<commit_message>
Daily IST report: add CSV/MD/XLSX
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J109"/>
+  <dimension ref="A1:K109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -438,8 +438,9 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,12 +484,17 @@
           <t>2026-02-19</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>2026-02-21</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -526,10 +532,13 @@
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K2" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -564,9 +573,12 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -605,7 +617,10 @@
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -640,9 +655,12 @@
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -683,6 +701,9 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -716,9 +737,12 @@
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -754,9 +778,12 @@
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" t="n">
         <v>2</v>
       </c>
     </row>
@@ -792,10 +819,13 @@
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K9" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -830,9 +860,12 @@
         <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" t="n">
         <v>2</v>
       </c>
     </row>
@@ -871,7 +904,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K11" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -906,10 +942,13 @@
         <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K12" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -944,10 +983,13 @@
         <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K13" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -982,9 +1024,12 @@
         <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1023,7 +1068,10 @@
         <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -1063,6 +1111,9 @@
       <c r="J16" t="n">
         <v>0</v>
       </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1096,9 +1147,12 @@
         <v>1</v>
       </c>
       <c r="I17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1134,10 +1188,13 @@
         <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J18" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K18" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -1172,10 +1229,13 @@
         <v>1</v>
       </c>
       <c r="I19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K19" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -1213,7 +1273,10 @@
         <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K20" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -1253,6 +1316,9 @@
       <c r="J21" t="n">
         <v>0</v>
       </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1291,6 +1357,9 @@
       <c r="J22" t="n">
         <v>0</v>
       </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1329,6 +1398,9 @@
       <c r="J23" t="n">
         <v>0</v>
       </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1365,7 +1437,10 @@
         <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -1400,9 +1475,12 @@
         <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
+        <v>2</v>
+      </c>
+      <c r="K25" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1443,6 +1521,9 @@
       <c r="J26" t="n">
         <v>0</v>
       </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1476,9 +1557,12 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
         <v>3</v>
       </c>
-      <c r="J27" t="n">
+      <c r="K27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1519,6 +1603,9 @@
       <c r="J28" t="n">
         <v>0</v>
       </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1557,6 +1644,9 @@
       <c r="J29" t="n">
         <v>0</v>
       </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1595,6 +1685,9 @@
       <c r="J30" t="n">
         <v>0</v>
       </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1628,10 +1721,13 @@
         <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K31" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -1666,9 +1762,12 @@
         <v>1</v>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
+        <v>2</v>
+      </c>
+      <c r="K32" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1704,9 +1803,12 @@
         <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1742,10 +1844,13 @@
         <v>1</v>
       </c>
       <c r="I34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K34" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -1780,10 +1885,13 @@
         <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J35" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K35" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="36">
@@ -1818,9 +1926,12 @@
         <v>1</v>
       </c>
       <c r="I36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1856,9 +1967,12 @@
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1899,6 +2013,9 @@
       <c r="J38" t="n">
         <v>0</v>
       </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1937,6 +2054,9 @@
       <c r="J39" t="n">
         <v>0</v>
       </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1970,10 +2090,13 @@
         <v>1</v>
       </c>
       <c r="I40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J40" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K40" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="41">
@@ -2008,9 +2131,12 @@
         <v>1</v>
       </c>
       <c r="I41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
+        <v>2</v>
+      </c>
+      <c r="K41" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2046,10 +2172,13 @@
         <v>1</v>
       </c>
       <c r="I42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J42" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K42" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="43">
@@ -2084,9 +2213,12 @@
         <v>0</v>
       </c>
       <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
         <v>21</v>
       </c>
-      <c r="J43" t="n">
+      <c r="K43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2127,6 +2259,9 @@
       <c r="J44" t="n">
         <v>0</v>
       </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2160,9 +2295,12 @@
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J45" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2198,10 +2336,13 @@
         <v>1</v>
       </c>
       <c r="I46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J46" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K46" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="47">
@@ -2236,10 +2377,13 @@
         <v>1</v>
       </c>
       <c r="I47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J47" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K47" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -2279,6 +2423,9 @@
       <c r="J48" t="n">
         <v>0</v>
       </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2312,10 +2459,13 @@
         <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J49" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K49" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -2353,7 +2503,10 @@
         <v>1</v>
       </c>
       <c r="J50" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K50" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="51">
@@ -2393,6 +2546,9 @@
       <c r="J51" t="n">
         <v>0</v>
       </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2426,9 +2582,12 @@
         <v>1</v>
       </c>
       <c r="I52" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J52" t="n">
+        <v>2</v>
+      </c>
+      <c r="K52" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2467,7 +2626,10 @@
         <v>1</v>
       </c>
       <c r="J53" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K53" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="54">
@@ -2507,6 +2669,9 @@
       <c r="J54" t="n">
         <v>0</v>
       </c>
+      <c r="K54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2540,9 +2705,12 @@
         <v>1</v>
       </c>
       <c r="I55" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J55" t="n">
+        <v>2</v>
+      </c>
+      <c r="K55" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2583,6 +2751,9 @@
       <c r="J56" t="n">
         <v>0</v>
       </c>
+      <c r="K56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2616,9 +2787,12 @@
         <v>1</v>
       </c>
       <c r="I57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J57" t="n">
+        <v>1</v>
+      </c>
+      <c r="K57" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2654,9 +2828,12 @@
         <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J58" t="n">
+        <v>1</v>
+      </c>
+      <c r="K58" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2692,9 +2869,12 @@
         <v>1</v>
       </c>
       <c r="I59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J59" t="n">
+        <v>1</v>
+      </c>
+      <c r="K59" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2730,10 +2910,13 @@
         <v>1</v>
       </c>
       <c r="I60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J60" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K60" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="61">
@@ -2771,7 +2954,10 @@
         <v>1</v>
       </c>
       <c r="J61" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K61" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="62">
@@ -2806,10 +2992,13 @@
         <v>0</v>
       </c>
       <c r="I62" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
+        <v>31</v>
+      </c>
+      <c r="K62" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -2844,10 +3033,13 @@
         <v>0</v>
       </c>
       <c r="I63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K63" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -2882,9 +3074,12 @@
         <v>1</v>
       </c>
       <c r="I64" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J64" t="n">
+        <v>2</v>
+      </c>
+      <c r="K64" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2925,6 +3120,9 @@
       <c r="J65" t="n">
         <v>0</v>
       </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2963,6 +3161,9 @@
       <c r="J66" t="n">
         <v>0</v>
       </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3001,6 +3202,9 @@
       <c r="J67" t="n">
         <v>0</v>
       </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3039,6 +3243,9 @@
       <c r="J68" t="n">
         <v>0</v>
       </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3077,6 +3284,9 @@
       <c r="J69" t="n">
         <v>0</v>
       </c>
+      <c r="K69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3110,10 +3320,13 @@
         <v>1</v>
       </c>
       <c r="I70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J70" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K70" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="71">
@@ -3153,6 +3366,9 @@
       <c r="J71" t="n">
         <v>0</v>
       </c>
+      <c r="K71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3191,6 +3407,9 @@
       <c r="J72" t="n">
         <v>0</v>
       </c>
+      <c r="K72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3229,6 +3448,9 @@
       <c r="J73" t="n">
         <v>0</v>
       </c>
+      <c r="K73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3262,9 +3484,12 @@
         <v>1</v>
       </c>
       <c r="I74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" t="n">
         <v>14</v>
       </c>
-      <c r="J74" t="n">
+      <c r="K74" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3305,6 +3530,9 @@
       <c r="J75" t="n">
         <v>0</v>
       </c>
+      <c r="K75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3341,7 +3569,10 @@
         <v>1</v>
       </c>
       <c r="J76" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K76" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="77">
@@ -3381,6 +3612,9 @@
       <c r="J77" t="n">
         <v>0</v>
       </c>
+      <c r="K77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3419,6 +3653,9 @@
       <c r="J78" t="n">
         <v>0</v>
       </c>
+      <c r="K78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3457,6 +3694,9 @@
       <c r="J79" t="n">
         <v>0</v>
       </c>
+      <c r="K79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3490,9 +3730,12 @@
         <v>1</v>
       </c>
       <c r="I80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K80" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3531,7 +3774,10 @@
         <v>1</v>
       </c>
       <c r="J81" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K81" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="82">
@@ -3566,10 +3812,13 @@
         <v>1</v>
       </c>
       <c r="I82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J82" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K82" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="83">
@@ -3609,6 +3858,9 @@
       <c r="J83" t="n">
         <v>0</v>
       </c>
+      <c r="K83" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3642,9 +3894,12 @@
         <v>0</v>
       </c>
       <c r="I84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J84" t="n">
+        <v>1</v>
+      </c>
+      <c r="K84" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3685,6 +3940,9 @@
       <c r="J85" t="n">
         <v>0</v>
       </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3718,9 +3976,12 @@
         <v>0</v>
       </c>
       <c r="I86" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J86" t="n">
+        <v>1</v>
+      </c>
+      <c r="K86" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3761,6 +4022,9 @@
       <c r="J87" t="n">
         <v>0</v>
       </c>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3797,7 +4061,10 @@
         <v>1</v>
       </c>
       <c r="J88" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K88" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="89">
@@ -3837,6 +4104,9 @@
       <c r="J89" t="n">
         <v>0</v>
       </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3875,6 +4145,9 @@
       <c r="J90" t="n">
         <v>0</v>
       </c>
+      <c r="K90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3913,6 +4186,9 @@
       <c r="J91" t="n">
         <v>0</v>
       </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3951,6 +4227,9 @@
       <c r="J92" t="n">
         <v>0</v>
       </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3989,6 +4268,9 @@
       <c r="J93" t="n">
         <v>0</v>
       </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4022,9 +4304,12 @@
         <v>1</v>
       </c>
       <c r="I94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J94" t="n">
+        <v>1</v>
+      </c>
+      <c r="K94" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4060,9 +4345,12 @@
         <v>1</v>
       </c>
       <c r="I95" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" t="n">
         <v>31</v>
       </c>
-      <c r="J95" t="n">
+      <c r="K95" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4103,6 +4391,9 @@
       <c r="J96" t="n">
         <v>0</v>
       </c>
+      <c r="K96" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4141,6 +4432,9 @@
       <c r="J97" t="n">
         <v>0</v>
       </c>
+      <c r="K97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4174,10 +4468,13 @@
         <v>0</v>
       </c>
       <c r="I98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J98" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K98" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -4217,6 +4514,9 @@
       <c r="J99" t="n">
         <v>0</v>
       </c>
+      <c r="K99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4250,9 +4550,12 @@
         <v>0</v>
       </c>
       <c r="I100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J100" t="n">
+        <v>1</v>
+      </c>
+      <c r="K100" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4288,10 +4591,13 @@
         <v>1</v>
       </c>
       <c r="I101" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J101" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K101" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="102">
@@ -4331,6 +4637,9 @@
       <c r="J102" t="n">
         <v>0</v>
       </c>
+      <c r="K102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4364,10 +4673,13 @@
         <v>1</v>
       </c>
       <c r="I103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J103" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K103" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="104">
@@ -4402,9 +4714,12 @@
         <v>0</v>
       </c>
       <c r="I104" t="n">
+        <v>0</v>
+      </c>
+      <c r="J104" t="n">
         <v>12</v>
       </c>
-      <c r="J104" t="n">
+      <c r="K104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4440,10 +4755,13 @@
         <v>1</v>
       </c>
       <c r="I105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J105" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K105" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="106">
@@ -4478,9 +4796,12 @@
         <v>1</v>
       </c>
       <c r="I106" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J106" t="n">
+        <v>2</v>
+      </c>
+      <c r="K106" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4521,6 +4842,9 @@
       <c r="J107" t="n">
         <v>0</v>
       </c>
+      <c r="K107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4557,7 +4881,10 @@
         <v>1</v>
       </c>
       <c r="J108" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K108" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="109">
@@ -4595,6 +4922,9 @@
         <v>0</v>
       </c>
       <c r="J109" t="n">
+        <v>0</v>
+      </c>
+      <c r="K109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1086)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O109"/>
+  <dimension ref="A1:P109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -443,8 +443,9 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,12 +514,17 @@
           <t>2026-02-27</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -571,11 +577,14 @@
         <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
         <v>6</v>
       </c>
+      <c r="P2" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -624,11 +633,14 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
         <v>5</v>
       </c>
+      <c r="P3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -677,10 +689,13 @@
         <v>1</v>
       </c>
       <c r="N4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="P4" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -730,11 +745,14 @@
         <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
         <v>7</v>
       </c>
+      <c r="P5" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -783,10 +801,13 @@
         <v>1</v>
       </c>
       <c r="N6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="P6" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -836,11 +857,14 @@
         <v>1</v>
       </c>
       <c r="N7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O7" t="n">
         <v>7</v>
       </c>
+      <c r="P7" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -889,11 +913,14 @@
         <v>1</v>
       </c>
       <c r="N8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
         <v>7</v>
       </c>
+      <c r="P8" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -942,10 +969,13 @@
         <v>1</v>
       </c>
       <c r="N9" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="P9" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -995,10 +1025,13 @@
         <v>1</v>
       </c>
       <c r="N10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O10" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="P10" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1048,11 +1081,14 @@
         <v>1</v>
       </c>
       <c r="N11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
         <v>6</v>
       </c>
+      <c r="P11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1101,10 +1137,13 @@
         <v>1</v>
       </c>
       <c r="N12" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O12" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="P12" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -1154,11 +1193,14 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
         <v>5</v>
       </c>
+      <c r="P13" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1207,11 +1249,14 @@
         <v>1</v>
       </c>
       <c r="N14" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O14" t="n">
         <v>7</v>
       </c>
+      <c r="P14" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1260,11 +1305,14 @@
         <v>1</v>
       </c>
       <c r="N15" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
         <v>5</v>
       </c>
+      <c r="P15" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1313,11 +1361,14 @@
         <v>1</v>
       </c>
       <c r="N16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
         <v>5</v>
       </c>
+      <c r="P16" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1366,11 +1417,14 @@
         <v>1</v>
       </c>
       <c r="N17" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O17" t="n">
         <v>7</v>
       </c>
+      <c r="P17" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1419,10 +1473,13 @@
         <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O18" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="P18" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="19">
@@ -1472,10 +1529,13 @@
         <v>1</v>
       </c>
       <c r="N19" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O19" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="P19" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -1525,11 +1585,14 @@
         <v>1</v>
       </c>
       <c r="N20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
         <v>6</v>
       </c>
+      <c r="P20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1583,6 +1646,9 @@
       <c r="O21" t="n">
         <v>0</v>
       </c>
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1636,6 +1702,9 @@
       <c r="O22" t="n">
         <v>0</v>
       </c>
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1684,11 +1753,14 @@
         <v>1</v>
       </c>
       <c r="N23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O23" t="n">
         <v>2</v>
       </c>
+      <c r="P23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1737,11 +1809,14 @@
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O24" t="n">
         <v>6</v>
       </c>
+      <c r="P24" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1790,11 +1865,14 @@
         <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O25" t="n">
         <v>5</v>
       </c>
+      <c r="P25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1843,11 +1921,14 @@
         <v>1</v>
       </c>
       <c r="N26" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O26" t="n">
         <v>4</v>
       </c>
+      <c r="P26" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1896,9 +1977,12 @@
         <v>1</v>
       </c>
       <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
         <v>8</v>
       </c>
-      <c r="O27" t="n">
+      <c r="P27" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1954,6 +2038,9 @@
       <c r="O28" t="n">
         <v>0</v>
       </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2007,6 +2094,9 @@
       <c r="O29" t="n">
         <v>0</v>
       </c>
+      <c r="P29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2060,6 +2150,9 @@
       <c r="O30" t="n">
         <v>0</v>
       </c>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2108,10 +2201,13 @@
         <v>1</v>
       </c>
       <c r="N31" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O31" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="P31" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="32">
@@ -2161,11 +2257,14 @@
         <v>1</v>
       </c>
       <c r="N32" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O32" t="n">
         <v>7</v>
       </c>
+      <c r="P32" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2214,11 +2313,14 @@
         <v>1</v>
       </c>
       <c r="N33" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O33" t="n">
         <v>7</v>
       </c>
+      <c r="P33" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2267,10 +2369,13 @@
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O34" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="P34" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="35">
@@ -2320,11 +2425,14 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O35" t="n">
         <v>5</v>
       </c>
+      <c r="P35" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2373,11 +2481,14 @@
         <v>1</v>
       </c>
       <c r="N36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O36" t="n">
         <v>6</v>
       </c>
+      <c r="P36" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2426,11 +2537,14 @@
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O37" t="n">
         <v>3</v>
       </c>
+      <c r="P37" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2484,6 +2598,9 @@
       <c r="O38" t="n">
         <v>0</v>
       </c>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2537,6 +2654,9 @@
       <c r="O39" t="n">
         <v>0</v>
       </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2585,11 +2705,14 @@
         <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O40" t="n">
         <v>7</v>
       </c>
+      <c r="P40" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2638,11 +2761,14 @@
         <v>1</v>
       </c>
       <c r="N41" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O41" t="n">
         <v>7</v>
       </c>
+      <c r="P41" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2691,10 +2817,13 @@
         <v>1</v>
       </c>
       <c r="N42" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O42" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="P42" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="43">
@@ -2744,9 +2873,12 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" t="n">
         <v>21</v>
       </c>
-      <c r="O43" t="n">
+      <c r="P43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2797,9 +2929,12 @@
         <v>1</v>
       </c>
       <c r="N44" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" t="n">
         <v>45</v>
       </c>
-      <c r="O44" t="n">
+      <c r="P44" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2850,10 +2985,13 @@
         <v>1</v>
       </c>
       <c r="N45" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O45" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="P45" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="46">
@@ -2903,10 +3041,13 @@
         <v>1</v>
       </c>
       <c r="N46" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O46" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="P46" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="47">
@@ -2956,11 +3097,14 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O47" t="n">
         <v>6</v>
       </c>
+      <c r="P47" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3014,6 +3158,9 @@
       <c r="O48" t="n">
         <v>0</v>
       </c>
+      <c r="P48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3062,10 +3209,13 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O49" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="P49" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="50">
@@ -3115,11 +3265,14 @@
         <v>1</v>
       </c>
       <c r="N50" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O50" t="n">
         <v>6</v>
       </c>
+      <c r="P50" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3168,11 +3321,14 @@
         <v>1</v>
       </c>
       <c r="N51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O51" t="n">
         <v>2</v>
       </c>
+      <c r="P51" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3221,11 +3377,14 @@
         <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O52" t="n">
         <v>3</v>
       </c>
+      <c r="P52" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3274,10 +3433,13 @@
         <v>1</v>
       </c>
       <c r="N53" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O53" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="P53" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="54">
@@ -3332,6 +3494,9 @@
       <c r="O54" t="n">
         <v>0</v>
       </c>
+      <c r="P54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3380,11 +3545,14 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O55" t="n">
         <v>6</v>
       </c>
+      <c r="P55" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3438,6 +3606,9 @@
       <c r="O56" t="n">
         <v>0</v>
       </c>
+      <c r="P56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3486,11 +3657,14 @@
         <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O57" t="n">
         <v>6</v>
       </c>
+      <c r="P57" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3539,11 +3713,14 @@
         <v>1</v>
       </c>
       <c r="N58" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O58" t="n">
         <v>6</v>
       </c>
+      <c r="P58" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3592,11 +3769,14 @@
         <v>0</v>
       </c>
       <c r="N59" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O59" t="n">
         <v>3</v>
       </c>
+      <c r="P59" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3645,10 +3825,13 @@
         <v>1</v>
       </c>
       <c r="N60" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O60" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="P60" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="61">
@@ -3698,9 +3881,12 @@
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O61" t="n">
+        <v>1</v>
+      </c>
+      <c r="P61" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3756,6 +3942,9 @@
       <c r="O62" t="n">
         <v>0</v>
       </c>
+      <c r="P62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3804,11 +3993,14 @@
         <v>1</v>
       </c>
       <c r="N63" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O63" t="n">
         <v>4</v>
       </c>
+      <c r="P63" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3857,11 +4049,14 @@
         <v>1</v>
       </c>
       <c r="N64" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O64" t="n">
         <v>7</v>
       </c>
+      <c r="P64" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3915,6 +4110,9 @@
       <c r="O65" t="n">
         <v>0</v>
       </c>
+      <c r="P65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3968,6 +4166,9 @@
       <c r="O66" t="n">
         <v>0</v>
       </c>
+      <c r="P66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4016,11 +4217,14 @@
         <v>1</v>
       </c>
       <c r="N67" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O67" t="n">
         <v>3</v>
       </c>
+      <c r="P67" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4074,6 +4278,9 @@
       <c r="O68" t="n">
         <v>0</v>
       </c>
+      <c r="P68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4127,6 +4334,9 @@
       <c r="O69" t="n">
         <v>0</v>
       </c>
+      <c r="P69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4175,10 +4385,13 @@
         <v>1</v>
       </c>
       <c r="N70" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O70" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="P70" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="71">
@@ -4228,9 +4441,12 @@
         <v>0</v>
       </c>
       <c r="N71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P71" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4286,6 +4502,9 @@
       <c r="O72" t="n">
         <v>0</v>
       </c>
+      <c r="P72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4334,11 +4553,14 @@
         <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O73" t="n">
         <v>3</v>
       </c>
+      <c r="P73" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4387,9 +4609,12 @@
         <v>1</v>
       </c>
       <c r="N74" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" t="n">
         <v>18</v>
       </c>
-      <c r="O74" t="n">
+      <c r="P74" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4440,11 +4665,14 @@
         <v>1</v>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O75" t="n">
         <v>2</v>
       </c>
+      <c r="P75" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4493,10 +4721,13 @@
         <v>1</v>
       </c>
       <c r="N76" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O76" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="P76" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="77">
@@ -4551,6 +4782,9 @@
       <c r="O77" t="n">
         <v>0</v>
       </c>
+      <c r="P77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4604,6 +4838,9 @@
       <c r="O78" t="n">
         <v>0</v>
       </c>
+      <c r="P78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4652,11 +4889,14 @@
         <v>0</v>
       </c>
       <c r="N79" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O79" t="n">
         <v>3</v>
       </c>
+      <c r="P79" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4705,11 +4945,14 @@
         <v>1</v>
       </c>
       <c r="N80" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O80" t="n">
         <v>6</v>
       </c>
+      <c r="P80" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4758,10 +5001,13 @@
         <v>1</v>
       </c>
       <c r="N81" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O81" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="P81" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="82">
@@ -4811,11 +5057,14 @@
         <v>1</v>
       </c>
       <c r="N82" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O82" t="n">
         <v>7</v>
       </c>
+      <c r="P82" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4864,11 +5113,14 @@
         <v>1</v>
       </c>
       <c r="N83" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O83" t="n">
         <v>4</v>
       </c>
+      <c r="P83" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4917,9 +5169,12 @@
         <v>0</v>
       </c>
       <c r="N84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O84" t="n">
+        <v>1</v>
+      </c>
+      <c r="P84" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4975,6 +5230,9 @@
       <c r="O85" t="n">
         <v>0</v>
       </c>
+      <c r="P85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5023,11 +5281,14 @@
         <v>1</v>
       </c>
       <c r="N86" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O86" t="n">
         <v>4</v>
       </c>
+      <c r="P86" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5081,6 +5342,9 @@
       <c r="O87" t="n">
         <v>0</v>
       </c>
+      <c r="P87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5129,11 +5393,14 @@
         <v>1</v>
       </c>
       <c r="N88" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O88" t="n">
         <v>3</v>
       </c>
+      <c r="P88" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5187,6 +5454,9 @@
       <c r="O89" t="n">
         <v>0</v>
       </c>
+      <c r="P89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5235,11 +5505,14 @@
         <v>0</v>
       </c>
       <c r="N90" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O90" t="n">
         <v>2</v>
       </c>
+      <c r="P90" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5293,6 +5566,9 @@
       <c r="O91" t="n">
         <v>0</v>
       </c>
+      <c r="P91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5346,6 +5622,9 @@
       <c r="O92" t="n">
         <v>0</v>
       </c>
+      <c r="P92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5394,11 +5673,14 @@
         <v>1</v>
       </c>
       <c r="N93" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O93" t="n">
         <v>4</v>
       </c>
+      <c r="P93" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5447,11 +5729,14 @@
         <v>1</v>
       </c>
       <c r="N94" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O94" t="n">
         <v>5</v>
       </c>
+      <c r="P94" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5500,9 +5785,12 @@
         <v>1</v>
       </c>
       <c r="N95" t="n">
+        <v>0</v>
+      </c>
+      <c r="O95" t="n">
         <v>34</v>
       </c>
-      <c r="O95" t="n">
+      <c r="P95" t="n">
         <v>5</v>
       </c>
     </row>
@@ -5553,11 +5841,14 @@
         <v>1</v>
       </c>
       <c r="N96" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O96" t="n">
         <v>2</v>
       </c>
+      <c r="P96" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5611,6 +5902,9 @@
       <c r="O97" t="n">
         <v>0</v>
       </c>
+      <c r="P97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5659,11 +5953,14 @@
         <v>1</v>
       </c>
       <c r="N98" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O98" t="n">
         <v>3</v>
       </c>
+      <c r="P98" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5717,6 +6014,9 @@
       <c r="O99" t="n">
         <v>0</v>
       </c>
+      <c r="P99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5765,11 +6065,14 @@
         <v>0</v>
       </c>
       <c r="N100" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O100" t="n">
         <v>2</v>
       </c>
+      <c r="P100" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5818,11 +6121,14 @@
         <v>1</v>
       </c>
       <c r="N101" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O101" t="n">
         <v>7</v>
       </c>
+      <c r="P101" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5876,6 +6182,9 @@
       <c r="O102" t="n">
         <v>0</v>
       </c>
+      <c r="P102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5924,10 +6233,13 @@
         <v>1</v>
       </c>
       <c r="N103" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O103" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="P103" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="104">
@@ -5977,9 +6289,12 @@
         <v>0</v>
       </c>
       <c r="N104" t="n">
+        <v>0</v>
+      </c>
+      <c r="O104" t="n">
         <v>12</v>
       </c>
-      <c r="O104" t="n">
+      <c r="P104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6030,11 +6345,14 @@
         <v>1</v>
       </c>
       <c r="N105" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O105" t="n">
         <v>7</v>
       </c>
+      <c r="P105" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -6083,11 +6401,14 @@
         <v>0</v>
       </c>
       <c r="N106" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O106" t="n">
         <v>6</v>
       </c>
+      <c r="P106" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -6141,6 +6462,9 @@
       <c r="O107" t="n">
         <v>0</v>
       </c>
+      <c r="P107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6189,11 +6513,14 @@
         <v>1</v>
       </c>
       <c r="N108" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O108" t="n">
         <v>6</v>
       </c>
+      <c r="P108" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6245,6 +6572,9 @@
         <v>0</v>
       </c>
       <c r="O109" t="n">
+        <v>0</v>
+      </c>
+      <c r="P109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1149)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P109"/>
+  <dimension ref="A1:Q109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -444,8 +444,9 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -519,12 +520,17 @@
           <t>2026-02-28</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -580,11 +586,14 @@
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
         <v>6</v>
       </c>
+      <c r="Q2" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -636,11 +645,14 @@
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
         <v>5</v>
       </c>
+      <c r="Q3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -692,11 +704,14 @@
         <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P4" t="n">
         <v>7</v>
       </c>
+      <c r="Q4" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -748,11 +763,14 @@
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
         <v>7</v>
       </c>
+      <c r="Q5" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -804,11 +822,14 @@
         <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
         <v>6</v>
       </c>
+      <c r="Q6" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -860,11 +881,14 @@
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
         <v>7</v>
       </c>
+      <c r="Q7" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -916,11 +940,14 @@
         <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
         <v>7</v>
       </c>
+      <c r="Q8" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -972,11 +999,14 @@
         <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P9" t="n">
         <v>8</v>
       </c>
+      <c r="Q9" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1028,11 +1058,14 @@
         <v>1</v>
       </c>
       <c r="O10" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
         <v>7</v>
       </c>
+      <c r="Q10" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1084,11 +1117,14 @@
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P11" t="n">
         <v>6</v>
       </c>
+      <c r="Q11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1140,11 +1176,14 @@
         <v>1</v>
       </c>
       <c r="O12" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P12" t="n">
         <v>8</v>
       </c>
+      <c r="Q12" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1196,11 +1235,14 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P13" t="n">
         <v>5</v>
       </c>
+      <c r="Q13" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1252,11 +1294,14 @@
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P14" t="n">
         <v>7</v>
       </c>
+      <c r="Q14" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1308,11 +1353,14 @@
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P15" t="n">
         <v>5</v>
       </c>
+      <c r="Q15" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1364,11 +1412,14 @@
         <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P16" t="n">
         <v>5</v>
       </c>
+      <c r="Q16" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1420,11 +1471,14 @@
         <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P17" t="n">
         <v>7</v>
       </c>
+      <c r="Q17" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1476,11 +1530,14 @@
         <v>1</v>
       </c>
       <c r="O18" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P18" t="n">
         <v>8</v>
       </c>
+      <c r="Q18" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1532,11 +1589,14 @@
         <v>1</v>
       </c>
       <c r="O19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P19" t="n">
         <v>6</v>
       </c>
+      <c r="Q19" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1588,11 +1648,14 @@
         <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P20" t="n">
         <v>6</v>
       </c>
+      <c r="Q20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1649,6 +1712,9 @@
       <c r="P21" t="n">
         <v>0</v>
       </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1705,6 +1771,9 @@
       <c r="P22" t="n">
         <v>0</v>
       </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1756,11 +1825,14 @@
         <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P23" t="n">
         <v>2</v>
       </c>
+      <c r="Q23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1812,11 +1884,14 @@
         <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P24" t="n">
         <v>6</v>
       </c>
+      <c r="Q24" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1868,11 +1943,14 @@
         <v>0</v>
       </c>
       <c r="O25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P25" t="n">
         <v>5</v>
       </c>
+      <c r="Q25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1924,11 +2002,14 @@
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P26" t="n">
         <v>4</v>
       </c>
+      <c r="Q26" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1980,9 +2061,12 @@
         <v>0</v>
       </c>
       <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
         <v>8</v>
       </c>
-      <c r="P27" t="n">
+      <c r="Q27" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2041,6 +2125,9 @@
       <c r="P28" t="n">
         <v>0</v>
       </c>
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2097,6 +2184,9 @@
       <c r="P29" t="n">
         <v>0</v>
       </c>
+      <c r="Q29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2153,6 +2243,9 @@
       <c r="P30" t="n">
         <v>0</v>
       </c>
+      <c r="Q30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2204,11 +2297,14 @@
         <v>1</v>
       </c>
       <c r="O31" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P31" t="n">
         <v>8</v>
       </c>
+      <c r="Q31" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2260,11 +2356,14 @@
         <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P32" t="n">
         <v>7</v>
       </c>
+      <c r="Q32" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2316,10 +2415,13 @@
         <v>0</v>
       </c>
       <c r="O33" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="P33" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="34">
@@ -2372,11 +2474,14 @@
         <v>1</v>
       </c>
       <c r="O34" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P34" t="n">
         <v>7</v>
       </c>
+      <c r="Q34" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2428,11 +2533,14 @@
         <v>0</v>
       </c>
       <c r="O35" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P35" t="n">
         <v>5</v>
       </c>
+      <c r="Q35" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2484,11 +2592,14 @@
         <v>0</v>
       </c>
       <c r="O36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P36" t="n">
         <v>6</v>
       </c>
+      <c r="Q36" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2540,11 +2651,14 @@
         <v>0</v>
       </c>
       <c r="O37" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P37" t="n">
         <v>3</v>
       </c>
+      <c r="Q37" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2601,6 +2715,9 @@
       <c r="P38" t="n">
         <v>0</v>
       </c>
+      <c r="Q38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2657,6 +2774,9 @@
       <c r="P39" t="n">
         <v>0</v>
       </c>
+      <c r="Q39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2708,11 +2828,14 @@
         <v>0</v>
       </c>
       <c r="O40" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P40" t="n">
         <v>7</v>
       </c>
+      <c r="Q40" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2764,11 +2887,14 @@
         <v>0</v>
       </c>
       <c r="O41" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P41" t="n">
         <v>7</v>
       </c>
+      <c r="Q41" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2820,11 +2946,14 @@
         <v>1</v>
       </c>
       <c r="O42" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P42" t="n">
         <v>8</v>
       </c>
+      <c r="Q42" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2876,9 +3005,12 @@
         <v>0</v>
       </c>
       <c r="O43" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" t="n">
         <v>21</v>
       </c>
-      <c r="P43" t="n">
+      <c r="Q43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2932,9 +3064,12 @@
         <v>0</v>
       </c>
       <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
         <v>45</v>
       </c>
-      <c r="P44" t="n">
+      <c r="Q44" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2988,11 +3123,14 @@
         <v>1</v>
       </c>
       <c r="O45" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
         <v>5</v>
       </c>
+      <c r="Q45" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3044,11 +3182,14 @@
         <v>1</v>
       </c>
       <c r="O46" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P46" t="n">
         <v>8</v>
       </c>
+      <c r="Q46" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3100,11 +3241,14 @@
         <v>0</v>
       </c>
       <c r="O47" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P47" t="n">
         <v>6</v>
       </c>
+      <c r="Q47" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3161,6 +3305,9 @@
       <c r="P48" t="n">
         <v>0</v>
       </c>
+      <c r="Q48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3212,11 +3359,14 @@
         <v>1</v>
       </c>
       <c r="O49" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P49" t="n">
         <v>7</v>
       </c>
+      <c r="Q49" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3268,11 +3418,14 @@
         <v>0</v>
       </c>
       <c r="O50" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P50" t="n">
         <v>6</v>
       </c>
+      <c r="Q50" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3324,11 +3477,14 @@
         <v>0</v>
       </c>
       <c r="O51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P51" t="n">
         <v>2</v>
       </c>
+      <c r="Q51" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3380,11 +3536,14 @@
         <v>0</v>
       </c>
       <c r="O52" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P52" t="n">
         <v>3</v>
       </c>
+      <c r="Q52" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3436,11 +3595,14 @@
         <v>1</v>
       </c>
       <c r="O53" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P53" t="n">
         <v>7</v>
       </c>
+      <c r="Q53" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3497,6 +3659,9 @@
       <c r="P54" t="n">
         <v>0</v>
       </c>
+      <c r="Q54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3548,11 +3713,14 @@
         <v>0</v>
       </c>
       <c r="O55" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P55" t="n">
         <v>6</v>
       </c>
+      <c r="Q55" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3609,6 +3777,9 @@
       <c r="P56" t="n">
         <v>0</v>
       </c>
+      <c r="Q56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3660,11 +3831,14 @@
         <v>0</v>
       </c>
       <c r="O57" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P57" t="n">
         <v>6</v>
       </c>
+      <c r="Q57" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3716,11 +3890,14 @@
         <v>0</v>
       </c>
       <c r="O58" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P58" t="n">
         <v>6</v>
       </c>
+      <c r="Q58" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3772,11 +3949,14 @@
         <v>0</v>
       </c>
       <c r="O59" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P59" t="n">
         <v>3</v>
       </c>
+      <c r="Q59" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3828,11 +4008,14 @@
         <v>1</v>
       </c>
       <c r="O60" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P60" t="n">
         <v>8</v>
       </c>
+      <c r="Q60" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3884,9 +4067,12 @@
         <v>0</v>
       </c>
       <c r="O61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P61" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q61" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3945,6 +4131,9 @@
       <c r="P62" t="n">
         <v>0</v>
       </c>
+      <c r="Q62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3996,11 +4185,14 @@
         <v>0</v>
       </c>
       <c r="O63" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P63" t="n">
         <v>4</v>
       </c>
+      <c r="Q63" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4052,11 +4244,14 @@
         <v>0</v>
       </c>
       <c r="O64" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P64" t="n">
         <v>7</v>
       </c>
+      <c r="Q64" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4113,6 +4308,9 @@
       <c r="P65" t="n">
         <v>0</v>
       </c>
+      <c r="Q65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4169,6 +4367,9 @@
       <c r="P66" t="n">
         <v>0</v>
       </c>
+      <c r="Q66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4220,11 +4421,14 @@
         <v>0</v>
       </c>
       <c r="O67" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P67" t="n">
         <v>3</v>
       </c>
+      <c r="Q67" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4281,6 +4485,9 @@
       <c r="P68" t="n">
         <v>0</v>
       </c>
+      <c r="Q68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4337,6 +4544,9 @@
       <c r="P69" t="n">
         <v>0</v>
       </c>
+      <c r="Q69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4388,11 +4598,14 @@
         <v>1</v>
       </c>
       <c r="O70" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P70" t="n">
         <v>8</v>
       </c>
+      <c r="Q70" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4444,9 +4657,12 @@
         <v>0</v>
       </c>
       <c r="O71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q71" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4505,6 +4721,9 @@
       <c r="P72" t="n">
         <v>0</v>
       </c>
+      <c r="Q72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4556,11 +4775,14 @@
         <v>0</v>
       </c>
       <c r="O73" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P73" t="n">
         <v>3</v>
       </c>
+      <c r="Q73" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4612,9 +4834,12 @@
         <v>0</v>
       </c>
       <c r="O74" t="n">
+        <v>0</v>
+      </c>
+      <c r="P74" t="n">
         <v>18</v>
       </c>
-      <c r="P74" t="n">
+      <c r="Q74" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4668,11 +4893,14 @@
         <v>0</v>
       </c>
       <c r="O75" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P75" t="n">
         <v>2</v>
       </c>
+      <c r="Q75" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4724,11 +4952,14 @@
         <v>1</v>
       </c>
       <c r="O76" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P76" t="n">
         <v>6</v>
       </c>
+      <c r="Q76" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4785,6 +5016,9 @@
       <c r="P77" t="n">
         <v>0</v>
       </c>
+      <c r="Q77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4841,6 +5075,9 @@
       <c r="P78" t="n">
         <v>0</v>
       </c>
+      <c r="Q78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4892,11 +5129,14 @@
         <v>0</v>
       </c>
       <c r="O79" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P79" t="n">
         <v>3</v>
       </c>
+      <c r="Q79" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4948,11 +5188,14 @@
         <v>0</v>
       </c>
       <c r="O80" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P80" t="n">
         <v>6</v>
       </c>
+      <c r="Q80" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5004,11 +5247,14 @@
         <v>1</v>
       </c>
       <c r="O81" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P81" t="n">
         <v>6</v>
       </c>
+      <c r="Q81" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5060,11 +5306,14 @@
         <v>0</v>
       </c>
       <c r="O82" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P82" t="n">
         <v>7</v>
       </c>
+      <c r="Q82" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5116,11 +5365,14 @@
         <v>0</v>
       </c>
       <c r="O83" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P83" t="n">
         <v>4</v>
       </c>
+      <c r="Q83" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5172,9 +5424,12 @@
         <v>0</v>
       </c>
       <c r="O84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P84" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q84" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5233,6 +5488,9 @@
       <c r="P85" t="n">
         <v>0</v>
       </c>
+      <c r="Q85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5284,11 +5542,14 @@
         <v>0</v>
       </c>
       <c r="O86" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P86" t="n">
         <v>4</v>
       </c>
+      <c r="Q86" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5345,6 +5606,9 @@
       <c r="P87" t="n">
         <v>0</v>
       </c>
+      <c r="Q87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5396,11 +5660,14 @@
         <v>0</v>
       </c>
       <c r="O88" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P88" t="n">
         <v>3</v>
       </c>
+      <c r="Q88" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5457,6 +5724,9 @@
       <c r="P89" t="n">
         <v>0</v>
       </c>
+      <c r="Q89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5508,11 +5778,14 @@
         <v>0</v>
       </c>
       <c r="O90" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P90" t="n">
         <v>2</v>
       </c>
+      <c r="Q90" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5569,6 +5842,9 @@
       <c r="P91" t="n">
         <v>0</v>
       </c>
+      <c r="Q91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5625,6 +5901,9 @@
       <c r="P92" t="n">
         <v>0</v>
       </c>
+      <c r="Q92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5676,11 +5955,14 @@
         <v>0</v>
       </c>
       <c r="O93" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P93" t="n">
         <v>4</v>
       </c>
+      <c r="Q93" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5732,11 +6014,14 @@
         <v>0</v>
       </c>
       <c r="O94" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P94" t="n">
         <v>5</v>
       </c>
+      <c r="Q94" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5788,9 +6073,12 @@
         <v>0</v>
       </c>
       <c r="O95" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" t="n">
         <v>34</v>
       </c>
-      <c r="P95" t="n">
+      <c r="Q95" t="n">
         <v>5</v>
       </c>
     </row>
@@ -5844,11 +6132,14 @@
         <v>0</v>
       </c>
       <c r="O96" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P96" t="n">
         <v>2</v>
       </c>
+      <c r="Q96" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5905,6 +6196,9 @@
       <c r="P97" t="n">
         <v>0</v>
       </c>
+      <c r="Q97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5956,11 +6250,14 @@
         <v>0</v>
       </c>
       <c r="O98" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P98" t="n">
         <v>3</v>
       </c>
+      <c r="Q98" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6017,6 +6314,9 @@
       <c r="P99" t="n">
         <v>0</v>
       </c>
+      <c r="Q99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6068,11 +6368,14 @@
         <v>0</v>
       </c>
       <c r="O100" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P100" t="n">
         <v>2</v>
       </c>
+      <c r="Q100" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6124,11 +6427,14 @@
         <v>0</v>
       </c>
       <c r="O101" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P101" t="n">
         <v>7</v>
       </c>
+      <c r="Q101" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6185,6 +6491,9 @@
       <c r="P102" t="n">
         <v>0</v>
       </c>
+      <c r="Q102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -6236,11 +6545,14 @@
         <v>1</v>
       </c>
       <c r="O103" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P103" t="n">
         <v>8</v>
       </c>
+      <c r="Q103" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6292,9 +6604,12 @@
         <v>0</v>
       </c>
       <c r="O104" t="n">
+        <v>0</v>
+      </c>
+      <c r="P104" t="n">
         <v>12</v>
       </c>
-      <c r="P104" t="n">
+      <c r="Q104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6348,11 +6663,14 @@
         <v>0</v>
       </c>
       <c r="O105" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P105" t="n">
         <v>7</v>
       </c>
+      <c r="Q105" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -6404,11 +6722,14 @@
         <v>0</v>
       </c>
       <c r="O106" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P106" t="n">
         <v>6</v>
       </c>
+      <c r="Q106" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -6465,6 +6786,9 @@
       <c r="P107" t="n">
         <v>0</v>
       </c>
+      <c r="Q107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6516,11 +6840,14 @@
         <v>0</v>
       </c>
       <c r="O108" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P108" t="n">
         <v>6</v>
       </c>
+      <c r="Q108" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6575,6 +6902,9 @@
         <v>0</v>
       </c>
       <c r="P109" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1251)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q109"/>
+  <dimension ref="A1:R109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -445,8 +445,9 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,12 +526,17 @@
           <t>2026-03-01</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -589,10 +595,13 @@
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R2" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -648,10 +657,13 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="R3" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -707,10 +719,13 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R4" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -766,10 +781,13 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R5" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -825,10 +843,13 @@
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R6" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -884,10 +905,13 @@
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R7" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -943,10 +967,13 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R8" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -1002,10 +1029,13 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="R9" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -1061,10 +1091,13 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R10" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -1120,10 +1153,13 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R11" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1179,10 +1215,13 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="R12" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -1238,11 +1277,14 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
         <v>5</v>
       </c>
+      <c r="R13" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1297,10 +1339,13 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R14" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -1356,10 +1401,13 @@
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="R15" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -1415,10 +1463,13 @@
         <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="R16" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -1474,10 +1525,13 @@
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R17" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="18">
@@ -1533,10 +1587,13 @@
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="R18" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="19">
@@ -1592,10 +1649,13 @@
         <v>0</v>
       </c>
       <c r="P19" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q19" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R19" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="20">
@@ -1651,10 +1711,13 @@
         <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q20" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R20" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="21">
@@ -1715,6 +1778,9 @@
       <c r="Q21" t="n">
         <v>0</v>
       </c>
+      <c r="R21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1774,6 +1840,9 @@
       <c r="Q22" t="n">
         <v>0</v>
       </c>
+      <c r="R22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1828,10 +1897,13 @@
         <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="R23" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -1887,10 +1959,13 @@
         <v>0</v>
       </c>
       <c r="P24" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q24" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R24" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="25">
@@ -1946,11 +2021,14 @@
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q25" t="n">
         <v>5</v>
       </c>
+      <c r="R25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2005,10 +2083,13 @@
         <v>0</v>
       </c>
       <c r="P26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q26" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="R26" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="27">
@@ -2064,10 +2145,13 @@
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Q27" t="n">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="R27" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="28">
@@ -2128,6 +2212,9 @@
       <c r="Q28" t="n">
         <v>0</v>
       </c>
+      <c r="R28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2187,6 +2274,9 @@
       <c r="Q29" t="n">
         <v>0</v>
       </c>
+      <c r="R29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2241,10 +2331,13 @@
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="R30" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -2300,11 +2393,14 @@
         <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q31" t="n">
         <v>8</v>
       </c>
+      <c r="R31" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2359,10 +2455,13 @@
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q32" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R32" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="33">
@@ -2418,11 +2517,14 @@
         <v>1</v>
       </c>
       <c r="P33" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q33" t="n">
         <v>8</v>
       </c>
+      <c r="R33" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2477,10 +2579,13 @@
         <v>0</v>
       </c>
       <c r="P34" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R34" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="35">
@@ -2536,11 +2641,14 @@
         <v>0</v>
       </c>
       <c r="P35" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q35" t="n">
         <v>5</v>
       </c>
+      <c r="R35" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2595,10 +2703,13 @@
         <v>0</v>
       </c>
       <c r="P36" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q36" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R36" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="37">
@@ -2654,11 +2765,14 @@
         <v>0</v>
       </c>
       <c r="P37" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q37" t="n">
         <v>3</v>
       </c>
+      <c r="R37" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2718,6 +2832,9 @@
       <c r="Q38" t="n">
         <v>0</v>
       </c>
+      <c r="R38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2772,10 +2889,13 @@
         <v>0</v>
       </c>
       <c r="P39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="R39" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -2831,10 +2951,13 @@
         <v>0</v>
       </c>
       <c r="P40" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R40" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="41">
@@ -2890,10 +3013,13 @@
         <v>0</v>
       </c>
       <c r="P41" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R41" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="42">
@@ -2949,10 +3075,13 @@
         <v>0</v>
       </c>
       <c r="P42" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="R42" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="43">
@@ -3008,9 +3137,12 @@
         <v>0</v>
       </c>
       <c r="P43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" t="n">
         <v>21</v>
       </c>
-      <c r="Q43" t="n">
+      <c r="R43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3067,9 +3199,12 @@
         <v>0</v>
       </c>
       <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="n">
         <v>45</v>
       </c>
-      <c r="Q44" t="n">
+      <c r="R44" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3126,10 +3261,13 @@
         <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q45" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="R45" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="46">
@@ -3185,10 +3323,13 @@
         <v>0</v>
       </c>
       <c r="P46" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Q46" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="R46" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="47">
@@ -3244,11 +3385,14 @@
         <v>0</v>
       </c>
       <c r="P47" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q47" t="n">
         <v>6</v>
       </c>
+      <c r="R47" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3308,6 +3452,9 @@
       <c r="Q48" t="n">
         <v>0</v>
       </c>
+      <c r="R48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3362,10 +3509,13 @@
         <v>0</v>
       </c>
       <c r="P49" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q49" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R49" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="50">
@@ -3421,10 +3571,13 @@
         <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q50" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R50" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="51">
@@ -3480,11 +3633,14 @@
         <v>0</v>
       </c>
       <c r="P51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q51" t="n">
         <v>2</v>
       </c>
+      <c r="R51" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3539,11 +3695,14 @@
         <v>0</v>
       </c>
       <c r="P52" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q52" t="n">
         <v>3</v>
       </c>
+      <c r="R52" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3598,10 +3757,13 @@
         <v>0</v>
       </c>
       <c r="P53" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q53" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R53" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="54">
@@ -3662,6 +3824,9 @@
       <c r="Q54" t="n">
         <v>0</v>
       </c>
+      <c r="R54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3716,10 +3881,13 @@
         <v>0</v>
       </c>
       <c r="P55" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q55" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R55" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="56">
@@ -3780,6 +3948,9 @@
       <c r="Q56" t="n">
         <v>0</v>
       </c>
+      <c r="R56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3834,10 +4005,13 @@
         <v>0</v>
       </c>
       <c r="P57" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q57" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R57" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="58">
@@ -3893,10 +4067,13 @@
         <v>0</v>
       </c>
       <c r="P58" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q58" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R58" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="59">
@@ -3952,11 +4129,14 @@
         <v>0</v>
       </c>
       <c r="P59" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q59" t="n">
         <v>3</v>
       </c>
+      <c r="R59" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4011,10 +4191,13 @@
         <v>0</v>
       </c>
       <c r="P60" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Q60" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="R60" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="61">
@@ -4073,7 +4256,10 @@
         <v>1</v>
       </c>
       <c r="Q61" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="R61" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="62">
@@ -4134,6 +4320,9 @@
       <c r="Q62" t="n">
         <v>0</v>
       </c>
+      <c r="R62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4188,10 +4377,13 @@
         <v>0</v>
       </c>
       <c r="P63" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q63" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="R63" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="64">
@@ -4247,10 +4439,13 @@
         <v>0</v>
       </c>
       <c r="P64" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q64" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R64" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="65">
@@ -4311,6 +4506,9 @@
       <c r="Q65" t="n">
         <v>0</v>
       </c>
+      <c r="R65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4370,6 +4568,9 @@
       <c r="Q66" t="n">
         <v>0</v>
       </c>
+      <c r="R66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4424,10 +4625,13 @@
         <v>0</v>
       </c>
       <c r="P67" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q67" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="R67" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="68">
@@ -4488,6 +4692,9 @@
       <c r="Q68" t="n">
         <v>0</v>
       </c>
+      <c r="R68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4547,6 +4754,9 @@
       <c r="Q69" t="n">
         <v>0</v>
       </c>
+      <c r="R69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4601,10 +4811,13 @@
         <v>0</v>
       </c>
       <c r="P70" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Q70" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="R70" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="71">
@@ -4660,9 +4873,12 @@
         <v>0</v>
       </c>
       <c r="P71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q71" t="n">
+        <v>1</v>
+      </c>
+      <c r="R71" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4724,6 +4940,9 @@
       <c r="Q72" t="n">
         <v>0</v>
       </c>
+      <c r="R72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4778,10 +4997,13 @@
         <v>0</v>
       </c>
       <c r="P73" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q73" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="R73" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="74">
@@ -4837,10 +5059,13 @@
         <v>0</v>
       </c>
       <c r="P74" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="Q74" t="n">
-        <v>6</v>
+        <v>19</v>
+      </c>
+      <c r="R74" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="75">
@@ -4896,11 +5121,14 @@
         <v>0</v>
       </c>
       <c r="P75" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q75" t="n">
         <v>2</v>
       </c>
+      <c r="R75" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4955,10 +5183,13 @@
         <v>0</v>
       </c>
       <c r="P76" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q76" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R76" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="77">
@@ -5019,6 +5250,9 @@
       <c r="Q77" t="n">
         <v>0</v>
       </c>
+      <c r="R77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5078,6 +5312,9 @@
       <c r="Q78" t="n">
         <v>0</v>
       </c>
+      <c r="R78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5132,10 +5369,13 @@
         <v>0</v>
       </c>
       <c r="P79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q79" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="R79" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="80">
@@ -5191,11 +5431,14 @@
         <v>0</v>
       </c>
       <c r="P80" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q80" t="n">
         <v>6</v>
       </c>
+      <c r="R80" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5250,10 +5493,13 @@
         <v>0</v>
       </c>
       <c r="P81" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q81" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R81" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="82">
@@ -5309,10 +5555,13 @@
         <v>0</v>
       </c>
       <c r="P82" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q82" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R82" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="83">
@@ -5368,10 +5617,13 @@
         <v>0</v>
       </c>
       <c r="P83" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q83" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="R83" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="84">
@@ -5427,9 +5679,12 @@
         <v>0</v>
       </c>
       <c r="P84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q84" t="n">
+        <v>1</v>
+      </c>
+      <c r="R84" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5491,6 +5746,9 @@
       <c r="Q85" t="n">
         <v>0</v>
       </c>
+      <c r="R85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5545,10 +5803,13 @@
         <v>0</v>
       </c>
       <c r="P86" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q86" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="R86" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="87">
@@ -5609,6 +5870,9 @@
       <c r="Q87" t="n">
         <v>0</v>
       </c>
+      <c r="R87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5663,10 +5927,13 @@
         <v>0</v>
       </c>
       <c r="P88" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q88" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="R88" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="89">
@@ -5727,6 +5994,9 @@
       <c r="Q89" t="n">
         <v>0</v>
       </c>
+      <c r="R89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5781,10 +6051,13 @@
         <v>0</v>
       </c>
       <c r="P90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q90" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="R90" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="91">
@@ -5845,6 +6118,9 @@
       <c r="Q91" t="n">
         <v>0</v>
       </c>
+      <c r="R91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5904,6 +6180,9 @@
       <c r="Q92" t="n">
         <v>0</v>
       </c>
+      <c r="R92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5958,10 +6237,13 @@
         <v>0</v>
       </c>
       <c r="P93" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q93" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="R93" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="94">
@@ -6017,11 +6299,14 @@
         <v>0</v>
       </c>
       <c r="P94" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q94" t="n">
         <v>5</v>
       </c>
+      <c r="R94" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6076,9 +6361,12 @@
         <v>0</v>
       </c>
       <c r="P95" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q95" t="n">
         <v>34</v>
       </c>
-      <c r="Q95" t="n">
+      <c r="R95" t="n">
         <v>5</v>
       </c>
     </row>
@@ -6135,10 +6423,13 @@
         <v>0</v>
       </c>
       <c r="P96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q96" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="R96" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="97">
@@ -6199,6 +6490,9 @@
       <c r="Q97" t="n">
         <v>0</v>
       </c>
+      <c r="R97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6253,10 +6547,13 @@
         <v>0</v>
       </c>
       <c r="P98" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q98" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="R98" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="99">
@@ -6312,10 +6609,13 @@
         <v>0</v>
       </c>
       <c r="P99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q99" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="R99" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="100">
@@ -6371,10 +6671,13 @@
         <v>0</v>
       </c>
       <c r="P100" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q100" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="R100" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="101">
@@ -6430,10 +6733,13 @@
         <v>0</v>
       </c>
       <c r="P101" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q101" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R101" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="102">
@@ -6494,6 +6800,9 @@
       <c r="Q102" t="n">
         <v>0</v>
       </c>
+      <c r="R102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -6548,10 +6857,13 @@
         <v>0</v>
       </c>
       <c r="P103" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Q103" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="R103" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="104">
@@ -6607,9 +6919,12 @@
         <v>0</v>
       </c>
       <c r="P104" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q104" t="n">
         <v>12</v>
       </c>
-      <c r="Q104" t="n">
+      <c r="R104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6666,10 +6981,13 @@
         <v>0</v>
       </c>
       <c r="P105" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q105" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="R105" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="106">
@@ -6725,10 +7043,13 @@
         <v>0</v>
       </c>
       <c r="P106" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q106" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R106" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="107">
@@ -6789,6 +7110,9 @@
       <c r="Q107" t="n">
         <v>0</v>
       </c>
+      <c r="R107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6843,10 +7167,13 @@
         <v>0</v>
       </c>
       <c r="P108" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q108" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R108" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="109">
@@ -6905,6 +7232,9 @@
         <v>0</v>
       </c>
       <c r="Q109" t="n">
+        <v>0</v>
+      </c>
+      <c r="R109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1356)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R109"/>
+  <dimension ref="A1:S109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -446,8 +446,9 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -531,12 +532,17 @@
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -598,11 +604,14 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
         <v>7</v>
       </c>
+      <c r="S2" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -660,11 +669,14 @@
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
         <v>6</v>
       </c>
+      <c r="S3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -722,10 +734,13 @@
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S4" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -784,10 +799,13 @@
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R5" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S5" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -846,10 +864,13 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R6" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S6" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -908,10 +929,13 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R7" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S7" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -970,10 +994,13 @@
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R8" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S8" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -1032,10 +1059,13 @@
         <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R9" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="S9" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -1094,10 +1124,13 @@
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R10" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S10" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -1156,10 +1189,13 @@
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R11" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S11" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1218,10 +1254,13 @@
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R12" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="S12" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -1280,11 +1319,14 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
+      <c r="S13" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1342,10 +1384,13 @@
         <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R14" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S14" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="15">
@@ -1404,10 +1449,13 @@
         <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R15" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="S15" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="16">
@@ -1466,10 +1514,13 @@
         <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R16" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="S16" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -1528,10 +1579,13 @@
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R17" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S17" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="18">
@@ -1590,10 +1644,13 @@
         <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R18" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="S18" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="19">
@@ -1652,10 +1709,13 @@
         <v>1</v>
       </c>
       <c r="Q19" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R19" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S19" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -1714,10 +1774,13 @@
         <v>1</v>
       </c>
       <c r="Q20" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R20" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S20" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="21">
@@ -1781,6 +1844,9 @@
       <c r="R21" t="n">
         <v>0</v>
       </c>
+      <c r="S21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1843,6 +1909,9 @@
       <c r="R22" t="n">
         <v>0</v>
       </c>
+      <c r="S22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1900,10 +1969,13 @@
         <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R23" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="S23" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="24">
@@ -1962,10 +2034,13 @@
         <v>1</v>
       </c>
       <c r="Q24" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R24" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S24" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="25">
@@ -2024,10 +2099,13 @@
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R25" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="S25" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -2086,10 +2164,13 @@
         <v>1</v>
       </c>
       <c r="Q26" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R26" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="S26" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -2148,10 +2229,13 @@
         <v>1</v>
       </c>
       <c r="Q27" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R27" t="n">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="S27" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -2215,6 +2299,9 @@
       <c r="R28" t="n">
         <v>0</v>
       </c>
+      <c r="S28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2277,6 +2364,9 @@
       <c r="R29" t="n">
         <v>0</v>
       </c>
+      <c r="S29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2337,7 +2427,10 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="S30" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -2396,10 +2489,13 @@
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R31" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S31" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="32">
@@ -2458,10 +2554,13 @@
         <v>1</v>
       </c>
       <c r="Q32" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R32" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S32" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="33">
@@ -2520,10 +2619,13 @@
         <v>0</v>
       </c>
       <c r="Q33" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R33" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S33" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="34">
@@ -2582,11 +2684,14 @@
         <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="R34" t="n">
         <v>8</v>
       </c>
+      <c r="S34" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2644,11 +2749,14 @@
         <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R35" t="n">
         <v>5</v>
       </c>
+      <c r="S35" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2706,10 +2814,13 @@
         <v>1</v>
       </c>
       <c r="Q36" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R36" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S36" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="37">
@@ -2768,11 +2879,14 @@
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R37" t="n">
         <v>3</v>
       </c>
+      <c r="S37" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2835,6 +2949,9 @@
       <c r="R38" t="n">
         <v>0</v>
       </c>
+      <c r="S38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2895,7 +3012,10 @@
         <v>1</v>
       </c>
       <c r="R39" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="S39" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="40">
@@ -2954,10 +3074,13 @@
         <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R40" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S40" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="41">
@@ -3016,10 +3139,13 @@
         <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R41" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S41" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="42">
@@ -3078,10 +3204,13 @@
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R42" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="S42" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="43">
@@ -3140,9 +3269,12 @@
         <v>0</v>
       </c>
       <c r="Q43" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" t="n">
         <v>21</v>
       </c>
-      <c r="R43" t="n">
+      <c r="S43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3202,10 +3334,13 @@
         <v>0</v>
       </c>
       <c r="Q44" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="R44" t="n">
-        <v>4</v>
+        <v>46</v>
+      </c>
+      <c r="S44" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="45">
@@ -3264,10 +3399,13 @@
         <v>1</v>
       </c>
       <c r="Q45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R45" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="S45" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="46">
@@ -3326,10 +3464,13 @@
         <v>1</v>
       </c>
       <c r="Q46" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R46" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="S46" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="47">
@@ -3388,10 +3529,13 @@
         <v>0</v>
       </c>
       <c r="Q47" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R47" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="S47" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="48">
@@ -3455,6 +3599,9 @@
       <c r="R48" t="n">
         <v>0</v>
       </c>
+      <c r="S48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3512,10 +3659,13 @@
         <v>1</v>
       </c>
       <c r="Q49" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R49" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S49" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="50">
@@ -3574,10 +3724,13 @@
         <v>1</v>
       </c>
       <c r="Q50" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R50" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S50" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="51">
@@ -3636,11 +3789,14 @@
         <v>0</v>
       </c>
       <c r="Q51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R51" t="n">
         <v>2</v>
       </c>
+      <c r="S51" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3698,10 +3854,13 @@
         <v>0</v>
       </c>
       <c r="Q52" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R52" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="S52" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="53">
@@ -3760,10 +3919,13 @@
         <v>1</v>
       </c>
       <c r="Q53" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R53" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S53" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="54">
@@ -3827,6 +3989,9 @@
       <c r="R54" t="n">
         <v>0</v>
       </c>
+      <c r="S54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3884,10 +4049,13 @@
         <v>1</v>
       </c>
       <c r="Q55" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R55" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S55" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="56">
@@ -3951,6 +4119,9 @@
       <c r="R56" t="n">
         <v>0</v>
       </c>
+      <c r="S56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4008,10 +4179,13 @@
         <v>1</v>
       </c>
       <c r="Q57" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R57" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S57" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="58">
@@ -4070,10 +4244,13 @@
         <v>1</v>
       </c>
       <c r="Q58" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R58" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S58" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="59">
@@ -4132,10 +4309,13 @@
         <v>0</v>
       </c>
       <c r="Q59" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R59" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="S59" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="60">
@@ -4194,10 +4374,13 @@
         <v>1</v>
       </c>
       <c r="Q60" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R60" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="S60" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="61">
@@ -4256,10 +4439,13 @@
         <v>1</v>
       </c>
       <c r="Q61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R61" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="S61" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="62">
@@ -4323,6 +4509,9 @@
       <c r="R62" t="n">
         <v>0</v>
       </c>
+      <c r="S62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4380,10 +4569,13 @@
         <v>1</v>
       </c>
       <c r="Q63" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R63" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="S63" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="64">
@@ -4442,10 +4634,13 @@
         <v>1</v>
       </c>
       <c r="Q64" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R64" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S64" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="65">
@@ -4509,6 +4704,9 @@
       <c r="R65" t="n">
         <v>0</v>
       </c>
+      <c r="S65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4571,6 +4769,9 @@
       <c r="R66" t="n">
         <v>0</v>
       </c>
+      <c r="S66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4628,11 +4829,14 @@
         <v>1</v>
       </c>
       <c r="Q67" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R67" t="n">
         <v>4</v>
       </c>
+      <c r="S67" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4695,6 +4899,9 @@
       <c r="R68" t="n">
         <v>0</v>
       </c>
+      <c r="S68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4757,6 +4964,9 @@
       <c r="R69" t="n">
         <v>0</v>
       </c>
+      <c r="S69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4814,10 +5024,13 @@
         <v>1</v>
       </c>
       <c r="Q70" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R70" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="S70" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="71">
@@ -4876,9 +5089,12 @@
         <v>0</v>
       </c>
       <c r="Q71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S71" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4943,6 +5159,9 @@
       <c r="R72" t="n">
         <v>0</v>
       </c>
+      <c r="S72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5000,10 +5219,13 @@
         <v>1</v>
       </c>
       <c r="Q73" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R73" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="S73" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="74">
@@ -5062,9 +5284,12 @@
         <v>1</v>
       </c>
       <c r="Q74" t="n">
+        <v>0</v>
+      </c>
+      <c r="R74" t="n">
         <v>19</v>
       </c>
-      <c r="R74" t="n">
+      <c r="S74" t="n">
         <v>7</v>
       </c>
     </row>
@@ -5124,10 +5349,13 @@
         <v>0</v>
       </c>
       <c r="Q75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R75" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="S75" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="76">
@@ -5186,10 +5414,13 @@
         <v>1</v>
       </c>
       <c r="Q76" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R76" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S76" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="77">
@@ -5253,6 +5484,9 @@
       <c r="R77" t="n">
         <v>0</v>
       </c>
+      <c r="S77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5315,6 +5549,9 @@
       <c r="R78" t="n">
         <v>0</v>
       </c>
+      <c r="S78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5372,10 +5609,13 @@
         <v>1</v>
       </c>
       <c r="Q79" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R79" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="S79" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="80">
@@ -5434,10 +5674,13 @@
         <v>0</v>
       </c>
       <c r="Q80" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R80" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="S80" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="81">
@@ -5496,10 +5739,13 @@
         <v>1</v>
       </c>
       <c r="Q81" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R81" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S81" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="82">
@@ -5558,10 +5804,13 @@
         <v>1</v>
       </c>
       <c r="Q82" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R82" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S82" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="83">
@@ -5620,10 +5869,13 @@
         <v>1</v>
       </c>
       <c r="Q83" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R83" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="S83" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="84">
@@ -5685,7 +5937,10 @@
         <v>1</v>
       </c>
       <c r="R84" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="S84" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="85">
@@ -5749,6 +6004,9 @@
       <c r="R85" t="n">
         <v>0</v>
       </c>
+      <c r="S85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5806,10 +6064,13 @@
         <v>1</v>
       </c>
       <c r="Q86" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R86" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="S86" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="87">
@@ -5873,6 +6134,9 @@
       <c r="R87" t="n">
         <v>0</v>
       </c>
+      <c r="S87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5930,10 +6194,13 @@
         <v>1</v>
       </c>
       <c r="Q88" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R88" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="S88" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="89">
@@ -5997,6 +6264,9 @@
       <c r="R89" t="n">
         <v>0</v>
       </c>
+      <c r="S89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6054,10 +6324,13 @@
         <v>1</v>
       </c>
       <c r="Q90" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R90" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="S90" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="91">
@@ -6121,6 +6394,9 @@
       <c r="R91" t="n">
         <v>0</v>
       </c>
+      <c r="S91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6183,6 +6459,9 @@
       <c r="R92" t="n">
         <v>0</v>
       </c>
+      <c r="S92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6240,10 +6519,13 @@
         <v>1</v>
       </c>
       <c r="Q93" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R93" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="S93" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="94">
@@ -6302,11 +6584,14 @@
         <v>0</v>
       </c>
       <c r="Q94" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R94" t="n">
         <v>5</v>
       </c>
+      <c r="S94" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6364,9 +6649,12 @@
         <v>0</v>
       </c>
       <c r="Q95" t="n">
+        <v>0</v>
+      </c>
+      <c r="R95" t="n">
         <v>34</v>
       </c>
-      <c r="R95" t="n">
+      <c r="S95" t="n">
         <v>5</v>
       </c>
     </row>
@@ -6426,10 +6714,13 @@
         <v>1</v>
       </c>
       <c r="Q96" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R96" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="S96" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="97">
@@ -6493,6 +6784,9 @@
       <c r="R97" t="n">
         <v>0</v>
       </c>
+      <c r="S97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6550,10 +6844,13 @@
         <v>1</v>
       </c>
       <c r="Q98" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R98" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="S98" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="99">
@@ -6612,9 +6909,12 @@
         <v>1</v>
       </c>
       <c r="Q99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R99" t="n">
+        <v>1</v>
+      </c>
+      <c r="S99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6674,11 +6974,14 @@
         <v>1</v>
       </c>
       <c r="Q100" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R100" t="n">
         <v>3</v>
       </c>
+      <c r="S100" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6736,10 +7039,13 @@
         <v>1</v>
       </c>
       <c r="Q101" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R101" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S101" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="102">
@@ -6803,6 +7109,9 @@
       <c r="R102" t="n">
         <v>0</v>
       </c>
+      <c r="S102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -6860,10 +7169,13 @@
         <v>1</v>
       </c>
       <c r="Q103" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R103" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="S103" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="104">
@@ -6922,9 +7234,12 @@
         <v>0</v>
       </c>
       <c r="Q104" t="n">
+        <v>0</v>
+      </c>
+      <c r="R104" t="n">
         <v>12</v>
       </c>
-      <c r="R104" t="n">
+      <c r="S104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6984,10 +7299,13 @@
         <v>1</v>
       </c>
       <c r="Q105" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R105" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="S105" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="106">
@@ -7046,10 +7364,13 @@
         <v>1</v>
       </c>
       <c r="Q106" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R106" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S106" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="107">
@@ -7113,6 +7434,9 @@
       <c r="R107" t="n">
         <v>0</v>
       </c>
+      <c r="S107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7170,10 +7494,13 @@
         <v>1</v>
       </c>
       <c r="Q108" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R108" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="S108" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="109">
@@ -7235,6 +7562,9 @@
         <v>0</v>
       </c>
       <c r="R109" t="n">
+        <v>0</v>
+      </c>
+      <c r="S109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1379)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S109"/>
+  <dimension ref="A1:T109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -447,8 +447,9 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -537,12 +538,17 @@
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -607,11 +613,14 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
         <v>7</v>
       </c>
+      <c r="T2" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -672,11 +681,14 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
         <v>6</v>
       </c>
+      <c r="T3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -737,11 +749,14 @@
         <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
         <v>9</v>
       </c>
+      <c r="T4" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -802,11 +817,14 @@
         <v>1</v>
       </c>
       <c r="R5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
         <v>9</v>
       </c>
+      <c r="T5" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -867,11 +885,14 @@
         <v>1</v>
       </c>
       <c r="R6" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S6" t="n">
         <v>8</v>
       </c>
+      <c r="T6" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -932,11 +953,14 @@
         <v>1</v>
       </c>
       <c r="R7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
         <v>9</v>
       </c>
+      <c r="T7" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -997,11 +1021,14 @@
         <v>1</v>
       </c>
       <c r="R8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
         <v>9</v>
       </c>
+      <c r="T8" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1062,11 +1089,14 @@
         <v>1</v>
       </c>
       <c r="R9" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
         <v>10</v>
       </c>
+      <c r="T9" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1127,11 +1157,14 @@
         <v>1</v>
       </c>
       <c r="R10" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
         <v>9</v>
       </c>
+      <c r="T10" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1192,11 +1225,14 @@
         <v>1</v>
       </c>
       <c r="R11" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
         <v>8</v>
       </c>
+      <c r="T11" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1257,11 +1293,14 @@
         <v>1</v>
       </c>
       <c r="R12" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S12" t="n">
         <v>10</v>
       </c>
+      <c r="T12" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1322,11 +1361,14 @@
         <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
         <v>5</v>
       </c>
+      <c r="T13" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1387,11 +1429,14 @@
         <v>1</v>
       </c>
       <c r="R14" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S14" t="n">
         <v>9</v>
       </c>
+      <c r="T14" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1452,11 +1497,14 @@
         <v>1</v>
       </c>
       <c r="R15" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
         <v>7</v>
       </c>
+      <c r="T15" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1517,11 +1565,14 @@
         <v>1</v>
       </c>
       <c r="R16" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
         <v>7</v>
       </c>
+      <c r="T16" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1582,11 +1633,14 @@
         <v>1</v>
       </c>
       <c r="R17" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
         <v>9</v>
       </c>
+      <c r="T17" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1647,11 +1701,14 @@
         <v>1</v>
       </c>
       <c r="R18" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S18" t="n">
         <v>10</v>
       </c>
+      <c r="T18" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1712,11 +1769,14 @@
         <v>1</v>
       </c>
       <c r="R19" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
         <v>8</v>
       </c>
+      <c r="T19" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1777,11 +1837,14 @@
         <v>1</v>
       </c>
       <c r="R20" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
         <v>8</v>
       </c>
+      <c r="T20" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1847,6 +1910,9 @@
       <c r="S21" t="n">
         <v>0</v>
       </c>
+      <c r="T21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1912,6 +1978,9 @@
       <c r="S22" t="n">
         <v>0</v>
       </c>
+      <c r="T22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1972,11 +2041,14 @@
         <v>1</v>
       </c>
       <c r="R23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
         <v>4</v>
       </c>
+      <c r="T23" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2037,11 +2109,14 @@
         <v>1</v>
       </c>
       <c r="R24" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S24" t="n">
         <v>8</v>
       </c>
+      <c r="T24" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2102,11 +2177,14 @@
         <v>1</v>
       </c>
       <c r="R25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S25" t="n">
         <v>6</v>
       </c>
+      <c r="T25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2167,11 +2245,14 @@
         <v>1</v>
       </c>
       <c r="R26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S26" t="n">
         <v>6</v>
       </c>
+      <c r="T26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2232,9 +2313,12 @@
         <v>1</v>
       </c>
       <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
         <v>10</v>
       </c>
-      <c r="S27" t="n">
+      <c r="T27" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2302,6 +2386,9 @@
       <c r="S28" t="n">
         <v>0</v>
       </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2367,6 +2454,9 @@
       <c r="S29" t="n">
         <v>0</v>
       </c>
+      <c r="T29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2427,11 +2517,14 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S30" t="n">
         <v>2</v>
       </c>
+      <c r="T30" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2492,11 +2585,14 @@
         <v>1</v>
       </c>
       <c r="R31" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S31" t="n">
         <v>9</v>
       </c>
+      <c r="T31" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2557,11 +2653,14 @@
         <v>1</v>
       </c>
       <c r="R32" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S32" t="n">
         <v>9</v>
       </c>
+      <c r="T32" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2622,11 +2721,14 @@
         <v>1</v>
       </c>
       <c r="R33" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S33" t="n">
         <v>9</v>
       </c>
+      <c r="T33" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2687,11 +2789,14 @@
         <v>0</v>
       </c>
       <c r="R34" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S34" t="n">
         <v>8</v>
       </c>
+      <c r="T34" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2752,11 +2857,14 @@
         <v>0</v>
       </c>
       <c r="R35" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S35" t="n">
         <v>5</v>
       </c>
+      <c r="T35" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2817,11 +2925,14 @@
         <v>1</v>
       </c>
       <c r="R36" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S36" t="n">
         <v>8</v>
       </c>
+      <c r="T36" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2882,11 +2993,14 @@
         <v>0</v>
       </c>
       <c r="R37" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S37" t="n">
         <v>3</v>
       </c>
+      <c r="T37" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2952,6 +3066,9 @@
       <c r="S38" t="n">
         <v>0</v>
       </c>
+      <c r="T38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3012,11 +3129,14 @@
         <v>1</v>
       </c>
       <c r="R39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S39" t="n">
         <v>2</v>
       </c>
+      <c r="T39" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3077,11 +3197,14 @@
         <v>1</v>
       </c>
       <c r="R40" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S40" t="n">
         <v>9</v>
       </c>
+      <c r="T40" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3142,11 +3265,14 @@
         <v>1</v>
       </c>
       <c r="R41" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S41" t="n">
         <v>9</v>
       </c>
+      <c r="T41" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3207,11 +3333,14 @@
         <v>1</v>
       </c>
       <c r="R42" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S42" t="n">
         <v>10</v>
       </c>
+      <c r="T42" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3272,9 +3401,12 @@
         <v>0</v>
       </c>
       <c r="R43" t="n">
+        <v>0</v>
+      </c>
+      <c r="S43" t="n">
         <v>21</v>
       </c>
-      <c r="S43" t="n">
+      <c r="T43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3337,9 +3469,12 @@
         <v>1</v>
       </c>
       <c r="R44" t="n">
+        <v>0</v>
+      </c>
+      <c r="S44" t="n">
         <v>46</v>
       </c>
-      <c r="S44" t="n">
+      <c r="T44" t="n">
         <v>5</v>
       </c>
     </row>
@@ -3402,11 +3537,14 @@
         <v>1</v>
       </c>
       <c r="R45" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S45" t="n">
         <v>7</v>
       </c>
+      <c r="T45" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3467,11 +3605,14 @@
         <v>1</v>
       </c>
       <c r="R46" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S46" t="n">
         <v>10</v>
       </c>
+      <c r="T46" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3532,11 +3673,14 @@
         <v>1</v>
       </c>
       <c r="R47" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S47" t="n">
         <v>7</v>
       </c>
+      <c r="T47" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3602,6 +3746,9 @@
       <c r="S48" t="n">
         <v>0</v>
       </c>
+      <c r="T48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3662,11 +3809,14 @@
         <v>1</v>
       </c>
       <c r="R49" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S49" t="n">
         <v>9</v>
       </c>
+      <c r="T49" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3727,11 +3877,14 @@
         <v>1</v>
       </c>
       <c r="R50" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S50" t="n">
         <v>8</v>
       </c>
+      <c r="T50" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3792,11 +3945,14 @@
         <v>0</v>
       </c>
       <c r="R51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S51" t="n">
         <v>2</v>
       </c>
+      <c r="T51" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3857,11 +4013,14 @@
         <v>1</v>
       </c>
       <c r="R52" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S52" t="n">
         <v>4</v>
       </c>
+      <c r="T52" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3922,11 +4081,14 @@
         <v>1</v>
       </c>
       <c r="R53" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S53" t="n">
         <v>9</v>
       </c>
+      <c r="T53" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3992,6 +4154,9 @@
       <c r="S54" t="n">
         <v>0</v>
       </c>
+      <c r="T54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4052,11 +4217,14 @@
         <v>1</v>
       </c>
       <c r="R55" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S55" t="n">
         <v>8</v>
       </c>
+      <c r="T55" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4122,6 +4290,9 @@
       <c r="S56" t="n">
         <v>0</v>
       </c>
+      <c r="T56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4182,11 +4353,14 @@
         <v>1</v>
       </c>
       <c r="R57" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S57" t="n">
         <v>8</v>
       </c>
+      <c r="T57" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4247,11 +4421,14 @@
         <v>1</v>
       </c>
       <c r="R58" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S58" t="n">
         <v>8</v>
       </c>
+      <c r="T58" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4312,11 +4489,14 @@
         <v>1</v>
       </c>
       <c r="R59" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S59" t="n">
         <v>4</v>
       </c>
+      <c r="T59" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4377,11 +4557,14 @@
         <v>1</v>
       </c>
       <c r="R60" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S60" t="n">
         <v>10</v>
       </c>
+      <c r="T60" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4442,11 +4625,14 @@
         <v>1</v>
       </c>
       <c r="R61" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S61" t="n">
         <v>3</v>
       </c>
+      <c r="T61" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4512,6 +4698,9 @@
       <c r="S62" t="n">
         <v>0</v>
       </c>
+      <c r="T62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4572,11 +4761,14 @@
         <v>1</v>
       </c>
       <c r="R63" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S63" t="n">
         <v>6</v>
       </c>
+      <c r="T63" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4637,11 +4829,14 @@
         <v>1</v>
       </c>
       <c r="R64" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S64" t="n">
         <v>9</v>
       </c>
+      <c r="T64" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4707,6 +4902,9 @@
       <c r="S65" t="n">
         <v>0</v>
       </c>
+      <c r="T65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4772,6 +4970,9 @@
       <c r="S66" t="n">
         <v>0</v>
       </c>
+      <c r="T66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4832,11 +5033,14 @@
         <v>0</v>
       </c>
       <c r="R67" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S67" t="n">
         <v>4</v>
       </c>
+      <c r="T67" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4902,6 +5106,9 @@
       <c r="S68" t="n">
         <v>0</v>
       </c>
+      <c r="T68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4967,6 +5174,9 @@
       <c r="S69" t="n">
         <v>0</v>
       </c>
+      <c r="T69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5027,11 +5237,14 @@
         <v>1</v>
       </c>
       <c r="R70" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S70" t="n">
         <v>10</v>
       </c>
+      <c r="T70" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5092,9 +5305,12 @@
         <v>0</v>
       </c>
       <c r="R71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S71" t="n">
+        <v>1</v>
+      </c>
+      <c r="T71" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5162,6 +5378,9 @@
       <c r="S72" t="n">
         <v>0</v>
       </c>
+      <c r="T72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5222,11 +5441,14 @@
         <v>1</v>
       </c>
       <c r="R73" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S73" t="n">
         <v>5</v>
       </c>
+      <c r="T73" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5287,9 +5509,12 @@
         <v>0</v>
       </c>
       <c r="R74" t="n">
+        <v>0</v>
+      </c>
+      <c r="S74" t="n">
         <v>19</v>
       </c>
-      <c r="S74" t="n">
+      <c r="T74" t="n">
         <v>7</v>
       </c>
     </row>
@@ -5352,11 +5577,14 @@
         <v>1</v>
       </c>
       <c r="R75" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S75" t="n">
         <v>3</v>
       </c>
+      <c r="T75" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5417,11 +5645,14 @@
         <v>1</v>
       </c>
       <c r="R76" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S76" t="n">
         <v>8</v>
       </c>
+      <c r="T76" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5487,6 +5718,9 @@
       <c r="S77" t="n">
         <v>0</v>
       </c>
+      <c r="T77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5552,6 +5786,9 @@
       <c r="S78" t="n">
         <v>0</v>
       </c>
+      <c r="T78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5612,11 +5849,14 @@
         <v>1</v>
       </c>
       <c r="R79" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S79" t="n">
         <v>5</v>
       </c>
+      <c r="T79" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5677,11 +5917,14 @@
         <v>1</v>
       </c>
       <c r="R80" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S80" t="n">
         <v>7</v>
       </c>
+      <c r="T80" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5742,11 +5985,14 @@
         <v>1</v>
       </c>
       <c r="R81" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S81" t="n">
         <v>8</v>
       </c>
+      <c r="T81" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5807,11 +6053,14 @@
         <v>1</v>
       </c>
       <c r="R82" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S82" t="n">
         <v>9</v>
       </c>
+      <c r="T82" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5872,11 +6121,14 @@
         <v>1</v>
       </c>
       <c r="R83" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S83" t="n">
         <v>6</v>
       </c>
+      <c r="T83" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5937,11 +6189,14 @@
         <v>1</v>
       </c>
       <c r="R84" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S84" t="n">
         <v>2</v>
       </c>
+      <c r="T84" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6007,6 +6262,9 @@
       <c r="S85" t="n">
         <v>0</v>
       </c>
+      <c r="T85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6067,11 +6325,14 @@
         <v>1</v>
       </c>
       <c r="R86" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S86" t="n">
         <v>6</v>
       </c>
+      <c r="T86" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6137,6 +6398,9 @@
       <c r="S87" t="n">
         <v>0</v>
       </c>
+      <c r="T87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6197,11 +6461,14 @@
         <v>1</v>
       </c>
       <c r="R88" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S88" t="n">
         <v>5</v>
       </c>
+      <c r="T88" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6267,6 +6534,9 @@
       <c r="S89" t="n">
         <v>0</v>
       </c>
+      <c r="T89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6327,11 +6597,14 @@
         <v>1</v>
       </c>
       <c r="R90" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S90" t="n">
         <v>4</v>
       </c>
+      <c r="T90" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6397,6 +6670,9 @@
       <c r="S91" t="n">
         <v>0</v>
       </c>
+      <c r="T91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6462,6 +6738,9 @@
       <c r="S92" t="n">
         <v>0</v>
       </c>
+      <c r="T92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6522,11 +6801,14 @@
         <v>1</v>
       </c>
       <c r="R93" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S93" t="n">
         <v>6</v>
       </c>
+      <c r="T93" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6587,11 +6869,14 @@
         <v>0</v>
       </c>
       <c r="R94" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S94" t="n">
         <v>5</v>
       </c>
+      <c r="T94" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6652,9 +6937,12 @@
         <v>0</v>
       </c>
       <c r="R95" t="n">
+        <v>0</v>
+      </c>
+      <c r="S95" t="n">
         <v>34</v>
       </c>
-      <c r="S95" t="n">
+      <c r="T95" t="n">
         <v>5</v>
       </c>
     </row>
@@ -6717,11 +7005,14 @@
         <v>1</v>
       </c>
       <c r="R96" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S96" t="n">
         <v>4</v>
       </c>
+      <c r="T96" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6787,6 +7078,9 @@
       <c r="S97" t="n">
         <v>0</v>
       </c>
+      <c r="T97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6847,11 +7141,14 @@
         <v>1</v>
       </c>
       <c r="R98" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S98" t="n">
         <v>5</v>
       </c>
+      <c r="T98" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6912,9 +7209,12 @@
         <v>0</v>
       </c>
       <c r="R99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S99" t="n">
+        <v>1</v>
+      </c>
+      <c r="T99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6977,11 +7277,14 @@
         <v>0</v>
       </c>
       <c r="R100" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S100" t="n">
         <v>3</v>
       </c>
+      <c r="T100" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7042,11 +7345,14 @@
         <v>1</v>
       </c>
       <c r="R101" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S101" t="n">
         <v>9</v>
       </c>
+      <c r="T101" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7112,6 +7418,9 @@
       <c r="S102" t="n">
         <v>0</v>
       </c>
+      <c r="T102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7172,11 +7481,14 @@
         <v>1</v>
       </c>
       <c r="R103" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S103" t="n">
         <v>10</v>
       </c>
+      <c r="T103" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7237,9 +7549,12 @@
         <v>0</v>
       </c>
       <c r="R104" t="n">
+        <v>0</v>
+      </c>
+      <c r="S104" t="n">
         <v>12</v>
       </c>
-      <c r="S104" t="n">
+      <c r="T104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7302,11 +7617,14 @@
         <v>1</v>
       </c>
       <c r="R105" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="S105" t="n">
         <v>9</v>
       </c>
+      <c r="T105" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7367,11 +7685,14 @@
         <v>1</v>
       </c>
       <c r="R106" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S106" t="n">
         <v>8</v>
       </c>
+      <c r="T106" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7437,6 +7758,9 @@
       <c r="S107" t="n">
         <v>0</v>
       </c>
+      <c r="T107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7497,11 +7821,14 @@
         <v>1</v>
       </c>
       <c r="R108" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S108" t="n">
         <v>8</v>
       </c>
+      <c r="T108" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7565,6 +7892,9 @@
         <v>0</v>
       </c>
       <c r="S109" t="n">
+        <v>0</v>
+      </c>
+      <c r="T109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1387)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T109"/>
+  <dimension ref="A1:U109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -448,8 +448,9 @@
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -543,12 +544,17 @@
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -616,11 +622,14 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="T2" t="n">
         <v>7</v>
       </c>
+      <c r="U2" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -684,11 +693,14 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
         <v>6</v>
       </c>
+      <c r="U3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -752,11 +764,14 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T4" t="n">
         <v>9</v>
       </c>
+      <c r="U4" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -820,11 +835,14 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T5" t="n">
         <v>9</v>
       </c>
+      <c r="U5" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -888,11 +906,14 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T6" t="n">
         <v>8</v>
       </c>
+      <c r="U6" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -956,11 +977,14 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T7" t="n">
         <v>9</v>
       </c>
+      <c r="U7" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1024,11 +1048,14 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T8" t="n">
         <v>9</v>
       </c>
+      <c r="U8" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1092,11 +1119,14 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T9" t="n">
         <v>10</v>
       </c>
+      <c r="U9" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1160,11 +1190,14 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
         <v>9</v>
       </c>
+      <c r="U10" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1228,11 +1261,14 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T11" t="n">
         <v>8</v>
       </c>
+      <c r="U11" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1296,11 +1332,14 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T12" t="n">
         <v>10</v>
       </c>
+      <c r="U12" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1364,11 +1403,14 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T13" t="n">
         <v>5</v>
       </c>
+      <c r="U13" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1432,11 +1474,14 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T14" t="n">
         <v>9</v>
       </c>
+      <c r="U14" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1500,11 +1545,14 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="T15" t="n">
         <v>7</v>
       </c>
+      <c r="U15" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1568,11 +1616,14 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="T16" t="n">
         <v>7</v>
       </c>
+      <c r="U16" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1636,11 +1687,14 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T17" t="n">
         <v>9</v>
       </c>
+      <c r="U17" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1704,11 +1758,14 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T18" t="n">
         <v>10</v>
       </c>
+      <c r="U18" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1772,11 +1829,14 @@
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T19" t="n">
         <v>8</v>
       </c>
+      <c r="U19" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1840,11 +1900,14 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T20" t="n">
         <v>8</v>
       </c>
+      <c r="U20" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1913,6 +1976,9 @@
       <c r="T21" t="n">
         <v>0</v>
       </c>
+      <c r="U21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1981,6 +2047,9 @@
       <c r="T22" t="n">
         <v>0</v>
       </c>
+      <c r="U22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2044,11 +2113,14 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T23" t="n">
         <v>4</v>
       </c>
+      <c r="U23" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2112,11 +2184,14 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T24" t="n">
         <v>8</v>
       </c>
+      <c r="U24" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2180,11 +2255,14 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T25" t="n">
         <v>6</v>
       </c>
+      <c r="U25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2248,11 +2326,14 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T26" t="n">
         <v>6</v>
       </c>
+      <c r="U26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2316,9 +2397,12 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" t="n">
         <v>10</v>
       </c>
-      <c r="T27" t="n">
+      <c r="U27" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2389,6 +2473,9 @@
       <c r="T28" t="n">
         <v>0</v>
       </c>
+      <c r="U28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2457,6 +2544,9 @@
       <c r="T29" t="n">
         <v>0</v>
       </c>
+      <c r="U29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2520,11 +2610,14 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T30" t="n">
         <v>2</v>
       </c>
+      <c r="U30" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2588,11 +2681,14 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T31" t="n">
         <v>9</v>
       </c>
+      <c r="U31" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2656,11 +2752,14 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T32" t="n">
         <v>9</v>
       </c>
+      <c r="U32" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2724,11 +2823,14 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T33" t="n">
         <v>9</v>
       </c>
+      <c r="U33" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2792,11 +2894,14 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T34" t="n">
         <v>8</v>
       </c>
+      <c r="U34" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2860,11 +2965,14 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T35" t="n">
         <v>5</v>
       </c>
+      <c r="U35" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2928,11 +3036,14 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T36" t="n">
         <v>8</v>
       </c>
+      <c r="U36" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2996,11 +3107,14 @@
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T37" t="n">
         <v>3</v>
       </c>
+      <c r="U37" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3069,6 +3183,9 @@
       <c r="T38" t="n">
         <v>0</v>
       </c>
+      <c r="U38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3132,11 +3249,14 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T39" t="n">
         <v>2</v>
       </c>
+      <c r="U39" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3200,11 +3320,14 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T40" t="n">
         <v>9</v>
       </c>
+      <c r="U40" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3268,11 +3391,14 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T41" t="n">
         <v>9</v>
       </c>
+      <c r="U41" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3336,11 +3462,14 @@
         <v>0</v>
       </c>
       <c r="S42" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T42" t="n">
         <v>10</v>
       </c>
+      <c r="U42" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3404,9 +3533,12 @@
         <v>0</v>
       </c>
       <c r="S43" t="n">
+        <v>0</v>
+      </c>
+      <c r="T43" t="n">
         <v>21</v>
       </c>
-      <c r="T43" t="n">
+      <c r="U43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3472,9 +3604,12 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
+        <v>0</v>
+      </c>
+      <c r="T44" t="n">
         <v>46</v>
       </c>
-      <c r="T44" t="n">
+      <c r="U44" t="n">
         <v>5</v>
       </c>
     </row>
@@ -3540,11 +3675,14 @@
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="T45" t="n">
         <v>7</v>
       </c>
+      <c r="U45" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3608,11 +3746,14 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T46" t="n">
         <v>10</v>
       </c>
+      <c r="U46" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3676,11 +3817,14 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="T47" t="n">
         <v>7</v>
       </c>
+      <c r="U47" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3749,6 +3893,9 @@
       <c r="T48" t="n">
         <v>0</v>
       </c>
+      <c r="U48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3812,11 +3959,14 @@
         <v>0</v>
       </c>
       <c r="S49" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T49" t="n">
         <v>9</v>
       </c>
+      <c r="U49" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3880,11 +4030,14 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T50" t="n">
         <v>8</v>
       </c>
+      <c r="U50" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3948,11 +4101,14 @@
         <v>0</v>
       </c>
       <c r="S51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T51" t="n">
         <v>2</v>
       </c>
+      <c r="U51" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4016,11 +4172,14 @@
         <v>0</v>
       </c>
       <c r="S52" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T52" t="n">
         <v>4</v>
       </c>
+      <c r="U52" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4084,11 +4243,14 @@
         <v>0</v>
       </c>
       <c r="S53" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T53" t="n">
         <v>9</v>
       </c>
+      <c r="U53" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4157,6 +4319,9 @@
       <c r="T54" t="n">
         <v>0</v>
       </c>
+      <c r="U54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4220,11 +4385,14 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T55" t="n">
         <v>8</v>
       </c>
+      <c r="U55" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4293,6 +4461,9 @@
       <c r="T56" t="n">
         <v>0</v>
       </c>
+      <c r="U56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4356,11 +4527,14 @@
         <v>0</v>
       </c>
       <c r="S57" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T57" t="n">
         <v>8</v>
       </c>
+      <c r="U57" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4424,11 +4598,14 @@
         <v>0</v>
       </c>
       <c r="S58" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T58" t="n">
         <v>8</v>
       </c>
+      <c r="U58" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4492,11 +4669,14 @@
         <v>0</v>
       </c>
       <c r="S59" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T59" t="n">
         <v>4</v>
       </c>
+      <c r="U59" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4560,11 +4740,14 @@
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T60" t="n">
         <v>10</v>
       </c>
+      <c r="U60" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4628,11 +4811,14 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T61" t="n">
         <v>3</v>
       </c>
+      <c r="U61" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4701,6 +4887,9 @@
       <c r="T62" t="n">
         <v>0</v>
       </c>
+      <c r="U62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4764,11 +4953,14 @@
         <v>0</v>
       </c>
       <c r="S63" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T63" t="n">
         <v>6</v>
       </c>
+      <c r="U63" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4832,11 +5024,14 @@
         <v>0</v>
       </c>
       <c r="S64" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T64" t="n">
         <v>9</v>
       </c>
+      <c r="U64" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4905,6 +5100,9 @@
       <c r="T65" t="n">
         <v>0</v>
       </c>
+      <c r="U65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4973,6 +5171,9 @@
       <c r="T66" t="n">
         <v>0</v>
       </c>
+      <c r="U66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5036,11 +5237,14 @@
         <v>0</v>
       </c>
       <c r="S67" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T67" t="n">
         <v>4</v>
       </c>
+      <c r="U67" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5109,6 +5313,9 @@
       <c r="T68" t="n">
         <v>0</v>
       </c>
+      <c r="U68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5177,6 +5384,9 @@
       <c r="T69" t="n">
         <v>0</v>
       </c>
+      <c r="U69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5240,11 +5450,14 @@
         <v>0</v>
       </c>
       <c r="S70" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T70" t="n">
         <v>10</v>
       </c>
+      <c r="U70" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5308,9 +5521,12 @@
         <v>0</v>
       </c>
       <c r="S71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T71" t="n">
+        <v>1</v>
+      </c>
+      <c r="U71" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5381,6 +5597,9 @@
       <c r="T72" t="n">
         <v>0</v>
       </c>
+      <c r="U72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5444,11 +5663,14 @@
         <v>0</v>
       </c>
       <c r="S73" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T73" t="n">
         <v>5</v>
       </c>
+      <c r="U73" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5512,9 +5734,12 @@
         <v>0</v>
       </c>
       <c r="S74" t="n">
+        <v>0</v>
+      </c>
+      <c r="T74" t="n">
         <v>19</v>
       </c>
-      <c r="T74" t="n">
+      <c r="U74" t="n">
         <v>7</v>
       </c>
     </row>
@@ -5580,11 +5805,14 @@
         <v>0</v>
       </c>
       <c r="S75" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T75" t="n">
         <v>3</v>
       </c>
+      <c r="U75" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5648,11 +5876,14 @@
         <v>0</v>
       </c>
       <c r="S76" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T76" t="n">
         <v>8</v>
       </c>
+      <c r="U76" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5721,6 +5952,9 @@
       <c r="T77" t="n">
         <v>0</v>
       </c>
+      <c r="U77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5789,6 +6023,9 @@
       <c r="T78" t="n">
         <v>0</v>
       </c>
+      <c r="U78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5852,11 +6089,14 @@
         <v>0</v>
       </c>
       <c r="S79" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T79" t="n">
         <v>5</v>
       </c>
+      <c r="U79" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5920,11 +6160,14 @@
         <v>0</v>
       </c>
       <c r="S80" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="T80" t="n">
         <v>7</v>
       </c>
+      <c r="U80" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5988,11 +6231,14 @@
         <v>0</v>
       </c>
       <c r="S81" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T81" t="n">
         <v>8</v>
       </c>
+      <c r="U81" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6056,11 +6302,14 @@
         <v>0</v>
       </c>
       <c r="S82" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T82" t="n">
         <v>9</v>
       </c>
+      <c r="U82" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6124,11 +6373,14 @@
         <v>0</v>
       </c>
       <c r="S83" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T83" t="n">
         <v>6</v>
       </c>
+      <c r="U83" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6192,11 +6444,14 @@
         <v>0</v>
       </c>
       <c r="S84" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T84" t="n">
         <v>2</v>
       </c>
+      <c r="U84" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6265,6 +6520,9 @@
       <c r="T85" t="n">
         <v>0</v>
       </c>
+      <c r="U85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6328,11 +6586,14 @@
         <v>0</v>
       </c>
       <c r="S86" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T86" t="n">
         <v>6</v>
       </c>
+      <c r="U86" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6401,6 +6662,9 @@
       <c r="T87" t="n">
         <v>0</v>
       </c>
+      <c r="U87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6464,11 +6728,14 @@
         <v>0</v>
       </c>
       <c r="S88" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T88" t="n">
         <v>5</v>
       </c>
+      <c r="U88" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6537,6 +6804,9 @@
       <c r="T89" t="n">
         <v>0</v>
       </c>
+      <c r="U89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6600,11 +6870,14 @@
         <v>0</v>
       </c>
       <c r="S90" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T90" t="n">
         <v>4</v>
       </c>
+      <c r="U90" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6673,6 +6946,9 @@
       <c r="T91" t="n">
         <v>0</v>
       </c>
+      <c r="U91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6741,6 +7017,9 @@
       <c r="T92" t="n">
         <v>0</v>
       </c>
+      <c r="U92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6804,11 +7083,14 @@
         <v>0</v>
       </c>
       <c r="S93" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T93" t="n">
         <v>6</v>
       </c>
+      <c r="U93" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6872,11 +7154,14 @@
         <v>0</v>
       </c>
       <c r="S94" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T94" t="n">
         <v>5</v>
       </c>
+      <c r="U94" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6940,9 +7225,12 @@
         <v>0</v>
       </c>
       <c r="S95" t="n">
+        <v>0</v>
+      </c>
+      <c r="T95" t="n">
         <v>34</v>
       </c>
-      <c r="T95" t="n">
+      <c r="U95" t="n">
         <v>5</v>
       </c>
     </row>
@@ -7008,11 +7296,14 @@
         <v>0</v>
       </c>
       <c r="S96" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T96" t="n">
         <v>4</v>
       </c>
+      <c r="U96" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7081,6 +7372,9 @@
       <c r="T97" t="n">
         <v>0</v>
       </c>
+      <c r="U97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7144,11 +7438,14 @@
         <v>0</v>
       </c>
       <c r="S98" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T98" t="n">
         <v>5</v>
       </c>
+      <c r="U98" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7212,9 +7509,12 @@
         <v>0</v>
       </c>
       <c r="S99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T99" t="n">
+        <v>1</v>
+      </c>
+      <c r="U99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7280,11 +7580,14 @@
         <v>0</v>
       </c>
       <c r="S100" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T100" t="n">
         <v>3</v>
       </c>
+      <c r="U100" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7348,11 +7651,14 @@
         <v>0</v>
       </c>
       <c r="S101" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T101" t="n">
         <v>9</v>
       </c>
+      <c r="U101" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7421,6 +7727,9 @@
       <c r="T102" t="n">
         <v>0</v>
       </c>
+      <c r="U102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7484,11 +7793,14 @@
         <v>0</v>
       </c>
       <c r="S103" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T103" t="n">
         <v>10</v>
       </c>
+      <c r="U103" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7552,9 +7864,12 @@
         <v>0</v>
       </c>
       <c r="S104" t="n">
+        <v>0</v>
+      </c>
+      <c r="T104" t="n">
         <v>12</v>
       </c>
-      <c r="T104" t="n">
+      <c r="U104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7620,11 +7935,14 @@
         <v>0</v>
       </c>
       <c r="S105" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T105" t="n">
         <v>9</v>
       </c>
+      <c r="U105" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7688,11 +8006,14 @@
         <v>0</v>
       </c>
       <c r="S106" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T106" t="n">
         <v>8</v>
       </c>
+      <c r="U106" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7761,6 +8082,9 @@
       <c r="T107" t="n">
         <v>0</v>
       </c>
+      <c r="U107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7824,11 +8148,14 @@
         <v>0</v>
       </c>
       <c r="S108" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T108" t="n">
         <v>8</v>
       </c>
+      <c r="U108" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7895,6 +8222,9 @@
         <v>0</v>
       </c>
       <c r="T109" t="n">
+        <v>0</v>
+      </c>
+      <c r="U109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1499)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U109"/>
+  <dimension ref="A1:V109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -449,8 +449,9 @@
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -549,12 +550,17 @@
           <t>2026-03-07</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -625,11 +631,14 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="U2" t="n">
         <v>7</v>
       </c>
+      <c r="V2" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -696,11 +705,14 @@
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U3" t="n">
         <v>6</v>
       </c>
+      <c r="V3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -767,11 +779,14 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
         <v>9</v>
       </c>
+      <c r="V4" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -838,11 +853,14 @@
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U5" t="n">
         <v>9</v>
       </c>
+      <c r="V5" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -909,11 +927,14 @@
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U6" t="n">
         <v>8</v>
       </c>
+      <c r="V6" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -980,11 +1001,14 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U7" t="n">
         <v>9</v>
       </c>
+      <c r="V7" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1051,11 +1075,14 @@
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U8" t="n">
         <v>9</v>
       </c>
+      <c r="V8" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1122,11 +1149,14 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U9" t="n">
         <v>10</v>
       </c>
+      <c r="V9" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1193,11 +1223,14 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
         <v>9</v>
       </c>
+      <c r="V10" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1264,11 +1297,14 @@
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U11" t="n">
         <v>8</v>
       </c>
+      <c r="V11" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1335,11 +1371,14 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U12" t="n">
         <v>10</v>
       </c>
+      <c r="V12" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1406,11 +1445,14 @@
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U13" t="n">
         <v>5</v>
       </c>
+      <c r="V13" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1477,11 +1519,14 @@
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U14" t="n">
         <v>9</v>
       </c>
+      <c r="V14" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1548,11 +1593,14 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="U15" t="n">
         <v>7</v>
       </c>
+      <c r="V15" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1619,11 +1667,14 @@
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="U16" t="n">
         <v>7</v>
       </c>
+      <c r="V16" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1690,11 +1741,14 @@
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U17" t="n">
         <v>9</v>
       </c>
+      <c r="V17" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1761,11 +1815,14 @@
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U18" t="n">
         <v>10</v>
       </c>
+      <c r="V18" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1832,11 +1889,14 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U19" t="n">
         <v>8</v>
       </c>
+      <c r="V19" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1903,11 +1963,14 @@
         <v>0</v>
       </c>
       <c r="T20" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U20" t="n">
         <v>8</v>
       </c>
+      <c r="V20" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1979,6 +2042,9 @@
       <c r="U21" t="n">
         <v>0</v>
       </c>
+      <c r="V21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2050,6 +2116,9 @@
       <c r="U22" t="n">
         <v>0</v>
       </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2116,11 +2185,14 @@
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U23" t="n">
         <v>4</v>
       </c>
+      <c r="V23" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2187,11 +2259,14 @@
         <v>0</v>
       </c>
       <c r="T24" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U24" t="n">
         <v>8</v>
       </c>
+      <c r="V24" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2258,11 +2333,14 @@
         <v>0</v>
       </c>
       <c r="T25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U25" t="n">
         <v>6</v>
       </c>
+      <c r="V25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2329,11 +2407,14 @@
         <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U26" t="n">
         <v>6</v>
       </c>
+      <c r="V26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2400,9 +2481,12 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" t="n">
         <v>10</v>
       </c>
-      <c r="U27" t="n">
+      <c r="V27" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2476,6 +2560,9 @@
       <c r="U28" t="n">
         <v>0</v>
       </c>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2547,6 +2634,9 @@
       <c r="U29" t="n">
         <v>0</v>
       </c>
+      <c r="V29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2613,11 +2703,14 @@
         <v>0</v>
       </c>
       <c r="T30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U30" t="n">
         <v>2</v>
       </c>
+      <c r="V30" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2684,11 +2777,14 @@
         <v>0</v>
       </c>
       <c r="T31" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U31" t="n">
         <v>9</v>
       </c>
+      <c r="V31" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2755,11 +2851,14 @@
         <v>0</v>
       </c>
       <c r="T32" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U32" t="n">
         <v>9</v>
       </c>
+      <c r="V32" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2826,11 +2925,14 @@
         <v>0</v>
       </c>
       <c r="T33" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U33" t="n">
         <v>9</v>
       </c>
+      <c r="V33" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2897,11 +2999,14 @@
         <v>0</v>
       </c>
       <c r="T34" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U34" t="n">
         <v>8</v>
       </c>
+      <c r="V34" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2968,11 +3073,14 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U35" t="n">
         <v>5</v>
       </c>
+      <c r="V35" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3039,11 +3147,14 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U36" t="n">
         <v>8</v>
       </c>
+      <c r="V36" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3110,11 +3221,14 @@
         <v>0</v>
       </c>
       <c r="T37" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="U37" t="n">
         <v>3</v>
       </c>
+      <c r="V37" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3186,6 +3300,9 @@
       <c r="U38" t="n">
         <v>0</v>
       </c>
+      <c r="V38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3252,11 +3369,14 @@
         <v>0</v>
       </c>
       <c r="T39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U39" t="n">
         <v>2</v>
       </c>
+      <c r="V39" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3323,11 +3443,14 @@
         <v>0</v>
       </c>
       <c r="T40" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U40" t="n">
         <v>9</v>
       </c>
+      <c r="V40" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3394,11 +3517,14 @@
         <v>0</v>
       </c>
       <c r="T41" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U41" t="n">
         <v>9</v>
       </c>
+      <c r="V41" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3465,11 +3591,14 @@
         <v>0</v>
       </c>
       <c r="T42" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U42" t="n">
         <v>10</v>
       </c>
+      <c r="V42" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3536,9 +3665,12 @@
         <v>0</v>
       </c>
       <c r="T43" t="n">
+        <v>0</v>
+      </c>
+      <c r="U43" t="n">
         <v>21</v>
       </c>
-      <c r="U43" t="n">
+      <c r="V43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3607,9 +3739,12 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
+        <v>0</v>
+      </c>
+      <c r="U44" t="n">
         <v>46</v>
       </c>
-      <c r="U44" t="n">
+      <c r="V44" t="n">
         <v>5</v>
       </c>
     </row>
@@ -3678,11 +3813,14 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="U45" t="n">
         <v>7</v>
       </c>
+      <c r="V45" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3749,11 +3887,14 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U46" t="n">
         <v>10</v>
       </c>
+      <c r="V46" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3820,11 +3961,14 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="U47" t="n">
         <v>7</v>
       </c>
+      <c r="V47" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3896,6 +4040,9 @@
       <c r="U48" t="n">
         <v>0</v>
       </c>
+      <c r="V48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3962,11 +4109,14 @@
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U49" t="n">
         <v>9</v>
       </c>
+      <c r="V49" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4033,11 +4183,14 @@
         <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U50" t="n">
         <v>8</v>
       </c>
+      <c r="V50" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4104,11 +4257,14 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U51" t="n">
         <v>2</v>
       </c>
+      <c r="V51" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4175,11 +4331,14 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U52" t="n">
         <v>4</v>
       </c>
+      <c r="V52" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4246,11 +4405,14 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U53" t="n">
         <v>9</v>
       </c>
+      <c r="V53" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4322,6 +4484,9 @@
       <c r="U54" t="n">
         <v>0</v>
       </c>
+      <c r="V54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4388,11 +4553,14 @@
         <v>0</v>
       </c>
       <c r="T55" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U55" t="n">
         <v>8</v>
       </c>
+      <c r="V55" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4464,6 +4632,9 @@
       <c r="U56" t="n">
         <v>0</v>
       </c>
+      <c r="V56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4530,11 +4701,14 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U57" t="n">
         <v>8</v>
       </c>
+      <c r="V57" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4601,11 +4775,14 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U58" t="n">
         <v>8</v>
       </c>
+      <c r="V58" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4672,11 +4849,14 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U59" t="n">
         <v>4</v>
       </c>
+      <c r="V59" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4743,11 +4923,14 @@
         <v>0</v>
       </c>
       <c r="T60" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U60" t="n">
         <v>10</v>
       </c>
+      <c r="V60" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4814,11 +4997,14 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="U61" t="n">
         <v>3</v>
       </c>
+      <c r="V61" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4890,6 +5076,9 @@
       <c r="U62" t="n">
         <v>0</v>
       </c>
+      <c r="V62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4956,11 +5145,14 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U63" t="n">
         <v>6</v>
       </c>
+      <c r="V63" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5027,11 +5219,14 @@
         <v>0</v>
       </c>
       <c r="T64" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U64" t="n">
         <v>9</v>
       </c>
+      <c r="V64" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5103,6 +5298,9 @@
       <c r="U65" t="n">
         <v>0</v>
       </c>
+      <c r="V65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5174,6 +5372,9 @@
       <c r="U66" t="n">
         <v>0</v>
       </c>
+      <c r="V66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5240,11 +5441,14 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U67" t="n">
         <v>4</v>
       </c>
+      <c r="V67" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5316,6 +5520,9 @@
       <c r="U68" t="n">
         <v>0</v>
       </c>
+      <c r="V68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5387,6 +5594,9 @@
       <c r="U69" t="n">
         <v>0</v>
       </c>
+      <c r="V69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5453,11 +5663,14 @@
         <v>0</v>
       </c>
       <c r="T70" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U70" t="n">
         <v>10</v>
       </c>
+      <c r="V70" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5524,9 +5737,12 @@
         <v>0</v>
       </c>
       <c r="T71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U71" t="n">
+        <v>1</v>
+      </c>
+      <c r="V71" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5600,6 +5816,9 @@
       <c r="U72" t="n">
         <v>0</v>
       </c>
+      <c r="V72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5666,11 +5885,14 @@
         <v>0</v>
       </c>
       <c r="T73" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U73" t="n">
         <v>5</v>
       </c>
+      <c r="V73" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5737,9 +5959,12 @@
         <v>0</v>
       </c>
       <c r="T74" t="n">
+        <v>0</v>
+      </c>
+      <c r="U74" t="n">
         <v>19</v>
       </c>
-      <c r="U74" t="n">
+      <c r="V74" t="n">
         <v>7</v>
       </c>
     </row>
@@ -5808,11 +6033,14 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="U75" t="n">
         <v>3</v>
       </c>
+      <c r="V75" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5879,11 +6107,14 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U76" t="n">
         <v>8</v>
       </c>
+      <c r="V76" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5955,6 +6186,9 @@
       <c r="U77" t="n">
         <v>0</v>
       </c>
+      <c r="V77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6026,6 +6260,9 @@
       <c r="U78" t="n">
         <v>0</v>
       </c>
+      <c r="V78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6092,11 +6329,14 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U79" t="n">
         <v>5</v>
       </c>
+      <c r="V79" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6163,11 +6403,14 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="U80" t="n">
         <v>7</v>
       </c>
+      <c r="V80" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6234,11 +6477,14 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U81" t="n">
         <v>8</v>
       </c>
+      <c r="V81" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6305,11 +6551,14 @@
         <v>0</v>
       </c>
       <c r="T82" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U82" t="n">
         <v>9</v>
       </c>
+      <c r="V82" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6376,11 +6625,14 @@
         <v>0</v>
       </c>
       <c r="T83" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U83" t="n">
         <v>6</v>
       </c>
+      <c r="V83" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6447,11 +6699,14 @@
         <v>0</v>
       </c>
       <c r="T84" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U84" t="n">
         <v>2</v>
       </c>
+      <c r="V84" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6523,6 +6778,9 @@
       <c r="U85" t="n">
         <v>0</v>
       </c>
+      <c r="V85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6589,11 +6847,14 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U86" t="n">
         <v>6</v>
       </c>
+      <c r="V86" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6665,6 +6926,9 @@
       <c r="U87" t="n">
         <v>0</v>
       </c>
+      <c r="V87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6731,11 +6995,14 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U88" t="n">
         <v>5</v>
       </c>
+      <c r="V88" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6807,6 +7074,9 @@
       <c r="U89" t="n">
         <v>0</v>
       </c>
+      <c r="V89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6873,11 +7143,14 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U90" t="n">
         <v>4</v>
       </c>
+      <c r="V90" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6949,6 +7222,9 @@
       <c r="U91" t="n">
         <v>0</v>
       </c>
+      <c r="V91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7020,6 +7296,9 @@
       <c r="U92" t="n">
         <v>0</v>
       </c>
+      <c r="V92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7086,11 +7365,14 @@
         <v>0</v>
       </c>
       <c r="T93" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U93" t="n">
         <v>6</v>
       </c>
+      <c r="V93" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7157,11 +7439,14 @@
         <v>0</v>
       </c>
       <c r="T94" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U94" t="n">
         <v>5</v>
       </c>
+      <c r="V94" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7228,9 +7513,12 @@
         <v>0</v>
       </c>
       <c r="T95" t="n">
+        <v>0</v>
+      </c>
+      <c r="U95" t="n">
         <v>34</v>
       </c>
-      <c r="U95" t="n">
+      <c r="V95" t="n">
         <v>5</v>
       </c>
     </row>
@@ -7299,11 +7587,14 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U96" t="n">
         <v>4</v>
       </c>
+      <c r="V96" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7375,6 +7666,9 @@
       <c r="U97" t="n">
         <v>0</v>
       </c>
+      <c r="V97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7441,11 +7735,14 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U98" t="n">
         <v>5</v>
       </c>
+      <c r="V98" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7512,9 +7809,12 @@
         <v>0</v>
       </c>
       <c r="T99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U99" t="n">
+        <v>1</v>
+      </c>
+      <c r="V99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7583,11 +7883,14 @@
         <v>0</v>
       </c>
       <c r="T100" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="U100" t="n">
         <v>3</v>
       </c>
+      <c r="V100" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7654,11 +7957,14 @@
         <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U101" t="n">
         <v>9</v>
       </c>
+      <c r="V101" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7730,6 +8036,9 @@
       <c r="U102" t="n">
         <v>0</v>
       </c>
+      <c r="V102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7796,11 +8105,14 @@
         <v>0</v>
       </c>
       <c r="T103" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U103" t="n">
         <v>10</v>
       </c>
+      <c r="V103" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7867,9 +8179,12 @@
         <v>0</v>
       </c>
       <c r="T104" t="n">
+        <v>0</v>
+      </c>
+      <c r="U104" t="n">
         <v>12</v>
       </c>
-      <c r="U104" t="n">
+      <c r="V104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7938,11 +8253,14 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="U105" t="n">
         <v>9</v>
       </c>
+      <c r="V105" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -8009,11 +8327,14 @@
         <v>0</v>
       </c>
       <c r="T106" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U106" t="n">
         <v>8</v>
       </c>
+      <c r="V106" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -8085,6 +8406,9 @@
       <c r="U107" t="n">
         <v>0</v>
       </c>
+      <c r="V107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8151,11 +8475,14 @@
         <v>0</v>
       </c>
       <c r="T108" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U108" t="n">
         <v>8</v>
       </c>
+      <c r="V108" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -8225,6 +8552,9 @@
         <v>0</v>
       </c>
       <c r="U109" t="n">
+        <v>0</v>
+      </c>
+      <c r="V109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1604)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V109"/>
+  <dimension ref="A1:W109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -450,8 +450,9 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
     <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -555,12 +556,17 @@
           <t>2026-03-08</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -634,10 +640,13 @@
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="V2" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="W2" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -708,11 +717,14 @@
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V3" t="n">
         <v>6</v>
       </c>
+      <c r="W3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -782,10 +794,13 @@
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V4" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W4" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -856,10 +871,13 @@
         <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V5" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W5" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -930,10 +948,13 @@
         <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V6" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W6" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -1004,11 +1025,14 @@
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="V7" t="n">
         <v>9</v>
       </c>
+      <c r="W7" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1078,10 +1102,13 @@
         <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V8" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W8" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -1152,10 +1179,13 @@
         <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="V9" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="W9" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -1226,10 +1256,13 @@
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V10" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W10" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -1300,10 +1333,13 @@
         <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W11" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -1374,10 +1410,13 @@
         <v>0</v>
       </c>
       <c r="U12" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="W12" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -1448,10 +1487,13 @@
         <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V13" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="W13" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -1522,10 +1564,13 @@
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V14" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W14" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -1596,10 +1641,13 @@
         <v>0</v>
       </c>
       <c r="U15" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="V15" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="W15" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -1670,10 +1718,13 @@
         <v>0</v>
       </c>
       <c r="U16" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="V16" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="W16" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="17">
@@ -1744,11 +1795,14 @@
         <v>0</v>
       </c>
       <c r="U17" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="V17" t="n">
         <v>9</v>
       </c>
+      <c r="W17" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1818,10 +1872,13 @@
         <v>0</v>
       </c>
       <c r="U18" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="V18" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="W18" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="19">
@@ -1892,10 +1949,13 @@
         <v>0</v>
       </c>
       <c r="U19" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V19" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W19" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="20">
@@ -1966,10 +2026,13 @@
         <v>0</v>
       </c>
       <c r="U20" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V20" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W20" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="21">
@@ -2045,6 +2108,9 @@
       <c r="V21" t="n">
         <v>0</v>
       </c>
+      <c r="W21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2119,6 +2185,9 @@
       <c r="V22" t="n">
         <v>0</v>
       </c>
+      <c r="W22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2188,11 +2257,14 @@
         <v>0</v>
       </c>
       <c r="U23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V23" t="n">
         <v>4</v>
       </c>
+      <c r="W23" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2262,10 +2334,13 @@
         <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V24" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W24" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -2336,11 +2411,14 @@
         <v>0</v>
       </c>
       <c r="U25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V25" t="n">
         <v>6</v>
       </c>
+      <c r="W25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2410,10 +2488,13 @@
         <v>0</v>
       </c>
       <c r="U26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="V26" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="W26" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="27">
@@ -2484,10 +2565,13 @@
         <v>0</v>
       </c>
       <c r="U27" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="V27" t="n">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="W27" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="28">
@@ -2563,6 +2647,9 @@
       <c r="V28" t="n">
         <v>0</v>
       </c>
+      <c r="W28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2637,6 +2724,9 @@
       <c r="V29" t="n">
         <v>0</v>
       </c>
+      <c r="W29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2706,11 +2796,14 @@
         <v>0</v>
       </c>
       <c r="U30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V30" t="n">
         <v>2</v>
       </c>
+      <c r="W30" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2780,11 +2873,14 @@
         <v>0</v>
       </c>
       <c r="U31" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="V31" t="n">
         <v>9</v>
       </c>
+      <c r="W31" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2854,10 +2950,13 @@
         <v>0</v>
       </c>
       <c r="U32" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V32" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W32" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="33">
@@ -2928,11 +3027,14 @@
         <v>0</v>
       </c>
       <c r="U33" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="V33" t="n">
         <v>9</v>
       </c>
+      <c r="W33" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3002,10 +3104,13 @@
         <v>0</v>
       </c>
       <c r="U34" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V34" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W34" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="35">
@@ -3076,10 +3181,13 @@
         <v>0</v>
       </c>
       <c r="U35" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V35" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="W35" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="36">
@@ -3150,10 +3258,13 @@
         <v>0</v>
       </c>
       <c r="U36" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V36" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W36" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="37">
@@ -3224,10 +3335,13 @@
         <v>0</v>
       </c>
       <c r="U37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V37" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="W37" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="38">
@@ -3303,6 +3417,9 @@
       <c r="V38" t="n">
         <v>0</v>
       </c>
+      <c r="W38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3372,11 +3489,14 @@
         <v>0</v>
       </c>
       <c r="U39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V39" t="n">
         <v>2</v>
       </c>
+      <c r="W39" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3446,10 +3566,13 @@
         <v>0</v>
       </c>
       <c r="U40" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V40" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W40" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="41">
@@ -3520,10 +3643,13 @@
         <v>0</v>
       </c>
       <c r="U41" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V41" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W41" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="42">
@@ -3594,10 +3720,13 @@
         <v>0</v>
       </c>
       <c r="U42" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="V42" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="W42" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="43">
@@ -3668,9 +3797,12 @@
         <v>0</v>
       </c>
       <c r="U43" t="n">
+        <v>0</v>
+      </c>
+      <c r="V43" t="n">
         <v>21</v>
       </c>
-      <c r="V43" t="n">
+      <c r="W43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3742,10 +3874,13 @@
         <v>0</v>
       </c>
       <c r="U44" t="n">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="V44" t="n">
-        <v>5</v>
+        <v>47</v>
+      </c>
+      <c r="W44" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="45">
@@ -3816,10 +3951,13 @@
         <v>0</v>
       </c>
       <c r="U45" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="V45" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="W45" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="46">
@@ -3890,10 +4028,13 @@
         <v>0</v>
       </c>
       <c r="U46" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="V46" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="W46" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="47">
@@ -3964,10 +4105,13 @@
         <v>0</v>
       </c>
       <c r="U47" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="V47" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="W47" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="48">
@@ -4043,6 +4187,9 @@
       <c r="V48" t="n">
         <v>0</v>
       </c>
+      <c r="W48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4112,10 +4259,13 @@
         <v>0</v>
       </c>
       <c r="U49" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V49" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W49" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="50">
@@ -4186,10 +4336,13 @@
         <v>0</v>
       </c>
       <c r="U50" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V50" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W50" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="51">
@@ -4260,11 +4413,14 @@
         <v>0</v>
       </c>
       <c r="U51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V51" t="n">
         <v>2</v>
       </c>
+      <c r="W51" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4334,10 +4490,13 @@
         <v>0</v>
       </c>
       <c r="U52" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V52" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="W52" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="53">
@@ -4408,10 +4567,13 @@
         <v>0</v>
       </c>
       <c r="U53" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V53" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W53" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="54">
@@ -4487,6 +4649,9 @@
       <c r="V54" t="n">
         <v>0</v>
       </c>
+      <c r="W54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4556,10 +4721,13 @@
         <v>0</v>
       </c>
       <c r="U55" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V55" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W55" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="56">
@@ -4635,6 +4803,9 @@
       <c r="V56" t="n">
         <v>0</v>
       </c>
+      <c r="W56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4704,10 +4875,13 @@
         <v>0</v>
       </c>
       <c r="U57" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V57" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W57" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="58">
@@ -4778,10 +4952,13 @@
         <v>0</v>
       </c>
       <c r="U58" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V58" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W58" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="59">
@@ -4852,10 +5029,13 @@
         <v>0</v>
       </c>
       <c r="U59" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V59" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="W59" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="60">
@@ -4926,10 +5106,13 @@
         <v>0</v>
       </c>
       <c r="U60" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="V60" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="W60" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="61">
@@ -5000,11 +5183,14 @@
         <v>0</v>
       </c>
       <c r="U61" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V61" t="n">
         <v>3</v>
       </c>
+      <c r="W61" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5079,6 +5265,9 @@
       <c r="V62" t="n">
         <v>0</v>
       </c>
+      <c r="W62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5148,10 +5337,13 @@
         <v>0</v>
       </c>
       <c r="U63" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="V63" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="W63" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="64">
@@ -5222,10 +5414,13 @@
         <v>0</v>
       </c>
       <c r="U64" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V64" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W64" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="65">
@@ -5301,6 +5496,9 @@
       <c r="V65" t="n">
         <v>0</v>
       </c>
+      <c r="W65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5375,6 +5573,9 @@
       <c r="V66" t="n">
         <v>0</v>
       </c>
+      <c r="W66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5444,11 +5645,14 @@
         <v>0</v>
       </c>
       <c r="U67" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V67" t="n">
         <v>4</v>
       </c>
+      <c r="W67" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5523,6 +5727,9 @@
       <c r="V68" t="n">
         <v>0</v>
       </c>
+      <c r="W68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5597,6 +5804,9 @@
       <c r="V69" t="n">
         <v>0</v>
       </c>
+      <c r="W69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5666,10 +5876,13 @@
         <v>0</v>
       </c>
       <c r="U70" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="V70" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="W70" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="71">
@@ -5743,7 +5956,10 @@
         <v>1</v>
       </c>
       <c r="V71" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="W71" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="72">
@@ -5819,6 +6035,9 @@
       <c r="V72" t="n">
         <v>0</v>
       </c>
+      <c r="W72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5888,10 +6107,13 @@
         <v>0</v>
       </c>
       <c r="U73" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V73" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="W73" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="74">
@@ -5962,9 +6184,12 @@
         <v>0</v>
       </c>
       <c r="U74" t="n">
+        <v>0</v>
+      </c>
+      <c r="V74" t="n">
         <v>19</v>
       </c>
-      <c r="V74" t="n">
+      <c r="W74" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6036,10 +6261,13 @@
         <v>0</v>
       </c>
       <c r="U75" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V75" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="W75" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="76">
@@ -6110,10 +6338,13 @@
         <v>0</v>
       </c>
       <c r="U76" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V76" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W76" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="77">
@@ -6189,6 +6420,9 @@
       <c r="V77" t="n">
         <v>0</v>
       </c>
+      <c r="W77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6263,6 +6497,9 @@
       <c r="V78" t="n">
         <v>0</v>
       </c>
+      <c r="W78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6332,11 +6569,14 @@
         <v>0</v>
       </c>
       <c r="U79" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="V79" t="n">
         <v>5</v>
       </c>
+      <c r="W79" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6406,11 +6646,14 @@
         <v>0</v>
       </c>
       <c r="U80" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="V80" t="n">
         <v>7</v>
       </c>
+      <c r="W80" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6480,10 +6723,13 @@
         <v>0</v>
       </c>
       <c r="U81" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V81" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W81" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="82">
@@ -6554,10 +6800,13 @@
         <v>0</v>
       </c>
       <c r="U82" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V82" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W82" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="83">
@@ -6628,10 +6877,13 @@
         <v>0</v>
       </c>
       <c r="U83" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="V83" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="W83" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="84">
@@ -6702,11 +6954,14 @@
         <v>0</v>
       </c>
       <c r="U84" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V84" t="n">
         <v>2</v>
       </c>
+      <c r="W84" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6781,6 +7036,9 @@
       <c r="V85" t="n">
         <v>0</v>
       </c>
+      <c r="W85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6850,10 +7108,13 @@
         <v>0</v>
       </c>
       <c r="U86" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="V86" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="W86" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="87">
@@ -6929,6 +7190,9 @@
       <c r="V87" t="n">
         <v>0</v>
       </c>
+      <c r="W87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6998,10 +7262,13 @@
         <v>0</v>
       </c>
       <c r="U88" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V88" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="W88" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="89">
@@ -7077,6 +7344,9 @@
       <c r="V89" t="n">
         <v>0</v>
       </c>
+      <c r="W89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7146,10 +7416,13 @@
         <v>0</v>
       </c>
       <c r="U90" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V90" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="W90" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="91">
@@ -7225,6 +7498,9 @@
       <c r="V91" t="n">
         <v>0</v>
       </c>
+      <c r="W91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7299,6 +7575,9 @@
       <c r="V92" t="n">
         <v>0</v>
       </c>
+      <c r="W92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7368,10 +7647,13 @@
         <v>0</v>
       </c>
       <c r="U93" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="V93" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="W93" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="94">
@@ -7442,10 +7724,13 @@
         <v>0</v>
       </c>
       <c r="U94" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V94" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="W94" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="95">
@@ -7516,10 +7801,13 @@
         <v>0</v>
       </c>
       <c r="U95" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="V95" t="n">
-        <v>5</v>
+        <v>35</v>
+      </c>
+      <c r="W95" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="96">
@@ -7590,11 +7878,14 @@
         <v>0</v>
       </c>
       <c r="U96" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V96" t="n">
         <v>4</v>
       </c>
+      <c r="W96" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7669,6 +7960,9 @@
       <c r="V97" t="n">
         <v>0</v>
       </c>
+      <c r="W97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7738,11 +8032,14 @@
         <v>0</v>
       </c>
       <c r="U98" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="V98" t="n">
         <v>5</v>
       </c>
+      <c r="W98" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7812,9 +8109,12 @@
         <v>0</v>
       </c>
       <c r="U99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V99" t="n">
+        <v>1</v>
+      </c>
+      <c r="W99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7886,11 +8186,14 @@
         <v>0</v>
       </c>
       <c r="U100" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V100" t="n">
         <v>3</v>
       </c>
+      <c r="W100" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7960,10 +8263,13 @@
         <v>0</v>
       </c>
       <c r="U101" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V101" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W101" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="102">
@@ -8039,6 +8345,9 @@
       <c r="V102" t="n">
         <v>0</v>
       </c>
+      <c r="W102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8108,10 +8417,13 @@
         <v>0</v>
       </c>
       <c r="U103" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="V103" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="W103" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="104">
@@ -8182,9 +8494,12 @@
         <v>0</v>
       </c>
       <c r="U104" t="n">
+        <v>0</v>
+      </c>
+      <c r="V104" t="n">
         <v>12</v>
       </c>
-      <c r="V104" t="n">
+      <c r="W104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8256,10 +8571,13 @@
         <v>0</v>
       </c>
       <c r="U105" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="V105" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="W105" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="106">
@@ -8330,10 +8648,13 @@
         <v>0</v>
       </c>
       <c r="U106" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V106" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W106" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="107">
@@ -8409,6 +8730,9 @@
       <c r="V107" t="n">
         <v>0</v>
       </c>
+      <c r="W107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8478,10 +8802,13 @@
         <v>0</v>
       </c>
       <c r="U108" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V108" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="W108" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="109">
@@ -8555,6 +8882,9 @@
         <v>0</v>
       </c>
       <c r="V109" t="n">
+        <v>0</v>
+      </c>
+      <c r="W109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1703)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W109"/>
+  <dimension ref="A1:X109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -451,8 +451,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -561,12 +562,17 @@
           <t>2026-03-09</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -643,10 +649,13 @@
         <v>1</v>
       </c>
       <c r="V2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="W2" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="X2" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -720,11 +729,14 @@
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W3" t="n">
         <v>6</v>
       </c>
+      <c r="X3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -797,10 +809,13 @@
         <v>1</v>
       </c>
       <c r="V4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W4" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X4" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -874,10 +889,13 @@
         <v>1</v>
       </c>
       <c r="V5" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W5" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X5" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -951,10 +969,13 @@
         <v>1</v>
       </c>
       <c r="V6" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W6" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X6" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -1028,11 +1049,14 @@
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="W7" t="n">
         <v>9</v>
       </c>
+      <c r="X7" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1105,10 +1129,13 @@
         <v>1</v>
       </c>
       <c r="V8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W8" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X8" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -1182,10 +1209,13 @@
         <v>1</v>
       </c>
       <c r="V9" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="W9" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="X9" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -1259,10 +1289,13 @@
         <v>1</v>
       </c>
       <c r="V10" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W10" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X10" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -1336,10 +1369,13 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W11" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X11" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -1413,10 +1449,13 @@
         <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="W12" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="X12" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -1490,11 +1529,14 @@
         <v>1</v>
       </c>
       <c r="V13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W13" t="n">
         <v>6</v>
       </c>
+      <c r="X13" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1567,10 +1609,13 @@
         <v>1</v>
       </c>
       <c r="V14" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W14" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X14" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="15">
@@ -1644,10 +1689,13 @@
         <v>1</v>
       </c>
       <c r="V15" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="W15" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="X15" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -1721,10 +1769,13 @@
         <v>1</v>
       </c>
       <c r="V16" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="W16" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="X16" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="17">
@@ -1798,10 +1849,13 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W17" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X17" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="18">
@@ -1875,11 +1929,14 @@
         <v>1</v>
       </c>
       <c r="V18" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="W18" t="n">
         <v>11</v>
       </c>
+      <c r="X18" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1952,11 +2009,14 @@
         <v>1</v>
       </c>
       <c r="V19" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="W19" t="n">
         <v>9</v>
       </c>
+      <c r="X19" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2029,10 +2089,13 @@
         <v>1</v>
       </c>
       <c r="V20" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W20" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X20" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -2111,6 +2174,9 @@
       <c r="W21" t="n">
         <v>0</v>
       </c>
+      <c r="X21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2188,6 +2254,9 @@
       <c r="W22" t="n">
         <v>0</v>
       </c>
+      <c r="X22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2260,10 +2329,13 @@
         <v>0</v>
       </c>
       <c r="V23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W23" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="X23" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="24">
@@ -2337,10 +2409,13 @@
         <v>1</v>
       </c>
       <c r="V24" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W24" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X24" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="25">
@@ -2414,11 +2489,14 @@
         <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W25" t="n">
         <v>6</v>
       </c>
+      <c r="X25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2491,10 +2569,13 @@
         <v>1</v>
       </c>
       <c r="V26" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="W26" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="X26" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="27">
@@ -2568,10 +2649,13 @@
         <v>1</v>
       </c>
       <c r="V27" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="W27" t="n">
-        <v>9</v>
+        <v>12</v>
+      </c>
+      <c r="X27" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="28">
@@ -2650,6 +2734,9 @@
       <c r="W28" t="n">
         <v>0</v>
       </c>
+      <c r="X28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2727,6 +2814,9 @@
       <c r="W29" t="n">
         <v>0</v>
       </c>
+      <c r="X29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2799,10 +2889,13 @@
         <v>0</v>
       </c>
       <c r="V30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W30" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="X30" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="31">
@@ -2876,11 +2969,14 @@
         <v>0</v>
       </c>
       <c r="V31" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="W31" t="n">
         <v>9</v>
       </c>
+      <c r="X31" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2953,11 +3049,14 @@
         <v>1</v>
       </c>
       <c r="V32" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="W32" t="n">
         <v>10</v>
       </c>
+      <c r="X32" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3030,10 +3129,13 @@
         <v>0</v>
       </c>
       <c r="V33" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W33" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X33" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="34">
@@ -3107,10 +3209,13 @@
         <v>1</v>
       </c>
       <c r="V34" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W34" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X34" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="35">
@@ -3184,11 +3289,14 @@
         <v>1</v>
       </c>
       <c r="V35" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W35" t="n">
         <v>6</v>
       </c>
+      <c r="X35" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3261,10 +3369,13 @@
         <v>1</v>
       </c>
       <c r="V36" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W36" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X36" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="37">
@@ -3338,10 +3449,13 @@
         <v>1</v>
       </c>
       <c r="V37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W37" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="X37" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="38">
@@ -3420,6 +3534,9 @@
       <c r="W38" t="n">
         <v>0</v>
       </c>
+      <c r="X38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3492,11 +3609,14 @@
         <v>0</v>
       </c>
       <c r="V39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W39" t="n">
         <v>2</v>
       </c>
+      <c r="X39" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3569,10 +3689,13 @@
         <v>1</v>
       </c>
       <c r="V40" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W40" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X40" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="41">
@@ -3646,11 +3769,14 @@
         <v>1</v>
       </c>
       <c r="V41" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="W41" t="n">
         <v>10</v>
       </c>
+      <c r="X41" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3723,10 +3849,13 @@
         <v>1</v>
       </c>
       <c r="V42" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="W42" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="X42" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="43">
@@ -3800,9 +3929,12 @@
         <v>0</v>
       </c>
       <c r="V43" t="n">
+        <v>0</v>
+      </c>
+      <c r="W43" t="n">
         <v>21</v>
       </c>
-      <c r="W43" t="n">
+      <c r="X43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3877,10 +4009,13 @@
         <v>1</v>
       </c>
       <c r="V44" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="W44" t="n">
-        <v>6</v>
+        <v>48</v>
+      </c>
+      <c r="X44" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="45">
@@ -3954,10 +4089,13 @@
         <v>1</v>
       </c>
       <c r="V45" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="W45" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="X45" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="46">
@@ -4031,10 +4169,13 @@
         <v>1</v>
       </c>
       <c r="V46" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="W46" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="X46" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="47">
@@ -4108,10 +4249,13 @@
         <v>1</v>
       </c>
       <c r="V47" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="W47" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="X47" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="48">
@@ -4190,6 +4334,9 @@
       <c r="W48" t="n">
         <v>0</v>
       </c>
+      <c r="X48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4262,10 +4409,13 @@
         <v>1</v>
       </c>
       <c r="V49" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W49" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X49" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="50">
@@ -4339,10 +4489,13 @@
         <v>1</v>
       </c>
       <c r="V50" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W50" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X50" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="51">
@@ -4416,11 +4569,14 @@
         <v>0</v>
       </c>
       <c r="V51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W51" t="n">
         <v>2</v>
       </c>
+      <c r="X51" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4493,11 +4649,14 @@
         <v>1</v>
       </c>
       <c r="V52" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W52" t="n">
         <v>5</v>
       </c>
+      <c r="X52" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4570,10 +4729,13 @@
         <v>1</v>
       </c>
       <c r="V53" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W53" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X53" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="54">
@@ -4652,6 +4814,9 @@
       <c r="W54" t="n">
         <v>0</v>
       </c>
+      <c r="X54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4724,11 +4889,14 @@
         <v>1</v>
       </c>
       <c r="V55" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="W55" t="n">
         <v>9</v>
       </c>
+      <c r="X55" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4806,6 +4974,9 @@
       <c r="W56" t="n">
         <v>0</v>
       </c>
+      <c r="X56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4878,10 +5049,13 @@
         <v>1</v>
       </c>
       <c r="V57" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W57" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X57" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="58">
@@ -4955,10 +5129,13 @@
         <v>1</v>
       </c>
       <c r="V58" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W58" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X58" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="59">
@@ -5032,10 +5209,13 @@
         <v>1</v>
       </c>
       <c r="V59" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="W59" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="X59" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="60">
@@ -5109,10 +5289,13 @@
         <v>1</v>
       </c>
       <c r="V60" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="W60" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="X60" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="61">
@@ -5186,11 +5369,14 @@
         <v>0</v>
       </c>
       <c r="V61" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W61" t="n">
         <v>3</v>
       </c>
+      <c r="X61" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5268,6 +5454,9 @@
       <c r="W62" t="n">
         <v>0</v>
       </c>
+      <c r="X62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5340,10 +5529,13 @@
         <v>1</v>
       </c>
       <c r="V63" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="W63" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="X63" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="64">
@@ -5417,10 +5609,13 @@
         <v>1</v>
       </c>
       <c r="V64" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W64" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X64" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="65">
@@ -5499,6 +5694,9 @@
       <c r="W65" t="n">
         <v>0</v>
       </c>
+      <c r="X65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5576,6 +5774,9 @@
       <c r="W66" t="n">
         <v>0</v>
       </c>
+      <c r="X66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5648,10 +5849,13 @@
         <v>0</v>
       </c>
       <c r="V67" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W67" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="X67" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="68">
@@ -5730,6 +5934,9 @@
       <c r="W68" t="n">
         <v>0</v>
       </c>
+      <c r="X68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5807,6 +6014,9 @@
       <c r="W69" t="n">
         <v>0</v>
       </c>
+      <c r="X69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5879,10 +6089,13 @@
         <v>1</v>
       </c>
       <c r="V70" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="W70" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="X70" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="71">
@@ -5959,7 +6172,10 @@
         <v>2</v>
       </c>
       <c r="W71" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="X71" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="72">
@@ -6038,6 +6254,9 @@
       <c r="W72" t="n">
         <v>0</v>
       </c>
+      <c r="X72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6110,10 +6329,13 @@
         <v>1</v>
       </c>
       <c r="V73" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="W73" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="X73" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="74">
@@ -6187,10 +6409,13 @@
         <v>0</v>
       </c>
       <c r="V74" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="W74" t="n">
-        <v>7</v>
+        <v>20</v>
+      </c>
+      <c r="X74" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="75">
@@ -6264,10 +6489,13 @@
         <v>1</v>
       </c>
       <c r="V75" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W75" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="X75" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="76">
@@ -6341,10 +6569,13 @@
         <v>1</v>
       </c>
       <c r="V76" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W76" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X76" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="77">
@@ -6423,6 +6654,9 @@
       <c r="W77" t="n">
         <v>0</v>
       </c>
+      <c r="X77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6500,6 +6734,9 @@
       <c r="W78" t="n">
         <v>0</v>
       </c>
+      <c r="X78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6572,10 +6809,13 @@
         <v>0</v>
       </c>
       <c r="V79" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="W79" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="X79" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="80">
@@ -6649,10 +6889,13 @@
         <v>0</v>
       </c>
       <c r="V80" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="W80" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="X80" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="81">
@@ -6726,10 +6969,13 @@
         <v>1</v>
       </c>
       <c r="V81" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W81" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X81" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="82">
@@ -6803,10 +7049,13 @@
         <v>1</v>
       </c>
       <c r="V82" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W82" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X82" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="83">
@@ -6880,10 +7129,13 @@
         <v>1</v>
       </c>
       <c r="V83" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="W83" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="X83" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="84">
@@ -6957,11 +7209,14 @@
         <v>0</v>
       </c>
       <c r="V84" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W84" t="n">
         <v>2</v>
       </c>
+      <c r="X84" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7039,6 +7294,9 @@
       <c r="W85" t="n">
         <v>0</v>
       </c>
+      <c r="X85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7111,10 +7369,13 @@
         <v>1</v>
       </c>
       <c r="V86" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="W86" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="X86" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="87">
@@ -7193,6 +7454,9 @@
       <c r="W87" t="n">
         <v>0</v>
       </c>
+      <c r="X87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7265,11 +7529,14 @@
         <v>1</v>
       </c>
       <c r="V88" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W88" t="n">
         <v>6</v>
       </c>
+      <c r="X88" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7347,6 +7614,9 @@
       <c r="W89" t="n">
         <v>0</v>
       </c>
+      <c r="X89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7419,10 +7689,13 @@
         <v>1</v>
       </c>
       <c r="V90" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="W90" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="X90" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="91">
@@ -7501,6 +7774,9 @@
       <c r="W91" t="n">
         <v>0</v>
       </c>
+      <c r="X91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7578,6 +7854,9 @@
       <c r="W92" t="n">
         <v>0</v>
       </c>
+      <c r="X92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7650,10 +7929,13 @@
         <v>1</v>
       </c>
       <c r="V93" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="W93" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="X93" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="94">
@@ -7727,10 +8009,13 @@
         <v>1</v>
       </c>
       <c r="V94" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="W94" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="X94" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="95">
@@ -7804,10 +8089,13 @@
         <v>1</v>
       </c>
       <c r="V95" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="W95" t="n">
-        <v>6</v>
+        <v>36</v>
+      </c>
+      <c r="X95" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="96">
@@ -7881,11 +8169,14 @@
         <v>0</v>
       </c>
       <c r="V96" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W96" t="n">
         <v>4</v>
       </c>
+      <c r="X96" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7963,6 +8254,9 @@
       <c r="W97" t="n">
         <v>0</v>
       </c>
+      <c r="X97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8035,10 +8329,13 @@
         <v>0</v>
       </c>
       <c r="V98" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="W98" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="X98" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="99">
@@ -8112,9 +8409,12 @@
         <v>0</v>
       </c>
       <c r="V99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W99" t="n">
+        <v>1</v>
+      </c>
+      <c r="X99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8189,10 +8489,13 @@
         <v>0</v>
       </c>
       <c r="V100" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W100" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="X100" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="101">
@@ -8266,10 +8569,13 @@
         <v>1</v>
       </c>
       <c r="V101" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W101" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X101" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="102">
@@ -8348,6 +8654,9 @@
       <c r="W102" t="n">
         <v>0</v>
       </c>
+      <c r="X102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8420,10 +8729,13 @@
         <v>1</v>
       </c>
       <c r="V103" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="W103" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="X103" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="104">
@@ -8497,9 +8809,12 @@
         <v>0</v>
       </c>
       <c r="V104" t="n">
+        <v>0</v>
+      </c>
+      <c r="W104" t="n">
         <v>12</v>
       </c>
-      <c r="W104" t="n">
+      <c r="X104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8574,10 +8889,13 @@
         <v>1</v>
       </c>
       <c r="V105" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W105" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="X105" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="106">
@@ -8651,10 +8969,13 @@
         <v>1</v>
       </c>
       <c r="V106" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W106" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X106" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="107">
@@ -8733,6 +9054,9 @@
       <c r="W107" t="n">
         <v>0</v>
       </c>
+      <c r="X107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8805,10 +9129,13 @@
         <v>1</v>
       </c>
       <c r="V108" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W108" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="X108" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="109">
@@ -8882,10 +9209,13 @@
         <v>0</v>
       </c>
       <c r="V109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W109" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="X109" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1816)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y109"/>
+  <dimension ref="A1:Z109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -453,8 +453,9 @@
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
     <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -573,12 +574,17 @@
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -661,11 +667,14 @@
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Y2" t="n">
         <v>9</v>
       </c>
+      <c r="Z2" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -744,11 +753,14 @@
         <v>1</v>
       </c>
       <c r="X3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Y3" t="n">
         <v>7</v>
       </c>
+      <c r="Z3" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -827,11 +839,14 @@
         <v>1</v>
       </c>
       <c r="X4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y4" t="n">
         <v>12</v>
       </c>
+      <c r="Z4" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -910,11 +925,14 @@
         <v>1</v>
       </c>
       <c r="X5" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y5" t="n">
         <v>12</v>
       </c>
+      <c r="Z5" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -993,11 +1011,14 @@
         <v>1</v>
       </c>
       <c r="X6" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y6" t="n">
         <v>11</v>
       </c>
+      <c r="Z6" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1076,11 +1097,14 @@
         <v>1</v>
       </c>
       <c r="X7" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y7" t="n">
         <v>10</v>
       </c>
+      <c r="Z7" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1159,11 +1183,14 @@
         <v>1</v>
       </c>
       <c r="X8" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y8" t="n">
         <v>12</v>
       </c>
+      <c r="Z8" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1242,11 +1269,14 @@
         <v>1</v>
       </c>
       <c r="X9" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Y9" t="n">
         <v>13</v>
       </c>
+      <c r="Z9" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1325,11 +1355,14 @@
         <v>1</v>
       </c>
       <c r="X10" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="n">
         <v>12</v>
       </c>
+      <c r="Z10" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1408,11 +1441,14 @@
         <v>1</v>
       </c>
       <c r="X11" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y11" t="n">
         <v>11</v>
       </c>
+      <c r="Z11" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1491,11 +1527,14 @@
         <v>1</v>
       </c>
       <c r="X12" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Y12" t="n">
         <v>13</v>
       </c>
+      <c r="Z12" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1574,11 +1613,14 @@
         <v>1</v>
       </c>
       <c r="X13" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Y13" t="n">
         <v>7</v>
       </c>
+      <c r="Z13" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1657,11 +1699,14 @@
         <v>1</v>
       </c>
       <c r="X14" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y14" t="n">
         <v>12</v>
       </c>
+      <c r="Z14" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1740,11 +1785,14 @@
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Y15" t="n">
         <v>9</v>
       </c>
+      <c r="Z15" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1823,11 +1871,14 @@
         <v>1</v>
       </c>
       <c r="X16" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y16" t="n">
         <v>10</v>
       </c>
+      <c r="Z16" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1906,11 +1957,14 @@
         <v>1</v>
       </c>
       <c r="X17" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y17" t="n">
         <v>11</v>
       </c>
+      <c r="Z17" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1989,11 +2043,14 @@
         <v>0</v>
       </c>
       <c r="X18" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y18" t="n">
         <v>11</v>
       </c>
+      <c r="Z18" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2077,6 +2134,9 @@
       <c r="Y19" t="n">
         <v>0</v>
       </c>
+      <c r="Z19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2155,11 +2215,14 @@
         <v>1</v>
       </c>
       <c r="X20" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y20" t="n">
         <v>10</v>
       </c>
+      <c r="Z20" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2238,11 +2301,14 @@
         <v>1</v>
       </c>
       <c r="X21" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y21" t="n">
         <v>11</v>
       </c>
+      <c r="Z21" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2326,6 +2392,9 @@
       <c r="Y22" t="n">
         <v>0</v>
       </c>
+      <c r="Z22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2404,11 +2473,14 @@
         <v>1</v>
       </c>
       <c r="X23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y23" t="n">
         <v>6</v>
       </c>
+      <c r="Z23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2487,11 +2559,14 @@
         <v>1</v>
       </c>
       <c r="X24" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y24" t="n">
         <v>11</v>
       </c>
+      <c r="Z24" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2570,11 +2645,14 @@
         <v>0</v>
       </c>
       <c r="X25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y25" t="n">
         <v>6</v>
       </c>
+      <c r="Z25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2653,11 +2731,14 @@
         <v>1</v>
       </c>
       <c r="X26" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Y26" t="n">
         <v>9</v>
       </c>
+      <c r="Z26" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2736,9 +2817,12 @@
         <v>1</v>
       </c>
       <c r="X27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y27" t="n">
         <v>13</v>
       </c>
-      <c r="Y27" t="n">
+      <c r="Z27" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2819,9 +2903,12 @@
         <v>1</v>
       </c>
       <c r="X28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y28" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2902,11 +2989,14 @@
         <v>1</v>
       </c>
       <c r="X29" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Y29" t="n">
         <v>4</v>
       </c>
+      <c r="Z29" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2985,11 +3075,14 @@
         <v>1</v>
       </c>
       <c r="X30" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y30" t="n">
         <v>10</v>
       </c>
+      <c r="Z30" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3068,11 +3161,14 @@
         <v>0</v>
       </c>
       <c r="X31" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y31" t="n">
         <v>10</v>
       </c>
+      <c r="Z31" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3151,11 +3247,14 @@
         <v>0</v>
       </c>
       <c r="X32" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y32" t="n">
         <v>10</v>
       </c>
+      <c r="Z32" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3234,11 +3333,14 @@
         <v>1</v>
       </c>
       <c r="X33" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y33" t="n">
         <v>11</v>
       </c>
+      <c r="Z33" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3317,11 +3419,14 @@
         <v>0</v>
       </c>
       <c r="X34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y34" t="n">
         <v>6</v>
       </c>
+      <c r="Z34" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3400,11 +3505,14 @@
         <v>1</v>
       </c>
       <c r="X35" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y35" t="n">
         <v>11</v>
       </c>
+      <c r="Z35" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3483,11 +3591,14 @@
         <v>1</v>
       </c>
       <c r="X36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y36" t="n">
         <v>6</v>
       </c>
+      <c r="Z36" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3571,6 +3682,9 @@
       <c r="Y37" t="n">
         <v>0</v>
       </c>
+      <c r="Z37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3649,11 +3763,14 @@
         <v>0</v>
       </c>
       <c r="X38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y38" t="n">
         <v>2</v>
       </c>
+      <c r="Z38" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3732,11 +3849,14 @@
         <v>1</v>
       </c>
       <c r="X39" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y39" t="n">
         <v>12</v>
       </c>
+      <c r="Z39" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3815,11 +3935,14 @@
         <v>1</v>
       </c>
       <c r="X40" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y40" t="n">
         <v>11</v>
       </c>
+      <c r="Z40" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3898,11 +4021,14 @@
         <v>1</v>
       </c>
       <c r="X41" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Y41" t="n">
         <v>13</v>
       </c>
+      <c r="Z41" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3981,9 +4107,12 @@
         <v>0</v>
       </c>
       <c r="X42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y42" t="n">
         <v>21</v>
       </c>
-      <c r="Y42" t="n">
+      <c r="Z42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4064,9 +4193,12 @@
         <v>1</v>
       </c>
       <c r="X43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y43" t="n">
         <v>49</v>
       </c>
-      <c r="Y43" t="n">
+      <c r="Z43" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4147,11 +4279,14 @@
         <v>1</v>
       </c>
       <c r="X44" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y44" t="n">
         <v>10</v>
       </c>
+      <c r="Z44" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4230,11 +4365,14 @@
         <v>0</v>
       </c>
       <c r="X45" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y45" t="n">
         <v>12</v>
       </c>
+      <c r="Z45" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4313,11 +4451,14 @@
         <v>1</v>
       </c>
       <c r="X46" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y46" t="n">
         <v>10</v>
       </c>
+      <c r="Z46" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4401,6 +4542,9 @@
       <c r="Y47" t="n">
         <v>0</v>
       </c>
+      <c r="Z47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4479,11 +4623,14 @@
         <v>1</v>
       </c>
       <c r="X48" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y48" t="n">
         <v>12</v>
       </c>
+      <c r="Z48" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4562,11 +4709,14 @@
         <v>1</v>
       </c>
       <c r="X49" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y49" t="n">
         <v>11</v>
       </c>
+      <c r="Z49" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4645,11 +4795,14 @@
         <v>1</v>
       </c>
       <c r="X50" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y50" t="n">
         <v>6</v>
       </c>
+      <c r="Z50" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4728,11 +4881,14 @@
         <v>1</v>
       </c>
       <c r="X51" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y51" t="n">
         <v>12</v>
       </c>
+      <c r="Z51" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4816,6 +4972,9 @@
       <c r="Y52" t="n">
         <v>0</v>
       </c>
+      <c r="Z52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4894,11 +5053,14 @@
         <v>1</v>
       </c>
       <c r="X53" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y53" t="n">
         <v>10</v>
       </c>
+      <c r="Z53" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4982,6 +5144,9 @@
       <c r="Y54" t="n">
         <v>0</v>
       </c>
+      <c r="Z54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5060,11 +5225,14 @@
         <v>1</v>
       </c>
       <c r="X55" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y55" t="n">
         <v>11</v>
       </c>
+      <c r="Z55" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5143,11 +5311,14 @@
         <v>1</v>
       </c>
       <c r="X56" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y56" t="n">
         <v>11</v>
       </c>
+      <c r="Z56" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5226,11 +5397,14 @@
         <v>1</v>
       </c>
       <c r="X57" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Y57" t="n">
         <v>7</v>
       </c>
+      <c r="Z57" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5309,11 +5483,14 @@
         <v>0</v>
       </c>
       <c r="X58" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y58" t="n">
         <v>12</v>
       </c>
+      <c r="Z58" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5392,11 +5569,14 @@
         <v>0</v>
       </c>
       <c r="X59" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y59" t="n">
         <v>3</v>
       </c>
+      <c r="Z59" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5480,6 +5660,9 @@
       <c r="Y60" t="n">
         <v>0</v>
       </c>
+      <c r="Z60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5558,11 +5741,14 @@
         <v>1</v>
       </c>
       <c r="X61" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Y61" t="n">
         <v>9</v>
       </c>
+      <c r="Z61" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5641,11 +5827,14 @@
         <v>1</v>
       </c>
       <c r="X62" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y62" t="n">
         <v>12</v>
       </c>
+      <c r="Z62" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5724,9 +5913,12 @@
         <v>1</v>
       </c>
       <c r="X63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y63" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z63" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5812,6 +6004,9 @@
       <c r="Y64" t="n">
         <v>0</v>
       </c>
+      <c r="Z64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5890,11 +6085,14 @@
         <v>0</v>
       </c>
       <c r="X65" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Y65" t="n">
         <v>5</v>
       </c>
+      <c r="Z65" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5973,9 +6171,12 @@
         <v>1</v>
       </c>
       <c r="X66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y66" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6056,11 +6257,14 @@
         <v>1</v>
       </c>
       <c r="X67" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Y67" t="n">
         <v>13</v>
       </c>
+      <c r="Z67" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6139,9 +6343,12 @@
         <v>1</v>
       </c>
       <c r="X68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y68" t="n">
         <v>5</v>
       </c>
-      <c r="Y68" t="n">
+      <c r="Z68" t="n">
         <v>4</v>
       </c>
     </row>
@@ -6222,11 +6429,14 @@
         <v>0</v>
       </c>
       <c r="X69" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Y69" t="n">
         <v>7</v>
       </c>
+      <c r="Z69" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6305,9 +6515,12 @@
         <v>1</v>
       </c>
       <c r="X70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y70" t="n">
         <v>21</v>
       </c>
-      <c r="Y70" t="n">
+      <c r="Z70" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6388,11 +6601,14 @@
         <v>1</v>
       </c>
       <c r="X71" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y71" t="n">
         <v>6</v>
       </c>
+      <c r="Z71" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6471,11 +6687,14 @@
         <v>0</v>
       </c>
       <c r="X72" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y72" t="n">
         <v>10</v>
       </c>
+      <c r="Z72" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6559,6 +6778,9 @@
       <c r="Y73" t="n">
         <v>0</v>
       </c>
+      <c r="Z73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6642,6 +6864,9 @@
       <c r="Y74" t="n">
         <v>0</v>
       </c>
+      <c r="Z74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6720,11 +6945,14 @@
         <v>1</v>
       </c>
       <c r="X75" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Y75" t="n">
         <v>7</v>
       </c>
+      <c r="Z75" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6803,11 +7031,14 @@
         <v>1</v>
       </c>
       <c r="X76" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Y76" t="n">
         <v>9</v>
       </c>
+      <c r="Z76" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6886,11 +7117,14 @@
         <v>1</v>
       </c>
       <c r="X77" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y77" t="n">
         <v>11</v>
       </c>
+      <c r="Z77" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6969,11 +7203,14 @@
         <v>1</v>
       </c>
       <c r="X78" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y78" t="n">
         <v>12</v>
       </c>
+      <c r="Z78" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7052,11 +7289,14 @@
         <v>1</v>
       </c>
       <c r="X79" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Y79" t="n">
         <v>9</v>
       </c>
+      <c r="Z79" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7135,11 +7375,14 @@
         <v>1</v>
       </c>
       <c r="X80" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y80" t="n">
         <v>3</v>
       </c>
+      <c r="Z80" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7218,9 +7461,12 @@
         <v>1</v>
       </c>
       <c r="X81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y81" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z81" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7306,6 +7552,9 @@
       <c r="Y82" t="n">
         <v>0</v>
       </c>
+      <c r="Z82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7384,11 +7633,14 @@
         <v>1</v>
       </c>
       <c r="X83" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Y83" t="n">
         <v>9</v>
       </c>
+      <c r="Z83" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7467,9 +7719,12 @@
         <v>1</v>
       </c>
       <c r="X84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y84" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z84" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7550,11 +7805,14 @@
         <v>1</v>
       </c>
       <c r="X85" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Y85" t="n">
         <v>7</v>
       </c>
+      <c r="Z85" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7638,6 +7896,9 @@
       <c r="Y86" t="n">
         <v>0</v>
       </c>
+      <c r="Z86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7716,11 +7977,14 @@
         <v>1</v>
       </c>
       <c r="X87" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Y87" t="n">
         <v>7</v>
       </c>
+      <c r="Z87" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7804,6 +8068,9 @@
       <c r="Y88" t="n">
         <v>0</v>
       </c>
+      <c r="Z88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7882,11 +8149,14 @@
         <v>1</v>
       </c>
       <c r="X89" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Y89" t="n">
         <v>9</v>
       </c>
+      <c r="Z89" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7965,11 +8235,14 @@
         <v>1</v>
       </c>
       <c r="X90" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Y90" t="n">
         <v>8</v>
       </c>
+      <c r="Z90" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -8048,9 +8321,12 @@
         <v>1</v>
       </c>
       <c r="X91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y91" t="n">
         <v>37</v>
       </c>
-      <c r="Y91" t="n">
+      <c r="Z91" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8131,11 +8407,14 @@
         <v>0</v>
       </c>
       <c r="X92" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Y92" t="n">
         <v>4</v>
       </c>
+      <c r="Z92" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -8219,6 +8498,9 @@
       <c r="Y93" t="n">
         <v>0</v>
       </c>
+      <c r="Z93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -8297,11 +8579,14 @@
         <v>0</v>
       </c>
       <c r="X94" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y94" t="n">
         <v>6</v>
       </c>
+      <c r="Z94" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -8380,11 +8665,14 @@
         <v>1</v>
       </c>
       <c r="X95" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Y95" t="n">
         <v>5</v>
       </c>
+      <c r="Z95" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -8463,11 +8751,14 @@
         <v>1</v>
       </c>
       <c r="X96" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y96" t="n">
         <v>12</v>
       </c>
+      <c r="Z96" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -8551,6 +8842,9 @@
       <c r="Y97" t="n">
         <v>0</v>
       </c>
+      <c r="Z97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8629,11 +8923,14 @@
         <v>1</v>
       </c>
       <c r="X98" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Y98" t="n">
         <v>13</v>
       </c>
+      <c r="Z98" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -8712,9 +9009,12 @@
         <v>1</v>
       </c>
       <c r="X99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y99" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8800,6 +9100,9 @@
       <c r="Y100" t="n">
         <v>0</v>
       </c>
+      <c r="Z100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8878,11 +9181,14 @@
         <v>1</v>
       </c>
       <c r="X101" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y101" t="n">
         <v>12</v>
       </c>
+      <c r="Z101" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8961,11 +9267,14 @@
         <v>1</v>
       </c>
       <c r="X102" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y102" t="n">
         <v>11</v>
       </c>
+      <c r="Z102" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -9044,11 +9353,14 @@
         <v>1</v>
       </c>
       <c r="X103" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Y103" t="n">
         <v>11</v>
       </c>
+      <c r="Z103" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9127,11 +9439,14 @@
         <v>1</v>
       </c>
       <c r="X104" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y104" t="n">
         <v>2</v>
       </c>
+      <c r="Z104" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9210,9 +9525,12 @@
         <v>1</v>
       </c>
       <c r="X105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y105" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z105" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9293,9 +9611,12 @@
         <v>1</v>
       </c>
       <c r="X106" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y106" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z106" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9376,9 +9697,12 @@
         <v>1</v>
       </c>
       <c r="X107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y107" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z107" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9459,9 +9783,12 @@
         <v>1</v>
       </c>
       <c r="X108" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y108" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z108" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9545,6 +9872,9 @@
         <v>0</v>
       </c>
       <c r="Y109" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1819)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z109"/>
+  <dimension ref="A1:AA109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -454,8 +454,9 @@
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
-    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
     <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -579,12 +580,17 @@
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -670,11 +676,14 @@
         <v>0</v>
       </c>
       <c r="Y2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Z2" t="n">
         <v>9</v>
       </c>
+      <c r="AA2" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -756,11 +765,14 @@
         <v>0</v>
       </c>
       <c r="Y3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z3" t="n">
         <v>7</v>
       </c>
+      <c r="AA3" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -842,11 +854,14 @@
         <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z4" t="n">
         <v>12</v>
       </c>
+      <c r="AA4" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -928,11 +943,14 @@
         <v>0</v>
       </c>
       <c r="Y5" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z5" t="n">
         <v>12</v>
       </c>
+      <c r="AA5" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1014,11 +1032,14 @@
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z6" t="n">
         <v>11</v>
       </c>
+      <c r="AA6" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1100,11 +1121,14 @@
         <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Z7" t="n">
         <v>10</v>
       </c>
+      <c r="AA7" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1186,11 +1210,14 @@
         <v>0</v>
       </c>
       <c r="Y8" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z8" t="n">
         <v>12</v>
       </c>
+      <c r="AA8" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1272,11 +1299,14 @@
         <v>0</v>
       </c>
       <c r="Y9" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Z9" t="n">
         <v>13</v>
       </c>
+      <c r="AA9" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1358,11 +1388,14 @@
         <v>0</v>
       </c>
       <c r="Y10" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="n">
         <v>12</v>
       </c>
+      <c r="AA10" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1444,11 +1477,14 @@
         <v>0</v>
       </c>
       <c r="Y11" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z11" t="n">
         <v>11</v>
       </c>
+      <c r="AA11" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1530,11 +1566,14 @@
         <v>0</v>
       </c>
       <c r="Y12" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Z12" t="n">
         <v>13</v>
       </c>
+      <c r="AA12" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1616,11 +1655,14 @@
         <v>0</v>
       </c>
       <c r="Y13" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z13" t="n">
         <v>7</v>
       </c>
+      <c r="AA13" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1702,11 +1744,14 @@
         <v>0</v>
       </c>
       <c r="Y14" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z14" t="n">
         <v>12</v>
       </c>
+      <c r="AA14" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1788,11 +1833,14 @@
         <v>0</v>
       </c>
       <c r="Y15" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Z15" t="n">
         <v>9</v>
       </c>
+      <c r="AA15" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1874,11 +1922,14 @@
         <v>0</v>
       </c>
       <c r="Y16" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Z16" t="n">
         <v>10</v>
       </c>
+      <c r="AA16" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1960,11 +2011,14 @@
         <v>0</v>
       </c>
       <c r="Y17" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z17" t="n">
         <v>11</v>
       </c>
+      <c r="AA17" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2046,11 +2100,14 @@
         <v>0</v>
       </c>
       <c r="Y18" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z18" t="n">
         <v>11</v>
       </c>
+      <c r="AA18" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2137,6 +2194,9 @@
       <c r="Z19" t="n">
         <v>0</v>
       </c>
+      <c r="AA19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2218,11 +2278,14 @@
         <v>0</v>
       </c>
       <c r="Y20" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Z20" t="n">
         <v>10</v>
       </c>
+      <c r="AA20" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2304,11 +2367,14 @@
         <v>0</v>
       </c>
       <c r="Y21" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z21" t="n">
         <v>11</v>
       </c>
+      <c r="AA21" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2395,6 +2461,9 @@
       <c r="Z22" t="n">
         <v>0</v>
       </c>
+      <c r="AA22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2476,11 +2545,14 @@
         <v>0</v>
       </c>
       <c r="Y23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z23" t="n">
         <v>6</v>
       </c>
+      <c r="AA23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2562,11 +2634,14 @@
         <v>0</v>
       </c>
       <c r="Y24" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z24" t="n">
         <v>11</v>
       </c>
+      <c r="AA24" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2648,11 +2723,14 @@
         <v>0</v>
       </c>
       <c r="Y25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z25" t="n">
         <v>6</v>
       </c>
+      <c r="AA25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2734,11 +2812,14 @@
         <v>0</v>
       </c>
       <c r="Y26" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Z26" t="n">
         <v>9</v>
       </c>
+      <c r="AA26" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2820,9 +2901,12 @@
         <v>0</v>
       </c>
       <c r="Y27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z27" t="n">
         <v>13</v>
       </c>
-      <c r="Z27" t="n">
+      <c r="AA27" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2906,9 +2990,12 @@
         <v>0</v>
       </c>
       <c r="Y28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2992,11 +3079,14 @@
         <v>0</v>
       </c>
       <c r="Y29" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Z29" t="n">
         <v>4</v>
       </c>
+      <c r="AA29" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3078,11 +3168,14 @@
         <v>0</v>
       </c>
       <c r="Y30" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Z30" t="n">
         <v>10</v>
       </c>
+      <c r="AA30" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3164,11 +3257,14 @@
         <v>0</v>
       </c>
       <c r="Y31" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Z31" t="n">
         <v>10</v>
       </c>
+      <c r="AA31" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3250,11 +3346,14 @@
         <v>0</v>
       </c>
       <c r="Y32" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Z32" t="n">
         <v>10</v>
       </c>
+      <c r="AA32" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3336,11 +3435,14 @@
         <v>0</v>
       </c>
       <c r="Y33" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z33" t="n">
         <v>11</v>
       </c>
+      <c r="AA33" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3422,11 +3524,14 @@
         <v>0</v>
       </c>
       <c r="Y34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z34" t="n">
         <v>6</v>
       </c>
+      <c r="AA34" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3508,11 +3613,14 @@
         <v>0</v>
       </c>
       <c r="Y35" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z35" t="n">
         <v>11</v>
       </c>
+      <c r="AA35" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3594,11 +3702,14 @@
         <v>0</v>
       </c>
       <c r="Y36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z36" t="n">
         <v>6</v>
       </c>
+      <c r="AA36" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3685,6 +3796,9 @@
       <c r="Z37" t="n">
         <v>0</v>
       </c>
+      <c r="AA37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3766,11 +3880,14 @@
         <v>0</v>
       </c>
       <c r="Y38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z38" t="n">
         <v>2</v>
       </c>
+      <c r="AA38" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3852,11 +3969,14 @@
         <v>0</v>
       </c>
       <c r="Y39" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z39" t="n">
         <v>12</v>
       </c>
+      <c r="AA39" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3938,11 +4058,14 @@
         <v>0</v>
       </c>
       <c r="Y40" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z40" t="n">
         <v>11</v>
       </c>
+      <c r="AA40" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4024,11 +4147,14 @@
         <v>0</v>
       </c>
       <c r="Y41" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Z41" t="n">
         <v>13</v>
       </c>
+      <c r="AA41" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4110,9 +4236,12 @@
         <v>0</v>
       </c>
       <c r="Y42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z42" t="n">
         <v>21</v>
       </c>
-      <c r="Z42" t="n">
+      <c r="AA42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4196,9 +4325,12 @@
         <v>0</v>
       </c>
       <c r="Y43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z43" t="n">
         <v>49</v>
       </c>
-      <c r="Z43" t="n">
+      <c r="AA43" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4282,11 +4414,14 @@
         <v>0</v>
       </c>
       <c r="Y44" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Z44" t="n">
         <v>10</v>
       </c>
+      <c r="AA44" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4368,11 +4503,14 @@
         <v>0</v>
       </c>
       <c r="Y45" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z45" t="n">
         <v>12</v>
       </c>
+      <c r="AA45" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4454,11 +4592,14 @@
         <v>0</v>
       </c>
       <c r="Y46" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Z46" t="n">
         <v>10</v>
       </c>
+      <c r="AA46" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4545,6 +4686,9 @@
       <c r="Z47" t="n">
         <v>0</v>
       </c>
+      <c r="AA47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4626,11 +4770,14 @@
         <v>0</v>
       </c>
       <c r="Y48" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z48" t="n">
         <v>12</v>
       </c>
+      <c r="AA48" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4712,11 +4859,14 @@
         <v>0</v>
       </c>
       <c r="Y49" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z49" t="n">
         <v>11</v>
       </c>
+      <c r="AA49" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4798,11 +4948,14 @@
         <v>0</v>
       </c>
       <c r="Y50" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z50" t="n">
         <v>6</v>
       </c>
+      <c r="AA50" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4884,11 +5037,14 @@
         <v>0</v>
       </c>
       <c r="Y51" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z51" t="n">
         <v>12</v>
       </c>
+      <c r="AA51" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4975,6 +5131,9 @@
       <c r="Z52" t="n">
         <v>0</v>
       </c>
+      <c r="AA52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5056,11 +5215,14 @@
         <v>0</v>
       </c>
       <c r="Y53" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Z53" t="n">
         <v>10</v>
       </c>
+      <c r="AA53" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5147,6 +5309,9 @@
       <c r="Z54" t="n">
         <v>0</v>
       </c>
+      <c r="AA54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5228,11 +5393,14 @@
         <v>0</v>
       </c>
       <c r="Y55" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z55" t="n">
         <v>11</v>
       </c>
+      <c r="AA55" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5314,11 +5482,14 @@
         <v>0</v>
       </c>
       <c r="Y56" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z56" t="n">
         <v>11</v>
       </c>
+      <c r="AA56" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5400,11 +5571,14 @@
         <v>0</v>
       </c>
       <c r="Y57" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z57" t="n">
         <v>7</v>
       </c>
+      <c r="AA57" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5486,11 +5660,14 @@
         <v>0</v>
       </c>
       <c r="Y58" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z58" t="n">
         <v>12</v>
       </c>
+      <c r="AA58" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5572,11 +5749,14 @@
         <v>0</v>
       </c>
       <c r="Y59" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z59" t="n">
         <v>3</v>
       </c>
+      <c r="AA59" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5663,6 +5843,9 @@
       <c r="Z60" t="n">
         <v>0</v>
       </c>
+      <c r="AA60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5744,11 +5927,14 @@
         <v>0</v>
       </c>
       <c r="Y61" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Z61" t="n">
         <v>9</v>
       </c>
+      <c r="AA61" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5830,11 +6016,14 @@
         <v>0</v>
       </c>
       <c r="Y62" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z62" t="n">
         <v>12</v>
       </c>
+      <c r="AA62" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5916,9 +6105,12 @@
         <v>0</v>
       </c>
       <c r="Y63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA63" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6007,6 +6199,9 @@
       <c r="Z64" t="n">
         <v>0</v>
       </c>
+      <c r="AA64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6088,11 +6283,14 @@
         <v>0</v>
       </c>
       <c r="Y65" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Z65" t="n">
         <v>5</v>
       </c>
+      <c r="AA65" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6174,9 +6372,12 @@
         <v>0</v>
       </c>
       <c r="Y66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6260,11 +6461,14 @@
         <v>0</v>
       </c>
       <c r="Y67" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Z67" t="n">
         <v>13</v>
       </c>
+      <c r="AA67" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6346,9 +6550,12 @@
         <v>0</v>
       </c>
       <c r="Y68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z68" t="n">
         <v>5</v>
       </c>
-      <c r="Z68" t="n">
+      <c r="AA68" t="n">
         <v>4</v>
       </c>
     </row>
@@ -6432,11 +6639,14 @@
         <v>0</v>
       </c>
       <c r="Y69" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z69" t="n">
         <v>7</v>
       </c>
+      <c r="AA69" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6518,9 +6728,12 @@
         <v>0</v>
       </c>
       <c r="Y70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z70" t="n">
         <v>21</v>
       </c>
-      <c r="Z70" t="n">
+      <c r="AA70" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6604,11 +6817,14 @@
         <v>0</v>
       </c>
       <c r="Y71" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z71" t="n">
         <v>6</v>
       </c>
+      <c r="AA71" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6690,11 +6906,14 @@
         <v>0</v>
       </c>
       <c r="Y72" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Z72" t="n">
         <v>10</v>
       </c>
+      <c r="AA72" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6781,6 +7000,9 @@
       <c r="Z73" t="n">
         <v>0</v>
       </c>
+      <c r="AA73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6867,6 +7089,9 @@
       <c r="Z74" t="n">
         <v>0</v>
       </c>
+      <c r="AA74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6948,11 +7173,14 @@
         <v>0</v>
       </c>
       <c r="Y75" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z75" t="n">
         <v>7</v>
       </c>
+      <c r="AA75" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7034,11 +7262,14 @@
         <v>0</v>
       </c>
       <c r="Y76" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Z76" t="n">
         <v>9</v>
       </c>
+      <c r="AA76" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7120,11 +7351,14 @@
         <v>0</v>
       </c>
       <c r="Y77" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z77" t="n">
         <v>11</v>
       </c>
+      <c r="AA77" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7206,11 +7440,14 @@
         <v>0</v>
       </c>
       <c r="Y78" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z78" t="n">
         <v>12</v>
       </c>
+      <c r="AA78" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7292,11 +7529,14 @@
         <v>0</v>
       </c>
       <c r="Y79" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Z79" t="n">
         <v>9</v>
       </c>
+      <c r="AA79" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7378,11 +7618,14 @@
         <v>0</v>
       </c>
       <c r="Y80" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z80" t="n">
         <v>3</v>
       </c>
+      <c r="AA80" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7464,9 +7707,12 @@
         <v>0</v>
       </c>
       <c r="Y81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA81" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7555,6 +7801,9 @@
       <c r="Z82" t="n">
         <v>0</v>
       </c>
+      <c r="AA82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7636,11 +7885,14 @@
         <v>0</v>
       </c>
       <c r="Y83" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Z83" t="n">
         <v>9</v>
       </c>
+      <c r="AA83" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7722,9 +7974,12 @@
         <v>0</v>
       </c>
       <c r="Y84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z84" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA84" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7808,11 +8063,14 @@
         <v>0</v>
       </c>
       <c r="Y85" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z85" t="n">
         <v>7</v>
       </c>
+      <c r="AA85" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7899,6 +8157,9 @@
       <c r="Z86" t="n">
         <v>0</v>
       </c>
+      <c r="AA86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7980,11 +8241,14 @@
         <v>0</v>
       </c>
       <c r="Y87" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z87" t="n">
         <v>7</v>
       </c>
+      <c r="AA87" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -8071,6 +8335,9 @@
       <c r="Z88" t="n">
         <v>0</v>
       </c>
+      <c r="AA88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -8152,11 +8419,14 @@
         <v>0</v>
       </c>
       <c r="Y89" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Z89" t="n">
         <v>9</v>
       </c>
+      <c r="AA89" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -8238,11 +8508,14 @@
         <v>0</v>
       </c>
       <c r="Y90" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Z90" t="n">
         <v>8</v>
       </c>
+      <c r="AA90" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -8324,9 +8597,12 @@
         <v>0</v>
       </c>
       <c r="Y91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z91" t="n">
         <v>37</v>
       </c>
-      <c r="Z91" t="n">
+      <c r="AA91" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8410,11 +8686,14 @@
         <v>0</v>
       </c>
       <c r="Y92" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Z92" t="n">
         <v>4</v>
       </c>
+      <c r="AA92" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -8501,6 +8780,9 @@
       <c r="Z93" t="n">
         <v>0</v>
       </c>
+      <c r="AA93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -8582,11 +8864,14 @@
         <v>0</v>
       </c>
       <c r="Y94" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z94" t="n">
         <v>6</v>
       </c>
+      <c r="AA94" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -8668,11 +8953,14 @@
         <v>0</v>
       </c>
       <c r="Y95" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Z95" t="n">
         <v>5</v>
       </c>
+      <c r="AA95" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -8754,11 +9042,14 @@
         <v>0</v>
       </c>
       <c r="Y96" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z96" t="n">
         <v>12</v>
       </c>
+      <c r="AA96" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -8845,6 +9136,9 @@
       <c r="Z97" t="n">
         <v>0</v>
       </c>
+      <c r="AA97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8926,11 +9220,14 @@
         <v>0</v>
       </c>
       <c r="Y98" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Z98" t="n">
         <v>13</v>
       </c>
+      <c r="AA98" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -9012,9 +9309,12 @@
         <v>0</v>
       </c>
       <c r="Y99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z99" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9103,6 +9403,9 @@
       <c r="Z100" t="n">
         <v>0</v>
       </c>
+      <c r="AA100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9184,11 +9487,14 @@
         <v>0</v>
       </c>
       <c r="Y101" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Z101" t="n">
         <v>12</v>
       </c>
+      <c r="AA101" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -9270,11 +9576,14 @@
         <v>0</v>
       </c>
       <c r="Y102" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z102" t="n">
         <v>11</v>
       </c>
+      <c r="AA102" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -9356,11 +9665,14 @@
         <v>0</v>
       </c>
       <c r="Y103" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="Z103" t="n">
         <v>11</v>
       </c>
+      <c r="AA103" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9442,11 +9754,14 @@
         <v>0</v>
       </c>
       <c r="Y104" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z104" t="n">
         <v>2</v>
       </c>
+      <c r="AA104" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9528,9 +9843,12 @@
         <v>0</v>
       </c>
       <c r="Y105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z105" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA105" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9614,9 +9932,12 @@
         <v>0</v>
       </c>
       <c r="Y106" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z106" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA106" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9700,9 +10021,12 @@
         <v>0</v>
       </c>
       <c r="Y107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA107" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9786,9 +10110,12 @@
         <v>0</v>
       </c>
       <c r="Y108" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z108" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA108" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9875,6 +10202,9 @@
         <v>0</v>
       </c>
       <c r="Z109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1911)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -455,8 +455,9 @@
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
-    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
     <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -585,12 +586,17 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -679,11 +685,14 @@
         <v>0</v>
       </c>
       <c r="Z2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="n">
         <v>9</v>
       </c>
+      <c r="AB2" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -768,11 +777,14 @@
         <v>0</v>
       </c>
       <c r="Z3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AA3" t="n">
         <v>7</v>
       </c>
+      <c r="AB3" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -857,11 +869,14 @@
         <v>0</v>
       </c>
       <c r="Z4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA4" t="n">
         <v>12</v>
       </c>
+      <c r="AB4" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -946,11 +961,14 @@
         <v>0</v>
       </c>
       <c r="Z5" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA5" t="n">
         <v>12</v>
       </c>
+      <c r="AB5" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1035,11 +1053,14 @@
         <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA6" t="n">
         <v>11</v>
       </c>
+      <c r="AB6" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1124,11 +1145,14 @@
         <v>0</v>
       </c>
       <c r="Z7" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA7" t="n">
         <v>10</v>
       </c>
+      <c r="AB7" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1213,11 +1237,14 @@
         <v>0</v>
       </c>
       <c r="Z8" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA8" t="n">
         <v>12</v>
       </c>
+      <c r="AB8" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1302,11 +1329,14 @@
         <v>0</v>
       </c>
       <c r="Z9" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AA9" t="n">
         <v>13</v>
       </c>
+      <c r="AB9" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1391,11 +1421,14 @@
         <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA10" t="n">
         <v>12</v>
       </c>
+      <c r="AB10" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1480,11 +1513,14 @@
         <v>0</v>
       </c>
       <c r="Z11" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA11" t="n">
         <v>11</v>
       </c>
+      <c r="AB11" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1569,11 +1605,14 @@
         <v>0</v>
       </c>
       <c r="Z12" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AA12" t="n">
         <v>13</v>
       </c>
+      <c r="AB12" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1658,11 +1697,14 @@
         <v>0</v>
       </c>
       <c r="Z13" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AA13" t="n">
         <v>7</v>
       </c>
+      <c r="AB13" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1747,11 +1789,14 @@
         <v>0</v>
       </c>
       <c r="Z14" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA14" t="n">
         <v>12</v>
       </c>
+      <c r="AB14" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1836,11 +1881,14 @@
         <v>0</v>
       </c>
       <c r="Z15" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AA15" t="n">
         <v>9</v>
       </c>
+      <c r="AB15" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1925,10 +1973,13 @@
         <v>0</v>
       </c>
       <c r="Z16" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AA16" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="17">
@@ -2014,11 +2065,14 @@
         <v>0</v>
       </c>
       <c r="Z17" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA17" t="n">
         <v>11</v>
       </c>
+      <c r="AB17" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2103,11 +2157,14 @@
         <v>0</v>
       </c>
       <c r="Z18" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA18" t="n">
         <v>11</v>
       </c>
+      <c r="AB18" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2197,6 +2254,9 @@
       <c r="AA19" t="n">
         <v>0</v>
       </c>
+      <c r="AB19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2281,11 +2341,14 @@
         <v>0</v>
       </c>
       <c r="Z20" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA20" t="n">
         <v>10</v>
       </c>
+      <c r="AB20" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2370,11 +2433,14 @@
         <v>0</v>
       </c>
       <c r="Z21" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA21" t="n">
         <v>11</v>
       </c>
+      <c r="AB21" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2464,6 +2530,9 @@
       <c r="AA22" t="n">
         <v>0</v>
       </c>
+      <c r="AB22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2548,11 +2617,14 @@
         <v>0</v>
       </c>
       <c r="Z23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA23" t="n">
         <v>6</v>
       </c>
+      <c r="AB23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2637,11 +2709,14 @@
         <v>0</v>
       </c>
       <c r="Z24" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA24" t="n">
         <v>11</v>
       </c>
+      <c r="AB24" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2726,11 +2801,14 @@
         <v>0</v>
       </c>
       <c r="Z25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA25" t="n">
         <v>6</v>
       </c>
+      <c r="AB25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2815,11 +2893,14 @@
         <v>0</v>
       </c>
       <c r="Z26" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AA26" t="n">
         <v>9</v>
       </c>
+      <c r="AB26" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2904,9 +2985,12 @@
         <v>0</v>
       </c>
       <c r="Z27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA27" t="n">
         <v>13</v>
       </c>
-      <c r="AA27" t="n">
+      <c r="AB27" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2993,9 +3077,12 @@
         <v>0</v>
       </c>
       <c r="Z28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3082,11 +3169,14 @@
         <v>0</v>
       </c>
       <c r="Z29" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AA29" t="n">
         <v>4</v>
       </c>
+      <c r="AB29" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3171,11 +3261,14 @@
         <v>0</v>
       </c>
       <c r="Z30" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA30" t="n">
         <v>10</v>
       </c>
+      <c r="AB30" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3260,11 +3353,14 @@
         <v>0</v>
       </c>
       <c r="Z31" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA31" t="n">
         <v>10</v>
       </c>
+      <c r="AB31" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3349,11 +3445,14 @@
         <v>0</v>
       </c>
       <c r="Z32" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA32" t="n">
         <v>10</v>
       </c>
+      <c r="AB32" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3438,11 +3537,14 @@
         <v>0</v>
       </c>
       <c r="Z33" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA33" t="n">
         <v>11</v>
       </c>
+      <c r="AB33" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3527,11 +3629,14 @@
         <v>0</v>
       </c>
       <c r="Z34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA34" t="n">
         <v>6</v>
       </c>
+      <c r="AB34" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3616,11 +3721,14 @@
         <v>0</v>
       </c>
       <c r="Z35" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA35" t="n">
         <v>11</v>
       </c>
+      <c r="AB35" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3705,11 +3813,14 @@
         <v>0</v>
       </c>
       <c r="Z36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA36" t="n">
         <v>6</v>
       </c>
+      <c r="AB36" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3799,6 +3910,9 @@
       <c r="AA37" t="n">
         <v>0</v>
       </c>
+      <c r="AB37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3883,11 +3997,14 @@
         <v>0</v>
       </c>
       <c r="Z38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA38" t="n">
         <v>2</v>
       </c>
+      <c r="AB38" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3972,11 +4089,14 @@
         <v>0</v>
       </c>
       <c r="Z39" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA39" t="n">
         <v>12</v>
       </c>
+      <c r="AB39" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4061,11 +4181,14 @@
         <v>0</v>
       </c>
       <c r="Z40" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA40" t="n">
         <v>11</v>
       </c>
+      <c r="AB40" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4150,11 +4273,14 @@
         <v>0</v>
       </c>
       <c r="Z41" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AA41" t="n">
         <v>13</v>
       </c>
+      <c r="AB41" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4239,9 +4365,12 @@
         <v>0</v>
       </c>
       <c r="Z42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA42" t="n">
         <v>21</v>
       </c>
-      <c r="AA42" t="n">
+      <c r="AB42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4328,9 +4457,12 @@
         <v>0</v>
       </c>
       <c r="Z43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA43" t="n">
         <v>49</v>
       </c>
-      <c r="AA43" t="n">
+      <c r="AB43" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4417,11 +4549,14 @@
         <v>0</v>
       </c>
       <c r="Z44" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA44" t="n">
         <v>10</v>
       </c>
+      <c r="AB44" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4506,11 +4641,14 @@
         <v>0</v>
       </c>
       <c r="Z45" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA45" t="n">
         <v>12</v>
       </c>
+      <c r="AB45" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4595,11 +4733,14 @@
         <v>0</v>
       </c>
       <c r="Z46" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA46" t="n">
         <v>10</v>
       </c>
+      <c r="AB46" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4689,6 +4830,9 @@
       <c r="AA47" t="n">
         <v>0</v>
       </c>
+      <c r="AB47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4773,11 +4917,14 @@
         <v>0</v>
       </c>
       <c r="Z48" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA48" t="n">
         <v>12</v>
       </c>
+      <c r="AB48" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4862,11 +5009,14 @@
         <v>0</v>
       </c>
       <c r="Z49" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA49" t="n">
         <v>11</v>
       </c>
+      <c r="AB49" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4951,11 +5101,14 @@
         <v>0</v>
       </c>
       <c r="Z50" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA50" t="n">
         <v>6</v>
       </c>
+      <c r="AB50" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5040,11 +5193,14 @@
         <v>0</v>
       </c>
       <c r="Z51" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA51" t="n">
         <v>12</v>
       </c>
+      <c r="AB51" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5134,6 +5290,9 @@
       <c r="AA52" t="n">
         <v>0</v>
       </c>
+      <c r="AB52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5218,11 +5377,14 @@
         <v>0</v>
       </c>
       <c r="Z53" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA53" t="n">
         <v>10</v>
       </c>
+      <c r="AB53" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5312,6 +5474,9 @@
       <c r="AA54" t="n">
         <v>0</v>
       </c>
+      <c r="AB54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5396,11 +5561,14 @@
         <v>0</v>
       </c>
       <c r="Z55" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA55" t="n">
         <v>11</v>
       </c>
+      <c r="AB55" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5485,11 +5653,14 @@
         <v>0</v>
       </c>
       <c r="Z56" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA56" t="n">
         <v>11</v>
       </c>
+      <c r="AB56" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5574,11 +5745,14 @@
         <v>0</v>
       </c>
       <c r="Z57" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AA57" t="n">
         <v>7</v>
       </c>
+      <c r="AB57" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5663,11 +5837,14 @@
         <v>0</v>
       </c>
       <c r="Z58" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA58" t="n">
         <v>12</v>
       </c>
+      <c r="AB58" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5752,11 +5929,14 @@
         <v>0</v>
       </c>
       <c r="Z59" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA59" t="n">
         <v>3</v>
       </c>
+      <c r="AB59" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5846,6 +6026,9 @@
       <c r="AA60" t="n">
         <v>0</v>
       </c>
+      <c r="AB60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5930,11 +6113,14 @@
         <v>0</v>
       </c>
       <c r="Z61" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AA61" t="n">
         <v>9</v>
       </c>
+      <c r="AB61" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6019,11 +6205,14 @@
         <v>0</v>
       </c>
       <c r="Z62" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA62" t="n">
         <v>12</v>
       </c>
+      <c r="AB62" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6108,9 +6297,12 @@
         <v>0</v>
       </c>
       <c r="Z63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB63" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6202,6 +6394,9 @@
       <c r="AA64" t="n">
         <v>0</v>
       </c>
+      <c r="AB64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6286,11 +6481,14 @@
         <v>0</v>
       </c>
       <c r="Z65" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA65" t="n">
         <v>5</v>
       </c>
+      <c r="AB65" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6375,9 +6573,12 @@
         <v>0</v>
       </c>
       <c r="Z66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6464,11 +6665,14 @@
         <v>0</v>
       </c>
       <c r="Z67" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AA67" t="n">
         <v>13</v>
       </c>
+      <c r="AB67" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6553,9 +6757,12 @@
         <v>0</v>
       </c>
       <c r="Z68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA68" t="n">
         <v>5</v>
       </c>
-      <c r="AA68" t="n">
+      <c r="AB68" t="n">
         <v>4</v>
       </c>
     </row>
@@ -6642,11 +6849,14 @@
         <v>0</v>
       </c>
       <c r="Z69" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AA69" t="n">
         <v>7</v>
       </c>
+      <c r="AB69" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6731,9 +6941,12 @@
         <v>0</v>
       </c>
       <c r="Z70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA70" t="n">
         <v>21</v>
       </c>
-      <c r="AA70" t="n">
+      <c r="AB70" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6820,11 +7033,14 @@
         <v>0</v>
       </c>
       <c r="Z71" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA71" t="n">
         <v>6</v>
       </c>
+      <c r="AB71" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6909,11 +7125,14 @@
         <v>0</v>
       </c>
       <c r="Z72" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA72" t="n">
         <v>10</v>
       </c>
+      <c r="AB72" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -7003,6 +7222,9 @@
       <c r="AA73" t="n">
         <v>0</v>
       </c>
+      <c r="AB73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7092,6 +7314,9 @@
       <c r="AA74" t="n">
         <v>0</v>
       </c>
+      <c r="AB74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7176,11 +7401,14 @@
         <v>0</v>
       </c>
       <c r="Z75" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AA75" t="n">
         <v>7</v>
       </c>
+      <c r="AB75" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7265,11 +7493,14 @@
         <v>0</v>
       </c>
       <c r="Z76" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AA76" t="n">
         <v>9</v>
       </c>
+      <c r="AB76" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7354,11 +7585,14 @@
         <v>0</v>
       </c>
       <c r="Z77" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA77" t="n">
         <v>11</v>
       </c>
+      <c r="AB77" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7443,11 +7677,14 @@
         <v>0</v>
       </c>
       <c r="Z78" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA78" t="n">
         <v>12</v>
       </c>
+      <c r="AB78" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7532,11 +7769,14 @@
         <v>0</v>
       </c>
       <c r="Z79" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AA79" t="n">
         <v>9</v>
       </c>
+      <c r="AB79" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7621,11 +7861,14 @@
         <v>0</v>
       </c>
       <c r="Z80" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA80" t="n">
         <v>3</v>
       </c>
+      <c r="AB80" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7710,9 +7953,12 @@
         <v>0</v>
       </c>
       <c r="Z81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB81" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7804,6 +8050,9 @@
       <c r="AA82" t="n">
         <v>0</v>
       </c>
+      <c r="AB82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7888,11 +8137,14 @@
         <v>0</v>
       </c>
       <c r="Z83" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AA83" t="n">
         <v>9</v>
       </c>
+      <c r="AB83" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7977,9 +8229,12 @@
         <v>0</v>
       </c>
       <c r="Z84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA84" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB84" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8066,11 +8321,14 @@
         <v>0</v>
       </c>
       <c r="Z85" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AA85" t="n">
         <v>7</v>
       </c>
+      <c r="AB85" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -8160,6 +8418,9 @@
       <c r="AA86" t="n">
         <v>0</v>
       </c>
+      <c r="AB86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8244,11 +8505,14 @@
         <v>0</v>
       </c>
       <c r="Z87" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AA87" t="n">
         <v>7</v>
       </c>
+      <c r="AB87" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -8338,6 +8602,9 @@
       <c r="AA88" t="n">
         <v>0</v>
       </c>
+      <c r="AB88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -8422,11 +8689,14 @@
         <v>0</v>
       </c>
       <c r="Z89" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AA89" t="n">
         <v>9</v>
       </c>
+      <c r="AB89" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -8511,11 +8781,14 @@
         <v>0</v>
       </c>
       <c r="Z90" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AA90" t="n">
         <v>8</v>
       </c>
+      <c r="AB90" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -8600,9 +8873,12 @@
         <v>0</v>
       </c>
       <c r="Z91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA91" t="n">
         <v>37</v>
       </c>
-      <c r="AA91" t="n">
+      <c r="AB91" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8689,11 +8965,14 @@
         <v>0</v>
       </c>
       <c r="Z92" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AA92" t="n">
         <v>4</v>
       </c>
+      <c r="AB92" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -8783,6 +9062,9 @@
       <c r="AA93" t="n">
         <v>0</v>
       </c>
+      <c r="AB93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -8867,11 +9149,14 @@
         <v>0</v>
       </c>
       <c r="Z94" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA94" t="n">
         <v>6</v>
       </c>
+      <c r="AB94" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -8956,11 +9241,14 @@
         <v>0</v>
       </c>
       <c r="Z95" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA95" t="n">
         <v>5</v>
       </c>
+      <c r="AB95" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -9045,11 +9333,14 @@
         <v>0</v>
       </c>
       <c r="Z96" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA96" t="n">
         <v>12</v>
       </c>
+      <c r="AB96" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -9139,6 +9430,9 @@
       <c r="AA97" t="n">
         <v>0</v>
       </c>
+      <c r="AB97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -9223,11 +9517,14 @@
         <v>0</v>
       </c>
       <c r="Z98" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AA98" t="n">
         <v>13</v>
       </c>
+      <c r="AB98" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -9312,9 +9609,12 @@
         <v>0</v>
       </c>
       <c r="Z99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA99" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9406,6 +9706,9 @@
       <c r="AA100" t="n">
         <v>0</v>
       </c>
+      <c r="AB100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9490,11 +9793,14 @@
         <v>0</v>
       </c>
       <c r="Z101" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AA101" t="n">
         <v>12</v>
       </c>
+      <c r="AB101" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -9579,11 +9885,14 @@
         <v>0</v>
       </c>
       <c r="Z102" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA102" t="n">
         <v>11</v>
       </c>
+      <c r="AB102" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -9668,11 +9977,14 @@
         <v>0</v>
       </c>
       <c r="Z103" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA103" t="n">
         <v>11</v>
       </c>
+      <c r="AB103" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9757,11 +10069,14 @@
         <v>0</v>
       </c>
       <c r="Z104" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA104" t="n">
         <v>2</v>
       </c>
+      <c r="AB104" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9846,9 +10161,12 @@
         <v>0</v>
       </c>
       <c r="Z105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA105" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB105" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9935,9 +10253,12 @@
         <v>0</v>
       </c>
       <c r="Z106" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA106" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB106" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10024,9 +10345,12 @@
         <v>0</v>
       </c>
       <c r="Z107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB107" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10113,9 +10437,12 @@
         <v>0</v>
       </c>
       <c r="Z108" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA108" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB108" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10205,6 +10532,9 @@
         <v>0</v>
       </c>
       <c r="AA109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1921)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB109"/>
+  <dimension ref="A1:AC109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -456,8 +456,9 @@
     <col width="12" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
     <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -591,12 +592,17 @@
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -688,9 +694,12 @@
         <v>0</v>
       </c>
       <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
         <v>9</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AC2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -780,9 +789,12 @@
         <v>0</v>
       </c>
       <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="n">
         <v>7</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -872,9 +884,12 @@
         <v>0</v>
       </c>
       <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="n">
         <v>12</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AC4" t="n">
         <v>12</v>
       </c>
     </row>
@@ -964,9 +979,12 @@
         <v>0</v>
       </c>
       <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="n">
         <v>12</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AC5" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1056,9 +1074,12 @@
         <v>0</v>
       </c>
       <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="n">
         <v>11</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AC6" t="n">
         <v>11</v>
       </c>
     </row>
@@ -1148,9 +1169,12 @@
         <v>0</v>
       </c>
       <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="n">
         <v>10</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AC7" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1240,9 +1264,12 @@
         <v>0</v>
       </c>
       <c r="AA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="n">
         <v>12</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AC8" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1332,9 +1359,12 @@
         <v>0</v>
       </c>
       <c r="AA9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="n">
         <v>13</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AC9" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1424,9 +1454,12 @@
         <v>0</v>
       </c>
       <c r="AA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="n">
         <v>12</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AC10" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1516,9 +1549,12 @@
         <v>0</v>
       </c>
       <c r="AA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="n">
         <v>11</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AC11" t="n">
         <v>11</v>
       </c>
     </row>
@@ -1608,9 +1644,12 @@
         <v>0</v>
       </c>
       <c r="AA12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="n">
         <v>13</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AC12" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1700,9 +1739,12 @@
         <v>0</v>
       </c>
       <c r="AA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="n">
         <v>7</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AC13" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1792,9 +1834,12 @@
         <v>0</v>
       </c>
       <c r="AA14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="n">
         <v>12</v>
       </c>
-      <c r="AB14" t="n">
+      <c r="AC14" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1884,9 +1929,12 @@
         <v>0</v>
       </c>
       <c r="AA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" t="n">
         <v>9</v>
       </c>
-      <c r="AB15" t="n">
+      <c r="AC15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1976,9 +2024,12 @@
         <v>1</v>
       </c>
       <c r="AA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="n">
         <v>11</v>
       </c>
-      <c r="AB16" t="n">
+      <c r="AC16" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2068,9 +2119,12 @@
         <v>0</v>
       </c>
       <c r="AA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="n">
         <v>11</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AC17" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2160,9 +2214,12 @@
         <v>0</v>
       </c>
       <c r="AA18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB18" t="n">
         <v>11</v>
       </c>
-      <c r="AB18" t="n">
+      <c r="AC18" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2257,6 +2314,9 @@
       <c r="AB19" t="n">
         <v>0</v>
       </c>
+      <c r="AC19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2344,9 +2404,12 @@
         <v>0</v>
       </c>
       <c r="AA20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB20" t="n">
         <v>10</v>
       </c>
-      <c r="AB20" t="n">
+      <c r="AC20" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2436,9 +2499,12 @@
         <v>0</v>
       </c>
       <c r="AA21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB21" t="n">
         <v>11</v>
       </c>
-      <c r="AB21" t="n">
+      <c r="AC21" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2533,6 +2599,9 @@
       <c r="AB22" t="n">
         <v>0</v>
       </c>
+      <c r="AC22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2620,9 +2689,12 @@
         <v>0</v>
       </c>
       <c r="AA23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB23" t="n">
         <v>6</v>
       </c>
-      <c r="AB23" t="n">
+      <c r="AC23" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2712,9 +2784,12 @@
         <v>0</v>
       </c>
       <c r="AA24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB24" t="n">
         <v>11</v>
       </c>
-      <c r="AB24" t="n">
+      <c r="AC24" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2804,9 +2879,12 @@
         <v>0</v>
       </c>
       <c r="AA25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB25" t="n">
         <v>6</v>
       </c>
-      <c r="AB25" t="n">
+      <c r="AC25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2896,9 +2974,12 @@
         <v>0</v>
       </c>
       <c r="AA26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB26" t="n">
         <v>9</v>
       </c>
-      <c r="AB26" t="n">
+      <c r="AC26" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2988,9 +3069,12 @@
         <v>0</v>
       </c>
       <c r="AA27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB27" t="n">
         <v>13</v>
       </c>
-      <c r="AB27" t="n">
+      <c r="AC27" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3080,9 +3164,12 @@
         <v>0</v>
       </c>
       <c r="AA28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3172,9 +3259,12 @@
         <v>0</v>
       </c>
       <c r="AA29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB29" t="n">
         <v>4</v>
       </c>
-      <c r="AB29" t="n">
+      <c r="AC29" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3264,9 +3354,12 @@
         <v>0</v>
       </c>
       <c r="AA30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB30" t="n">
         <v>10</v>
       </c>
-      <c r="AB30" t="n">
+      <c r="AC30" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3356,9 +3449,12 @@
         <v>0</v>
       </c>
       <c r="AA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB31" t="n">
         <v>10</v>
       </c>
-      <c r="AB31" t="n">
+      <c r="AC31" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3448,9 +3544,12 @@
         <v>0</v>
       </c>
       <c r="AA32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB32" t="n">
         <v>10</v>
       </c>
-      <c r="AB32" t="n">
+      <c r="AC32" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3540,9 +3639,12 @@
         <v>0</v>
       </c>
       <c r="AA33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB33" t="n">
         <v>11</v>
       </c>
-      <c r="AB33" t="n">
+      <c r="AC33" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3632,9 +3734,12 @@
         <v>0</v>
       </c>
       <c r="AA34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB34" t="n">
         <v>6</v>
       </c>
-      <c r="AB34" t="n">
+      <c r="AC34" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3724,9 +3829,12 @@
         <v>0</v>
       </c>
       <c r="AA35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB35" t="n">
         <v>11</v>
       </c>
-      <c r="AB35" t="n">
+      <c r="AC35" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3816,9 +3924,12 @@
         <v>0</v>
       </c>
       <c r="AA36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB36" t="n">
         <v>6</v>
       </c>
-      <c r="AB36" t="n">
+      <c r="AC36" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3913,6 +4024,9 @@
       <c r="AB37" t="n">
         <v>0</v>
       </c>
+      <c r="AC37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4000,9 +4114,12 @@
         <v>0</v>
       </c>
       <c r="AA38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB38" t="n">
         <v>2</v>
       </c>
-      <c r="AB38" t="n">
+      <c r="AC38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4092,9 +4209,12 @@
         <v>0</v>
       </c>
       <c r="AA39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB39" t="n">
         <v>12</v>
       </c>
-      <c r="AB39" t="n">
+      <c r="AC39" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4184,9 +4304,12 @@
         <v>0</v>
       </c>
       <c r="AA40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB40" t="n">
         <v>11</v>
       </c>
-      <c r="AB40" t="n">
+      <c r="AC40" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4276,9 +4399,12 @@
         <v>0</v>
       </c>
       <c r="AA41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB41" t="n">
         <v>13</v>
       </c>
-      <c r="AB41" t="n">
+      <c r="AC41" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4368,9 +4494,12 @@
         <v>0</v>
       </c>
       <c r="AA42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB42" t="n">
         <v>21</v>
       </c>
-      <c r="AB42" t="n">
+      <c r="AC42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4460,9 +4589,12 @@
         <v>0</v>
       </c>
       <c r="AA43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB43" t="n">
         <v>49</v>
       </c>
-      <c r="AB43" t="n">
+      <c r="AC43" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4552,9 +4684,12 @@
         <v>0</v>
       </c>
       <c r="AA44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB44" t="n">
         <v>10</v>
       </c>
-      <c r="AB44" t="n">
+      <c r="AC44" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4644,9 +4779,12 @@
         <v>0</v>
       </c>
       <c r="AA45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB45" t="n">
         <v>12</v>
       </c>
-      <c r="AB45" t="n">
+      <c r="AC45" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4736,9 +4874,12 @@
         <v>0</v>
       </c>
       <c r="AA46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB46" t="n">
         <v>10</v>
       </c>
-      <c r="AB46" t="n">
+      <c r="AC46" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4833,6 +4974,9 @@
       <c r="AB47" t="n">
         <v>0</v>
       </c>
+      <c r="AC47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4920,9 +5064,12 @@
         <v>0</v>
       </c>
       <c r="AA48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB48" t="n">
         <v>12</v>
       </c>
-      <c r="AB48" t="n">
+      <c r="AC48" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5012,9 +5159,12 @@
         <v>0</v>
       </c>
       <c r="AA49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB49" t="n">
         <v>11</v>
       </c>
-      <c r="AB49" t="n">
+      <c r="AC49" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5104,9 +5254,12 @@
         <v>0</v>
       </c>
       <c r="AA50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB50" t="n">
         <v>6</v>
       </c>
-      <c r="AB50" t="n">
+      <c r="AC50" t="n">
         <v>6</v>
       </c>
     </row>
@@ -5196,9 +5349,12 @@
         <v>0</v>
       </c>
       <c r="AA51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB51" t="n">
         <v>12</v>
       </c>
-      <c r="AB51" t="n">
+      <c r="AC51" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5293,6 +5449,9 @@
       <c r="AB52" t="n">
         <v>0</v>
       </c>
+      <c r="AC52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5380,9 +5539,12 @@
         <v>0</v>
       </c>
       <c r="AA53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB53" t="n">
         <v>10</v>
       </c>
-      <c r="AB53" t="n">
+      <c r="AC53" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5477,6 +5639,9 @@
       <c r="AB54" t="n">
         <v>0</v>
       </c>
+      <c r="AC54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5564,9 +5729,12 @@
         <v>0</v>
       </c>
       <c r="AA55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB55" t="n">
         <v>11</v>
       </c>
-      <c r="AB55" t="n">
+      <c r="AC55" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5656,9 +5824,12 @@
         <v>0</v>
       </c>
       <c r="AA56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB56" t="n">
         <v>11</v>
       </c>
-      <c r="AB56" t="n">
+      <c r="AC56" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5748,9 +5919,12 @@
         <v>0</v>
       </c>
       <c r="AA57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB57" t="n">
         <v>7</v>
       </c>
-      <c r="AB57" t="n">
+      <c r="AC57" t="n">
         <v>7</v>
       </c>
     </row>
@@ -5840,9 +6014,12 @@
         <v>0</v>
       </c>
       <c r="AA58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB58" t="n">
         <v>12</v>
       </c>
-      <c r="AB58" t="n">
+      <c r="AC58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5932,9 +6109,12 @@
         <v>0</v>
       </c>
       <c r="AA59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB59" t="n">
         <v>3</v>
       </c>
-      <c r="AB59" t="n">
+      <c r="AC59" t="n">
         <v>3</v>
       </c>
     </row>
@@ -6029,6 +6209,9 @@
       <c r="AB60" t="n">
         <v>0</v>
       </c>
+      <c r="AC60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6116,9 +6299,12 @@
         <v>0</v>
       </c>
       <c r="AA61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB61" t="n">
         <v>9</v>
       </c>
-      <c r="AB61" t="n">
+      <c r="AC61" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6208,9 +6394,12 @@
         <v>0</v>
       </c>
       <c r="AA62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB62" t="n">
         <v>12</v>
       </c>
-      <c r="AB62" t="n">
+      <c r="AC62" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6300,9 +6489,12 @@
         <v>0</v>
       </c>
       <c r="AA63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC63" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6397,6 +6589,9 @@
       <c r="AB64" t="n">
         <v>0</v>
       </c>
+      <c r="AC64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6484,9 +6679,12 @@
         <v>0</v>
       </c>
       <c r="AA65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB65" t="n">
         <v>5</v>
       </c>
-      <c r="AB65" t="n">
+      <c r="AC65" t="n">
         <v>5</v>
       </c>
     </row>
@@ -6576,9 +6774,12 @@
         <v>0</v>
       </c>
       <c r="AA66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6668,9 +6869,12 @@
         <v>0</v>
       </c>
       <c r="AA67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB67" t="n">
         <v>13</v>
       </c>
-      <c r="AB67" t="n">
+      <c r="AC67" t="n">
         <v>13</v>
       </c>
     </row>
@@ -6760,9 +6964,12 @@
         <v>0</v>
       </c>
       <c r="AA68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB68" t="n">
         <v>5</v>
       </c>
-      <c r="AB68" t="n">
+      <c r="AC68" t="n">
         <v>4</v>
       </c>
     </row>
@@ -6852,9 +7059,12 @@
         <v>0</v>
       </c>
       <c r="AA69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB69" t="n">
         <v>7</v>
       </c>
-      <c r="AB69" t="n">
+      <c r="AC69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6944,9 +7154,12 @@
         <v>0</v>
       </c>
       <c r="AA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB70" t="n">
         <v>21</v>
       </c>
-      <c r="AB70" t="n">
+      <c r="AC70" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7036,9 +7249,12 @@
         <v>0</v>
       </c>
       <c r="AA71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB71" t="n">
         <v>6</v>
       </c>
-      <c r="AB71" t="n">
+      <c r="AC71" t="n">
         <v>6</v>
       </c>
     </row>
@@ -7128,9 +7344,12 @@
         <v>0</v>
       </c>
       <c r="AA72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB72" t="n">
         <v>10</v>
       </c>
-      <c r="AB72" t="n">
+      <c r="AC72" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7225,6 +7444,9 @@
       <c r="AB73" t="n">
         <v>0</v>
       </c>
+      <c r="AC73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7317,6 +7539,9 @@
       <c r="AB74" t="n">
         <v>0</v>
       </c>
+      <c r="AC74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7404,9 +7629,12 @@
         <v>0</v>
       </c>
       <c r="AA75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB75" t="n">
         <v>7</v>
       </c>
-      <c r="AB75" t="n">
+      <c r="AC75" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7496,9 +7724,12 @@
         <v>0</v>
       </c>
       <c r="AA76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB76" t="n">
         <v>9</v>
       </c>
-      <c r="AB76" t="n">
+      <c r="AC76" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7588,9 +7819,12 @@
         <v>0</v>
       </c>
       <c r="AA77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB77" t="n">
         <v>11</v>
       </c>
-      <c r="AB77" t="n">
+      <c r="AC77" t="n">
         <v>11</v>
       </c>
     </row>
@@ -7680,9 +7914,12 @@
         <v>0</v>
       </c>
       <c r="AA78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB78" t="n">
         <v>12</v>
       </c>
-      <c r="AB78" t="n">
+      <c r="AC78" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7772,9 +8009,12 @@
         <v>0</v>
       </c>
       <c r="AA79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB79" t="n">
         <v>9</v>
       </c>
-      <c r="AB79" t="n">
+      <c r="AC79" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7864,9 +8104,12 @@
         <v>0</v>
       </c>
       <c r="AA80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB80" t="n">
         <v>3</v>
       </c>
-      <c r="AB80" t="n">
+      <c r="AC80" t="n">
         <v>3</v>
       </c>
     </row>
@@ -7956,9 +8199,12 @@
         <v>0</v>
       </c>
       <c r="AA81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC81" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8053,6 +8299,9 @@
       <c r="AB82" t="n">
         <v>0</v>
       </c>
+      <c r="AC82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8140,9 +8389,12 @@
         <v>0</v>
       </c>
       <c r="AA83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB83" t="n">
         <v>9</v>
       </c>
-      <c r="AB83" t="n">
+      <c r="AC83" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8232,9 +8484,12 @@
         <v>0</v>
       </c>
       <c r="AA84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB84" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC84" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8324,9 +8579,12 @@
         <v>0</v>
       </c>
       <c r="AA85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB85" t="n">
         <v>7</v>
       </c>
-      <c r="AB85" t="n">
+      <c r="AC85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8421,6 +8679,9 @@
       <c r="AB86" t="n">
         <v>0</v>
       </c>
+      <c r="AC86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8508,9 +8769,12 @@
         <v>0</v>
       </c>
       <c r="AA87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB87" t="n">
         <v>7</v>
       </c>
-      <c r="AB87" t="n">
+      <c r="AC87" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8605,6 +8869,9 @@
       <c r="AB88" t="n">
         <v>0</v>
       </c>
+      <c r="AC88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -8692,9 +8959,12 @@
         <v>0</v>
       </c>
       <c r="AA89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB89" t="n">
         <v>9</v>
       </c>
-      <c r="AB89" t="n">
+      <c r="AC89" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8784,9 +9054,12 @@
         <v>0</v>
       </c>
       <c r="AA90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB90" t="n">
         <v>8</v>
       </c>
-      <c r="AB90" t="n">
+      <c r="AC90" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8876,9 +9149,12 @@
         <v>0</v>
       </c>
       <c r="AA91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB91" t="n">
         <v>37</v>
       </c>
-      <c r="AB91" t="n">
+      <c r="AC91" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8968,9 +9244,12 @@
         <v>0</v>
       </c>
       <c r="AA92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB92" t="n">
         <v>4</v>
       </c>
-      <c r="AB92" t="n">
+      <c r="AC92" t="n">
         <v>4</v>
       </c>
     </row>
@@ -9065,6 +9344,9 @@
       <c r="AB93" t="n">
         <v>0</v>
       </c>
+      <c r="AC93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -9152,9 +9434,12 @@
         <v>0</v>
       </c>
       <c r="AA94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB94" t="n">
         <v>6</v>
       </c>
-      <c r="AB94" t="n">
+      <c r="AC94" t="n">
         <v>6</v>
       </c>
     </row>
@@ -9244,9 +9529,12 @@
         <v>0</v>
       </c>
       <c r="AA95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB95" t="n">
         <v>5</v>
       </c>
-      <c r="AB95" t="n">
+      <c r="AC95" t="n">
         <v>5</v>
       </c>
     </row>
@@ -9336,9 +9624,12 @@
         <v>0</v>
       </c>
       <c r="AA96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB96" t="n">
         <v>12</v>
       </c>
-      <c r="AB96" t="n">
+      <c r="AC96" t="n">
         <v>12</v>
       </c>
     </row>
@@ -9433,6 +9724,9 @@
       <c r="AB97" t="n">
         <v>0</v>
       </c>
+      <c r="AC97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -9520,9 +9814,12 @@
         <v>0</v>
       </c>
       <c r="AA98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB98" t="n">
         <v>13</v>
       </c>
-      <c r="AB98" t="n">
+      <c r="AC98" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9612,9 +9909,12 @@
         <v>0</v>
       </c>
       <c r="AA99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB99" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9709,6 +10009,9 @@
       <c r="AB100" t="n">
         <v>0</v>
       </c>
+      <c r="AC100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9796,9 +10099,12 @@
         <v>0</v>
       </c>
       <c r="AA101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB101" t="n">
         <v>12</v>
       </c>
-      <c r="AB101" t="n">
+      <c r="AC101" t="n">
         <v>12</v>
       </c>
     </row>
@@ -9888,9 +10194,12 @@
         <v>0</v>
       </c>
       <c r="AA102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB102" t="n">
         <v>11</v>
       </c>
-      <c r="AB102" t="n">
+      <c r="AC102" t="n">
         <v>11</v>
       </c>
     </row>
@@ -9980,9 +10289,12 @@
         <v>0</v>
       </c>
       <c r="AA103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB103" t="n">
         <v>11</v>
       </c>
-      <c r="AB103" t="n">
+      <c r="AC103" t="n">
         <v>11</v>
       </c>
     </row>
@@ -10072,9 +10384,12 @@
         <v>0</v>
       </c>
       <c r="AA104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB104" t="n">
         <v>2</v>
       </c>
-      <c r="AB104" t="n">
+      <c r="AC104" t="n">
         <v>2</v>
       </c>
     </row>
@@ -10164,9 +10479,12 @@
         <v>0</v>
       </c>
       <c r="AA105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB105" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC105" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10256,9 +10574,12 @@
         <v>0</v>
       </c>
       <c r="AA106" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB106" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC106" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10348,9 +10669,12 @@
         <v>0</v>
       </c>
       <c r="AA107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC107" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10440,9 +10764,12 @@
         <v>0</v>
       </c>
       <c r="AA108" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB108" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC108" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10535,6 +10862,9 @@
         <v>0</v>
       </c>
       <c r="AB109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#1988)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC109"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -457,8 +457,9 @@
     <col width="12" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
-    <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
     <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -597,12 +598,17 @@
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -697,9 +703,12 @@
         <v>0</v>
       </c>
       <c r="AB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="n">
         <v>9</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -792,9 +801,12 @@
         <v>0</v>
       </c>
       <c r="AB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="n">
         <v>7</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -887,10 +899,13 @@
         <v>0</v>
       </c>
       <c r="AB4" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC4" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -982,10 +997,13 @@
         <v>0</v>
       </c>
       <c r="AB5" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC5" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -1077,10 +1095,13 @@
         <v>0</v>
       </c>
       <c r="AB6" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC6" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -1172,9 +1193,12 @@
         <v>0</v>
       </c>
       <c r="AB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="n">
         <v>10</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AD7" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1267,10 +1291,13 @@
         <v>0</v>
       </c>
       <c r="AB8" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC8" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="9">
@@ -1362,10 +1389,13 @@
         <v>0</v>
       </c>
       <c r="AB9" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AC9" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -1457,10 +1487,13 @@
         <v>0</v>
       </c>
       <c r="AB10" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC10" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="11">
@@ -1552,10 +1585,13 @@
         <v>0</v>
       </c>
       <c r="AB11" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC11" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="12">
@@ -1647,10 +1683,13 @@
         <v>0</v>
       </c>
       <c r="AB12" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AC12" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -1742,10 +1781,13 @@
         <v>0</v>
       </c>
       <c r="AB13" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AC13" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -1837,10 +1879,13 @@
         <v>0</v>
       </c>
       <c r="AB14" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC14" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="15">
@@ -1932,9 +1977,12 @@
         <v>0</v>
       </c>
       <c r="AB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" t="n">
         <v>9</v>
       </c>
-      <c r="AC15" t="n">
+      <c r="AD15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2027,9 +2075,12 @@
         <v>0</v>
       </c>
       <c r="AB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" t="n">
         <v>11</v>
       </c>
-      <c r="AC16" t="n">
+      <c r="AD16" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2122,9 +2173,12 @@
         <v>0</v>
       </c>
       <c r="AB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" t="n">
         <v>11</v>
       </c>
-      <c r="AC17" t="n">
+      <c r="AD17" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2217,10 +2271,13 @@
         <v>0</v>
       </c>
       <c r="AB18" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC18" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="19">
@@ -2317,6 +2374,9 @@
       <c r="AC19" t="n">
         <v>0</v>
       </c>
+      <c r="AD19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2407,10 +2467,13 @@
         <v>0</v>
       </c>
       <c r="AB20" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AC20" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="21">
@@ -2502,10 +2565,13 @@
         <v>0</v>
       </c>
       <c r="AB21" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC21" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="22">
@@ -2602,6 +2668,9 @@
       <c r="AC22" t="n">
         <v>0</v>
       </c>
+      <c r="AD22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2692,10 +2761,13 @@
         <v>0</v>
       </c>
       <c r="AB23" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AC23" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="24">
@@ -2787,10 +2859,13 @@
         <v>0</v>
       </c>
       <c r="AB24" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC24" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="25">
@@ -2882,9 +2957,12 @@
         <v>0</v>
       </c>
       <c r="AB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" t="n">
         <v>6</v>
       </c>
-      <c r="AC25" t="n">
+      <c r="AD25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2977,10 +3055,13 @@
         <v>0</v>
       </c>
       <c r="AB26" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AC26" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="27">
@@ -3072,10 +3153,13 @@
         <v>0</v>
       </c>
       <c r="AB27" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AC27" t="n">
-        <v>11</v>
+        <v>14</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="28">
@@ -3170,7 +3254,10 @@
         <v>1</v>
       </c>
       <c r="AC28" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -3262,9 +3349,12 @@
         <v>0</v>
       </c>
       <c r="AB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC29" t="n">
         <v>4</v>
       </c>
-      <c r="AC29" t="n">
+      <c r="AD29" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3357,9 +3447,12 @@
         <v>0</v>
       </c>
       <c r="AB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC30" t="n">
         <v>10</v>
       </c>
-      <c r="AC30" t="n">
+      <c r="AD30" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3452,10 +3545,13 @@
         <v>0</v>
       </c>
       <c r="AB31" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AC31" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="32">
@@ -3547,9 +3643,12 @@
         <v>0</v>
       </c>
       <c r="AB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC32" t="n">
         <v>10</v>
       </c>
-      <c r="AC32" t="n">
+      <c r="AD32" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3642,9 +3741,12 @@
         <v>0</v>
       </c>
       <c r="AB33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC33" t="n">
         <v>11</v>
       </c>
-      <c r="AC33" t="n">
+      <c r="AD33" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3737,9 +3839,12 @@
         <v>0</v>
       </c>
       <c r="AB34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC34" t="n">
         <v>6</v>
       </c>
-      <c r="AC34" t="n">
+      <c r="AD34" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3832,9 +3937,12 @@
         <v>0</v>
       </c>
       <c r="AB35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC35" t="n">
         <v>11</v>
       </c>
-      <c r="AC35" t="n">
+      <c r="AD35" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3927,9 +4035,12 @@
         <v>0</v>
       </c>
       <c r="AB36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC36" t="n">
         <v>6</v>
       </c>
-      <c r="AC36" t="n">
+      <c r="AD36" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4027,6 +4138,9 @@
       <c r="AC37" t="n">
         <v>0</v>
       </c>
+      <c r="AD37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4117,9 +4231,12 @@
         <v>0</v>
       </c>
       <c r="AB38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC38" t="n">
         <v>2</v>
       </c>
-      <c r="AC38" t="n">
+      <c r="AD38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4212,10 +4329,13 @@
         <v>0</v>
       </c>
       <c r="AB39" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC39" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="40">
@@ -4307,10 +4427,13 @@
         <v>0</v>
       </c>
       <c r="AB40" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC40" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AD40" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="41">
@@ -4402,10 +4525,13 @@
         <v>0</v>
       </c>
       <c r="AB41" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AC41" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AD41" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="42">
@@ -4497,9 +4623,12 @@
         <v>0</v>
       </c>
       <c r="AB42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC42" t="n">
         <v>21</v>
       </c>
-      <c r="AC42" t="n">
+      <c r="AD42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4592,9 +4721,12 @@
         <v>0</v>
       </c>
       <c r="AB43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC43" t="n">
         <v>49</v>
       </c>
-      <c r="AC43" t="n">
+      <c r="AD43" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4687,10 +4819,13 @@
         <v>0</v>
       </c>
       <c r="AB44" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AC44" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AD44" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="45">
@@ -4782,10 +4917,13 @@
         <v>0</v>
       </c>
       <c r="AB45" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC45" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="46">
@@ -4877,10 +5015,13 @@
         <v>0</v>
       </c>
       <c r="AB46" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AC46" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AD46" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="47">
@@ -4977,6 +5118,9 @@
       <c r="AC47" t="n">
         <v>0</v>
       </c>
+      <c r="AD47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5067,10 +5211,13 @@
         <v>0</v>
       </c>
       <c r="AB48" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC48" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD48" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="49">
@@ -5162,10 +5309,13 @@
         <v>0</v>
       </c>
       <c r="AB49" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC49" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AD49" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="50">
@@ -5257,9 +5407,12 @@
         <v>0</v>
       </c>
       <c r="AB50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC50" t="n">
         <v>6</v>
       </c>
-      <c r="AC50" t="n">
+      <c r="AD50" t="n">
         <v>6</v>
       </c>
     </row>
@@ -5352,10 +5505,13 @@
         <v>0</v>
       </c>
       <c r="AB51" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC51" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD51" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="52">
@@ -5452,6 +5608,9 @@
       <c r="AC52" t="n">
         <v>0</v>
       </c>
+      <c r="AD52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5542,10 +5701,13 @@
         <v>0</v>
       </c>
       <c r="AB53" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AC53" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AD53" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="54">
@@ -5642,6 +5804,9 @@
       <c r="AC54" t="n">
         <v>0</v>
       </c>
+      <c r="AD54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5732,10 +5897,13 @@
         <v>0</v>
       </c>
       <c r="AB55" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC55" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AD55" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="56">
@@ -5827,9 +5995,12 @@
         <v>0</v>
       </c>
       <c r="AB56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC56" t="n">
         <v>11</v>
       </c>
-      <c r="AC56" t="n">
+      <c r="AD56" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5922,9 +6093,12 @@
         <v>0</v>
       </c>
       <c r="AB57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC57" t="n">
         <v>7</v>
       </c>
-      <c r="AC57" t="n">
+      <c r="AD57" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6017,9 +6191,12 @@
         <v>0</v>
       </c>
       <c r="AB58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC58" t="n">
         <v>12</v>
       </c>
-      <c r="AC58" t="n">
+      <c r="AD58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6112,9 +6289,12 @@
         <v>0</v>
       </c>
       <c r="AB59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC59" t="n">
         <v>3</v>
       </c>
-      <c r="AC59" t="n">
+      <c r="AD59" t="n">
         <v>3</v>
       </c>
     </row>
@@ -6212,6 +6392,9 @@
       <c r="AC60" t="n">
         <v>0</v>
       </c>
+      <c r="AD60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6302,10 +6485,13 @@
         <v>0</v>
       </c>
       <c r="AB61" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AC61" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AD61" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="62">
@@ -6397,10 +6583,13 @@
         <v>0</v>
       </c>
       <c r="AB62" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC62" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD62" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="63">
@@ -6495,7 +6684,10 @@
         <v>1</v>
       </c>
       <c r="AC63" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AD63" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="64">
@@ -6592,6 +6784,9 @@
       <c r="AC64" t="n">
         <v>0</v>
       </c>
+      <c r="AD64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6682,9 +6877,12 @@
         <v>0</v>
       </c>
       <c r="AB65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC65" t="n">
         <v>5</v>
       </c>
-      <c r="AC65" t="n">
+      <c r="AD65" t="n">
         <v>5</v>
       </c>
     </row>
@@ -6777,9 +6975,12 @@
         <v>0</v>
       </c>
       <c r="AB66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6872,10 +7073,13 @@
         <v>0</v>
       </c>
       <c r="AB67" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AC67" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AD67" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="68">
@@ -6967,10 +7171,13 @@
         <v>0</v>
       </c>
       <c r="AB68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC68" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD68" t="n">
         <v>5</v>
-      </c>
-      <c r="AC68" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="69">
@@ -7062,9 +7269,12 @@
         <v>0</v>
       </c>
       <c r="AB69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC69" t="n">
         <v>7</v>
       </c>
-      <c r="AC69" t="n">
+      <c r="AD69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7157,9 +7367,12 @@
         <v>0</v>
       </c>
       <c r="AB70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC70" t="n">
         <v>21</v>
       </c>
-      <c r="AC70" t="n">
+      <c r="AD70" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7252,10 +7465,13 @@
         <v>0</v>
       </c>
       <c r="AB71" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AC71" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AD71" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="72">
@@ -7347,10 +7563,13 @@
         <v>0</v>
       </c>
       <c r="AB72" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AC72" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AD72" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="73">
@@ -7447,6 +7666,9 @@
       <c r="AC73" t="n">
         <v>0</v>
       </c>
+      <c r="AD73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7542,6 +7764,9 @@
       <c r="AC74" t="n">
         <v>0</v>
       </c>
+      <c r="AD74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7632,9 +7857,12 @@
         <v>0</v>
       </c>
       <c r="AB75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC75" t="n">
         <v>7</v>
       </c>
-      <c r="AC75" t="n">
+      <c r="AD75" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7727,9 +7955,12 @@
         <v>0</v>
       </c>
       <c r="AB76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC76" t="n">
         <v>9</v>
       </c>
-      <c r="AC76" t="n">
+      <c r="AD76" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7822,10 +8053,13 @@
         <v>0</v>
       </c>
       <c r="AB77" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC77" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AD77" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="78">
@@ -7917,10 +8151,13 @@
         <v>0</v>
       </c>
       <c r="AB78" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC78" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD78" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="79">
@@ -8012,9 +8249,12 @@
         <v>0</v>
       </c>
       <c r="AB79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC79" t="n">
         <v>9</v>
       </c>
-      <c r="AC79" t="n">
+      <c r="AD79" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8107,10 +8347,13 @@
         <v>0</v>
       </c>
       <c r="AB80" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AC80" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AD80" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="81">
@@ -8205,7 +8448,10 @@
         <v>1</v>
       </c>
       <c r="AC81" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AD81" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="82">
@@ -8302,6 +8548,9 @@
       <c r="AC82" t="n">
         <v>0</v>
       </c>
+      <c r="AD82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8392,9 +8641,12 @@
         <v>0</v>
       </c>
       <c r="AB83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC83" t="n">
         <v>9</v>
       </c>
-      <c r="AC83" t="n">
+      <c r="AD83" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8490,7 +8742,10 @@
         <v>1</v>
       </c>
       <c r="AC84" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AD84" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="85">
@@ -8582,9 +8837,12 @@
         <v>0</v>
       </c>
       <c r="AB85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC85" t="n">
         <v>7</v>
       </c>
-      <c r="AC85" t="n">
+      <c r="AD85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8682,6 +8940,9 @@
       <c r="AC86" t="n">
         <v>0</v>
       </c>
+      <c r="AD86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8772,10 +9033,13 @@
         <v>0</v>
       </c>
       <c r="AB87" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AC87" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AD87" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="88">
@@ -8872,6 +9136,9 @@
       <c r="AC88" t="n">
         <v>0</v>
       </c>
+      <c r="AD88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -8962,10 +9229,13 @@
         <v>0</v>
       </c>
       <c r="AB89" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AC89" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AD89" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="90">
@@ -9057,10 +9327,13 @@
         <v>0</v>
       </c>
       <c r="AB90" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AC90" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AD90" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="91">
@@ -9152,9 +9425,12 @@
         <v>0</v>
       </c>
       <c r="AB91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC91" t="n">
         <v>37</v>
       </c>
-      <c r="AC91" t="n">
+      <c r="AD91" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9247,9 +9523,12 @@
         <v>0</v>
       </c>
       <c r="AB92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC92" t="n">
         <v>4</v>
       </c>
-      <c r="AC92" t="n">
+      <c r="AD92" t="n">
         <v>4</v>
       </c>
     </row>
@@ -9347,6 +9626,9 @@
       <c r="AC93" t="n">
         <v>0</v>
       </c>
+      <c r="AD93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -9437,10 +9719,13 @@
         <v>0</v>
       </c>
       <c r="AB94" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AC94" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AD94" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="95">
@@ -9532,10 +9817,13 @@
         <v>0</v>
       </c>
       <c r="AB95" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC95" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AD95" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="96">
@@ -9627,10 +9915,13 @@
         <v>0</v>
       </c>
       <c r="AB96" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC96" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD96" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="97">
@@ -9727,6 +10018,9 @@
       <c r="AC97" t="n">
         <v>0</v>
       </c>
+      <c r="AD97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -9817,10 +10111,13 @@
         <v>0</v>
       </c>
       <c r="AB98" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AC98" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AD98" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="99">
@@ -9912,9 +10209,12 @@
         <v>0</v>
       </c>
       <c r="AB99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC99" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10012,6 +10312,9 @@
       <c r="AC100" t="n">
         <v>0</v>
       </c>
+      <c r="AD100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -10102,10 +10405,13 @@
         <v>0</v>
       </c>
       <c r="AB101" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC101" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AD101" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="102">
@@ -10197,10 +10503,13 @@
         <v>0</v>
       </c>
       <c r="AB102" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC102" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AD102" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="103">
@@ -10292,10 +10601,13 @@
         <v>0</v>
       </c>
       <c r="AB103" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC103" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AD103" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="104">
@@ -10387,9 +10699,12 @@
         <v>0</v>
       </c>
       <c r="AB104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC104" t="n">
         <v>2</v>
       </c>
-      <c r="AC104" t="n">
+      <c r="AD104" t="n">
         <v>2</v>
       </c>
     </row>
@@ -10485,7 +10800,10 @@
         <v>1</v>
       </c>
       <c r="AC105" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AD105" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="106">
@@ -10577,9 +10895,12 @@
         <v>0</v>
       </c>
       <c r="AB106" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC106" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD106" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10672,9 +10993,12 @@
         <v>0</v>
       </c>
       <c r="AB107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD107" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10770,7 +11094,10 @@
         <v>1</v>
       </c>
       <c r="AC108" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AD108" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="109">
@@ -10865,6 +11192,9 @@
         <v>0</v>
       </c>
       <c r="AC109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2047)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AE109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -458,8 +458,9 @@
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
     <col width="12" customWidth="1" min="28" max="28"/>
-    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
     <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -603,12 +604,17 @@
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AD1" s="2" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -706,9 +712,12 @@
         <v>0</v>
       </c>
       <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="n">
         <v>9</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AE2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -804,9 +813,12 @@
         <v>0</v>
       </c>
       <c r="AC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="n">
         <v>7</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AE3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -902,9 +914,12 @@
         <v>1</v>
       </c>
       <c r="AC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" t="n">
         <v>13</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AE4" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1000,9 +1015,12 @@
         <v>1</v>
       </c>
       <c r="AC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" t="n">
         <v>13</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AE5" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1098,9 +1116,12 @@
         <v>1</v>
       </c>
       <c r="AC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="n">
         <v>12</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AE6" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1196,9 +1217,12 @@
         <v>0</v>
       </c>
       <c r="AC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="n">
         <v>10</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AE7" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1294,9 +1318,12 @@
         <v>1</v>
       </c>
       <c r="AC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="n">
         <v>13</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AE8" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1392,9 +1419,12 @@
         <v>1</v>
       </c>
       <c r="AC9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" t="n">
         <v>14</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AE9" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1490,9 +1520,12 @@
         <v>1</v>
       </c>
       <c r="AC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" t="n">
         <v>13</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AE10" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1588,9 +1621,12 @@
         <v>1</v>
       </c>
       <c r="AC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD11" t="n">
         <v>12</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AE11" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1686,9 +1722,12 @@
         <v>1</v>
       </c>
       <c r="AC12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" t="n">
         <v>14</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AE12" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1784,9 +1823,12 @@
         <v>1</v>
       </c>
       <c r="AC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" t="n">
         <v>8</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AE13" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1882,9 +1924,12 @@
         <v>1</v>
       </c>
       <c r="AC14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD14" t="n">
         <v>13</v>
       </c>
-      <c r="AD14" t="n">
+      <c r="AE14" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1980,9 +2025,12 @@
         <v>0</v>
       </c>
       <c r="AC15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD15" t="n">
         <v>9</v>
       </c>
-      <c r="AD15" t="n">
+      <c r="AE15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2078,9 +2126,12 @@
         <v>0</v>
       </c>
       <c r="AC16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD16" t="n">
         <v>11</v>
       </c>
-      <c r="AD16" t="n">
+      <c r="AE16" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2176,9 +2227,12 @@
         <v>0</v>
       </c>
       <c r="AC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD17" t="n">
         <v>11</v>
       </c>
-      <c r="AD17" t="n">
+      <c r="AE17" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2274,9 +2328,12 @@
         <v>1</v>
       </c>
       <c r="AC18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" t="n">
         <v>12</v>
       </c>
-      <c r="AD18" t="n">
+      <c r="AE18" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2377,6 +2434,9 @@
       <c r="AD19" t="n">
         <v>0</v>
       </c>
+      <c r="AE19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2470,9 +2530,12 @@
         <v>1</v>
       </c>
       <c r="AC20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD20" t="n">
         <v>11</v>
       </c>
-      <c r="AD20" t="n">
+      <c r="AE20" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2568,9 +2631,12 @@
         <v>1</v>
       </c>
       <c r="AC21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD21" t="n">
         <v>12</v>
       </c>
-      <c r="AD21" t="n">
+      <c r="AE21" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2671,6 +2737,9 @@
       <c r="AD22" t="n">
         <v>0</v>
       </c>
+      <c r="AE22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2764,9 +2833,12 @@
         <v>1</v>
       </c>
       <c r="AC23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD23" t="n">
         <v>7</v>
       </c>
-      <c r="AD23" t="n">
+      <c r="AE23" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2862,9 +2934,12 @@
         <v>1</v>
       </c>
       <c r="AC24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD24" t="n">
         <v>12</v>
       </c>
-      <c r="AD24" t="n">
+      <c r="AE24" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2960,9 +3035,12 @@
         <v>0</v>
       </c>
       <c r="AC25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD25" t="n">
         <v>6</v>
       </c>
-      <c r="AD25" t="n">
+      <c r="AE25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3058,10 +3136,13 @@
         <v>1</v>
       </c>
       <c r="AC26" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AD26" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="27">
@@ -3156,9 +3237,12 @@
         <v>1</v>
       </c>
       <c r="AC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD27" t="n">
         <v>14</v>
       </c>
-      <c r="AD27" t="n">
+      <c r="AE27" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3254,9 +3338,12 @@
         <v>1</v>
       </c>
       <c r="AC28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD28" t="n">
         <v>2</v>
       </c>
-      <c r="AD28" t="n">
+      <c r="AE28" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3352,9 +3439,12 @@
         <v>0</v>
       </c>
       <c r="AC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD29" t="n">
         <v>4</v>
       </c>
-      <c r="AD29" t="n">
+      <c r="AE29" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3450,9 +3540,12 @@
         <v>0</v>
       </c>
       <c r="AC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" t="n">
         <v>10</v>
       </c>
-      <c r="AD30" t="n">
+      <c r="AE30" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3548,9 +3641,12 @@
         <v>1</v>
       </c>
       <c r="AC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" t="n">
         <v>11</v>
       </c>
-      <c r="AD31" t="n">
+      <c r="AE31" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3646,9 +3742,12 @@
         <v>0</v>
       </c>
       <c r="AC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD32" t="n">
         <v>10</v>
       </c>
-      <c r="AD32" t="n">
+      <c r="AE32" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3744,9 +3843,12 @@
         <v>0</v>
       </c>
       <c r="AC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD33" t="n">
         <v>11</v>
       </c>
-      <c r="AD33" t="n">
+      <c r="AE33" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3842,9 +3944,12 @@
         <v>0</v>
       </c>
       <c r="AC34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD34" t="n">
         <v>6</v>
       </c>
-      <c r="AD34" t="n">
+      <c r="AE34" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3940,9 +4045,12 @@
         <v>0</v>
       </c>
       <c r="AC35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD35" t="n">
         <v>11</v>
       </c>
-      <c r="AD35" t="n">
+      <c r="AE35" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4038,9 +4146,12 @@
         <v>0</v>
       </c>
       <c r="AC36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD36" t="n">
         <v>6</v>
       </c>
-      <c r="AD36" t="n">
+      <c r="AE36" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4141,6 +4252,9 @@
       <c r="AD37" t="n">
         <v>0</v>
       </c>
+      <c r="AE37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4234,9 +4348,12 @@
         <v>0</v>
       </c>
       <c r="AC38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD38" t="n">
         <v>2</v>
       </c>
-      <c r="AD38" t="n">
+      <c r="AE38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4332,9 +4449,12 @@
         <v>1</v>
       </c>
       <c r="AC39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD39" t="n">
         <v>13</v>
       </c>
-      <c r="AD39" t="n">
+      <c r="AE39" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4430,9 +4550,12 @@
         <v>1</v>
       </c>
       <c r="AC40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD40" t="n">
         <v>12</v>
       </c>
-      <c r="AD40" t="n">
+      <c r="AE40" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4528,9 +4651,12 @@
         <v>1</v>
       </c>
       <c r="AC41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD41" t="n">
         <v>14</v>
       </c>
-      <c r="AD41" t="n">
+      <c r="AE41" t="n">
         <v>14</v>
       </c>
     </row>
@@ -4626,9 +4752,12 @@
         <v>0</v>
       </c>
       <c r="AC42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD42" t="n">
         <v>21</v>
       </c>
-      <c r="AD42" t="n">
+      <c r="AE42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4724,9 +4853,12 @@
         <v>0</v>
       </c>
       <c r="AC43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD43" t="n">
         <v>49</v>
       </c>
-      <c r="AD43" t="n">
+      <c r="AE43" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4822,9 +4954,12 @@
         <v>1</v>
       </c>
       <c r="AC44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD44" t="n">
         <v>11</v>
       </c>
-      <c r="AD44" t="n">
+      <c r="AE44" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4920,9 +5055,12 @@
         <v>1</v>
       </c>
       <c r="AC45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD45" t="n">
         <v>13</v>
       </c>
-      <c r="AD45" t="n">
+      <c r="AE45" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5018,9 +5156,12 @@
         <v>1</v>
       </c>
       <c r="AC46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD46" t="n">
         <v>11</v>
       </c>
-      <c r="AD46" t="n">
+      <c r="AE46" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5121,6 +5262,9 @@
       <c r="AD47" t="n">
         <v>0</v>
       </c>
+      <c r="AE47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5214,9 +5358,12 @@
         <v>1</v>
       </c>
       <c r="AC48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD48" t="n">
         <v>13</v>
       </c>
-      <c r="AD48" t="n">
+      <c r="AE48" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5312,9 +5459,12 @@
         <v>1</v>
       </c>
       <c r="AC49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD49" t="n">
         <v>12</v>
       </c>
-      <c r="AD49" t="n">
+      <c r="AE49" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5410,9 +5560,12 @@
         <v>0</v>
       </c>
       <c r="AC50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD50" t="n">
         <v>6</v>
       </c>
-      <c r="AD50" t="n">
+      <c r="AE50" t="n">
         <v>6</v>
       </c>
     </row>
@@ -5508,9 +5661,12 @@
         <v>1</v>
       </c>
       <c r="AC51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD51" t="n">
         <v>13</v>
       </c>
-      <c r="AD51" t="n">
+      <c r="AE51" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5611,6 +5767,9 @@
       <c r="AD52" t="n">
         <v>0</v>
       </c>
+      <c r="AE52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5704,9 +5863,12 @@
         <v>1</v>
       </c>
       <c r="AC53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD53" t="n">
         <v>11</v>
       </c>
-      <c r="AD53" t="n">
+      <c r="AE53" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5807,6 +5969,9 @@
       <c r="AD54" t="n">
         <v>0</v>
       </c>
+      <c r="AE54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5900,9 +6065,12 @@
         <v>1</v>
       </c>
       <c r="AC55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD55" t="n">
         <v>12</v>
       </c>
-      <c r="AD55" t="n">
+      <c r="AE55" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5998,10 +6166,13 @@
         <v>0</v>
       </c>
       <c r="AC56" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AD56" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AE56" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="57">
@@ -6096,9 +6267,12 @@
         <v>0</v>
       </c>
       <c r="AC57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD57" t="n">
         <v>7</v>
       </c>
-      <c r="AD57" t="n">
+      <c r="AE57" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6194,9 +6368,12 @@
         <v>0</v>
       </c>
       <c r="AC58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD58" t="n">
         <v>12</v>
       </c>
-      <c r="AD58" t="n">
+      <c r="AE58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6292,9 +6469,12 @@
         <v>0</v>
       </c>
       <c r="AC59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD59" t="n">
         <v>3</v>
       </c>
-      <c r="AD59" t="n">
+      <c r="AE59" t="n">
         <v>3</v>
       </c>
     </row>
@@ -6395,6 +6575,9 @@
       <c r="AD60" t="n">
         <v>0</v>
       </c>
+      <c r="AE60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6488,9 +6671,12 @@
         <v>1</v>
       </c>
       <c r="AC61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD61" t="n">
         <v>10</v>
       </c>
-      <c r="AD61" t="n">
+      <c r="AE61" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6586,9 +6772,12 @@
         <v>1</v>
       </c>
       <c r="AC62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD62" t="n">
         <v>13</v>
       </c>
-      <c r="AD62" t="n">
+      <c r="AE62" t="n">
         <v>13</v>
       </c>
     </row>
@@ -6684,9 +6873,12 @@
         <v>1</v>
       </c>
       <c r="AC63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD63" t="n">
         <v>2</v>
       </c>
-      <c r="AD63" t="n">
+      <c r="AE63" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6787,6 +6979,9 @@
       <c r="AD64" t="n">
         <v>0</v>
       </c>
+      <c r="AE64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6880,9 +7075,12 @@
         <v>0</v>
       </c>
       <c r="AC65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD65" t="n">
         <v>5</v>
       </c>
-      <c r="AD65" t="n">
+      <c r="AE65" t="n">
         <v>5</v>
       </c>
     </row>
@@ -6978,9 +7176,12 @@
         <v>0</v>
       </c>
       <c r="AC66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7076,9 +7277,12 @@
         <v>1</v>
       </c>
       <c r="AC67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD67" t="n">
         <v>14</v>
       </c>
-      <c r="AD67" t="n">
+      <c r="AE67" t="n">
         <v>14</v>
       </c>
     </row>
@@ -7174,9 +7378,12 @@
         <v>1</v>
       </c>
       <c r="AC68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD68" t="n">
         <v>6</v>
       </c>
-      <c r="AD68" t="n">
+      <c r="AE68" t="n">
         <v>5</v>
       </c>
     </row>
@@ -7272,9 +7479,12 @@
         <v>0</v>
       </c>
       <c r="AC69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD69" t="n">
         <v>7</v>
       </c>
-      <c r="AD69" t="n">
+      <c r="AE69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7370,9 +7580,12 @@
         <v>0</v>
       </c>
       <c r="AC70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD70" t="n">
         <v>21</v>
       </c>
-      <c r="AD70" t="n">
+      <c r="AE70" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7468,9 +7681,12 @@
         <v>1</v>
       </c>
       <c r="AC71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD71" t="n">
         <v>7</v>
       </c>
-      <c r="AD71" t="n">
+      <c r="AE71" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7566,9 +7782,12 @@
         <v>1</v>
       </c>
       <c r="AC72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD72" t="n">
         <v>11</v>
       </c>
-      <c r="AD72" t="n">
+      <c r="AE72" t="n">
         <v>11</v>
       </c>
     </row>
@@ -7669,6 +7888,9 @@
       <c r="AD73" t="n">
         <v>0</v>
       </c>
+      <c r="AE73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7767,6 +7989,9 @@
       <c r="AD74" t="n">
         <v>0</v>
       </c>
+      <c r="AE74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7860,9 +8085,12 @@
         <v>0</v>
       </c>
       <c r="AC75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD75" t="n">
         <v>7</v>
       </c>
-      <c r="AD75" t="n">
+      <c r="AE75" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7958,9 +8186,12 @@
         <v>0</v>
       </c>
       <c r="AC76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD76" t="n">
         <v>9</v>
       </c>
-      <c r="AD76" t="n">
+      <c r="AE76" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8056,9 +8287,12 @@
         <v>1</v>
       </c>
       <c r="AC77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD77" t="n">
         <v>12</v>
       </c>
-      <c r="AD77" t="n">
+      <c r="AE77" t="n">
         <v>12</v>
       </c>
     </row>
@@ -8154,9 +8388,12 @@
         <v>1</v>
       </c>
       <c r="AC78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD78" t="n">
         <v>13</v>
       </c>
-      <c r="AD78" t="n">
+      <c r="AE78" t="n">
         <v>13</v>
       </c>
     </row>
@@ -8252,9 +8489,12 @@
         <v>0</v>
       </c>
       <c r="AC79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD79" t="n">
         <v>9</v>
       </c>
-      <c r="AD79" t="n">
+      <c r="AE79" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8350,9 +8590,12 @@
         <v>1</v>
       </c>
       <c r="AC80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD80" t="n">
         <v>4</v>
       </c>
-      <c r="AD80" t="n">
+      <c r="AE80" t="n">
         <v>4</v>
       </c>
     </row>
@@ -8448,9 +8691,12 @@
         <v>1</v>
       </c>
       <c r="AC81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD81" t="n">
         <v>2</v>
       </c>
-      <c r="AD81" t="n">
+      <c r="AE81" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8551,6 +8797,9 @@
       <c r="AD82" t="n">
         <v>0</v>
       </c>
+      <c r="AE82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8644,9 +8893,12 @@
         <v>0</v>
       </c>
       <c r="AC83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD83" t="n">
         <v>9</v>
       </c>
-      <c r="AD83" t="n">
+      <c r="AE83" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8742,9 +8994,12 @@
         <v>1</v>
       </c>
       <c r="AC84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD84" t="n">
         <v>2</v>
       </c>
-      <c r="AD84" t="n">
+      <c r="AE84" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8840,9 +9095,12 @@
         <v>0</v>
       </c>
       <c r="AC85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD85" t="n">
         <v>7</v>
       </c>
-      <c r="AD85" t="n">
+      <c r="AE85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8943,6 +9201,9 @@
       <c r="AD86" t="n">
         <v>0</v>
       </c>
+      <c r="AE86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -9036,9 +9297,12 @@
         <v>1</v>
       </c>
       <c r="AC87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD87" t="n">
         <v>8</v>
       </c>
-      <c r="AD87" t="n">
+      <c r="AE87" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9139,6 +9403,9 @@
       <c r="AD88" t="n">
         <v>0</v>
       </c>
+      <c r="AE88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -9232,9 +9499,12 @@
         <v>1</v>
       </c>
       <c r="AC89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD89" t="n">
         <v>10</v>
       </c>
-      <c r="AD89" t="n">
+      <c r="AE89" t="n">
         <v>10</v>
       </c>
     </row>
@@ -9330,9 +9600,12 @@
         <v>1</v>
       </c>
       <c r="AC90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD90" t="n">
         <v>9</v>
       </c>
-      <c r="AD90" t="n">
+      <c r="AE90" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9428,9 +9701,12 @@
         <v>0</v>
       </c>
       <c r="AC91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD91" t="n">
         <v>37</v>
       </c>
-      <c r="AD91" t="n">
+      <c r="AE91" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9526,9 +9802,12 @@
         <v>0</v>
       </c>
       <c r="AC92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD92" t="n">
         <v>4</v>
       </c>
-      <c r="AD92" t="n">
+      <c r="AE92" t="n">
         <v>4</v>
       </c>
     </row>
@@ -9629,6 +9908,9 @@
       <c r="AD93" t="n">
         <v>0</v>
       </c>
+      <c r="AE93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -9722,9 +10004,12 @@
         <v>1</v>
       </c>
       <c r="AC94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD94" t="n">
         <v>7</v>
       </c>
-      <c r="AD94" t="n">
+      <c r="AE94" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9820,9 +10105,12 @@
         <v>1</v>
       </c>
       <c r="AC95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD95" t="n">
         <v>6</v>
       </c>
-      <c r="AD95" t="n">
+      <c r="AE95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -9918,9 +10206,12 @@
         <v>1</v>
       </c>
       <c r="AC96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD96" t="n">
         <v>13</v>
       </c>
-      <c r="AD96" t="n">
+      <c r="AE96" t="n">
         <v>13</v>
       </c>
     </row>
@@ -10021,6 +10312,9 @@
       <c r="AD97" t="n">
         <v>0</v>
       </c>
+      <c r="AE97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -10114,10 +10408,13 @@
         <v>1</v>
       </c>
       <c r="AC98" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AD98" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AE98" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="99">
@@ -10212,9 +10509,12 @@
         <v>0</v>
       </c>
       <c r="AC99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD99" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE99" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10315,6 +10615,9 @@
       <c r="AD100" t="n">
         <v>0</v>
       </c>
+      <c r="AE100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -10408,10 +10711,13 @@
         <v>1</v>
       </c>
       <c r="AC101" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AD101" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AE101" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="102">
@@ -10506,9 +10812,12 @@
         <v>1</v>
       </c>
       <c r="AC102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD102" t="n">
         <v>12</v>
       </c>
-      <c r="AD102" t="n">
+      <c r="AE102" t="n">
         <v>12</v>
       </c>
     </row>
@@ -10604,9 +10913,12 @@
         <v>1</v>
       </c>
       <c r="AC103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD103" t="n">
         <v>12</v>
       </c>
-      <c r="AD103" t="n">
+      <c r="AE103" t="n">
         <v>12</v>
       </c>
     </row>
@@ -10702,9 +11014,12 @@
         <v>0</v>
       </c>
       <c r="AC104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD104" t="n">
         <v>2</v>
       </c>
-      <c r="AD104" t="n">
+      <c r="AE104" t="n">
         <v>2</v>
       </c>
     </row>
@@ -10800,9 +11115,12 @@
         <v>1</v>
       </c>
       <c r="AC105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD105" t="n">
         <v>2</v>
       </c>
-      <c r="AD105" t="n">
+      <c r="AE105" t="n">
         <v>2</v>
       </c>
     </row>
@@ -10898,9 +11216,12 @@
         <v>0</v>
       </c>
       <c r="AC106" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD106" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE106" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10996,9 +11317,12 @@
         <v>0</v>
       </c>
       <c r="AC107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE107" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11094,9 +11418,12 @@
         <v>1</v>
       </c>
       <c r="AC108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD108" t="n">
         <v>2</v>
       </c>
-      <c r="AD108" t="n">
+      <c r="AE108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -11195,6 +11522,9 @@
         <v>0</v>
       </c>
       <c r="AD109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2124)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE109"/>
+  <dimension ref="A1:AF109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -459,8 +459,9 @@
     <col width="12" customWidth="1" min="27" max="27"/>
     <col width="12" customWidth="1" min="28" max="28"/>
     <col width="12" customWidth="1" min="29" max="29"/>
-    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -609,12 +610,17 @@
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="AD1" s="2" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AE1" s="2" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -715,10 +721,13 @@
         <v>0</v>
       </c>
       <c r="AD2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AE2" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -816,10 +825,13 @@
         <v>0</v>
       </c>
       <c r="AD3" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AE3" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -917,10 +929,13 @@
         <v>0</v>
       </c>
       <c r="AD4" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AE4" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -1018,9 +1033,12 @@
         <v>0</v>
       </c>
       <c r="AD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" t="n">
         <v>13</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AF5" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1119,9 +1137,12 @@
         <v>0</v>
       </c>
       <c r="AD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="n">
         <v>12</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AF6" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1220,10 +1241,13 @@
         <v>0</v>
       </c>
       <c r="AD7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AE7" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -1321,10 +1345,13 @@
         <v>0</v>
       </c>
       <c r="AD8" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AE8" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -1422,10 +1449,13 @@
         <v>0</v>
       </c>
       <c r="AD9" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AE9" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1523,10 +1553,13 @@
         <v>0</v>
       </c>
       <c r="AD10" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AE10" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="11">
@@ -1624,10 +1657,13 @@
         <v>0</v>
       </c>
       <c r="AD11" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AE11" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="12">
@@ -1725,9 +1761,12 @@
         <v>0</v>
       </c>
       <c r="AD12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE12" t="n">
         <v>14</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AF12" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1826,9 +1865,12 @@
         <v>0</v>
       </c>
       <c r="AD13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE13" t="n">
         <v>8</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AF13" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1927,10 +1969,13 @@
         <v>0</v>
       </c>
       <c r="AD14" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AE14" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="15">
@@ -2028,9 +2073,12 @@
         <v>0</v>
       </c>
       <c r="AD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE15" t="n">
         <v>9</v>
       </c>
-      <c r="AE15" t="n">
+      <c r="AF15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2129,10 +2177,13 @@
         <v>0</v>
       </c>
       <c r="AD16" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AE16" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -2230,10 +2281,13 @@
         <v>0</v>
       </c>
       <c r="AD17" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AE17" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="18">
@@ -2331,10 +2385,13 @@
         <v>0</v>
       </c>
       <c r="AD18" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AE18" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="19">
@@ -2437,6 +2494,9 @@
       <c r="AE19" t="n">
         <v>0</v>
       </c>
+      <c r="AF19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2533,9 +2593,12 @@
         <v>0</v>
       </c>
       <c r="AD20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE20" t="n">
         <v>11</v>
       </c>
-      <c r="AE20" t="n">
+      <c r="AF20" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2634,10 +2697,13 @@
         <v>0</v>
       </c>
       <c r="AD21" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AE21" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="22">
@@ -2740,6 +2806,9 @@
       <c r="AE22" t="n">
         <v>0</v>
       </c>
+      <c r="AF22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2836,9 +2905,12 @@
         <v>0</v>
       </c>
       <c r="AD23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE23" t="n">
         <v>7</v>
       </c>
-      <c r="AE23" t="n">
+      <c r="AF23" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2937,10 +3009,13 @@
         <v>0</v>
       </c>
       <c r="AD24" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AE24" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="25">
@@ -3038,9 +3113,12 @@
         <v>0</v>
       </c>
       <c r="AD25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" t="n">
         <v>6</v>
       </c>
-      <c r="AE25" t="n">
+      <c r="AF25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3139,10 +3217,13 @@
         <v>1</v>
       </c>
       <c r="AD26" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AE26" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="27">
@@ -3240,10 +3321,13 @@
         <v>0</v>
       </c>
       <c r="AD27" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AE27" t="n">
-        <v>12</v>
+        <v>15</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="28">
@@ -3341,10 +3425,13 @@
         <v>0</v>
       </c>
       <c r="AD28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE28" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="29">
@@ -3442,10 +3529,13 @@
         <v>0</v>
       </c>
       <c r="AD29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AE29" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="30">
@@ -3543,10 +3633,13 @@
         <v>0</v>
       </c>
       <c r="AD30" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AE30" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="31">
@@ -3644,10 +3737,13 @@
         <v>0</v>
       </c>
       <c r="AD31" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AE31" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="32">
@@ -3745,10 +3841,13 @@
         <v>0</v>
       </c>
       <c r="AD32" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AE32" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="33">
@@ -3846,10 +3945,13 @@
         <v>0</v>
       </c>
       <c r="AD33" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AE33" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="34">
@@ -3947,9 +4049,12 @@
         <v>0</v>
       </c>
       <c r="AD34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE34" t="n">
         <v>6</v>
       </c>
-      <c r="AE34" t="n">
+      <c r="AF34" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4048,9 +4153,12 @@
         <v>0</v>
       </c>
       <c r="AD35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE35" t="n">
         <v>11</v>
       </c>
-      <c r="AE35" t="n">
+      <c r="AF35" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4149,10 +4257,13 @@
         <v>0</v>
       </c>
       <c r="AD36" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AE36" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="37">
@@ -4255,6 +4366,9 @@
       <c r="AE37" t="n">
         <v>0</v>
       </c>
+      <c r="AF37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4351,9 +4465,12 @@
         <v>0</v>
       </c>
       <c r="AD38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE38" t="n">
         <v>2</v>
       </c>
-      <c r="AE38" t="n">
+      <c r="AF38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4452,10 +4569,13 @@
         <v>0</v>
       </c>
       <c r="AD39" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AE39" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="40">
@@ -4553,10 +4673,13 @@
         <v>0</v>
       </c>
       <c r="AD40" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AE40" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AF40" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="41">
@@ -4654,10 +4777,13 @@
         <v>0</v>
       </c>
       <c r="AD41" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AE41" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AF41" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="42">
@@ -4755,9 +4881,12 @@
         <v>0</v>
       </c>
       <c r="AD42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE42" t="n">
         <v>21</v>
       </c>
-      <c r="AE42" t="n">
+      <c r="AF42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4856,9 +4985,12 @@
         <v>0</v>
       </c>
       <c r="AD43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE43" t="n">
         <v>49</v>
       </c>
-      <c r="AE43" t="n">
+      <c r="AF43" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4957,9 +5089,12 @@
         <v>0</v>
       </c>
       <c r="AD44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE44" t="n">
         <v>11</v>
       </c>
-      <c r="AE44" t="n">
+      <c r="AF44" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5058,10 +5193,13 @@
         <v>0</v>
       </c>
       <c r="AD45" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AE45" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="46">
@@ -5159,10 +5297,13 @@
         <v>0</v>
       </c>
       <c r="AD46" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AE46" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AF46" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="47">
@@ -5265,6 +5406,9 @@
       <c r="AE47" t="n">
         <v>0</v>
       </c>
+      <c r="AF47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5361,10 +5505,13 @@
         <v>0</v>
       </c>
       <c r="AD48" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AE48" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AF48" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="49">
@@ -5462,9 +5609,12 @@
         <v>0</v>
       </c>
       <c r="AD49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE49" t="n">
         <v>12</v>
       </c>
-      <c r="AE49" t="n">
+      <c r="AF49" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5563,9 +5713,12 @@
         <v>0</v>
       </c>
       <c r="AD50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE50" t="n">
         <v>6</v>
       </c>
-      <c r="AE50" t="n">
+      <c r="AF50" t="n">
         <v>6</v>
       </c>
     </row>
@@ -5664,10 +5817,13 @@
         <v>0</v>
       </c>
       <c r="AD51" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AE51" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AF51" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="52">
@@ -5770,6 +5926,9 @@
       <c r="AE52" t="n">
         <v>0</v>
       </c>
+      <c r="AF52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5866,10 +6025,13 @@
         <v>0</v>
       </c>
       <c r="AD53" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AE53" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AF53" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="54">
@@ -5972,6 +6134,9 @@
       <c r="AE54" t="n">
         <v>0</v>
       </c>
+      <c r="AF54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6068,10 +6233,13 @@
         <v>0</v>
       </c>
       <c r="AD55" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AE55" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AF55" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="56">
@@ -6169,10 +6337,13 @@
         <v>1</v>
       </c>
       <c r="AD56" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AE56" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AF56" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="57">
@@ -6270,9 +6441,12 @@
         <v>0</v>
       </c>
       <c r="AD57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE57" t="n">
         <v>7</v>
       </c>
-      <c r="AE57" t="n">
+      <c r="AF57" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6371,9 +6545,12 @@
         <v>0</v>
       </c>
       <c r="AD58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE58" t="n">
         <v>12</v>
       </c>
-      <c r="AE58" t="n">
+      <c r="AF58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6472,9 +6649,12 @@
         <v>0</v>
       </c>
       <c r="AD59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE59" t="n">
         <v>3</v>
       </c>
-      <c r="AE59" t="n">
+      <c r="AF59" t="n">
         <v>3</v>
       </c>
     </row>
@@ -6578,6 +6758,9 @@
       <c r="AE60" t="n">
         <v>0</v>
       </c>
+      <c r="AF60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6674,10 +6857,13 @@
         <v>0</v>
       </c>
       <c r="AD61" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AE61" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AF61" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="62">
@@ -6775,9 +6961,12 @@
         <v>0</v>
       </c>
       <c r="AD62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE62" t="n">
         <v>13</v>
       </c>
-      <c r="AE62" t="n">
+      <c r="AF62" t="n">
         <v>13</v>
       </c>
     </row>
@@ -6876,10 +7065,13 @@
         <v>0</v>
       </c>
       <c r="AD63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE63" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AF63" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="64">
@@ -6982,6 +7174,9 @@
       <c r="AE64" t="n">
         <v>0</v>
       </c>
+      <c r="AF64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7078,10 +7273,13 @@
         <v>0</v>
       </c>
       <c r="AD65" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE65" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AF65" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="66">
@@ -7179,9 +7377,12 @@
         <v>0</v>
       </c>
       <c r="AD66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7280,10 +7481,13 @@
         <v>0</v>
       </c>
       <c r="AD67" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AE67" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AF67" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="68">
@@ -7381,10 +7585,13 @@
         <v>0</v>
       </c>
       <c r="AD68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE68" t="n">
+        <v>7</v>
+      </c>
+      <c r="AF68" t="n">
         <v>6</v>
-      </c>
-      <c r="AE68" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="69">
@@ -7482,9 +7689,12 @@
         <v>0</v>
       </c>
       <c r="AD69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE69" t="n">
         <v>7</v>
       </c>
-      <c r="AE69" t="n">
+      <c r="AF69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7583,10 +7793,13 @@
         <v>0</v>
       </c>
       <c r="AD70" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AE70" t="n">
-        <v>9</v>
+        <v>22</v>
+      </c>
+      <c r="AF70" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="71">
@@ -7684,10 +7897,13 @@
         <v>0</v>
       </c>
       <c r="AD71" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AE71" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AF71" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="72">
@@ -7785,10 +8001,13 @@
         <v>0</v>
       </c>
       <c r="AD72" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AE72" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AF72" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="73">
@@ -7891,6 +8110,9 @@
       <c r="AE73" t="n">
         <v>0</v>
       </c>
+      <c r="AF73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7992,6 +8214,9 @@
       <c r="AE74" t="n">
         <v>0</v>
       </c>
+      <c r="AF74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8088,10 +8313,13 @@
         <v>0</v>
       </c>
       <c r="AD75" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AE75" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AF75" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="76">
@@ -8189,10 +8417,13 @@
         <v>0</v>
       </c>
       <c r="AD76" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AE76" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AF76" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="77">
@@ -8290,9 +8521,12 @@
         <v>0</v>
       </c>
       <c r="AD77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE77" t="n">
         <v>12</v>
       </c>
-      <c r="AE77" t="n">
+      <c r="AF77" t="n">
         <v>12</v>
       </c>
     </row>
@@ -8391,9 +8625,12 @@
         <v>0</v>
       </c>
       <c r="AD78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE78" t="n">
         <v>13</v>
       </c>
-      <c r="AE78" t="n">
+      <c r="AF78" t="n">
         <v>13</v>
       </c>
     </row>
@@ -8492,10 +8729,13 @@
         <v>0</v>
       </c>
       <c r="AD79" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AE79" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AF79" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="80">
@@ -8593,10 +8833,13 @@
         <v>0</v>
       </c>
       <c r="AD80" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AE80" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AF80" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="81">
@@ -8694,9 +8937,12 @@
         <v>0</v>
       </c>
       <c r="AD81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE81" t="n">
         <v>2</v>
       </c>
-      <c r="AE81" t="n">
+      <c r="AF81" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8795,10 +9041,13 @@
         <v>0</v>
       </c>
       <c r="AD82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE82" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AF82" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -8896,10 +9145,13 @@
         <v>0</v>
       </c>
       <c r="AD83" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AE83" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AF83" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="84">
@@ -8997,9 +9249,12 @@
         <v>0</v>
       </c>
       <c r="AD84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE84" t="n">
         <v>2</v>
       </c>
-      <c r="AE84" t="n">
+      <c r="AF84" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9098,9 +9353,12 @@
         <v>0</v>
       </c>
       <c r="AD85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE85" t="n">
         <v>7</v>
       </c>
-      <c r="AE85" t="n">
+      <c r="AF85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9204,6 +9462,9 @@
       <c r="AE86" t="n">
         <v>0</v>
       </c>
+      <c r="AF86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -9300,9 +9561,12 @@
         <v>0</v>
       </c>
       <c r="AD87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE87" t="n">
         <v>8</v>
       </c>
-      <c r="AE87" t="n">
+      <c r="AF87" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9406,6 +9670,9 @@
       <c r="AE88" t="n">
         <v>0</v>
       </c>
+      <c r="AF88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -9502,9 +9769,12 @@
         <v>0</v>
       </c>
       <c r="AD89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE89" t="n">
         <v>10</v>
       </c>
-      <c r="AE89" t="n">
+      <c r="AF89" t="n">
         <v>10</v>
       </c>
     </row>
@@ -9603,9 +9873,12 @@
         <v>0</v>
       </c>
       <c r="AD90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE90" t="n">
         <v>9</v>
       </c>
-      <c r="AE90" t="n">
+      <c r="AF90" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9704,9 +9977,12 @@
         <v>0</v>
       </c>
       <c r="AD91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE91" t="n">
         <v>37</v>
       </c>
-      <c r="AE91" t="n">
+      <c r="AF91" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9805,9 +10081,12 @@
         <v>0</v>
       </c>
       <c r="AD92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE92" t="n">
         <v>4</v>
       </c>
-      <c r="AE92" t="n">
+      <c r="AF92" t="n">
         <v>4</v>
       </c>
     </row>
@@ -9911,6 +10190,9 @@
       <c r="AE93" t="n">
         <v>0</v>
       </c>
+      <c r="AF93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10007,9 +10289,12 @@
         <v>0</v>
       </c>
       <c r="AD94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE94" t="n">
         <v>7</v>
       </c>
-      <c r="AE94" t="n">
+      <c r="AF94" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10108,9 +10393,12 @@
         <v>0</v>
       </c>
       <c r="AD95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE95" t="n">
         <v>6</v>
       </c>
-      <c r="AE95" t="n">
+      <c r="AF95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10209,10 +10497,13 @@
         <v>0</v>
       </c>
       <c r="AD96" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AE96" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AF96" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="97">
@@ -10315,6 +10606,9 @@
       <c r="AE97" t="n">
         <v>0</v>
       </c>
+      <c r="AF97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -10411,9 +10705,12 @@
         <v>1</v>
       </c>
       <c r="AD98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE98" t="n">
         <v>15</v>
       </c>
-      <c r="AE98" t="n">
+      <c r="AF98" t="n">
         <v>15</v>
       </c>
     </row>
@@ -10515,7 +10812,10 @@
         <v>1</v>
       </c>
       <c r="AE99" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AF99" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="100">
@@ -10618,6 +10918,9 @@
       <c r="AE100" t="n">
         <v>0</v>
       </c>
+      <c r="AF100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -10714,9 +11017,12 @@
         <v>1</v>
       </c>
       <c r="AD101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE101" t="n">
         <v>14</v>
       </c>
-      <c r="AE101" t="n">
+      <c r="AF101" t="n">
         <v>14</v>
       </c>
     </row>
@@ -10815,10 +11121,13 @@
         <v>0</v>
       </c>
       <c r="AD102" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AE102" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AF102" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="103">
@@ -10916,10 +11225,13 @@
         <v>0</v>
       </c>
       <c r="AD103" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AE103" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AF103" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="104">
@@ -11017,10 +11329,13 @@
         <v>0</v>
       </c>
       <c r="AD104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE104" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AF104" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="105">
@@ -11118,10 +11433,13 @@
         <v>0</v>
       </c>
       <c r="AD105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE105" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AF105" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="106">
@@ -11222,7 +11540,10 @@
         <v>1</v>
       </c>
       <c r="AE106" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AF106" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="107">
@@ -11323,7 +11644,10 @@
         <v>1</v>
       </c>
       <c r="AE107" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AF107" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="108">
@@ -11421,9 +11745,12 @@
         <v>0</v>
       </c>
       <c r="AD108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE108" t="n">
         <v>2</v>
       </c>
-      <c r="AE108" t="n">
+      <c r="AF108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -11525,6 +11852,9 @@
         <v>0</v>
       </c>
       <c r="AE109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2178)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF109"/>
+  <dimension ref="A1:AG109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -460,8 +460,9 @@
     <col width="12" customWidth="1" min="28" max="28"/>
     <col width="12" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
-    <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
     <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -615,12 +616,17 @@
           <t>2026-03-20</t>
         </is>
       </c>
-      <c r="AE1" s="2" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AF1" s="2" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -724,9 +730,12 @@
         <v>1</v>
       </c>
       <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
         <v>10</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="AG2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -828,9 +837,12 @@
         <v>1</v>
       </c>
       <c r="AE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" t="n">
         <v>8</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="AG3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -932,9 +944,12 @@
         <v>1</v>
       </c>
       <c r="AE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF4" t="n">
         <v>14</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="AG4" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1036,9 +1051,12 @@
         <v>0</v>
       </c>
       <c r="AE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" t="n">
         <v>13</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="AG5" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1140,9 +1158,12 @@
         <v>0</v>
       </c>
       <c r="AE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="n">
         <v>12</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="AG6" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1244,9 +1265,12 @@
         <v>1</v>
       </c>
       <c r="AE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="n">
         <v>11</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="AG7" t="n">
         <v>11</v>
       </c>
     </row>
@@ -1348,9 +1372,12 @@
         <v>1</v>
       </c>
       <c r="AE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="n">
         <v>14</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="AG8" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1452,9 +1479,12 @@
         <v>1</v>
       </c>
       <c r="AE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" t="n">
         <v>15</v>
       </c>
-      <c r="AF9" t="n">
+      <c r="AG9" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1556,9 +1586,12 @@
         <v>1</v>
       </c>
       <c r="AE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" t="n">
         <v>14</v>
       </c>
-      <c r="AF10" t="n">
+      <c r="AG10" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1660,9 +1693,12 @@
         <v>1</v>
       </c>
       <c r="AE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF11" t="n">
         <v>13</v>
       </c>
-      <c r="AF11" t="n">
+      <c r="AG11" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1764,9 +1800,12 @@
         <v>0</v>
       </c>
       <c r="AE12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF12" t="n">
         <v>14</v>
       </c>
-      <c r="AF12" t="n">
+      <c r="AG12" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1868,9 +1907,12 @@
         <v>0</v>
       </c>
       <c r="AE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF13" t="n">
         <v>8</v>
       </c>
-      <c r="AF13" t="n">
+      <c r="AG13" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1972,9 +2014,12 @@
         <v>1</v>
       </c>
       <c r="AE14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF14" t="n">
         <v>14</v>
       </c>
-      <c r="AF14" t="n">
+      <c r="AG14" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2076,9 +2121,12 @@
         <v>0</v>
       </c>
       <c r="AE15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF15" t="n">
         <v>9</v>
       </c>
-      <c r="AF15" t="n">
+      <c r="AG15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2180,9 +2228,12 @@
         <v>1</v>
       </c>
       <c r="AE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF16" t="n">
         <v>12</v>
       </c>
-      <c r="AF16" t="n">
+      <c r="AG16" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2284,9 +2335,12 @@
         <v>1</v>
       </c>
       <c r="AE17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF17" t="n">
         <v>12</v>
       </c>
-      <c r="AF17" t="n">
+      <c r="AG17" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2388,9 +2442,12 @@
         <v>1</v>
       </c>
       <c r="AE18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF18" t="n">
         <v>13</v>
       </c>
-      <c r="AF18" t="n">
+      <c r="AG18" t="n">
         <v>13</v>
       </c>
     </row>
@@ -2497,6 +2554,9 @@
       <c r="AF19" t="n">
         <v>0</v>
       </c>
+      <c r="AG19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2596,9 +2656,12 @@
         <v>0</v>
       </c>
       <c r="AE20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF20" t="n">
         <v>11</v>
       </c>
-      <c r="AF20" t="n">
+      <c r="AG20" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2700,9 +2763,12 @@
         <v>1</v>
       </c>
       <c r="AE21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF21" t="n">
         <v>13</v>
       </c>
-      <c r="AF21" t="n">
+      <c r="AG21" t="n">
         <v>13</v>
       </c>
     </row>
@@ -2809,6 +2875,9 @@
       <c r="AF22" t="n">
         <v>0</v>
       </c>
+      <c r="AG22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2908,9 +2977,12 @@
         <v>0</v>
       </c>
       <c r="AE23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF23" t="n">
         <v>7</v>
       </c>
-      <c r="AF23" t="n">
+      <c r="AG23" t="n">
         <v>7</v>
       </c>
     </row>
@@ -3012,9 +3084,12 @@
         <v>1</v>
       </c>
       <c r="AE24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF24" t="n">
         <v>13</v>
       </c>
-      <c r="AF24" t="n">
+      <c r="AG24" t="n">
         <v>13</v>
       </c>
     </row>
@@ -3116,9 +3191,12 @@
         <v>0</v>
       </c>
       <c r="AE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="n">
         <v>6</v>
       </c>
-      <c r="AF25" t="n">
+      <c r="AG25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3220,9 +3298,12 @@
         <v>1</v>
       </c>
       <c r="AE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF26" t="n">
         <v>12</v>
       </c>
-      <c r="AF26" t="n">
+      <c r="AG26" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3324,9 +3405,12 @@
         <v>1</v>
       </c>
       <c r="AE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF27" t="n">
         <v>15</v>
       </c>
-      <c r="AF27" t="n">
+      <c r="AG27" t="n">
         <v>13</v>
       </c>
     </row>
@@ -3428,9 +3512,12 @@
         <v>1</v>
       </c>
       <c r="AE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF28" t="n">
         <v>3</v>
       </c>
-      <c r="AF28" t="n">
+      <c r="AG28" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3532,9 +3619,12 @@
         <v>1</v>
       </c>
       <c r="AE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF29" t="n">
         <v>5</v>
       </c>
-      <c r="AF29" t="n">
+      <c r="AG29" t="n">
         <v>5</v>
       </c>
     </row>
@@ -3636,9 +3726,12 @@
         <v>1</v>
       </c>
       <c r="AE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" t="n">
         <v>11</v>
       </c>
-      <c r="AF30" t="n">
+      <c r="AG30" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3740,9 +3833,12 @@
         <v>1</v>
       </c>
       <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
         <v>12</v>
       </c>
-      <c r="AF31" t="n">
+      <c r="AG31" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3844,9 +3940,12 @@
         <v>1</v>
       </c>
       <c r="AE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="n">
         <v>11</v>
       </c>
-      <c r="AF32" t="n">
+      <c r="AG32" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3948,9 +4047,12 @@
         <v>1</v>
       </c>
       <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
         <v>12</v>
       </c>
-      <c r="AF33" t="n">
+      <c r="AG33" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4052,9 +4154,12 @@
         <v>0</v>
       </c>
       <c r="AE34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF34" t="n">
         <v>6</v>
       </c>
-      <c r="AF34" t="n">
+      <c r="AG34" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4156,9 +4261,12 @@
         <v>0</v>
       </c>
       <c r="AE35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF35" t="n">
         <v>11</v>
       </c>
-      <c r="AF35" t="n">
+      <c r="AG35" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4260,9 +4368,12 @@
         <v>1</v>
       </c>
       <c r="AE36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF36" t="n">
         <v>7</v>
       </c>
-      <c r="AF36" t="n">
+      <c r="AG36" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4369,6 +4480,9 @@
       <c r="AF37" t="n">
         <v>0</v>
       </c>
+      <c r="AG37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4468,9 +4582,12 @@
         <v>0</v>
       </c>
       <c r="AE38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF38" t="n">
         <v>2</v>
       </c>
-      <c r="AF38" t="n">
+      <c r="AG38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4572,9 +4689,12 @@
         <v>1</v>
       </c>
       <c r="AE39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF39" t="n">
         <v>14</v>
       </c>
-      <c r="AF39" t="n">
+      <c r="AG39" t="n">
         <v>14</v>
       </c>
     </row>
@@ -4676,9 +4796,12 @@
         <v>1</v>
       </c>
       <c r="AE40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF40" t="n">
         <v>13</v>
       </c>
-      <c r="AF40" t="n">
+      <c r="AG40" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4780,9 +4903,12 @@
         <v>1</v>
       </c>
       <c r="AE41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF41" t="n">
         <v>15</v>
       </c>
-      <c r="AF41" t="n">
+      <c r="AG41" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4884,9 +5010,12 @@
         <v>0</v>
       </c>
       <c r="AE42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF42" t="n">
         <v>21</v>
       </c>
-      <c r="AF42" t="n">
+      <c r="AG42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4988,9 +5117,12 @@
         <v>0</v>
       </c>
       <c r="AE43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF43" t="n">
         <v>49</v>
       </c>
-      <c r="AF43" t="n">
+      <c r="AG43" t="n">
         <v>8</v>
       </c>
     </row>
@@ -5092,9 +5224,12 @@
         <v>0</v>
       </c>
       <c r="AE44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF44" t="n">
         <v>11</v>
       </c>
-      <c r="AF44" t="n">
+      <c r="AG44" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5196,9 +5331,12 @@
         <v>1</v>
       </c>
       <c r="AE45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF45" t="n">
         <v>14</v>
       </c>
-      <c r="AF45" t="n">
+      <c r="AG45" t="n">
         <v>14</v>
       </c>
     </row>
@@ -5300,9 +5438,12 @@
         <v>1</v>
       </c>
       <c r="AE46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF46" t="n">
         <v>12</v>
       </c>
-      <c r="AF46" t="n">
+      <c r="AG46" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5409,6 +5550,9 @@
       <c r="AF47" t="n">
         <v>0</v>
       </c>
+      <c r="AG47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5508,9 +5652,12 @@
         <v>1</v>
       </c>
       <c r="AE48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF48" t="n">
         <v>14</v>
       </c>
-      <c r="AF48" t="n">
+      <c r="AG48" t="n">
         <v>14</v>
       </c>
     </row>
@@ -5612,9 +5759,12 @@
         <v>0</v>
       </c>
       <c r="AE49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF49" t="n">
         <v>12</v>
       </c>
-      <c r="AF49" t="n">
+      <c r="AG49" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5716,9 +5866,12 @@
         <v>0</v>
       </c>
       <c r="AE50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF50" t="n">
         <v>6</v>
       </c>
-      <c r="AF50" t="n">
+      <c r="AG50" t="n">
         <v>6</v>
       </c>
     </row>
@@ -5820,9 +5973,12 @@
         <v>1</v>
       </c>
       <c r="AE51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF51" t="n">
         <v>14</v>
       </c>
-      <c r="AF51" t="n">
+      <c r="AG51" t="n">
         <v>14</v>
       </c>
     </row>
@@ -5929,6 +6085,9 @@
       <c r="AF52" t="n">
         <v>0</v>
       </c>
+      <c r="AG52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6028,9 +6187,12 @@
         <v>1</v>
       </c>
       <c r="AE53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF53" t="n">
         <v>12</v>
       </c>
-      <c r="AF53" t="n">
+      <c r="AG53" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6137,6 +6299,9 @@
       <c r="AF54" t="n">
         <v>0</v>
       </c>
+      <c r="AG54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6236,9 +6401,12 @@
         <v>1</v>
       </c>
       <c r="AE55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF55" t="n">
         <v>13</v>
       </c>
-      <c r="AF55" t="n">
+      <c r="AG55" t="n">
         <v>13</v>
       </c>
     </row>
@@ -6340,9 +6508,12 @@
         <v>1</v>
       </c>
       <c r="AE56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF56" t="n">
         <v>13</v>
       </c>
-      <c r="AF56" t="n">
+      <c r="AG56" t="n">
         <v>13</v>
       </c>
     </row>
@@ -6444,9 +6615,12 @@
         <v>0</v>
       </c>
       <c r="AE57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF57" t="n">
         <v>7</v>
       </c>
-      <c r="AF57" t="n">
+      <c r="AG57" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6548,9 +6722,12 @@
         <v>0</v>
       </c>
       <c r="AE58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF58" t="n">
         <v>12</v>
       </c>
-      <c r="AF58" t="n">
+      <c r="AG58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6652,9 +6829,12 @@
         <v>0</v>
       </c>
       <c r="AE59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF59" t="n">
         <v>3</v>
       </c>
-      <c r="AF59" t="n">
+      <c r="AG59" t="n">
         <v>3</v>
       </c>
     </row>
@@ -6761,6 +6941,9 @@
       <c r="AF60" t="n">
         <v>0</v>
       </c>
+      <c r="AG60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6860,9 +7043,12 @@
         <v>1</v>
       </c>
       <c r="AE61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF61" t="n">
         <v>11</v>
       </c>
-      <c r="AF61" t="n">
+      <c r="AG61" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6964,9 +7150,12 @@
         <v>0</v>
       </c>
       <c r="AE62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF62" t="n">
         <v>13</v>
       </c>
-      <c r="AF62" t="n">
+      <c r="AG62" t="n">
         <v>13</v>
       </c>
     </row>
@@ -7068,9 +7257,12 @@
         <v>1</v>
       </c>
       <c r="AE63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF63" t="n">
         <v>3</v>
       </c>
-      <c r="AF63" t="n">
+      <c r="AG63" t="n">
         <v>3</v>
       </c>
     </row>
@@ -7177,6 +7369,9 @@
       <c r="AF64" t="n">
         <v>0</v>
       </c>
+      <c r="AG64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7276,9 +7471,12 @@
         <v>1</v>
       </c>
       <c r="AE65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF65" t="n">
         <v>6</v>
       </c>
-      <c r="AF65" t="n">
+      <c r="AG65" t="n">
         <v>6</v>
       </c>
     </row>
@@ -7380,9 +7578,12 @@
         <v>0</v>
       </c>
       <c r="AE66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7484,9 +7685,12 @@
         <v>1</v>
       </c>
       <c r="AE67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF67" t="n">
         <v>15</v>
       </c>
-      <c r="AF67" t="n">
+      <c r="AG67" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7588,9 +7792,12 @@
         <v>1</v>
       </c>
       <c r="AE68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF68" t="n">
         <v>7</v>
       </c>
-      <c r="AF68" t="n">
+      <c r="AG68" t="n">
         <v>6</v>
       </c>
     </row>
@@ -7692,9 +7899,12 @@
         <v>0</v>
       </c>
       <c r="AE69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF69" t="n">
         <v>7</v>
       </c>
-      <c r="AF69" t="n">
+      <c r="AG69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7796,9 +8006,12 @@
         <v>1</v>
       </c>
       <c r="AE70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF70" t="n">
         <v>22</v>
       </c>
-      <c r="AF70" t="n">
+      <c r="AG70" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7900,9 +8113,12 @@
         <v>1</v>
       </c>
       <c r="AE71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF71" t="n">
         <v>8</v>
       </c>
-      <c r="AF71" t="n">
+      <c r="AG71" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8004,9 +8220,12 @@
         <v>1</v>
       </c>
       <c r="AE72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF72" t="n">
         <v>12</v>
       </c>
-      <c r="AF72" t="n">
+      <c r="AG72" t="n">
         <v>12</v>
       </c>
     </row>
@@ -8113,6 +8332,9 @@
       <c r="AF73" t="n">
         <v>0</v>
       </c>
+      <c r="AG73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8217,6 +8439,9 @@
       <c r="AF74" t="n">
         <v>0</v>
       </c>
+      <c r="AG74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8316,9 +8541,12 @@
         <v>1</v>
       </c>
       <c r="AE75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF75" t="n">
         <v>8</v>
       </c>
-      <c r="AF75" t="n">
+      <c r="AG75" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8420,9 +8648,12 @@
         <v>1</v>
       </c>
       <c r="AE76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF76" t="n">
         <v>10</v>
       </c>
-      <c r="AF76" t="n">
+      <c r="AG76" t="n">
         <v>10</v>
       </c>
     </row>
@@ -8524,9 +8755,12 @@
         <v>0</v>
       </c>
       <c r="AE77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF77" t="n">
         <v>12</v>
       </c>
-      <c r="AF77" t="n">
+      <c r="AG77" t="n">
         <v>12</v>
       </c>
     </row>
@@ -8628,9 +8862,12 @@
         <v>0</v>
       </c>
       <c r="AE78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF78" t="n">
         <v>13</v>
       </c>
-      <c r="AF78" t="n">
+      <c r="AG78" t="n">
         <v>13</v>
       </c>
     </row>
@@ -8732,9 +8969,12 @@
         <v>1</v>
       </c>
       <c r="AE79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF79" t="n">
         <v>10</v>
       </c>
-      <c r="AF79" t="n">
+      <c r="AG79" t="n">
         <v>10</v>
       </c>
     </row>
@@ -8836,9 +9076,12 @@
         <v>1</v>
       </c>
       <c r="AE80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF80" t="n">
         <v>5</v>
       </c>
-      <c r="AF80" t="n">
+      <c r="AG80" t="n">
         <v>5</v>
       </c>
     </row>
@@ -8940,9 +9183,12 @@
         <v>0</v>
       </c>
       <c r="AE81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF81" t="n">
         <v>2</v>
       </c>
-      <c r="AF81" t="n">
+      <c r="AG81" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9044,9 +9290,12 @@
         <v>1</v>
       </c>
       <c r="AE82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF82" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG82" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9148,9 +9397,12 @@
         <v>1</v>
       </c>
       <c r="AE83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF83" t="n">
         <v>10</v>
       </c>
-      <c r="AF83" t="n">
+      <c r="AG83" t="n">
         <v>10</v>
       </c>
     </row>
@@ -9252,9 +9504,12 @@
         <v>0</v>
       </c>
       <c r="AE84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF84" t="n">
         <v>2</v>
       </c>
-      <c r="AF84" t="n">
+      <c r="AG84" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9356,9 +9611,12 @@
         <v>0</v>
       </c>
       <c r="AE85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF85" t="n">
         <v>7</v>
       </c>
-      <c r="AF85" t="n">
+      <c r="AG85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9465,6 +9723,9 @@
       <c r="AF86" t="n">
         <v>0</v>
       </c>
+      <c r="AG86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -9564,9 +9825,12 @@
         <v>0</v>
       </c>
       <c r="AE87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF87" t="n">
         <v>8</v>
       </c>
-      <c r="AF87" t="n">
+      <c r="AG87" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9673,6 +9937,9 @@
       <c r="AF88" t="n">
         <v>0</v>
       </c>
+      <c r="AG88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -9772,9 +10039,12 @@
         <v>0</v>
       </c>
       <c r="AE89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF89" t="n">
         <v>10</v>
       </c>
-      <c r="AF89" t="n">
+      <c r="AG89" t="n">
         <v>10</v>
       </c>
     </row>
@@ -9876,9 +10146,12 @@
         <v>0</v>
       </c>
       <c r="AE90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF90" t="n">
         <v>9</v>
       </c>
-      <c r="AF90" t="n">
+      <c r="AG90" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9980,9 +10253,12 @@
         <v>0</v>
       </c>
       <c r="AE91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF91" t="n">
         <v>37</v>
       </c>
-      <c r="AF91" t="n">
+      <c r="AG91" t="n">
         <v>8</v>
       </c>
     </row>
@@ -10084,9 +10360,12 @@
         <v>0</v>
       </c>
       <c r="AE92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF92" t="n">
         <v>4</v>
       </c>
-      <c r="AF92" t="n">
+      <c r="AG92" t="n">
         <v>4</v>
       </c>
     </row>
@@ -10193,6 +10472,9 @@
       <c r="AF93" t="n">
         <v>0</v>
       </c>
+      <c r="AG93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10292,9 +10574,12 @@
         <v>0</v>
       </c>
       <c r="AE94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF94" t="n">
         <v>7</v>
       </c>
-      <c r="AF94" t="n">
+      <c r="AG94" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10396,9 +10681,12 @@
         <v>0</v>
       </c>
       <c r="AE95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF95" t="n">
         <v>6</v>
       </c>
-      <c r="AF95" t="n">
+      <c r="AG95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10500,9 +10788,12 @@
         <v>1</v>
       </c>
       <c r="AE96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF96" t="n">
         <v>14</v>
       </c>
-      <c r="AF96" t="n">
+      <c r="AG96" t="n">
         <v>14</v>
       </c>
     </row>
@@ -10609,6 +10900,9 @@
       <c r="AF97" t="n">
         <v>0</v>
       </c>
+      <c r="AG97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -10708,9 +11002,12 @@
         <v>0</v>
       </c>
       <c r="AE98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF98" t="n">
         <v>15</v>
       </c>
-      <c r="AF98" t="n">
+      <c r="AG98" t="n">
         <v>15</v>
       </c>
     </row>
@@ -10812,9 +11109,12 @@
         <v>1</v>
       </c>
       <c r="AE99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF99" t="n">
         <v>2</v>
       </c>
-      <c r="AF99" t="n">
+      <c r="AG99" t="n">
         <v>2</v>
       </c>
     </row>
@@ -10921,6 +11221,9 @@
       <c r="AF100" t="n">
         <v>0</v>
       </c>
+      <c r="AG100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -11020,10 +11323,13 @@
         <v>0</v>
       </c>
       <c r="AE101" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AF101" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AG101" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="102">
@@ -11124,9 +11430,12 @@
         <v>1</v>
       </c>
       <c r="AE102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF102" t="n">
         <v>13</v>
       </c>
-      <c r="AF102" t="n">
+      <c r="AG102" t="n">
         <v>13</v>
       </c>
     </row>
@@ -11228,9 +11537,12 @@
         <v>1</v>
       </c>
       <c r="AE103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF103" t="n">
         <v>13</v>
       </c>
-      <c r="AF103" t="n">
+      <c r="AG103" t="n">
         <v>13</v>
       </c>
     </row>
@@ -11332,9 +11644,12 @@
         <v>1</v>
       </c>
       <c r="AE104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF104" t="n">
         <v>3</v>
       </c>
-      <c r="AF104" t="n">
+      <c r="AG104" t="n">
         <v>3</v>
       </c>
     </row>
@@ -11436,9 +11751,12 @@
         <v>1</v>
       </c>
       <c r="AE105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF105" t="n">
         <v>3</v>
       </c>
-      <c r="AF105" t="n">
+      <c r="AG105" t="n">
         <v>3</v>
       </c>
     </row>
@@ -11540,9 +11858,12 @@
         <v>1</v>
       </c>
       <c r="AE106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF106" t="n">
         <v>2</v>
       </c>
-      <c r="AF106" t="n">
+      <c r="AG106" t="n">
         <v>2</v>
       </c>
     </row>
@@ -11644,9 +11965,12 @@
         <v>1</v>
       </c>
       <c r="AE107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF107" t="n">
         <v>2</v>
       </c>
-      <c r="AF107" t="n">
+      <c r="AG107" t="n">
         <v>2</v>
       </c>
     </row>
@@ -11748,9 +12072,12 @@
         <v>0</v>
       </c>
       <c r="AE108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF108" t="n">
         <v>2</v>
       </c>
-      <c r="AF108" t="n">
+      <c r="AG108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -11855,6 +12182,9 @@
         <v>0</v>
       </c>
       <c r="AF109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2245)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG109"/>
+  <dimension ref="A1:AH109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -461,8 +461,9 @@
     <col width="12" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
     <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="13" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -621,12 +622,17 @@
           <t>2026-03-22</t>
         </is>
       </c>
-      <c r="AF1" s="2" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AG1" s="2" t="inlineStr">
+      <c r="AH1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -733,9 +739,12 @@
         <v>0</v>
       </c>
       <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
         <v>10</v>
       </c>
-      <c r="AG2" t="n">
+      <c r="AH2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -840,9 +849,12 @@
         <v>0</v>
       </c>
       <c r="AF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG3" t="n">
         <v>8</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="AH3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -947,10 +959,13 @@
         <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AG4" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -1054,9 +1069,12 @@
         <v>0</v>
       </c>
       <c r="AF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" t="n">
         <v>13</v>
       </c>
-      <c r="AG5" t="n">
+      <c r="AH5" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1161,10 +1179,13 @@
         <v>0</v>
       </c>
       <c r="AF6" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AG6" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -1268,10 +1289,13 @@
         <v>0</v>
       </c>
       <c r="AF7" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AG7" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -1375,10 +1399,13 @@
         <v>0</v>
       </c>
       <c r="AF8" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AG8" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -1482,9 +1509,12 @@
         <v>0</v>
       </c>
       <c r="AF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" t="n">
         <v>15</v>
       </c>
-      <c r="AG9" t="n">
+      <c r="AH9" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1589,10 +1619,13 @@
         <v>0</v>
       </c>
       <c r="AF10" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AG10" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="11">
@@ -1696,9 +1729,12 @@
         <v>0</v>
       </c>
       <c r="AF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="n">
         <v>13</v>
       </c>
-      <c r="AG11" t="n">
+      <c r="AH11" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1803,10 +1839,13 @@
         <v>0</v>
       </c>
       <c r="AF12" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AG12" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -1910,10 +1949,13 @@
         <v>0</v>
       </c>
       <c r="AF13" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AG13" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -2017,10 +2059,13 @@
         <v>0</v>
       </c>
       <c r="AF14" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AG14" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -2124,9 +2169,12 @@
         <v>0</v>
       </c>
       <c r="AF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG15" t="n">
         <v>9</v>
       </c>
-      <c r="AG15" t="n">
+      <c r="AH15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2231,10 +2279,13 @@
         <v>0</v>
       </c>
       <c r="AF16" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AG16" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="17">
@@ -2338,10 +2389,13 @@
         <v>0</v>
       </c>
       <c r="AF17" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AG17" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="18">
@@ -2445,10 +2499,13 @@
         <v>0</v>
       </c>
       <c r="AF18" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AG18" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="19">
@@ -2557,6 +2614,9 @@
       <c r="AG19" t="n">
         <v>0</v>
       </c>
+      <c r="AH19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2659,10 +2719,13 @@
         <v>0</v>
       </c>
       <c r="AF20" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AG20" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="21">
@@ -2766,10 +2829,13 @@
         <v>0</v>
       </c>
       <c r="AF21" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AG21" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="22">
@@ -2878,6 +2944,9 @@
       <c r="AG22" t="n">
         <v>0</v>
       </c>
+      <c r="AH22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2980,10 +3049,13 @@
         <v>0</v>
       </c>
       <c r="AF23" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AG23" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="24">
@@ -3087,10 +3159,13 @@
         <v>0</v>
       </c>
       <c r="AF24" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AG24" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="25">
@@ -3194,9 +3269,12 @@
         <v>0</v>
       </c>
       <c r="AF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG25" t="n">
         <v>6</v>
       </c>
-      <c r="AG25" t="n">
+      <c r="AH25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3301,10 +3379,13 @@
         <v>0</v>
       </c>
       <c r="AF26" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AG26" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="27">
@@ -3408,10 +3489,13 @@
         <v>0</v>
       </c>
       <c r="AF27" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AG27" t="n">
-        <v>13</v>
+        <v>16</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="28">
@@ -3515,10 +3599,13 @@
         <v>0</v>
       </c>
       <c r="AF28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AG28" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="29">
@@ -3622,9 +3709,12 @@
         <v>0</v>
       </c>
       <c r="AF29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG29" t="n">
         <v>5</v>
       </c>
-      <c r="AG29" t="n">
+      <c r="AH29" t="n">
         <v>5</v>
       </c>
     </row>
@@ -3729,9 +3819,12 @@
         <v>0</v>
       </c>
       <c r="AF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG30" t="n">
         <v>11</v>
       </c>
-      <c r="AG30" t="n">
+      <c r="AH30" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3836,9 +3929,12 @@
         <v>0</v>
       </c>
       <c r="AF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG31" t="n">
         <v>12</v>
       </c>
-      <c r="AG31" t="n">
+      <c r="AH31" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3943,9 +4039,12 @@
         <v>0</v>
       </c>
       <c r="AF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG32" t="n">
         <v>11</v>
       </c>
-      <c r="AG32" t="n">
+      <c r="AH32" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4050,9 +4149,12 @@
         <v>0</v>
       </c>
       <c r="AF33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG33" t="n">
         <v>12</v>
       </c>
-      <c r="AG33" t="n">
+      <c r="AH33" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4157,10 +4259,13 @@
         <v>0</v>
       </c>
       <c r="AF34" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG34" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AH34" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="35">
@@ -4264,9 +4369,12 @@
         <v>0</v>
       </c>
       <c r="AF35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG35" t="n">
         <v>11</v>
       </c>
-      <c r="AG35" t="n">
+      <c r="AH35" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4371,10 +4479,13 @@
         <v>0</v>
       </c>
       <c r="AF36" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AG36" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AH36" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="37">
@@ -4483,6 +4594,9 @@
       <c r="AG37" t="n">
         <v>0</v>
       </c>
+      <c r="AH37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4585,9 +4699,12 @@
         <v>0</v>
       </c>
       <c r="AF38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG38" t="n">
         <v>2</v>
       </c>
-      <c r="AG38" t="n">
+      <c r="AH38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4692,10 +4809,13 @@
         <v>0</v>
       </c>
       <c r="AF39" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AG39" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AH39" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="40">
@@ -4799,10 +4919,13 @@
         <v>0</v>
       </c>
       <c r="AF40" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AG40" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AH40" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="41">
@@ -4906,10 +5029,13 @@
         <v>0</v>
       </c>
       <c r="AF41" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AG41" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AH41" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="42">
@@ -5013,9 +5139,12 @@
         <v>0</v>
       </c>
       <c r="AF42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG42" t="n">
         <v>21</v>
       </c>
-      <c r="AG42" t="n">
+      <c r="AH42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5120,10 +5249,13 @@
         <v>0</v>
       </c>
       <c r="AF43" t="n">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="AG43" t="n">
-        <v>8</v>
+        <v>50</v>
+      </c>
+      <c r="AH43" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="44">
@@ -5227,10 +5359,13 @@
         <v>0</v>
       </c>
       <c r="AF44" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AG44" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AH44" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="45">
@@ -5334,10 +5469,13 @@
         <v>0</v>
       </c>
       <c r="AF45" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AG45" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AH45" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="46">
@@ -5441,10 +5579,13 @@
         <v>0</v>
       </c>
       <c r="AF46" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AG46" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AH46" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="47">
@@ -5553,6 +5694,9 @@
       <c r="AG47" t="n">
         <v>0</v>
       </c>
+      <c r="AH47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5655,10 +5799,13 @@
         <v>0</v>
       </c>
       <c r="AF48" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AG48" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AH48" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="49">
@@ -5762,9 +5909,12 @@
         <v>0</v>
       </c>
       <c r="AF49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG49" t="n">
         <v>12</v>
       </c>
-      <c r="AG49" t="n">
+      <c r="AH49" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5869,9 +6019,12 @@
         <v>0</v>
       </c>
       <c r="AF50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG50" t="n">
         <v>6</v>
       </c>
-      <c r="AG50" t="n">
+      <c r="AH50" t="n">
         <v>6</v>
       </c>
     </row>
@@ -5976,10 +6129,13 @@
         <v>0</v>
       </c>
       <c r="AF51" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AG51" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AH51" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="52">
@@ -6088,6 +6244,9 @@
       <c r="AG52" t="n">
         <v>0</v>
       </c>
+      <c r="AH52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6190,9 +6349,12 @@
         <v>0</v>
       </c>
       <c r="AF53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG53" t="n">
         <v>12</v>
       </c>
-      <c r="AG53" t="n">
+      <c r="AH53" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6302,6 +6464,9 @@
       <c r="AG54" t="n">
         <v>0</v>
       </c>
+      <c r="AH54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6404,10 +6569,13 @@
         <v>0</v>
       </c>
       <c r="AF55" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AG55" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AH55" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="56">
@@ -6511,10 +6679,13 @@
         <v>0</v>
       </c>
       <c r="AF56" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AG56" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AH56" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="57">
@@ -6618,10 +6789,13 @@
         <v>0</v>
       </c>
       <c r="AF57" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AG57" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AH57" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="58">
@@ -6725,9 +6899,12 @@
         <v>0</v>
       </c>
       <c r="AF58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG58" t="n">
         <v>12</v>
       </c>
-      <c r="AG58" t="n">
+      <c r="AH58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6832,9 +7009,12 @@
         <v>0</v>
       </c>
       <c r="AF59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG59" t="n">
         <v>3</v>
       </c>
-      <c r="AG59" t="n">
+      <c r="AH59" t="n">
         <v>3</v>
       </c>
     </row>
@@ -6944,6 +7124,9 @@
       <c r="AG60" t="n">
         <v>0</v>
       </c>
+      <c r="AH60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7046,10 +7229,13 @@
         <v>0</v>
       </c>
       <c r="AF61" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AG61" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AH61" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="62">
@@ -7153,10 +7339,13 @@
         <v>0</v>
       </c>
       <c r="AF62" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AG62" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AH62" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="63">
@@ -7260,10 +7449,13 @@
         <v>0</v>
       </c>
       <c r="AF63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AG63" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AH63" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="64">
@@ -7372,6 +7564,9 @@
       <c r="AG64" t="n">
         <v>0</v>
       </c>
+      <c r="AH64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7474,10 +7669,13 @@
         <v>0</v>
       </c>
       <c r="AF65" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG65" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AH65" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="66">
@@ -7581,9 +7779,12 @@
         <v>0</v>
       </c>
       <c r="AF66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7688,10 +7889,13 @@
         <v>0</v>
       </c>
       <c r="AF67" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AG67" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AH67" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="68">
@@ -7795,9 +7999,12 @@
         <v>0</v>
       </c>
       <c r="AF68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG68" t="n">
         <v>7</v>
       </c>
-      <c r="AG68" t="n">
+      <c r="AH68" t="n">
         <v>6</v>
       </c>
     </row>
@@ -7902,9 +8109,12 @@
         <v>0</v>
       </c>
       <c r="AF69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG69" t="n">
         <v>7</v>
       </c>
-      <c r="AG69" t="n">
+      <c r="AH69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8009,9 +8219,12 @@
         <v>0</v>
       </c>
       <c r="AF70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG70" t="n">
         <v>22</v>
       </c>
-      <c r="AG70" t="n">
+      <c r="AH70" t="n">
         <v>10</v>
       </c>
     </row>
@@ -8116,10 +8329,13 @@
         <v>0</v>
       </c>
       <c r="AF71" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AG71" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AH71" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="72">
@@ -8223,9 +8439,12 @@
         <v>0</v>
       </c>
       <c r="AF72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG72" t="n">
         <v>12</v>
       </c>
-      <c r="AG72" t="n">
+      <c r="AH72" t="n">
         <v>12</v>
       </c>
     </row>
@@ -8335,6 +8554,9 @@
       <c r="AG73" t="n">
         <v>0</v>
       </c>
+      <c r="AH73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8442,6 +8664,9 @@
       <c r="AG74" t="n">
         <v>0</v>
       </c>
+      <c r="AH74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8544,10 +8769,13 @@
         <v>0</v>
       </c>
       <c r="AF75" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AG75" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AH75" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="76">
@@ -8651,9 +8879,12 @@
         <v>0</v>
       </c>
       <c r="AF76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG76" t="n">
         <v>10</v>
       </c>
-      <c r="AG76" t="n">
+      <c r="AH76" t="n">
         <v>10</v>
       </c>
     </row>
@@ -8758,10 +8989,13 @@
         <v>0</v>
       </c>
       <c r="AF77" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AG77" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AH77" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="78">
@@ -8865,10 +9099,13 @@
         <v>0</v>
       </c>
       <c r="AF78" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AG78" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AH78" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="79">
@@ -8972,10 +9209,13 @@
         <v>0</v>
       </c>
       <c r="AF79" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AG79" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AH79" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="80">
@@ -9079,9 +9319,12 @@
         <v>0</v>
       </c>
       <c r="AF80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG80" t="n">
         <v>5</v>
       </c>
-      <c r="AG80" t="n">
+      <c r="AH80" t="n">
         <v>5</v>
       </c>
     </row>
@@ -9186,9 +9429,12 @@
         <v>0</v>
       </c>
       <c r="AF81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG81" t="n">
         <v>2</v>
       </c>
-      <c r="AG81" t="n">
+      <c r="AH81" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9296,7 +9542,10 @@
         <v>1</v>
       </c>
       <c r="AG82" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AH82" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="83">
@@ -9400,10 +9649,13 @@
         <v>0</v>
       </c>
       <c r="AF83" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AG83" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AH83" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="84">
@@ -9507,10 +9759,13 @@
         <v>0</v>
       </c>
       <c r="AF84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG84" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AH84" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="85">
@@ -9614,9 +9869,12 @@
         <v>0</v>
       </c>
       <c r="AF85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG85" t="n">
         <v>7</v>
       </c>
-      <c r="AG85" t="n">
+      <c r="AH85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9726,6 +9984,9 @@
       <c r="AG86" t="n">
         <v>0</v>
       </c>
+      <c r="AH86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -9828,9 +10089,12 @@
         <v>0</v>
       </c>
       <c r="AF87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG87" t="n">
         <v>8</v>
       </c>
-      <c r="AG87" t="n">
+      <c r="AH87" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9940,6 +10204,9 @@
       <c r="AG88" t="n">
         <v>0</v>
       </c>
+      <c r="AH88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -10042,10 +10309,13 @@
         <v>0</v>
       </c>
       <c r="AF89" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AG89" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AH89" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="90">
@@ -10149,10 +10419,13 @@
         <v>0</v>
       </c>
       <c r="AF90" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AG90" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AH90" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="91">
@@ -10256,10 +10529,13 @@
         <v>0</v>
       </c>
       <c r="AF91" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="AG91" t="n">
-        <v>8</v>
+        <v>38</v>
+      </c>
+      <c r="AH91" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="92">
@@ -10363,10 +10639,13 @@
         <v>0</v>
       </c>
       <c r="AF92" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AG92" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AH92" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="93">
@@ -10475,6 +10754,9 @@
       <c r="AG93" t="n">
         <v>0</v>
       </c>
+      <c r="AH93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10577,10 +10859,13 @@
         <v>0</v>
       </c>
       <c r="AF94" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AG94" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AH94" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="95">
@@ -10684,9 +10969,12 @@
         <v>0</v>
       </c>
       <c r="AF95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG95" t="n">
         <v>6</v>
       </c>
-      <c r="AG95" t="n">
+      <c r="AH95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10791,9 +11079,12 @@
         <v>0</v>
       </c>
       <c r="AF96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG96" t="n">
         <v>14</v>
       </c>
-      <c r="AG96" t="n">
+      <c r="AH96" t="n">
         <v>14</v>
       </c>
     </row>
@@ -10903,6 +11194,9 @@
       <c r="AG97" t="n">
         <v>0</v>
       </c>
+      <c r="AH97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -11005,10 +11299,13 @@
         <v>0</v>
       </c>
       <c r="AF98" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AG98" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AH98" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="99">
@@ -11112,10 +11409,13 @@
         <v>0</v>
       </c>
       <c r="AF99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG99" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AH99" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="100">
@@ -11224,6 +11524,9 @@
       <c r="AG100" t="n">
         <v>0</v>
       </c>
+      <c r="AH100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -11326,10 +11629,13 @@
         <v>1</v>
       </c>
       <c r="AF101" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AG101" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AH101" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="102">
@@ -11433,10 +11739,13 @@
         <v>0</v>
       </c>
       <c r="AF102" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AG102" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AH102" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="103">
@@ -11540,10 +11849,13 @@
         <v>0</v>
       </c>
       <c r="AF103" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AG103" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AH103" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="104">
@@ -11647,9 +11959,12 @@
         <v>0</v>
       </c>
       <c r="AF104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG104" t="n">
         <v>3</v>
       </c>
-      <c r="AG104" t="n">
+      <c r="AH104" t="n">
         <v>3</v>
       </c>
     </row>
@@ -11754,10 +12069,13 @@
         <v>0</v>
       </c>
       <c r="AF105" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AG105" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AH105" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="106">
@@ -11861,10 +12179,13 @@
         <v>0</v>
       </c>
       <c r="AF106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG106" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AH106" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="107">
@@ -11968,9 +12289,12 @@
         <v>0</v>
       </c>
       <c r="AF107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG107" t="n">
         <v>2</v>
       </c>
-      <c r="AG107" t="n">
+      <c r="AH107" t="n">
         <v>2</v>
       </c>
     </row>
@@ -12075,9 +12399,12 @@
         <v>0</v>
       </c>
       <c r="AF108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG108" t="n">
         <v>2</v>
       </c>
-      <c r="AG108" t="n">
+      <c r="AH108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -12185,6 +12512,9 @@
         <v>0</v>
       </c>
       <c r="AG109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH109" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2333)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH109"/>
+  <dimension ref="A1:AI109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -462,8 +462,9 @@
     <col width="12" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
     <col width="12" customWidth="1" min="32" max="32"/>
-    <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
     <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -627,12 +628,17 @@
           <t>2026-03-23</t>
         </is>
       </c>
-      <c r="AG1" s="2" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="AH1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AH1" s="2" t="inlineStr">
+      <c r="AI1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -742,9 +748,12 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" t="n">
         <v>10</v>
       </c>
-      <c r="AH2" t="n">
+      <c r="AI2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -852,9 +861,12 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH3" t="n">
         <v>8</v>
       </c>
-      <c r="AH3" t="n">
+      <c r="AI3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -962,10 +974,13 @@
         <v>1</v>
       </c>
       <c r="AG4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AH4" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -1072,10 +1087,13 @@
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AH5" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -1182,9 +1200,12 @@
         <v>1</v>
       </c>
       <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="n">
         <v>13</v>
       </c>
-      <c r="AH6" t="n">
+      <c r="AI6" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1292,10 +1313,13 @@
         <v>1</v>
       </c>
       <c r="AG7" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AH7" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -1402,10 +1426,13 @@
         <v>1</v>
       </c>
       <c r="AG8" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AH8" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -1512,10 +1539,13 @@
         <v>0</v>
       </c>
       <c r="AG9" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AH9" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -1622,10 +1652,13 @@
         <v>1</v>
       </c>
       <c r="AG10" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AH10" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="11">
@@ -1732,9 +1765,12 @@
         <v>0</v>
       </c>
       <c r="AG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" t="n">
         <v>13</v>
       </c>
-      <c r="AH11" t="n">
+      <c r="AI11" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1842,10 +1878,13 @@
         <v>1</v>
       </c>
       <c r="AG12" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AH12" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="13">
@@ -1952,9 +1991,12 @@
         <v>1</v>
       </c>
       <c r="AG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH13" t="n">
         <v>9</v>
       </c>
-      <c r="AH13" t="n">
+      <c r="AI13" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2062,10 +2104,13 @@
         <v>1</v>
       </c>
       <c r="AG14" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AH14" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="15">
@@ -2172,9 +2217,12 @@
         <v>0</v>
       </c>
       <c r="AG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH15" t="n">
         <v>9</v>
       </c>
-      <c r="AH15" t="n">
+      <c r="AI15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2282,9 +2330,12 @@
         <v>1</v>
       </c>
       <c r="AG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH16" t="n">
         <v>13</v>
       </c>
-      <c r="AH16" t="n">
+      <c r="AI16" t="n">
         <v>13</v>
       </c>
     </row>
@@ -2392,9 +2443,12 @@
         <v>1</v>
       </c>
       <c r="AG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH17" t="n">
         <v>13</v>
       </c>
-      <c r="AH17" t="n">
+      <c r="AI17" t="n">
         <v>13</v>
       </c>
     </row>
@@ -2502,10 +2556,13 @@
         <v>1</v>
       </c>
       <c r="AG18" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AH18" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="19">
@@ -2617,6 +2674,9 @@
       <c r="AH19" t="n">
         <v>0</v>
       </c>
+      <c r="AI19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2722,10 +2782,13 @@
         <v>1</v>
       </c>
       <c r="AG20" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AH20" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="21">
@@ -2832,10 +2895,13 @@
         <v>1</v>
       </c>
       <c r="AG21" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AH21" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="22">
@@ -2947,6 +3013,9 @@
       <c r="AH22" t="n">
         <v>0</v>
       </c>
+      <c r="AI22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3052,10 +3121,13 @@
         <v>1</v>
       </c>
       <c r="AG23" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AH23" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="24">
@@ -3162,10 +3234,13 @@
         <v>1</v>
       </c>
       <c r="AG24" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AH24" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AI24" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="25">
@@ -3272,9 +3347,12 @@
         <v>0</v>
       </c>
       <c r="AG25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH25" t="n">
         <v>6</v>
       </c>
-      <c r="AH25" t="n">
+      <c r="AI25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3382,10 +3460,13 @@
         <v>1</v>
       </c>
       <c r="AG26" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AH26" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="27">
@@ -3492,10 +3573,13 @@
         <v>1</v>
       </c>
       <c r="AG27" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AH27" t="n">
-        <v>14</v>
+        <v>17</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="28">
@@ -3602,10 +3686,13 @@
         <v>1</v>
       </c>
       <c r="AG28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AH28" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AI28" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -3712,10 +3799,13 @@
         <v>0</v>
       </c>
       <c r="AG29" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AH29" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AI29" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="30">
@@ -3822,9 +3912,12 @@
         <v>0</v>
       </c>
       <c r="AG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH30" t="n">
         <v>11</v>
       </c>
-      <c r="AH30" t="n">
+      <c r="AI30" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3932,10 +4025,13 @@
         <v>0</v>
       </c>
       <c r="AG31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AH31" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="32">
@@ -4042,9 +4138,12 @@
         <v>0</v>
       </c>
       <c r="AG32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH32" t="n">
         <v>11</v>
       </c>
-      <c r="AH32" t="n">
+      <c r="AI32" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4152,9 +4251,12 @@
         <v>0</v>
       </c>
       <c r="AG33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH33" t="n">
         <v>12</v>
       </c>
-      <c r="AH33" t="n">
+      <c r="AI33" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4262,9 +4364,12 @@
         <v>1</v>
       </c>
       <c r="AG34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH34" t="n">
         <v>7</v>
       </c>
-      <c r="AH34" t="n">
+      <c r="AI34" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4372,10 +4477,13 @@
         <v>0</v>
       </c>
       <c r="AG35" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AH35" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AI35" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="36">
@@ -4482,10 +4590,13 @@
         <v>1</v>
       </c>
       <c r="AG36" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AH36" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AI36" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="37">
@@ -4597,6 +4708,9 @@
       <c r="AH37" t="n">
         <v>0</v>
       </c>
+      <c r="AI37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4702,9 +4816,12 @@
         <v>0</v>
       </c>
       <c r="AG38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH38" t="n">
         <v>2</v>
       </c>
-      <c r="AH38" t="n">
+      <c r="AI38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4812,10 +4929,13 @@
         <v>1</v>
       </c>
       <c r="AG39" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AH39" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AI39" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="40">
@@ -4922,9 +5042,12 @@
         <v>1</v>
       </c>
       <c r="AG40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH40" t="n">
         <v>14</v>
       </c>
-      <c r="AH40" t="n">
+      <c r="AI40" t="n">
         <v>14</v>
       </c>
     </row>
@@ -5032,10 +5155,13 @@
         <v>1</v>
       </c>
       <c r="AG41" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AH41" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AI41" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="42">
@@ -5142,9 +5268,12 @@
         <v>0</v>
       </c>
       <c r="AG42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH42" t="n">
         <v>21</v>
       </c>
-      <c r="AH42" t="n">
+      <c r="AI42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5252,10 +5381,13 @@
         <v>1</v>
       </c>
       <c r="AG43" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="AH43" t="n">
-        <v>9</v>
+        <v>51</v>
+      </c>
+      <c r="AI43" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="44">
@@ -5362,10 +5494,13 @@
         <v>1</v>
       </c>
       <c r="AG44" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AH44" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AI44" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="45">
@@ -5472,10 +5607,13 @@
         <v>1</v>
       </c>
       <c r="AG45" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AH45" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AI45" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="46">
@@ -5582,10 +5720,13 @@
         <v>1</v>
       </c>
       <c r="AG46" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AH46" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AI46" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="47">
@@ -5697,6 +5838,9 @@
       <c r="AH47" t="n">
         <v>0</v>
       </c>
+      <c r="AI47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5802,9 +5946,12 @@
         <v>1</v>
       </c>
       <c r="AG48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH48" t="n">
         <v>15</v>
       </c>
-      <c r="AH48" t="n">
+      <c r="AI48" t="n">
         <v>15</v>
       </c>
     </row>
@@ -5912,10 +6059,13 @@
         <v>0</v>
       </c>
       <c r="AG49" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AH49" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AI49" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="50">
@@ -6022,10 +6172,13 @@
         <v>0</v>
       </c>
       <c r="AG50" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AH50" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AI50" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="51">
@@ -6132,10 +6285,13 @@
         <v>1</v>
       </c>
       <c r="AG51" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AH51" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AI51" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="52">
@@ -6247,6 +6403,9 @@
       <c r="AH52" t="n">
         <v>0</v>
       </c>
+      <c r="AI52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6352,9 +6511,12 @@
         <v>0</v>
       </c>
       <c r="AG53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH53" t="n">
         <v>12</v>
       </c>
-      <c r="AH53" t="n">
+      <c r="AI53" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6467,6 +6629,9 @@
       <c r="AH54" t="n">
         <v>0</v>
       </c>
+      <c r="AI54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6572,10 +6737,13 @@
         <v>1</v>
       </c>
       <c r="AG55" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AH55" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AI55" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="56">
@@ -6682,10 +6850,13 @@
         <v>1</v>
       </c>
       <c r="AG56" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AH56" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AI56" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="57">
@@ -6792,9 +6963,12 @@
         <v>1</v>
       </c>
       <c r="AG57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH57" t="n">
         <v>8</v>
       </c>
-      <c r="AH57" t="n">
+      <c r="AI57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -6902,9 +7076,12 @@
         <v>0</v>
       </c>
       <c r="AG58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH58" t="n">
         <v>12</v>
       </c>
-      <c r="AH58" t="n">
+      <c r="AI58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7012,9 +7189,12 @@
         <v>0</v>
       </c>
       <c r="AG59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH59" t="n">
         <v>3</v>
       </c>
-      <c r="AH59" t="n">
+      <c r="AI59" t="n">
         <v>3</v>
       </c>
     </row>
@@ -7127,6 +7307,9 @@
       <c r="AH60" t="n">
         <v>0</v>
       </c>
+      <c r="AI60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7232,10 +7415,13 @@
         <v>1</v>
       </c>
       <c r="AG61" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AH61" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AI61" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="62">
@@ -7342,10 +7528,13 @@
         <v>1</v>
       </c>
       <c r="AG62" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AH62" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AI62" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="63">
@@ -7452,10 +7641,13 @@
         <v>1</v>
       </c>
       <c r="AG63" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AH63" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AI63" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="64">
@@ -7567,6 +7759,9 @@
       <c r="AH64" t="n">
         <v>0</v>
       </c>
+      <c r="AI64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7672,10 +7867,13 @@
         <v>1</v>
       </c>
       <c r="AG65" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AH65" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AI65" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="66">
@@ -7782,9 +7980,12 @@
         <v>0</v>
       </c>
       <c r="AG66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7892,10 +8093,13 @@
         <v>1</v>
       </c>
       <c r="AG67" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AH67" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AI67" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="68">
@@ -8002,10 +8206,13 @@
         <v>0</v>
       </c>
       <c r="AG68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH68" t="n">
+        <v>8</v>
+      </c>
+      <c r="AI68" t="n">
         <v>7</v>
-      </c>
-      <c r="AH68" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="69">
@@ -8112,9 +8319,12 @@
         <v>0</v>
       </c>
       <c r="AG69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH69" t="n">
         <v>7</v>
       </c>
-      <c r="AH69" t="n">
+      <c r="AI69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8222,10 +8432,13 @@
         <v>0</v>
       </c>
       <c r="AG70" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AH70" t="n">
-        <v>10</v>
+        <v>23</v>
+      </c>
+      <c r="AI70" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="71">
@@ -8332,10 +8545,13 @@
         <v>1</v>
       </c>
       <c r="AG71" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AH71" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AI71" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="72">
@@ -8442,10 +8658,13 @@
         <v>0</v>
       </c>
       <c r="AG72" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AH72" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AI72" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="73">
@@ -8557,6 +8776,9 @@
       <c r="AH73" t="n">
         <v>0</v>
       </c>
+      <c r="AI73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8667,6 +8889,9 @@
       <c r="AH74" t="n">
         <v>0</v>
       </c>
+      <c r="AI74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8772,10 +8997,13 @@
         <v>1</v>
       </c>
       <c r="AG75" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AH75" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AI75" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="76">
@@ -8882,9 +9110,12 @@
         <v>0</v>
       </c>
       <c r="AG76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH76" t="n">
         <v>10</v>
       </c>
-      <c r="AH76" t="n">
+      <c r="AI76" t="n">
         <v>10</v>
       </c>
     </row>
@@ -8992,9 +9223,12 @@
         <v>1</v>
       </c>
       <c r="AG77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH77" t="n">
         <v>13</v>
       </c>
-      <c r="AH77" t="n">
+      <c r="AI77" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9102,10 +9336,13 @@
         <v>1</v>
       </c>
       <c r="AG78" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AH78" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AI78" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="79">
@@ -9212,10 +9449,13 @@
         <v>1</v>
       </c>
       <c r="AG79" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AH79" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AI79" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="80">
@@ -9322,10 +9562,13 @@
         <v>0</v>
       </c>
       <c r="AG80" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AH80" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AI80" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="81">
@@ -9432,9 +9675,12 @@
         <v>0</v>
       </c>
       <c r="AG81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH81" t="n">
         <v>2</v>
       </c>
-      <c r="AH81" t="n">
+      <c r="AI81" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9542,10 +9788,13 @@
         <v>1</v>
       </c>
       <c r="AG82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH82" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AI82" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="83">
@@ -9652,10 +9901,13 @@
         <v>1</v>
       </c>
       <c r="AG83" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AH83" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AI83" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="84">
@@ -9762,10 +10014,13 @@
         <v>1</v>
       </c>
       <c r="AG84" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AH84" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AI84" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="85">
@@ -9872,9 +10127,12 @@
         <v>0</v>
       </c>
       <c r="AG85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH85" t="n">
         <v>7</v>
       </c>
-      <c r="AH85" t="n">
+      <c r="AI85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9987,6 +10245,9 @@
       <c r="AH86" t="n">
         <v>0</v>
       </c>
+      <c r="AI86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -10092,10 +10353,13 @@
         <v>0</v>
       </c>
       <c r="AG87" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AH87" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AI87" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="88">
@@ -10207,6 +10471,9 @@
       <c r="AH88" t="n">
         <v>0</v>
       </c>
+      <c r="AI88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -10312,10 +10579,13 @@
         <v>1</v>
       </c>
       <c r="AG89" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AH89" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AI89" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="90">
@@ -10422,10 +10692,13 @@
         <v>1</v>
       </c>
       <c r="AG90" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AH90" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AI90" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="91">
@@ -10532,10 +10805,13 @@
         <v>1</v>
       </c>
       <c r="AG91" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="AH91" t="n">
-        <v>9</v>
+        <v>39</v>
+      </c>
+      <c r="AI91" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="92">
@@ -10642,9 +10918,12 @@
         <v>1</v>
       </c>
       <c r="AG92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH92" t="n">
         <v>5</v>
       </c>
-      <c r="AH92" t="n">
+      <c r="AI92" t="n">
         <v>5</v>
       </c>
     </row>
@@ -10757,6 +11036,9 @@
       <c r="AH93" t="n">
         <v>0</v>
       </c>
+      <c r="AI93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10862,9 +11144,12 @@
         <v>1</v>
       </c>
       <c r="AG94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH94" t="n">
         <v>8</v>
       </c>
-      <c r="AH94" t="n">
+      <c r="AI94" t="n">
         <v>8</v>
       </c>
     </row>
@@ -10972,9 +11257,12 @@
         <v>0</v>
       </c>
       <c r="AG95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH95" t="n">
         <v>6</v>
       </c>
-      <c r="AH95" t="n">
+      <c r="AI95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -11082,9 +11370,12 @@
         <v>0</v>
       </c>
       <c r="AG96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH96" t="n">
         <v>14</v>
       </c>
-      <c r="AH96" t="n">
+      <c r="AI96" t="n">
         <v>14</v>
       </c>
     </row>
@@ -11197,6 +11488,9 @@
       <c r="AH97" t="n">
         <v>0</v>
       </c>
+      <c r="AI97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -11302,10 +11596,13 @@
         <v>1</v>
       </c>
       <c r="AG98" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AH98" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AI98" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="99">
@@ -11412,9 +11709,12 @@
         <v>1</v>
       </c>
       <c r="AG99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH99" t="n">
         <v>3</v>
       </c>
-      <c r="AH99" t="n">
+      <c r="AI99" t="n">
         <v>3</v>
       </c>
     </row>
@@ -11527,6 +11827,9 @@
       <c r="AH100" t="n">
         <v>0</v>
       </c>
+      <c r="AI100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -11632,10 +11935,13 @@
         <v>1</v>
       </c>
       <c r="AG101" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AH101" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AI101" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="102">
@@ -11742,10 +12048,13 @@
         <v>1</v>
       </c>
       <c r="AG102" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AH102" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AI102" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="103">
@@ -11852,10 +12161,13 @@
         <v>1</v>
       </c>
       <c r="AG103" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AH103" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AI103" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="104">
@@ -11962,10 +12274,13 @@
         <v>0</v>
       </c>
       <c r="AG104" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AH104" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AI104" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="105">
@@ -12072,10 +12387,13 @@
         <v>1</v>
       </c>
       <c r="AG105" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AH105" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AI105" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="106">
@@ -12182,10 +12500,13 @@
         <v>1</v>
       </c>
       <c r="AG106" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AH106" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AI106" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="107">
@@ -12292,10 +12613,13 @@
         <v>0</v>
       </c>
       <c r="AG107" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH107" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AI107" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="108">
@@ -12402,9 +12726,12 @@
         <v>0</v>
       </c>
       <c r="AG108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH108" t="n">
         <v>2</v>
       </c>
-      <c r="AH108" t="n">
+      <c r="AI108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -12512,10 +12839,13 @@
         <v>0</v>
       </c>
       <c r="AG109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH109" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AI109" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2405)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI109"/>
+  <dimension ref="A1:AJ109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -463,8 +463,9 @@
     <col width="12" customWidth="1" min="31" max="31"/>
     <col width="12" customWidth="1" min="32" max="32"/>
     <col width="12" customWidth="1" min="33" max="33"/>
-    <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
     <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -633,12 +634,17 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="AH1" s="2" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="AI1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AI1" s="2" t="inlineStr">
+      <c r="AJ1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -751,9 +757,12 @@
         <v>0</v>
       </c>
       <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="n">
         <v>10</v>
       </c>
-      <c r="AI2" t="n">
+      <c r="AJ2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -864,9 +873,12 @@
         <v>0</v>
       </c>
       <c r="AH3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI3" t="n">
         <v>8</v>
       </c>
-      <c r="AI3" t="n">
+      <c r="AJ3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -977,10 +989,13 @@
         <v>1</v>
       </c>
       <c r="AH4" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AI4" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -1090,9 +1105,12 @@
         <v>1</v>
       </c>
       <c r="AH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" t="n">
         <v>14</v>
       </c>
-      <c r="AI5" t="n">
+      <c r="AJ5" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1203,9 +1221,12 @@
         <v>0</v>
       </c>
       <c r="AH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" t="n">
         <v>13</v>
       </c>
-      <c r="AI6" t="n">
+      <c r="AJ6" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1316,9 +1337,12 @@
         <v>1</v>
       </c>
       <c r="AH7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI7" t="n">
         <v>13</v>
       </c>
-      <c r="AI7" t="n">
+      <c r="AJ7" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1429,10 +1453,13 @@
         <v>1</v>
       </c>
       <c r="AH8" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AI8" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1542,10 +1569,13 @@
         <v>1</v>
       </c>
       <c r="AH9" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AI9" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -1655,10 +1685,13 @@
         <v>1</v>
       </c>
       <c r="AH10" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AI10" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="11">
@@ -1768,10 +1801,13 @@
         <v>0</v>
       </c>
       <c r="AH11" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AI11" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -1881,10 +1917,13 @@
         <v>1</v>
       </c>
       <c r="AH12" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AI12" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="13">
@@ -1994,9 +2033,12 @@
         <v>0</v>
       </c>
       <c r="AH13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI13" t="n">
         <v>9</v>
       </c>
-      <c r="AI13" t="n">
+      <c r="AJ13" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2107,10 +2149,13 @@
         <v>1</v>
       </c>
       <c r="AH14" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AI14" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="15">
@@ -2220,9 +2265,12 @@
         <v>0</v>
       </c>
       <c r="AH15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI15" t="n">
         <v>9</v>
       </c>
-      <c r="AI15" t="n">
+      <c r="AJ15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2333,10 +2381,13 @@
         <v>0</v>
       </c>
       <c r="AH16" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AI16" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="17">
@@ -2446,10 +2497,13 @@
         <v>0</v>
       </c>
       <c r="AH17" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AI17" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="18">
@@ -2559,10 +2613,13 @@
         <v>1</v>
       </c>
       <c r="AH18" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AI18" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="19">
@@ -2677,6 +2734,9 @@
       <c r="AI19" t="n">
         <v>0</v>
       </c>
+      <c r="AJ19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2785,9 +2845,12 @@
         <v>1</v>
       </c>
       <c r="AH20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI20" t="n">
         <v>13</v>
       </c>
-      <c r="AI20" t="n">
+      <c r="AJ20" t="n">
         <v>13</v>
       </c>
     </row>
@@ -2898,10 +2961,13 @@
         <v>1</v>
       </c>
       <c r="AH21" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AI21" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="22">
@@ -3016,6 +3082,9 @@
       <c r="AI22" t="n">
         <v>0</v>
       </c>
+      <c r="AJ22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3124,9 +3193,12 @@
         <v>1</v>
       </c>
       <c r="AH23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI23" t="n">
         <v>9</v>
       </c>
-      <c r="AI23" t="n">
+      <c r="AJ23" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3237,10 +3309,13 @@
         <v>1</v>
       </c>
       <c r="AH24" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AI24" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="25">
@@ -3350,9 +3425,12 @@
         <v>0</v>
       </c>
       <c r="AH25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI25" t="n">
         <v>6</v>
       </c>
-      <c r="AI25" t="n">
+      <c r="AJ25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3463,10 +3541,13 @@
         <v>1</v>
       </c>
       <c r="AH26" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AI26" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="27">
@@ -3576,10 +3657,13 @@
         <v>1</v>
       </c>
       <c r="AH27" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AI27" t="n">
-        <v>15</v>
+        <v>18</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="28">
@@ -3689,9 +3773,12 @@
         <v>1</v>
       </c>
       <c r="AH28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI28" t="n">
         <v>5</v>
       </c>
-      <c r="AI28" t="n">
+      <c r="AJ28" t="n">
         <v>5</v>
       </c>
     </row>
@@ -3802,9 +3889,12 @@
         <v>1</v>
       </c>
       <c r="AH29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI29" t="n">
         <v>6</v>
       </c>
-      <c r="AI29" t="n">
+      <c r="AJ29" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3915,10 +4005,13 @@
         <v>0</v>
       </c>
       <c r="AH30" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AI30" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="31">
@@ -4028,10 +4121,13 @@
         <v>1</v>
       </c>
       <c r="AH31" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AI31" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="32">
@@ -4141,10 +4237,13 @@
         <v>0</v>
       </c>
       <c r="AH32" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AI32" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AJ32" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="33">
@@ -4254,9 +4353,12 @@
         <v>0</v>
       </c>
       <c r="AH33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI33" t="n">
         <v>12</v>
       </c>
-      <c r="AI33" t="n">
+      <c r="AJ33" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4367,9 +4469,12 @@
         <v>0</v>
       </c>
       <c r="AH34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI34" t="n">
         <v>7</v>
       </c>
-      <c r="AI34" t="n">
+      <c r="AJ34" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4480,10 +4585,13 @@
         <v>1</v>
       </c>
       <c r="AH35" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AI35" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AJ35" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="36">
@@ -4593,9 +4701,12 @@
         <v>1</v>
       </c>
       <c r="AH36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI36" t="n">
         <v>9</v>
       </c>
-      <c r="AI36" t="n">
+      <c r="AJ36" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4711,6 +4822,9 @@
       <c r="AI37" t="n">
         <v>0</v>
       </c>
+      <c r="AJ37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4819,9 +4933,12 @@
         <v>0</v>
       </c>
       <c r="AH38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI38" t="n">
         <v>2</v>
       </c>
-      <c r="AI38" t="n">
+      <c r="AJ38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4932,10 +5049,13 @@
         <v>1</v>
       </c>
       <c r="AH39" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AI39" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AJ39" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="40">
@@ -5045,9 +5165,12 @@
         <v>0</v>
       </c>
       <c r="AH40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI40" t="n">
         <v>14</v>
       </c>
-      <c r="AI40" t="n">
+      <c r="AJ40" t="n">
         <v>14</v>
       </c>
     </row>
@@ -5158,10 +5281,13 @@
         <v>1</v>
       </c>
       <c r="AH41" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AI41" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AJ41" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="42">
@@ -5271,9 +5397,12 @@
         <v>0</v>
       </c>
       <c r="AH42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI42" t="n">
         <v>21</v>
       </c>
-      <c r="AI42" t="n">
+      <c r="AJ42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5384,10 +5513,13 @@
         <v>1</v>
       </c>
       <c r="AH43" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="AI43" t="n">
-        <v>10</v>
+        <v>52</v>
+      </c>
+      <c r="AJ43" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="44">
@@ -5497,9 +5629,12 @@
         <v>1</v>
       </c>
       <c r="AH44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI44" t="n">
         <v>13</v>
       </c>
-      <c r="AI44" t="n">
+      <c r="AJ44" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5610,9 +5745,12 @@
         <v>1</v>
       </c>
       <c r="AH45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI45" t="n">
         <v>16</v>
       </c>
-      <c r="AI45" t="n">
+      <c r="AJ45" t="n">
         <v>16</v>
       </c>
     </row>
@@ -5723,9 +5861,12 @@
         <v>1</v>
       </c>
       <c r="AH46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI46" t="n">
         <v>14</v>
       </c>
-      <c r="AI46" t="n">
+      <c r="AJ46" t="n">
         <v>14</v>
       </c>
     </row>
@@ -5841,6 +5982,9 @@
       <c r="AI47" t="n">
         <v>0</v>
       </c>
+      <c r="AJ47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5949,10 +6093,13 @@
         <v>0</v>
       </c>
       <c r="AH48" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AI48" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AJ48" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="49">
@@ -6062,10 +6209,13 @@
         <v>1</v>
       </c>
       <c r="AH49" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AI49" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AJ49" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="50">
@@ -6175,9 +6325,12 @@
         <v>1</v>
       </c>
       <c r="AH50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI50" t="n">
         <v>7</v>
       </c>
-      <c r="AI50" t="n">
+      <c r="AJ50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6288,10 +6441,13 @@
         <v>1</v>
       </c>
       <c r="AH51" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AI51" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AJ51" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="52">
@@ -6406,6 +6562,9 @@
       <c r="AI52" t="n">
         <v>0</v>
       </c>
+      <c r="AJ52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6514,9 +6673,12 @@
         <v>0</v>
       </c>
       <c r="AH53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI53" t="n">
         <v>12</v>
       </c>
-      <c r="AI53" t="n">
+      <c r="AJ53" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6632,6 +6794,9 @@
       <c r="AI54" t="n">
         <v>0</v>
       </c>
+      <c r="AJ54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6740,10 +6905,13 @@
         <v>1</v>
       </c>
       <c r="AH55" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AI55" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AJ55" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="56">
@@ -6853,10 +7021,13 @@
         <v>1</v>
       </c>
       <c r="AH56" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AI56" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AJ56" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="57">
@@ -6966,9 +7137,12 @@
         <v>0</v>
       </c>
       <c r="AH57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI57" t="n">
         <v>8</v>
       </c>
-      <c r="AI57" t="n">
+      <c r="AJ57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7079,9 +7253,12 @@
         <v>0</v>
       </c>
       <c r="AH58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI58" t="n">
         <v>12</v>
       </c>
-      <c r="AI58" t="n">
+      <c r="AJ58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7192,9 +7369,12 @@
         <v>0</v>
       </c>
       <c r="AH59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI59" t="n">
         <v>3</v>
       </c>
-      <c r="AI59" t="n">
+      <c r="AJ59" t="n">
         <v>3</v>
       </c>
     </row>
@@ -7310,6 +7490,9 @@
       <c r="AI60" t="n">
         <v>0</v>
       </c>
+      <c r="AJ60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7418,10 +7601,13 @@
         <v>1</v>
       </c>
       <c r="AH61" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AI61" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AJ61" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="62">
@@ -7531,10 +7717,13 @@
         <v>1</v>
       </c>
       <c r="AH62" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AI62" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AJ62" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="63">
@@ -7644,10 +7833,13 @@
         <v>1</v>
       </c>
       <c r="AH63" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AI63" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AJ63" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="64">
@@ -7762,6 +7954,9 @@
       <c r="AI64" t="n">
         <v>0</v>
       </c>
+      <c r="AJ64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7870,9 +8065,12 @@
         <v>1</v>
       </c>
       <c r="AH65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI65" t="n">
         <v>8</v>
       </c>
-      <c r="AI65" t="n">
+      <c r="AJ65" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7986,7 +8184,10 @@
         <v>1</v>
       </c>
       <c r="AI66" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AJ66" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="67">
@@ -8096,10 +8297,13 @@
         <v>1</v>
       </c>
       <c r="AH67" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AI67" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AJ67" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="68">
@@ -8209,10 +8413,13 @@
         <v>1</v>
       </c>
       <c r="AH68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI68" t="n">
+        <v>9</v>
+      </c>
+      <c r="AJ68" t="n">
         <v>8</v>
-      </c>
-      <c r="AI68" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="69">
@@ -8322,9 +8529,12 @@
         <v>0</v>
       </c>
       <c r="AH69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI69" t="n">
         <v>7</v>
       </c>
-      <c r="AI69" t="n">
+      <c r="AJ69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8435,9 +8645,12 @@
         <v>1</v>
       </c>
       <c r="AH70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI70" t="n">
         <v>23</v>
       </c>
-      <c r="AI70" t="n">
+      <c r="AJ70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -8548,10 +8761,13 @@
         <v>1</v>
       </c>
       <c r="AH71" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AI71" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AJ71" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="72">
@@ -8661,9 +8877,12 @@
         <v>1</v>
       </c>
       <c r="AH72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI72" t="n">
         <v>13</v>
       </c>
-      <c r="AI72" t="n">
+      <c r="AJ72" t="n">
         <v>13</v>
       </c>
     </row>
@@ -8779,6 +8998,9 @@
       <c r="AI73" t="n">
         <v>0</v>
       </c>
+      <c r="AJ73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8892,6 +9114,9 @@
       <c r="AI74" t="n">
         <v>0</v>
       </c>
+      <c r="AJ74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -9000,10 +9225,13 @@
         <v>1</v>
       </c>
       <c r="AH75" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AI75" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AJ75" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="76">
@@ -9113,10 +9341,13 @@
         <v>0</v>
       </c>
       <c r="AH76" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AI76" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AJ76" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="77">
@@ -9226,9 +9457,12 @@
         <v>0</v>
       </c>
       <c r="AH77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI77" t="n">
         <v>13</v>
       </c>
-      <c r="AI77" t="n">
+      <c r="AJ77" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9339,10 +9573,13 @@
         <v>1</v>
       </c>
       <c r="AH78" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AI78" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AJ78" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="79">
@@ -9452,10 +9689,13 @@
         <v>1</v>
       </c>
       <c r="AH79" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AI79" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AJ79" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="80">
@@ -9565,10 +9805,13 @@
         <v>1</v>
       </c>
       <c r="AH80" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AI80" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AJ80" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="81">
@@ -9678,9 +9921,12 @@
         <v>0</v>
       </c>
       <c r="AH81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI81" t="n">
         <v>2</v>
       </c>
-      <c r="AI81" t="n">
+      <c r="AJ81" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9791,10 +10037,13 @@
         <v>1</v>
       </c>
       <c r="AH82" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AI82" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AJ82" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="83">
@@ -9904,9 +10153,12 @@
         <v>1</v>
       </c>
       <c r="AH83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI83" t="n">
         <v>12</v>
       </c>
-      <c r="AI83" t="n">
+      <c r="AJ83" t="n">
         <v>12</v>
       </c>
     </row>
@@ -10017,10 +10269,13 @@
         <v>1</v>
       </c>
       <c r="AH84" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AI84" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AJ84" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="85">
@@ -10130,9 +10385,12 @@
         <v>0</v>
       </c>
       <c r="AH85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI85" t="n">
         <v>7</v>
       </c>
-      <c r="AI85" t="n">
+      <c r="AJ85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10248,6 +10506,9 @@
       <c r="AI86" t="n">
         <v>0</v>
       </c>
+      <c r="AJ86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -10356,9 +10617,12 @@
         <v>1</v>
       </c>
       <c r="AH87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI87" t="n">
         <v>9</v>
       </c>
-      <c r="AI87" t="n">
+      <c r="AJ87" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10474,6 +10738,9 @@
       <c r="AI88" t="n">
         <v>0</v>
       </c>
+      <c r="AJ88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -10582,10 +10849,13 @@
         <v>1</v>
       </c>
       <c r="AH89" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AI89" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AJ89" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="90">
@@ -10695,9 +10965,12 @@
         <v>1</v>
       </c>
       <c r="AH90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI90" t="n">
         <v>11</v>
       </c>
-      <c r="AI90" t="n">
+      <c r="AJ90" t="n">
         <v>11</v>
       </c>
     </row>
@@ -10808,9 +11081,12 @@
         <v>1</v>
       </c>
       <c r="AH91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI91" t="n">
         <v>39</v>
       </c>
-      <c r="AI91" t="n">
+      <c r="AJ91" t="n">
         <v>10</v>
       </c>
     </row>
@@ -10921,10 +11197,13 @@
         <v>0</v>
       </c>
       <c r="AH92" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AI92" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AJ92" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="93">
@@ -11039,6 +11318,9 @@
       <c r="AI93" t="n">
         <v>0</v>
       </c>
+      <c r="AJ93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -11147,10 +11429,13 @@
         <v>0</v>
       </c>
       <c r="AH94" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AI94" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AJ94" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="95">
@@ -11260,9 +11545,12 @@
         <v>0</v>
       </c>
       <c r="AH95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI95" t="n">
         <v>6</v>
       </c>
-      <c r="AI95" t="n">
+      <c r="AJ95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -11373,9 +11661,12 @@
         <v>0</v>
       </c>
       <c r="AH96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI96" t="n">
         <v>14</v>
       </c>
-      <c r="AI96" t="n">
+      <c r="AJ96" t="n">
         <v>14</v>
       </c>
     </row>
@@ -11491,6 +11782,9 @@
       <c r="AI97" t="n">
         <v>0</v>
       </c>
+      <c r="AJ97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -11599,10 +11893,13 @@
         <v>1</v>
       </c>
       <c r="AH98" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AI98" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AJ98" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="99">
@@ -11712,9 +12009,12 @@
         <v>0</v>
       </c>
       <c r="AH99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI99" t="n">
         <v>3</v>
       </c>
-      <c r="AI99" t="n">
+      <c r="AJ99" t="n">
         <v>3</v>
       </c>
     </row>
@@ -11830,6 +12130,9 @@
       <c r="AI100" t="n">
         <v>0</v>
       </c>
+      <c r="AJ100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -11938,9 +12241,12 @@
         <v>1</v>
       </c>
       <c r="AH101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI101" t="n">
         <v>17</v>
       </c>
-      <c r="AI101" t="n">
+      <c r="AJ101" t="n">
         <v>17</v>
       </c>
     </row>
@@ -12051,9 +12357,12 @@
         <v>1</v>
       </c>
       <c r="AH102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI102" t="n">
         <v>15</v>
       </c>
-      <c r="AI102" t="n">
+      <c r="AJ102" t="n">
         <v>15</v>
       </c>
     </row>
@@ -12164,10 +12473,13 @@
         <v>1</v>
       </c>
       <c r="AH103" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AI103" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AJ103" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="104">
@@ -12277,10 +12589,13 @@
         <v>1</v>
       </c>
       <c r="AH104" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AI104" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AJ104" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="105">
@@ -12390,10 +12705,13 @@
         <v>1</v>
       </c>
       <c r="AH105" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AI105" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AJ105" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="106">
@@ -12503,10 +12821,13 @@
         <v>1</v>
       </c>
       <c r="AH106" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AI106" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AJ106" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="107">
@@ -12616,10 +12937,13 @@
         <v>1</v>
       </c>
       <c r="AH107" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AI107" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AJ107" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="108">
@@ -12729,9 +13053,12 @@
         <v>0</v>
       </c>
       <c r="AH108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI108" t="n">
         <v>2</v>
       </c>
-      <c r="AI108" t="n">
+      <c r="AJ108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -12845,7 +13172,10 @@
         <v>1</v>
       </c>
       <c r="AI109" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AJ109" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2501)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ109"/>
+  <dimension ref="A1:AK109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -464,8 +464,9 @@
     <col width="12" customWidth="1" min="32" max="32"/>
     <col width="12" customWidth="1" min="33" max="33"/>
     <col width="12" customWidth="1" min="34" max="34"/>
-    <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="35" max="35"/>
     <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="13" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -639,12 +640,17 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="AI1" s="2" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="AJ1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AJ1" s="2" t="inlineStr">
+      <c r="AK1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -760,9 +766,12 @@
         <v>0</v>
       </c>
       <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
         <v>10</v>
       </c>
-      <c r="AJ2" t="n">
+      <c r="AK2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -876,9 +885,12 @@
         <v>0</v>
       </c>
       <c r="AI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ3" t="n">
         <v>8</v>
       </c>
-      <c r="AJ3" t="n">
+      <c r="AK3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -992,10 +1004,13 @@
         <v>1</v>
       </c>
       <c r="AI4" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AJ4" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -1108,10 +1123,13 @@
         <v>0</v>
       </c>
       <c r="AI5" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AJ5" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -1224,10 +1242,13 @@
         <v>0</v>
       </c>
       <c r="AI6" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AJ6" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -1340,9 +1361,12 @@
         <v>0</v>
       </c>
       <c r="AI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="n">
         <v>13</v>
       </c>
-      <c r="AJ7" t="n">
+      <c r="AK7" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1456,10 +1480,13 @@
         <v>1</v>
       </c>
       <c r="AI8" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AJ8" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -1572,9 +1599,12 @@
         <v>1</v>
       </c>
       <c r="AI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" t="n">
         <v>17</v>
       </c>
-      <c r="AJ9" t="n">
+      <c r="AK9" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1688,10 +1718,13 @@
         <v>1</v>
       </c>
       <c r="AI10" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AJ10" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="11">
@@ -1804,10 +1837,13 @@
         <v>1</v>
       </c>
       <c r="AI11" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AJ11" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -1920,10 +1956,13 @@
         <v>1</v>
       </c>
       <c r="AI12" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AJ12" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -2036,10 +2075,13 @@
         <v>0</v>
       </c>
       <c r="AI13" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AJ13" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -2152,10 +2194,13 @@
         <v>1</v>
       </c>
       <c r="AI14" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AJ14" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="15">
@@ -2268,9 +2313,12 @@
         <v>0</v>
       </c>
       <c r="AI15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ15" t="n">
         <v>9</v>
       </c>
-      <c r="AJ15" t="n">
+      <c r="AK15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2384,9 +2432,12 @@
         <v>1</v>
       </c>
       <c r="AI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ16" t="n">
         <v>14</v>
       </c>
-      <c r="AJ16" t="n">
+      <c r="AK16" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2500,9 +2551,12 @@
         <v>1</v>
       </c>
       <c r="AI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ17" t="n">
         <v>14</v>
       </c>
-      <c r="AJ17" t="n">
+      <c r="AK17" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2616,9 +2670,12 @@
         <v>1</v>
       </c>
       <c r="AI18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ18" t="n">
         <v>16</v>
       </c>
-      <c r="AJ18" t="n">
+      <c r="AK18" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2737,6 +2794,9 @@
       <c r="AJ19" t="n">
         <v>0</v>
       </c>
+      <c r="AK19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2848,10 +2908,13 @@
         <v>0</v>
       </c>
       <c r="AI20" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AJ20" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="21">
@@ -2964,10 +3027,13 @@
         <v>1</v>
       </c>
       <c r="AI21" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AJ21" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="22">
@@ -3085,6 +3151,9 @@
       <c r="AJ22" t="n">
         <v>0</v>
       </c>
+      <c r="AK22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3196,10 +3265,13 @@
         <v>0</v>
       </c>
       <c r="AI23" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AJ23" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="24">
@@ -3312,10 +3384,13 @@
         <v>1</v>
       </c>
       <c r="AI24" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AJ24" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="25">
@@ -3428,9 +3503,12 @@
         <v>0</v>
       </c>
       <c r="AI25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ25" t="n">
         <v>6</v>
       </c>
-      <c r="AJ25" t="n">
+      <c r="AK25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3544,10 +3622,13 @@
         <v>1</v>
       </c>
       <c r="AI26" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AJ26" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="27">
@@ -3660,10 +3741,13 @@
         <v>1</v>
       </c>
       <c r="AI27" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AJ27" t="n">
-        <v>16</v>
+        <v>19</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="28">
@@ -3776,10 +3860,13 @@
         <v>0</v>
       </c>
       <c r="AI28" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AJ28" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AK28" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -3892,9 +3979,12 @@
         <v>0</v>
       </c>
       <c r="AI29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ29" t="n">
         <v>6</v>
       </c>
-      <c r="AJ29" t="n">
+      <c r="AK29" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4008,10 +4098,13 @@
         <v>1</v>
       </c>
       <c r="AI30" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AJ30" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AK30" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="31">
@@ -4124,10 +4217,13 @@
         <v>1</v>
       </c>
       <c r="AI31" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AJ31" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="32">
@@ -4240,9 +4336,12 @@
         <v>1</v>
       </c>
       <c r="AI32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ32" t="n">
         <v>12</v>
       </c>
-      <c r="AJ32" t="n">
+      <c r="AK32" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4356,10 +4455,13 @@
         <v>0</v>
       </c>
       <c r="AI33" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AJ33" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="34">
@@ -4472,9 +4574,12 @@
         <v>0</v>
       </c>
       <c r="AI34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ34" t="n">
         <v>7</v>
       </c>
-      <c r="AJ34" t="n">
+      <c r="AK34" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4588,10 +4693,13 @@
         <v>1</v>
       </c>
       <c r="AI35" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AJ35" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AK35" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="36">
@@ -4704,9 +4812,12 @@
         <v>0</v>
       </c>
       <c r="AI36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ36" t="n">
         <v>9</v>
       </c>
-      <c r="AJ36" t="n">
+      <c r="AK36" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4825,6 +4936,9 @@
       <c r="AJ37" t="n">
         <v>0</v>
       </c>
+      <c r="AK37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4936,9 +5050,12 @@
         <v>0</v>
       </c>
       <c r="AI38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ38" t="n">
         <v>2</v>
       </c>
-      <c r="AJ38" t="n">
+      <c r="AK38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5052,10 +5169,13 @@
         <v>1</v>
       </c>
       <c r="AI39" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AJ39" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AK39" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="40">
@@ -5168,10 +5288,13 @@
         <v>0</v>
       </c>
       <c r="AI40" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AJ40" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AK40" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="41">
@@ -5284,10 +5407,13 @@
         <v>1</v>
       </c>
       <c r="AI41" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AJ41" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AK41" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="42">
@@ -5400,9 +5526,12 @@
         <v>0</v>
       </c>
       <c r="AI42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ42" t="n">
         <v>21</v>
       </c>
-      <c r="AJ42" t="n">
+      <c r="AK42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5516,10 +5645,13 @@
         <v>1</v>
       </c>
       <c r="AI43" t="n">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="AJ43" t="n">
-        <v>11</v>
+        <v>53</v>
+      </c>
+      <c r="AK43" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="44">
@@ -5632,10 +5764,13 @@
         <v>0</v>
       </c>
       <c r="AI44" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AJ44" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AK44" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="45">
@@ -5748,10 +5883,13 @@
         <v>0</v>
       </c>
       <c r="AI45" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AJ45" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AK45" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="46">
@@ -5864,10 +6002,13 @@
         <v>0</v>
       </c>
       <c r="AI46" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AJ46" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AK46" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="47">
@@ -5985,6 +6126,9 @@
       <c r="AJ47" t="n">
         <v>0</v>
       </c>
+      <c r="AK47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6096,10 +6240,13 @@
         <v>1</v>
       </c>
       <c r="AI48" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AJ48" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AK48" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="49">
@@ -6212,9 +6359,12 @@
         <v>1</v>
       </c>
       <c r="AI49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ49" t="n">
         <v>14</v>
       </c>
-      <c r="AJ49" t="n">
+      <c r="AK49" t="n">
         <v>14</v>
       </c>
     </row>
@@ -6328,9 +6478,12 @@
         <v>0</v>
       </c>
       <c r="AI50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ50" t="n">
         <v>7</v>
       </c>
-      <c r="AJ50" t="n">
+      <c r="AK50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6444,10 +6597,13 @@
         <v>1</v>
       </c>
       <c r="AI51" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AJ51" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AK51" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="52">
@@ -6565,6 +6721,9 @@
       <c r="AJ52" t="n">
         <v>0</v>
       </c>
+      <c r="AK52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6676,9 +6835,12 @@
         <v>0</v>
       </c>
       <c r="AI53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ53" t="n">
         <v>12</v>
       </c>
-      <c r="AJ53" t="n">
+      <c r="AK53" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6797,6 +6959,9 @@
       <c r="AJ54" t="n">
         <v>0</v>
       </c>
+      <c r="AK54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6908,10 +7073,13 @@
         <v>1</v>
       </c>
       <c r="AI55" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AJ55" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AK55" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="56">
@@ -7024,10 +7192,13 @@
         <v>1</v>
       </c>
       <c r="AI56" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AJ56" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AK56" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="57">
@@ -7140,9 +7311,12 @@
         <v>0</v>
       </c>
       <c r="AI57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ57" t="n">
         <v>8</v>
       </c>
-      <c r="AJ57" t="n">
+      <c r="AK57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7256,9 +7430,12 @@
         <v>0</v>
       </c>
       <c r="AI58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ58" t="n">
         <v>12</v>
       </c>
-      <c r="AJ58" t="n">
+      <c r="AK58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7372,9 +7549,12 @@
         <v>0</v>
       </c>
       <c r="AI59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ59" t="n">
         <v>3</v>
       </c>
-      <c r="AJ59" t="n">
+      <c r="AK59" t="n">
         <v>3</v>
       </c>
     </row>
@@ -7493,6 +7673,9 @@
       <c r="AJ60" t="n">
         <v>0</v>
       </c>
+      <c r="AK60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7604,10 +7787,13 @@
         <v>1</v>
       </c>
       <c r="AI61" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AJ61" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AK61" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="62">
@@ -7720,10 +7906,13 @@
         <v>1</v>
       </c>
       <c r="AI62" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AJ62" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AK62" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="63">
@@ -7836,10 +8025,13 @@
         <v>1</v>
       </c>
       <c r="AI63" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AJ63" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AK63" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="64">
@@ -7957,6 +8149,9 @@
       <c r="AJ64" t="n">
         <v>0</v>
       </c>
+      <c r="AK64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8068,10 +8263,13 @@
         <v>0</v>
       </c>
       <c r="AI65" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AJ65" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AK65" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="66">
@@ -8184,9 +8382,12 @@
         <v>1</v>
       </c>
       <c r="AI66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ66" t="n">
         <v>2</v>
       </c>
-      <c r="AJ66" t="n">
+      <c r="AK66" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8300,10 +8501,13 @@
         <v>1</v>
       </c>
       <c r="AI67" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AJ67" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AK67" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="68">
@@ -8416,10 +8620,13 @@
         <v>1</v>
       </c>
       <c r="AI68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ68" t="n">
+        <v>10</v>
+      </c>
+      <c r="AK68" t="n">
         <v>9</v>
-      </c>
-      <c r="AJ68" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="69">
@@ -8532,9 +8739,12 @@
         <v>0</v>
       </c>
       <c r="AI69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ69" t="n">
         <v>7</v>
       </c>
-      <c r="AJ69" t="n">
+      <c r="AK69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8648,9 +8858,12 @@
         <v>0</v>
       </c>
       <c r="AI70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ70" t="n">
         <v>23</v>
       </c>
-      <c r="AJ70" t="n">
+      <c r="AK70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -8764,10 +8977,13 @@
         <v>1</v>
       </c>
       <c r="AI71" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AJ71" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AK71" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="72">
@@ -8880,9 +9096,12 @@
         <v>0</v>
       </c>
       <c r="AI72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ72" t="n">
         <v>13</v>
       </c>
-      <c r="AJ72" t="n">
+      <c r="AK72" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9001,6 +9220,9 @@
       <c r="AJ73" t="n">
         <v>0</v>
       </c>
+      <c r="AK73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9117,6 +9339,9 @@
       <c r="AJ74" t="n">
         <v>0</v>
       </c>
+      <c r="AK74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -9228,10 +9453,13 @@
         <v>1</v>
       </c>
       <c r="AI75" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AJ75" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AK75" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="76">
@@ -9344,10 +9572,13 @@
         <v>1</v>
       </c>
       <c r="AI76" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AJ76" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AK76" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="77">
@@ -9460,10 +9691,13 @@
         <v>0</v>
       </c>
       <c r="AI77" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AJ77" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AK77" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="78">
@@ -9576,10 +9810,13 @@
         <v>1</v>
       </c>
       <c r="AI78" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AJ78" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AK78" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="79">
@@ -9692,10 +9929,13 @@
         <v>1</v>
       </c>
       <c r="AI79" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AJ79" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AK79" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="80">
@@ -9808,10 +10048,13 @@
         <v>1</v>
       </c>
       <c r="AI80" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AJ80" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AK80" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="81">
@@ -9924,10 +10167,13 @@
         <v>0</v>
       </c>
       <c r="AI81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AJ81" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AK81" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="82">
@@ -10040,10 +10286,13 @@
         <v>1</v>
       </c>
       <c r="AI82" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AJ82" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AK82" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="83">
@@ -10156,10 +10405,13 @@
         <v>0</v>
       </c>
       <c r="AI83" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AJ83" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AK83" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="84">
@@ -10272,9 +10524,12 @@
         <v>1</v>
       </c>
       <c r="AI84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ84" t="n">
         <v>5</v>
       </c>
-      <c r="AJ84" t="n">
+      <c r="AK84" t="n">
         <v>5</v>
       </c>
     </row>
@@ -10388,9 +10643,12 @@
         <v>0</v>
       </c>
       <c r="AI85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ85" t="n">
         <v>7</v>
       </c>
-      <c r="AJ85" t="n">
+      <c r="AK85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10509,6 +10767,9 @@
       <c r="AJ86" t="n">
         <v>0</v>
       </c>
+      <c r="AK86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -10620,9 +10881,12 @@
         <v>0</v>
       </c>
       <c r="AI87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ87" t="n">
         <v>9</v>
       </c>
-      <c r="AJ87" t="n">
+      <c r="AK87" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10741,6 +11005,9 @@
       <c r="AJ88" t="n">
         <v>0</v>
       </c>
+      <c r="AK88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -10852,10 +11119,13 @@
         <v>1</v>
       </c>
       <c r="AI89" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AJ89" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AK89" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="90">
@@ -10968,9 +11238,12 @@
         <v>0</v>
       </c>
       <c r="AI90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ90" t="n">
         <v>11</v>
       </c>
-      <c r="AJ90" t="n">
+      <c r="AK90" t="n">
         <v>11</v>
       </c>
     </row>
@@ -11084,10 +11357,13 @@
         <v>0</v>
       </c>
       <c r="AI91" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="AJ91" t="n">
-        <v>10</v>
+        <v>40</v>
+      </c>
+      <c r="AK91" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="92">
@@ -11200,10 +11476,13 @@
         <v>1</v>
       </c>
       <c r="AI92" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AJ92" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AK92" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="93">
@@ -11321,6 +11600,9 @@
       <c r="AJ93" t="n">
         <v>0</v>
       </c>
+      <c r="AK93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -11432,10 +11714,13 @@
         <v>1</v>
       </c>
       <c r="AI94" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AJ94" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AK94" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="95">
@@ -11548,9 +11833,12 @@
         <v>0</v>
       </c>
       <c r="AI95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ95" t="n">
         <v>6</v>
       </c>
-      <c r="AJ95" t="n">
+      <c r="AK95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -11664,9 +11952,12 @@
         <v>0</v>
       </c>
       <c r="AI96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ96" t="n">
         <v>14</v>
       </c>
-      <c r="AJ96" t="n">
+      <c r="AK96" t="n">
         <v>14</v>
       </c>
     </row>
@@ -11785,6 +12076,9 @@
       <c r="AJ97" t="n">
         <v>0</v>
       </c>
+      <c r="AK97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -11896,10 +12190,13 @@
         <v>1</v>
       </c>
       <c r="AI98" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AJ98" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AK98" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="99">
@@ -12012,10 +12309,13 @@
         <v>0</v>
       </c>
       <c r="AI99" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AJ99" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AK99" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="100">
@@ -12133,6 +12433,9 @@
       <c r="AJ100" t="n">
         <v>0</v>
       </c>
+      <c r="AK100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -12244,10 +12547,13 @@
         <v>0</v>
       </c>
       <c r="AI101" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AJ101" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AK101" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="102">
@@ -12360,10 +12666,13 @@
         <v>0</v>
       </c>
       <c r="AI102" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AJ102" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AK102" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="103">
@@ -12476,10 +12785,13 @@
         <v>1</v>
       </c>
       <c r="AI103" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AJ103" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AK103" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="104">
@@ -12592,10 +12904,13 @@
         <v>1</v>
       </c>
       <c r="AI104" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AJ104" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AK104" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="105">
@@ -12708,10 +13023,13 @@
         <v>1</v>
       </c>
       <c r="AI105" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AJ105" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AK105" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="106">
@@ -12824,10 +13142,13 @@
         <v>1</v>
       </c>
       <c r="AI106" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AJ106" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AK106" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="107">
@@ -12940,10 +13261,13 @@
         <v>1</v>
       </c>
       <c r="AI107" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AJ107" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AK107" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="108">
@@ -13056,9 +13380,12 @@
         <v>0</v>
       </c>
       <c r="AI108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ108" t="n">
         <v>2</v>
       </c>
-      <c r="AJ108" t="n">
+      <c r="AK108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -13172,9 +13499,12 @@
         <v>1</v>
       </c>
       <c r="AI109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ109" t="n">
         <v>2</v>
       </c>
-      <c r="AJ109" t="n">
+      <c r="AK109" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2521)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK109"/>
+  <dimension ref="A1:AL109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -465,8 +465,9 @@
     <col width="12" customWidth="1" min="33" max="33"/>
     <col width="12" customWidth="1" min="34" max="34"/>
     <col width="12" customWidth="1" min="35" max="35"/>
-    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
     <col width="13" customWidth="1" min="37" max="37"/>
+    <col width="13" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -645,12 +646,17 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="AJ1" s="2" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="AK1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AK1" s="2" t="inlineStr">
+      <c r="AL1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -769,9 +775,12 @@
         <v>0</v>
       </c>
       <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="n">
         <v>10</v>
       </c>
-      <c r="AK2" t="n">
+      <c r="AL2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -888,9 +897,12 @@
         <v>0</v>
       </c>
       <c r="AJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" t="n">
         <v>8</v>
       </c>
-      <c r="AK3" t="n">
+      <c r="AL3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1007,10 +1019,13 @@
         <v>1</v>
       </c>
       <c r="AJ4" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AK4" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -1126,9 +1141,12 @@
         <v>1</v>
       </c>
       <c r="AJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" t="n">
         <v>15</v>
       </c>
-      <c r="AK5" t="n">
+      <c r="AL5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1245,9 +1263,12 @@
         <v>1</v>
       </c>
       <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" t="n">
         <v>14</v>
       </c>
-      <c r="AK6" t="n">
+      <c r="AL6" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1364,9 +1385,12 @@
         <v>0</v>
       </c>
       <c r="AJ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="n">
         <v>13</v>
       </c>
-      <c r="AK7" t="n">
+      <c r="AL7" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1483,9 +1507,12 @@
         <v>1</v>
       </c>
       <c r="AJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" t="n">
         <v>18</v>
       </c>
-      <c r="AK8" t="n">
+      <c r="AL8" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1602,9 +1629,12 @@
         <v>0</v>
       </c>
       <c r="AJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" t="n">
         <v>17</v>
       </c>
-      <c r="AK9" t="n">
+      <c r="AL9" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1721,10 +1751,13 @@
         <v>1</v>
       </c>
       <c r="AJ10" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AK10" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="11">
@@ -1840,9 +1873,12 @@
         <v>1</v>
       </c>
       <c r="AJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK11" t="n">
         <v>15</v>
       </c>
-      <c r="AK11" t="n">
+      <c r="AL11" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1959,9 +1995,12 @@
         <v>1</v>
       </c>
       <c r="AJ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK12" t="n">
         <v>18</v>
       </c>
-      <c r="AK12" t="n">
+      <c r="AL12" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2078,9 +2117,12 @@
         <v>1</v>
       </c>
       <c r="AJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK13" t="n">
         <v>10</v>
       </c>
-      <c r="AK13" t="n">
+      <c r="AL13" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2197,9 +2239,12 @@
         <v>1</v>
       </c>
       <c r="AJ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK14" t="n">
         <v>18</v>
       </c>
-      <c r="AK14" t="n">
+      <c r="AL14" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2316,9 +2361,12 @@
         <v>0</v>
       </c>
       <c r="AJ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK15" t="n">
         <v>9</v>
       </c>
-      <c r="AK15" t="n">
+      <c r="AL15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2435,9 +2483,12 @@
         <v>0</v>
       </c>
       <c r="AJ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK16" t="n">
         <v>14</v>
       </c>
-      <c r="AK16" t="n">
+      <c r="AL16" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2554,9 +2605,12 @@
         <v>0</v>
       </c>
       <c r="AJ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK17" t="n">
         <v>14</v>
       </c>
-      <c r="AK17" t="n">
+      <c r="AL17" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2673,9 +2727,12 @@
         <v>0</v>
       </c>
       <c r="AJ18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK18" t="n">
         <v>16</v>
       </c>
-      <c r="AK18" t="n">
+      <c r="AL18" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2797,6 +2854,9 @@
       <c r="AK19" t="n">
         <v>0</v>
       </c>
+      <c r="AL19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2911,9 +2971,12 @@
         <v>1</v>
       </c>
       <c r="AJ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK20" t="n">
         <v>14</v>
       </c>
-      <c r="AK20" t="n">
+      <c r="AL20" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3030,9 +3093,12 @@
         <v>1</v>
       </c>
       <c r="AJ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK21" t="n">
         <v>17</v>
       </c>
-      <c r="AK21" t="n">
+      <c r="AL21" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3154,6 +3220,9 @@
       <c r="AK22" t="n">
         <v>0</v>
       </c>
+      <c r="AL22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3268,9 +3337,12 @@
         <v>1</v>
       </c>
       <c r="AJ23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK23" t="n">
         <v>10</v>
       </c>
-      <c r="AK23" t="n">
+      <c r="AL23" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3387,9 +3459,12 @@
         <v>1</v>
       </c>
       <c r="AJ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK24" t="n">
         <v>17</v>
       </c>
-      <c r="AK24" t="n">
+      <c r="AL24" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3506,9 +3581,12 @@
         <v>0</v>
       </c>
       <c r="AJ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK25" t="n">
         <v>6</v>
       </c>
-      <c r="AK25" t="n">
+      <c r="AL25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3625,9 +3703,12 @@
         <v>1</v>
       </c>
       <c r="AJ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK26" t="n">
         <v>16</v>
       </c>
-      <c r="AK26" t="n">
+      <c r="AL26" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3744,9 +3825,12 @@
         <v>1</v>
       </c>
       <c r="AJ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK27" t="n">
         <v>19</v>
       </c>
-      <c r="AK27" t="n">
+      <c r="AL27" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3863,9 +3947,12 @@
         <v>1</v>
       </c>
       <c r="AJ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK28" t="n">
         <v>6</v>
       </c>
-      <c r="AK28" t="n">
+      <c r="AL28" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3982,9 +4069,12 @@
         <v>0</v>
       </c>
       <c r="AJ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK29" t="n">
         <v>6</v>
       </c>
-      <c r="AK29" t="n">
+      <c r="AL29" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4101,9 +4191,12 @@
         <v>1</v>
       </c>
       <c r="AJ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK30" t="n">
         <v>13</v>
       </c>
-      <c r="AK30" t="n">
+      <c r="AL30" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4220,9 +4313,12 @@
         <v>1</v>
       </c>
       <c r="AJ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK31" t="n">
         <v>15</v>
       </c>
-      <c r="AK31" t="n">
+      <c r="AL31" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4339,9 +4435,12 @@
         <v>0</v>
       </c>
       <c r="AJ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK32" t="n">
         <v>12</v>
       </c>
-      <c r="AK32" t="n">
+      <c r="AL32" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4458,9 +4557,12 @@
         <v>1</v>
       </c>
       <c r="AJ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK33" t="n">
         <v>13</v>
       </c>
-      <c r="AK33" t="n">
+      <c r="AL33" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4577,9 +4679,12 @@
         <v>0</v>
       </c>
       <c r="AJ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK34" t="n">
         <v>7</v>
       </c>
-      <c r="AK34" t="n">
+      <c r="AL34" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4696,9 +4801,12 @@
         <v>1</v>
       </c>
       <c r="AJ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK35" t="n">
         <v>14</v>
       </c>
-      <c r="AK35" t="n">
+      <c r="AL35" t="n">
         <v>14</v>
       </c>
     </row>
@@ -4815,9 +4923,12 @@
         <v>0</v>
       </c>
       <c r="AJ36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK36" t="n">
         <v>9</v>
       </c>
-      <c r="AK36" t="n">
+      <c r="AL36" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4939,6 +5050,9 @@
       <c r="AK37" t="n">
         <v>0</v>
       </c>
+      <c r="AL37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5053,9 +5167,12 @@
         <v>0</v>
       </c>
       <c r="AJ38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK38" t="n">
         <v>2</v>
       </c>
-      <c r="AK38" t="n">
+      <c r="AL38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5172,9 +5289,12 @@
         <v>1</v>
       </c>
       <c r="AJ39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK39" t="n">
         <v>18</v>
       </c>
-      <c r="AK39" t="n">
+      <c r="AL39" t="n">
         <v>18</v>
       </c>
     </row>
@@ -5291,9 +5411,12 @@
         <v>1</v>
       </c>
       <c r="AJ40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK40" t="n">
         <v>15</v>
       </c>
-      <c r="AK40" t="n">
+      <c r="AL40" t="n">
         <v>15</v>
       </c>
     </row>
@@ -5410,9 +5533,12 @@
         <v>1</v>
       </c>
       <c r="AJ41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK41" t="n">
         <v>19</v>
       </c>
-      <c r="AK41" t="n">
+      <c r="AL41" t="n">
         <v>19</v>
       </c>
     </row>
@@ -5529,9 +5655,12 @@
         <v>0</v>
       </c>
       <c r="AJ42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK42" t="n">
         <v>21</v>
       </c>
-      <c r="AK42" t="n">
+      <c r="AL42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5648,9 +5777,12 @@
         <v>1</v>
       </c>
       <c r="AJ43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK43" t="n">
         <v>53</v>
       </c>
-      <c r="AK43" t="n">
+      <c r="AL43" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5767,9 +5899,12 @@
         <v>1</v>
       </c>
       <c r="AJ44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK44" t="n">
         <v>14</v>
       </c>
-      <c r="AK44" t="n">
+      <c r="AL44" t="n">
         <v>14</v>
       </c>
     </row>
@@ -5886,9 +6021,12 @@
         <v>1</v>
       </c>
       <c r="AJ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK45" t="n">
         <v>17</v>
       </c>
-      <c r="AK45" t="n">
+      <c r="AL45" t="n">
         <v>17</v>
       </c>
     </row>
@@ -6005,9 +6143,12 @@
         <v>1</v>
       </c>
       <c r="AJ46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK46" t="n">
         <v>15</v>
       </c>
-      <c r="AK46" t="n">
+      <c r="AL46" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6129,6 +6270,9 @@
       <c r="AK47" t="n">
         <v>0</v>
       </c>
+      <c r="AL47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6243,9 +6387,12 @@
         <v>1</v>
       </c>
       <c r="AJ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK48" t="n">
         <v>17</v>
       </c>
-      <c r="AK48" t="n">
+      <c r="AL48" t="n">
         <v>17</v>
       </c>
     </row>
@@ -6362,9 +6509,12 @@
         <v>0</v>
       </c>
       <c r="AJ49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK49" t="n">
         <v>14</v>
       </c>
-      <c r="AK49" t="n">
+      <c r="AL49" t="n">
         <v>14</v>
       </c>
     </row>
@@ -6481,9 +6631,12 @@
         <v>0</v>
       </c>
       <c r="AJ50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK50" t="n">
         <v>7</v>
       </c>
-      <c r="AK50" t="n">
+      <c r="AL50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6600,9 +6753,12 @@
         <v>1</v>
       </c>
       <c r="AJ51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK51" t="n">
         <v>18</v>
       </c>
-      <c r="AK51" t="n">
+      <c r="AL51" t="n">
         <v>18</v>
       </c>
     </row>
@@ -6724,6 +6880,9 @@
       <c r="AK52" t="n">
         <v>0</v>
       </c>
+      <c r="AL52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6838,9 +6997,12 @@
         <v>0</v>
       </c>
       <c r="AJ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK53" t="n">
         <v>12</v>
       </c>
-      <c r="AK53" t="n">
+      <c r="AL53" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6962,6 +7124,9 @@
       <c r="AK54" t="n">
         <v>0</v>
       </c>
+      <c r="AL54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7076,10 +7241,13 @@
         <v>1</v>
       </c>
       <c r="AJ55" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AK55" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AL55" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="56">
@@ -7195,9 +7363,12 @@
         <v>1</v>
       </c>
       <c r="AJ56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK56" t="n">
         <v>17</v>
       </c>
-      <c r="AK56" t="n">
+      <c r="AL56" t="n">
         <v>17</v>
       </c>
     </row>
@@ -7314,9 +7485,12 @@
         <v>0</v>
       </c>
       <c r="AJ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK57" t="n">
         <v>8</v>
       </c>
-      <c r="AK57" t="n">
+      <c r="AL57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7433,9 +7607,12 @@
         <v>0</v>
       </c>
       <c r="AJ58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK58" t="n">
         <v>12</v>
       </c>
-      <c r="AK58" t="n">
+      <c r="AL58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7552,9 +7729,12 @@
         <v>0</v>
       </c>
       <c r="AJ59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK59" t="n">
         <v>3</v>
       </c>
-      <c r="AK59" t="n">
+      <c r="AL59" t="n">
         <v>3</v>
       </c>
     </row>
@@ -7676,6 +7856,9 @@
       <c r="AK60" t="n">
         <v>0</v>
       </c>
+      <c r="AL60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7790,9 +7973,12 @@
         <v>1</v>
       </c>
       <c r="AJ61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK61" t="n">
         <v>15</v>
       </c>
-      <c r="AK61" t="n">
+      <c r="AL61" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7909,9 +8095,12 @@
         <v>1</v>
       </c>
       <c r="AJ62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK62" t="n">
         <v>17</v>
       </c>
-      <c r="AK62" t="n">
+      <c r="AL62" t="n">
         <v>17</v>
       </c>
     </row>
@@ -8028,9 +8217,12 @@
         <v>1</v>
       </c>
       <c r="AJ63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK63" t="n">
         <v>7</v>
       </c>
-      <c r="AK63" t="n">
+      <c r="AL63" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8152,6 +8344,9 @@
       <c r="AK64" t="n">
         <v>0</v>
       </c>
+      <c r="AL64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8266,9 +8461,12 @@
         <v>1</v>
       </c>
       <c r="AJ65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK65" t="n">
         <v>9</v>
       </c>
-      <c r="AK65" t="n">
+      <c r="AL65" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8385,9 +8583,12 @@
         <v>0</v>
       </c>
       <c r="AJ66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK66" t="n">
         <v>2</v>
       </c>
-      <c r="AK66" t="n">
+      <c r="AL66" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8504,9 +8705,12 @@
         <v>1</v>
       </c>
       <c r="AJ67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK67" t="n">
         <v>19</v>
       </c>
-      <c r="AK67" t="n">
+      <c r="AL67" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8623,9 +8827,12 @@
         <v>1</v>
       </c>
       <c r="AJ68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK68" t="n">
         <v>10</v>
       </c>
-      <c r="AK68" t="n">
+      <c r="AL68" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8742,9 +8949,12 @@
         <v>0</v>
       </c>
       <c r="AJ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK69" t="n">
         <v>7</v>
       </c>
-      <c r="AK69" t="n">
+      <c r="AL69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8861,9 +9071,12 @@
         <v>0</v>
       </c>
       <c r="AJ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK70" t="n">
         <v>23</v>
       </c>
-      <c r="AK70" t="n">
+      <c r="AL70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -8980,9 +9193,12 @@
         <v>1</v>
       </c>
       <c r="AJ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK71" t="n">
         <v>12</v>
       </c>
-      <c r="AK71" t="n">
+      <c r="AL71" t="n">
         <v>12</v>
       </c>
     </row>
@@ -9099,9 +9315,12 @@
         <v>0</v>
       </c>
       <c r="AJ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK72" t="n">
         <v>13</v>
       </c>
-      <c r="AK72" t="n">
+      <c r="AL72" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9223,6 +9442,9 @@
       <c r="AK73" t="n">
         <v>0</v>
       </c>
+      <c r="AL73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9342,6 +9564,9 @@
       <c r="AK74" t="n">
         <v>0</v>
       </c>
+      <c r="AL74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -9456,9 +9681,12 @@
         <v>1</v>
       </c>
       <c r="AJ75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK75" t="n">
         <v>12</v>
       </c>
-      <c r="AK75" t="n">
+      <c r="AL75" t="n">
         <v>12</v>
       </c>
     </row>
@@ -9575,10 +9803,13 @@
         <v>1</v>
       </c>
       <c r="AJ76" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AK76" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AL76" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="77">
@@ -9694,9 +9925,12 @@
         <v>1</v>
       </c>
       <c r="AJ77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK77" t="n">
         <v>14</v>
       </c>
-      <c r="AK77" t="n">
+      <c r="AL77" t="n">
         <v>14</v>
       </c>
     </row>
@@ -9813,9 +10047,12 @@
         <v>1</v>
       </c>
       <c r="AJ78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK78" t="n">
         <v>17</v>
       </c>
-      <c r="AK78" t="n">
+      <c r="AL78" t="n">
         <v>17</v>
       </c>
     </row>
@@ -9932,9 +10169,12 @@
         <v>1</v>
       </c>
       <c r="AJ79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK79" t="n">
         <v>14</v>
       </c>
-      <c r="AK79" t="n">
+      <c r="AL79" t="n">
         <v>14</v>
       </c>
     </row>
@@ -10051,9 +10291,12 @@
         <v>1</v>
       </c>
       <c r="AJ80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK80" t="n">
         <v>8</v>
       </c>
-      <c r="AK80" t="n">
+      <c r="AL80" t="n">
         <v>8</v>
       </c>
     </row>
@@ -10170,9 +10413,12 @@
         <v>1</v>
       </c>
       <c r="AJ81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK81" t="n">
         <v>3</v>
       </c>
-      <c r="AK81" t="n">
+      <c r="AL81" t="n">
         <v>3</v>
       </c>
     </row>
@@ -10289,9 +10535,12 @@
         <v>1</v>
       </c>
       <c r="AJ82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK82" t="n">
         <v>5</v>
       </c>
-      <c r="AK82" t="n">
+      <c r="AL82" t="n">
         <v>5</v>
       </c>
     </row>
@@ -10408,9 +10657,12 @@
         <v>1</v>
       </c>
       <c r="AJ83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK83" t="n">
         <v>13</v>
       </c>
-      <c r="AK83" t="n">
+      <c r="AL83" t="n">
         <v>13</v>
       </c>
     </row>
@@ -10527,9 +10779,12 @@
         <v>0</v>
       </c>
       <c r="AJ84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK84" t="n">
         <v>5</v>
       </c>
-      <c r="AK84" t="n">
+      <c r="AL84" t="n">
         <v>5</v>
       </c>
     </row>
@@ -10646,9 +10901,12 @@
         <v>0</v>
       </c>
       <c r="AJ85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK85" t="n">
         <v>7</v>
       </c>
-      <c r="AK85" t="n">
+      <c r="AL85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10770,6 +11028,9 @@
       <c r="AK86" t="n">
         <v>0</v>
       </c>
+      <c r="AL86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -10884,9 +11145,12 @@
         <v>0</v>
       </c>
       <c r="AJ87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK87" t="n">
         <v>9</v>
       </c>
-      <c r="AK87" t="n">
+      <c r="AL87" t="n">
         <v>9</v>
       </c>
     </row>
@@ -11008,6 +11272,9 @@
       <c r="AK88" t="n">
         <v>0</v>
       </c>
+      <c r="AL88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -11122,9 +11389,12 @@
         <v>1</v>
       </c>
       <c r="AJ89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK89" t="n">
         <v>14</v>
       </c>
-      <c r="AK89" t="n">
+      <c r="AL89" t="n">
         <v>14</v>
       </c>
     </row>
@@ -11241,9 +11511,12 @@
         <v>0</v>
       </c>
       <c r="AJ90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK90" t="n">
         <v>11</v>
       </c>
-      <c r="AK90" t="n">
+      <c r="AL90" t="n">
         <v>11</v>
       </c>
     </row>
@@ -11360,9 +11633,12 @@
         <v>1</v>
       </c>
       <c r="AJ91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK91" t="n">
         <v>40</v>
       </c>
-      <c r="AK91" t="n">
+      <c r="AL91" t="n">
         <v>11</v>
       </c>
     </row>
@@ -11479,9 +11755,12 @@
         <v>1</v>
       </c>
       <c r="AJ92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK92" t="n">
         <v>7</v>
       </c>
-      <c r="AK92" t="n">
+      <c r="AL92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11603,6 +11882,9 @@
       <c r="AK93" t="n">
         <v>0</v>
       </c>
+      <c r="AL93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -11717,9 +11999,12 @@
         <v>1</v>
       </c>
       <c r="AJ94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK94" t="n">
         <v>10</v>
       </c>
-      <c r="AK94" t="n">
+      <c r="AL94" t="n">
         <v>10</v>
       </c>
     </row>
@@ -11836,9 +12121,12 @@
         <v>0</v>
       </c>
       <c r="AJ95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK95" t="n">
         <v>6</v>
       </c>
-      <c r="AK95" t="n">
+      <c r="AL95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -11955,9 +12243,12 @@
         <v>0</v>
       </c>
       <c r="AJ96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK96" t="n">
         <v>14</v>
       </c>
-      <c r="AK96" t="n">
+      <c r="AL96" t="n">
         <v>14</v>
       </c>
     </row>
@@ -12079,6 +12370,9 @@
       <c r="AK97" t="n">
         <v>0</v>
       </c>
+      <c r="AL97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -12193,9 +12487,12 @@
         <v>1</v>
       </c>
       <c r="AJ98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK98" t="n">
         <v>19</v>
       </c>
-      <c r="AK98" t="n">
+      <c r="AL98" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12312,9 +12609,12 @@
         <v>1</v>
       </c>
       <c r="AJ99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK99" t="n">
         <v>4</v>
       </c>
-      <c r="AK99" t="n">
+      <c r="AL99" t="n">
         <v>4</v>
       </c>
     </row>
@@ -12436,6 +12736,9 @@
       <c r="AK100" t="n">
         <v>0</v>
       </c>
+      <c r="AL100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -12550,9 +12853,12 @@
         <v>1</v>
       </c>
       <c r="AJ101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK101" t="n">
         <v>18</v>
       </c>
-      <c r="AK101" t="n">
+      <c r="AL101" t="n">
         <v>18</v>
       </c>
     </row>
@@ -12669,10 +12975,13 @@
         <v>1</v>
       </c>
       <c r="AJ102" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AK102" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AL102" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="103">
@@ -12788,9 +13097,12 @@
         <v>1</v>
       </c>
       <c r="AJ103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK103" t="n">
         <v>17</v>
       </c>
-      <c r="AK103" t="n">
+      <c r="AL103" t="n">
         <v>17</v>
       </c>
     </row>
@@ -12907,9 +13219,12 @@
         <v>1</v>
       </c>
       <c r="AJ104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK104" t="n">
         <v>6</v>
       </c>
-      <c r="AK104" t="n">
+      <c r="AL104" t="n">
         <v>6</v>
       </c>
     </row>
@@ -13026,10 +13341,13 @@
         <v>1</v>
       </c>
       <c r="AJ105" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AK105" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AL105" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="106">
@@ -13145,9 +13463,12 @@
         <v>1</v>
       </c>
       <c r="AJ106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK106" t="n">
         <v>6</v>
       </c>
-      <c r="AK106" t="n">
+      <c r="AL106" t="n">
         <v>6</v>
       </c>
     </row>
@@ -13264,9 +13585,12 @@
         <v>1</v>
       </c>
       <c r="AJ107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK107" t="n">
         <v>5</v>
       </c>
-      <c r="AK107" t="n">
+      <c r="AL107" t="n">
         <v>5</v>
       </c>
     </row>
@@ -13383,9 +13707,12 @@
         <v>0</v>
       </c>
       <c r="AJ108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK108" t="n">
         <v>2</v>
       </c>
-      <c r="AK108" t="n">
+      <c r="AL108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -13502,9 +13829,12 @@
         <v>0</v>
       </c>
       <c r="AJ109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK109" t="n">
         <v>2</v>
       </c>
-      <c r="AK109" t="n">
+      <c r="AL109" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2549)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL109"/>
+  <dimension ref="A1:AM109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -466,8 +466,9 @@
     <col width="12" customWidth="1" min="34" max="34"/>
     <col width="12" customWidth="1" min="35" max="35"/>
     <col width="12" customWidth="1" min="36" max="36"/>
-    <col width="13" customWidth="1" min="37" max="37"/>
+    <col width="12" customWidth="1" min="37" max="37"/>
     <col width="13" customWidth="1" min="38" max="38"/>
+    <col width="13" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -651,12 +652,17 @@
           <t>2026-03-28</t>
         </is>
       </c>
-      <c r="AK1" s="2" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="AL1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AL1" s="2" t="inlineStr">
+      <c r="AM1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -778,9 +784,12 @@
         <v>0</v>
       </c>
       <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="n">
         <v>10</v>
       </c>
-      <c r="AL2" t="n">
+      <c r="AM2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -900,9 +909,12 @@
         <v>0</v>
       </c>
       <c r="AK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL3" t="n">
         <v>8</v>
       </c>
-      <c r="AL3" t="n">
+      <c r="AM3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1022,9 +1034,12 @@
         <v>1</v>
       </c>
       <c r="AK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="n">
         <v>19</v>
       </c>
-      <c r="AL4" t="n">
+      <c r="AM4" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1144,9 +1159,12 @@
         <v>0</v>
       </c>
       <c r="AK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="n">
         <v>15</v>
       </c>
-      <c r="AL5" t="n">
+      <c r="AM5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1266,9 +1284,12 @@
         <v>0</v>
       </c>
       <c r="AK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="n">
         <v>14</v>
       </c>
-      <c r="AL6" t="n">
+      <c r="AM6" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1388,9 +1409,12 @@
         <v>0</v>
       </c>
       <c r="AK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="n">
         <v>13</v>
       </c>
-      <c r="AL7" t="n">
+      <c r="AM7" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1510,9 +1534,12 @@
         <v>0</v>
       </c>
       <c r="AK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL8" t="n">
         <v>18</v>
       </c>
-      <c r="AL8" t="n">
+      <c r="AM8" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1632,9 +1659,12 @@
         <v>0</v>
       </c>
       <c r="AK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" t="n">
         <v>17</v>
       </c>
-      <c r="AL9" t="n">
+      <c r="AM9" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1754,9 +1784,12 @@
         <v>1</v>
       </c>
       <c r="AK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="n">
         <v>19</v>
       </c>
-      <c r="AL10" t="n">
+      <c r="AM10" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1876,9 +1909,12 @@
         <v>0</v>
       </c>
       <c r="AK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="n">
         <v>15</v>
       </c>
-      <c r="AL11" t="n">
+      <c r="AM11" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1998,9 +2034,12 @@
         <v>0</v>
       </c>
       <c r="AK12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL12" t="n">
         <v>18</v>
       </c>
-      <c r="AL12" t="n">
+      <c r="AM12" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2120,9 +2159,12 @@
         <v>0</v>
       </c>
       <c r="AK13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL13" t="n">
         <v>10</v>
       </c>
-      <c r="AL13" t="n">
+      <c r="AM13" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2242,9 +2284,12 @@
         <v>0</v>
       </c>
       <c r="AK14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL14" t="n">
         <v>18</v>
       </c>
-      <c r="AL14" t="n">
+      <c r="AM14" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2364,9 +2409,12 @@
         <v>0</v>
       </c>
       <c r="AK15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL15" t="n">
         <v>9</v>
       </c>
-      <c r="AL15" t="n">
+      <c r="AM15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2486,9 +2534,12 @@
         <v>0</v>
       </c>
       <c r="AK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL16" t="n">
         <v>14</v>
       </c>
-      <c r="AL16" t="n">
+      <c r="AM16" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2608,9 +2659,12 @@
         <v>0</v>
       </c>
       <c r="AK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL17" t="n">
         <v>14</v>
       </c>
-      <c r="AL17" t="n">
+      <c r="AM17" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2730,9 +2784,12 @@
         <v>0</v>
       </c>
       <c r="AK18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL18" t="n">
         <v>16</v>
       </c>
-      <c r="AL18" t="n">
+      <c r="AM18" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2857,6 +2914,9 @@
       <c r="AL19" t="n">
         <v>0</v>
       </c>
+      <c r="AM19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2974,9 +3034,12 @@
         <v>0</v>
       </c>
       <c r="AK20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL20" t="n">
         <v>14</v>
       </c>
-      <c r="AL20" t="n">
+      <c r="AM20" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3096,9 +3159,12 @@
         <v>0</v>
       </c>
       <c r="AK21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL21" t="n">
         <v>17</v>
       </c>
-      <c r="AL21" t="n">
+      <c r="AM21" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3223,6 +3289,9 @@
       <c r="AL22" t="n">
         <v>0</v>
       </c>
+      <c r="AM22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3340,9 +3409,12 @@
         <v>0</v>
       </c>
       <c r="AK23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL23" t="n">
         <v>10</v>
       </c>
-      <c r="AL23" t="n">
+      <c r="AM23" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3462,9 +3534,12 @@
         <v>0</v>
       </c>
       <c r="AK24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL24" t="n">
         <v>17</v>
       </c>
-      <c r="AL24" t="n">
+      <c r="AM24" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3584,9 +3659,12 @@
         <v>0</v>
       </c>
       <c r="AK25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL25" t="n">
         <v>6</v>
       </c>
-      <c r="AL25" t="n">
+      <c r="AM25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3706,9 +3784,12 @@
         <v>0</v>
       </c>
       <c r="AK26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL26" t="n">
         <v>16</v>
       </c>
-      <c r="AL26" t="n">
+      <c r="AM26" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3828,9 +3909,12 @@
         <v>0</v>
       </c>
       <c r="AK27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL27" t="n">
         <v>19</v>
       </c>
-      <c r="AL27" t="n">
+      <c r="AM27" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3950,9 +4034,12 @@
         <v>0</v>
       </c>
       <c r="AK28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL28" t="n">
         <v>6</v>
       </c>
-      <c r="AL28" t="n">
+      <c r="AM28" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4072,9 +4159,12 @@
         <v>0</v>
       </c>
       <c r="AK29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL29" t="n">
         <v>6</v>
       </c>
-      <c r="AL29" t="n">
+      <c r="AM29" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4194,9 +4284,12 @@
         <v>0</v>
       </c>
       <c r="AK30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL30" t="n">
         <v>13</v>
       </c>
-      <c r="AL30" t="n">
+      <c r="AM30" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4316,9 +4409,12 @@
         <v>0</v>
       </c>
       <c r="AK31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL31" t="n">
         <v>15</v>
       </c>
-      <c r="AL31" t="n">
+      <c r="AM31" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4438,9 +4534,12 @@
         <v>0</v>
       </c>
       <c r="AK32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL32" t="n">
         <v>12</v>
       </c>
-      <c r="AL32" t="n">
+      <c r="AM32" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4560,9 +4659,12 @@
         <v>0</v>
       </c>
       <c r="AK33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL33" t="n">
         <v>13</v>
       </c>
-      <c r="AL33" t="n">
+      <c r="AM33" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4682,9 +4784,12 @@
         <v>0</v>
       </c>
       <c r="AK34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL34" t="n">
         <v>7</v>
       </c>
-      <c r="AL34" t="n">
+      <c r="AM34" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4804,9 +4909,12 @@
         <v>0</v>
       </c>
       <c r="AK35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL35" t="n">
         <v>14</v>
       </c>
-      <c r="AL35" t="n">
+      <c r="AM35" t="n">
         <v>14</v>
       </c>
     </row>
@@ -4926,9 +5034,12 @@
         <v>0</v>
       </c>
       <c r="AK36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL36" t="n">
         <v>9</v>
       </c>
-      <c r="AL36" t="n">
+      <c r="AM36" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5053,6 +5164,9 @@
       <c r="AL37" t="n">
         <v>0</v>
       </c>
+      <c r="AM37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5170,9 +5284,12 @@
         <v>0</v>
       </c>
       <c r="AK38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL38" t="n">
         <v>2</v>
       </c>
-      <c r="AL38" t="n">
+      <c r="AM38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5292,9 +5409,12 @@
         <v>0</v>
       </c>
       <c r="AK39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL39" t="n">
         <v>18</v>
       </c>
-      <c r="AL39" t="n">
+      <c r="AM39" t="n">
         <v>18</v>
       </c>
     </row>
@@ -5414,9 +5534,12 @@
         <v>0</v>
       </c>
       <c r="AK40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL40" t="n">
         <v>15</v>
       </c>
-      <c r="AL40" t="n">
+      <c r="AM40" t="n">
         <v>15</v>
       </c>
     </row>
@@ -5536,9 +5659,12 @@
         <v>0</v>
       </c>
       <c r="AK41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL41" t="n">
         <v>19</v>
       </c>
-      <c r="AL41" t="n">
+      <c r="AM41" t="n">
         <v>19</v>
       </c>
     </row>
@@ -5658,9 +5784,12 @@
         <v>0</v>
       </c>
       <c r="AK42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL42" t="n">
         <v>21</v>
       </c>
-      <c r="AL42" t="n">
+      <c r="AM42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5780,9 +5909,12 @@
         <v>0</v>
       </c>
       <c r="AK43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL43" t="n">
         <v>53</v>
       </c>
-      <c r="AL43" t="n">
+      <c r="AM43" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5902,9 +6034,12 @@
         <v>0</v>
       </c>
       <c r="AK44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL44" t="n">
         <v>14</v>
       </c>
-      <c r="AL44" t="n">
+      <c r="AM44" t="n">
         <v>14</v>
       </c>
     </row>
@@ -6024,9 +6159,12 @@
         <v>0</v>
       </c>
       <c r="AK45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL45" t="n">
         <v>17</v>
       </c>
-      <c r="AL45" t="n">
+      <c r="AM45" t="n">
         <v>17</v>
       </c>
     </row>
@@ -6146,9 +6284,12 @@
         <v>0</v>
       </c>
       <c r="AK46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL46" t="n">
         <v>15</v>
       </c>
-      <c r="AL46" t="n">
+      <c r="AM46" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6273,6 +6414,9 @@
       <c r="AL47" t="n">
         <v>0</v>
       </c>
+      <c r="AM47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6390,9 +6534,12 @@
         <v>0</v>
       </c>
       <c r="AK48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL48" t="n">
         <v>17</v>
       </c>
-      <c r="AL48" t="n">
+      <c r="AM48" t="n">
         <v>17</v>
       </c>
     </row>
@@ -6512,9 +6659,12 @@
         <v>0</v>
       </c>
       <c r="AK49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL49" t="n">
         <v>14</v>
       </c>
-      <c r="AL49" t="n">
+      <c r="AM49" t="n">
         <v>14</v>
       </c>
     </row>
@@ -6634,9 +6784,12 @@
         <v>0</v>
       </c>
       <c r="AK50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL50" t="n">
         <v>7</v>
       </c>
-      <c r="AL50" t="n">
+      <c r="AM50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6756,9 +6909,12 @@
         <v>0</v>
       </c>
       <c r="AK51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL51" t="n">
         <v>18</v>
       </c>
-      <c r="AL51" t="n">
+      <c r="AM51" t="n">
         <v>18</v>
       </c>
     </row>
@@ -6883,6 +7039,9 @@
       <c r="AL52" t="n">
         <v>0</v>
       </c>
+      <c r="AM52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7000,9 +7159,12 @@
         <v>0</v>
       </c>
       <c r="AK53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL53" t="n">
         <v>12</v>
       </c>
-      <c r="AL53" t="n">
+      <c r="AM53" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7127,6 +7289,9 @@
       <c r="AL54" t="n">
         <v>0</v>
       </c>
+      <c r="AM54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7244,9 +7409,12 @@
         <v>1</v>
       </c>
       <c r="AK55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL55" t="n">
         <v>18</v>
       </c>
-      <c r="AL55" t="n">
+      <c r="AM55" t="n">
         <v>18</v>
       </c>
     </row>
@@ -7366,9 +7534,12 @@
         <v>0</v>
       </c>
       <c r="AK56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL56" t="n">
         <v>17</v>
       </c>
-      <c r="AL56" t="n">
+      <c r="AM56" t="n">
         <v>17</v>
       </c>
     </row>
@@ -7488,9 +7659,12 @@
         <v>0</v>
       </c>
       <c r="AK57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL57" t="n">
         <v>8</v>
       </c>
-      <c r="AL57" t="n">
+      <c r="AM57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7610,9 +7784,12 @@
         <v>0</v>
       </c>
       <c r="AK58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL58" t="n">
         <v>12</v>
       </c>
-      <c r="AL58" t="n">
+      <c r="AM58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7732,9 +7909,12 @@
         <v>0</v>
       </c>
       <c r="AK59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL59" t="n">
         <v>3</v>
       </c>
-      <c r="AL59" t="n">
+      <c r="AM59" t="n">
         <v>3</v>
       </c>
     </row>
@@ -7859,6 +8039,9 @@
       <c r="AL60" t="n">
         <v>0</v>
       </c>
+      <c r="AM60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7976,9 +8159,12 @@
         <v>0</v>
       </c>
       <c r="AK61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL61" t="n">
         <v>15</v>
       </c>
-      <c r="AL61" t="n">
+      <c r="AM61" t="n">
         <v>15</v>
       </c>
     </row>
@@ -8098,9 +8284,12 @@
         <v>0</v>
       </c>
       <c r="AK62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL62" t="n">
         <v>17</v>
       </c>
-      <c r="AL62" t="n">
+      <c r="AM62" t="n">
         <v>17</v>
       </c>
     </row>
@@ -8220,9 +8409,12 @@
         <v>0</v>
       </c>
       <c r="AK63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL63" t="n">
         <v>7</v>
       </c>
-      <c r="AL63" t="n">
+      <c r="AM63" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8347,6 +8539,9 @@
       <c r="AL64" t="n">
         <v>0</v>
       </c>
+      <c r="AM64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8464,9 +8659,12 @@
         <v>0</v>
       </c>
       <c r="AK65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL65" t="n">
         <v>9</v>
       </c>
-      <c r="AL65" t="n">
+      <c r="AM65" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8586,9 +8784,12 @@
         <v>0</v>
       </c>
       <c r="AK66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL66" t="n">
         <v>2</v>
       </c>
-      <c r="AL66" t="n">
+      <c r="AM66" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8708,9 +8909,12 @@
         <v>0</v>
       </c>
       <c r="AK67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL67" t="n">
         <v>19</v>
       </c>
-      <c r="AL67" t="n">
+      <c r="AM67" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8830,9 +9034,12 @@
         <v>0</v>
       </c>
       <c r="AK68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL68" t="n">
         <v>10</v>
       </c>
-      <c r="AL68" t="n">
+      <c r="AM68" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8952,9 +9159,12 @@
         <v>0</v>
       </c>
       <c r="AK69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL69" t="n">
         <v>7</v>
       </c>
-      <c r="AL69" t="n">
+      <c r="AM69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9074,9 +9284,12 @@
         <v>0</v>
       </c>
       <c r="AK70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL70" t="n">
         <v>23</v>
       </c>
-      <c r="AL70" t="n">
+      <c r="AM70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -9196,9 +9409,12 @@
         <v>0</v>
       </c>
       <c r="AK71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL71" t="n">
         <v>12</v>
       </c>
-      <c r="AL71" t="n">
+      <c r="AM71" t="n">
         <v>12</v>
       </c>
     </row>
@@ -9318,9 +9534,12 @@
         <v>0</v>
       </c>
       <c r="AK72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL72" t="n">
         <v>13</v>
       </c>
-      <c r="AL72" t="n">
+      <c r="AM72" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9445,6 +9664,9 @@
       <c r="AL73" t="n">
         <v>0</v>
       </c>
+      <c r="AM73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9567,6 +9789,9 @@
       <c r="AL74" t="n">
         <v>0</v>
       </c>
+      <c r="AM74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -9684,9 +9909,12 @@
         <v>0</v>
       </c>
       <c r="AK75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL75" t="n">
         <v>12</v>
       </c>
-      <c r="AL75" t="n">
+      <c r="AM75" t="n">
         <v>12</v>
       </c>
     </row>
@@ -9806,9 +10034,12 @@
         <v>1</v>
       </c>
       <c r="AK76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL76" t="n">
         <v>13</v>
       </c>
-      <c r="AL76" t="n">
+      <c r="AM76" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9928,9 +10159,12 @@
         <v>0</v>
       </c>
       <c r="AK77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL77" t="n">
         <v>14</v>
       </c>
-      <c r="AL77" t="n">
+      <c r="AM77" t="n">
         <v>14</v>
       </c>
     </row>
@@ -10050,9 +10284,12 @@
         <v>0</v>
       </c>
       <c r="AK78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL78" t="n">
         <v>17</v>
       </c>
-      <c r="AL78" t="n">
+      <c r="AM78" t="n">
         <v>17</v>
       </c>
     </row>
@@ -10172,9 +10409,12 @@
         <v>0</v>
       </c>
       <c r="AK79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL79" t="n">
         <v>14</v>
       </c>
-      <c r="AL79" t="n">
+      <c r="AM79" t="n">
         <v>14</v>
       </c>
     </row>
@@ -10294,9 +10534,12 @@
         <v>0</v>
       </c>
       <c r="AK80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL80" t="n">
         <v>8</v>
       </c>
-      <c r="AL80" t="n">
+      <c r="AM80" t="n">
         <v>8</v>
       </c>
     </row>
@@ -10416,9 +10659,12 @@
         <v>0</v>
       </c>
       <c r="AK81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL81" t="n">
         <v>3</v>
       </c>
-      <c r="AL81" t="n">
+      <c r="AM81" t="n">
         <v>3</v>
       </c>
     </row>
@@ -10538,9 +10784,12 @@
         <v>0</v>
       </c>
       <c r="AK82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL82" t="n">
         <v>5</v>
       </c>
-      <c r="AL82" t="n">
+      <c r="AM82" t="n">
         <v>5</v>
       </c>
     </row>
@@ -10660,9 +10909,12 @@
         <v>0</v>
       </c>
       <c r="AK83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL83" t="n">
         <v>13</v>
       </c>
-      <c r="AL83" t="n">
+      <c r="AM83" t="n">
         <v>13</v>
       </c>
     </row>
@@ -10782,9 +11034,12 @@
         <v>0</v>
       </c>
       <c r="AK84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL84" t="n">
         <v>5</v>
       </c>
-      <c r="AL84" t="n">
+      <c r="AM84" t="n">
         <v>5</v>
       </c>
     </row>
@@ -10904,9 +11159,12 @@
         <v>0</v>
       </c>
       <c r="AK85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL85" t="n">
         <v>7</v>
       </c>
-      <c r="AL85" t="n">
+      <c r="AM85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11031,6 +11289,9 @@
       <c r="AL86" t="n">
         <v>0</v>
       </c>
+      <c r="AM86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -11148,9 +11409,12 @@
         <v>0</v>
       </c>
       <c r="AK87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL87" t="n">
         <v>9</v>
       </c>
-      <c r="AL87" t="n">
+      <c r="AM87" t="n">
         <v>9</v>
       </c>
     </row>
@@ -11275,6 +11539,9 @@
       <c r="AL88" t="n">
         <v>0</v>
       </c>
+      <c r="AM88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -11392,9 +11659,12 @@
         <v>0</v>
       </c>
       <c r="AK89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL89" t="n">
         <v>14</v>
       </c>
-      <c r="AL89" t="n">
+      <c r="AM89" t="n">
         <v>14</v>
       </c>
     </row>
@@ -11514,9 +11784,12 @@
         <v>0</v>
       </c>
       <c r="AK90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL90" t="n">
         <v>11</v>
       </c>
-      <c r="AL90" t="n">
+      <c r="AM90" t="n">
         <v>11</v>
       </c>
     </row>
@@ -11636,9 +11909,12 @@
         <v>0</v>
       </c>
       <c r="AK91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL91" t="n">
         <v>40</v>
       </c>
-      <c r="AL91" t="n">
+      <c r="AM91" t="n">
         <v>11</v>
       </c>
     </row>
@@ -11758,9 +12034,12 @@
         <v>0</v>
       </c>
       <c r="AK92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL92" t="n">
         <v>7</v>
       </c>
-      <c r="AL92" t="n">
+      <c r="AM92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11885,6 +12164,9 @@
       <c r="AL93" t="n">
         <v>0</v>
       </c>
+      <c r="AM93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -12002,9 +12284,12 @@
         <v>0</v>
       </c>
       <c r="AK94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL94" t="n">
         <v>10</v>
       </c>
-      <c r="AL94" t="n">
+      <c r="AM94" t="n">
         <v>10</v>
       </c>
     </row>
@@ -12124,9 +12409,12 @@
         <v>0</v>
       </c>
       <c r="AK95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL95" t="n">
         <v>6</v>
       </c>
-      <c r="AL95" t="n">
+      <c r="AM95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -12246,9 +12534,12 @@
         <v>0</v>
       </c>
       <c r="AK96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL96" t="n">
         <v>14</v>
       </c>
-      <c r="AL96" t="n">
+      <c r="AM96" t="n">
         <v>14</v>
       </c>
     </row>
@@ -12373,6 +12664,9 @@
       <c r="AL97" t="n">
         <v>0</v>
       </c>
+      <c r="AM97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -12490,9 +12784,12 @@
         <v>0</v>
       </c>
       <c r="AK98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL98" t="n">
         <v>19</v>
       </c>
-      <c r="AL98" t="n">
+      <c r="AM98" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12612,9 +12909,12 @@
         <v>0</v>
       </c>
       <c r="AK99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL99" t="n">
         <v>4</v>
       </c>
-      <c r="AL99" t="n">
+      <c r="AM99" t="n">
         <v>4</v>
       </c>
     </row>
@@ -12739,6 +13039,9 @@
       <c r="AL100" t="n">
         <v>0</v>
       </c>
+      <c r="AM100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -12856,10 +13159,13 @@
         <v>0</v>
       </c>
       <c r="AK101" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AL101" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AM101" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="102">
@@ -12978,9 +13284,12 @@
         <v>1</v>
       </c>
       <c r="AK102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL102" t="n">
         <v>17</v>
       </c>
-      <c r="AL102" t="n">
+      <c r="AM102" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13100,9 +13409,12 @@
         <v>0</v>
       </c>
       <c r="AK103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL103" t="n">
         <v>17</v>
       </c>
-      <c r="AL103" t="n">
+      <c r="AM103" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13222,9 +13534,12 @@
         <v>0</v>
       </c>
       <c r="AK104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL104" t="n">
         <v>6</v>
       </c>
-      <c r="AL104" t="n">
+      <c r="AM104" t="n">
         <v>6</v>
       </c>
     </row>
@@ -13344,9 +13659,12 @@
         <v>1</v>
       </c>
       <c r="AK105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL105" t="n">
         <v>8</v>
       </c>
-      <c r="AL105" t="n">
+      <c r="AM105" t="n">
         <v>8</v>
       </c>
     </row>
@@ -13466,9 +13784,12 @@
         <v>0</v>
       </c>
       <c r="AK106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL106" t="n">
         <v>6</v>
       </c>
-      <c r="AL106" t="n">
+      <c r="AM106" t="n">
         <v>6</v>
       </c>
     </row>
@@ -13588,9 +13909,12 @@
         <v>0</v>
       </c>
       <c r="AK107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL107" t="n">
         <v>5</v>
       </c>
-      <c r="AL107" t="n">
+      <c r="AM107" t="n">
         <v>5</v>
       </c>
     </row>
@@ -13710,9 +14034,12 @@
         <v>0</v>
       </c>
       <c r="AK108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL108" t="n">
         <v>2</v>
       </c>
-      <c r="AL108" t="n">
+      <c r="AM108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -13832,9 +14159,12 @@
         <v>0</v>
       </c>
       <c r="AK109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL109" t="n">
         <v>2</v>
       </c>
-      <c r="AL109" t="n">
+      <c r="AM109" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2631)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM109"/>
+  <dimension ref="A1:AN109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -467,8 +467,9 @@
     <col width="12" customWidth="1" min="35" max="35"/>
     <col width="12" customWidth="1" min="36" max="36"/>
     <col width="12" customWidth="1" min="37" max="37"/>
-    <col width="13" customWidth="1" min="38" max="38"/>
+    <col width="12" customWidth="1" min="38" max="38"/>
     <col width="13" customWidth="1" min="39" max="39"/>
+    <col width="13" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -657,12 +658,17 @@
           <t>2026-03-29</t>
         </is>
       </c>
-      <c r="AL1" s="2" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="AM1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AM1" s="2" t="inlineStr">
+      <c r="AN1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -787,9 +793,12 @@
         <v>0</v>
       </c>
       <c r="AL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="n">
         <v>10</v>
       </c>
-      <c r="AM2" t="n">
+      <c r="AN2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -912,9 +921,12 @@
         <v>0</v>
       </c>
       <c r="AL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM3" t="n">
         <v>8</v>
       </c>
-      <c r="AM3" t="n">
+      <c r="AN3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1037,10 +1049,13 @@
         <v>0</v>
       </c>
       <c r="AL4" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AM4" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -1162,9 +1177,12 @@
         <v>0</v>
       </c>
       <c r="AL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" t="n">
         <v>15</v>
       </c>
-      <c r="AM5" t="n">
+      <c r="AN5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1287,10 +1305,13 @@
         <v>0</v>
       </c>
       <c r="AL6" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AM6" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -1412,10 +1433,13 @@
         <v>0</v>
       </c>
       <c r="AL7" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AM7" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -1537,10 +1561,13 @@
         <v>0</v>
       </c>
       <c r="AL8" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AM8" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -1662,10 +1689,13 @@
         <v>0</v>
       </c>
       <c r="AL9" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AM9" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -1787,10 +1817,13 @@
         <v>0</v>
       </c>
       <c r="AL10" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AM10" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -1912,10 +1945,13 @@
         <v>0</v>
       </c>
       <c r="AL11" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AM11" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="12">
@@ -2037,10 +2073,13 @@
         <v>0</v>
       </c>
       <c r="AL12" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AM12" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="13">
@@ -2162,10 +2201,13 @@
         <v>0</v>
       </c>
       <c r="AL13" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AM13" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -2287,10 +2329,13 @@
         <v>0</v>
       </c>
       <c r="AL14" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AM14" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="15">
@@ -2412,9 +2457,12 @@
         <v>0</v>
       </c>
       <c r="AL15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM15" t="n">
         <v>9</v>
       </c>
-      <c r="AM15" t="n">
+      <c r="AN15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2537,9 +2585,12 @@
         <v>0</v>
       </c>
       <c r="AL16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM16" t="n">
         <v>14</v>
       </c>
-      <c r="AM16" t="n">
+      <c r="AN16" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2662,9 +2713,12 @@
         <v>0</v>
       </c>
       <c r="AL17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM17" t="n">
         <v>14</v>
       </c>
-      <c r="AM17" t="n">
+      <c r="AN17" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2787,10 +2841,13 @@
         <v>0</v>
       </c>
       <c r="AL18" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AM18" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="19">
@@ -2917,6 +2974,9 @@
       <c r="AM19" t="n">
         <v>0</v>
       </c>
+      <c r="AN19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3037,9 +3097,12 @@
         <v>0</v>
       </c>
       <c r="AL20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM20" t="n">
         <v>14</v>
       </c>
-      <c r="AM20" t="n">
+      <c r="AN20" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3162,10 +3225,13 @@
         <v>0</v>
       </c>
       <c r="AL21" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AM21" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="22">
@@ -3292,6 +3358,9 @@
       <c r="AM22" t="n">
         <v>0</v>
       </c>
+      <c r="AN22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3412,10 +3481,13 @@
         <v>0</v>
       </c>
       <c r="AL23" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AM23" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AN23" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="24">
@@ -3537,10 +3609,13 @@
         <v>0</v>
       </c>
       <c r="AL24" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AM24" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="25">
@@ -3662,9 +3737,12 @@
         <v>0</v>
       </c>
       <c r="AL25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM25" t="n">
         <v>6</v>
       </c>
-      <c r="AM25" t="n">
+      <c r="AN25" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3787,10 +3865,13 @@
         <v>0</v>
       </c>
       <c r="AL26" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AM26" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="27">
@@ -3912,10 +3993,13 @@
         <v>0</v>
       </c>
       <c r="AL27" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AM27" t="n">
-        <v>17</v>
+        <v>20</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="28">
@@ -4037,9 +4121,12 @@
         <v>0</v>
       </c>
       <c r="AL28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM28" t="n">
         <v>6</v>
       </c>
-      <c r="AM28" t="n">
+      <c r="AN28" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4162,9 +4249,12 @@
         <v>0</v>
       </c>
       <c r="AL29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM29" t="n">
         <v>6</v>
       </c>
-      <c r="AM29" t="n">
+      <c r="AN29" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4287,10 +4377,13 @@
         <v>0</v>
       </c>
       <c r="AL30" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AM30" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="31">
@@ -4412,10 +4505,13 @@
         <v>0</v>
       </c>
       <c r="AL31" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AM31" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="32">
@@ -4537,9 +4633,12 @@
         <v>0</v>
       </c>
       <c r="AL32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM32" t="n">
         <v>12</v>
       </c>
-      <c r="AM32" t="n">
+      <c r="AN32" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4662,9 +4761,12 @@
         <v>0</v>
       </c>
       <c r="AL33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM33" t="n">
         <v>13</v>
       </c>
-      <c r="AM33" t="n">
+      <c r="AN33" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4787,10 +4889,13 @@
         <v>0</v>
       </c>
       <c r="AL34" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AM34" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AN34" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="35">
@@ -4912,10 +5017,13 @@
         <v>0</v>
       </c>
       <c r="AL35" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AM35" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AN35" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="36">
@@ -5037,9 +5145,12 @@
         <v>0</v>
       </c>
       <c r="AL36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM36" t="n">
         <v>9</v>
       </c>
-      <c r="AM36" t="n">
+      <c r="AN36" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5167,6 +5278,9 @@
       <c r="AM37" t="n">
         <v>0</v>
       </c>
+      <c r="AN37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5287,9 +5401,12 @@
         <v>0</v>
       </c>
       <c r="AL38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM38" t="n">
         <v>2</v>
       </c>
-      <c r="AM38" t="n">
+      <c r="AN38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5412,10 +5529,13 @@
         <v>0</v>
       </c>
       <c r="AL39" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AM39" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AN39" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="40">
@@ -5537,10 +5657,13 @@
         <v>0</v>
       </c>
       <c r="AL40" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AM40" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AN40" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="41">
@@ -5662,10 +5785,13 @@
         <v>0</v>
       </c>
       <c r="AL41" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AM41" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AN41" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="42">
@@ -5787,9 +5913,12 @@
         <v>0</v>
       </c>
       <c r="AL42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM42" t="n">
         <v>21</v>
       </c>
-      <c r="AM42" t="n">
+      <c r="AN42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5912,10 +6041,13 @@
         <v>0</v>
       </c>
       <c r="AL43" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="AM43" t="n">
-        <v>12</v>
+        <v>54</v>
+      </c>
+      <c r="AN43" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="44">
@@ -6037,10 +6169,13 @@
         <v>0</v>
       </c>
       <c r="AL44" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AM44" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AN44" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="45">
@@ -6162,10 +6297,13 @@
         <v>0</v>
       </c>
       <c r="AL45" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AM45" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AN45" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="46">
@@ -6287,10 +6425,13 @@
         <v>0</v>
       </c>
       <c r="AL46" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AM46" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AN46" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="47">
@@ -6417,6 +6558,9 @@
       <c r="AM47" t="n">
         <v>0</v>
       </c>
+      <c r="AN47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6537,10 +6681,13 @@
         <v>0</v>
       </c>
       <c r="AL48" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AM48" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AN48" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="49">
@@ -6662,10 +6809,13 @@
         <v>0</v>
       </c>
       <c r="AL49" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AM49" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AN49" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="50">
@@ -6787,9 +6937,12 @@
         <v>0</v>
       </c>
       <c r="AL50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM50" t="n">
         <v>7</v>
       </c>
-      <c r="AM50" t="n">
+      <c r="AN50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6912,10 +7065,13 @@
         <v>0</v>
       </c>
       <c r="AL51" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AM51" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AN51" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="52">
@@ -7042,6 +7198,9 @@
       <c r="AM52" t="n">
         <v>0</v>
       </c>
+      <c r="AN52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7162,9 +7321,12 @@
         <v>0</v>
       </c>
       <c r="AL53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM53" t="n">
         <v>12</v>
       </c>
-      <c r="AM53" t="n">
+      <c r="AN53" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7292,6 +7454,9 @@
       <c r="AM54" t="n">
         <v>0</v>
       </c>
+      <c r="AN54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7412,10 +7577,13 @@
         <v>0</v>
       </c>
       <c r="AL55" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AM55" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AN55" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="56">
@@ -7537,10 +7705,13 @@
         <v>0</v>
       </c>
       <c r="AL56" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AM56" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AN56" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="57">
@@ -7662,9 +7833,12 @@
         <v>0</v>
       </c>
       <c r="AL57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM57" t="n">
         <v>8</v>
       </c>
-      <c r="AM57" t="n">
+      <c r="AN57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7787,9 +7961,12 @@
         <v>0</v>
       </c>
       <c r="AL58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM58" t="n">
         <v>12</v>
       </c>
-      <c r="AM58" t="n">
+      <c r="AN58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7912,10 +8089,13 @@
         <v>0</v>
       </c>
       <c r="AL59" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AM59" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AN59" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="60">
@@ -8042,6 +8222,9 @@
       <c r="AM60" t="n">
         <v>0</v>
       </c>
+      <c r="AN60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8162,10 +8345,13 @@
         <v>0</v>
       </c>
       <c r="AL61" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AM61" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AN61" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="62">
@@ -8287,10 +8473,13 @@
         <v>0</v>
       </c>
       <c r="AL62" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AM62" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AN62" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="63">
@@ -8412,10 +8601,13 @@
         <v>0</v>
       </c>
       <c r="AL63" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AM63" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AN63" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="64">
@@ -8542,6 +8734,9 @@
       <c r="AM64" t="n">
         <v>0</v>
       </c>
+      <c r="AN64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8662,10 +8857,13 @@
         <v>0</v>
       </c>
       <c r="AL65" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AM65" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AN65" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="66">
@@ -8787,10 +8985,13 @@
         <v>0</v>
       </c>
       <c r="AL66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM66" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AN66" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="67">
@@ -8912,10 +9113,13 @@
         <v>0</v>
       </c>
       <c r="AL67" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AM67" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AN67" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="68">
@@ -9037,10 +9241,13 @@
         <v>0</v>
       </c>
       <c r="AL68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM68" t="n">
+        <v>11</v>
+      </c>
+      <c r="AN68" t="n">
         <v>10</v>
-      </c>
-      <c r="AM68" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="69">
@@ -9162,9 +9369,12 @@
         <v>0</v>
       </c>
       <c r="AL69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM69" t="n">
         <v>7</v>
       </c>
-      <c r="AM69" t="n">
+      <c r="AN69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9287,9 +9497,12 @@
         <v>0</v>
       </c>
       <c r="AL70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM70" t="n">
         <v>23</v>
       </c>
-      <c r="AM70" t="n">
+      <c r="AN70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -9412,10 +9625,13 @@
         <v>0</v>
       </c>
       <c r="AL71" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AM71" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AN71" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="72">
@@ -9537,10 +9753,13 @@
         <v>0</v>
       </c>
       <c r="AL72" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AM72" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AN72" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="73">
@@ -9667,6 +9886,9 @@
       <c r="AM73" t="n">
         <v>0</v>
       </c>
+      <c r="AN73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9792,6 +10014,9 @@
       <c r="AM74" t="n">
         <v>0</v>
       </c>
+      <c r="AN74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -9912,10 +10137,13 @@
         <v>0</v>
       </c>
       <c r="AL75" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AM75" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AN75" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="76">
@@ -10037,10 +10265,13 @@
         <v>0</v>
       </c>
       <c r="AL76" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AM76" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AN76" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="77">
@@ -10162,10 +10393,13 @@
         <v>0</v>
       </c>
       <c r="AL77" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AM77" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AN77" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="78">
@@ -10287,9 +10521,12 @@
         <v>0</v>
       </c>
       <c r="AL78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM78" t="n">
         <v>17</v>
       </c>
-      <c r="AM78" t="n">
+      <c r="AN78" t="n">
         <v>17</v>
       </c>
     </row>
@@ -10412,10 +10649,13 @@
         <v>0</v>
       </c>
       <c r="AL79" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AM79" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AN79" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="80">
@@ -10537,9 +10777,12 @@
         <v>0</v>
       </c>
       <c r="AL80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM80" t="n">
         <v>8</v>
       </c>
-      <c r="AM80" t="n">
+      <c r="AN80" t="n">
         <v>8</v>
       </c>
     </row>
@@ -10662,9 +10905,12 @@
         <v>0</v>
       </c>
       <c r="AL81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM81" t="n">
         <v>3</v>
       </c>
-      <c r="AM81" t="n">
+      <c r="AN81" t="n">
         <v>3</v>
       </c>
     </row>
@@ -10787,9 +11033,12 @@
         <v>0</v>
       </c>
       <c r="AL82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM82" t="n">
         <v>5</v>
       </c>
-      <c r="AM82" t="n">
+      <c r="AN82" t="n">
         <v>5</v>
       </c>
     </row>
@@ -10912,10 +11161,13 @@
         <v>0</v>
       </c>
       <c r="AL83" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AM83" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AN83" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="84">
@@ -11037,9 +11289,12 @@
         <v>0</v>
       </c>
       <c r="AL84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM84" t="n">
         <v>5</v>
       </c>
-      <c r="AM84" t="n">
+      <c r="AN84" t="n">
         <v>5</v>
       </c>
     </row>
@@ -11162,9 +11417,12 @@
         <v>0</v>
       </c>
       <c r="AL85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM85" t="n">
         <v>7</v>
       </c>
-      <c r="AM85" t="n">
+      <c r="AN85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11292,6 +11550,9 @@
       <c r="AM86" t="n">
         <v>0</v>
       </c>
+      <c r="AN86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -11412,10 +11673,13 @@
         <v>0</v>
       </c>
       <c r="AL87" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AM87" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AN87" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="88">
@@ -11542,6 +11806,9 @@
       <c r="AM88" t="n">
         <v>0</v>
       </c>
+      <c r="AN88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -11662,9 +11929,12 @@
         <v>0</v>
       </c>
       <c r="AL89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM89" t="n">
         <v>14</v>
       </c>
-      <c r="AM89" t="n">
+      <c r="AN89" t="n">
         <v>14</v>
       </c>
     </row>
@@ -11787,10 +12057,13 @@
         <v>0</v>
       </c>
       <c r="AL90" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AM90" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AN90" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="91">
@@ -11912,10 +12185,13 @@
         <v>0</v>
       </c>
       <c r="AL91" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="AM91" t="n">
-        <v>11</v>
+        <v>41</v>
+      </c>
+      <c r="AN91" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="92">
@@ -12037,9 +12313,12 @@
         <v>0</v>
       </c>
       <c r="AL92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM92" t="n">
         <v>7</v>
       </c>
-      <c r="AM92" t="n">
+      <c r="AN92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12167,6 +12446,9 @@
       <c r="AM93" t="n">
         <v>0</v>
       </c>
+      <c r="AN93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -12287,10 +12569,13 @@
         <v>0</v>
       </c>
       <c r="AL94" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AM94" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AN94" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="95">
@@ -12412,9 +12697,12 @@
         <v>0</v>
       </c>
       <c r="AL95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM95" t="n">
         <v>6</v>
       </c>
-      <c r="AM95" t="n">
+      <c r="AN95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -12537,10 +12825,13 @@
         <v>0</v>
       </c>
       <c r="AL96" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AM96" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AN96" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="97">
@@ -12667,6 +12958,9 @@
       <c r="AM97" t="n">
         <v>0</v>
       </c>
+      <c r="AN97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -12787,9 +13081,12 @@
         <v>0</v>
       </c>
       <c r="AL98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM98" t="n">
         <v>19</v>
       </c>
-      <c r="AM98" t="n">
+      <c r="AN98" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12912,10 +13209,13 @@
         <v>0</v>
       </c>
       <c r="AL99" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AM99" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AN99" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="100">
@@ -13042,6 +13342,9 @@
       <c r="AM100" t="n">
         <v>0</v>
       </c>
+      <c r="AN100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -13162,10 +13465,13 @@
         <v>1</v>
       </c>
       <c r="AL101" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AM101" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AN101" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="102">
@@ -13287,10 +13593,13 @@
         <v>0</v>
       </c>
       <c r="AL102" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AM102" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AN102" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="103">
@@ -13412,9 +13721,12 @@
         <v>0</v>
       </c>
       <c r="AL103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM103" t="n">
         <v>17</v>
       </c>
-      <c r="AM103" t="n">
+      <c r="AN103" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13537,10 +13849,13 @@
         <v>0</v>
       </c>
       <c r="AL104" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AM104" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AN104" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="105">
@@ -13662,10 +13977,13 @@
         <v>0</v>
       </c>
       <c r="AL105" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AM105" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AN105" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="106">
@@ -13787,10 +14105,13 @@
         <v>0</v>
       </c>
       <c r="AL106" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AM106" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AN106" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="107">
@@ -13912,10 +14233,13 @@
         <v>0</v>
       </c>
       <c r="AL107" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AM107" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AN107" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="108">
@@ -14037,9 +14361,12 @@
         <v>0</v>
       </c>
       <c r="AL108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM108" t="n">
         <v>2</v>
       </c>
-      <c r="AM108" t="n">
+      <c r="AN108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -14162,9 +14489,12 @@
         <v>0</v>
       </c>
       <c r="AL109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM109" t="n">
         <v>2</v>
       </c>
-      <c r="AM109" t="n">
+      <c r="AN109" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2774)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN109"/>
+  <dimension ref="A1:AO109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -468,8 +468,9 @@
     <col width="12" customWidth="1" min="36" max="36"/>
     <col width="12" customWidth="1" min="37" max="37"/>
     <col width="12" customWidth="1" min="38" max="38"/>
-    <col width="13" customWidth="1" min="39" max="39"/>
+    <col width="12" customWidth="1" min="39" max="39"/>
     <col width="13" customWidth="1" min="40" max="40"/>
+    <col width="13" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -663,12 +664,17 @@
           <t>2026-03-30</t>
         </is>
       </c>
-      <c r="AM1" s="2" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="AN1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AN1" s="2" t="inlineStr">
+      <c r="AO1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -796,9 +802,12 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN2" t="n">
         <v>10</v>
       </c>
-      <c r="AN2" t="n">
+      <c r="AO2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -924,9 +933,12 @@
         <v>0</v>
       </c>
       <c r="AM3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN3" t="n">
         <v>8</v>
       </c>
-      <c r="AN3" t="n">
+      <c r="AO3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1052,10 +1064,13 @@
         <v>1</v>
       </c>
       <c r="AM4" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AN4" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -1180,9 +1195,12 @@
         <v>0</v>
       </c>
       <c r="AM5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN5" t="n">
         <v>15</v>
       </c>
-      <c r="AN5" t="n">
+      <c r="AO5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1308,10 +1326,13 @@
         <v>1</v>
       </c>
       <c r="AM6" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AN6" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -1436,10 +1457,13 @@
         <v>1</v>
       </c>
       <c r="AM7" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AN7" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -1564,10 +1588,13 @@
         <v>1</v>
       </c>
       <c r="AM8" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AN8" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -1692,9 +1719,12 @@
         <v>1</v>
       </c>
       <c r="AM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN9" t="n">
         <v>18</v>
       </c>
-      <c r="AN9" t="n">
+      <c r="AO9" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1820,10 +1850,13 @@
         <v>1</v>
       </c>
       <c r="AM10" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AN10" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="11">
@@ -1948,10 +1981,13 @@
         <v>1</v>
       </c>
       <c r="AM11" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AN11" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="12">
@@ -2076,10 +2112,13 @@
         <v>1</v>
       </c>
       <c r="AM12" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AN12" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="13">
@@ -2204,9 +2243,12 @@
         <v>1</v>
       </c>
       <c r="AM13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN13" t="n">
         <v>11</v>
       </c>
-      <c r="AN13" t="n">
+      <c r="AO13" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2332,10 +2374,13 @@
         <v>1</v>
       </c>
       <c r="AM14" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AN14" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="15">
@@ -2460,9 +2505,12 @@
         <v>0</v>
       </c>
       <c r="AM15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN15" t="n">
         <v>9</v>
       </c>
-      <c r="AN15" t="n">
+      <c r="AO15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2588,10 +2636,13 @@
         <v>0</v>
       </c>
       <c r="AM16" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AN16" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -2716,10 +2767,13 @@
         <v>0</v>
       </c>
       <c r="AM17" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AN17" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="18">
@@ -2844,10 +2898,13 @@
         <v>1</v>
       </c>
       <c r="AM18" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AN18" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="19">
@@ -2977,6 +3034,9 @@
       <c r="AN19" t="n">
         <v>0</v>
       </c>
+      <c r="AO19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3100,9 +3160,12 @@
         <v>0</v>
       </c>
       <c r="AM20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN20" t="n">
         <v>14</v>
       </c>
-      <c r="AN20" t="n">
+      <c r="AO20" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3228,10 +3291,13 @@
         <v>1</v>
       </c>
       <c r="AM21" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AN21" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AO21" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="22">
@@ -3361,6 +3427,9 @@
       <c r="AN22" t="n">
         <v>0</v>
       </c>
+      <c r="AO22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3484,10 +3553,13 @@
         <v>1</v>
       </c>
       <c r="AM23" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AN23" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AO23" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="24">
@@ -3612,10 +3684,13 @@
         <v>1</v>
       </c>
       <c r="AM24" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AN24" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="25">
@@ -3740,10 +3815,13 @@
         <v>0</v>
       </c>
       <c r="AM25" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AN25" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AO25" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="26">
@@ -3868,10 +3946,13 @@
         <v>1</v>
       </c>
       <c r="AM26" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AN26" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AO26" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="27">
@@ -3996,9 +4077,12 @@
         <v>1</v>
       </c>
       <c r="AM27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN27" t="n">
         <v>20</v>
       </c>
-      <c r="AN27" t="n">
+      <c r="AO27" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4124,10 +4208,13 @@
         <v>0</v>
       </c>
       <c r="AM28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AN28" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="29">
@@ -4252,10 +4339,13 @@
         <v>0</v>
       </c>
       <c r="AM29" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AN29" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AO29" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="30">
@@ -4380,10 +4470,13 @@
         <v>1</v>
       </c>
       <c r="AM30" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AN30" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="31">
@@ -4508,9 +4601,12 @@
         <v>1</v>
       </c>
       <c r="AM31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN31" t="n">
         <v>16</v>
       </c>
-      <c r="AN31" t="n">
+      <c r="AO31" t="n">
         <v>16</v>
       </c>
     </row>
@@ -4636,10 +4732,13 @@
         <v>0</v>
       </c>
       <c r="AM32" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AN32" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="33">
@@ -4764,9 +4863,12 @@
         <v>0</v>
       </c>
       <c r="AM33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN33" t="n">
         <v>13</v>
       </c>
-      <c r="AN33" t="n">
+      <c r="AO33" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4892,9 +4994,12 @@
         <v>1</v>
       </c>
       <c r="AM34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN34" t="n">
         <v>8</v>
       </c>
-      <c r="AN34" t="n">
+      <c r="AO34" t="n">
         <v>8</v>
       </c>
     </row>
@@ -5020,10 +5125,13 @@
         <v>1</v>
       </c>
       <c r="AM35" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AN35" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AO35" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="36">
@@ -5148,9 +5256,12 @@
         <v>0</v>
       </c>
       <c r="AM36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN36" t="n">
         <v>9</v>
       </c>
-      <c r="AN36" t="n">
+      <c r="AO36" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5281,6 +5392,9 @@
       <c r="AN37" t="n">
         <v>0</v>
       </c>
+      <c r="AO37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5404,9 +5518,12 @@
         <v>0</v>
       </c>
       <c r="AM38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN38" t="n">
         <v>2</v>
       </c>
-      <c r="AN38" t="n">
+      <c r="AO38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5532,10 +5649,13 @@
         <v>1</v>
       </c>
       <c r="AM39" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AN39" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AO39" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="40">
@@ -5660,9 +5780,12 @@
         <v>1</v>
       </c>
       <c r="AM40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN40" t="n">
         <v>16</v>
       </c>
-      <c r="AN40" t="n">
+      <c r="AO40" t="n">
         <v>16</v>
       </c>
     </row>
@@ -5788,10 +5911,13 @@
         <v>1</v>
       </c>
       <c r="AM41" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AN41" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AO41" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="42">
@@ -5916,9 +6042,12 @@
         <v>0</v>
       </c>
       <c r="AM42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN42" t="n">
         <v>21</v>
       </c>
-      <c r="AN42" t="n">
+      <c r="AO42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6044,10 +6173,13 @@
         <v>1</v>
       </c>
       <c r="AM43" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="AN43" t="n">
-        <v>13</v>
+        <v>55</v>
+      </c>
+      <c r="AO43" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="44">
@@ -6172,10 +6304,13 @@
         <v>1</v>
       </c>
       <c r="AM44" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AN44" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AO44" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="45">
@@ -6300,10 +6435,13 @@
         <v>1</v>
       </c>
       <c r="AM45" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AN45" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AO45" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="46">
@@ -6428,9 +6566,12 @@
         <v>1</v>
       </c>
       <c r="AM46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN46" t="n">
         <v>16</v>
       </c>
-      <c r="AN46" t="n">
+      <c r="AO46" t="n">
         <v>16</v>
       </c>
     </row>
@@ -6561,6 +6702,9 @@
       <c r="AN47" t="n">
         <v>0</v>
       </c>
+      <c r="AO47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6684,10 +6828,13 @@
         <v>1</v>
       </c>
       <c r="AM48" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AN48" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AO48" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="49">
@@ -6812,10 +6959,13 @@
         <v>1</v>
       </c>
       <c r="AM49" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AN49" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AO49" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="50">
@@ -6940,9 +7090,12 @@
         <v>0</v>
       </c>
       <c r="AM50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN50" t="n">
         <v>7</v>
       </c>
-      <c r="AN50" t="n">
+      <c r="AO50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7068,10 +7221,13 @@
         <v>1</v>
       </c>
       <c r="AM51" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AN51" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AO51" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="52">
@@ -7201,6 +7357,9 @@
       <c r="AN52" t="n">
         <v>0</v>
       </c>
+      <c r="AO52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7324,9 +7483,12 @@
         <v>0</v>
       </c>
       <c r="AM53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN53" t="n">
         <v>12</v>
       </c>
-      <c r="AN53" t="n">
+      <c r="AO53" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7457,6 +7619,9 @@
       <c r="AN54" t="n">
         <v>0</v>
       </c>
+      <c r="AO54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7580,10 +7745,13 @@
         <v>1</v>
       </c>
       <c r="AM55" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AN55" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AO55" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="56">
@@ -7708,9 +7876,12 @@
         <v>1</v>
       </c>
       <c r="AM56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN56" t="n">
         <v>18</v>
       </c>
-      <c r="AN56" t="n">
+      <c r="AO56" t="n">
         <v>18</v>
       </c>
     </row>
@@ -7836,9 +8007,12 @@
         <v>0</v>
       </c>
       <c r="AM57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN57" t="n">
         <v>8</v>
       </c>
-      <c r="AN57" t="n">
+      <c r="AO57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7964,9 +8138,12 @@
         <v>0</v>
       </c>
       <c r="AM58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN58" t="n">
         <v>12</v>
       </c>
-      <c r="AN58" t="n">
+      <c r="AO58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -8092,10 +8269,13 @@
         <v>1</v>
       </c>
       <c r="AM59" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AN59" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AO59" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="60">
@@ -8225,6 +8405,9 @@
       <c r="AN60" t="n">
         <v>0</v>
       </c>
+      <c r="AO60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8348,10 +8531,13 @@
         <v>1</v>
       </c>
       <c r="AM61" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AN61" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AO61" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="62">
@@ -8476,10 +8662,13 @@
         <v>1</v>
       </c>
       <c r="AM62" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AN62" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AO62" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="63">
@@ -8604,9 +8793,12 @@
         <v>1</v>
       </c>
       <c r="AM63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN63" t="n">
         <v>8</v>
       </c>
-      <c r="AN63" t="n">
+      <c r="AO63" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8737,6 +8929,9 @@
       <c r="AN64" t="n">
         <v>0</v>
       </c>
+      <c r="AO64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8860,9 +9055,12 @@
         <v>1</v>
       </c>
       <c r="AM65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN65" t="n">
         <v>10</v>
       </c>
-      <c r="AN65" t="n">
+      <c r="AO65" t="n">
         <v>10</v>
       </c>
     </row>
@@ -8988,9 +9186,12 @@
         <v>1</v>
       </c>
       <c r="AM66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN66" t="n">
         <v>3</v>
       </c>
-      <c r="AN66" t="n">
+      <c r="AO66" t="n">
         <v>3</v>
       </c>
     </row>
@@ -9116,10 +9317,13 @@
         <v>1</v>
       </c>
       <c r="AM67" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AN67" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AO67" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="68">
@@ -9244,10 +9448,13 @@
         <v>1</v>
       </c>
       <c r="AM68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN68" t="n">
+        <v>12</v>
+      </c>
+      <c r="AO68" t="n">
         <v>11</v>
-      </c>
-      <c r="AN68" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="69">
@@ -9372,9 +9579,12 @@
         <v>0</v>
       </c>
       <c r="AM69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN69" t="n">
         <v>7</v>
       </c>
-      <c r="AN69" t="n">
+      <c r="AO69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9500,9 +9710,12 @@
         <v>0</v>
       </c>
       <c r="AM70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN70" t="n">
         <v>23</v>
       </c>
-      <c r="AN70" t="n">
+      <c r="AO70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -9628,10 +9841,13 @@
         <v>1</v>
       </c>
       <c r="AM71" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AN71" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AO71" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="72">
@@ -9756,9 +9972,12 @@
         <v>1</v>
       </c>
       <c r="AM72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN72" t="n">
         <v>14</v>
       </c>
-      <c r="AN72" t="n">
+      <c r="AO72" t="n">
         <v>14</v>
       </c>
     </row>
@@ -9889,6 +10108,9 @@
       <c r="AN73" t="n">
         <v>0</v>
       </c>
+      <c r="AO73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10017,6 +10239,9 @@
       <c r="AN74" t="n">
         <v>0</v>
       </c>
+      <c r="AO74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10140,10 +10365,13 @@
         <v>1</v>
       </c>
       <c r="AM75" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AN75" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AO75" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="76">
@@ -10268,10 +10496,13 @@
         <v>1</v>
       </c>
       <c r="AM76" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AN76" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AO76" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="77">
@@ -10396,9 +10627,12 @@
         <v>1</v>
       </c>
       <c r="AM77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN77" t="n">
         <v>15</v>
       </c>
-      <c r="AN77" t="n">
+      <c r="AO77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -10524,10 +10758,13 @@
         <v>0</v>
       </c>
       <c r="AM78" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AN78" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AO78" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="79">
@@ -10652,10 +10889,13 @@
         <v>1</v>
       </c>
       <c r="AM79" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AN79" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AO79" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="80">
@@ -10780,9 +11020,12 @@
         <v>0</v>
       </c>
       <c r="AM80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN80" t="n">
         <v>8</v>
       </c>
-      <c r="AN80" t="n">
+      <c r="AO80" t="n">
         <v>8</v>
       </c>
     </row>
@@ -10908,9 +11151,12 @@
         <v>0</v>
       </c>
       <c r="AM81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN81" t="n">
         <v>3</v>
       </c>
-      <c r="AN81" t="n">
+      <c r="AO81" t="n">
         <v>3</v>
       </c>
     </row>
@@ -11036,9 +11282,12 @@
         <v>0</v>
       </c>
       <c r="AM82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN82" t="n">
         <v>5</v>
       </c>
-      <c r="AN82" t="n">
+      <c r="AO82" t="n">
         <v>5</v>
       </c>
     </row>
@@ -11164,10 +11413,13 @@
         <v>1</v>
       </c>
       <c r="AM83" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AN83" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AO83" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="84">
@@ -11292,10 +11544,13 @@
         <v>0</v>
       </c>
       <c r="AM84" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AN84" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AO84" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="85">
@@ -11420,9 +11675,12 @@
         <v>0</v>
       </c>
       <c r="AM85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN85" t="n">
         <v>7</v>
       </c>
-      <c r="AN85" t="n">
+      <c r="AO85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11553,6 +11811,9 @@
       <c r="AN86" t="n">
         <v>0</v>
       </c>
+      <c r="AO86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -11676,10 +11937,13 @@
         <v>1</v>
       </c>
       <c r="AM87" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AN87" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AO87" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="88">
@@ -11809,6 +12073,9 @@
       <c r="AN88" t="n">
         <v>0</v>
       </c>
+      <c r="AO88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -11932,10 +12199,13 @@
         <v>0</v>
       </c>
       <c r="AM89" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AN89" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AO89" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="90">
@@ -12060,10 +12330,13 @@
         <v>1</v>
       </c>
       <c r="AM90" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AN90" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AO90" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="91">
@@ -12188,10 +12461,13 @@
         <v>1</v>
       </c>
       <c r="AM91" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="AN91" t="n">
-        <v>12</v>
+        <v>42</v>
+      </c>
+      <c r="AO91" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="92">
@@ -12316,9 +12592,12 @@
         <v>0</v>
       </c>
       <c r="AM92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN92" t="n">
         <v>7</v>
       </c>
-      <c r="AN92" t="n">
+      <c r="AO92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12449,6 +12728,9 @@
       <c r="AN93" t="n">
         <v>0</v>
       </c>
+      <c r="AO93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -12572,9 +12854,12 @@
         <v>1</v>
       </c>
       <c r="AM94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN94" t="n">
         <v>11</v>
       </c>
-      <c r="AN94" t="n">
+      <c r="AO94" t="n">
         <v>11</v>
       </c>
     </row>
@@ -12700,9 +12985,12 @@
         <v>0</v>
       </c>
       <c r="AM95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN95" t="n">
         <v>6</v>
       </c>
-      <c r="AN95" t="n">
+      <c r="AO95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -12828,10 +13116,13 @@
         <v>1</v>
       </c>
       <c r="AM96" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AN96" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AO96" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="97">
@@ -12961,6 +13252,9 @@
       <c r="AN97" t="n">
         <v>0</v>
       </c>
+      <c r="AO97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -13084,9 +13378,12 @@
         <v>0</v>
       </c>
       <c r="AM98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN98" t="n">
         <v>19</v>
       </c>
-      <c r="AN98" t="n">
+      <c r="AO98" t="n">
         <v>19</v>
       </c>
     </row>
@@ -13212,9 +13509,12 @@
         <v>1</v>
       </c>
       <c r="AM99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN99" t="n">
         <v>5</v>
       </c>
-      <c r="AN99" t="n">
+      <c r="AO99" t="n">
         <v>5</v>
       </c>
     </row>
@@ -13345,6 +13645,9 @@
       <c r="AN100" t="n">
         <v>0</v>
       </c>
+      <c r="AO100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -13468,10 +13771,13 @@
         <v>1</v>
       </c>
       <c r="AM101" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AN101" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AO101" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="102">
@@ -13596,10 +13902,13 @@
         <v>1</v>
       </c>
       <c r="AM102" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AN102" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AO102" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="103">
@@ -13724,10 +14033,13 @@
         <v>0</v>
       </c>
       <c r="AM103" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AN103" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AO103" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="104">
@@ -13852,10 +14164,13 @@
         <v>1</v>
       </c>
       <c r="AM104" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AN104" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AO104" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="105">
@@ -13980,10 +14295,13 @@
         <v>1</v>
       </c>
       <c r="AM105" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AN105" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AO105" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="106">
@@ -14108,9 +14426,12 @@
         <v>1</v>
       </c>
       <c r="AM106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN106" t="n">
         <v>7</v>
       </c>
-      <c r="AN106" t="n">
+      <c r="AO106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14236,10 +14557,13 @@
         <v>1</v>
       </c>
       <c r="AM107" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AN107" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AO107" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="108">
@@ -14364,9 +14688,12 @@
         <v>0</v>
       </c>
       <c r="AM108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN108" t="n">
         <v>2</v>
       </c>
-      <c r="AN108" t="n">
+      <c r="AO108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -14492,9 +14819,12 @@
         <v>0</v>
       </c>
       <c r="AM109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN109" t="n">
         <v>2</v>
       </c>
-      <c r="AN109" t="n">
+      <c r="AO109" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2838)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO109"/>
+  <dimension ref="A1:AP109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -469,8 +469,9 @@
     <col width="12" customWidth="1" min="37" max="37"/>
     <col width="12" customWidth="1" min="38" max="38"/>
     <col width="12" customWidth="1" min="39" max="39"/>
-    <col width="13" customWidth="1" min="40" max="40"/>
+    <col width="12" customWidth="1" min="40" max="40"/>
     <col width="13" customWidth="1" min="41" max="41"/>
+    <col width="13" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -669,12 +670,17 @@
           <t>2026-03-31</t>
         </is>
       </c>
-      <c r="AN1" s="2" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="AO1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AO1" s="2" t="inlineStr">
+      <c r="AP1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -805,9 +811,12 @@
         <v>0</v>
       </c>
       <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
         <v>10</v>
       </c>
-      <c r="AO2" t="n">
+      <c r="AP2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -936,10 +945,13 @@
         <v>0</v>
       </c>
       <c r="AN3" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AO3" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -1067,10 +1079,13 @@
         <v>1</v>
       </c>
       <c r="AN4" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AO4" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -1198,9 +1213,12 @@
         <v>0</v>
       </c>
       <c r="AN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO5" t="n">
         <v>15</v>
       </c>
-      <c r="AO5" t="n">
+      <c r="AP5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1329,9 +1347,12 @@
         <v>1</v>
       </c>
       <c r="AN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO6" t="n">
         <v>16</v>
       </c>
-      <c r="AO6" t="n">
+      <c r="AP6" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1460,9 +1481,12 @@
         <v>1</v>
       </c>
       <c r="AN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="n">
         <v>15</v>
       </c>
-      <c r="AO7" t="n">
+      <c r="AP7" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1591,10 +1615,13 @@
         <v>1</v>
       </c>
       <c r="AN8" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AO8" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -1722,10 +1749,13 @@
         <v>0</v>
       </c>
       <c r="AN9" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AO9" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="10">
@@ -1853,10 +1883,13 @@
         <v>1</v>
       </c>
       <c r="AN10" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AO10" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="11">
@@ -1984,10 +2017,13 @@
         <v>1</v>
       </c>
       <c r="AN11" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AO11" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="12">
@@ -2115,10 +2151,13 @@
         <v>1</v>
       </c>
       <c r="AN12" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AO12" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="13">
@@ -2246,10 +2285,13 @@
         <v>0</v>
       </c>
       <c r="AN13" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AO13" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -2377,10 +2419,13 @@
         <v>1</v>
       </c>
       <c r="AN14" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AO14" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -2508,9 +2553,12 @@
         <v>0</v>
       </c>
       <c r="AN15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO15" t="n">
         <v>9</v>
       </c>
-      <c r="AO15" t="n">
+      <c r="AP15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2639,10 +2687,13 @@
         <v>1</v>
       </c>
       <c r="AN16" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AO16" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="17">
@@ -2770,9 +2821,12 @@
         <v>1</v>
       </c>
       <c r="AN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO17" t="n">
         <v>15</v>
       </c>
-      <c r="AO17" t="n">
+      <c r="AP17" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2901,10 +2955,13 @@
         <v>1</v>
       </c>
       <c r="AN18" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AO18" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AP18" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="19">
@@ -3037,6 +3094,9 @@
       <c r="AO19" t="n">
         <v>0</v>
       </c>
+      <c r="AP19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3163,10 +3223,13 @@
         <v>0</v>
       </c>
       <c r="AN20" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AO20" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AP20" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="21">
@@ -3294,10 +3357,13 @@
         <v>1</v>
       </c>
       <c r="AN21" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AO21" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AP21" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="22">
@@ -3430,6 +3496,9 @@
       <c r="AO22" t="n">
         <v>0</v>
       </c>
+      <c r="AP22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3556,10 +3625,13 @@
         <v>1</v>
       </c>
       <c r="AN23" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AO23" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AP23" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="24">
@@ -3687,10 +3759,13 @@
         <v>1</v>
       </c>
       <c r="AN24" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AO24" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="25">
@@ -3818,9 +3893,12 @@
         <v>1</v>
       </c>
       <c r="AN25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO25" t="n">
         <v>7</v>
       </c>
-      <c r="AO25" t="n">
+      <c r="AP25" t="n">
         <v>7</v>
       </c>
     </row>
@@ -3949,10 +4027,13 @@
         <v>1</v>
       </c>
       <c r="AN26" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AO26" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AP26" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="27">
@@ -4080,10 +4161,13 @@
         <v>0</v>
       </c>
       <c r="AN27" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AO27" t="n">
-        <v>18</v>
+        <v>21</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="28">
@@ -4211,10 +4295,13 @@
         <v>1</v>
       </c>
       <c r="AN28" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AO28" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="29">
@@ -4342,9 +4429,12 @@
         <v>1</v>
       </c>
       <c r="AN29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO29" t="n">
         <v>7</v>
       </c>
-      <c r="AO29" t="n">
+      <c r="AP29" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4473,10 +4563,13 @@
         <v>1</v>
       </c>
       <c r="AN30" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AO30" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="31">
@@ -4604,10 +4697,13 @@
         <v>0</v>
       </c>
       <c r="AN31" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AO31" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="32">
@@ -4735,9 +4831,12 @@
         <v>1</v>
       </c>
       <c r="AN32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO32" t="n">
         <v>13</v>
       </c>
-      <c r="AO32" t="n">
+      <c r="AP32" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4866,9 +4965,12 @@
         <v>0</v>
       </c>
       <c r="AN33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO33" t="n">
         <v>13</v>
       </c>
-      <c r="AO33" t="n">
+      <c r="AP33" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4997,9 +5099,12 @@
         <v>0</v>
       </c>
       <c r="AN34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO34" t="n">
         <v>8</v>
       </c>
-      <c r="AO34" t="n">
+      <c r="AP34" t="n">
         <v>8</v>
       </c>
     </row>
@@ -5128,10 +5233,13 @@
         <v>1</v>
       </c>
       <c r="AN35" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AO35" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AP35" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="36">
@@ -5259,10 +5367,13 @@
         <v>0</v>
       </c>
       <c r="AN36" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AO36" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AP36" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="37">
@@ -5395,6 +5506,9 @@
       <c r="AO37" t="n">
         <v>0</v>
       </c>
+      <c r="AP37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5521,9 +5635,12 @@
         <v>0</v>
       </c>
       <c r="AN38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO38" t="n">
         <v>2</v>
       </c>
-      <c r="AO38" t="n">
+      <c r="AP38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5652,10 +5769,13 @@
         <v>1</v>
       </c>
       <c r="AN39" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AO39" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AP39" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="40">
@@ -5783,9 +5903,12 @@
         <v>0</v>
       </c>
       <c r="AN40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO40" t="n">
         <v>16</v>
       </c>
-      <c r="AO40" t="n">
+      <c r="AP40" t="n">
         <v>16</v>
       </c>
     </row>
@@ -5914,10 +6037,13 @@
         <v>1</v>
       </c>
       <c r="AN41" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AO41" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AP41" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="42">
@@ -6045,9 +6171,12 @@
         <v>0</v>
       </c>
       <c r="AN42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO42" t="n">
         <v>21</v>
       </c>
-      <c r="AO42" t="n">
+      <c r="AP42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6176,10 +6305,13 @@
         <v>1</v>
       </c>
       <c r="AN43" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="AO43" t="n">
-        <v>14</v>
+        <v>56</v>
+      </c>
+      <c r="AP43" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="44">
@@ -6307,10 +6439,13 @@
         <v>1</v>
       </c>
       <c r="AN44" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AO44" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AP44" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="45">
@@ -6438,10 +6573,13 @@
         <v>1</v>
       </c>
       <c r="AN45" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AO45" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AP45" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="46">
@@ -6569,10 +6707,13 @@
         <v>0</v>
       </c>
       <c r="AN46" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AO46" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AP46" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="47">
@@ -6705,6 +6846,9 @@
       <c r="AO47" t="n">
         <v>0</v>
       </c>
+      <c r="AP47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6831,10 +6975,13 @@
         <v>1</v>
       </c>
       <c r="AN48" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AO48" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AP48" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="49">
@@ -6962,9 +7109,12 @@
         <v>1</v>
       </c>
       <c r="AN49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO49" t="n">
         <v>16</v>
       </c>
-      <c r="AO49" t="n">
+      <c r="AP49" t="n">
         <v>16</v>
       </c>
     </row>
@@ -7093,9 +7243,12 @@
         <v>0</v>
       </c>
       <c r="AN50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO50" t="n">
         <v>7</v>
       </c>
-      <c r="AO50" t="n">
+      <c r="AP50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7224,10 +7377,13 @@
         <v>1</v>
       </c>
       <c r="AN51" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AO51" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AP51" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="52">
@@ -7360,6 +7516,9 @@
       <c r="AO52" t="n">
         <v>0</v>
       </c>
+      <c r="AP52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7486,9 +7645,12 @@
         <v>0</v>
       </c>
       <c r="AN53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO53" t="n">
         <v>12</v>
       </c>
-      <c r="AO53" t="n">
+      <c r="AP53" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7622,6 +7784,9 @@
       <c r="AO54" t="n">
         <v>0</v>
       </c>
+      <c r="AP54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7748,10 +7913,13 @@
         <v>1</v>
       </c>
       <c r="AN55" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AO55" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AP55" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="56">
@@ -7879,10 +8047,13 @@
         <v>0</v>
       </c>
       <c r="AN56" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AO56" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AP56" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="57">
@@ -8010,9 +8181,12 @@
         <v>0</v>
       </c>
       <c r="AN57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO57" t="n">
         <v>8</v>
       </c>
-      <c r="AO57" t="n">
+      <c r="AP57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8141,9 +8315,12 @@
         <v>0</v>
       </c>
       <c r="AN58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO58" t="n">
         <v>12</v>
       </c>
-      <c r="AO58" t="n">
+      <c r="AP58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -8272,9 +8449,12 @@
         <v>1</v>
       </c>
       <c r="AN59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO59" t="n">
         <v>5</v>
       </c>
-      <c r="AO59" t="n">
+      <c r="AP59" t="n">
         <v>5</v>
       </c>
     </row>
@@ -8408,6 +8588,9 @@
       <c r="AO60" t="n">
         <v>0</v>
       </c>
+      <c r="AP60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8534,10 +8717,13 @@
         <v>1</v>
       </c>
       <c r="AN61" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AO61" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AP61" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="62">
@@ -8665,9 +8851,12 @@
         <v>1</v>
       </c>
       <c r="AN62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO62" t="n">
         <v>19</v>
       </c>
-      <c r="AO62" t="n">
+      <c r="AP62" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8796,9 +8985,12 @@
         <v>0</v>
       </c>
       <c r="AN63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO63" t="n">
         <v>8</v>
       </c>
-      <c r="AO63" t="n">
+      <c r="AP63" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8932,6 +9124,9 @@
       <c r="AO64" t="n">
         <v>0</v>
       </c>
+      <c r="AP64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -9058,9 +9253,12 @@
         <v>0</v>
       </c>
       <c r="AN65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO65" t="n">
         <v>10</v>
       </c>
-      <c r="AO65" t="n">
+      <c r="AP65" t="n">
         <v>10</v>
       </c>
     </row>
@@ -9189,10 +9387,13 @@
         <v>0</v>
       </c>
       <c r="AN66" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AO66" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AP66" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="67">
@@ -9320,10 +9521,13 @@
         <v>1</v>
       </c>
       <c r="AN67" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AO67" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AP67" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="68">
@@ -9451,9 +9655,12 @@
         <v>1</v>
       </c>
       <c r="AN68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO68" t="n">
         <v>12</v>
       </c>
-      <c r="AO68" t="n">
+      <c r="AP68" t="n">
         <v>11</v>
       </c>
     </row>
@@ -9582,9 +9789,12 @@
         <v>0</v>
       </c>
       <c r="AN69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO69" t="n">
         <v>7</v>
       </c>
-      <c r="AO69" t="n">
+      <c r="AP69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9713,9 +9923,12 @@
         <v>0</v>
       </c>
       <c r="AN70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO70" t="n">
         <v>23</v>
       </c>
-      <c r="AO70" t="n">
+      <c r="AP70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -9844,10 +10057,13 @@
         <v>1</v>
       </c>
       <c r="AN71" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AO71" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AP71" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="72">
@@ -9975,9 +10191,12 @@
         <v>0</v>
       </c>
       <c r="AN72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO72" t="n">
         <v>14</v>
       </c>
-      <c r="AO72" t="n">
+      <c r="AP72" t="n">
         <v>14</v>
       </c>
     </row>
@@ -10111,6 +10330,9 @@
       <c r="AO73" t="n">
         <v>0</v>
       </c>
+      <c r="AP73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10242,6 +10464,9 @@
       <c r="AO74" t="n">
         <v>0</v>
       </c>
+      <c r="AP74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10368,9 +10593,12 @@
         <v>1</v>
       </c>
       <c r="AN75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO75" t="n">
         <v>14</v>
       </c>
-      <c r="AO75" t="n">
+      <c r="AP75" t="n">
         <v>14</v>
       </c>
     </row>
@@ -10499,10 +10727,13 @@
         <v>1</v>
       </c>
       <c r="AN76" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AO76" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AP76" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="77">
@@ -10630,9 +10861,12 @@
         <v>0</v>
       </c>
       <c r="AN77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO77" t="n">
         <v>15</v>
       </c>
-      <c r="AO77" t="n">
+      <c r="AP77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -10761,10 +10995,13 @@
         <v>1</v>
       </c>
       <c r="AN78" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AO78" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AP78" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="79">
@@ -10892,10 +11129,13 @@
         <v>1</v>
       </c>
       <c r="AN79" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AO79" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AP79" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="80">
@@ -11023,9 +11263,12 @@
         <v>0</v>
       </c>
       <c r="AN80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO80" t="n">
         <v>8</v>
       </c>
-      <c r="AO80" t="n">
+      <c r="AP80" t="n">
         <v>8</v>
       </c>
     </row>
@@ -11154,9 +11397,12 @@
         <v>0</v>
       </c>
       <c r="AN81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO81" t="n">
         <v>3</v>
       </c>
-      <c r="AO81" t="n">
+      <c r="AP81" t="n">
         <v>3</v>
       </c>
     </row>
@@ -11285,9 +11531,12 @@
         <v>0</v>
       </c>
       <c r="AN82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO82" t="n">
         <v>5</v>
       </c>
-      <c r="AO82" t="n">
+      <c r="AP82" t="n">
         <v>5</v>
       </c>
     </row>
@@ -11416,9 +11665,12 @@
         <v>1</v>
       </c>
       <c r="AN83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO83" t="n">
         <v>15</v>
       </c>
-      <c r="AO83" t="n">
+      <c r="AP83" t="n">
         <v>15</v>
       </c>
     </row>
@@ -11547,9 +11799,12 @@
         <v>1</v>
       </c>
       <c r="AN84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO84" t="n">
         <v>6</v>
       </c>
-      <c r="AO84" t="n">
+      <c r="AP84" t="n">
         <v>6</v>
       </c>
     </row>
@@ -11678,9 +11933,12 @@
         <v>0</v>
       </c>
       <c r="AN85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO85" t="n">
         <v>7</v>
       </c>
-      <c r="AO85" t="n">
+      <c r="AP85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11814,6 +12072,9 @@
       <c r="AO86" t="n">
         <v>0</v>
       </c>
+      <c r="AP86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -11940,10 +12201,13 @@
         <v>1</v>
       </c>
       <c r="AN87" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AO87" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AP87" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="88">
@@ -12076,6 +12340,9 @@
       <c r="AO88" t="n">
         <v>0</v>
       </c>
+      <c r="AP88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -12202,10 +12469,13 @@
         <v>1</v>
       </c>
       <c r="AN89" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AO89" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AP89" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="90">
@@ -12333,10 +12603,13 @@
         <v>1</v>
       </c>
       <c r="AN90" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AO90" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AP90" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="91">
@@ -12464,9 +12737,12 @@
         <v>1</v>
       </c>
       <c r="AN91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO91" t="n">
         <v>42</v>
       </c>
-      <c r="AO91" t="n">
+      <c r="AP91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -12595,9 +12871,12 @@
         <v>0</v>
       </c>
       <c r="AN92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO92" t="n">
         <v>7</v>
       </c>
-      <c r="AO92" t="n">
+      <c r="AP92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12731,6 +13010,9 @@
       <c r="AO93" t="n">
         <v>0</v>
       </c>
+      <c r="AP93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -12857,10 +13139,13 @@
         <v>0</v>
       </c>
       <c r="AN94" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AO94" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AP94" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="95">
@@ -12988,9 +13273,12 @@
         <v>0</v>
       </c>
       <c r="AN95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO95" t="n">
         <v>6</v>
       </c>
-      <c r="AO95" t="n">
+      <c r="AP95" t="n">
         <v>6</v>
       </c>
     </row>
@@ -13119,10 +13407,13 @@
         <v>1</v>
       </c>
       <c r="AN96" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AO96" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AP96" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="97">
@@ -13255,6 +13546,9 @@
       <c r="AO97" t="n">
         <v>0</v>
       </c>
+      <c r="AP97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -13381,10 +13675,13 @@
         <v>0</v>
       </c>
       <c r="AN98" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AO98" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AP98" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="99">
@@ -13512,10 +13809,13 @@
         <v>0</v>
       </c>
       <c r="AN99" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AO99" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AP99" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="100">
@@ -13648,6 +13948,9 @@
       <c r="AO100" t="n">
         <v>0</v>
       </c>
+      <c r="AP100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -13774,10 +14077,13 @@
         <v>1</v>
       </c>
       <c r="AN101" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AO101" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AP101" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="102">
@@ -13905,10 +14211,13 @@
         <v>1</v>
       </c>
       <c r="AN102" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AO102" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AP102" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="103">
@@ -14036,10 +14345,13 @@
         <v>1</v>
       </c>
       <c r="AN103" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AO103" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AP103" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="104">
@@ -14167,10 +14479,13 @@
         <v>1</v>
       </c>
       <c r="AN104" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AO104" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AP104" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="105">
@@ -14298,10 +14613,13 @@
         <v>1</v>
       </c>
       <c r="AN105" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AO105" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AP105" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="106">
@@ -14429,9 +14747,12 @@
         <v>0</v>
       </c>
       <c r="AN106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO106" t="n">
         <v>7</v>
       </c>
-      <c r="AO106" t="n">
+      <c r="AP106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14560,10 +14881,13 @@
         <v>1</v>
       </c>
       <c r="AN107" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AO107" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AP107" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="108">
@@ -14691,9 +15015,12 @@
         <v>0</v>
       </c>
       <c r="AN108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO108" t="n">
         <v>2</v>
       </c>
-      <c r="AO108" t="n">
+      <c r="AP108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -14822,9 +15149,12 @@
         <v>0</v>
       </c>
       <c r="AN109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO109" t="n">
         <v>2</v>
       </c>
-      <c r="AO109" t="n">
+      <c r="AP109" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2916)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP109"/>
+  <dimension ref="A1:AQ109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -470,8 +470,9 @@
     <col width="12" customWidth="1" min="38" max="38"/>
     <col width="12" customWidth="1" min="39" max="39"/>
     <col width="12" customWidth="1" min="40" max="40"/>
-    <col width="13" customWidth="1" min="41" max="41"/>
+    <col width="12" customWidth="1" min="41" max="41"/>
     <col width="13" customWidth="1" min="42" max="42"/>
+    <col width="13" customWidth="1" min="43" max="43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -675,12 +676,17 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="AO1" s="2" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="AP1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AP1" s="2" t="inlineStr">
+      <c r="AQ1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -814,9 +820,12 @@
         <v>0</v>
       </c>
       <c r="AO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP2" t="n">
         <v>10</v>
       </c>
-      <c r="AP2" t="n">
+      <c r="AQ2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -948,9 +957,12 @@
         <v>1</v>
       </c>
       <c r="AO3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP3" t="n">
         <v>9</v>
       </c>
-      <c r="AP3" t="n">
+      <c r="AQ3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1082,10 +1094,13 @@
         <v>1</v>
       </c>
       <c r="AO4" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AP4" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="5">
@@ -1216,9 +1231,12 @@
         <v>0</v>
       </c>
       <c r="AO5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP5" t="n">
         <v>15</v>
       </c>
-      <c r="AP5" t="n">
+      <c r="AQ5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1350,9 +1368,12 @@
         <v>0</v>
       </c>
       <c r="AO6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP6" t="n">
         <v>16</v>
       </c>
-      <c r="AP6" t="n">
+      <c r="AQ6" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1484,10 +1505,13 @@
         <v>0</v>
       </c>
       <c r="AO7" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AP7" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -1618,10 +1642,13 @@
         <v>1</v>
       </c>
       <c r="AO8" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AP8" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -1752,10 +1779,13 @@
         <v>1</v>
       </c>
       <c r="AO9" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AP9" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -1886,10 +1916,13 @@
         <v>1</v>
       </c>
       <c r="AO10" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AP10" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="11">
@@ -2020,10 +2053,13 @@
         <v>1</v>
       </c>
       <c r="AO11" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AP11" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="12">
@@ -2154,10 +2190,13 @@
         <v>1</v>
       </c>
       <c r="AO12" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AP12" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="13">
@@ -2288,9 +2327,12 @@
         <v>1</v>
       </c>
       <c r="AO13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP13" t="n">
         <v>12</v>
       </c>
-      <c r="AP13" t="n">
+      <c r="AQ13" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2422,10 +2464,13 @@
         <v>1</v>
       </c>
       <c r="AO14" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AP14" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="15">
@@ -2556,9 +2601,12 @@
         <v>0</v>
       </c>
       <c r="AO15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP15" t="n">
         <v>9</v>
       </c>
-      <c r="AP15" t="n">
+      <c r="AQ15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2690,9 +2738,12 @@
         <v>1</v>
       </c>
       <c r="AO16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP16" t="n">
         <v>16</v>
       </c>
-      <c r="AP16" t="n">
+      <c r="AQ16" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2824,10 +2875,13 @@
         <v>0</v>
       </c>
       <c r="AO17" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AP17" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="18">
@@ -2958,9 +3012,12 @@
         <v>1</v>
       </c>
       <c r="AO18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP18" t="n">
         <v>19</v>
       </c>
-      <c r="AP18" t="n">
+      <c r="AQ18" t="n">
         <v>19</v>
       </c>
     </row>
@@ -3097,6 +3154,9 @@
       <c r="AP19" t="n">
         <v>0</v>
       </c>
+      <c r="AQ19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3226,9 +3286,12 @@
         <v>1</v>
       </c>
       <c r="AO20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP20" t="n">
         <v>15</v>
       </c>
-      <c r="AP20" t="n">
+      <c r="AQ20" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3360,10 +3423,13 @@
         <v>1</v>
       </c>
       <c r="AO21" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AP21" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AQ21" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="22">
@@ -3499,6 +3565,9 @@
       <c r="AP22" t="n">
         <v>0</v>
       </c>
+      <c r="AQ22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3628,10 +3697,13 @@
         <v>1</v>
       </c>
       <c r="AO23" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AP23" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="24">
@@ -3762,10 +3834,13 @@
         <v>1</v>
       </c>
       <c r="AO24" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AP24" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="25">
@@ -3896,10 +3971,13 @@
         <v>0</v>
       </c>
       <c r="AO25" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AP25" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="26">
@@ -4030,10 +4108,13 @@
         <v>1</v>
       </c>
       <c r="AO26" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AP26" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="27">
@@ -4164,9 +4245,12 @@
         <v>1</v>
       </c>
       <c r="AO27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP27" t="n">
         <v>21</v>
       </c>
-      <c r="AP27" t="n">
+      <c r="AQ27" t="n">
         <v>19</v>
       </c>
     </row>
@@ -4298,10 +4382,13 @@
         <v>1</v>
       </c>
       <c r="AO28" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AP28" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="29">
@@ -4432,10 +4519,13 @@
         <v>0</v>
       </c>
       <c r="AO29" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AP29" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="30">
@@ -4566,10 +4656,13 @@
         <v>1</v>
       </c>
       <c r="AO30" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AP30" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="31">
@@ -4700,9 +4793,12 @@
         <v>1</v>
       </c>
       <c r="AO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP31" t="n">
         <v>17</v>
       </c>
-      <c r="AP31" t="n">
+      <c r="AQ31" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4834,10 +4930,13 @@
         <v>0</v>
       </c>
       <c r="AO32" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AP32" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="33">
@@ -4968,9 +5067,12 @@
         <v>0</v>
       </c>
       <c r="AO33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP33" t="n">
         <v>13</v>
       </c>
-      <c r="AP33" t="n">
+      <c r="AQ33" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5102,9 +5204,12 @@
         <v>0</v>
       </c>
       <c r="AO34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP34" t="n">
         <v>8</v>
       </c>
-      <c r="AP34" t="n">
+      <c r="AQ34" t="n">
         <v>8</v>
       </c>
     </row>
@@ -5236,9 +5341,12 @@
         <v>1</v>
       </c>
       <c r="AO35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP35" t="n">
         <v>17</v>
       </c>
-      <c r="AP35" t="n">
+      <c r="AQ35" t="n">
         <v>17</v>
       </c>
     </row>
@@ -5370,10 +5478,13 @@
         <v>1</v>
       </c>
       <c r="AO36" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AP36" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AQ36" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="37">
@@ -5509,6 +5620,9 @@
       <c r="AP37" t="n">
         <v>0</v>
       </c>
+      <c r="AQ37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5638,9 +5752,12 @@
         <v>0</v>
       </c>
       <c r="AO38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP38" t="n">
         <v>2</v>
       </c>
-      <c r="AP38" t="n">
+      <c r="AQ38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5772,10 +5889,13 @@
         <v>1</v>
       </c>
       <c r="AO39" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AP39" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AQ39" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="40">
@@ -5906,10 +6026,13 @@
         <v>0</v>
       </c>
       <c r="AO40" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AP40" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AQ40" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="41">
@@ -6040,10 +6163,13 @@
         <v>1</v>
       </c>
       <c r="AO41" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AP41" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AQ41" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="42">
@@ -6174,9 +6300,12 @@
         <v>0</v>
       </c>
       <c r="AO42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP42" t="n">
         <v>21</v>
       </c>
-      <c r="AP42" t="n">
+      <c r="AQ42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6308,9 +6437,12 @@
         <v>1</v>
       </c>
       <c r="AO43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP43" t="n">
         <v>56</v>
       </c>
-      <c r="AP43" t="n">
+      <c r="AQ43" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6442,10 +6574,13 @@
         <v>1</v>
       </c>
       <c r="AO44" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AP44" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AQ44" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="45">
@@ -6576,10 +6711,13 @@
         <v>1</v>
       </c>
       <c r="AO45" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AP45" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="46">
@@ -6710,10 +6848,13 @@
         <v>1</v>
       </c>
       <c r="AO46" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AP46" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AQ46" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="47">
@@ -6849,6 +6990,9 @@
       <c r="AP47" t="n">
         <v>0</v>
       </c>
+      <c r="AQ47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6978,10 +7122,13 @@
         <v>1</v>
       </c>
       <c r="AO48" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AP48" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AQ48" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="49">
@@ -7112,9 +7259,12 @@
         <v>0</v>
       </c>
       <c r="AO49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP49" t="n">
         <v>16</v>
       </c>
-      <c r="AP49" t="n">
+      <c r="AQ49" t="n">
         <v>16</v>
       </c>
     </row>
@@ -7246,9 +7396,12 @@
         <v>0</v>
       </c>
       <c r="AO50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP50" t="n">
         <v>7</v>
       </c>
-      <c r="AP50" t="n">
+      <c r="AQ50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7380,10 +7533,13 @@
         <v>1</v>
       </c>
       <c r="AO51" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AP51" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AQ51" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="52">
@@ -7519,6 +7675,9 @@
       <c r="AP52" t="n">
         <v>0</v>
       </c>
+      <c r="AQ52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7648,9 +7807,12 @@
         <v>0</v>
       </c>
       <c r="AO53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP53" t="n">
         <v>12</v>
       </c>
-      <c r="AP53" t="n">
+      <c r="AQ53" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7787,6 +7949,9 @@
       <c r="AP54" t="n">
         <v>0</v>
       </c>
+      <c r="AQ54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7916,10 +8081,13 @@
         <v>1</v>
       </c>
       <c r="AO55" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AP55" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AQ55" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="56">
@@ -8050,10 +8218,13 @@
         <v>1</v>
       </c>
       <c r="AO56" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AP56" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AQ56" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="57">
@@ -8184,9 +8355,12 @@
         <v>0</v>
       </c>
       <c r="AO57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP57" t="n">
         <v>8</v>
       </c>
-      <c r="AP57" t="n">
+      <c r="AQ57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8318,9 +8492,12 @@
         <v>0</v>
       </c>
       <c r="AO58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP58" t="n">
         <v>12</v>
       </c>
-      <c r="AP58" t="n">
+      <c r="AQ58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -8452,9 +8629,12 @@
         <v>0</v>
       </c>
       <c r="AO59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP59" t="n">
         <v>5</v>
       </c>
-      <c r="AP59" t="n">
+      <c r="AQ59" t="n">
         <v>5</v>
       </c>
     </row>
@@ -8591,6 +8771,9 @@
       <c r="AP60" t="n">
         <v>0</v>
       </c>
+      <c r="AQ60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8720,10 +8903,13 @@
         <v>1</v>
       </c>
       <c r="AO61" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AP61" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AQ61" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="62">
@@ -8854,10 +9040,13 @@
         <v>0</v>
       </c>
       <c r="AO62" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AP62" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AQ62" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="63">
@@ -8988,9 +9177,12 @@
         <v>0</v>
       </c>
       <c r="AO63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP63" t="n">
         <v>8</v>
       </c>
-      <c r="AP63" t="n">
+      <c r="AQ63" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9127,6 +9319,9 @@
       <c r="AP64" t="n">
         <v>0</v>
       </c>
+      <c r="AQ64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -9256,9 +9451,12 @@
         <v>0</v>
       </c>
       <c r="AO65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP65" t="n">
         <v>10</v>
       </c>
-      <c r="AP65" t="n">
+      <c r="AQ65" t="n">
         <v>10</v>
       </c>
     </row>
@@ -9390,9 +9588,12 @@
         <v>1</v>
       </c>
       <c r="AO66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP66" t="n">
         <v>4</v>
       </c>
-      <c r="AP66" t="n">
+      <c r="AQ66" t="n">
         <v>4</v>
       </c>
     </row>
@@ -9524,10 +9725,13 @@
         <v>1</v>
       </c>
       <c r="AO67" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AP67" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AQ67" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="68">
@@ -9658,10 +9862,13 @@
         <v>0</v>
       </c>
       <c r="AO68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP68" t="n">
+        <v>13</v>
+      </c>
+      <c r="AQ68" t="n">
         <v>12</v>
-      </c>
-      <c r="AP68" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="69">
@@ -9792,9 +9999,12 @@
         <v>0</v>
       </c>
       <c r="AO69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP69" t="n">
         <v>7</v>
       </c>
-      <c r="AP69" t="n">
+      <c r="AQ69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9926,9 +10136,12 @@
         <v>0</v>
       </c>
       <c r="AO70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP70" t="n">
         <v>23</v>
       </c>
-      <c r="AP70" t="n">
+      <c r="AQ70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -10060,9 +10273,12 @@
         <v>1</v>
       </c>
       <c r="AO71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP71" t="n">
         <v>15</v>
       </c>
-      <c r="AP71" t="n">
+      <c r="AQ71" t="n">
         <v>15</v>
       </c>
     </row>
@@ -10194,10 +10410,13 @@
         <v>0</v>
       </c>
       <c r="AO72" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AP72" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AQ72" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="73">
@@ -10333,6 +10552,9 @@
       <c r="AP73" t="n">
         <v>0</v>
       </c>
+      <c r="AQ73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10467,6 +10689,9 @@
       <c r="AP74" t="n">
         <v>0</v>
       </c>
+      <c r="AQ74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10596,10 +10821,13 @@
         <v>0</v>
       </c>
       <c r="AO75" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AP75" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AQ75" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="76">
@@ -10730,9 +10958,12 @@
         <v>1</v>
       </c>
       <c r="AO76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP76" t="n">
         <v>16</v>
       </c>
-      <c r="AP76" t="n">
+      <c r="AQ76" t="n">
         <v>16</v>
       </c>
     </row>
@@ -10864,9 +11095,12 @@
         <v>0</v>
       </c>
       <c r="AO77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP77" t="n">
         <v>15</v>
       </c>
-      <c r="AP77" t="n">
+      <c r="AQ77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -10998,10 +11232,13 @@
         <v>1</v>
       </c>
       <c r="AO78" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AP78" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AQ78" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="79">
@@ -11132,9 +11369,12 @@
         <v>1</v>
       </c>
       <c r="AO79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP79" t="n">
         <v>17</v>
       </c>
-      <c r="AP79" t="n">
+      <c r="AQ79" t="n">
         <v>17</v>
       </c>
     </row>
@@ -11266,9 +11506,12 @@
         <v>0</v>
       </c>
       <c r="AO80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP80" t="n">
         <v>8</v>
       </c>
-      <c r="AP80" t="n">
+      <c r="AQ80" t="n">
         <v>8</v>
       </c>
     </row>
@@ -11400,9 +11643,12 @@
         <v>0</v>
       </c>
       <c r="AO81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP81" t="n">
         <v>3</v>
       </c>
-      <c r="AP81" t="n">
+      <c r="AQ81" t="n">
         <v>3</v>
       </c>
     </row>
@@ -11534,10 +11780,13 @@
         <v>0</v>
       </c>
       <c r="AO82" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AP82" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AQ82" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="83">
@@ -11668,10 +11917,13 @@
         <v>0</v>
       </c>
       <c r="AO83" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AP83" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AQ83" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="84">
@@ -11802,10 +12054,13 @@
         <v>0</v>
       </c>
       <c r="AO84" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AP84" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AQ84" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="85">
@@ -11936,9 +12191,12 @@
         <v>0</v>
       </c>
       <c r="AO85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP85" t="n">
         <v>7</v>
       </c>
-      <c r="AP85" t="n">
+      <c r="AQ85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12075,6 +12333,9 @@
       <c r="AP86" t="n">
         <v>0</v>
       </c>
+      <c r="AQ86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -12204,10 +12465,13 @@
         <v>1</v>
       </c>
       <c r="AO87" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AP87" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AQ87" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="88">
@@ -12343,6 +12607,9 @@
       <c r="AP88" t="n">
         <v>0</v>
       </c>
+      <c r="AQ88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -12472,9 +12739,12 @@
         <v>1</v>
       </c>
       <c r="AO89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP89" t="n">
         <v>16</v>
       </c>
-      <c r="AP89" t="n">
+      <c r="AQ89" t="n">
         <v>16</v>
       </c>
     </row>
@@ -12606,9 +12876,12 @@
         <v>1</v>
       </c>
       <c r="AO90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP90" t="n">
         <v>14</v>
       </c>
-      <c r="AP90" t="n">
+      <c r="AQ90" t="n">
         <v>14</v>
       </c>
     </row>
@@ -12740,9 +13013,12 @@
         <v>0</v>
       </c>
       <c r="AO91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP91" t="n">
         <v>42</v>
       </c>
-      <c r="AP91" t="n">
+      <c r="AQ91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -12874,9 +13150,12 @@
         <v>0</v>
       </c>
       <c r="AO92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP92" t="n">
         <v>7</v>
       </c>
-      <c r="AP92" t="n">
+      <c r="AQ92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13013,6 +13292,9 @@
       <c r="AP93" t="n">
         <v>0</v>
       </c>
+      <c r="AQ93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -13142,10 +13424,13 @@
         <v>1</v>
       </c>
       <c r="AO94" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AP94" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AQ94" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="95">
@@ -13276,10 +13561,13 @@
         <v>0</v>
       </c>
       <c r="AO95" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AP95" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AQ95" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="96">
@@ -13410,9 +13698,12 @@
         <v>1</v>
       </c>
       <c r="AO96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP96" t="n">
         <v>17</v>
       </c>
-      <c r="AP96" t="n">
+      <c r="AQ96" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13549,6 +13840,9 @@
       <c r="AP97" t="n">
         <v>0</v>
       </c>
+      <c r="AQ97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -13678,9 +13972,12 @@
         <v>1</v>
       </c>
       <c r="AO98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP98" t="n">
         <v>20</v>
       </c>
-      <c r="AP98" t="n">
+      <c r="AQ98" t="n">
         <v>20</v>
       </c>
     </row>
@@ -13812,9 +14109,12 @@
         <v>1</v>
       </c>
       <c r="AO99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP99" t="n">
         <v>6</v>
       </c>
-      <c r="AP99" t="n">
+      <c r="AQ99" t="n">
         <v>6</v>
       </c>
     </row>
@@ -13951,6 +14251,9 @@
       <c r="AP100" t="n">
         <v>0</v>
       </c>
+      <c r="AQ100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -14080,10 +14383,13 @@
         <v>1</v>
       </c>
       <c r="AO101" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AP101" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AQ101" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="102">
@@ -14214,10 +14520,13 @@
         <v>1</v>
       </c>
       <c r="AO102" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AP102" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AQ102" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="103">
@@ -14348,10 +14657,13 @@
         <v>1</v>
       </c>
       <c r="AO103" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AP103" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AQ103" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="104">
@@ -14482,10 +14794,13 @@
         <v>1</v>
       </c>
       <c r="AO104" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AP104" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AQ104" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="105">
@@ -14616,10 +14931,13 @@
         <v>1</v>
       </c>
       <c r="AO105" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AP105" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AQ105" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="106">
@@ -14750,9 +15068,12 @@
         <v>0</v>
       </c>
       <c r="AO106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP106" t="n">
         <v>7</v>
       </c>
-      <c r="AP106" t="n">
+      <c r="AQ106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14884,10 +15205,13 @@
         <v>1</v>
       </c>
       <c r="AO107" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AP107" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AQ107" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="108">
@@ -15018,9 +15342,12 @@
         <v>0</v>
       </c>
       <c r="AO108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP108" t="n">
         <v>2</v>
       </c>
-      <c r="AP108" t="n">
+      <c r="AQ108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -15152,9 +15479,12 @@
         <v>0</v>
       </c>
       <c r="AO109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP109" t="n">
         <v>2</v>
       </c>
-      <c r="AP109" t="n">
+      <c r="AQ109" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2984)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ109"/>
+  <dimension ref="A1:AR109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -471,8 +471,9 @@
     <col width="12" customWidth="1" min="39" max="39"/>
     <col width="12" customWidth="1" min="40" max="40"/>
     <col width="12" customWidth="1" min="41" max="41"/>
-    <col width="13" customWidth="1" min="42" max="42"/>
+    <col width="12" customWidth="1" min="42" max="42"/>
     <col width="13" customWidth="1" min="43" max="43"/>
+    <col width="13" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -681,12 +682,17 @@
           <t>2026-04-02</t>
         </is>
       </c>
-      <c r="AP1" s="2" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="AQ1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AQ1" s="2" t="inlineStr">
+      <c r="AR1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -823,9 +829,12 @@
         <v>0</v>
       </c>
       <c r="AP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="n">
         <v>10</v>
       </c>
-      <c r="AQ2" t="n">
+      <c r="AR2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -960,9 +969,12 @@
         <v>0</v>
       </c>
       <c r="AP3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ3" t="n">
         <v>9</v>
       </c>
-      <c r="AQ3" t="n">
+      <c r="AR3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1097,10 +1109,13 @@
         <v>1</v>
       </c>
       <c r="AP4" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AQ4" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="5">
@@ -1234,9 +1249,12 @@
         <v>0</v>
       </c>
       <c r="AP5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ5" t="n">
         <v>15</v>
       </c>
-      <c r="AQ5" t="n">
+      <c r="AR5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1371,10 +1389,13 @@
         <v>0</v>
       </c>
       <c r="AP6" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AQ6" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -1508,9 +1529,12 @@
         <v>1</v>
       </c>
       <c r="AP7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ7" t="n">
         <v>16</v>
       </c>
-      <c r="AQ7" t="n">
+      <c r="AR7" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1645,9 +1669,12 @@
         <v>1</v>
       </c>
       <c r="AP8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ8" t="n">
         <v>22</v>
       </c>
-      <c r="AQ8" t="n">
+      <c r="AR8" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1782,10 +1809,13 @@
         <v>1</v>
       </c>
       <c r="AP9" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AQ9" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -1919,10 +1949,13 @@
         <v>1</v>
       </c>
       <c r="AP10" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AQ10" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="11">
@@ -2056,9 +2089,12 @@
         <v>1</v>
       </c>
       <c r="AP11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ11" t="n">
         <v>19</v>
       </c>
-      <c r="AQ11" t="n">
+      <c r="AR11" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2193,10 +2229,13 @@
         <v>1</v>
       </c>
       <c r="AP12" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AQ12" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="13">
@@ -2330,9 +2369,12 @@
         <v>0</v>
       </c>
       <c r="AP13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ13" t="n">
         <v>12</v>
       </c>
-      <c r="AQ13" t="n">
+      <c r="AR13" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2467,9 +2509,12 @@
         <v>1</v>
       </c>
       <c r="AP14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ14" t="n">
         <v>22</v>
       </c>
-      <c r="AQ14" t="n">
+      <c r="AR14" t="n">
         <v>22</v>
       </c>
     </row>
@@ -2604,9 +2649,12 @@
         <v>0</v>
       </c>
       <c r="AP15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ15" t="n">
         <v>9</v>
       </c>
-      <c r="AQ15" t="n">
+      <c r="AR15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2741,10 +2789,13 @@
         <v>0</v>
       </c>
       <c r="AP16" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AQ16" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="17">
@@ -2878,9 +2929,12 @@
         <v>1</v>
       </c>
       <c r="AP17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ17" t="n">
         <v>16</v>
       </c>
-      <c r="AQ17" t="n">
+      <c r="AR17" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3015,10 +3069,13 @@
         <v>0</v>
       </c>
       <c r="AP18" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AQ18" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AR18" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="19">
@@ -3157,6 +3214,9 @@
       <c r="AQ19" t="n">
         <v>0</v>
       </c>
+      <c r="AR19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3289,9 +3349,12 @@
         <v>0</v>
       </c>
       <c r="AP20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ20" t="n">
         <v>15</v>
       </c>
-      <c r="AQ20" t="n">
+      <c r="AR20" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3426,9 +3489,12 @@
         <v>1</v>
       </c>
       <c r="AP21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ21" t="n">
         <v>21</v>
       </c>
-      <c r="AQ21" t="n">
+      <c r="AR21" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3568,6 +3634,9 @@
       <c r="AQ22" t="n">
         <v>0</v>
       </c>
+      <c r="AR22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3700,9 +3769,12 @@
         <v>1</v>
       </c>
       <c r="AP23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ23" t="n">
         <v>14</v>
       </c>
-      <c r="AQ23" t="n">
+      <c r="AR23" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3837,9 +3909,12 @@
         <v>1</v>
       </c>
       <c r="AP24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ24" t="n">
         <v>21</v>
       </c>
-      <c r="AQ24" t="n">
+      <c r="AR24" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3974,9 +4049,12 @@
         <v>1</v>
       </c>
       <c r="AP25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ25" t="n">
         <v>8</v>
       </c>
-      <c r="AQ25" t="n">
+      <c r="AR25" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4111,10 +4189,13 @@
         <v>1</v>
       </c>
       <c r="AP26" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AQ26" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="27">
@@ -4248,9 +4329,12 @@
         <v>0</v>
       </c>
       <c r="AP27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ27" t="n">
         <v>21</v>
       </c>
-      <c r="AQ27" t="n">
+      <c r="AR27" t="n">
         <v>19</v>
       </c>
     </row>
@@ -4385,10 +4469,13 @@
         <v>1</v>
       </c>
       <c r="AP28" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AQ28" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AR28" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="29">
@@ -4522,9 +4609,12 @@
         <v>1</v>
       </c>
       <c r="AP29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ29" t="n">
         <v>8</v>
       </c>
-      <c r="AQ29" t="n">
+      <c r="AR29" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4659,10 +4749,13 @@
         <v>1</v>
       </c>
       <c r="AP30" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AQ30" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="31">
@@ -4796,9 +4889,12 @@
         <v>0</v>
       </c>
       <c r="AP31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ31" t="n">
         <v>17</v>
       </c>
-      <c r="AQ31" t="n">
+      <c r="AR31" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4933,10 +5029,13 @@
         <v>1</v>
       </c>
       <c r="AP32" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AQ32" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="33">
@@ -5070,9 +5169,12 @@
         <v>0</v>
       </c>
       <c r="AP33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ33" t="n">
         <v>13</v>
       </c>
-      <c r="AQ33" t="n">
+      <c r="AR33" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5207,10 +5309,13 @@
         <v>0</v>
       </c>
       <c r="AP34" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AQ34" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AR34" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="35">
@@ -5344,9 +5449,12 @@
         <v>0</v>
       </c>
       <c r="AP35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ35" t="n">
         <v>17</v>
       </c>
-      <c r="AQ35" t="n">
+      <c r="AR35" t="n">
         <v>17</v>
       </c>
     </row>
@@ -5481,10 +5589,13 @@
         <v>1</v>
       </c>
       <c r="AP36" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AQ36" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AR36" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="37">
@@ -5623,6 +5734,9 @@
       <c r="AQ37" t="n">
         <v>0</v>
       </c>
+      <c r="AR37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5755,9 +5869,12 @@
         <v>0</v>
       </c>
       <c r="AP38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ38" t="n">
         <v>2</v>
       </c>
-      <c r="AQ38" t="n">
+      <c r="AR38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5892,10 +6009,13 @@
         <v>1</v>
       </c>
       <c r="AP39" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AQ39" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AR39" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="40">
@@ -6029,10 +6149,13 @@
         <v>1</v>
       </c>
       <c r="AP40" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AQ40" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AR40" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="41">
@@ -6166,9 +6289,12 @@
         <v>1</v>
       </c>
       <c r="AP41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ41" t="n">
         <v>23</v>
       </c>
-      <c r="AQ41" t="n">
+      <c r="AR41" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6303,9 +6429,12 @@
         <v>0</v>
       </c>
       <c r="AP42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ42" t="n">
         <v>21</v>
       </c>
-      <c r="AQ42" t="n">
+      <c r="AR42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6440,9 +6569,12 @@
         <v>0</v>
       </c>
       <c r="AP43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ43" t="n">
         <v>56</v>
       </c>
-      <c r="AQ43" t="n">
+      <c r="AR43" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6577,10 +6709,13 @@
         <v>1</v>
       </c>
       <c r="AP44" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AQ44" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AR44" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="45">
@@ -6714,10 +6849,13 @@
         <v>1</v>
       </c>
       <c r="AP45" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AQ45" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="46">
@@ -6851,10 +6989,13 @@
         <v>1</v>
       </c>
       <c r="AP46" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AQ46" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AR46" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="47">
@@ -6993,6 +7134,9 @@
       <c r="AQ47" t="n">
         <v>0</v>
       </c>
+      <c r="AR47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7125,10 +7269,13 @@
         <v>1</v>
       </c>
       <c r="AP48" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AQ48" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AR48" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="49">
@@ -7262,10 +7409,13 @@
         <v>0</v>
       </c>
       <c r="AP49" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AQ49" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AR49" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="50">
@@ -7399,9 +7549,12 @@
         <v>0</v>
       </c>
       <c r="AP50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ50" t="n">
         <v>7</v>
       </c>
-      <c r="AQ50" t="n">
+      <c r="AR50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7536,10 +7689,13 @@
         <v>1</v>
       </c>
       <c r="AP51" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AQ51" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AR51" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="52">
@@ -7678,6 +7834,9 @@
       <c r="AQ52" t="n">
         <v>0</v>
       </c>
+      <c r="AR52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7810,10 +7969,13 @@
         <v>0</v>
       </c>
       <c r="AP53" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AQ53" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AR53" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="54">
@@ -7952,6 +8114,9 @@
       <c r="AQ54" t="n">
         <v>0</v>
       </c>
+      <c r="AR54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8084,10 +8249,13 @@
         <v>1</v>
       </c>
       <c r="AP55" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AQ55" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AR55" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="56">
@@ -8221,10 +8389,13 @@
         <v>1</v>
       </c>
       <c r="AP56" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AQ56" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AR56" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="57">
@@ -8358,9 +8529,12 @@
         <v>0</v>
       </c>
       <c r="AP57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ57" t="n">
         <v>8</v>
       </c>
-      <c r="AQ57" t="n">
+      <c r="AR57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8495,9 +8669,12 @@
         <v>0</v>
       </c>
       <c r="AP58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ58" t="n">
         <v>12</v>
       </c>
-      <c r="AQ58" t="n">
+      <c r="AR58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -8632,9 +8809,12 @@
         <v>0</v>
       </c>
       <c r="AP59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ59" t="n">
         <v>5</v>
       </c>
-      <c r="AQ59" t="n">
+      <c r="AR59" t="n">
         <v>5</v>
       </c>
     </row>
@@ -8774,6 +8954,9 @@
       <c r="AQ60" t="n">
         <v>0</v>
       </c>
+      <c r="AR60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8906,10 +9089,13 @@
         <v>1</v>
       </c>
       <c r="AP61" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AQ61" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AR61" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="62">
@@ -9043,10 +9229,13 @@
         <v>1</v>
       </c>
       <c r="AP62" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AQ62" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AR62" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="63">
@@ -9180,9 +9369,12 @@
         <v>0</v>
       </c>
       <c r="AP63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ63" t="n">
         <v>8</v>
       </c>
-      <c r="AQ63" t="n">
+      <c r="AR63" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9322,6 +9514,9 @@
       <c r="AQ64" t="n">
         <v>0</v>
       </c>
+      <c r="AR64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -9454,10 +9649,13 @@
         <v>0</v>
       </c>
       <c r="AP65" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AQ65" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AR65" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="66">
@@ -9591,9 +9789,12 @@
         <v>0</v>
       </c>
       <c r="AP66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ66" t="n">
         <v>4</v>
       </c>
-      <c r="AQ66" t="n">
+      <c r="AR66" t="n">
         <v>4</v>
       </c>
     </row>
@@ -9728,10 +9929,13 @@
         <v>1</v>
       </c>
       <c r="AP67" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AQ67" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AR67" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="68">
@@ -9865,10 +10069,13 @@
         <v>1</v>
       </c>
       <c r="AP68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ68" t="n">
+        <v>14</v>
+      </c>
+      <c r="AR68" t="n">
         <v>13</v>
-      </c>
-      <c r="AQ68" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="69">
@@ -10002,9 +10209,12 @@
         <v>0</v>
       </c>
       <c r="AP69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ69" t="n">
         <v>7</v>
       </c>
-      <c r="AQ69" t="n">
+      <c r="AR69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10139,9 +10349,12 @@
         <v>0</v>
       </c>
       <c r="AP70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ70" t="n">
         <v>23</v>
       </c>
-      <c r="AQ70" t="n">
+      <c r="AR70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -10276,10 +10489,13 @@
         <v>0</v>
       </c>
       <c r="AP71" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AQ71" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AR71" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="72">
@@ -10413,9 +10629,12 @@
         <v>1</v>
       </c>
       <c r="AP72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ72" t="n">
         <v>15</v>
       </c>
-      <c r="AQ72" t="n">
+      <c r="AR72" t="n">
         <v>15</v>
       </c>
     </row>
@@ -10555,6 +10774,9 @@
       <c r="AQ73" t="n">
         <v>0</v>
       </c>
+      <c r="AR73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10692,6 +10914,9 @@
       <c r="AQ74" t="n">
         <v>0</v>
       </c>
+      <c r="AR74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10824,10 +11049,13 @@
         <v>1</v>
       </c>
       <c r="AP75" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AQ75" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AR75" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="76">
@@ -10961,9 +11189,12 @@
         <v>0</v>
       </c>
       <c r="AP76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ76" t="n">
         <v>16</v>
       </c>
-      <c r="AQ76" t="n">
+      <c r="AR76" t="n">
         <v>16</v>
       </c>
     </row>
@@ -11098,9 +11329,12 @@
         <v>0</v>
       </c>
       <c r="AP77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ77" t="n">
         <v>15</v>
       </c>
-      <c r="AQ77" t="n">
+      <c r="AR77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -11235,10 +11469,13 @@
         <v>1</v>
       </c>
       <c r="AP78" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AQ78" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AR78" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="79">
@@ -11372,10 +11609,13 @@
         <v>0</v>
       </c>
       <c r="AP79" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AQ79" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AR79" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="80">
@@ -11509,10 +11749,13 @@
         <v>0</v>
       </c>
       <c r="AP80" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AQ80" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AR80" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="81">
@@ -11646,9 +11889,12 @@
         <v>0</v>
       </c>
       <c r="AP81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ81" t="n">
         <v>3</v>
       </c>
-      <c r="AQ81" t="n">
+      <c r="AR81" t="n">
         <v>3</v>
       </c>
     </row>
@@ -11783,10 +12029,13 @@
         <v>1</v>
       </c>
       <c r="AP82" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AQ82" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AR82" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="83">
@@ -11920,9 +12169,12 @@
         <v>1</v>
       </c>
       <c r="AP83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ83" t="n">
         <v>16</v>
       </c>
-      <c r="AQ83" t="n">
+      <c r="AR83" t="n">
         <v>16</v>
       </c>
     </row>
@@ -12057,10 +12309,13 @@
         <v>1</v>
       </c>
       <c r="AP84" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AQ84" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AR84" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="85">
@@ -12194,9 +12449,12 @@
         <v>0</v>
       </c>
       <c r="AP85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ85" t="n">
         <v>7</v>
       </c>
-      <c r="AQ85" t="n">
+      <c r="AR85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12336,6 +12594,9 @@
       <c r="AQ86" t="n">
         <v>0</v>
       </c>
+      <c r="AR86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -12468,9 +12729,12 @@
         <v>1</v>
       </c>
       <c r="AP87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ87" t="n">
         <v>13</v>
       </c>
-      <c r="AQ87" t="n">
+      <c r="AR87" t="n">
         <v>13</v>
       </c>
     </row>
@@ -12610,6 +12874,9 @@
       <c r="AQ88" t="n">
         <v>0</v>
       </c>
+      <c r="AR88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -12742,9 +13009,12 @@
         <v>0</v>
       </c>
       <c r="AP89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ89" t="n">
         <v>16</v>
       </c>
-      <c r="AQ89" t="n">
+      <c r="AR89" t="n">
         <v>16</v>
       </c>
     </row>
@@ -12879,9 +13149,12 @@
         <v>0</v>
       </c>
       <c r="AP90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ90" t="n">
         <v>14</v>
       </c>
-      <c r="AQ90" t="n">
+      <c r="AR90" t="n">
         <v>14</v>
       </c>
     </row>
@@ -13016,9 +13289,12 @@
         <v>0</v>
       </c>
       <c r="AP91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ91" t="n">
         <v>42</v>
       </c>
-      <c r="AQ91" t="n">
+      <c r="AR91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -13153,9 +13429,12 @@
         <v>0</v>
       </c>
       <c r="AP92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ92" t="n">
         <v>7</v>
       </c>
-      <c r="AQ92" t="n">
+      <c r="AR92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13295,6 +13574,9 @@
       <c r="AQ93" t="n">
         <v>0</v>
       </c>
+      <c r="AR93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -13427,9 +13709,12 @@
         <v>1</v>
       </c>
       <c r="AP94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ94" t="n">
         <v>13</v>
       </c>
-      <c r="AQ94" t="n">
+      <c r="AR94" t="n">
         <v>13</v>
       </c>
     </row>
@@ -13564,9 +13849,12 @@
         <v>1</v>
       </c>
       <c r="AP95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ95" t="n">
         <v>7</v>
       </c>
-      <c r="AQ95" t="n">
+      <c r="AR95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13701,10 +13989,13 @@
         <v>0</v>
       </c>
       <c r="AP96" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AQ96" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AR96" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="97">
@@ -13843,6 +14134,9 @@
       <c r="AQ97" t="n">
         <v>0</v>
       </c>
+      <c r="AR97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -13975,10 +14269,13 @@
         <v>0</v>
       </c>
       <c r="AP98" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AQ98" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AR98" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="99">
@@ -14112,9 +14409,12 @@
         <v>0</v>
       </c>
       <c r="AP99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ99" t="n">
         <v>6</v>
       </c>
-      <c r="AQ99" t="n">
+      <c r="AR99" t="n">
         <v>6</v>
       </c>
     </row>
@@ -14254,6 +14554,9 @@
       <c r="AQ100" t="n">
         <v>0</v>
       </c>
+      <c r="AR100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -14386,9 +14689,12 @@
         <v>1</v>
       </c>
       <c r="AP101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ101" t="n">
         <v>23</v>
       </c>
-      <c r="AQ101" t="n">
+      <c r="AR101" t="n">
         <v>23</v>
       </c>
     </row>
@@ -14523,10 +14829,13 @@
         <v>1</v>
       </c>
       <c r="AP102" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AQ102" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AR102" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="103">
@@ -14660,9 +14969,12 @@
         <v>1</v>
       </c>
       <c r="AP103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ103" t="n">
         <v>20</v>
       </c>
-      <c r="AQ103" t="n">
+      <c r="AR103" t="n">
         <v>20</v>
       </c>
     </row>
@@ -14797,9 +15109,12 @@
         <v>1</v>
       </c>
       <c r="AP104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ104" t="n">
         <v>10</v>
       </c>
-      <c r="AQ104" t="n">
+      <c r="AR104" t="n">
         <v>10</v>
       </c>
     </row>
@@ -14934,10 +15249,13 @@
         <v>1</v>
       </c>
       <c r="AP105" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AQ105" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AR105" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="106">
@@ -15071,9 +15389,12 @@
         <v>0</v>
       </c>
       <c r="AP106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ106" t="n">
         <v>7</v>
       </c>
-      <c r="AQ106" t="n">
+      <c r="AR106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15208,9 +15529,12 @@
         <v>1</v>
       </c>
       <c r="AP107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ107" t="n">
         <v>9</v>
       </c>
-      <c r="AQ107" t="n">
+      <c r="AR107" t="n">
         <v>9</v>
       </c>
     </row>
@@ -15345,9 +15669,12 @@
         <v>0</v>
       </c>
       <c r="AP108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ108" t="n">
         <v>2</v>
       </c>
-      <c r="AQ108" t="n">
+      <c r="AR108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -15482,9 +15809,12 @@
         <v>0</v>
       </c>
       <c r="AP109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ109" t="n">
         <v>2</v>
       </c>
-      <c r="AQ109" t="n">
+      <c r="AR109" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#2999)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR109"/>
+  <dimension ref="A1:AS109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -472,8 +472,9 @@
     <col width="12" customWidth="1" min="40" max="40"/>
     <col width="12" customWidth="1" min="41" max="41"/>
     <col width="12" customWidth="1" min="42" max="42"/>
-    <col width="13" customWidth="1" min="43" max="43"/>
+    <col width="12" customWidth="1" min="43" max="43"/>
     <col width="13" customWidth="1" min="44" max="44"/>
+    <col width="13" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -687,12 +688,17 @@
           <t>2026-04-03</t>
         </is>
       </c>
-      <c r="AQ1" s="2" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="AR1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AR1" s="2" t="inlineStr">
+      <c r="AS1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -832,9 +838,12 @@
         <v>0</v>
       </c>
       <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
         <v>10</v>
       </c>
-      <c r="AR2" t="n">
+      <c r="AS2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -972,9 +981,12 @@
         <v>0</v>
       </c>
       <c r="AQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR3" t="n">
         <v>9</v>
       </c>
-      <c r="AR3" t="n">
+      <c r="AS3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1112,9 +1124,12 @@
         <v>1</v>
       </c>
       <c r="AQ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR4" t="n">
         <v>24</v>
       </c>
-      <c r="AR4" t="n">
+      <c r="AS4" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1252,9 +1267,12 @@
         <v>0</v>
       </c>
       <c r="AQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR5" t="n">
         <v>15</v>
       </c>
-      <c r="AR5" t="n">
+      <c r="AS5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1392,9 +1410,12 @@
         <v>1</v>
       </c>
       <c r="AQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR6" t="n">
         <v>17</v>
       </c>
-      <c r="AR6" t="n">
+      <c r="AS6" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1532,9 +1553,12 @@
         <v>0</v>
       </c>
       <c r="AQ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR7" t="n">
         <v>16</v>
       </c>
-      <c r="AR7" t="n">
+      <c r="AS7" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1672,10 +1696,13 @@
         <v>0</v>
       </c>
       <c r="AQ8" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AR8" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -1812,9 +1839,12 @@
         <v>1</v>
       </c>
       <c r="AQ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR9" t="n">
         <v>21</v>
       </c>
-      <c r="AR9" t="n">
+      <c r="AS9" t="n">
         <v>21</v>
       </c>
     </row>
@@ -1952,9 +1982,12 @@
         <v>1</v>
       </c>
       <c r="AQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR10" t="n">
         <v>24</v>
       </c>
-      <c r="AR10" t="n">
+      <c r="AS10" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2092,9 +2125,12 @@
         <v>0</v>
       </c>
       <c r="AQ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR11" t="n">
         <v>19</v>
       </c>
-      <c r="AR11" t="n">
+      <c r="AS11" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2232,9 +2268,12 @@
         <v>1</v>
       </c>
       <c r="AQ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR12" t="n">
         <v>23</v>
       </c>
-      <c r="AR12" t="n">
+      <c r="AS12" t="n">
         <v>23</v>
       </c>
     </row>
@@ -2372,9 +2411,12 @@
         <v>0</v>
       </c>
       <c r="AQ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR13" t="n">
         <v>12</v>
       </c>
-      <c r="AR13" t="n">
+      <c r="AS13" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2512,9 +2554,12 @@
         <v>0</v>
       </c>
       <c r="AQ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR14" t="n">
         <v>22</v>
       </c>
-      <c r="AR14" t="n">
+      <c r="AS14" t="n">
         <v>22</v>
       </c>
     </row>
@@ -2652,9 +2697,12 @@
         <v>0</v>
       </c>
       <c r="AQ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR15" t="n">
         <v>9</v>
       </c>
-      <c r="AR15" t="n">
+      <c r="AS15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2792,9 +2840,12 @@
         <v>1</v>
       </c>
       <c r="AQ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR16" t="n">
         <v>17</v>
       </c>
-      <c r="AR16" t="n">
+      <c r="AS16" t="n">
         <v>17</v>
       </c>
     </row>
@@ -2932,9 +2983,12 @@
         <v>0</v>
       </c>
       <c r="AQ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR17" t="n">
         <v>16</v>
       </c>
-      <c r="AR17" t="n">
+      <c r="AS17" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3072,9 +3126,12 @@
         <v>1</v>
       </c>
       <c r="AQ18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR18" t="n">
         <v>20</v>
       </c>
-      <c r="AR18" t="n">
+      <c r="AS18" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3217,6 +3274,9 @@
       <c r="AR19" t="n">
         <v>0</v>
       </c>
+      <c r="AS19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3352,9 +3412,12 @@
         <v>0</v>
       </c>
       <c r="AQ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR20" t="n">
         <v>15</v>
       </c>
-      <c r="AR20" t="n">
+      <c r="AS20" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3492,9 +3555,12 @@
         <v>0</v>
       </c>
       <c r="AQ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR21" t="n">
         <v>21</v>
       </c>
-      <c r="AR21" t="n">
+      <c r="AS21" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3637,6 +3703,9 @@
       <c r="AR22" t="n">
         <v>0</v>
       </c>
+      <c r="AS22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3772,9 +3841,12 @@
         <v>0</v>
       </c>
       <c r="AQ23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR23" t="n">
         <v>14</v>
       </c>
-      <c r="AR23" t="n">
+      <c r="AS23" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3912,10 +3984,13 @@
         <v>0</v>
       </c>
       <c r="AQ24" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AR24" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="25">
@@ -4052,9 +4127,12 @@
         <v>0</v>
       </c>
       <c r="AQ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR25" t="n">
         <v>8</v>
       </c>
-      <c r="AR25" t="n">
+      <c r="AS25" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4192,9 +4270,12 @@
         <v>1</v>
       </c>
       <c r="AQ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR26" t="n">
         <v>21</v>
       </c>
-      <c r="AR26" t="n">
+      <c r="AS26" t="n">
         <v>21</v>
       </c>
     </row>
@@ -4332,9 +4413,12 @@
         <v>0</v>
       </c>
       <c r="AQ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR27" t="n">
         <v>21</v>
       </c>
-      <c r="AR27" t="n">
+      <c r="AS27" t="n">
         <v>19</v>
       </c>
     </row>
@@ -4472,10 +4556,13 @@
         <v>1</v>
       </c>
       <c r="AQ28" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AR28" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="29">
@@ -4612,9 +4699,12 @@
         <v>0</v>
       </c>
       <c r="AQ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR29" t="n">
         <v>8</v>
       </c>
-      <c r="AR29" t="n">
+      <c r="AS29" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4752,9 +4842,12 @@
         <v>1</v>
       </c>
       <c r="AQ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR30" t="n">
         <v>18</v>
       </c>
-      <c r="AR30" t="n">
+      <c r="AS30" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4892,9 +4985,12 @@
         <v>0</v>
       </c>
       <c r="AQ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR31" t="n">
         <v>17</v>
       </c>
-      <c r="AR31" t="n">
+      <c r="AS31" t="n">
         <v>17</v>
       </c>
     </row>
@@ -5032,9 +5128,12 @@
         <v>1</v>
       </c>
       <c r="AQ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR32" t="n">
         <v>15</v>
       </c>
-      <c r="AR32" t="n">
+      <c r="AS32" t="n">
         <v>15</v>
       </c>
     </row>
@@ -5172,9 +5271,12 @@
         <v>0</v>
       </c>
       <c r="AQ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR33" t="n">
         <v>13</v>
       </c>
-      <c r="AR33" t="n">
+      <c r="AS33" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5312,9 +5414,12 @@
         <v>1</v>
       </c>
       <c r="AQ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR34" t="n">
         <v>9</v>
       </c>
-      <c r="AR34" t="n">
+      <c r="AS34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5452,9 +5557,12 @@
         <v>0</v>
       </c>
       <c r="AQ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR35" t="n">
         <v>17</v>
       </c>
-      <c r="AR35" t="n">
+      <c r="AS35" t="n">
         <v>17</v>
       </c>
     </row>
@@ -5592,9 +5700,12 @@
         <v>1</v>
       </c>
       <c r="AQ36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR36" t="n">
         <v>12</v>
       </c>
-      <c r="AR36" t="n">
+      <c r="AS36" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5737,6 +5848,9 @@
       <c r="AR37" t="n">
         <v>0</v>
       </c>
+      <c r="AS37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5872,9 +5986,12 @@
         <v>0</v>
       </c>
       <c r="AQ38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR38" t="n">
         <v>2</v>
       </c>
-      <c r="AR38" t="n">
+      <c r="AS38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6012,9 +6129,12 @@
         <v>1</v>
       </c>
       <c r="AQ39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR39" t="n">
         <v>23</v>
       </c>
-      <c r="AR39" t="n">
+      <c r="AS39" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6152,9 +6272,12 @@
         <v>1</v>
       </c>
       <c r="AQ40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR40" t="n">
         <v>18</v>
       </c>
-      <c r="AR40" t="n">
+      <c r="AS40" t="n">
         <v>18</v>
       </c>
     </row>
@@ -6292,9 +6415,12 @@
         <v>0</v>
       </c>
       <c r="AQ41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR41" t="n">
         <v>23</v>
       </c>
-      <c r="AR41" t="n">
+      <c r="AS41" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6432,9 +6558,12 @@
         <v>0</v>
       </c>
       <c r="AQ42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR42" t="n">
         <v>21</v>
       </c>
-      <c r="AR42" t="n">
+      <c r="AS42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6572,9 +6701,12 @@
         <v>0</v>
       </c>
       <c r="AQ43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR43" t="n">
         <v>56</v>
       </c>
-      <c r="AR43" t="n">
+      <c r="AS43" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6712,9 +6844,12 @@
         <v>1</v>
       </c>
       <c r="AQ44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR44" t="n">
         <v>19</v>
       </c>
-      <c r="AR44" t="n">
+      <c r="AS44" t="n">
         <v>19</v>
       </c>
     </row>
@@ -6852,9 +6987,12 @@
         <v>1</v>
       </c>
       <c r="AQ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR45" t="n">
         <v>22</v>
       </c>
-      <c r="AR45" t="n">
+      <c r="AS45" t="n">
         <v>22</v>
       </c>
     </row>
@@ -6992,9 +7130,12 @@
         <v>1</v>
       </c>
       <c r="AQ46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR46" t="n">
         <v>19</v>
       </c>
-      <c r="AR46" t="n">
+      <c r="AS46" t="n">
         <v>19</v>
       </c>
     </row>
@@ -7137,6 +7278,9 @@
       <c r="AR47" t="n">
         <v>0</v>
       </c>
+      <c r="AS47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7272,9 +7416,12 @@
         <v>1</v>
       </c>
       <c r="AQ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR48" t="n">
         <v>22</v>
       </c>
-      <c r="AR48" t="n">
+      <c r="AS48" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7412,9 +7559,12 @@
         <v>1</v>
       </c>
       <c r="AQ49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR49" t="n">
         <v>17</v>
       </c>
-      <c r="AR49" t="n">
+      <c r="AS49" t="n">
         <v>17</v>
       </c>
     </row>
@@ -7552,9 +7702,12 @@
         <v>0</v>
       </c>
       <c r="AQ50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR50" t="n">
         <v>7</v>
       </c>
-      <c r="AR50" t="n">
+      <c r="AS50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7692,9 +7845,12 @@
         <v>1</v>
       </c>
       <c r="AQ51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR51" t="n">
         <v>23</v>
       </c>
-      <c r="AR51" t="n">
+      <c r="AS51" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7837,6 +7993,9 @@
       <c r="AR52" t="n">
         <v>0</v>
       </c>
+      <c r="AS52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7972,9 +8131,12 @@
         <v>1</v>
       </c>
       <c r="AQ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR53" t="n">
         <v>13</v>
       </c>
-      <c r="AR53" t="n">
+      <c r="AS53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -8117,6 +8279,9 @@
       <c r="AR54" t="n">
         <v>0</v>
       </c>
+      <c r="AS54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8252,10 +8417,13 @@
         <v>1</v>
       </c>
       <c r="AQ55" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AR55" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AS55" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="56">
@@ -8392,9 +8560,12 @@
         <v>1</v>
       </c>
       <c r="AQ56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR56" t="n">
         <v>21</v>
       </c>
-      <c r="AR56" t="n">
+      <c r="AS56" t="n">
         <v>21</v>
       </c>
     </row>
@@ -8532,9 +8703,12 @@
         <v>0</v>
       </c>
       <c r="AQ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR57" t="n">
         <v>8</v>
       </c>
-      <c r="AR57" t="n">
+      <c r="AS57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8672,9 +8846,12 @@
         <v>0</v>
       </c>
       <c r="AQ58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR58" t="n">
         <v>12</v>
       </c>
-      <c r="AR58" t="n">
+      <c r="AS58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -8812,9 +8989,12 @@
         <v>0</v>
       </c>
       <c r="AQ59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR59" t="n">
         <v>5</v>
       </c>
-      <c r="AR59" t="n">
+      <c r="AS59" t="n">
         <v>5</v>
       </c>
     </row>
@@ -8957,6 +9137,9 @@
       <c r="AR60" t="n">
         <v>0</v>
       </c>
+      <c r="AS60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -9092,9 +9275,12 @@
         <v>1</v>
       </c>
       <c r="AQ61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR61" t="n">
         <v>20</v>
       </c>
-      <c r="AR61" t="n">
+      <c r="AS61" t="n">
         <v>20</v>
       </c>
     </row>
@@ -9232,9 +9418,12 @@
         <v>1</v>
       </c>
       <c r="AQ62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR62" t="n">
         <v>21</v>
       </c>
-      <c r="AR62" t="n">
+      <c r="AS62" t="n">
         <v>21</v>
       </c>
     </row>
@@ -9372,9 +9561,12 @@
         <v>0</v>
       </c>
       <c r="AQ63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR63" t="n">
         <v>8</v>
       </c>
-      <c r="AR63" t="n">
+      <c r="AS63" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9517,6 +9709,9 @@
       <c r="AR64" t="n">
         <v>0</v>
       </c>
+      <c r="AS64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -9652,9 +9847,12 @@
         <v>1</v>
       </c>
       <c r="AQ65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR65" t="n">
         <v>11</v>
       </c>
-      <c r="AR65" t="n">
+      <c r="AS65" t="n">
         <v>11</v>
       </c>
     </row>
@@ -9792,9 +9990,12 @@
         <v>0</v>
       </c>
       <c r="AQ66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR66" t="n">
         <v>4</v>
       </c>
-      <c r="AR66" t="n">
+      <c r="AS66" t="n">
         <v>4</v>
       </c>
     </row>
@@ -9932,9 +10133,12 @@
         <v>1</v>
       </c>
       <c r="AQ67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR67" t="n">
         <v>24</v>
       </c>
-      <c r="AR67" t="n">
+      <c r="AS67" t="n">
         <v>24</v>
       </c>
     </row>
@@ -10072,9 +10276,12 @@
         <v>1</v>
       </c>
       <c r="AQ68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR68" t="n">
         <v>14</v>
       </c>
-      <c r="AR68" t="n">
+      <c r="AS68" t="n">
         <v>13</v>
       </c>
     </row>
@@ -10212,9 +10419,12 @@
         <v>0</v>
       </c>
       <c r="AQ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR69" t="n">
         <v>7</v>
       </c>
-      <c r="AR69" t="n">
+      <c r="AS69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10352,9 +10562,12 @@
         <v>0</v>
       </c>
       <c r="AQ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR70" t="n">
         <v>23</v>
       </c>
-      <c r="AR70" t="n">
+      <c r="AS70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -10492,9 +10705,12 @@
         <v>1</v>
       </c>
       <c r="AQ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR71" t="n">
         <v>16</v>
       </c>
-      <c r="AR71" t="n">
+      <c r="AS71" t="n">
         <v>16</v>
       </c>
     </row>
@@ -10632,9 +10848,12 @@
         <v>0</v>
       </c>
       <c r="AQ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR72" t="n">
         <v>15</v>
       </c>
-      <c r="AR72" t="n">
+      <c r="AS72" t="n">
         <v>15</v>
       </c>
     </row>
@@ -10777,6 +10996,9 @@
       <c r="AR73" t="n">
         <v>0</v>
       </c>
+      <c r="AS73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10917,6 +11139,9 @@
       <c r="AR74" t="n">
         <v>0</v>
       </c>
+      <c r="AS74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -11052,9 +11277,12 @@
         <v>1</v>
       </c>
       <c r="AQ75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR75" t="n">
         <v>16</v>
       </c>
-      <c r="AR75" t="n">
+      <c r="AS75" t="n">
         <v>16</v>
       </c>
     </row>
@@ -11192,9 +11420,12 @@
         <v>0</v>
       </c>
       <c r="AQ76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR76" t="n">
         <v>16</v>
       </c>
-      <c r="AR76" t="n">
+      <c r="AS76" t="n">
         <v>16</v>
       </c>
     </row>
@@ -11332,9 +11563,12 @@
         <v>0</v>
       </c>
       <c r="AQ77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR77" t="n">
         <v>15</v>
       </c>
-      <c r="AR77" t="n">
+      <c r="AS77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -11472,9 +11706,12 @@
         <v>1</v>
       </c>
       <c r="AQ78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR78" t="n">
         <v>21</v>
       </c>
-      <c r="AR78" t="n">
+      <c r="AS78" t="n">
         <v>21</v>
       </c>
     </row>
@@ -11612,9 +11849,12 @@
         <v>1</v>
       </c>
       <c r="AQ79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR79" t="n">
         <v>18</v>
       </c>
-      <c r="AR79" t="n">
+      <c r="AS79" t="n">
         <v>18</v>
       </c>
     </row>
@@ -11752,9 +11992,12 @@
         <v>1</v>
       </c>
       <c r="AQ80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR80" t="n">
         <v>9</v>
       </c>
-      <c r="AR80" t="n">
+      <c r="AS80" t="n">
         <v>9</v>
       </c>
     </row>
@@ -11892,9 +12135,12 @@
         <v>0</v>
       </c>
       <c r="AQ81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR81" t="n">
         <v>3</v>
       </c>
-      <c r="AR81" t="n">
+      <c r="AS81" t="n">
         <v>3</v>
       </c>
     </row>
@@ -12032,9 +12278,12 @@
         <v>1</v>
       </c>
       <c r="AQ82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR82" t="n">
         <v>7</v>
       </c>
-      <c r="AR82" t="n">
+      <c r="AS82" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12172,9 +12421,12 @@
         <v>0</v>
       </c>
       <c r="AQ83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR83" t="n">
         <v>16</v>
       </c>
-      <c r="AR83" t="n">
+      <c r="AS83" t="n">
         <v>16</v>
       </c>
     </row>
@@ -12312,9 +12564,12 @@
         <v>1</v>
       </c>
       <c r="AQ84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR84" t="n">
         <v>8</v>
       </c>
-      <c r="AR84" t="n">
+      <c r="AS84" t="n">
         <v>8</v>
       </c>
     </row>
@@ -12452,9 +12707,12 @@
         <v>0</v>
       </c>
       <c r="AQ85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR85" t="n">
         <v>7</v>
       </c>
-      <c r="AR85" t="n">
+      <c r="AS85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12597,6 +12855,9 @@
       <c r="AR86" t="n">
         <v>0</v>
       </c>
+      <c r="AS86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -12732,9 +12993,12 @@
         <v>0</v>
       </c>
       <c r="AQ87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR87" t="n">
         <v>13</v>
       </c>
-      <c r="AR87" t="n">
+      <c r="AS87" t="n">
         <v>13</v>
       </c>
     </row>
@@ -12877,6 +13141,9 @@
       <c r="AR88" t="n">
         <v>0</v>
       </c>
+      <c r="AS88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -13012,9 +13279,12 @@
         <v>0</v>
       </c>
       <c r="AQ89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR89" t="n">
         <v>16</v>
       </c>
-      <c r="AR89" t="n">
+      <c r="AS89" t="n">
         <v>16</v>
       </c>
     </row>
@@ -13152,9 +13422,12 @@
         <v>0</v>
       </c>
       <c r="AQ90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR90" t="n">
         <v>14</v>
       </c>
-      <c r="AR90" t="n">
+      <c r="AS90" t="n">
         <v>14</v>
       </c>
     </row>
@@ -13292,9 +13565,12 @@
         <v>0</v>
       </c>
       <c r="AQ91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR91" t="n">
         <v>42</v>
       </c>
-      <c r="AR91" t="n">
+      <c r="AS91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -13432,9 +13708,12 @@
         <v>0</v>
       </c>
       <c r="AQ92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR92" t="n">
         <v>7</v>
       </c>
-      <c r="AR92" t="n">
+      <c r="AS92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13577,6 +13856,9 @@
       <c r="AR93" t="n">
         <v>0</v>
       </c>
+      <c r="AS93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -13712,9 +13994,12 @@
         <v>0</v>
       </c>
       <c r="AQ94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR94" t="n">
         <v>13</v>
       </c>
-      <c r="AR94" t="n">
+      <c r="AS94" t="n">
         <v>13</v>
       </c>
     </row>
@@ -13852,9 +14137,12 @@
         <v>0</v>
       </c>
       <c r="AQ95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR95" t="n">
         <v>7</v>
       </c>
-      <c r="AR95" t="n">
+      <c r="AS95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13992,9 +14280,12 @@
         <v>1</v>
       </c>
       <c r="AQ96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR96" t="n">
         <v>18</v>
       </c>
-      <c r="AR96" t="n">
+      <c r="AS96" t="n">
         <v>18</v>
       </c>
     </row>
@@ -14137,6 +14428,9 @@
       <c r="AR97" t="n">
         <v>0</v>
       </c>
+      <c r="AS97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -14272,10 +14566,13 @@
         <v>1</v>
       </c>
       <c r="AQ98" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AR98" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AS98" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="99">
@@ -14412,9 +14709,12 @@
         <v>0</v>
       </c>
       <c r="AQ99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR99" t="n">
         <v>6</v>
       </c>
-      <c r="AR99" t="n">
+      <c r="AS99" t="n">
         <v>6</v>
       </c>
     </row>
@@ -14557,6 +14857,9 @@
       <c r="AR100" t="n">
         <v>0</v>
       </c>
+      <c r="AS100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -14692,9 +14995,12 @@
         <v>0</v>
       </c>
       <c r="AQ101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR101" t="n">
         <v>23</v>
       </c>
-      <c r="AR101" t="n">
+      <c r="AS101" t="n">
         <v>23</v>
       </c>
     </row>
@@ -14832,9 +15138,12 @@
         <v>1</v>
       </c>
       <c r="AQ102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR102" t="n">
         <v>22</v>
       </c>
-      <c r="AR102" t="n">
+      <c r="AS102" t="n">
         <v>22</v>
       </c>
     </row>
@@ -14972,10 +15281,13 @@
         <v>0</v>
       </c>
       <c r="AQ103" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AR103" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AS103" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="104">
@@ -15112,9 +15424,12 @@
         <v>0</v>
       </c>
       <c r="AQ104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR104" t="n">
         <v>10</v>
       </c>
-      <c r="AR104" t="n">
+      <c r="AS104" t="n">
         <v>10</v>
       </c>
     </row>
@@ -15252,10 +15567,13 @@
         <v>1</v>
       </c>
       <c r="AQ105" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AR105" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AS105" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="106">
@@ -15392,9 +15710,12 @@
         <v>0</v>
       </c>
       <c r="AQ106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR106" t="n">
         <v>7</v>
       </c>
-      <c r="AR106" t="n">
+      <c r="AS106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15532,9 +15853,12 @@
         <v>0</v>
       </c>
       <c r="AQ107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR107" t="n">
         <v>9</v>
       </c>
-      <c r="AR107" t="n">
+      <c r="AS107" t="n">
         <v>9</v>
       </c>
     </row>
@@ -15672,9 +15996,12 @@
         <v>0</v>
       </c>
       <c r="AQ108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR108" t="n">
         <v>2</v>
       </c>
-      <c r="AR108" t="n">
+      <c r="AS108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -15812,9 +16139,12 @@
         <v>0</v>
       </c>
       <c r="AQ109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR109" t="n">
         <v>2</v>
       </c>
-      <c r="AR109" t="n">
+      <c r="AS109" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3048)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS109"/>
+  <dimension ref="A1:AT109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -473,8 +473,9 @@
     <col width="12" customWidth="1" min="41" max="41"/>
     <col width="12" customWidth="1" min="42" max="42"/>
     <col width="12" customWidth="1" min="43" max="43"/>
-    <col width="13" customWidth="1" min="44" max="44"/>
+    <col width="12" customWidth="1" min="44" max="44"/>
     <col width="13" customWidth="1" min="45" max="45"/>
+    <col width="13" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -693,12 +694,17 @@
           <t>2026-04-04</t>
         </is>
       </c>
-      <c r="AR1" s="2" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="AS1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AS1" s="2" t="inlineStr">
+      <c r="AT1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -841,9 +847,12 @@
         <v>0</v>
       </c>
       <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
         <v>10</v>
       </c>
-      <c r="AS2" t="n">
+      <c r="AT2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -984,9 +993,12 @@
         <v>0</v>
       </c>
       <c r="AR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS3" t="n">
         <v>9</v>
       </c>
-      <c r="AS3" t="n">
+      <c r="AT3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1127,9 +1139,12 @@
         <v>0</v>
       </c>
       <c r="AR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="n">
         <v>24</v>
       </c>
-      <c r="AS4" t="n">
+      <c r="AT4" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1270,9 +1285,12 @@
         <v>0</v>
       </c>
       <c r="AR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS5" t="n">
         <v>15</v>
       </c>
-      <c r="AS5" t="n">
+      <c r="AT5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1413,9 +1431,12 @@
         <v>0</v>
       </c>
       <c r="AR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS6" t="n">
         <v>17</v>
       </c>
-      <c r="AS6" t="n">
+      <c r="AT6" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1556,9 +1577,12 @@
         <v>0</v>
       </c>
       <c r="AR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS7" t="n">
         <v>16</v>
       </c>
-      <c r="AS7" t="n">
+      <c r="AT7" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1699,9 +1723,12 @@
         <v>1</v>
       </c>
       <c r="AR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS8" t="n">
         <v>23</v>
       </c>
-      <c r="AS8" t="n">
+      <c r="AT8" t="n">
         <v>23</v>
       </c>
     </row>
@@ -1842,9 +1869,12 @@
         <v>0</v>
       </c>
       <c r="AR9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS9" t="n">
         <v>21</v>
       </c>
-      <c r="AS9" t="n">
+      <c r="AT9" t="n">
         <v>21</v>
       </c>
     </row>
@@ -1985,9 +2015,12 @@
         <v>0</v>
       </c>
       <c r="AR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS10" t="n">
         <v>24</v>
       </c>
-      <c r="AS10" t="n">
+      <c r="AT10" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2128,9 +2161,12 @@
         <v>0</v>
       </c>
       <c r="AR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS11" t="n">
         <v>19</v>
       </c>
-      <c r="AS11" t="n">
+      <c r="AT11" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2271,9 +2307,12 @@
         <v>0</v>
       </c>
       <c r="AR12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS12" t="n">
         <v>23</v>
       </c>
-      <c r="AS12" t="n">
+      <c r="AT12" t="n">
         <v>23</v>
       </c>
     </row>
@@ -2414,9 +2453,12 @@
         <v>0</v>
       </c>
       <c r="AR13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS13" t="n">
         <v>12</v>
       </c>
-      <c r="AS13" t="n">
+      <c r="AT13" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2557,9 +2599,12 @@
         <v>0</v>
       </c>
       <c r="AR14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS14" t="n">
         <v>22</v>
       </c>
-      <c r="AS14" t="n">
+      <c r="AT14" t="n">
         <v>22</v>
       </c>
     </row>
@@ -2700,9 +2745,12 @@
         <v>0</v>
       </c>
       <c r="AR15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS15" t="n">
         <v>9</v>
       </c>
-      <c r="AS15" t="n">
+      <c r="AT15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2843,9 +2891,12 @@
         <v>0</v>
       </c>
       <c r="AR16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS16" t="n">
         <v>17</v>
       </c>
-      <c r="AS16" t="n">
+      <c r="AT16" t="n">
         <v>17</v>
       </c>
     </row>
@@ -2986,9 +3037,12 @@
         <v>0</v>
       </c>
       <c r="AR17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS17" t="n">
         <v>16</v>
       </c>
-      <c r="AS17" t="n">
+      <c r="AT17" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3129,9 +3183,12 @@
         <v>0</v>
       </c>
       <c r="AR18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS18" t="n">
         <v>20</v>
       </c>
-      <c r="AS18" t="n">
+      <c r="AT18" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3277,6 +3334,9 @@
       <c r="AS19" t="n">
         <v>0</v>
       </c>
+      <c r="AT19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3415,9 +3475,12 @@
         <v>0</v>
       </c>
       <c r="AR20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS20" t="n">
         <v>15</v>
       </c>
-      <c r="AS20" t="n">
+      <c r="AT20" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3558,9 +3621,12 @@
         <v>0</v>
       </c>
       <c r="AR21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS21" t="n">
         <v>21</v>
       </c>
-      <c r="AS21" t="n">
+      <c r="AT21" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3706,6 +3772,9 @@
       <c r="AS22" t="n">
         <v>0</v>
       </c>
+      <c r="AT22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3844,9 +3913,12 @@
         <v>0</v>
       </c>
       <c r="AR23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS23" t="n">
         <v>14</v>
       </c>
-      <c r="AS23" t="n">
+      <c r="AT23" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3987,9 +4059,12 @@
         <v>1</v>
       </c>
       <c r="AR24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS24" t="n">
         <v>22</v>
       </c>
-      <c r="AS24" t="n">
+      <c r="AT24" t="n">
         <v>22</v>
       </c>
     </row>
@@ -4130,9 +4205,12 @@
         <v>0</v>
       </c>
       <c r="AR25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS25" t="n">
         <v>8</v>
       </c>
-      <c r="AS25" t="n">
+      <c r="AT25" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4273,9 +4351,12 @@
         <v>0</v>
       </c>
       <c r="AR26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS26" t="n">
         <v>21</v>
       </c>
-      <c r="AS26" t="n">
+      <c r="AT26" t="n">
         <v>21</v>
       </c>
     </row>
@@ -4416,9 +4497,12 @@
         <v>0</v>
       </c>
       <c r="AR27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS27" t="n">
         <v>21</v>
       </c>
-      <c r="AS27" t="n">
+      <c r="AT27" t="n">
         <v>19</v>
       </c>
     </row>
@@ -4559,9 +4643,12 @@
         <v>1</v>
       </c>
       <c r="AR28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS28" t="n">
         <v>11</v>
       </c>
-      <c r="AS28" t="n">
+      <c r="AT28" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4702,9 +4789,12 @@
         <v>0</v>
       </c>
       <c r="AR29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS29" t="n">
         <v>8</v>
       </c>
-      <c r="AS29" t="n">
+      <c r="AT29" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4845,9 +4935,12 @@
         <v>0</v>
       </c>
       <c r="AR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS30" t="n">
         <v>18</v>
       </c>
-      <c r="AS30" t="n">
+      <c r="AT30" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4988,9 +5081,12 @@
         <v>0</v>
       </c>
       <c r="AR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS31" t="n">
         <v>17</v>
       </c>
-      <c r="AS31" t="n">
+      <c r="AT31" t="n">
         <v>17</v>
       </c>
     </row>
@@ -5131,9 +5227,12 @@
         <v>0</v>
       </c>
       <c r="AR32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS32" t="n">
         <v>15</v>
       </c>
-      <c r="AS32" t="n">
+      <c r="AT32" t="n">
         <v>15</v>
       </c>
     </row>
@@ -5274,9 +5373,12 @@
         <v>0</v>
       </c>
       <c r="AR33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS33" t="n">
         <v>13</v>
       </c>
-      <c r="AS33" t="n">
+      <c r="AT33" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5417,9 +5519,12 @@
         <v>0</v>
       </c>
       <c r="AR34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS34" t="n">
         <v>9</v>
       </c>
-      <c r="AS34" t="n">
+      <c r="AT34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5560,9 +5665,12 @@
         <v>0</v>
       </c>
       <c r="AR35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS35" t="n">
         <v>17</v>
       </c>
-      <c r="AS35" t="n">
+      <c r="AT35" t="n">
         <v>17</v>
       </c>
     </row>
@@ -5703,9 +5811,12 @@
         <v>0</v>
       </c>
       <c r="AR36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS36" t="n">
         <v>12</v>
       </c>
-      <c r="AS36" t="n">
+      <c r="AT36" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5851,6 +5962,9 @@
       <c r="AS37" t="n">
         <v>0</v>
       </c>
+      <c r="AT37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5989,9 +6103,12 @@
         <v>0</v>
       </c>
       <c r="AR38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS38" t="n">
         <v>2</v>
       </c>
-      <c r="AS38" t="n">
+      <c r="AT38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6132,9 +6249,12 @@
         <v>0</v>
       </c>
       <c r="AR39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS39" t="n">
         <v>23</v>
       </c>
-      <c r="AS39" t="n">
+      <c r="AT39" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6275,9 +6395,12 @@
         <v>0</v>
       </c>
       <c r="AR40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS40" t="n">
         <v>18</v>
       </c>
-      <c r="AS40" t="n">
+      <c r="AT40" t="n">
         <v>18</v>
       </c>
     </row>
@@ -6418,9 +6541,12 @@
         <v>0</v>
       </c>
       <c r="AR41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS41" t="n">
         <v>23</v>
       </c>
-      <c r="AS41" t="n">
+      <c r="AT41" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6561,9 +6687,12 @@
         <v>0</v>
       </c>
       <c r="AR42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS42" t="n">
         <v>21</v>
       </c>
-      <c r="AS42" t="n">
+      <c r="AT42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6704,9 +6833,12 @@
         <v>0</v>
       </c>
       <c r="AR43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS43" t="n">
         <v>56</v>
       </c>
-      <c r="AS43" t="n">
+      <c r="AT43" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6847,10 +6979,13 @@
         <v>0</v>
       </c>
       <c r="AR44" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AS44" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AT44" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="45">
@@ -6990,9 +7125,12 @@
         <v>0</v>
       </c>
       <c r="AR45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS45" t="n">
         <v>22</v>
       </c>
-      <c r="AS45" t="n">
+      <c r="AT45" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7133,9 +7271,12 @@
         <v>0</v>
       </c>
       <c r="AR46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS46" t="n">
         <v>19</v>
       </c>
-      <c r="AS46" t="n">
+      <c r="AT46" t="n">
         <v>19</v>
       </c>
     </row>
@@ -7281,6 +7422,9 @@
       <c r="AS47" t="n">
         <v>0</v>
       </c>
+      <c r="AT47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7419,9 +7563,12 @@
         <v>0</v>
       </c>
       <c r="AR48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS48" t="n">
         <v>22</v>
       </c>
-      <c r="AS48" t="n">
+      <c r="AT48" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7562,9 +7709,12 @@
         <v>0</v>
       </c>
       <c r="AR49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS49" t="n">
         <v>17</v>
       </c>
-      <c r="AS49" t="n">
+      <c r="AT49" t="n">
         <v>17</v>
       </c>
     </row>
@@ -7705,9 +7855,12 @@
         <v>0</v>
       </c>
       <c r="AR50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS50" t="n">
         <v>7</v>
       </c>
-      <c r="AS50" t="n">
+      <c r="AT50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7848,9 +8001,12 @@
         <v>0</v>
       </c>
       <c r="AR51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS51" t="n">
         <v>23</v>
       </c>
-      <c r="AS51" t="n">
+      <c r="AT51" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7996,6 +8152,9 @@
       <c r="AS52" t="n">
         <v>0</v>
       </c>
+      <c r="AT52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8134,9 +8293,12 @@
         <v>0</v>
       </c>
       <c r="AR53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS53" t="n">
         <v>13</v>
       </c>
-      <c r="AS53" t="n">
+      <c r="AT53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -8282,6 +8444,9 @@
       <c r="AS54" t="n">
         <v>0</v>
       </c>
+      <c r="AT54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8420,9 +8585,12 @@
         <v>1</v>
       </c>
       <c r="AR55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS55" t="n">
         <v>24</v>
       </c>
-      <c r="AS55" t="n">
+      <c r="AT55" t="n">
         <v>24</v>
       </c>
     </row>
@@ -8563,9 +8731,12 @@
         <v>0</v>
       </c>
       <c r="AR56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS56" t="n">
         <v>21</v>
       </c>
-      <c r="AS56" t="n">
+      <c r="AT56" t="n">
         <v>21</v>
       </c>
     </row>
@@ -8706,9 +8877,12 @@
         <v>0</v>
       </c>
       <c r="AR57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS57" t="n">
         <v>8</v>
       </c>
-      <c r="AS57" t="n">
+      <c r="AT57" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8849,9 +9023,12 @@
         <v>0</v>
       </c>
       <c r="AR58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS58" t="n">
         <v>12</v>
       </c>
-      <c r="AS58" t="n">
+      <c r="AT58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -8992,9 +9169,12 @@
         <v>0</v>
       </c>
       <c r="AR59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS59" t="n">
         <v>5</v>
       </c>
-      <c r="AS59" t="n">
+      <c r="AT59" t="n">
         <v>5</v>
       </c>
     </row>
@@ -9140,6 +9320,9 @@
       <c r="AS60" t="n">
         <v>0</v>
       </c>
+      <c r="AT60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -9278,9 +9461,12 @@
         <v>0</v>
       </c>
       <c r="AR61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS61" t="n">
         <v>20</v>
       </c>
-      <c r="AS61" t="n">
+      <c r="AT61" t="n">
         <v>20</v>
       </c>
     </row>
@@ -9421,9 +9607,12 @@
         <v>0</v>
       </c>
       <c r="AR62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS62" t="n">
         <v>21</v>
       </c>
-      <c r="AS62" t="n">
+      <c r="AT62" t="n">
         <v>21</v>
       </c>
     </row>
@@ -9564,9 +9753,12 @@
         <v>0</v>
       </c>
       <c r="AR63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS63" t="n">
         <v>8</v>
       </c>
-      <c r="AS63" t="n">
+      <c r="AT63" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9712,6 +9904,9 @@
       <c r="AS64" t="n">
         <v>0</v>
       </c>
+      <c r="AT64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -9850,9 +10045,12 @@
         <v>0</v>
       </c>
       <c r="AR65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS65" t="n">
         <v>11</v>
       </c>
-      <c r="AS65" t="n">
+      <c r="AT65" t="n">
         <v>11</v>
       </c>
     </row>
@@ -9993,9 +10191,12 @@
         <v>0</v>
       </c>
       <c r="AR66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS66" t="n">
         <v>4</v>
       </c>
-      <c r="AS66" t="n">
+      <c r="AT66" t="n">
         <v>4</v>
       </c>
     </row>
@@ -10136,9 +10337,12 @@
         <v>0</v>
       </c>
       <c r="AR67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS67" t="n">
         <v>24</v>
       </c>
-      <c r="AS67" t="n">
+      <c r="AT67" t="n">
         <v>24</v>
       </c>
     </row>
@@ -10279,9 +10483,12 @@
         <v>0</v>
       </c>
       <c r="AR68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS68" t="n">
         <v>14</v>
       </c>
-      <c r="AS68" t="n">
+      <c r="AT68" t="n">
         <v>13</v>
       </c>
     </row>
@@ -10422,9 +10629,12 @@
         <v>0</v>
       </c>
       <c r="AR69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS69" t="n">
         <v>7</v>
       </c>
-      <c r="AS69" t="n">
+      <c r="AT69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10565,9 +10775,12 @@
         <v>0</v>
       </c>
       <c r="AR70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS70" t="n">
         <v>23</v>
       </c>
-      <c r="AS70" t="n">
+      <c r="AT70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -10708,9 +10921,12 @@
         <v>0</v>
       </c>
       <c r="AR71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS71" t="n">
         <v>16</v>
       </c>
-      <c r="AS71" t="n">
+      <c r="AT71" t="n">
         <v>16</v>
       </c>
     </row>
@@ -10851,9 +11067,12 @@
         <v>0</v>
       </c>
       <c r="AR72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS72" t="n">
         <v>15</v>
       </c>
-      <c r="AS72" t="n">
+      <c r="AT72" t="n">
         <v>15</v>
       </c>
     </row>
@@ -10999,6 +11218,9 @@
       <c r="AS73" t="n">
         <v>0</v>
       </c>
+      <c r="AT73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -11142,6 +11364,9 @@
       <c r="AS74" t="n">
         <v>0</v>
       </c>
+      <c r="AT74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -11280,9 +11505,12 @@
         <v>0</v>
       </c>
       <c r="AR75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS75" t="n">
         <v>16</v>
       </c>
-      <c r="AS75" t="n">
+      <c r="AT75" t="n">
         <v>16</v>
       </c>
     </row>
@@ -11423,10 +11651,13 @@
         <v>0</v>
       </c>
       <c r="AR76" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AS76" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AT76" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="77">
@@ -11566,9 +11797,12 @@
         <v>0</v>
       </c>
       <c r="AR77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS77" t="n">
         <v>15</v>
       </c>
-      <c r="AS77" t="n">
+      <c r="AT77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -11709,9 +11943,12 @@
         <v>0</v>
       </c>
       <c r="AR78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS78" t="n">
         <v>21</v>
       </c>
-      <c r="AS78" t="n">
+      <c r="AT78" t="n">
         <v>21</v>
       </c>
     </row>
@@ -11852,9 +12089,12 @@
         <v>0</v>
       </c>
       <c r="AR79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS79" t="n">
         <v>18</v>
       </c>
-      <c r="AS79" t="n">
+      <c r="AT79" t="n">
         <v>18</v>
       </c>
     </row>
@@ -11995,9 +12235,12 @@
         <v>0</v>
       </c>
       <c r="AR80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS80" t="n">
         <v>9</v>
       </c>
-      <c r="AS80" t="n">
+      <c r="AT80" t="n">
         <v>9</v>
       </c>
     </row>
@@ -12138,9 +12381,12 @@
         <v>0</v>
       </c>
       <c r="AR81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS81" t="n">
         <v>3</v>
       </c>
-      <c r="AS81" t="n">
+      <c r="AT81" t="n">
         <v>3</v>
       </c>
     </row>
@@ -12281,10 +12527,13 @@
         <v>0</v>
       </c>
       <c r="AR82" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AS82" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AT82" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="83">
@@ -12424,9 +12673,12 @@
         <v>0</v>
       </c>
       <c r="AR83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS83" t="n">
         <v>16</v>
       </c>
-      <c r="AS83" t="n">
+      <c r="AT83" t="n">
         <v>16</v>
       </c>
     </row>
@@ -12567,9 +12819,12 @@
         <v>0</v>
       </c>
       <c r="AR84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS84" t="n">
         <v>8</v>
       </c>
-      <c r="AS84" t="n">
+      <c r="AT84" t="n">
         <v>8</v>
       </c>
     </row>
@@ -12710,9 +12965,12 @@
         <v>0</v>
       </c>
       <c r="AR85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS85" t="n">
         <v>7</v>
       </c>
-      <c r="AS85" t="n">
+      <c r="AT85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12858,6 +13116,9 @@
       <c r="AS86" t="n">
         <v>0</v>
       </c>
+      <c r="AT86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -12996,9 +13257,12 @@
         <v>0</v>
       </c>
       <c r="AR87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS87" t="n">
         <v>13</v>
       </c>
-      <c r="AS87" t="n">
+      <c r="AT87" t="n">
         <v>13</v>
       </c>
     </row>
@@ -13144,6 +13408,9 @@
       <c r="AS88" t="n">
         <v>0</v>
       </c>
+      <c r="AT88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -13282,9 +13549,12 @@
         <v>0</v>
       </c>
       <c r="AR89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS89" t="n">
         <v>16</v>
       </c>
-      <c r="AS89" t="n">
+      <c r="AT89" t="n">
         <v>16</v>
       </c>
     </row>
@@ -13425,9 +13695,12 @@
         <v>0</v>
       </c>
       <c r="AR90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS90" t="n">
         <v>14</v>
       </c>
-      <c r="AS90" t="n">
+      <c r="AT90" t="n">
         <v>14</v>
       </c>
     </row>
@@ -13568,9 +13841,12 @@
         <v>0</v>
       </c>
       <c r="AR91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS91" t="n">
         <v>42</v>
       </c>
-      <c r="AS91" t="n">
+      <c r="AT91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -13711,9 +13987,12 @@
         <v>0</v>
       </c>
       <c r="AR92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS92" t="n">
         <v>7</v>
       </c>
-      <c r="AS92" t="n">
+      <c r="AT92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13859,6 +14138,9 @@
       <c r="AS93" t="n">
         <v>0</v>
       </c>
+      <c r="AT93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -13997,9 +14279,12 @@
         <v>0</v>
       </c>
       <c r="AR94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS94" t="n">
         <v>13</v>
       </c>
-      <c r="AS94" t="n">
+      <c r="AT94" t="n">
         <v>13</v>
       </c>
     </row>
@@ -14140,9 +14425,12 @@
         <v>0</v>
       </c>
       <c r="AR95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS95" t="n">
         <v>7</v>
       </c>
-      <c r="AS95" t="n">
+      <c r="AT95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14283,9 +14571,12 @@
         <v>0</v>
       </c>
       <c r="AR96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS96" t="n">
         <v>18</v>
       </c>
-      <c r="AS96" t="n">
+      <c r="AT96" t="n">
         <v>18</v>
       </c>
     </row>
@@ -14431,6 +14722,9 @@
       <c r="AS97" t="n">
         <v>0</v>
       </c>
+      <c r="AT97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -14569,9 +14863,12 @@
         <v>1</v>
       </c>
       <c r="AR98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS98" t="n">
         <v>22</v>
       </c>
-      <c r="AS98" t="n">
+      <c r="AT98" t="n">
         <v>22</v>
       </c>
     </row>
@@ -14712,9 +15009,12 @@
         <v>0</v>
       </c>
       <c r="AR99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS99" t="n">
         <v>6</v>
       </c>
-      <c r="AS99" t="n">
+      <c r="AT99" t="n">
         <v>6</v>
       </c>
     </row>
@@ -14860,6 +15160,9 @@
       <c r="AS100" t="n">
         <v>0</v>
       </c>
+      <c r="AT100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -14998,9 +15301,12 @@
         <v>0</v>
       </c>
       <c r="AR101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS101" t="n">
         <v>23</v>
       </c>
-      <c r="AS101" t="n">
+      <c r="AT101" t="n">
         <v>23</v>
       </c>
     </row>
@@ -15141,9 +15447,12 @@
         <v>0</v>
       </c>
       <c r="AR102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS102" t="n">
         <v>22</v>
       </c>
-      <c r="AS102" t="n">
+      <c r="AT102" t="n">
         <v>22</v>
       </c>
     </row>
@@ -15284,9 +15593,12 @@
         <v>1</v>
       </c>
       <c r="AR103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS103" t="n">
         <v>21</v>
       </c>
-      <c r="AS103" t="n">
+      <c r="AT103" t="n">
         <v>21</v>
       </c>
     </row>
@@ -15427,9 +15739,12 @@
         <v>0</v>
       </c>
       <c r="AR104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS104" t="n">
         <v>10</v>
       </c>
-      <c r="AS104" t="n">
+      <c r="AT104" t="n">
         <v>10</v>
       </c>
     </row>
@@ -15570,9 +15885,12 @@
         <v>1</v>
       </c>
       <c r="AR105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS105" t="n">
         <v>14</v>
       </c>
-      <c r="AS105" t="n">
+      <c r="AT105" t="n">
         <v>14</v>
       </c>
     </row>
@@ -15713,9 +16031,12 @@
         <v>0</v>
       </c>
       <c r="AR106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS106" t="n">
         <v>7</v>
       </c>
-      <c r="AS106" t="n">
+      <c r="AT106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15856,9 +16177,12 @@
         <v>0</v>
       </c>
       <c r="AR107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS107" t="n">
         <v>9</v>
       </c>
-      <c r="AS107" t="n">
+      <c r="AT107" t="n">
         <v>9</v>
       </c>
     </row>
@@ -15999,9 +16323,12 @@
         <v>0</v>
       </c>
       <c r="AR108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS108" t="n">
         <v>2</v>
       </c>
-      <c r="AS108" t="n">
+      <c r="AT108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -16142,9 +16469,12 @@
         <v>0</v>
       </c>
       <c r="AR109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS109" t="n">
         <v>2</v>
       </c>
-      <c r="AS109" t="n">
+      <c r="AT109" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3132)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT109"/>
+  <dimension ref="A1:AU109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -474,8 +474,9 @@
     <col width="12" customWidth="1" min="42" max="42"/>
     <col width="12" customWidth="1" min="43" max="43"/>
     <col width="12" customWidth="1" min="44" max="44"/>
-    <col width="13" customWidth="1" min="45" max="45"/>
+    <col width="12" customWidth="1" min="45" max="45"/>
     <col width="13" customWidth="1" min="46" max="46"/>
+    <col width="13" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -699,12 +700,17 @@
           <t>2026-04-05</t>
         </is>
       </c>
-      <c r="AS1" s="2" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="AT1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AT1" s="2" t="inlineStr">
+      <c r="AU1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -850,10 +856,13 @@
         <v>0</v>
       </c>
       <c r="AS2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AT2" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -996,9 +1005,12 @@
         <v>0</v>
       </c>
       <c r="AS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="n">
         <v>9</v>
       </c>
-      <c r="AT3" t="n">
+      <c r="AU3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1142,10 +1154,13 @@
         <v>0</v>
       </c>
       <c r="AS4" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AT4" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -1288,9 +1303,12 @@
         <v>0</v>
       </c>
       <c r="AS5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT5" t="n">
         <v>15</v>
       </c>
-      <c r="AT5" t="n">
+      <c r="AU5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1434,9 +1452,12 @@
         <v>0</v>
       </c>
       <c r="AS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT6" t="n">
         <v>17</v>
       </c>
-      <c r="AT6" t="n">
+      <c r="AU6" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1580,9 +1601,12 @@
         <v>0</v>
       </c>
       <c r="AS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT7" t="n">
         <v>16</v>
       </c>
-      <c r="AT7" t="n">
+      <c r="AU7" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1726,10 +1750,13 @@
         <v>0</v>
       </c>
       <c r="AS8" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AT8" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -1872,10 +1899,13 @@
         <v>0</v>
       </c>
       <c r="AS9" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AT9" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="10">
@@ -2018,10 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AS10" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AT10" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="11">
@@ -2164,10 +2197,13 @@
         <v>0</v>
       </c>
       <c r="AS11" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AT11" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="12">
@@ -2310,10 +2346,13 @@
         <v>0</v>
       </c>
       <c r="AS12" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AT12" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="13">
@@ -2456,10 +2495,13 @@
         <v>0</v>
       </c>
       <c r="AS13" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AT13" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="14">
@@ -2602,10 +2644,13 @@
         <v>0</v>
       </c>
       <c r="AS14" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AT14" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="15">
@@ -2748,9 +2793,12 @@
         <v>0</v>
       </c>
       <c r="AS15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT15" t="n">
         <v>9</v>
       </c>
-      <c r="AT15" t="n">
+      <c r="AU15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2894,10 +2942,13 @@
         <v>0</v>
       </c>
       <c r="AS16" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AT16" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="17">
@@ -3040,10 +3091,13 @@
         <v>0</v>
       </c>
       <c r="AS17" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AT17" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="18">
@@ -3186,10 +3240,13 @@
         <v>0</v>
       </c>
       <c r="AS18" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AT18" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="19">
@@ -3337,6 +3394,9 @@
       <c r="AT19" t="n">
         <v>0</v>
       </c>
+      <c r="AU19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3478,10 +3538,13 @@
         <v>0</v>
       </c>
       <c r="AS20" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AT20" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="21">
@@ -3624,9 +3687,12 @@
         <v>0</v>
       </c>
       <c r="AS21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT21" t="n">
         <v>21</v>
       </c>
-      <c r="AT21" t="n">
+      <c r="AU21" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3775,6 +3841,9 @@
       <c r="AT22" t="n">
         <v>0</v>
       </c>
+      <c r="AU22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3916,10 +3985,13 @@
         <v>0</v>
       </c>
       <c r="AS23" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AT23" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="24">
@@ -4062,9 +4134,12 @@
         <v>0</v>
       </c>
       <c r="AS24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT24" t="n">
         <v>22</v>
       </c>
-      <c r="AT24" t="n">
+      <c r="AU24" t="n">
         <v>22</v>
       </c>
     </row>
@@ -4208,10 +4283,13 @@
         <v>0</v>
       </c>
       <c r="AS25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AT25" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="26">
@@ -4354,10 +4432,13 @@
         <v>0</v>
       </c>
       <c r="AS26" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AT26" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="27">
@@ -4500,9 +4581,12 @@
         <v>0</v>
       </c>
       <c r="AS27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT27" t="n">
         <v>21</v>
       </c>
-      <c r="AT27" t="n">
+      <c r="AU27" t="n">
         <v>19</v>
       </c>
     </row>
@@ -4646,10 +4730,13 @@
         <v>0</v>
       </c>
       <c r="AS28" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AT28" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="29">
@@ -4792,10 +4879,13 @@
         <v>0</v>
       </c>
       <c r="AS29" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AT29" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AU29" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="30">
@@ -4938,10 +5028,13 @@
         <v>0</v>
       </c>
       <c r="AS30" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AT30" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="31">
@@ -5084,10 +5177,13 @@
         <v>0</v>
       </c>
       <c r="AS31" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AT31" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="32">
@@ -5230,10 +5326,13 @@
         <v>0</v>
       </c>
       <c r="AS32" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AT32" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="33">
@@ -5376,9 +5475,12 @@
         <v>0</v>
       </c>
       <c r="AS33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT33" t="n">
         <v>13</v>
       </c>
-      <c r="AT33" t="n">
+      <c r="AU33" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5522,9 +5624,12 @@
         <v>0</v>
       </c>
       <c r="AS34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT34" t="n">
         <v>9</v>
       </c>
-      <c r="AT34" t="n">
+      <c r="AU34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5668,10 +5773,13 @@
         <v>0</v>
       </c>
       <c r="AS35" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AT35" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AU35" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="36">
@@ -5814,9 +5922,12 @@
         <v>0</v>
       </c>
       <c r="AS36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT36" t="n">
         <v>12</v>
       </c>
-      <c r="AT36" t="n">
+      <c r="AU36" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5965,6 +6076,9 @@
       <c r="AT37" t="n">
         <v>0</v>
       </c>
+      <c r="AU37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6106,9 +6220,12 @@
         <v>0</v>
       </c>
       <c r="AS38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT38" t="n">
         <v>2</v>
       </c>
-      <c r="AT38" t="n">
+      <c r="AU38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6252,10 +6369,13 @@
         <v>0</v>
       </c>
       <c r="AS39" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AT39" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AU39" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="40">
@@ -6398,10 +6518,13 @@
         <v>0</v>
       </c>
       <c r="AS40" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AT40" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AU40" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="41">
@@ -6544,10 +6667,13 @@
         <v>0</v>
       </c>
       <c r="AS41" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AT41" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AU41" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="42">
@@ -6690,9 +6816,12 @@
         <v>0</v>
       </c>
       <c r="AS42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT42" t="n">
         <v>21</v>
       </c>
-      <c r="AT42" t="n">
+      <c r="AU42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6836,10 +6965,13 @@
         <v>0</v>
       </c>
       <c r="AS43" t="n">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="AT43" t="n">
-        <v>15</v>
+        <v>57</v>
+      </c>
+      <c r="AU43" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="44">
@@ -6982,10 +7114,13 @@
         <v>1</v>
       </c>
       <c r="AS44" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AT44" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AU44" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="45">
@@ -7128,10 +7263,13 @@
         <v>0</v>
       </c>
       <c r="AS45" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AT45" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AU45" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="46">
@@ -7274,10 +7412,13 @@
         <v>0</v>
       </c>
       <c r="AS46" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AT46" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AU46" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="47">
@@ -7425,6 +7566,9 @@
       <c r="AT47" t="n">
         <v>0</v>
       </c>
+      <c r="AU47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7566,9 +7710,12 @@
         <v>0</v>
       </c>
       <c r="AS48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT48" t="n">
         <v>22</v>
       </c>
-      <c r="AT48" t="n">
+      <c r="AU48" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7712,10 +7859,13 @@
         <v>0</v>
       </c>
       <c r="AS49" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AT49" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AU49" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="50">
@@ -7858,9 +8008,12 @@
         <v>0</v>
       </c>
       <c r="AS50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT50" t="n">
         <v>7</v>
       </c>
-      <c r="AT50" t="n">
+      <c r="AU50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8004,10 +8157,13 @@
         <v>0</v>
       </c>
       <c r="AS51" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AT51" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AU51" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="52">
@@ -8155,6 +8311,9 @@
       <c r="AT52" t="n">
         <v>0</v>
       </c>
+      <c r="AU52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8296,9 +8455,12 @@
         <v>0</v>
       </c>
       <c r="AS53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT53" t="n">
         <v>13</v>
       </c>
-      <c r="AT53" t="n">
+      <c r="AU53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -8447,6 +8609,9 @@
       <c r="AT54" t="n">
         <v>0</v>
       </c>
+      <c r="AU54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8588,10 +8753,13 @@
         <v>0</v>
       </c>
       <c r="AS55" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AT55" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AU55" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="56">
@@ -8734,10 +8902,13 @@
         <v>0</v>
       </c>
       <c r="AS56" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AT56" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AU56" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="57">
@@ -8880,10 +9051,13 @@
         <v>0</v>
       </c>
       <c r="AS57" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AT57" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AU57" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="58">
@@ -9026,9 +9200,12 @@
         <v>0</v>
       </c>
       <c r="AS58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT58" t="n">
         <v>12</v>
       </c>
-      <c r="AT58" t="n">
+      <c r="AU58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -9172,9 +9349,12 @@
         <v>0</v>
       </c>
       <c r="AS59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT59" t="n">
         <v>5</v>
       </c>
-      <c r="AT59" t="n">
+      <c r="AU59" t="n">
         <v>5</v>
       </c>
     </row>
@@ -9323,6 +9503,9 @@
       <c r="AT60" t="n">
         <v>0</v>
       </c>
+      <c r="AU60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -9464,10 +9647,13 @@
         <v>0</v>
       </c>
       <c r="AS61" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AT61" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AU61" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="62">
@@ -9610,10 +9796,13 @@
         <v>0</v>
       </c>
       <c r="AS62" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AT62" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AU62" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="63">
@@ -9756,10 +9945,13 @@
         <v>0</v>
       </c>
       <c r="AS63" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AT63" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AU63" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="64">
@@ -9907,6 +10099,9 @@
       <c r="AT64" t="n">
         <v>0</v>
       </c>
+      <c r="AU64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -10048,9 +10243,12 @@
         <v>0</v>
       </c>
       <c r="AS65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT65" t="n">
         <v>11</v>
       </c>
-      <c r="AT65" t="n">
+      <c r="AU65" t="n">
         <v>11</v>
       </c>
     </row>
@@ -10194,10 +10392,13 @@
         <v>0</v>
       </c>
       <c r="AS66" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AT66" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AU66" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="67">
@@ -10340,10 +10541,13 @@
         <v>0</v>
       </c>
       <c r="AS67" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AT67" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AU67" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="68">
@@ -10486,10 +10690,13 @@
         <v>0</v>
       </c>
       <c r="AS68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT68" t="n">
+        <v>15</v>
+      </c>
+      <c r="AU68" t="n">
         <v>14</v>
-      </c>
-      <c r="AT68" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="69">
@@ -10632,9 +10839,12 @@
         <v>0</v>
       </c>
       <c r="AS69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT69" t="n">
         <v>7</v>
       </c>
-      <c r="AT69" t="n">
+      <c r="AU69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10778,9 +10988,12 @@
         <v>0</v>
       </c>
       <c r="AS70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT70" t="n">
         <v>23</v>
       </c>
-      <c r="AT70" t="n">
+      <c r="AU70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -10924,10 +11137,13 @@
         <v>0</v>
       </c>
       <c r="AS71" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AT71" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AU71" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="72">
@@ -11070,10 +11286,13 @@
         <v>0</v>
       </c>
       <c r="AS72" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AT72" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AU72" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="73">
@@ -11221,6 +11440,9 @@
       <c r="AT73" t="n">
         <v>0</v>
       </c>
+      <c r="AU73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -11367,6 +11589,9 @@
       <c r="AT74" t="n">
         <v>0</v>
       </c>
+      <c r="AU74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -11508,10 +11733,13 @@
         <v>0</v>
       </c>
       <c r="AS75" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AT75" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AU75" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="76">
@@ -11654,10 +11882,13 @@
         <v>1</v>
       </c>
       <c r="AS76" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AT76" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AU76" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="77">
@@ -11800,9 +12031,12 @@
         <v>0</v>
       </c>
       <c r="AS77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT77" t="n">
         <v>15</v>
       </c>
-      <c r="AT77" t="n">
+      <c r="AU77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -11946,10 +12180,13 @@
         <v>0</v>
       </c>
       <c r="AS78" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AT78" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AU78" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="79">
@@ -12092,10 +12329,13 @@
         <v>0</v>
       </c>
       <c r="AS79" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AT79" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AU79" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="80">
@@ -12238,10 +12478,13 @@
         <v>0</v>
       </c>
       <c r="AS80" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AT80" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AU80" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="81">
@@ -12384,10 +12627,13 @@
         <v>0</v>
       </c>
       <c r="AS81" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AT81" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AU81" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="82">
@@ -12530,10 +12776,13 @@
         <v>1</v>
       </c>
       <c r="AS82" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AT82" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AU82" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="83">
@@ -12676,10 +12925,13 @@
         <v>0</v>
       </c>
       <c r="AS83" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AT83" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AU83" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="84">
@@ -12822,10 +13074,13 @@
         <v>0</v>
       </c>
       <c r="AS84" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AT84" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AU84" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="85">
@@ -12968,9 +13223,12 @@
         <v>0</v>
       </c>
       <c r="AS85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT85" t="n">
         <v>7</v>
       </c>
-      <c r="AT85" t="n">
+      <c r="AU85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13119,6 +13377,9 @@
       <c r="AT86" t="n">
         <v>0</v>
       </c>
+      <c r="AU86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -13260,10 +13521,13 @@
         <v>0</v>
       </c>
       <c r="AS87" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AT87" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AU87" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="88">
@@ -13411,6 +13675,9 @@
       <c r="AT88" t="n">
         <v>0</v>
       </c>
+      <c r="AU88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -13552,9 +13819,12 @@
         <v>0</v>
       </c>
       <c r="AS89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT89" t="n">
         <v>16</v>
       </c>
-      <c r="AT89" t="n">
+      <c r="AU89" t="n">
         <v>16</v>
       </c>
     </row>
@@ -13698,9 +13968,12 @@
         <v>0</v>
       </c>
       <c r="AS90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT90" t="n">
         <v>14</v>
       </c>
-      <c r="AT90" t="n">
+      <c r="AU90" t="n">
         <v>14</v>
       </c>
     </row>
@@ -13844,9 +14117,12 @@
         <v>0</v>
       </c>
       <c r="AS91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT91" t="n">
         <v>42</v>
       </c>
-      <c r="AT91" t="n">
+      <c r="AU91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -13990,9 +14266,12 @@
         <v>0</v>
       </c>
       <c r="AS92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT92" t="n">
         <v>7</v>
       </c>
-      <c r="AT92" t="n">
+      <c r="AU92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14141,6 +14420,9 @@
       <c r="AT93" t="n">
         <v>0</v>
       </c>
+      <c r="AU93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -14282,9 +14564,12 @@
         <v>0</v>
       </c>
       <c r="AS94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT94" t="n">
         <v>13</v>
       </c>
-      <c r="AT94" t="n">
+      <c r="AU94" t="n">
         <v>13</v>
       </c>
     </row>
@@ -14428,9 +14713,12 @@
         <v>0</v>
       </c>
       <c r="AS95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT95" t="n">
         <v>7</v>
       </c>
-      <c r="AT95" t="n">
+      <c r="AU95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14574,10 +14862,13 @@
         <v>0</v>
       </c>
       <c r="AS96" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AT96" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AU96" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="97">
@@ -14725,6 +15016,9 @@
       <c r="AT97" t="n">
         <v>0</v>
       </c>
+      <c r="AU97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -14866,10 +15160,13 @@
         <v>0</v>
       </c>
       <c r="AS98" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AT98" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AU98" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="99">
@@ -15012,10 +15309,13 @@
         <v>0</v>
       </c>
       <c r="AS99" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AT99" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AU99" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="100">
@@ -15163,6 +15463,9 @@
       <c r="AT100" t="n">
         <v>0</v>
       </c>
+      <c r="AU100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -15304,9 +15607,12 @@
         <v>0</v>
       </c>
       <c r="AS101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT101" t="n">
         <v>23</v>
       </c>
-      <c r="AT101" t="n">
+      <c r="AU101" t="n">
         <v>23</v>
       </c>
     </row>
@@ -15450,9 +15756,12 @@
         <v>0</v>
       </c>
       <c r="AS102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT102" t="n">
         <v>22</v>
       </c>
-      <c r="AT102" t="n">
+      <c r="AU102" t="n">
         <v>22</v>
       </c>
     </row>
@@ -15596,10 +15905,13 @@
         <v>0</v>
       </c>
       <c r="AS103" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AT103" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AU103" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="104">
@@ -15742,10 +16054,13 @@
         <v>0</v>
       </c>
       <c r="AS104" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AT104" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AU104" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="105">
@@ -15888,10 +16203,13 @@
         <v>0</v>
       </c>
       <c r="AS105" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AT105" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AU105" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="106">
@@ -16034,9 +16352,12 @@
         <v>0</v>
       </c>
       <c r="AS106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT106" t="n">
         <v>7</v>
       </c>
-      <c r="AT106" t="n">
+      <c r="AU106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16180,10 +16501,13 @@
         <v>0</v>
       </c>
       <c r="AS107" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AT107" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AU107" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="108">
@@ -16326,9 +16650,12 @@
         <v>0</v>
       </c>
       <c r="AS108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT108" t="n">
         <v>2</v>
       </c>
-      <c r="AT108" t="n">
+      <c r="AU108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -16472,9 +16799,12 @@
         <v>0</v>
       </c>
       <c r="AS109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT109" t="n">
         <v>2</v>
       </c>
-      <c r="AT109" t="n">
+      <c r="AU109" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3209)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU109"/>
+  <dimension ref="A1:AV109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -475,8 +475,9 @@
     <col width="12" customWidth="1" min="43" max="43"/>
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
-    <col width="13" customWidth="1" min="46" max="46"/>
+    <col width="12" customWidth="1" min="46" max="46"/>
     <col width="13" customWidth="1" min="47" max="47"/>
+    <col width="13" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -705,12 +706,17 @@
           <t>2026-04-06</t>
         </is>
       </c>
-      <c r="AT1" s="2" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="AU1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AU1" s="2" t="inlineStr">
+      <c r="AV1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -859,10 +865,13 @@
         <v>1</v>
       </c>
       <c r="AT2" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AU2" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -1008,9 +1017,12 @@
         <v>0</v>
       </c>
       <c r="AT3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU3" t="n">
         <v>9</v>
       </c>
-      <c r="AU3" t="n">
+      <c r="AV3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1157,10 +1169,13 @@
         <v>1</v>
       </c>
       <c r="AT4" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AU4" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -1306,9 +1321,12 @@
         <v>0</v>
       </c>
       <c r="AT5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU5" t="n">
         <v>15</v>
       </c>
-      <c r="AU5" t="n">
+      <c r="AV5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1455,10 +1473,13 @@
         <v>0</v>
       </c>
       <c r="AT6" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AU6" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -1604,10 +1625,13 @@
         <v>0</v>
       </c>
       <c r="AT7" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AU7" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -1753,10 +1777,13 @@
         <v>1</v>
       </c>
       <c r="AT8" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AU8" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="9">
@@ -1902,10 +1929,13 @@
         <v>1</v>
       </c>
       <c r="AT9" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AU9" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="10">
@@ -2051,10 +2081,13 @@
         <v>1</v>
       </c>
       <c r="AT10" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AU10" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="11">
@@ -2200,10 +2233,13 @@
         <v>1</v>
       </c>
       <c r="AT11" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AU11" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="12">
@@ -2349,10 +2385,13 @@
         <v>1</v>
       </c>
       <c r="AT12" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AU12" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="13">
@@ -2498,10 +2537,13 @@
         <v>1</v>
       </c>
       <c r="AT13" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AU13" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -2647,10 +2689,13 @@
         <v>1</v>
       </c>
       <c r="AT14" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AU14" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="15">
@@ -2796,9 +2841,12 @@
         <v>0</v>
       </c>
       <c r="AT15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU15" t="n">
         <v>9</v>
       </c>
-      <c r="AU15" t="n">
+      <c r="AV15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2945,10 +2993,13 @@
         <v>1</v>
       </c>
       <c r="AT16" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AU16" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="17">
@@ -3094,9 +3145,12 @@
         <v>1</v>
       </c>
       <c r="AT17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU17" t="n">
         <v>17</v>
       </c>
-      <c r="AU17" t="n">
+      <c r="AV17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3243,10 +3297,13 @@
         <v>1</v>
       </c>
       <c r="AT18" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AU18" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="19">
@@ -3397,6 +3454,9 @@
       <c r="AU19" t="n">
         <v>0</v>
       </c>
+      <c r="AV19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3541,9 +3601,12 @@
         <v>1</v>
       </c>
       <c r="AT20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU20" t="n">
         <v>16</v>
       </c>
-      <c r="AU20" t="n">
+      <c r="AV20" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3690,9 +3753,12 @@
         <v>0</v>
       </c>
       <c r="AT21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU21" t="n">
         <v>21</v>
       </c>
-      <c r="AU21" t="n">
+      <c r="AV21" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3844,6 +3910,9 @@
       <c r="AU22" t="n">
         <v>0</v>
       </c>
+      <c r="AV22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3988,10 +4057,13 @@
         <v>1</v>
       </c>
       <c r="AT23" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AU23" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AV23" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="24">
@@ -4137,10 +4209,13 @@
         <v>0</v>
       </c>
       <c r="AT24" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AU24" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="25">
@@ -4286,9 +4361,12 @@
         <v>1</v>
       </c>
       <c r="AT25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU25" t="n">
         <v>9</v>
       </c>
-      <c r="AU25" t="n">
+      <c r="AV25" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4435,9 +4513,12 @@
         <v>1</v>
       </c>
       <c r="AT26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU26" t="n">
         <v>22</v>
       </c>
-      <c r="AU26" t="n">
+      <c r="AV26" t="n">
         <v>22</v>
       </c>
     </row>
@@ -4584,10 +4665,13 @@
         <v>0</v>
       </c>
       <c r="AT27" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AU27" t="n">
-        <v>19</v>
+        <v>22</v>
+      </c>
+      <c r="AV27" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="28">
@@ -4733,10 +4817,13 @@
         <v>1</v>
       </c>
       <c r="AT28" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AU28" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="29">
@@ -4882,9 +4969,12 @@
         <v>1</v>
       </c>
       <c r="AT29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU29" t="n">
         <v>9</v>
       </c>
-      <c r="AU29" t="n">
+      <c r="AV29" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5031,10 +5121,13 @@
         <v>1</v>
       </c>
       <c r="AT30" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AU30" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AV30" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="31">
@@ -5180,10 +5273,13 @@
         <v>1</v>
       </c>
       <c r="AT31" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AU31" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="32">
@@ -5329,9 +5425,12 @@
         <v>1</v>
       </c>
       <c r="AT32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU32" t="n">
         <v>16</v>
       </c>
-      <c r="AU32" t="n">
+      <c r="AV32" t="n">
         <v>16</v>
       </c>
     </row>
@@ -5478,10 +5577,13 @@
         <v>0</v>
       </c>
       <c r="AT33" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AU33" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="34">
@@ -5627,9 +5729,12 @@
         <v>0</v>
       </c>
       <c r="AT34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU34" t="n">
         <v>9</v>
       </c>
-      <c r="AU34" t="n">
+      <c r="AV34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5776,10 +5881,13 @@
         <v>1</v>
       </c>
       <c r="AT35" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AU35" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AV35" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="36">
@@ -5925,9 +6033,12 @@
         <v>0</v>
       </c>
       <c r="AT36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU36" t="n">
         <v>12</v>
       </c>
-      <c r="AU36" t="n">
+      <c r="AV36" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6079,6 +6190,9 @@
       <c r="AU37" t="n">
         <v>0</v>
       </c>
+      <c r="AV37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6223,9 +6337,12 @@
         <v>0</v>
       </c>
       <c r="AT38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU38" t="n">
         <v>2</v>
       </c>
-      <c r="AU38" t="n">
+      <c r="AV38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6372,10 +6489,13 @@
         <v>1</v>
       </c>
       <c r="AT39" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AU39" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AV39" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="40">
@@ -6521,10 +6641,13 @@
         <v>1</v>
       </c>
       <c r="AT40" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AU40" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AV40" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="41">
@@ -6670,10 +6793,13 @@
         <v>1</v>
       </c>
       <c r="AT41" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AU41" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AV41" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="42">
@@ -6819,9 +6945,12 @@
         <v>0</v>
       </c>
       <c r="AT42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU42" t="n">
         <v>21</v>
       </c>
-      <c r="AU42" t="n">
+      <c r="AV42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6968,10 +7097,13 @@
         <v>1</v>
       </c>
       <c r="AT43" t="n">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="AU43" t="n">
-        <v>16</v>
+        <v>58</v>
+      </c>
+      <c r="AV43" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="44">
@@ -7117,10 +7249,13 @@
         <v>1</v>
       </c>
       <c r="AT44" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AU44" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AV44" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="45">
@@ -7266,9 +7401,12 @@
         <v>1</v>
       </c>
       <c r="AT45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU45" t="n">
         <v>23</v>
       </c>
-      <c r="AU45" t="n">
+      <c r="AV45" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7415,10 +7553,13 @@
         <v>1</v>
       </c>
       <c r="AT46" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AU46" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AV46" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="47">
@@ -7569,6 +7710,9 @@
       <c r="AU47" t="n">
         <v>0</v>
       </c>
+      <c r="AV47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7713,10 +7857,13 @@
         <v>0</v>
       </c>
       <c r="AT48" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AU48" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AV48" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="49">
@@ -7862,9 +8009,12 @@
         <v>1</v>
       </c>
       <c r="AT49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU49" t="n">
         <v>18</v>
       </c>
-      <c r="AU49" t="n">
+      <c r="AV49" t="n">
         <v>18</v>
       </c>
     </row>
@@ -8011,9 +8161,12 @@
         <v>0</v>
       </c>
       <c r="AT50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU50" t="n">
         <v>7</v>
       </c>
-      <c r="AU50" t="n">
+      <c r="AV50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8160,10 +8313,13 @@
         <v>1</v>
       </c>
       <c r="AT51" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AU51" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AV51" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="52">
@@ -8314,6 +8470,9 @@
       <c r="AU52" t="n">
         <v>0</v>
       </c>
+      <c r="AV52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8458,9 +8617,12 @@
         <v>0</v>
       </c>
       <c r="AT53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU53" t="n">
         <v>13</v>
       </c>
-      <c r="AU53" t="n">
+      <c r="AV53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -8612,6 +8774,9 @@
       <c r="AU54" t="n">
         <v>0</v>
       </c>
+      <c r="AV54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8756,10 +8921,13 @@
         <v>1</v>
       </c>
       <c r="AT55" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AU55" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="AV55" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="56">
@@ -8905,9 +9073,12 @@
         <v>1</v>
       </c>
       <c r="AT56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU56" t="n">
         <v>22</v>
       </c>
-      <c r="AU56" t="n">
+      <c r="AV56" t="n">
         <v>22</v>
       </c>
     </row>
@@ -9054,9 +9225,12 @@
         <v>1</v>
       </c>
       <c r="AT57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU57" t="n">
         <v>9</v>
       </c>
-      <c r="AU57" t="n">
+      <c r="AV57" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9203,9 +9377,12 @@
         <v>0</v>
       </c>
       <c r="AT58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU58" t="n">
         <v>12</v>
       </c>
-      <c r="AU58" t="n">
+      <c r="AV58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -9352,9 +9529,12 @@
         <v>0</v>
       </c>
       <c r="AT59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU59" t="n">
         <v>5</v>
       </c>
-      <c r="AU59" t="n">
+      <c r="AV59" t="n">
         <v>5</v>
       </c>
     </row>
@@ -9506,6 +9686,9 @@
       <c r="AU60" t="n">
         <v>0</v>
       </c>
+      <c r="AV60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -9650,10 +9833,13 @@
         <v>1</v>
       </c>
       <c r="AT61" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AU61" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AV61" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="62">
@@ -9799,10 +9985,13 @@
         <v>1</v>
       </c>
       <c r="AT62" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AU62" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AV62" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="63">
@@ -9948,9 +10137,12 @@
         <v>1</v>
       </c>
       <c r="AT63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU63" t="n">
         <v>9</v>
       </c>
-      <c r="AU63" t="n">
+      <c r="AV63" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10102,6 +10294,9 @@
       <c r="AU64" t="n">
         <v>0</v>
       </c>
+      <c r="AV64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -10246,10 +10441,13 @@
         <v>0</v>
       </c>
       <c r="AT65" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AU65" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AV65" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="66">
@@ -10395,10 +10593,13 @@
         <v>1</v>
       </c>
       <c r="AT66" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AU66" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AV66" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="67">
@@ -10544,10 +10745,13 @@
         <v>1</v>
       </c>
       <c r="AT67" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AU67" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="AV67" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="68">
@@ -10693,10 +10897,13 @@
         <v>1</v>
       </c>
       <c r="AT68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU68" t="n">
+        <v>16</v>
+      </c>
+      <c r="AV68" t="n">
         <v>15</v>
-      </c>
-      <c r="AU68" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="69">
@@ -10842,9 +11049,12 @@
         <v>0</v>
       </c>
       <c r="AT69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU69" t="n">
         <v>7</v>
       </c>
-      <c r="AU69" t="n">
+      <c r="AV69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10991,9 +11201,12 @@
         <v>0</v>
       </c>
       <c r="AT70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU70" t="n">
         <v>23</v>
       </c>
-      <c r="AU70" t="n">
+      <c r="AV70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -11140,10 +11353,13 @@
         <v>1</v>
       </c>
       <c r="AT71" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AU71" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AV71" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="72">
@@ -11289,10 +11505,13 @@
         <v>1</v>
       </c>
       <c r="AT72" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AU72" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AV72" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="73">
@@ -11443,6 +11662,9 @@
       <c r="AU73" t="n">
         <v>0</v>
       </c>
+      <c r="AV73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -11592,6 +11814,9 @@
       <c r="AU74" t="n">
         <v>0</v>
       </c>
+      <c r="AV74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -11736,10 +11961,13 @@
         <v>1</v>
       </c>
       <c r="AT75" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AU75" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AV75" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="76">
@@ -11885,10 +12113,13 @@
         <v>1</v>
       </c>
       <c r="AT76" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AU76" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AV76" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="77">
@@ -12034,9 +12265,12 @@
         <v>0</v>
       </c>
       <c r="AT77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU77" t="n">
         <v>15</v>
       </c>
-      <c r="AU77" t="n">
+      <c r="AV77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -12183,10 +12417,13 @@
         <v>1</v>
       </c>
       <c r="AT78" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AU78" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AV78" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="79">
@@ -12332,10 +12569,13 @@
         <v>1</v>
       </c>
       <c r="AT79" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AU79" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AV79" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="80">
@@ -12481,9 +12721,12 @@
         <v>1</v>
       </c>
       <c r="AT80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU80" t="n">
         <v>10</v>
       </c>
-      <c r="AU80" t="n">
+      <c r="AV80" t="n">
         <v>10</v>
       </c>
     </row>
@@ -12630,9 +12873,12 @@
         <v>1</v>
       </c>
       <c r="AT81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU81" t="n">
         <v>4</v>
       </c>
-      <c r="AU81" t="n">
+      <c r="AV81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -12779,10 +13025,13 @@
         <v>1</v>
       </c>
       <c r="AT82" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AU82" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AV82" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="83">
@@ -12928,9 +13177,12 @@
         <v>1</v>
       </c>
       <c r="AT83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU83" t="n">
         <v>17</v>
       </c>
-      <c r="AU83" t="n">
+      <c r="AV83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13077,10 +13329,13 @@
         <v>1</v>
       </c>
       <c r="AT84" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AU84" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AV84" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="85">
@@ -13226,9 +13481,12 @@
         <v>0</v>
       </c>
       <c r="AT85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU85" t="n">
         <v>7</v>
       </c>
-      <c r="AU85" t="n">
+      <c r="AV85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13380,6 +13638,9 @@
       <c r="AU86" t="n">
         <v>0</v>
       </c>
+      <c r="AV86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -13524,10 +13785,13 @@
         <v>1</v>
       </c>
       <c r="AT87" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AU87" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AV87" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="88">
@@ -13678,6 +13942,9 @@
       <c r="AU88" t="n">
         <v>0</v>
       </c>
+      <c r="AV88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -13822,9 +14089,12 @@
         <v>0</v>
       </c>
       <c r="AT89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU89" t="n">
         <v>16</v>
       </c>
-      <c r="AU89" t="n">
+      <c r="AV89" t="n">
         <v>16</v>
       </c>
     </row>
@@ -13971,9 +14241,12 @@
         <v>0</v>
       </c>
       <c r="AT90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU90" t="n">
         <v>14</v>
       </c>
-      <c r="AU90" t="n">
+      <c r="AV90" t="n">
         <v>14</v>
       </c>
     </row>
@@ -14120,9 +14393,12 @@
         <v>0</v>
       </c>
       <c r="AT91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU91" t="n">
         <v>42</v>
       </c>
-      <c r="AU91" t="n">
+      <c r="AV91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -14269,9 +14545,12 @@
         <v>0</v>
       </c>
       <c r="AT92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU92" t="n">
         <v>7</v>
       </c>
-      <c r="AU92" t="n">
+      <c r="AV92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14423,6 +14702,9 @@
       <c r="AU93" t="n">
         <v>0</v>
       </c>
+      <c r="AV93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -14567,9 +14849,12 @@
         <v>0</v>
       </c>
       <c r="AT94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU94" t="n">
         <v>13</v>
       </c>
-      <c r="AU94" t="n">
+      <c r="AV94" t="n">
         <v>13</v>
       </c>
     </row>
@@ -14716,9 +15001,12 @@
         <v>0</v>
       </c>
       <c r="AT95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU95" t="n">
         <v>7</v>
       </c>
-      <c r="AU95" t="n">
+      <c r="AV95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14865,9 +15153,12 @@
         <v>1</v>
       </c>
       <c r="AT96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU96" t="n">
         <v>19</v>
       </c>
-      <c r="AU96" t="n">
+      <c r="AV96" t="n">
         <v>19</v>
       </c>
     </row>
@@ -15019,6 +15310,9 @@
       <c r="AU97" t="n">
         <v>0</v>
       </c>
+      <c r="AV97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -15163,10 +15457,13 @@
         <v>1</v>
       </c>
       <c r="AT98" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AU98" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AV98" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="99">
@@ -15312,10 +15609,13 @@
         <v>1</v>
       </c>
       <c r="AT99" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AU99" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="AV99" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="100">
@@ -15466,6 +15766,9 @@
       <c r="AU100" t="n">
         <v>0</v>
       </c>
+      <c r="AV100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -15610,10 +15913,13 @@
         <v>0</v>
       </c>
       <c r="AT101" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AU101" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AV101" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="102">
@@ -15759,9 +16065,12 @@
         <v>0</v>
       </c>
       <c r="AT102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU102" t="n">
         <v>22</v>
       </c>
-      <c r="AU102" t="n">
+      <c r="AV102" t="n">
         <v>22</v>
       </c>
     </row>
@@ -15908,10 +16217,13 @@
         <v>1</v>
       </c>
       <c r="AT103" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AU103" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AV103" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="104">
@@ -16057,9 +16369,12 @@
         <v>1</v>
       </c>
       <c r="AT104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU104" t="n">
         <v>11</v>
       </c>
-      <c r="AU104" t="n">
+      <c r="AV104" t="n">
         <v>11</v>
       </c>
     </row>
@@ -16206,10 +16521,13 @@
         <v>1</v>
       </c>
       <c r="AT105" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AU105" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AV105" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="106">
@@ -16355,9 +16673,12 @@
         <v>0</v>
       </c>
       <c r="AT106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU106" t="n">
         <v>7</v>
       </c>
-      <c r="AU106" t="n">
+      <c r="AV106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16504,10 +16825,13 @@
         <v>1</v>
       </c>
       <c r="AT107" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AU107" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AV107" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="108">
@@ -16653,9 +16977,12 @@
         <v>0</v>
       </c>
       <c r="AT108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU108" t="n">
         <v>2</v>
       </c>
-      <c r="AU108" t="n">
+      <c r="AV108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -16802,10 +17129,13 @@
         <v>0</v>
       </c>
       <c r="AT109" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AU109" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AV109" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3288)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV109"/>
+  <dimension ref="A1:AW109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -476,8 +476,9 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="13" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
+    <col width="13" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -711,12 +712,17 @@
           <t>2026-04-07</t>
         </is>
       </c>
-      <c r="AU1" s="2" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="AV1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AV1" s="2" t="inlineStr">
+      <c r="AW1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -868,9 +874,12 @@
         <v>1</v>
       </c>
       <c r="AU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="n">
         <v>12</v>
       </c>
-      <c r="AV2" t="n">
+      <c r="AW2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1020,9 +1029,12 @@
         <v>0</v>
       </c>
       <c r="AU3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV3" t="n">
         <v>9</v>
       </c>
-      <c r="AV3" t="n">
+      <c r="AW3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1172,10 +1184,13 @@
         <v>1</v>
       </c>
       <c r="AU4" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="AV4" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -1324,9 +1339,12 @@
         <v>0</v>
       </c>
       <c r="AU5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV5" t="n">
         <v>15</v>
       </c>
-      <c r="AV5" t="n">
+      <c r="AW5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1476,9 +1494,12 @@
         <v>1</v>
       </c>
       <c r="AU6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV6" t="n">
         <v>18</v>
       </c>
-      <c r="AV6" t="n">
+      <c r="AW6" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1628,10 +1649,13 @@
         <v>1</v>
       </c>
       <c r="AU7" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AV7" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="8">
@@ -1780,10 +1804,13 @@
         <v>1</v>
       </c>
       <c r="AU8" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AV8" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -1932,9 +1959,12 @@
         <v>1</v>
       </c>
       <c r="AU9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV9" t="n">
         <v>23</v>
       </c>
-      <c r="AV9" t="n">
+      <c r="AW9" t="n">
         <v>23</v>
       </c>
     </row>
@@ -2084,10 +2114,13 @@
         <v>1</v>
       </c>
       <c r="AU10" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="AV10" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="11">
@@ -2236,10 +2269,13 @@
         <v>1</v>
       </c>
       <c r="AU11" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AV11" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="12">
@@ -2388,10 +2424,13 @@
         <v>1</v>
       </c>
       <c r="AU12" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AV12" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="13">
@@ -2540,9 +2579,12 @@
         <v>1</v>
       </c>
       <c r="AU13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV13" t="n">
         <v>14</v>
       </c>
-      <c r="AV13" t="n">
+      <c r="AW13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2692,9 +2734,12 @@
         <v>1</v>
       </c>
       <c r="AU14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV14" t="n">
         <v>24</v>
       </c>
-      <c r="AV14" t="n">
+      <c r="AW14" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2844,9 +2889,12 @@
         <v>0</v>
       </c>
       <c r="AU15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV15" t="n">
         <v>9</v>
       </c>
-      <c r="AV15" t="n">
+      <c r="AW15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2996,9 +3044,12 @@
         <v>1</v>
       </c>
       <c r="AU16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV16" t="n">
         <v>19</v>
       </c>
-      <c r="AV16" t="n">
+      <c r="AW16" t="n">
         <v>19</v>
       </c>
     </row>
@@ -3148,9 +3199,12 @@
         <v>0</v>
       </c>
       <c r="AU17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV17" t="n">
         <v>17</v>
       </c>
-      <c r="AV17" t="n">
+      <c r="AW17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3300,10 +3354,13 @@
         <v>1</v>
       </c>
       <c r="AU18" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AV18" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AW18" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="19">
@@ -3457,6 +3514,9 @@
       <c r="AV19" t="n">
         <v>0</v>
       </c>
+      <c r="AW19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3604,10 +3664,13 @@
         <v>0</v>
       </c>
       <c r="AU20" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AV20" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="21">
@@ -3756,10 +3819,13 @@
         <v>0</v>
       </c>
       <c r="AU21" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AV21" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="22">
@@ -3913,6 +3979,9 @@
       <c r="AV22" t="n">
         <v>0</v>
       </c>
+      <c r="AW22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4060,9 +4129,12 @@
         <v>1</v>
       </c>
       <c r="AU23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV23" t="n">
         <v>16</v>
       </c>
-      <c r="AV23" t="n">
+      <c r="AW23" t="n">
         <v>16</v>
       </c>
     </row>
@@ -4212,9 +4284,12 @@
         <v>1</v>
       </c>
       <c r="AU24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV24" t="n">
         <v>23</v>
       </c>
-      <c r="AV24" t="n">
+      <c r="AW24" t="n">
         <v>23</v>
       </c>
     </row>
@@ -4364,9 +4439,12 @@
         <v>0</v>
       </c>
       <c r="AU25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV25" t="n">
         <v>9</v>
       </c>
-      <c r="AV25" t="n">
+      <c r="AW25" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4516,10 +4594,13 @@
         <v>0</v>
       </c>
       <c r="AU26" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AV26" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="27">
@@ -4668,10 +4749,13 @@
         <v>1</v>
       </c>
       <c r="AU27" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AV27" t="n">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="AW27" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="28">
@@ -4820,10 +4904,13 @@
         <v>1</v>
       </c>
       <c r="AU28" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AV28" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="29">
@@ -4972,10 +5059,13 @@
         <v>0</v>
       </c>
       <c r="AU29" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AV29" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AW29" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="30">
@@ -5124,10 +5214,13 @@
         <v>1</v>
       </c>
       <c r="AU30" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AV30" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AW30" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="31">
@@ -5276,9 +5369,12 @@
         <v>1</v>
       </c>
       <c r="AU31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV31" t="n">
         <v>19</v>
       </c>
-      <c r="AV31" t="n">
+      <c r="AW31" t="n">
         <v>19</v>
       </c>
     </row>
@@ -5428,9 +5524,12 @@
         <v>0</v>
       </c>
       <c r="AU32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV32" t="n">
         <v>16</v>
       </c>
-      <c r="AV32" t="n">
+      <c r="AW32" t="n">
         <v>16</v>
       </c>
     </row>
@@ -5580,10 +5679,13 @@
         <v>1</v>
       </c>
       <c r="AU33" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AV33" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="34">
@@ -5732,9 +5834,12 @@
         <v>0</v>
       </c>
       <c r="AU34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV34" t="n">
         <v>9</v>
       </c>
-      <c r="AV34" t="n">
+      <c r="AW34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5884,10 +5989,13 @@
         <v>1</v>
       </c>
       <c r="AU35" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AV35" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AW35" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="36">
@@ -6036,9 +6144,12 @@
         <v>0</v>
       </c>
       <c r="AU36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV36" t="n">
         <v>12</v>
       </c>
-      <c r="AV36" t="n">
+      <c r="AW36" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6193,6 +6304,9 @@
       <c r="AV37" t="n">
         <v>0</v>
       </c>
+      <c r="AW37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6340,9 +6454,12 @@
         <v>0</v>
       </c>
       <c r="AU38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV38" t="n">
         <v>2</v>
       </c>
-      <c r="AV38" t="n">
+      <c r="AW38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6492,10 +6609,13 @@
         <v>1</v>
       </c>
       <c r="AU39" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AV39" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="AW39" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="40">
@@ -6644,9 +6764,12 @@
         <v>1</v>
       </c>
       <c r="AU40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV40" t="n">
         <v>20</v>
       </c>
-      <c r="AV40" t="n">
+      <c r="AW40" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6796,10 +6919,13 @@
         <v>1</v>
       </c>
       <c r="AU41" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AV41" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="AW41" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="42">
@@ -6948,9 +7074,12 @@
         <v>0</v>
       </c>
       <c r="AU42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV42" t="n">
         <v>21</v>
       </c>
-      <c r="AV42" t="n">
+      <c r="AW42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7100,9 +7229,12 @@
         <v>1</v>
       </c>
       <c r="AU43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV43" t="n">
         <v>58</v>
       </c>
-      <c r="AV43" t="n">
+      <c r="AW43" t="n">
         <v>17</v>
       </c>
     </row>
@@ -7252,9 +7384,12 @@
         <v>1</v>
       </c>
       <c r="AU44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV44" t="n">
         <v>22</v>
       </c>
-      <c r="AV44" t="n">
+      <c r="AW44" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7404,9 +7539,12 @@
         <v>0</v>
       </c>
       <c r="AU45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV45" t="n">
         <v>23</v>
       </c>
-      <c r="AV45" t="n">
+      <c r="AW45" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7556,10 +7694,13 @@
         <v>1</v>
       </c>
       <c r="AU46" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AV46" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AW46" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="47">
@@ -7713,6 +7854,9 @@
       <c r="AV47" t="n">
         <v>0</v>
       </c>
+      <c r="AW47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7860,10 +8004,13 @@
         <v>1</v>
       </c>
       <c r="AU48" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AV48" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AW48" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="49">
@@ -8012,9 +8159,12 @@
         <v>0</v>
       </c>
       <c r="AU49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV49" t="n">
         <v>18</v>
       </c>
-      <c r="AV49" t="n">
+      <c r="AW49" t="n">
         <v>18</v>
       </c>
     </row>
@@ -8164,9 +8314,12 @@
         <v>0</v>
       </c>
       <c r="AU50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV50" t="n">
         <v>7</v>
       </c>
-      <c r="AV50" t="n">
+      <c r="AW50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8316,10 +8469,13 @@
         <v>1</v>
       </c>
       <c r="AU51" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AV51" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="AW51" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="52">
@@ -8473,6 +8629,9 @@
       <c r="AV52" t="n">
         <v>0</v>
       </c>
+      <c r="AW52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8620,9 +8779,12 @@
         <v>0</v>
       </c>
       <c r="AU53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV53" t="n">
         <v>13</v>
       </c>
-      <c r="AV53" t="n">
+      <c r="AW53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -8777,6 +8939,9 @@
       <c r="AV54" t="n">
         <v>0</v>
       </c>
+      <c r="AW54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8924,10 +9089,13 @@
         <v>1</v>
       </c>
       <c r="AU55" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="AV55" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="AW55" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="56">
@@ -9076,10 +9244,13 @@
         <v>0</v>
       </c>
       <c r="AU56" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AV56" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AW56" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="57">
@@ -9228,9 +9399,12 @@
         <v>0</v>
       </c>
       <c r="AU57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV57" t="n">
         <v>9</v>
       </c>
-      <c r="AV57" t="n">
+      <c r="AW57" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9380,9 +9554,12 @@
         <v>0</v>
       </c>
       <c r="AU58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV58" t="n">
         <v>12</v>
       </c>
-      <c r="AV58" t="n">
+      <c r="AW58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -9532,10 +9709,13 @@
         <v>0</v>
       </c>
       <c r="AU59" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AV59" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="AW59" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="60">
@@ -9689,6 +9869,9 @@
       <c r="AV60" t="n">
         <v>0</v>
       </c>
+      <c r="AW60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -9836,10 +10019,13 @@
         <v>1</v>
       </c>
       <c r="AU61" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AV61" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AW61" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="62">
@@ -9988,10 +10174,13 @@
         <v>1</v>
       </c>
       <c r="AU62" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AV62" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AW62" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="63">
@@ -10140,9 +10329,12 @@
         <v>0</v>
       </c>
       <c r="AU63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV63" t="n">
         <v>9</v>
       </c>
-      <c r="AV63" t="n">
+      <c r="AW63" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10297,6 +10489,9 @@
       <c r="AV64" t="n">
         <v>0</v>
       </c>
+      <c r="AW64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -10444,10 +10639,13 @@
         <v>1</v>
       </c>
       <c r="AU65" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AV65" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AW65" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="66">
@@ -10596,9 +10794,12 @@
         <v>1</v>
       </c>
       <c r="AU66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV66" t="n">
         <v>6</v>
       </c>
-      <c r="AV66" t="n">
+      <c r="AW66" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10748,10 +10949,13 @@
         <v>1</v>
       </c>
       <c r="AU67" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="AV67" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="AW67" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="68">
@@ -10900,10 +11104,13 @@
         <v>1</v>
       </c>
       <c r="AU68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV68" t="n">
+        <v>17</v>
+      </c>
+      <c r="AW68" t="n">
         <v>16</v>
-      </c>
-      <c r="AV68" t="n">
-        <v>15</v>
       </c>
     </row>
     <row r="69">
@@ -11052,9 +11259,12 @@
         <v>0</v>
       </c>
       <c r="AU69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV69" t="n">
         <v>7</v>
       </c>
-      <c r="AV69" t="n">
+      <c r="AW69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11204,9 +11414,12 @@
         <v>0</v>
       </c>
       <c r="AU70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV70" t="n">
         <v>23</v>
       </c>
-      <c r="AV70" t="n">
+      <c r="AW70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -11356,10 +11569,13 @@
         <v>1</v>
       </c>
       <c r="AU71" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AV71" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AW71" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="72">
@@ -11508,10 +11724,13 @@
         <v>1</v>
       </c>
       <c r="AU72" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AV72" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AW72" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="73">
@@ -11665,6 +11884,9 @@
       <c r="AV73" t="n">
         <v>0</v>
       </c>
+      <c r="AW73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -11817,6 +12039,9 @@
       <c r="AV74" t="n">
         <v>0</v>
       </c>
+      <c r="AW74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -11964,10 +12189,13 @@
         <v>1</v>
       </c>
       <c r="AU75" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AV75" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AW75" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="76">
@@ -12116,9 +12344,12 @@
         <v>1</v>
       </c>
       <c r="AU76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV76" t="n">
         <v>19</v>
       </c>
-      <c r="AV76" t="n">
+      <c r="AW76" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12268,9 +12499,12 @@
         <v>0</v>
       </c>
       <c r="AU77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV77" t="n">
         <v>15</v>
       </c>
-      <c r="AV77" t="n">
+      <c r="AW77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -12420,10 +12654,13 @@
         <v>1</v>
       </c>
       <c r="AU78" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AV78" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AW78" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="79">
@@ -12572,10 +12809,13 @@
         <v>1</v>
       </c>
       <c r="AU79" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AV79" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AW79" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="80">
@@ -12724,9 +12964,12 @@
         <v>0</v>
       </c>
       <c r="AU80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV80" t="n">
         <v>10</v>
       </c>
-      <c r="AV80" t="n">
+      <c r="AW80" t="n">
         <v>10</v>
       </c>
     </row>
@@ -12876,9 +13119,12 @@
         <v>0</v>
       </c>
       <c r="AU81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV81" t="n">
         <v>4</v>
       </c>
-      <c r="AV81" t="n">
+      <c r="AW81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -13028,10 +13274,13 @@
         <v>1</v>
       </c>
       <c r="AU82" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AV82" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AW82" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="83">
@@ -13180,9 +13429,12 @@
         <v>0</v>
       </c>
       <c r="AU83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV83" t="n">
         <v>17</v>
       </c>
-      <c r="AV83" t="n">
+      <c r="AW83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13332,10 +13584,13 @@
         <v>1</v>
       </c>
       <c r="AU84" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AV84" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AW84" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="85">
@@ -13484,9 +13739,12 @@
         <v>0</v>
       </c>
       <c r="AU85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV85" t="n">
         <v>7</v>
       </c>
-      <c r="AV85" t="n">
+      <c r="AW85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13641,6 +13899,9 @@
       <c r="AV86" t="n">
         <v>0</v>
       </c>
+      <c r="AW86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -13788,10 +14049,13 @@
         <v>1</v>
       </c>
       <c r="AU87" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AV87" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="AW87" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="88">
@@ -13945,6 +14209,9 @@
       <c r="AV88" t="n">
         <v>0</v>
       </c>
+      <c r="AW88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -14092,9 +14359,12 @@
         <v>0</v>
       </c>
       <c r="AU89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV89" t="n">
         <v>16</v>
       </c>
-      <c r="AV89" t="n">
+      <c r="AW89" t="n">
         <v>16</v>
       </c>
     </row>
@@ -14244,9 +14514,12 @@
         <v>0</v>
       </c>
       <c r="AU90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV90" t="n">
         <v>14</v>
       </c>
-      <c r="AV90" t="n">
+      <c r="AW90" t="n">
         <v>14</v>
       </c>
     </row>
@@ -14396,9 +14669,12 @@
         <v>0</v>
       </c>
       <c r="AU91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV91" t="n">
         <v>42</v>
       </c>
-      <c r="AV91" t="n">
+      <c r="AW91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -14548,9 +14824,12 @@
         <v>0</v>
       </c>
       <c r="AU92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV92" t="n">
         <v>7</v>
       </c>
-      <c r="AV92" t="n">
+      <c r="AW92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14705,6 +14984,9 @@
       <c r="AV93" t="n">
         <v>0</v>
       </c>
+      <c r="AW93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -14852,10 +15134,13 @@
         <v>0</v>
       </c>
       <c r="AU94" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AV94" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AW94" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="95">
@@ -15004,9 +15289,12 @@
         <v>0</v>
       </c>
       <c r="AU95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV95" t="n">
         <v>7</v>
       </c>
-      <c r="AV95" t="n">
+      <c r="AW95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15156,10 +15444,13 @@
         <v>0</v>
       </c>
       <c r="AU96" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AV96" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AW96" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="97">
@@ -15313,6 +15604,9 @@
       <c r="AV97" t="n">
         <v>0</v>
       </c>
+      <c r="AW97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -15460,10 +15754,13 @@
         <v>1</v>
       </c>
       <c r="AU98" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AV98" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AW98" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="99">
@@ -15612,9 +15909,12 @@
         <v>1</v>
       </c>
       <c r="AU99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV99" t="n">
         <v>8</v>
       </c>
-      <c r="AV99" t="n">
+      <c r="AW99" t="n">
         <v>8</v>
       </c>
     </row>
@@ -15769,6 +16069,9 @@
       <c r="AV100" t="n">
         <v>0</v>
       </c>
+      <c r="AW100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -15916,9 +16219,12 @@
         <v>1</v>
       </c>
       <c r="AU101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV101" t="n">
         <v>24</v>
       </c>
-      <c r="AV101" t="n">
+      <c r="AW101" t="n">
         <v>24</v>
       </c>
     </row>
@@ -16068,10 +16374,13 @@
         <v>0</v>
       </c>
       <c r="AU102" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AV102" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AW102" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="103">
@@ -16220,10 +16529,13 @@
         <v>1</v>
       </c>
       <c r="AU103" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AV103" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AW103" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="104">
@@ -16372,9 +16684,12 @@
         <v>0</v>
       </c>
       <c r="AU104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV104" t="n">
         <v>11</v>
       </c>
-      <c r="AV104" t="n">
+      <c r="AW104" t="n">
         <v>11</v>
       </c>
     </row>
@@ -16524,10 +16839,13 @@
         <v>1</v>
       </c>
       <c r="AU105" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AV105" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AW105" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="106">
@@ -16676,9 +16994,12 @@
         <v>0</v>
       </c>
       <c r="AU106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV106" t="n">
         <v>7</v>
       </c>
-      <c r="AV106" t="n">
+      <c r="AW106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16828,9 +17149,12 @@
         <v>1</v>
       </c>
       <c r="AU107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV107" t="n">
         <v>11</v>
       </c>
-      <c r="AV107" t="n">
+      <c r="AW107" t="n">
         <v>11</v>
       </c>
     </row>
@@ -16980,9 +17304,12 @@
         <v>0</v>
       </c>
       <c r="AU108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV108" t="n">
         <v>2</v>
       </c>
-      <c r="AV108" t="n">
+      <c r="AW108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -17132,10 +17459,13 @@
         <v>1</v>
       </c>
       <c r="AU109" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AV109" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="AW109" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3386)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW109"/>
+  <dimension ref="A1:AX109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -477,8 +477,9 @@
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
     <col width="12" customWidth="1" min="47" max="47"/>
-    <col width="13" customWidth="1" min="48" max="48"/>
+    <col width="12" customWidth="1" min="48" max="48"/>
     <col width="13" customWidth="1" min="49" max="49"/>
+    <col width="13" customWidth="1" min="50" max="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -717,12 +718,17 @@
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="AV1" s="2" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="AW1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AW1" s="2" t="inlineStr">
+      <c r="AX1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -877,9 +883,12 @@
         <v>0</v>
       </c>
       <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="n">
         <v>12</v>
       </c>
-      <c r="AW2" t="n">
+      <c r="AX2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1032,9 +1041,12 @@
         <v>0</v>
       </c>
       <c r="AV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW3" t="n">
         <v>9</v>
       </c>
-      <c r="AW3" t="n">
+      <c r="AX3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1187,10 +1199,13 @@
         <v>1</v>
       </c>
       <c r="AV4" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="AW4" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="5">
@@ -1342,9 +1357,12 @@
         <v>0</v>
       </c>
       <c r="AV5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW5" t="n">
         <v>15</v>
       </c>
-      <c r="AW5" t="n">
+      <c r="AX5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1497,9 +1515,12 @@
         <v>0</v>
       </c>
       <c r="AV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW6" t="n">
         <v>18</v>
       </c>
-      <c r="AW6" t="n">
+      <c r="AX6" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1652,9 +1673,12 @@
         <v>1</v>
       </c>
       <c r="AV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW7" t="n">
         <v>18</v>
       </c>
-      <c r="AW7" t="n">
+      <c r="AX7" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1807,10 +1831,13 @@
         <v>1</v>
       </c>
       <c r="AV8" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="AW8" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="9">
@@ -1962,10 +1989,13 @@
         <v>0</v>
       </c>
       <c r="AV9" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AW9" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -2117,10 +2147,13 @@
         <v>1</v>
       </c>
       <c r="AV10" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="AW10" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="11">
@@ -2272,10 +2305,13 @@
         <v>1</v>
       </c>
       <c r="AV11" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AW11" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="12">
@@ -2427,10 +2463,13 @@
         <v>1</v>
       </c>
       <c r="AV12" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="AW12" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="13">
@@ -2582,9 +2621,12 @@
         <v>0</v>
       </c>
       <c r="AV13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW13" t="n">
         <v>14</v>
       </c>
-      <c r="AW13" t="n">
+      <c r="AX13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2737,9 +2779,12 @@
         <v>0</v>
       </c>
       <c r="AV14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW14" t="n">
         <v>24</v>
       </c>
-      <c r="AW14" t="n">
+      <c r="AX14" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2892,9 +2937,12 @@
         <v>0</v>
       </c>
       <c r="AV15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW15" t="n">
         <v>9</v>
       </c>
-      <c r="AW15" t="n">
+      <c r="AX15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3047,10 +3095,13 @@
         <v>0</v>
       </c>
       <c r="AV16" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AW16" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AX16" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="17">
@@ -3202,9 +3253,12 @@
         <v>0</v>
       </c>
       <c r="AV17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW17" t="n">
         <v>17</v>
       </c>
-      <c r="AW17" t="n">
+      <c r="AX17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3357,10 +3411,13 @@
         <v>1</v>
       </c>
       <c r="AV18" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AW18" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AX18" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="19">
@@ -3517,6 +3574,9 @@
       <c r="AW19" t="n">
         <v>0</v>
       </c>
+      <c r="AX19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3667,10 +3727,13 @@
         <v>1</v>
       </c>
       <c r="AV20" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AW20" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AX20" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="21">
@@ -3822,10 +3885,13 @@
         <v>1</v>
       </c>
       <c r="AV21" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AW21" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AX21" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="22">
@@ -3982,6 +4048,9 @@
       <c r="AW22" t="n">
         <v>0</v>
       </c>
+      <c r="AX22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4132,10 +4201,13 @@
         <v>0</v>
       </c>
       <c r="AV23" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AW23" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AX23" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="24">
@@ -4287,10 +4359,13 @@
         <v>0</v>
       </c>
       <c r="AV24" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AW24" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AX24" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="25">
@@ -4442,9 +4517,12 @@
         <v>0</v>
       </c>
       <c r="AV25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW25" t="n">
         <v>9</v>
       </c>
-      <c r="AW25" t="n">
+      <c r="AX25" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4597,10 +4675,13 @@
         <v>1</v>
       </c>
       <c r="AV26" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AW26" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AX26" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="27">
@@ -4752,10 +4833,13 @@
         <v>1</v>
       </c>
       <c r="AV27" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AW27" t="n">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="AX27" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="28">
@@ -4907,10 +4991,13 @@
         <v>1</v>
       </c>
       <c r="AV28" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AW28" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AX28" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="29">
@@ -5062,10 +5149,13 @@
         <v>1</v>
       </c>
       <c r="AV29" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AW29" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AX29" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="30">
@@ -5217,10 +5307,13 @@
         <v>1</v>
       </c>
       <c r="AV30" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AW30" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="AX30" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="31">
@@ -5372,9 +5465,12 @@
         <v>0</v>
       </c>
       <c r="AV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
         <v>19</v>
       </c>
-      <c r="AW31" t="n">
+      <c r="AX31" t="n">
         <v>19</v>
       </c>
     </row>
@@ -5527,10 +5623,13 @@
         <v>0</v>
       </c>
       <c r="AV32" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AW32" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AX32" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="33">
@@ -5682,9 +5781,12 @@
         <v>1</v>
       </c>
       <c r="AV33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW33" t="n">
         <v>15</v>
       </c>
-      <c r="AW33" t="n">
+      <c r="AX33" t="n">
         <v>15</v>
       </c>
     </row>
@@ -5837,9 +5939,12 @@
         <v>0</v>
       </c>
       <c r="AV34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW34" t="n">
         <v>9</v>
       </c>
-      <c r="AW34" t="n">
+      <c r="AX34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5992,10 +6097,13 @@
         <v>1</v>
       </c>
       <c r="AV35" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AW35" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AX35" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="36">
@@ -6147,10 +6255,13 @@
         <v>0</v>
       </c>
       <c r="AV36" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AW36" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="AX36" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="37">
@@ -6307,6 +6418,9 @@
       <c r="AW37" t="n">
         <v>0</v>
       </c>
+      <c r="AX37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6457,9 +6571,12 @@
         <v>0</v>
       </c>
       <c r="AV38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW38" t="n">
         <v>2</v>
       </c>
-      <c r="AW38" t="n">
+      <c r="AX38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6612,10 +6729,13 @@
         <v>1</v>
       </c>
       <c r="AV39" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="AW39" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="AX39" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="40">
@@ -6767,10 +6887,13 @@
         <v>0</v>
       </c>
       <c r="AV40" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AW40" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AX40" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="41">
@@ -6922,10 +7045,13 @@
         <v>1</v>
       </c>
       <c r="AV41" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="AW41" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="AX41" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="42">
@@ -7077,9 +7203,12 @@
         <v>0</v>
       </c>
       <c r="AV42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW42" t="n">
         <v>21</v>
       </c>
-      <c r="AW42" t="n">
+      <c r="AX42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7232,10 +7361,13 @@
         <v>0</v>
       </c>
       <c r="AV43" t="n">
-        <v>58</v>
+        <v>1</v>
       </c>
       <c r="AW43" t="n">
-        <v>17</v>
+        <v>59</v>
+      </c>
+      <c r="AX43" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="44">
@@ -7387,9 +7519,12 @@
         <v>0</v>
       </c>
       <c r="AV44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW44" t="n">
         <v>22</v>
       </c>
-      <c r="AW44" t="n">
+      <c r="AX44" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7542,9 +7677,12 @@
         <v>0</v>
       </c>
       <c r="AV45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW45" t="n">
         <v>23</v>
       </c>
-      <c r="AW45" t="n">
+      <c r="AX45" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7697,10 +7835,13 @@
         <v>1</v>
       </c>
       <c r="AV46" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AW46" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AX46" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="47">
@@ -7857,6 +7998,9 @@
       <c r="AW47" t="n">
         <v>0</v>
       </c>
+      <c r="AX47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8007,10 +8151,13 @@
         <v>1</v>
       </c>
       <c r="AV48" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AW48" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AX48" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="49">
@@ -8162,10 +8309,13 @@
         <v>0</v>
       </c>
       <c r="AV49" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AW49" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AX49" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="50">
@@ -8317,9 +8467,12 @@
         <v>0</v>
       </c>
       <c r="AV50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW50" t="n">
         <v>7</v>
       </c>
-      <c r="AW50" t="n">
+      <c r="AX50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8472,9 +8625,12 @@
         <v>1</v>
       </c>
       <c r="AV51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW51" t="n">
         <v>26</v>
       </c>
-      <c r="AW51" t="n">
+      <c r="AX51" t="n">
         <v>26</v>
       </c>
     </row>
@@ -8632,6 +8788,9 @@
       <c r="AW52" t="n">
         <v>0</v>
       </c>
+      <c r="AX52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8782,9 +8941,12 @@
         <v>0</v>
       </c>
       <c r="AV53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW53" t="n">
         <v>13</v>
       </c>
-      <c r="AW53" t="n">
+      <c r="AX53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -8942,6 +9104,9 @@
       <c r="AW54" t="n">
         <v>0</v>
       </c>
+      <c r="AX54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9092,10 +9257,13 @@
         <v>1</v>
       </c>
       <c r="AV55" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="AW55" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="AX55" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="56">
@@ -9247,10 +9415,13 @@
         <v>1</v>
       </c>
       <c r="AV56" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AW56" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AX56" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="57">
@@ -9402,9 +9573,12 @@
         <v>0</v>
       </c>
       <c r="AV57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW57" t="n">
         <v>9</v>
       </c>
-      <c r="AW57" t="n">
+      <c r="AX57" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9557,9 +9731,12 @@
         <v>0</v>
       </c>
       <c r="AV58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW58" t="n">
         <v>12</v>
       </c>
-      <c r="AW58" t="n">
+      <c r="AX58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -9712,9 +9889,12 @@
         <v>1</v>
       </c>
       <c r="AV59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW59" t="n">
         <v>6</v>
       </c>
-      <c r="AW59" t="n">
+      <c r="AX59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -9872,6 +10052,9 @@
       <c r="AW60" t="n">
         <v>0</v>
       </c>
+      <c r="AX60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10022,10 +10205,13 @@
         <v>1</v>
       </c>
       <c r="AV61" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AW61" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AX61" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="62">
@@ -10177,9 +10363,12 @@
         <v>1</v>
       </c>
       <c r="AV62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW62" t="n">
         <v>24</v>
       </c>
-      <c r="AW62" t="n">
+      <c r="AX62" t="n">
         <v>24</v>
       </c>
     </row>
@@ -10332,9 +10521,12 @@
         <v>0</v>
       </c>
       <c r="AV63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW63" t="n">
         <v>9</v>
       </c>
-      <c r="AW63" t="n">
+      <c r="AX63" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10492,6 +10684,9 @@
       <c r="AW64" t="n">
         <v>0</v>
       </c>
+      <c r="AX64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -10642,10 +10837,13 @@
         <v>1</v>
       </c>
       <c r="AV65" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AW65" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="AX65" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="66">
@@ -10797,10 +10995,13 @@
         <v>0</v>
       </c>
       <c r="AV66" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AW66" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="AX66" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="67">
@@ -10952,10 +11153,13 @@
         <v>1</v>
       </c>
       <c r="AV67" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="AW67" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="AX67" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="68">
@@ -11107,10 +11311,13 @@
         <v>1</v>
       </c>
       <c r="AV68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW68" t="n">
+        <v>18</v>
+      </c>
+      <c r="AX68" t="n">
         <v>17</v>
-      </c>
-      <c r="AW68" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="69">
@@ -11262,9 +11469,12 @@
         <v>0</v>
       </c>
       <c r="AV69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW69" t="n">
         <v>7</v>
       </c>
-      <c r="AW69" t="n">
+      <c r="AX69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11417,9 +11627,12 @@
         <v>0</v>
       </c>
       <c r="AV70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW70" t="n">
         <v>23</v>
       </c>
-      <c r="AW70" t="n">
+      <c r="AX70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -11572,10 +11785,13 @@
         <v>1</v>
       </c>
       <c r="AV71" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AW71" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="AX71" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="72">
@@ -11727,10 +11943,13 @@
         <v>1</v>
       </c>
       <c r="AV72" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AW72" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="AX72" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="73">
@@ -11887,6 +12106,9 @@
       <c r="AW73" t="n">
         <v>0</v>
       </c>
+      <c r="AX73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12042,6 +12264,9 @@
       <c r="AW74" t="n">
         <v>0</v>
       </c>
+      <c r="AX74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12192,9 +12417,12 @@
         <v>1</v>
       </c>
       <c r="AV75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW75" t="n">
         <v>19</v>
       </c>
-      <c r="AW75" t="n">
+      <c r="AX75" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12347,9 +12575,12 @@
         <v>0</v>
       </c>
       <c r="AV76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW76" t="n">
         <v>19</v>
       </c>
-      <c r="AW76" t="n">
+      <c r="AX76" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12502,9 +12733,12 @@
         <v>0</v>
       </c>
       <c r="AV77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW77" t="n">
         <v>15</v>
       </c>
-      <c r="AW77" t="n">
+      <c r="AX77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -12657,10 +12891,13 @@
         <v>1</v>
       </c>
       <c r="AV78" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AW78" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AX78" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="79">
@@ -12812,9 +13049,12 @@
         <v>1</v>
       </c>
       <c r="AV79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW79" t="n">
         <v>21</v>
       </c>
-      <c r="AW79" t="n">
+      <c r="AX79" t="n">
         <v>21</v>
       </c>
     </row>
@@ -12967,10 +13207,13 @@
         <v>0</v>
       </c>
       <c r="AV80" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AW80" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="AX80" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="81">
@@ -13122,9 +13365,12 @@
         <v>0</v>
       </c>
       <c r="AV81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW81" t="n">
         <v>4</v>
       </c>
-      <c r="AW81" t="n">
+      <c r="AX81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -13277,9 +13523,12 @@
         <v>1</v>
       </c>
       <c r="AV82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW82" t="n">
         <v>11</v>
       </c>
-      <c r="AW82" t="n">
+      <c r="AX82" t="n">
         <v>11</v>
       </c>
     </row>
@@ -13432,9 +13681,12 @@
         <v>0</v>
       </c>
       <c r="AV83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW83" t="n">
         <v>17</v>
       </c>
-      <c r="AW83" t="n">
+      <c r="AX83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13587,10 +13839,13 @@
         <v>1</v>
       </c>
       <c r="AV84" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AW84" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="AX84" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="85">
@@ -13742,9 +13997,12 @@
         <v>0</v>
       </c>
       <c r="AV85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW85" t="n">
         <v>7</v>
       </c>
-      <c r="AW85" t="n">
+      <c r="AX85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13902,6 +14160,9 @@
       <c r="AW86" t="n">
         <v>0</v>
       </c>
+      <c r="AX86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -14052,10 +14313,13 @@
         <v>1</v>
       </c>
       <c r="AV87" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AW87" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AX87" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="88">
@@ -14212,6 +14476,9 @@
       <c r="AW88" t="n">
         <v>0</v>
       </c>
+      <c r="AX88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -14362,10 +14629,13 @@
         <v>0</v>
       </c>
       <c r="AV89" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AW89" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="AX89" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="90">
@@ -14517,10 +14787,13 @@
         <v>0</v>
       </c>
       <c r="AV90" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AW90" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="AX90" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="91">
@@ -14672,9 +14945,12 @@
         <v>0</v>
       </c>
       <c r="AV91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW91" t="n">
         <v>42</v>
       </c>
-      <c r="AW91" t="n">
+      <c r="AX91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -14827,9 +15103,12 @@
         <v>0</v>
       </c>
       <c r="AV92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW92" t="n">
         <v>7</v>
       </c>
-      <c r="AW92" t="n">
+      <c r="AX92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14987,6 +15266,9 @@
       <c r="AW93" t="n">
         <v>0</v>
       </c>
+      <c r="AX93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -15137,9 +15419,12 @@
         <v>1</v>
       </c>
       <c r="AV94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW94" t="n">
         <v>14</v>
       </c>
-      <c r="AW94" t="n">
+      <c r="AX94" t="n">
         <v>14</v>
       </c>
     </row>
@@ -15292,9 +15577,12 @@
         <v>0</v>
       </c>
       <c r="AV95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW95" t="n">
         <v>7</v>
       </c>
-      <c r="AW95" t="n">
+      <c r="AX95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15447,10 +15735,13 @@
         <v>1</v>
       </c>
       <c r="AV96" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AW96" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="AX96" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="97">
@@ -15607,6 +15898,9 @@
       <c r="AW97" t="n">
         <v>0</v>
       </c>
+      <c r="AX97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -15757,10 +16051,13 @@
         <v>1</v>
       </c>
       <c r="AV98" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AW98" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="AX98" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="99">
@@ -15912,10 +16209,13 @@
         <v>0</v>
       </c>
       <c r="AV99" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AW99" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="AX99" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="100">
@@ -16072,6 +16372,9 @@
       <c r="AW100" t="n">
         <v>0</v>
       </c>
+      <c r="AX100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -16222,10 +16525,13 @@
         <v>0</v>
       </c>
       <c r="AV101" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AW101" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AX101" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="102">
@@ -16377,10 +16683,13 @@
         <v>1</v>
       </c>
       <c r="AV102" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AW102" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AX102" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="103">
@@ -16532,10 +16841,13 @@
         <v>1</v>
       </c>
       <c r="AV103" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AW103" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AX103" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="104">
@@ -16687,9 +16999,12 @@
         <v>0</v>
       </c>
       <c r="AV104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW104" t="n">
         <v>11</v>
       </c>
-      <c r="AW104" t="n">
+      <c r="AX104" t="n">
         <v>11</v>
       </c>
     </row>
@@ -16842,10 +17157,13 @@
         <v>1</v>
       </c>
       <c r="AV105" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AW105" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AX105" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="106">
@@ -16997,9 +17315,12 @@
         <v>0</v>
       </c>
       <c r="AV106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW106" t="n">
         <v>7</v>
       </c>
-      <c r="AW106" t="n">
+      <c r="AX106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17152,9 +17473,12 @@
         <v>0</v>
       </c>
       <c r="AV107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW107" t="n">
         <v>11</v>
       </c>
-      <c r="AW107" t="n">
+      <c r="AX107" t="n">
         <v>11</v>
       </c>
     </row>
@@ -17307,9 +17631,12 @@
         <v>0</v>
       </c>
       <c r="AV108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW108" t="n">
         <v>2</v>
       </c>
-      <c r="AW108" t="n">
+      <c r="AX108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -17462,9 +17789,12 @@
         <v>1</v>
       </c>
       <c r="AV109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW109" t="n">
         <v>4</v>
       </c>
-      <c r="AW109" t="n">
+      <c r="AX109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3452)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX109"/>
+  <dimension ref="A1:AY109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -478,8 +478,9 @@
     <col width="12" customWidth="1" min="46" max="46"/>
     <col width="12" customWidth="1" min="47" max="47"/>
     <col width="12" customWidth="1" min="48" max="48"/>
-    <col width="13" customWidth="1" min="49" max="49"/>
+    <col width="12" customWidth="1" min="49" max="49"/>
     <col width="13" customWidth="1" min="50" max="50"/>
+    <col width="13" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -723,12 +724,17 @@
           <t>2026-04-09</t>
         </is>
       </c>
-      <c r="AW1" s="2" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="AX1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AX1" s="2" t="inlineStr">
+      <c r="AY1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -886,9 +892,12 @@
         <v>0</v>
       </c>
       <c r="AW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX2" t="n">
         <v>12</v>
       </c>
-      <c r="AX2" t="n">
+      <c r="AY2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1044,9 +1053,12 @@
         <v>0</v>
       </c>
       <c r="AW3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX3" t="n">
         <v>9</v>
       </c>
-      <c r="AX3" t="n">
+      <c r="AY3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1202,9 +1214,12 @@
         <v>1</v>
       </c>
       <c r="AW4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX4" t="n">
         <v>28</v>
       </c>
-      <c r="AX4" t="n">
+      <c r="AY4" t="n">
         <v>28</v>
       </c>
     </row>
@@ -1360,9 +1375,12 @@
         <v>0</v>
       </c>
       <c r="AW5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX5" t="n">
         <v>15</v>
       </c>
-      <c r="AX5" t="n">
+      <c r="AY5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1518,9 +1536,12 @@
         <v>0</v>
       </c>
       <c r="AW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX6" t="n">
         <v>18</v>
       </c>
-      <c r="AX6" t="n">
+      <c r="AY6" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1676,9 +1697,12 @@
         <v>0</v>
       </c>
       <c r="AW7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX7" t="n">
         <v>18</v>
       </c>
-      <c r="AX7" t="n">
+      <c r="AY7" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1834,9 +1858,12 @@
         <v>1</v>
       </c>
       <c r="AW8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX8" t="n">
         <v>27</v>
       </c>
-      <c r="AX8" t="n">
+      <c r="AY8" t="n">
         <v>27</v>
       </c>
     </row>
@@ -1992,9 +2019,12 @@
         <v>1</v>
       </c>
       <c r="AW9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX9" t="n">
         <v>24</v>
       </c>
-      <c r="AX9" t="n">
+      <c r="AY9" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2150,9 +2180,12 @@
         <v>1</v>
       </c>
       <c r="AW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX10" t="n">
         <v>28</v>
       </c>
-      <c r="AX10" t="n">
+      <c r="AY10" t="n">
         <v>28</v>
       </c>
     </row>
@@ -2308,9 +2341,12 @@
         <v>1</v>
       </c>
       <c r="AW11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX11" t="n">
         <v>23</v>
       </c>
-      <c r="AX11" t="n">
+      <c r="AY11" t="n">
         <v>23</v>
       </c>
     </row>
@@ -2466,9 +2502,12 @@
         <v>1</v>
       </c>
       <c r="AW12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX12" t="n">
         <v>27</v>
       </c>
-      <c r="AX12" t="n">
+      <c r="AY12" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2624,9 +2663,12 @@
         <v>0</v>
       </c>
       <c r="AW13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX13" t="n">
         <v>14</v>
       </c>
-      <c r="AX13" t="n">
+      <c r="AY13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2782,9 +2824,12 @@
         <v>0</v>
       </c>
       <c r="AW14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX14" t="n">
         <v>24</v>
       </c>
-      <c r="AX14" t="n">
+      <c r="AY14" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2940,9 +2985,12 @@
         <v>0</v>
       </c>
       <c r="AW15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX15" t="n">
         <v>9</v>
       </c>
-      <c r="AX15" t="n">
+      <c r="AY15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3098,9 +3146,12 @@
         <v>1</v>
       </c>
       <c r="AW16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX16" t="n">
         <v>20</v>
       </c>
-      <c r="AX16" t="n">
+      <c r="AY16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3256,9 +3307,12 @@
         <v>0</v>
       </c>
       <c r="AW17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX17" t="n">
         <v>17</v>
       </c>
-      <c r="AX17" t="n">
+      <c r="AY17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3414,9 +3468,12 @@
         <v>1</v>
       </c>
       <c r="AW18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX18" t="n">
         <v>24</v>
       </c>
-      <c r="AX18" t="n">
+      <c r="AY18" t="n">
         <v>24</v>
       </c>
     </row>
@@ -3577,6 +3634,9 @@
       <c r="AX19" t="n">
         <v>0</v>
       </c>
+      <c r="AY19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3730,9 +3790,12 @@
         <v>1</v>
       </c>
       <c r="AW20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX20" t="n">
         <v>18</v>
       </c>
-      <c r="AX20" t="n">
+      <c r="AY20" t="n">
         <v>18</v>
       </c>
     </row>
@@ -3888,9 +3951,12 @@
         <v>1</v>
       </c>
       <c r="AW21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX21" t="n">
         <v>23</v>
       </c>
-      <c r="AX21" t="n">
+      <c r="AY21" t="n">
         <v>23</v>
       </c>
     </row>
@@ -4051,6 +4117,9 @@
       <c r="AX22" t="n">
         <v>0</v>
       </c>
+      <c r="AY22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4204,9 +4273,12 @@
         <v>1</v>
       </c>
       <c r="AW23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX23" t="n">
         <v>17</v>
       </c>
-      <c r="AX23" t="n">
+      <c r="AY23" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4362,9 +4434,12 @@
         <v>1</v>
       </c>
       <c r="AW24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX24" t="n">
         <v>24</v>
       </c>
-      <c r="AX24" t="n">
+      <c r="AY24" t="n">
         <v>24</v>
       </c>
     </row>
@@ -4520,9 +4595,12 @@
         <v>0</v>
       </c>
       <c r="AW25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX25" t="n">
         <v>9</v>
       </c>
-      <c r="AX25" t="n">
+      <c r="AY25" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4678,9 +4756,12 @@
         <v>1</v>
       </c>
       <c r="AW26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX26" t="n">
         <v>24</v>
       </c>
-      <c r="AX26" t="n">
+      <c r="AY26" t="n">
         <v>24</v>
       </c>
     </row>
@@ -4836,9 +4917,12 @@
         <v>1</v>
       </c>
       <c r="AW27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX27" t="n">
         <v>24</v>
       </c>
-      <c r="AX27" t="n">
+      <c r="AY27" t="n">
         <v>22</v>
       </c>
     </row>
@@ -4994,9 +5078,12 @@
         <v>1</v>
       </c>
       <c r="AW28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX28" t="n">
         <v>15</v>
       </c>
-      <c r="AX28" t="n">
+      <c r="AY28" t="n">
         <v>15</v>
       </c>
     </row>
@@ -5152,9 +5239,12 @@
         <v>1</v>
       </c>
       <c r="AW29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX29" t="n">
         <v>11</v>
       </c>
-      <c r="AX29" t="n">
+      <c r="AY29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5310,9 +5400,12 @@
         <v>1</v>
       </c>
       <c r="AW30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX30" t="n">
         <v>22</v>
       </c>
-      <c r="AX30" t="n">
+      <c r="AY30" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5468,9 +5561,12 @@
         <v>0</v>
       </c>
       <c r="AW31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX31" t="n">
         <v>19</v>
       </c>
-      <c r="AX31" t="n">
+      <c r="AY31" t="n">
         <v>19</v>
       </c>
     </row>
@@ -5626,10 +5722,13 @@
         <v>1</v>
       </c>
       <c r="AW32" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AX32" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="AY32" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="33">
@@ -5784,9 +5883,12 @@
         <v>0</v>
       </c>
       <c r="AW33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX33" t="n">
         <v>15</v>
       </c>
-      <c r="AX33" t="n">
+      <c r="AY33" t="n">
         <v>15</v>
       </c>
     </row>
@@ -5942,9 +6044,12 @@
         <v>0</v>
       </c>
       <c r="AW34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX34" t="n">
         <v>9</v>
       </c>
-      <c r="AX34" t="n">
+      <c r="AY34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6100,9 +6205,12 @@
         <v>1</v>
       </c>
       <c r="AW35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX35" t="n">
         <v>21</v>
       </c>
-      <c r="AX35" t="n">
+      <c r="AY35" t="n">
         <v>21</v>
       </c>
     </row>
@@ -6258,9 +6366,12 @@
         <v>1</v>
       </c>
       <c r="AW36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX36" t="n">
         <v>13</v>
       </c>
-      <c r="AX36" t="n">
+      <c r="AY36" t="n">
         <v>13</v>
       </c>
     </row>
@@ -6421,6 +6532,9 @@
       <c r="AX37" t="n">
         <v>0</v>
       </c>
+      <c r="AY37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6574,9 +6688,12 @@
         <v>0</v>
       </c>
       <c r="AW38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX38" t="n">
         <v>2</v>
       </c>
-      <c r="AX38" t="n">
+      <c r="AY38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6732,9 +6849,12 @@
         <v>1</v>
       </c>
       <c r="AW39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX39" t="n">
         <v>27</v>
       </c>
-      <c r="AX39" t="n">
+      <c r="AY39" t="n">
         <v>27</v>
       </c>
     </row>
@@ -6890,9 +7010,12 @@
         <v>1</v>
       </c>
       <c r="AW40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX40" t="n">
         <v>21</v>
       </c>
-      <c r="AX40" t="n">
+      <c r="AY40" t="n">
         <v>21</v>
       </c>
     </row>
@@ -7048,9 +7171,12 @@
         <v>1</v>
       </c>
       <c r="AW41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX41" t="n">
         <v>27</v>
       </c>
-      <c r="AX41" t="n">
+      <c r="AY41" t="n">
         <v>27</v>
       </c>
     </row>
@@ -7206,9 +7332,12 @@
         <v>0</v>
       </c>
       <c r="AW42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX42" t="n">
         <v>21</v>
       </c>
-      <c r="AX42" t="n">
+      <c r="AY42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7364,9 +7493,12 @@
         <v>1</v>
       </c>
       <c r="AW43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX43" t="n">
         <v>59</v>
       </c>
-      <c r="AX43" t="n">
+      <c r="AY43" t="n">
         <v>18</v>
       </c>
     </row>
@@ -7522,9 +7654,12 @@
         <v>0</v>
       </c>
       <c r="AW44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX44" t="n">
         <v>22</v>
       </c>
-      <c r="AX44" t="n">
+      <c r="AY44" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7680,9 +7815,12 @@
         <v>0</v>
       </c>
       <c r="AW45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX45" t="n">
         <v>23</v>
       </c>
-      <c r="AX45" t="n">
+      <c r="AY45" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7838,9 +7976,12 @@
         <v>1</v>
       </c>
       <c r="AW46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX46" t="n">
         <v>23</v>
       </c>
-      <c r="AX46" t="n">
+      <c r="AY46" t="n">
         <v>23</v>
       </c>
     </row>
@@ -8001,6 +8142,9 @@
       <c r="AX47" t="n">
         <v>0</v>
       </c>
+      <c r="AY47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8154,9 +8298,12 @@
         <v>1</v>
       </c>
       <c r="AW48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX48" t="n">
         <v>25</v>
       </c>
-      <c r="AX48" t="n">
+      <c r="AY48" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8312,9 +8459,12 @@
         <v>1</v>
       </c>
       <c r="AW49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX49" t="n">
         <v>19</v>
       </c>
-      <c r="AX49" t="n">
+      <c r="AY49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8470,9 +8620,12 @@
         <v>0</v>
       </c>
       <c r="AW50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX50" t="n">
         <v>7</v>
       </c>
-      <c r="AX50" t="n">
+      <c r="AY50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8628,9 +8781,12 @@
         <v>0</v>
       </c>
       <c r="AW51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX51" t="n">
         <v>26</v>
       </c>
-      <c r="AX51" t="n">
+      <c r="AY51" t="n">
         <v>26</v>
       </c>
     </row>
@@ -8791,6 +8947,9 @@
       <c r="AX52" t="n">
         <v>0</v>
       </c>
+      <c r="AY52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8944,9 +9103,12 @@
         <v>0</v>
       </c>
       <c r="AW53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX53" t="n">
         <v>13</v>
       </c>
-      <c r="AX53" t="n">
+      <c r="AY53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9107,6 +9269,9 @@
       <c r="AX54" t="n">
         <v>0</v>
       </c>
+      <c r="AY54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9260,9 +9425,12 @@
         <v>1</v>
       </c>
       <c r="AW55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX55" t="n">
         <v>28</v>
       </c>
-      <c r="AX55" t="n">
+      <c r="AY55" t="n">
         <v>28</v>
       </c>
     </row>
@@ -9418,10 +9586,13 @@
         <v>1</v>
       </c>
       <c r="AW56" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AX56" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="AY56" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="57">
@@ -9576,9 +9747,12 @@
         <v>0</v>
       </c>
       <c r="AW57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX57" t="n">
         <v>9</v>
       </c>
-      <c r="AX57" t="n">
+      <c r="AY57" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9734,9 +9908,12 @@
         <v>0</v>
       </c>
       <c r="AW58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX58" t="n">
         <v>12</v>
       </c>
-      <c r="AX58" t="n">
+      <c r="AY58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -9892,9 +10069,12 @@
         <v>0</v>
       </c>
       <c r="AW59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX59" t="n">
         <v>6</v>
       </c>
-      <c r="AX59" t="n">
+      <c r="AY59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10055,6 +10235,9 @@
       <c r="AX60" t="n">
         <v>0</v>
       </c>
+      <c r="AY60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10208,9 +10391,12 @@
         <v>1</v>
       </c>
       <c r="AW61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX61" t="n">
         <v>24</v>
       </c>
-      <c r="AX61" t="n">
+      <c r="AY61" t="n">
         <v>24</v>
       </c>
     </row>
@@ -10366,9 +10552,12 @@
         <v>0</v>
       </c>
       <c r="AW62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX62" t="n">
         <v>24</v>
       </c>
-      <c r="AX62" t="n">
+      <c r="AY62" t="n">
         <v>24</v>
       </c>
     </row>
@@ -10524,9 +10713,12 @@
         <v>0</v>
       </c>
       <c r="AW63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX63" t="n">
         <v>9</v>
       </c>
-      <c r="AX63" t="n">
+      <c r="AY63" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10687,6 +10879,9 @@
       <c r="AX64" t="n">
         <v>0</v>
       </c>
+      <c r="AY64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -10840,9 +11035,12 @@
         <v>1</v>
       </c>
       <c r="AW65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX65" t="n">
         <v>14</v>
       </c>
-      <c r="AX65" t="n">
+      <c r="AY65" t="n">
         <v>14</v>
       </c>
     </row>
@@ -10998,9 +11196,12 @@
         <v>1</v>
       </c>
       <c r="AW66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX66" t="n">
         <v>7</v>
       </c>
-      <c r="AX66" t="n">
+      <c r="AY66" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11156,9 +11357,12 @@
         <v>1</v>
       </c>
       <c r="AW67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX67" t="n">
         <v>28</v>
       </c>
-      <c r="AX67" t="n">
+      <c r="AY67" t="n">
         <v>28</v>
       </c>
     </row>
@@ -11314,9 +11518,12 @@
         <v>1</v>
       </c>
       <c r="AW68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX68" t="n">
         <v>18</v>
       </c>
-      <c r="AX68" t="n">
+      <c r="AY68" t="n">
         <v>17</v>
       </c>
     </row>
@@ -11472,9 +11679,12 @@
         <v>0</v>
       </c>
       <c r="AW69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX69" t="n">
         <v>7</v>
       </c>
-      <c r="AX69" t="n">
+      <c r="AY69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11630,9 +11840,12 @@
         <v>0</v>
       </c>
       <c r="AW70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX70" t="n">
         <v>23</v>
       </c>
-      <c r="AX70" t="n">
+      <c r="AY70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -11788,9 +12001,12 @@
         <v>1</v>
       </c>
       <c r="AW71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX71" t="n">
         <v>20</v>
       </c>
-      <c r="AX71" t="n">
+      <c r="AY71" t="n">
         <v>20</v>
       </c>
     </row>
@@ -11946,9 +12162,12 @@
         <v>1</v>
       </c>
       <c r="AW72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX72" t="n">
         <v>19</v>
       </c>
-      <c r="AX72" t="n">
+      <c r="AY72" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12109,6 +12328,9 @@
       <c r="AX73" t="n">
         <v>0</v>
       </c>
+      <c r="AY73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12267,6 +12489,9 @@
       <c r="AX74" t="n">
         <v>0</v>
       </c>
+      <c r="AY74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12420,9 +12645,12 @@
         <v>0</v>
       </c>
       <c r="AW75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX75" t="n">
         <v>19</v>
       </c>
-      <c r="AX75" t="n">
+      <c r="AY75" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12578,9 +12806,12 @@
         <v>0</v>
       </c>
       <c r="AW76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX76" t="n">
         <v>19</v>
       </c>
-      <c r="AX76" t="n">
+      <c r="AY76" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12736,9 +12967,12 @@
         <v>0</v>
       </c>
       <c r="AW77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX77" t="n">
         <v>15</v>
       </c>
-      <c r="AX77" t="n">
+      <c r="AY77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -12894,9 +13128,12 @@
         <v>1</v>
       </c>
       <c r="AW78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX78" t="n">
         <v>25</v>
       </c>
-      <c r="AX78" t="n">
+      <c r="AY78" t="n">
         <v>25</v>
       </c>
     </row>
@@ -13052,9 +13289,12 @@
         <v>0</v>
       </c>
       <c r="AW79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX79" t="n">
         <v>21</v>
       </c>
-      <c r="AX79" t="n">
+      <c r="AY79" t="n">
         <v>21</v>
       </c>
     </row>
@@ -13210,9 +13450,12 @@
         <v>1</v>
       </c>
       <c r="AW80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX80" t="n">
         <v>11</v>
       </c>
-      <c r="AX80" t="n">
+      <c r="AY80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -13368,9 +13611,12 @@
         <v>0</v>
       </c>
       <c r="AW81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX81" t="n">
         <v>4</v>
       </c>
-      <c r="AX81" t="n">
+      <c r="AY81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -13526,9 +13772,12 @@
         <v>0</v>
       </c>
       <c r="AW82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX82" t="n">
         <v>11</v>
       </c>
-      <c r="AX82" t="n">
+      <c r="AY82" t="n">
         <v>11</v>
       </c>
     </row>
@@ -13684,9 +13933,12 @@
         <v>0</v>
       </c>
       <c r="AW83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX83" t="n">
         <v>17</v>
       </c>
-      <c r="AX83" t="n">
+      <c r="AY83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13842,9 +14094,12 @@
         <v>1</v>
       </c>
       <c r="AW84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX84" t="n">
         <v>12</v>
       </c>
-      <c r="AX84" t="n">
+      <c r="AY84" t="n">
         <v>12</v>
       </c>
     </row>
@@ -14000,9 +14255,12 @@
         <v>0</v>
       </c>
       <c r="AW85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX85" t="n">
         <v>7</v>
       </c>
-      <c r="AX85" t="n">
+      <c r="AY85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14163,6 +14421,9 @@
       <c r="AX86" t="n">
         <v>0</v>
       </c>
+      <c r="AY86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -14316,9 +14577,12 @@
         <v>1</v>
       </c>
       <c r="AW87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX87" t="n">
         <v>17</v>
       </c>
-      <c r="AX87" t="n">
+      <c r="AY87" t="n">
         <v>17</v>
       </c>
     </row>
@@ -14479,6 +14743,9 @@
       <c r="AX88" t="n">
         <v>0</v>
       </c>
+      <c r="AY88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -14632,9 +14899,12 @@
         <v>1</v>
       </c>
       <c r="AW89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX89" t="n">
         <v>17</v>
       </c>
-      <c r="AX89" t="n">
+      <c r="AY89" t="n">
         <v>17</v>
       </c>
     </row>
@@ -14790,9 +15060,12 @@
         <v>1</v>
       </c>
       <c r="AW90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX90" t="n">
         <v>15</v>
       </c>
-      <c r="AX90" t="n">
+      <c r="AY90" t="n">
         <v>15</v>
       </c>
     </row>
@@ -14948,9 +15221,12 @@
         <v>0</v>
       </c>
       <c r="AW91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX91" t="n">
         <v>42</v>
       </c>
-      <c r="AX91" t="n">
+      <c r="AY91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -15106,9 +15382,12 @@
         <v>0</v>
       </c>
       <c r="AW92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX92" t="n">
         <v>7</v>
       </c>
-      <c r="AX92" t="n">
+      <c r="AY92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15269,6 +15548,9 @@
       <c r="AX93" t="n">
         <v>0</v>
       </c>
+      <c r="AY93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -15422,9 +15704,12 @@
         <v>0</v>
       </c>
       <c r="AW94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX94" t="n">
         <v>14</v>
       </c>
-      <c r="AX94" t="n">
+      <c r="AY94" t="n">
         <v>14</v>
       </c>
     </row>
@@ -15580,9 +15865,12 @@
         <v>0</v>
       </c>
       <c r="AW95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX95" t="n">
         <v>7</v>
       </c>
-      <c r="AX95" t="n">
+      <c r="AY95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15738,9 +16026,12 @@
         <v>1</v>
       </c>
       <c r="AW96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX96" t="n">
         <v>21</v>
       </c>
-      <c r="AX96" t="n">
+      <c r="AY96" t="n">
         <v>21</v>
       </c>
     </row>
@@ -15901,6 +16192,9 @@
       <c r="AX97" t="n">
         <v>0</v>
       </c>
+      <c r="AY97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -16054,9 +16348,12 @@
         <v>1</v>
       </c>
       <c r="AW98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX98" t="n">
         <v>26</v>
       </c>
-      <c r="AX98" t="n">
+      <c r="AY98" t="n">
         <v>26</v>
       </c>
     </row>
@@ -16212,10 +16509,13 @@
         <v>1</v>
       </c>
       <c r="AW99" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AX99" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AY99" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="100">
@@ -16375,6 +16675,9 @@
       <c r="AX100" t="n">
         <v>0</v>
       </c>
+      <c r="AY100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -16528,9 +16831,12 @@
         <v>1</v>
       </c>
       <c r="AW101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX101" t="n">
         <v>25</v>
       </c>
-      <c r="AX101" t="n">
+      <c r="AY101" t="n">
         <v>25</v>
       </c>
     </row>
@@ -16686,9 +16992,12 @@
         <v>1</v>
       </c>
       <c r="AW102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX102" t="n">
         <v>24</v>
       </c>
-      <c r="AX102" t="n">
+      <c r="AY102" t="n">
         <v>24</v>
       </c>
     </row>
@@ -16844,9 +17153,12 @@
         <v>1</v>
       </c>
       <c r="AW103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX103" t="n">
         <v>25</v>
       </c>
-      <c r="AX103" t="n">
+      <c r="AY103" t="n">
         <v>25</v>
       </c>
     </row>
@@ -17002,9 +17314,12 @@
         <v>0</v>
       </c>
       <c r="AW104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX104" t="n">
         <v>11</v>
       </c>
-      <c r="AX104" t="n">
+      <c r="AY104" t="n">
         <v>11</v>
       </c>
     </row>
@@ -17160,9 +17475,12 @@
         <v>1</v>
       </c>
       <c r="AW105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX105" t="n">
         <v>18</v>
       </c>
-      <c r="AX105" t="n">
+      <c r="AY105" t="n">
         <v>18</v>
       </c>
     </row>
@@ -17318,9 +17636,12 @@
         <v>0</v>
       </c>
       <c r="AW106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX106" t="n">
         <v>7</v>
       </c>
-      <c r="AX106" t="n">
+      <c r="AY106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17476,9 +17797,12 @@
         <v>0</v>
       </c>
       <c r="AW107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX107" t="n">
         <v>11</v>
       </c>
-      <c r="AX107" t="n">
+      <c r="AY107" t="n">
         <v>11</v>
       </c>
     </row>
@@ -17634,9 +17958,12 @@
         <v>0</v>
       </c>
       <c r="AW108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX108" t="n">
         <v>2</v>
       </c>
-      <c r="AX108" t="n">
+      <c r="AY108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -17792,9 +18119,12 @@
         <v>0</v>
       </c>
       <c r="AW109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX109" t="n">
         <v>4</v>
       </c>
-      <c r="AX109" t="n">
+      <c r="AY109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3491)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY109"/>
+  <dimension ref="A1:AZ109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -479,8 +479,9 @@
     <col width="12" customWidth="1" min="47" max="47"/>
     <col width="12" customWidth="1" min="48" max="48"/>
     <col width="12" customWidth="1" min="49" max="49"/>
-    <col width="13" customWidth="1" min="50" max="50"/>
+    <col width="12" customWidth="1" min="50" max="50"/>
     <col width="13" customWidth="1" min="51" max="51"/>
+    <col width="13" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -729,12 +730,17 @@
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="AX1" s="2" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="AY1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AY1" s="2" t="inlineStr">
+      <c r="AZ1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -895,9 +901,12 @@
         <v>0</v>
       </c>
       <c r="AX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY2" t="n">
         <v>12</v>
       </c>
-      <c r="AY2" t="n">
+      <c r="AZ2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1056,9 +1065,12 @@
         <v>0</v>
       </c>
       <c r="AX3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY3" t="n">
         <v>9</v>
       </c>
-      <c r="AY3" t="n">
+      <c r="AZ3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1217,9 +1229,12 @@
         <v>0</v>
       </c>
       <c r="AX4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY4" t="n">
         <v>28</v>
       </c>
-      <c r="AY4" t="n">
+      <c r="AZ4" t="n">
         <v>28</v>
       </c>
     </row>
@@ -1378,9 +1393,12 @@
         <v>0</v>
       </c>
       <c r="AX5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY5" t="n">
         <v>15</v>
       </c>
-      <c r="AY5" t="n">
+      <c r="AZ5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1539,9 +1557,12 @@
         <v>0</v>
       </c>
       <c r="AX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY6" t="n">
         <v>18</v>
       </c>
-      <c r="AY6" t="n">
+      <c r="AZ6" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1700,9 +1721,12 @@
         <v>0</v>
       </c>
       <c r="AX7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY7" t="n">
         <v>18</v>
       </c>
-      <c r="AY7" t="n">
+      <c r="AZ7" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1861,9 +1885,12 @@
         <v>0</v>
       </c>
       <c r="AX8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY8" t="n">
         <v>27</v>
       </c>
-      <c r="AY8" t="n">
+      <c r="AZ8" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2022,9 +2049,12 @@
         <v>0</v>
       </c>
       <c r="AX9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY9" t="n">
         <v>24</v>
       </c>
-      <c r="AY9" t="n">
+      <c r="AZ9" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2183,9 +2213,12 @@
         <v>0</v>
       </c>
       <c r="AX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY10" t="n">
         <v>28</v>
       </c>
-      <c r="AY10" t="n">
+      <c r="AZ10" t="n">
         <v>28</v>
       </c>
     </row>
@@ -2344,9 +2377,12 @@
         <v>0</v>
       </c>
       <c r="AX11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY11" t="n">
         <v>23</v>
       </c>
-      <c r="AY11" t="n">
+      <c r="AZ11" t="n">
         <v>23</v>
       </c>
     </row>
@@ -2505,9 +2541,12 @@
         <v>0</v>
       </c>
       <c r="AX12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY12" t="n">
         <v>27</v>
       </c>
-      <c r="AY12" t="n">
+      <c r="AZ12" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2666,9 +2705,12 @@
         <v>0</v>
       </c>
       <c r="AX13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY13" t="n">
         <v>14</v>
       </c>
-      <c r="AY13" t="n">
+      <c r="AZ13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2827,9 +2869,12 @@
         <v>0</v>
       </c>
       <c r="AX14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY14" t="n">
         <v>24</v>
       </c>
-      <c r="AY14" t="n">
+      <c r="AZ14" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2988,9 +3033,12 @@
         <v>0</v>
       </c>
       <c r="AX15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY15" t="n">
         <v>9</v>
       </c>
-      <c r="AY15" t="n">
+      <c r="AZ15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3149,9 +3197,12 @@
         <v>0</v>
       </c>
       <c r="AX16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY16" t="n">
         <v>20</v>
       </c>
-      <c r="AY16" t="n">
+      <c r="AZ16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3310,9 +3361,12 @@
         <v>0</v>
       </c>
       <c r="AX17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY17" t="n">
         <v>17</v>
       </c>
-      <c r="AY17" t="n">
+      <c r="AZ17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3471,9 +3525,12 @@
         <v>0</v>
       </c>
       <c r="AX18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY18" t="n">
         <v>24</v>
       </c>
-      <c r="AY18" t="n">
+      <c r="AZ18" t="n">
         <v>24</v>
       </c>
     </row>
@@ -3637,6 +3694,9 @@
       <c r="AY19" t="n">
         <v>0</v>
       </c>
+      <c r="AZ19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3793,9 +3853,12 @@
         <v>0</v>
       </c>
       <c r="AX20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY20" t="n">
         <v>18</v>
       </c>
-      <c r="AY20" t="n">
+      <c r="AZ20" t="n">
         <v>18</v>
       </c>
     </row>
@@ -3954,9 +4017,12 @@
         <v>0</v>
       </c>
       <c r="AX21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY21" t="n">
         <v>23</v>
       </c>
-      <c r="AY21" t="n">
+      <c r="AZ21" t="n">
         <v>23</v>
       </c>
     </row>
@@ -4120,6 +4186,9 @@
       <c r="AY22" t="n">
         <v>0</v>
       </c>
+      <c r="AZ22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4276,9 +4345,12 @@
         <v>0</v>
       </c>
       <c r="AX23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY23" t="n">
         <v>17</v>
       </c>
-      <c r="AY23" t="n">
+      <c r="AZ23" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4437,9 +4509,12 @@
         <v>0</v>
       </c>
       <c r="AX24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY24" t="n">
         <v>24</v>
       </c>
-      <c r="AY24" t="n">
+      <c r="AZ24" t="n">
         <v>24</v>
       </c>
     </row>
@@ -4598,9 +4673,12 @@
         <v>0</v>
       </c>
       <c r="AX25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY25" t="n">
         <v>9</v>
       </c>
-      <c r="AY25" t="n">
+      <c r="AZ25" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4759,9 +4837,12 @@
         <v>0</v>
       </c>
       <c r="AX26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY26" t="n">
         <v>24</v>
       </c>
-      <c r="AY26" t="n">
+      <c r="AZ26" t="n">
         <v>24</v>
       </c>
     </row>
@@ -4920,9 +5001,12 @@
         <v>0</v>
       </c>
       <c r="AX27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY27" t="n">
         <v>24</v>
       </c>
-      <c r="AY27" t="n">
+      <c r="AZ27" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5081,9 +5165,12 @@
         <v>0</v>
       </c>
       <c r="AX28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY28" t="n">
         <v>15</v>
       </c>
-      <c r="AY28" t="n">
+      <c r="AZ28" t="n">
         <v>15</v>
       </c>
     </row>
@@ -5242,9 +5329,12 @@
         <v>0</v>
       </c>
       <c r="AX29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY29" t="n">
         <v>11</v>
       </c>
-      <c r="AY29" t="n">
+      <c r="AZ29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5403,9 +5493,12 @@
         <v>0</v>
       </c>
       <c r="AX30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY30" t="n">
         <v>22</v>
       </c>
-      <c r="AY30" t="n">
+      <c r="AZ30" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5564,9 +5657,12 @@
         <v>0</v>
       </c>
       <c r="AX31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY31" t="n">
         <v>19</v>
       </c>
-      <c r="AY31" t="n">
+      <c r="AZ31" t="n">
         <v>19</v>
       </c>
     </row>
@@ -5725,9 +5821,12 @@
         <v>1</v>
       </c>
       <c r="AX32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY32" t="n">
         <v>18</v>
       </c>
-      <c r="AY32" t="n">
+      <c r="AZ32" t="n">
         <v>18</v>
       </c>
     </row>
@@ -5886,9 +5985,12 @@
         <v>0</v>
       </c>
       <c r="AX33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY33" t="n">
         <v>15</v>
       </c>
-      <c r="AY33" t="n">
+      <c r="AZ33" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6047,9 +6149,12 @@
         <v>0</v>
       </c>
       <c r="AX34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY34" t="n">
         <v>9</v>
       </c>
-      <c r="AY34" t="n">
+      <c r="AZ34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6208,9 +6313,12 @@
         <v>0</v>
       </c>
       <c r="AX35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY35" t="n">
         <v>21</v>
       </c>
-      <c r="AY35" t="n">
+      <c r="AZ35" t="n">
         <v>21</v>
       </c>
     </row>
@@ -6369,9 +6477,12 @@
         <v>0</v>
       </c>
       <c r="AX36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY36" t="n">
         <v>13</v>
       </c>
-      <c r="AY36" t="n">
+      <c r="AZ36" t="n">
         <v>13</v>
       </c>
     </row>
@@ -6535,6 +6646,9 @@
       <c r="AY37" t="n">
         <v>0</v>
       </c>
+      <c r="AZ37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6691,9 +6805,12 @@
         <v>0</v>
       </c>
       <c r="AX38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY38" t="n">
         <v>2</v>
       </c>
-      <c r="AY38" t="n">
+      <c r="AZ38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6852,9 +6969,12 @@
         <v>0</v>
       </c>
       <c r="AX39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY39" t="n">
         <v>27</v>
       </c>
-      <c r="AY39" t="n">
+      <c r="AZ39" t="n">
         <v>27</v>
       </c>
     </row>
@@ -7013,9 +7133,12 @@
         <v>0</v>
       </c>
       <c r="AX40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY40" t="n">
         <v>21</v>
       </c>
-      <c r="AY40" t="n">
+      <c r="AZ40" t="n">
         <v>21</v>
       </c>
     </row>
@@ -7174,9 +7297,12 @@
         <v>0</v>
       </c>
       <c r="AX41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY41" t="n">
         <v>27</v>
       </c>
-      <c r="AY41" t="n">
+      <c r="AZ41" t="n">
         <v>27</v>
       </c>
     </row>
@@ -7335,9 +7461,12 @@
         <v>0</v>
       </c>
       <c r="AX42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY42" t="n">
         <v>21</v>
       </c>
-      <c r="AY42" t="n">
+      <c r="AZ42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7496,9 +7625,12 @@
         <v>0</v>
       </c>
       <c r="AX43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY43" t="n">
         <v>59</v>
       </c>
-      <c r="AY43" t="n">
+      <c r="AZ43" t="n">
         <v>18</v>
       </c>
     </row>
@@ -7657,9 +7789,12 @@
         <v>0</v>
       </c>
       <c r="AX44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY44" t="n">
         <v>22</v>
       </c>
-      <c r="AY44" t="n">
+      <c r="AZ44" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7818,9 +7953,12 @@
         <v>0</v>
       </c>
       <c r="AX45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY45" t="n">
         <v>23</v>
       </c>
-      <c r="AY45" t="n">
+      <c r="AZ45" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7979,9 +8117,12 @@
         <v>0</v>
       </c>
       <c r="AX46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY46" t="n">
         <v>23</v>
       </c>
-      <c r="AY46" t="n">
+      <c r="AZ46" t="n">
         <v>23</v>
       </c>
     </row>
@@ -8145,6 +8286,9 @@
       <c r="AY47" t="n">
         <v>0</v>
       </c>
+      <c r="AZ47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8301,9 +8445,12 @@
         <v>0</v>
       </c>
       <c r="AX48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY48" t="n">
         <v>25</v>
       </c>
-      <c r="AY48" t="n">
+      <c r="AZ48" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8462,9 +8609,12 @@
         <v>0</v>
       </c>
       <c r="AX49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY49" t="n">
         <v>19</v>
       </c>
-      <c r="AY49" t="n">
+      <c r="AZ49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8623,9 +8773,12 @@
         <v>0</v>
       </c>
       <c r="AX50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY50" t="n">
         <v>7</v>
       </c>
-      <c r="AY50" t="n">
+      <c r="AZ50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8784,9 +8937,12 @@
         <v>0</v>
       </c>
       <c r="AX51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY51" t="n">
         <v>26</v>
       </c>
-      <c r="AY51" t="n">
+      <c r="AZ51" t="n">
         <v>26</v>
       </c>
     </row>
@@ -8950,6 +9106,9 @@
       <c r="AY52" t="n">
         <v>0</v>
       </c>
+      <c r="AZ52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9106,9 +9265,12 @@
         <v>0</v>
       </c>
       <c r="AX53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY53" t="n">
         <v>13</v>
       </c>
-      <c r="AY53" t="n">
+      <c r="AZ53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9272,6 +9434,9 @@
       <c r="AY54" t="n">
         <v>0</v>
       </c>
+      <c r="AZ54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9428,9 +9593,12 @@
         <v>0</v>
       </c>
       <c r="AX55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY55" t="n">
         <v>28</v>
       </c>
-      <c r="AY55" t="n">
+      <c r="AZ55" t="n">
         <v>28</v>
       </c>
     </row>
@@ -9589,9 +9757,12 @@
         <v>1</v>
       </c>
       <c r="AX56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY56" t="n">
         <v>25</v>
       </c>
-      <c r="AY56" t="n">
+      <c r="AZ56" t="n">
         <v>25</v>
       </c>
     </row>
@@ -9750,9 +9921,12 @@
         <v>0</v>
       </c>
       <c r="AX57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY57" t="n">
         <v>9</v>
       </c>
-      <c r="AY57" t="n">
+      <c r="AZ57" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9911,9 +10085,12 @@
         <v>0</v>
       </c>
       <c r="AX58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY58" t="n">
         <v>12</v>
       </c>
-      <c r="AY58" t="n">
+      <c r="AZ58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -10072,9 +10249,12 @@
         <v>0</v>
       </c>
       <c r="AX59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY59" t="n">
         <v>6</v>
       </c>
-      <c r="AY59" t="n">
+      <c r="AZ59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10238,6 +10418,9 @@
       <c r="AY60" t="n">
         <v>0</v>
       </c>
+      <c r="AZ60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10394,9 +10577,12 @@
         <v>0</v>
       </c>
       <c r="AX61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY61" t="n">
         <v>24</v>
       </c>
-      <c r="AY61" t="n">
+      <c r="AZ61" t="n">
         <v>24</v>
       </c>
     </row>
@@ -10555,9 +10741,12 @@
         <v>0</v>
       </c>
       <c r="AX62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY62" t="n">
         <v>24</v>
       </c>
-      <c r="AY62" t="n">
+      <c r="AZ62" t="n">
         <v>24</v>
       </c>
     </row>
@@ -10716,9 +10905,12 @@
         <v>0</v>
       </c>
       <c r="AX63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY63" t="n">
         <v>9</v>
       </c>
-      <c r="AY63" t="n">
+      <c r="AZ63" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10882,6 +11074,9 @@
       <c r="AY64" t="n">
         <v>0</v>
       </c>
+      <c r="AZ64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -11038,9 +11233,12 @@
         <v>0</v>
       </c>
       <c r="AX65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY65" t="n">
         <v>14</v>
       </c>
-      <c r="AY65" t="n">
+      <c r="AZ65" t="n">
         <v>14</v>
       </c>
     </row>
@@ -11199,9 +11397,12 @@
         <v>0</v>
       </c>
       <c r="AX66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY66" t="n">
         <v>7</v>
       </c>
-      <c r="AY66" t="n">
+      <c r="AZ66" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11360,9 +11561,12 @@
         <v>0</v>
       </c>
       <c r="AX67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY67" t="n">
         <v>28</v>
       </c>
-      <c r="AY67" t="n">
+      <c r="AZ67" t="n">
         <v>28</v>
       </c>
     </row>
@@ -11521,9 +11725,12 @@
         <v>0</v>
       </c>
       <c r="AX68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY68" t="n">
         <v>18</v>
       </c>
-      <c r="AY68" t="n">
+      <c r="AZ68" t="n">
         <v>17</v>
       </c>
     </row>
@@ -11682,9 +11889,12 @@
         <v>0</v>
       </c>
       <c r="AX69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY69" t="n">
         <v>7</v>
       </c>
-      <c r="AY69" t="n">
+      <c r="AZ69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11843,9 +12053,12 @@
         <v>0</v>
       </c>
       <c r="AX70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY70" t="n">
         <v>23</v>
       </c>
-      <c r="AY70" t="n">
+      <c r="AZ70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -12004,9 +12217,12 @@
         <v>0</v>
       </c>
       <c r="AX71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY71" t="n">
         <v>20</v>
       </c>
-      <c r="AY71" t="n">
+      <c r="AZ71" t="n">
         <v>20</v>
       </c>
     </row>
@@ -12165,9 +12381,12 @@
         <v>0</v>
       </c>
       <c r="AX72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY72" t="n">
         <v>19</v>
       </c>
-      <c r="AY72" t="n">
+      <c r="AZ72" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12331,6 +12550,9 @@
       <c r="AY73" t="n">
         <v>0</v>
       </c>
+      <c r="AZ73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12492,6 +12714,9 @@
       <c r="AY74" t="n">
         <v>0</v>
       </c>
+      <c r="AZ74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12648,9 +12873,12 @@
         <v>0</v>
       </c>
       <c r="AX75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY75" t="n">
         <v>19</v>
       </c>
-      <c r="AY75" t="n">
+      <c r="AZ75" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12809,9 +13037,12 @@
         <v>0</v>
       </c>
       <c r="AX76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY76" t="n">
         <v>19</v>
       </c>
-      <c r="AY76" t="n">
+      <c r="AZ76" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12970,9 +13201,12 @@
         <v>0</v>
       </c>
       <c r="AX77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY77" t="n">
         <v>15</v>
       </c>
-      <c r="AY77" t="n">
+      <c r="AZ77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -13131,9 +13365,12 @@
         <v>0</v>
       </c>
       <c r="AX78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY78" t="n">
         <v>25</v>
       </c>
-      <c r="AY78" t="n">
+      <c r="AZ78" t="n">
         <v>25</v>
       </c>
     </row>
@@ -13292,9 +13529,12 @@
         <v>0</v>
       </c>
       <c r="AX79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY79" t="n">
         <v>21</v>
       </c>
-      <c r="AY79" t="n">
+      <c r="AZ79" t="n">
         <v>21</v>
       </c>
     </row>
@@ -13453,9 +13693,12 @@
         <v>0</v>
       </c>
       <c r="AX80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY80" t="n">
         <v>11</v>
       </c>
-      <c r="AY80" t="n">
+      <c r="AZ80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -13614,9 +13857,12 @@
         <v>0</v>
       </c>
       <c r="AX81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY81" t="n">
         <v>4</v>
       </c>
-      <c r="AY81" t="n">
+      <c r="AZ81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -13775,9 +14021,12 @@
         <v>0</v>
       </c>
       <c r="AX82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY82" t="n">
         <v>11</v>
       </c>
-      <c r="AY82" t="n">
+      <c r="AZ82" t="n">
         <v>11</v>
       </c>
     </row>
@@ -13936,9 +14185,12 @@
         <v>0</v>
       </c>
       <c r="AX83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY83" t="n">
         <v>17</v>
       </c>
-      <c r="AY83" t="n">
+      <c r="AZ83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -14097,9 +14349,12 @@
         <v>0</v>
       </c>
       <c r="AX84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY84" t="n">
         <v>12</v>
       </c>
-      <c r="AY84" t="n">
+      <c r="AZ84" t="n">
         <v>12</v>
       </c>
     </row>
@@ -14258,9 +14513,12 @@
         <v>0</v>
       </c>
       <c r="AX85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY85" t="n">
         <v>7</v>
       </c>
-      <c r="AY85" t="n">
+      <c r="AZ85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14424,6 +14682,9 @@
       <c r="AY86" t="n">
         <v>0</v>
       </c>
+      <c r="AZ86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -14580,9 +14841,12 @@
         <v>0</v>
       </c>
       <c r="AX87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY87" t="n">
         <v>17</v>
       </c>
-      <c r="AY87" t="n">
+      <c r="AZ87" t="n">
         <v>17</v>
       </c>
     </row>
@@ -14746,6 +15010,9 @@
       <c r="AY88" t="n">
         <v>0</v>
       </c>
+      <c r="AZ88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -14902,9 +15169,12 @@
         <v>0</v>
       </c>
       <c r="AX89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY89" t="n">
         <v>17</v>
       </c>
-      <c r="AY89" t="n">
+      <c r="AZ89" t="n">
         <v>17</v>
       </c>
     </row>
@@ -15063,9 +15333,12 @@
         <v>0</v>
       </c>
       <c r="AX90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY90" t="n">
         <v>15</v>
       </c>
-      <c r="AY90" t="n">
+      <c r="AZ90" t="n">
         <v>15</v>
       </c>
     </row>
@@ -15224,9 +15497,12 @@
         <v>0</v>
       </c>
       <c r="AX91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY91" t="n">
         <v>42</v>
       </c>
-      <c r="AY91" t="n">
+      <c r="AZ91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -15385,9 +15661,12 @@
         <v>0</v>
       </c>
       <c r="AX92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY92" t="n">
         <v>7</v>
       </c>
-      <c r="AY92" t="n">
+      <c r="AZ92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15551,6 +15830,9 @@
       <c r="AY93" t="n">
         <v>0</v>
       </c>
+      <c r="AZ93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -15707,9 +15989,12 @@
         <v>0</v>
       </c>
       <c r="AX94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY94" t="n">
         <v>14</v>
       </c>
-      <c r="AY94" t="n">
+      <c r="AZ94" t="n">
         <v>14</v>
       </c>
     </row>
@@ -15868,9 +16153,12 @@
         <v>0</v>
       </c>
       <c r="AX95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY95" t="n">
         <v>7</v>
       </c>
-      <c r="AY95" t="n">
+      <c r="AZ95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16029,9 +16317,12 @@
         <v>0</v>
       </c>
       <c r="AX96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY96" t="n">
         <v>21</v>
       </c>
-      <c r="AY96" t="n">
+      <c r="AZ96" t="n">
         <v>21</v>
       </c>
     </row>
@@ -16195,6 +16486,9 @@
       <c r="AY97" t="n">
         <v>0</v>
       </c>
+      <c r="AZ97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -16351,9 +16645,12 @@
         <v>0</v>
       </c>
       <c r="AX98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY98" t="n">
         <v>26</v>
       </c>
-      <c r="AY98" t="n">
+      <c r="AZ98" t="n">
         <v>26</v>
       </c>
     </row>
@@ -16512,9 +16809,12 @@
         <v>1</v>
       </c>
       <c r="AX99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY99" t="n">
         <v>10</v>
       </c>
-      <c r="AY99" t="n">
+      <c r="AZ99" t="n">
         <v>10</v>
       </c>
     </row>
@@ -16678,6 +16978,9 @@
       <c r="AY100" t="n">
         <v>0</v>
       </c>
+      <c r="AZ100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -16834,9 +17137,12 @@
         <v>0</v>
       </c>
       <c r="AX101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY101" t="n">
         <v>25</v>
       </c>
-      <c r="AY101" t="n">
+      <c r="AZ101" t="n">
         <v>25</v>
       </c>
     </row>
@@ -16995,9 +17301,12 @@
         <v>0</v>
       </c>
       <c r="AX102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY102" t="n">
         <v>24</v>
       </c>
-      <c r="AY102" t="n">
+      <c r="AZ102" t="n">
         <v>24</v>
       </c>
     </row>
@@ -17156,9 +17465,12 @@
         <v>0</v>
       </c>
       <c r="AX103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY103" t="n">
         <v>25</v>
       </c>
-      <c r="AY103" t="n">
+      <c r="AZ103" t="n">
         <v>25</v>
       </c>
     </row>
@@ -17317,9 +17629,12 @@
         <v>0</v>
       </c>
       <c r="AX104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY104" t="n">
         <v>11</v>
       </c>
-      <c r="AY104" t="n">
+      <c r="AZ104" t="n">
         <v>11</v>
       </c>
     </row>
@@ -17478,9 +17793,12 @@
         <v>0</v>
       </c>
       <c r="AX105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY105" t="n">
         <v>18</v>
       </c>
-      <c r="AY105" t="n">
+      <c r="AZ105" t="n">
         <v>18</v>
       </c>
     </row>
@@ -17639,9 +17957,12 @@
         <v>0</v>
       </c>
       <c r="AX106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY106" t="n">
         <v>7</v>
       </c>
-      <c r="AY106" t="n">
+      <c r="AZ106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17800,9 +18121,12 @@
         <v>0</v>
       </c>
       <c r="AX107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY107" t="n">
         <v>11</v>
       </c>
-      <c r="AY107" t="n">
+      <c r="AZ107" t="n">
         <v>11</v>
       </c>
     </row>
@@ -17961,9 +18285,12 @@
         <v>0</v>
       </c>
       <c r="AX108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY108" t="n">
         <v>2</v>
       </c>
-      <c r="AY108" t="n">
+      <c r="AZ108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -18122,9 +18449,12 @@
         <v>0</v>
       </c>
       <c r="AX109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY109" t="n">
         <v>4</v>
       </c>
-      <c r="AY109" t="n">
+      <c r="AZ109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3561)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ109"/>
+  <dimension ref="A1:BA109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -480,8 +480,9 @@
     <col width="12" customWidth="1" min="48" max="48"/>
     <col width="12" customWidth="1" min="49" max="49"/>
     <col width="12" customWidth="1" min="50" max="50"/>
-    <col width="13" customWidth="1" min="51" max="51"/>
+    <col width="12" customWidth="1" min="51" max="51"/>
     <col width="13" customWidth="1" min="52" max="52"/>
+    <col width="13" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -735,12 +736,17 @@
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="AY1" s="2" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="AZ1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="AZ1" s="2" t="inlineStr">
+      <c r="BA1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -904,9 +910,12 @@
         <v>0</v>
       </c>
       <c r="AY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ2" t="n">
         <v>12</v>
       </c>
-      <c r="AZ2" t="n">
+      <c r="BA2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1068,9 +1077,12 @@
         <v>0</v>
       </c>
       <c r="AY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ3" t="n">
         <v>9</v>
       </c>
-      <c r="AZ3" t="n">
+      <c r="BA3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1232,10 +1244,13 @@
         <v>0</v>
       </c>
       <c r="AY4" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="AZ4" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -1396,9 +1411,12 @@
         <v>0</v>
       </c>
       <c r="AY5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ5" t="n">
         <v>15</v>
       </c>
-      <c r="AZ5" t="n">
+      <c r="BA5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1560,9 +1578,12 @@
         <v>0</v>
       </c>
       <c r="AY6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ6" t="n">
         <v>18</v>
       </c>
-      <c r="AZ6" t="n">
+      <c r="BA6" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1724,9 +1745,12 @@
         <v>0</v>
       </c>
       <c r="AY7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ7" t="n">
         <v>18</v>
       </c>
-      <c r="AZ7" t="n">
+      <c r="BA7" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1888,9 +1912,12 @@
         <v>0</v>
       </c>
       <c r="AY8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ8" t="n">
         <v>27</v>
       </c>
-      <c r="AZ8" t="n">
+      <c r="BA8" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2052,9 +2079,12 @@
         <v>0</v>
       </c>
       <c r="AY9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ9" t="n">
         <v>24</v>
       </c>
-      <c r="AZ9" t="n">
+      <c r="BA9" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2216,10 +2246,13 @@
         <v>0</v>
       </c>
       <c r="AY10" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="AZ10" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="11">
@@ -2380,10 +2413,13 @@
         <v>0</v>
       </c>
       <c r="AY11" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AZ11" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="12">
@@ -2544,10 +2580,13 @@
         <v>0</v>
       </c>
       <c r="AY12" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="AZ12" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="13">
@@ -2708,9 +2747,12 @@
         <v>0</v>
       </c>
       <c r="AY13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ13" t="n">
         <v>14</v>
       </c>
-      <c r="AZ13" t="n">
+      <c r="BA13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2872,9 +2914,12 @@
         <v>0</v>
       </c>
       <c r="AY14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ14" t="n">
         <v>24</v>
       </c>
-      <c r="AZ14" t="n">
+      <c r="BA14" t="n">
         <v>24</v>
       </c>
     </row>
@@ -3036,9 +3081,12 @@
         <v>0</v>
       </c>
       <c r="AY15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ15" t="n">
         <v>9</v>
       </c>
-      <c r="AZ15" t="n">
+      <c r="BA15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3200,9 +3248,12 @@
         <v>0</v>
       </c>
       <c r="AY16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ16" t="n">
         <v>20</v>
       </c>
-      <c r="AZ16" t="n">
+      <c r="BA16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3364,9 +3415,12 @@
         <v>0</v>
       </c>
       <c r="AY17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ17" t="n">
         <v>17</v>
       </c>
-      <c r="AZ17" t="n">
+      <c r="BA17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3528,10 +3582,13 @@
         <v>0</v>
       </c>
       <c r="AY18" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AZ18" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BA18" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="19">
@@ -3697,6 +3754,9 @@
       <c r="AZ19" t="n">
         <v>0</v>
       </c>
+      <c r="BA19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3856,9 +3916,12 @@
         <v>0</v>
       </c>
       <c r="AY20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ20" t="n">
         <v>18</v>
       </c>
-      <c r="AZ20" t="n">
+      <c r="BA20" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4020,10 +4083,13 @@
         <v>0</v>
       </c>
       <c r="AY21" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AZ21" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BA21" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="22">
@@ -4189,6 +4255,9 @@
       <c r="AZ22" t="n">
         <v>0</v>
       </c>
+      <c r="BA22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4348,10 +4417,13 @@
         <v>0</v>
       </c>
       <c r="AY23" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AZ23" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="BA23" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="24">
@@ -4512,9 +4584,12 @@
         <v>0</v>
       </c>
       <c r="AY24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ24" t="n">
         <v>24</v>
       </c>
-      <c r="AZ24" t="n">
+      <c r="BA24" t="n">
         <v>24</v>
       </c>
     </row>
@@ -4676,9 +4751,12 @@
         <v>0</v>
       </c>
       <c r="AY25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ25" t="n">
         <v>9</v>
       </c>
-      <c r="AZ25" t="n">
+      <c r="BA25" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4840,10 +4918,13 @@
         <v>0</v>
       </c>
       <c r="AY26" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AZ26" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BA26" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="27">
@@ -5004,9 +5085,12 @@
         <v>0</v>
       </c>
       <c r="AY27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ27" t="n">
         <v>24</v>
       </c>
-      <c r="AZ27" t="n">
+      <c r="BA27" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5168,10 +5252,13 @@
         <v>0</v>
       </c>
       <c r="AY28" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AZ28" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="29">
@@ -5332,9 +5419,12 @@
         <v>0</v>
       </c>
       <c r="AY29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ29" t="n">
         <v>11</v>
       </c>
-      <c r="AZ29" t="n">
+      <c r="BA29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5496,9 +5586,12 @@
         <v>0</v>
       </c>
       <c r="AY30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ30" t="n">
         <v>22</v>
       </c>
-      <c r="AZ30" t="n">
+      <c r="BA30" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5660,9 +5753,12 @@
         <v>0</v>
       </c>
       <c r="AY31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ31" t="n">
         <v>19</v>
       </c>
-      <c r="AZ31" t="n">
+      <c r="BA31" t="n">
         <v>19</v>
       </c>
     </row>
@@ -5824,9 +5920,12 @@
         <v>0</v>
       </c>
       <c r="AY32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ32" t="n">
         <v>18</v>
       </c>
-      <c r="AZ32" t="n">
+      <c r="BA32" t="n">
         <v>18</v>
       </c>
     </row>
@@ -5988,9 +6087,12 @@
         <v>0</v>
       </c>
       <c r="AY33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ33" t="n">
         <v>15</v>
       </c>
-      <c r="AZ33" t="n">
+      <c r="BA33" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6152,9 +6254,12 @@
         <v>0</v>
       </c>
       <c r="AY34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ34" t="n">
         <v>9</v>
       </c>
-      <c r="AZ34" t="n">
+      <c r="BA34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6316,10 +6421,13 @@
         <v>0</v>
       </c>
       <c r="AY35" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AZ35" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="BA35" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="36">
@@ -6480,10 +6588,13 @@
         <v>0</v>
       </c>
       <c r="AY36" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AZ36" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="BA36" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="37">
@@ -6649,6 +6760,9 @@
       <c r="AZ37" t="n">
         <v>0</v>
       </c>
+      <c r="BA37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6808,9 +6922,12 @@
         <v>0</v>
       </c>
       <c r="AY38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ38" t="n">
         <v>2</v>
       </c>
-      <c r="AZ38" t="n">
+      <c r="BA38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6972,10 +7089,13 @@
         <v>0</v>
       </c>
       <c r="AY39" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="AZ39" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BA39" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="40">
@@ -7136,10 +7256,13 @@
         <v>0</v>
       </c>
       <c r="AY40" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AZ40" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="BA40" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="41">
@@ -7300,10 +7423,13 @@
         <v>0</v>
       </c>
       <c r="AY41" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="AZ41" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BA41" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="42">
@@ -7464,9 +7590,12 @@
         <v>0</v>
       </c>
       <c r="AY42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ42" t="n">
         <v>21</v>
       </c>
-      <c r="AZ42" t="n">
+      <c r="BA42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7628,10 +7757,13 @@
         <v>0</v>
       </c>
       <c r="AY43" t="n">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="AZ43" t="n">
-        <v>18</v>
+        <v>60</v>
+      </c>
+      <c r="BA43" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="44">
@@ -7792,9 +7924,12 @@
         <v>0</v>
       </c>
       <c r="AY44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ44" t="n">
         <v>22</v>
       </c>
-      <c r="AZ44" t="n">
+      <c r="BA44" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7956,9 +8091,12 @@
         <v>0</v>
       </c>
       <c r="AY45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ45" t="n">
         <v>23</v>
       </c>
-      <c r="AZ45" t="n">
+      <c r="BA45" t="n">
         <v>23</v>
       </c>
     </row>
@@ -8120,10 +8258,13 @@
         <v>0</v>
       </c>
       <c r="AY46" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="AZ46" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BA46" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="47">
@@ -8289,6 +8430,9 @@
       <c r="AZ47" t="n">
         <v>0</v>
       </c>
+      <c r="BA47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8448,9 +8592,12 @@
         <v>0</v>
       </c>
       <c r="AY48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ48" t="n">
         <v>25</v>
       </c>
-      <c r="AZ48" t="n">
+      <c r="BA48" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8612,9 +8759,12 @@
         <v>0</v>
       </c>
       <c r="AY49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ49" t="n">
         <v>19</v>
       </c>
-      <c r="AZ49" t="n">
+      <c r="BA49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8776,9 +8926,12 @@
         <v>0</v>
       </c>
       <c r="AY50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ50" t="n">
         <v>7</v>
       </c>
-      <c r="AZ50" t="n">
+      <c r="BA50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8940,10 +9093,13 @@
         <v>0</v>
       </c>
       <c r="AY51" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="AZ51" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BA51" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="52">
@@ -9109,6 +9265,9 @@
       <c r="AZ52" t="n">
         <v>0</v>
       </c>
+      <c r="BA52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9268,9 +9427,12 @@
         <v>0</v>
       </c>
       <c r="AY53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ53" t="n">
         <v>13</v>
       </c>
-      <c r="AZ53" t="n">
+      <c r="BA53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9437,6 +9599,9 @@
       <c r="AZ54" t="n">
         <v>0</v>
       </c>
+      <c r="BA54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9596,10 +9761,13 @@
         <v>0</v>
       </c>
       <c r="AY55" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="AZ55" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BA55" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="56">
@@ -9760,10 +9928,13 @@
         <v>0</v>
       </c>
       <c r="AY56" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AZ56" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BA56" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="57">
@@ -9924,9 +10095,12 @@
         <v>0</v>
       </c>
       <c r="AY57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ57" t="n">
         <v>9</v>
       </c>
-      <c r="AZ57" t="n">
+      <c r="BA57" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10088,9 +10262,12 @@
         <v>0</v>
       </c>
       <c r="AY58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ58" t="n">
         <v>12</v>
       </c>
-      <c r="AZ58" t="n">
+      <c r="BA58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -10252,9 +10429,12 @@
         <v>0</v>
       </c>
       <c r="AY59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ59" t="n">
         <v>6</v>
       </c>
-      <c r="AZ59" t="n">
+      <c r="BA59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10421,6 +10601,9 @@
       <c r="AZ60" t="n">
         <v>0</v>
       </c>
+      <c r="BA60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10580,10 +10763,13 @@
         <v>0</v>
       </c>
       <c r="AY61" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AZ61" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BA61" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="62">
@@ -10744,10 +10930,13 @@
         <v>0</v>
       </c>
       <c r="AY62" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AZ62" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BA62" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="63">
@@ -10908,10 +11097,13 @@
         <v>0</v>
       </c>
       <c r="AY63" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AZ63" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="BA63" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="64">
@@ -11077,6 +11269,9 @@
       <c r="AZ64" t="n">
         <v>0</v>
       </c>
+      <c r="BA64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -11236,9 +11431,12 @@
         <v>0</v>
       </c>
       <c r="AY65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ65" t="n">
         <v>14</v>
       </c>
-      <c r="AZ65" t="n">
+      <c r="BA65" t="n">
         <v>14</v>
       </c>
     </row>
@@ -11400,9 +11598,12 @@
         <v>0</v>
       </c>
       <c r="AY66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ66" t="n">
         <v>7</v>
       </c>
-      <c r="AZ66" t="n">
+      <c r="BA66" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11564,10 +11765,13 @@
         <v>0</v>
       </c>
       <c r="AY67" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="AZ67" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BA67" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="68">
@@ -11728,10 +11932,13 @@
         <v>0</v>
       </c>
       <c r="AY68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ68" t="n">
+        <v>19</v>
+      </c>
+      <c r="BA68" t="n">
         <v>18</v>
-      </c>
-      <c r="AZ68" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="69">
@@ -11892,9 +12099,12 @@
         <v>0</v>
       </c>
       <c r="AY69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ69" t="n">
         <v>7</v>
       </c>
-      <c r="AZ69" t="n">
+      <c r="BA69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12056,9 +12266,12 @@
         <v>0</v>
       </c>
       <c r="AY70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ70" t="n">
         <v>23</v>
       </c>
-      <c r="AZ70" t="n">
+      <c r="BA70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -12220,9 +12433,12 @@
         <v>0</v>
       </c>
       <c r="AY71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ71" t="n">
         <v>20</v>
       </c>
-      <c r="AZ71" t="n">
+      <c r="BA71" t="n">
         <v>20</v>
       </c>
     </row>
@@ -12384,10 +12600,13 @@
         <v>0</v>
       </c>
       <c r="AY72" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AZ72" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="BA72" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="73">
@@ -12553,6 +12772,9 @@
       <c r="AZ73" t="n">
         <v>0</v>
       </c>
+      <c r="BA73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12717,6 +12939,9 @@
       <c r="AZ74" t="n">
         <v>0</v>
       </c>
+      <c r="BA74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12876,10 +13101,13 @@
         <v>0</v>
       </c>
       <c r="AY75" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AZ75" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="BA75" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="76">
@@ -13040,10 +13268,13 @@
         <v>0</v>
       </c>
       <c r="AY76" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AZ76" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="BA76" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="77">
@@ -13204,9 +13435,12 @@
         <v>0</v>
       </c>
       <c r="AY77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ77" t="n">
         <v>15</v>
       </c>
-      <c r="AZ77" t="n">
+      <c r="BA77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -13368,10 +13602,13 @@
         <v>0</v>
       </c>
       <c r="AY78" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AZ78" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BA78" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="79">
@@ -13532,9 +13769,12 @@
         <v>0</v>
       </c>
       <c r="AY79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ79" t="n">
         <v>21</v>
       </c>
-      <c r="AZ79" t="n">
+      <c r="BA79" t="n">
         <v>21</v>
       </c>
     </row>
@@ -13696,9 +13936,12 @@
         <v>0</v>
       </c>
       <c r="AY80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ80" t="n">
         <v>11</v>
       </c>
-      <c r="AZ80" t="n">
+      <c r="BA80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -13860,9 +14103,12 @@
         <v>0</v>
       </c>
       <c r="AY81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ81" t="n">
         <v>4</v>
       </c>
-      <c r="AZ81" t="n">
+      <c r="BA81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -14024,10 +14270,13 @@
         <v>0</v>
       </c>
       <c r="AY82" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AZ82" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="BA82" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="83">
@@ -14188,9 +14437,12 @@
         <v>0</v>
       </c>
       <c r="AY83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ83" t="n">
         <v>17</v>
       </c>
-      <c r="AZ83" t="n">
+      <c r="BA83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -14352,10 +14604,13 @@
         <v>0</v>
       </c>
       <c r="AY84" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AZ84" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="BA84" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="85">
@@ -14516,9 +14771,12 @@
         <v>0</v>
       </c>
       <c r="AY85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ85" t="n">
         <v>7</v>
       </c>
-      <c r="AZ85" t="n">
+      <c r="BA85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14685,6 +14943,9 @@
       <c r="AZ86" t="n">
         <v>0</v>
       </c>
+      <c r="BA86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -14844,9 +15105,12 @@
         <v>0</v>
       </c>
       <c r="AY87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ87" t="n">
         <v>17</v>
       </c>
-      <c r="AZ87" t="n">
+      <c r="BA87" t="n">
         <v>17</v>
       </c>
     </row>
@@ -15013,6 +15277,9 @@
       <c r="AZ88" t="n">
         <v>0</v>
       </c>
+      <c r="BA88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -15172,9 +15439,12 @@
         <v>0</v>
       </c>
       <c r="AY89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ89" t="n">
         <v>17</v>
       </c>
-      <c r="AZ89" t="n">
+      <c r="BA89" t="n">
         <v>17</v>
       </c>
     </row>
@@ -15336,9 +15606,12 @@
         <v>0</v>
       </c>
       <c r="AY90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ90" t="n">
         <v>15</v>
       </c>
-      <c r="AZ90" t="n">
+      <c r="BA90" t="n">
         <v>15</v>
       </c>
     </row>
@@ -15500,9 +15773,12 @@
         <v>0</v>
       </c>
       <c r="AY91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ91" t="n">
         <v>42</v>
       </c>
-      <c r="AZ91" t="n">
+      <c r="BA91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -15664,9 +15940,12 @@
         <v>0</v>
       </c>
       <c r="AY92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ92" t="n">
         <v>7</v>
       </c>
-      <c r="AZ92" t="n">
+      <c r="BA92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15833,6 +16112,9 @@
       <c r="AZ93" t="n">
         <v>0</v>
       </c>
+      <c r="BA93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -15992,10 +16274,13 @@
         <v>0</v>
       </c>
       <c r="AY94" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="AZ94" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="BA94" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="95">
@@ -16156,9 +16441,12 @@
         <v>0</v>
       </c>
       <c r="AY95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ95" t="n">
         <v>7</v>
       </c>
-      <c r="AZ95" t="n">
+      <c r="BA95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16320,10 +16608,13 @@
         <v>0</v>
       </c>
       <c r="AY96" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AZ96" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="BA96" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="97">
@@ -16489,6 +16780,9 @@
       <c r="AZ97" t="n">
         <v>0</v>
       </c>
+      <c r="BA97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -16648,10 +16942,13 @@
         <v>0</v>
       </c>
       <c r="AY98" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="AZ98" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BA98" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="99">
@@ -16812,10 +17109,13 @@
         <v>0</v>
       </c>
       <c r="AY99" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AZ99" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="BA99" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="100">
@@ -16981,6 +17281,9 @@
       <c r="AZ100" t="n">
         <v>0</v>
       </c>
+      <c r="BA100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -17140,10 +17443,13 @@
         <v>0</v>
       </c>
       <c r="AY101" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AZ101" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BA101" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="102">
@@ -17304,10 +17610,13 @@
         <v>0</v>
       </c>
       <c r="AY102" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="AZ102" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BA102" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="103">
@@ -17468,10 +17777,13 @@
         <v>0</v>
       </c>
       <c r="AY103" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="AZ103" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BA103" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="104">
@@ -17632,9 +17944,12 @@
         <v>0</v>
       </c>
       <c r="AY104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ104" t="n">
         <v>11</v>
       </c>
-      <c r="AZ104" t="n">
+      <c r="BA104" t="n">
         <v>11</v>
       </c>
     </row>
@@ -17796,10 +18111,13 @@
         <v>0</v>
       </c>
       <c r="AY105" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AZ105" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="BA105" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="106">
@@ -17960,9 +18278,12 @@
         <v>0</v>
       </c>
       <c r="AY106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ106" t="n">
         <v>7</v>
       </c>
-      <c r="AZ106" t="n">
+      <c r="BA106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18124,10 +18445,13 @@
         <v>0</v>
       </c>
       <c r="AY107" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AZ107" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="BA107" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="108">
@@ -18288,9 +18612,12 @@
         <v>0</v>
       </c>
       <c r="AY108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ108" t="n">
         <v>2</v>
       </c>
-      <c r="AZ108" t="n">
+      <c r="BA108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -18452,9 +18779,12 @@
         <v>0</v>
       </c>
       <c r="AY109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ109" t="n">
         <v>4</v>
       </c>
-      <c r="AZ109" t="n">
+      <c r="BA109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3645)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA109"/>
+  <dimension ref="A1:BB109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -481,8 +481,9 @@
     <col width="12" customWidth="1" min="49" max="49"/>
     <col width="12" customWidth="1" min="50" max="50"/>
     <col width="12" customWidth="1" min="51" max="51"/>
-    <col width="13" customWidth="1" min="52" max="52"/>
+    <col width="12" customWidth="1" min="52" max="52"/>
     <col width="13" customWidth="1" min="53" max="53"/>
+    <col width="13" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -741,12 +742,17 @@
           <t>2026-04-13</t>
         </is>
       </c>
-      <c r="AZ1" s="2" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="BA1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BA1" s="2" t="inlineStr">
+      <c r="BB1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -913,9 +919,12 @@
         <v>0</v>
       </c>
       <c r="AZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA2" t="n">
         <v>12</v>
       </c>
-      <c r="BA2" t="n">
+      <c r="BB2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1080,9 +1089,12 @@
         <v>0</v>
       </c>
       <c r="AZ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA3" t="n">
         <v>9</v>
       </c>
-      <c r="BA3" t="n">
+      <c r="BB3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1247,10 +1259,13 @@
         <v>1</v>
       </c>
       <c r="AZ4" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BA4" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="5">
@@ -1414,9 +1429,12 @@
         <v>0</v>
       </c>
       <c r="AZ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA5" t="n">
         <v>15</v>
       </c>
-      <c r="BA5" t="n">
+      <c r="BB5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1581,9 +1599,12 @@
         <v>0</v>
       </c>
       <c r="AZ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA6" t="n">
         <v>18</v>
       </c>
-      <c r="BA6" t="n">
+      <c r="BB6" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1748,10 +1769,13 @@
         <v>0</v>
       </c>
       <c r="AZ7" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="BA7" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="8">
@@ -1915,10 +1939,13 @@
         <v>0</v>
       </c>
       <c r="AZ8" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BA8" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -2082,10 +2109,13 @@
         <v>0</v>
       </c>
       <c r="AZ9" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BA9" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -2249,10 +2279,13 @@
         <v>1</v>
       </c>
       <c r="AZ10" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BA10" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="11">
@@ -2416,10 +2449,13 @@
         <v>1</v>
       </c>
       <c r="AZ11" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BA11" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="12">
@@ -2583,10 +2619,13 @@
         <v>1</v>
       </c>
       <c r="AZ12" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BA12" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BB12" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="13">
@@ -2750,9 +2789,12 @@
         <v>0</v>
       </c>
       <c r="AZ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA13" t="n">
         <v>14</v>
       </c>
-      <c r="BA13" t="n">
+      <c r="BB13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2917,9 +2959,12 @@
         <v>0</v>
       </c>
       <c r="AZ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA14" t="n">
         <v>24</v>
       </c>
-      <c r="BA14" t="n">
+      <c r="BB14" t="n">
         <v>24</v>
       </c>
     </row>
@@ -3084,9 +3129,12 @@
         <v>0</v>
       </c>
       <c r="AZ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA15" t="n">
         <v>9</v>
       </c>
-      <c r="BA15" t="n">
+      <c r="BB15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3251,9 +3299,12 @@
         <v>0</v>
       </c>
       <c r="AZ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA16" t="n">
         <v>20</v>
       </c>
-      <c r="BA16" t="n">
+      <c r="BB16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3418,9 +3469,12 @@
         <v>0</v>
       </c>
       <c r="AZ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA17" t="n">
         <v>17</v>
       </c>
-      <c r="BA17" t="n">
+      <c r="BB17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3585,10 +3639,13 @@
         <v>1</v>
       </c>
       <c r="AZ18" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BA18" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BB18" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="19">
@@ -3757,6 +3814,9 @@
       <c r="BA19" t="n">
         <v>0</v>
       </c>
+      <c r="BB19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3919,9 +3979,12 @@
         <v>0</v>
       </c>
       <c r="AZ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA20" t="n">
         <v>18</v>
       </c>
-      <c r="BA20" t="n">
+      <c r="BB20" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4086,9 +4149,12 @@
         <v>1</v>
       </c>
       <c r="AZ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA21" t="n">
         <v>24</v>
       </c>
-      <c r="BA21" t="n">
+      <c r="BB21" t="n">
         <v>24</v>
       </c>
     </row>
@@ -4258,6 +4324,9 @@
       <c r="BA22" t="n">
         <v>0</v>
       </c>
+      <c r="BB22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4420,10 +4489,13 @@
         <v>1</v>
       </c>
       <c r="AZ23" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="BA23" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="BB23" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="24">
@@ -4587,9 +4659,12 @@
         <v>0</v>
       </c>
       <c r="AZ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA24" t="n">
         <v>24</v>
       </c>
-      <c r="BA24" t="n">
+      <c r="BB24" t="n">
         <v>24</v>
       </c>
     </row>
@@ -4754,10 +4829,13 @@
         <v>0</v>
       </c>
       <c r="AZ25" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="BA25" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="BB25" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="26">
@@ -4921,10 +4999,13 @@
         <v>1</v>
       </c>
       <c r="AZ26" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BA26" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="27">
@@ -5088,9 +5169,12 @@
         <v>0</v>
       </c>
       <c r="AZ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA27" t="n">
         <v>24</v>
       </c>
-      <c r="BA27" t="n">
+      <c r="BB27" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5255,10 +5339,13 @@
         <v>1</v>
       </c>
       <c r="AZ28" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="BA28" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="BB28" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="29">
@@ -5422,9 +5509,12 @@
         <v>0</v>
       </c>
       <c r="AZ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA29" t="n">
         <v>11</v>
       </c>
-      <c r="BA29" t="n">
+      <c r="BB29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5589,9 +5679,12 @@
         <v>0</v>
       </c>
       <c r="AZ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA30" t="n">
         <v>22</v>
       </c>
-      <c r="BA30" t="n">
+      <c r="BB30" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5756,9 +5849,12 @@
         <v>0</v>
       </c>
       <c r="AZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA31" t="n">
         <v>19</v>
       </c>
-      <c r="BA31" t="n">
+      <c r="BB31" t="n">
         <v>19</v>
       </c>
     </row>
@@ -5923,10 +6019,13 @@
         <v>0</v>
       </c>
       <c r="AZ32" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="BA32" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="BB32" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="33">
@@ -6090,9 +6189,12 @@
         <v>0</v>
       </c>
       <c r="AZ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA33" t="n">
         <v>15</v>
       </c>
-      <c r="BA33" t="n">
+      <c r="BB33" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6257,9 +6359,12 @@
         <v>0</v>
       </c>
       <c r="AZ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA34" t="n">
         <v>9</v>
       </c>
-      <c r="BA34" t="n">
+      <c r="BB34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6424,10 +6529,13 @@
         <v>1</v>
       </c>
       <c r="AZ35" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="BA35" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="BB35" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="36">
@@ -6591,10 +6699,13 @@
         <v>1</v>
       </c>
       <c r="AZ36" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="BA36" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="BB36" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="37">
@@ -6763,6 +6874,9 @@
       <c r="BA37" t="n">
         <v>0</v>
       </c>
+      <c r="BB37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6925,9 +7039,12 @@
         <v>0</v>
       </c>
       <c r="AZ38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA38" t="n">
         <v>2</v>
       </c>
-      <c r="BA38" t="n">
+      <c r="BB38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7092,10 +7209,13 @@
         <v>1</v>
       </c>
       <c r="AZ39" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BA39" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BB39" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="40">
@@ -7259,10 +7379,13 @@
         <v>1</v>
       </c>
       <c r="AZ40" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="BA40" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="BB40" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="41">
@@ -7426,10 +7549,13 @@
         <v>1</v>
       </c>
       <c r="AZ41" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BA41" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BB41" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="42">
@@ -7593,9 +7719,12 @@
         <v>0</v>
       </c>
       <c r="AZ42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA42" t="n">
         <v>21</v>
       </c>
-      <c r="BA42" t="n">
+      <c r="BB42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7760,9 +7889,12 @@
         <v>1</v>
       </c>
       <c r="AZ43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA43" t="n">
         <v>60</v>
       </c>
-      <c r="BA43" t="n">
+      <c r="BB43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -7927,9 +8059,12 @@
         <v>0</v>
       </c>
       <c r="AZ44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA44" t="n">
         <v>22</v>
       </c>
-      <c r="BA44" t="n">
+      <c r="BB44" t="n">
         <v>22</v>
       </c>
     </row>
@@ -8094,9 +8229,12 @@
         <v>0</v>
       </c>
       <c r="AZ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA45" t="n">
         <v>23</v>
       </c>
-      <c r="BA45" t="n">
+      <c r="BB45" t="n">
         <v>23</v>
       </c>
     </row>
@@ -8261,10 +8399,13 @@
         <v>1</v>
       </c>
       <c r="AZ46" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BA46" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BB46" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="47">
@@ -8433,6 +8574,9 @@
       <c r="BA47" t="n">
         <v>0</v>
       </c>
+      <c r="BB47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8595,9 +8739,12 @@
         <v>0</v>
       </c>
       <c r="AZ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA48" t="n">
         <v>25</v>
       </c>
-      <c r="BA48" t="n">
+      <c r="BB48" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8762,9 +8909,12 @@
         <v>0</v>
       </c>
       <c r="AZ49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA49" t="n">
         <v>19</v>
       </c>
-      <c r="BA49" t="n">
+      <c r="BB49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8929,9 +9079,12 @@
         <v>0</v>
       </c>
       <c r="AZ50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA50" t="n">
         <v>7</v>
       </c>
-      <c r="BA50" t="n">
+      <c r="BB50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9096,10 +9249,13 @@
         <v>1</v>
       </c>
       <c r="AZ51" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BA51" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BB51" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="52">
@@ -9268,6 +9424,9 @@
       <c r="BA52" t="n">
         <v>0</v>
       </c>
+      <c r="BB52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9430,9 +9589,12 @@
         <v>0</v>
       </c>
       <c r="AZ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA53" t="n">
         <v>13</v>
       </c>
-      <c r="BA53" t="n">
+      <c r="BB53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9602,6 +9764,9 @@
       <c r="BA54" t="n">
         <v>0</v>
       </c>
+      <c r="BB54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9764,10 +9929,13 @@
         <v>1</v>
       </c>
       <c r="AZ55" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BA55" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BB55" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="56">
@@ -9931,9 +10099,12 @@
         <v>1</v>
       </c>
       <c r="AZ56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA56" t="n">
         <v>26</v>
       </c>
-      <c r="BA56" t="n">
+      <c r="BB56" t="n">
         <v>26</v>
       </c>
     </row>
@@ -10098,9 +10269,12 @@
         <v>0</v>
       </c>
       <c r="AZ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA57" t="n">
         <v>9</v>
       </c>
-      <c r="BA57" t="n">
+      <c r="BB57" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10265,9 +10439,12 @@
         <v>0</v>
       </c>
       <c r="AZ58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA58" t="n">
         <v>12</v>
       </c>
-      <c r="BA58" t="n">
+      <c r="BB58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -10432,9 +10609,12 @@
         <v>0</v>
       </c>
       <c r="AZ59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA59" t="n">
         <v>6</v>
       </c>
-      <c r="BA59" t="n">
+      <c r="BB59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10604,6 +10784,9 @@
       <c r="BA60" t="n">
         <v>0</v>
       </c>
+      <c r="BB60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10766,10 +10949,13 @@
         <v>1</v>
       </c>
       <c r="AZ61" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BA61" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BB61" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="62">
@@ -10933,10 +11119,13 @@
         <v>1</v>
       </c>
       <c r="AZ62" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BA62" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BB62" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="63">
@@ -11100,9 +11289,12 @@
         <v>1</v>
       </c>
       <c r="AZ63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA63" t="n">
         <v>10</v>
       </c>
-      <c r="BA63" t="n">
+      <c r="BB63" t="n">
         <v>10</v>
       </c>
     </row>
@@ -11272,6 +11464,9 @@
       <c r="BA64" t="n">
         <v>0</v>
       </c>
+      <c r="BB64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -11434,10 +11629,13 @@
         <v>0</v>
       </c>
       <c r="AZ65" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="BA65" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="BB65" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="66">
@@ -11601,9 +11799,12 @@
         <v>0</v>
       </c>
       <c r="AZ66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA66" t="n">
         <v>7</v>
       </c>
-      <c r="BA66" t="n">
+      <c r="BB66" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11768,10 +11969,13 @@
         <v>1</v>
       </c>
       <c r="AZ67" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BA67" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BB67" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="68">
@@ -11935,9 +12139,12 @@
         <v>1</v>
       </c>
       <c r="AZ68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA68" t="n">
         <v>19</v>
       </c>
-      <c r="BA68" t="n">
+      <c r="BB68" t="n">
         <v>18</v>
       </c>
     </row>
@@ -12102,9 +12309,12 @@
         <v>0</v>
       </c>
       <c r="AZ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA69" t="n">
         <v>7</v>
       </c>
-      <c r="BA69" t="n">
+      <c r="BB69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12269,9 +12479,12 @@
         <v>0</v>
       </c>
       <c r="AZ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA70" t="n">
         <v>23</v>
       </c>
-      <c r="BA70" t="n">
+      <c r="BB70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -12436,10 +12649,13 @@
         <v>0</v>
       </c>
       <c r="AZ71" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="BA71" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="BB71" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="72">
@@ -12603,10 +12819,13 @@
         <v>1</v>
       </c>
       <c r="AZ72" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="BA72" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="BB72" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="73">
@@ -12775,6 +12994,9 @@
       <c r="BA73" t="n">
         <v>0</v>
       </c>
+      <c r="BB73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12942,6 +13164,9 @@
       <c r="BA74" t="n">
         <v>0</v>
       </c>
+      <c r="BB74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -13104,10 +13329,13 @@
         <v>1</v>
       </c>
       <c r="AZ75" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="BA75" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="BB75" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="76">
@@ -13271,9 +13499,12 @@
         <v>1</v>
       </c>
       <c r="AZ76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA76" t="n">
         <v>20</v>
       </c>
-      <c r="BA76" t="n">
+      <c r="BB76" t="n">
         <v>20</v>
       </c>
     </row>
@@ -13438,9 +13669,12 @@
         <v>0</v>
       </c>
       <c r="AZ77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA77" t="n">
         <v>15</v>
       </c>
-      <c r="BA77" t="n">
+      <c r="BB77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -13605,10 +13839,13 @@
         <v>1</v>
       </c>
       <c r="AZ78" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BA78" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BB78" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="79">
@@ -13772,9 +14009,12 @@
         <v>0</v>
       </c>
       <c r="AZ79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA79" t="n">
         <v>21</v>
       </c>
-      <c r="BA79" t="n">
+      <c r="BB79" t="n">
         <v>21</v>
       </c>
     </row>
@@ -13939,9 +14179,12 @@
         <v>0</v>
       </c>
       <c r="AZ80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA80" t="n">
         <v>11</v>
       </c>
-      <c r="BA80" t="n">
+      <c r="BB80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -14106,9 +14349,12 @@
         <v>0</v>
       </c>
       <c r="AZ81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA81" t="n">
         <v>4</v>
       </c>
-      <c r="BA81" t="n">
+      <c r="BB81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -14273,10 +14519,13 @@
         <v>1</v>
       </c>
       <c r="AZ82" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="BA82" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="BB82" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="83">
@@ -14440,9 +14689,12 @@
         <v>0</v>
       </c>
       <c r="AZ83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA83" t="n">
         <v>17</v>
       </c>
-      <c r="BA83" t="n">
+      <c r="BB83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -14607,9 +14859,12 @@
         <v>1</v>
       </c>
       <c r="AZ84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA84" t="n">
         <v>13</v>
       </c>
-      <c r="BA84" t="n">
+      <c r="BB84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -14774,9 +15029,12 @@
         <v>0</v>
       </c>
       <c r="AZ85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA85" t="n">
         <v>7</v>
       </c>
-      <c r="BA85" t="n">
+      <c r="BB85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14946,6 +15204,9 @@
       <c r="BA86" t="n">
         <v>0</v>
       </c>
+      <c r="BB86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -15108,10 +15369,13 @@
         <v>0</v>
       </c>
       <c r="AZ87" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="BA87" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="BB87" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="88">
@@ -15280,6 +15544,9 @@
       <c r="BA88" t="n">
         <v>0</v>
       </c>
+      <c r="BB88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -15442,9 +15709,12 @@
         <v>0</v>
       </c>
       <c r="AZ89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA89" t="n">
         <v>17</v>
       </c>
-      <c r="BA89" t="n">
+      <c r="BB89" t="n">
         <v>17</v>
       </c>
     </row>
@@ -15609,9 +15879,12 @@
         <v>0</v>
       </c>
       <c r="AZ90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA90" t="n">
         <v>15</v>
       </c>
-      <c r="BA90" t="n">
+      <c r="BB90" t="n">
         <v>15</v>
       </c>
     </row>
@@ -15776,9 +16049,12 @@
         <v>0</v>
       </c>
       <c r="AZ91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA91" t="n">
         <v>42</v>
       </c>
-      <c r="BA91" t="n">
+      <c r="BB91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -15943,9 +16219,12 @@
         <v>0</v>
       </c>
       <c r="AZ92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA92" t="n">
         <v>7</v>
       </c>
-      <c r="BA92" t="n">
+      <c r="BB92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16115,6 +16394,9 @@
       <c r="BA93" t="n">
         <v>0</v>
       </c>
+      <c r="BB93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -16277,10 +16559,13 @@
         <v>1</v>
       </c>
       <c r="AZ94" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="BA94" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="BB94" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="95">
@@ -16444,9 +16729,12 @@
         <v>0</v>
       </c>
       <c r="AZ95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA95" t="n">
         <v>7</v>
       </c>
-      <c r="BA95" t="n">
+      <c r="BB95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16611,10 +16899,13 @@
         <v>1</v>
       </c>
       <c r="AZ96" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="BA96" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="BB96" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="97">
@@ -16783,6 +17074,9 @@
       <c r="BA97" t="n">
         <v>0</v>
       </c>
+      <c r="BB97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -16945,10 +17239,13 @@
         <v>1</v>
       </c>
       <c r="AZ98" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BA98" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BB98" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="99">
@@ -17112,10 +17409,13 @@
         <v>1</v>
       </c>
       <c r="AZ99" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="BA99" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="BB99" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="100">
@@ -17284,6 +17584,9 @@
       <c r="BA100" t="n">
         <v>0</v>
       </c>
+      <c r="BB100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -17446,9 +17749,12 @@
         <v>1</v>
       </c>
       <c r="AZ101" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA101" t="n">
         <v>26</v>
       </c>
-      <c r="BA101" t="n">
+      <c r="BB101" t="n">
         <v>26</v>
       </c>
     </row>
@@ -17613,10 +17919,13 @@
         <v>1</v>
       </c>
       <c r="AZ102" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BA102" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BB102" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="103">
@@ -17780,10 +18089,13 @@
         <v>1</v>
       </c>
       <c r="AZ103" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BA103" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BB103" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="104">
@@ -17947,10 +18259,13 @@
         <v>0</v>
       </c>
       <c r="AZ104" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="BA104" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="BB104" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="105">
@@ -18114,10 +18429,13 @@
         <v>1</v>
       </c>
       <c r="AZ105" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="BA105" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="BB105" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="106">
@@ -18281,9 +18599,12 @@
         <v>0</v>
       </c>
       <c r="AZ106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA106" t="n">
         <v>7</v>
       </c>
-      <c r="BA106" t="n">
+      <c r="BB106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18448,9 +18769,12 @@
         <v>1</v>
       </c>
       <c r="AZ107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA107" t="n">
         <v>12</v>
       </c>
-      <c r="BA107" t="n">
+      <c r="BB107" t="n">
         <v>12</v>
       </c>
     </row>
@@ -18615,9 +18939,12 @@
         <v>0</v>
       </c>
       <c r="AZ108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA108" t="n">
         <v>2</v>
       </c>
-      <c r="BA108" t="n">
+      <c r="BB108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -18782,9 +19109,12 @@
         <v>0</v>
       </c>
       <c r="AZ109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA109" t="n">
         <v>4</v>
       </c>
-      <c r="BA109" t="n">
+      <c r="BB109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3728)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB109"/>
+  <dimension ref="A1:BC109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -482,8 +482,9 @@
     <col width="12" customWidth="1" min="50" max="50"/>
     <col width="12" customWidth="1" min="51" max="51"/>
     <col width="12" customWidth="1" min="52" max="52"/>
-    <col width="13" customWidth="1" min="53" max="53"/>
+    <col width="12" customWidth="1" min="53" max="53"/>
     <col width="13" customWidth="1" min="54" max="54"/>
+    <col width="13" customWidth="1" min="55" max="55"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -747,12 +748,17 @@
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="BA1" s="2" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="BB1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BB1" s="2" t="inlineStr">
+      <c r="BC1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -922,9 +928,12 @@
         <v>0</v>
       </c>
       <c r="BA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB2" t="n">
         <v>12</v>
       </c>
-      <c r="BB2" t="n">
+      <c r="BC2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1092,9 +1101,12 @@
         <v>0</v>
       </c>
       <c r="BA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB3" t="n">
         <v>9</v>
       </c>
-      <c r="BB3" t="n">
+      <c r="BC3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1262,10 +1274,13 @@
         <v>1</v>
       </c>
       <c r="BA4" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BB4" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="5">
@@ -1432,9 +1447,12 @@
         <v>0</v>
       </c>
       <c r="BA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB5" t="n">
         <v>15</v>
       </c>
-      <c r="BB5" t="n">
+      <c r="BC5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1602,10 +1620,13 @@
         <v>0</v>
       </c>
       <c r="BA6" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="BB6" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -1772,9 +1793,12 @@
         <v>1</v>
       </c>
       <c r="BA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB7" t="n">
         <v>19</v>
       </c>
-      <c r="BB7" t="n">
+      <c r="BC7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1942,10 +1966,13 @@
         <v>1</v>
       </c>
       <c r="BA8" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BB8" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="9">
@@ -2112,9 +2139,12 @@
         <v>1</v>
       </c>
       <c r="BA9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB9" t="n">
         <v>25</v>
       </c>
-      <c r="BB9" t="n">
+      <c r="BC9" t="n">
         <v>25</v>
       </c>
     </row>
@@ -2282,10 +2312,13 @@
         <v>1</v>
       </c>
       <c r="BA10" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BB10" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="11">
@@ -2452,10 +2485,13 @@
         <v>1</v>
       </c>
       <c r="BA11" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BB11" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BC11" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -2622,9 +2658,12 @@
         <v>1</v>
       </c>
       <c r="BA12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB12" t="n">
         <v>29</v>
       </c>
-      <c r="BB12" t="n">
+      <c r="BC12" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2792,9 +2831,12 @@
         <v>0</v>
       </c>
       <c r="BA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB13" t="n">
         <v>14</v>
       </c>
-      <c r="BB13" t="n">
+      <c r="BC13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2962,10 +3004,13 @@
         <v>0</v>
       </c>
       <c r="BA14" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BB14" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="15">
@@ -3132,9 +3177,12 @@
         <v>0</v>
       </c>
       <c r="BA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB15" t="n">
         <v>9</v>
       </c>
-      <c r="BB15" t="n">
+      <c r="BC15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3302,9 +3350,12 @@
         <v>0</v>
       </c>
       <c r="BA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB16" t="n">
         <v>20</v>
       </c>
-      <c r="BB16" t="n">
+      <c r="BC16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3472,9 +3523,12 @@
         <v>0</v>
       </c>
       <c r="BA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB17" t="n">
         <v>17</v>
       </c>
-      <c r="BB17" t="n">
+      <c r="BC17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3642,10 +3696,13 @@
         <v>1</v>
       </c>
       <c r="BA18" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BB18" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BC18" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="19">
@@ -3817,6 +3874,9 @@
       <c r="BB19" t="n">
         <v>0</v>
       </c>
+      <c r="BC19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3982,9 +4042,12 @@
         <v>0</v>
       </c>
       <c r="BA20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB20" t="n">
         <v>18</v>
       </c>
-      <c r="BB20" t="n">
+      <c r="BC20" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4152,10 +4215,13 @@
         <v>0</v>
       </c>
       <c r="BA21" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BB21" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BC21" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="22">
@@ -4327,6 +4393,9 @@
       <c r="BB22" t="n">
         <v>0</v>
       </c>
+      <c r="BC22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4492,10 +4561,13 @@
         <v>1</v>
       </c>
       <c r="BA23" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="BB23" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="BC23" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="24">
@@ -4662,10 +4734,13 @@
         <v>0</v>
       </c>
       <c r="BA24" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BB24" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BC24" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="25">
@@ -4832,9 +4907,12 @@
         <v>1</v>
       </c>
       <c r="BA25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB25" t="n">
         <v>10</v>
       </c>
-      <c r="BB25" t="n">
+      <c r="BC25" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5002,10 +5080,13 @@
         <v>1</v>
       </c>
       <c r="BA26" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BB26" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BC26" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="27">
@@ -5172,9 +5253,12 @@
         <v>0</v>
       </c>
       <c r="BA27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB27" t="n">
         <v>24</v>
       </c>
-      <c r="BB27" t="n">
+      <c r="BC27" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5342,10 +5426,13 @@
         <v>1</v>
       </c>
       <c r="BA28" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="BB28" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="29">
@@ -5512,9 +5599,12 @@
         <v>0</v>
       </c>
       <c r="BA29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB29" t="n">
         <v>11</v>
       </c>
-      <c r="BB29" t="n">
+      <c r="BC29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5682,10 +5772,13 @@
         <v>0</v>
       </c>
       <c r="BA30" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="BB30" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="BC30" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="31">
@@ -5852,10 +5945,13 @@
         <v>0</v>
       </c>
       <c r="BA31" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="BB31" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="32">
@@ -6022,10 +6118,13 @@
         <v>1</v>
       </c>
       <c r="BA32" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="BB32" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="33">
@@ -6192,10 +6291,13 @@
         <v>0</v>
       </c>
       <c r="BA33" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="BB33" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="BC33" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="34">
@@ -6362,9 +6464,12 @@
         <v>0</v>
       </c>
       <c r="BA34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB34" t="n">
         <v>9</v>
       </c>
-      <c r="BB34" t="n">
+      <c r="BC34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6532,10 +6637,13 @@
         <v>1</v>
       </c>
       <c r="BA35" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="BB35" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BC35" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="36">
@@ -6702,9 +6810,12 @@
         <v>1</v>
       </c>
       <c r="BA36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB36" t="n">
         <v>15</v>
       </c>
-      <c r="BB36" t="n">
+      <c r="BC36" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6877,6 +6988,9 @@
       <c r="BB37" t="n">
         <v>0</v>
       </c>
+      <c r="BC37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7042,9 +7156,12 @@
         <v>0</v>
       </c>
       <c r="BA38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB38" t="n">
         <v>2</v>
       </c>
-      <c r="BB38" t="n">
+      <c r="BC38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7212,10 +7329,13 @@
         <v>1</v>
       </c>
       <c r="BA39" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BB39" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BC39" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="40">
@@ -7382,9 +7502,12 @@
         <v>1</v>
       </c>
       <c r="BA40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB40" t="n">
         <v>23</v>
       </c>
-      <c r="BB40" t="n">
+      <c r="BC40" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7552,10 +7675,13 @@
         <v>1</v>
       </c>
       <c r="BA41" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BB41" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BC41" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="42">
@@ -7722,9 +7848,12 @@
         <v>0</v>
       </c>
       <c r="BA42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB42" t="n">
         <v>21</v>
       </c>
-      <c r="BB42" t="n">
+      <c r="BC42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7892,9 +8021,12 @@
         <v>0</v>
       </c>
       <c r="BA43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB43" t="n">
         <v>60</v>
       </c>
-      <c r="BB43" t="n">
+      <c r="BC43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8062,10 +8194,13 @@
         <v>0</v>
       </c>
       <c r="BA44" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="BB44" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="BC44" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="45">
@@ -8232,10 +8367,13 @@
         <v>0</v>
       </c>
       <c r="BA45" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="BB45" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BC45" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="46">
@@ -8402,10 +8540,13 @@
         <v>1</v>
       </c>
       <c r="BA46" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BB46" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BC46" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="47">
@@ -8577,6 +8718,9 @@
       <c r="BB47" t="n">
         <v>0</v>
       </c>
+      <c r="BC47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8742,9 +8886,12 @@
         <v>0</v>
       </c>
       <c r="BA48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB48" t="n">
         <v>25</v>
       </c>
-      <c r="BB48" t="n">
+      <c r="BC48" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8912,9 +9059,12 @@
         <v>0</v>
       </c>
       <c r="BA49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB49" t="n">
         <v>19</v>
       </c>
-      <c r="BB49" t="n">
+      <c r="BC49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9082,9 +9232,12 @@
         <v>0</v>
       </c>
       <c r="BA50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB50" t="n">
         <v>7</v>
       </c>
-      <c r="BB50" t="n">
+      <c r="BC50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9252,10 +9405,13 @@
         <v>1</v>
       </c>
       <c r="BA51" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BB51" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BC51" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="52">
@@ -9427,6 +9583,9 @@
       <c r="BB52" t="n">
         <v>0</v>
       </c>
+      <c r="BC52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9592,9 +9751,12 @@
         <v>0</v>
       </c>
       <c r="BA53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB53" t="n">
         <v>13</v>
       </c>
-      <c r="BB53" t="n">
+      <c r="BC53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9767,6 +9929,9 @@
       <c r="BB54" t="n">
         <v>0</v>
       </c>
+      <c r="BC54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9932,10 +10097,13 @@
         <v>1</v>
       </c>
       <c r="BA55" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BB55" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BC55" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="56">
@@ -10102,10 +10270,13 @@
         <v>0</v>
       </c>
       <c r="BA56" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BB56" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BC56" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="57">
@@ -10272,9 +10443,12 @@
         <v>0</v>
       </c>
       <c r="BA57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB57" t="n">
         <v>9</v>
       </c>
-      <c r="BB57" t="n">
+      <c r="BC57" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10442,9 +10616,12 @@
         <v>0</v>
       </c>
       <c r="BA58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB58" t="n">
         <v>12</v>
       </c>
-      <c r="BB58" t="n">
+      <c r="BC58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -10612,9 +10789,12 @@
         <v>0</v>
       </c>
       <c r="BA59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB59" t="n">
         <v>6</v>
       </c>
-      <c r="BB59" t="n">
+      <c r="BC59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10787,6 +10967,9 @@
       <c r="BB60" t="n">
         <v>0</v>
       </c>
+      <c r="BC60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10952,10 +11135,13 @@
         <v>1</v>
       </c>
       <c r="BA61" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BB61" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BC61" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="62">
@@ -11122,10 +11308,13 @@
         <v>1</v>
       </c>
       <c r="BA62" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BB62" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BC62" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="63">
@@ -11292,10 +11481,13 @@
         <v>0</v>
       </c>
       <c r="BA63" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="BB63" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="BC63" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="64">
@@ -11467,6 +11659,9 @@
       <c r="BB64" t="n">
         <v>0</v>
       </c>
+      <c r="BC64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -11632,10 +11827,13 @@
         <v>1</v>
       </c>
       <c r="BA65" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="BB65" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="BC65" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="66">
@@ -11802,10 +12000,13 @@
         <v>0</v>
       </c>
       <c r="BA66" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="BB66" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="BC66" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="67">
@@ -11972,10 +12173,13 @@
         <v>1</v>
       </c>
       <c r="BA67" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BB67" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BC67" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="68">
@@ -12142,9 +12346,12 @@
         <v>0</v>
       </c>
       <c r="BA68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB68" t="n">
         <v>19</v>
       </c>
-      <c r="BB68" t="n">
+      <c r="BC68" t="n">
         <v>18</v>
       </c>
     </row>
@@ -12312,9 +12519,12 @@
         <v>0</v>
       </c>
       <c r="BA69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB69" t="n">
         <v>7</v>
       </c>
-      <c r="BB69" t="n">
+      <c r="BC69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12482,9 +12692,12 @@
         <v>0</v>
       </c>
       <c r="BA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB70" t="n">
         <v>23</v>
       </c>
-      <c r="BB70" t="n">
+      <c r="BC70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -12652,10 +12865,13 @@
         <v>1</v>
       </c>
       <c r="BA71" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="BB71" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="BC71" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="72">
@@ -12822,10 +13038,13 @@
         <v>1</v>
       </c>
       <c r="BA72" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="BB72" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="BC72" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="73">
@@ -12997,6 +13216,9 @@
       <c r="BB73" t="n">
         <v>0</v>
       </c>
+      <c r="BC73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -13167,6 +13389,9 @@
       <c r="BB74" t="n">
         <v>0</v>
       </c>
+      <c r="BC74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -13332,10 +13557,13 @@
         <v>1</v>
       </c>
       <c r="BA75" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="BB75" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="BC75" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="76">
@@ -13502,9 +13730,12 @@
         <v>0</v>
       </c>
       <c r="BA76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB76" t="n">
         <v>20</v>
       </c>
-      <c r="BB76" t="n">
+      <c r="BC76" t="n">
         <v>20</v>
       </c>
     </row>
@@ -13672,9 +13903,12 @@
         <v>0</v>
       </c>
       <c r="BA77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB77" t="n">
         <v>15</v>
       </c>
-      <c r="BB77" t="n">
+      <c r="BC77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -13842,10 +14076,13 @@
         <v>1</v>
       </c>
       <c r="BA78" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BB78" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BC78" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="79">
@@ -14012,10 +14249,13 @@
         <v>0</v>
       </c>
       <c r="BA79" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="BB79" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="BC79" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="80">
@@ -14182,9 +14422,12 @@
         <v>0</v>
       </c>
       <c r="BA80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB80" t="n">
         <v>11</v>
       </c>
-      <c r="BB80" t="n">
+      <c r="BC80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -14352,9 +14595,12 @@
         <v>0</v>
       </c>
       <c r="BA81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB81" t="n">
         <v>4</v>
       </c>
-      <c r="BB81" t="n">
+      <c r="BC81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -14522,10 +14768,13 @@
         <v>1</v>
       </c>
       <c r="BA82" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="BB82" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="BC82" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="83">
@@ -14692,9 +14941,12 @@
         <v>0</v>
       </c>
       <c r="BA83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB83" t="n">
         <v>17</v>
       </c>
-      <c r="BB83" t="n">
+      <c r="BC83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -14862,9 +15114,12 @@
         <v>0</v>
       </c>
       <c r="BA84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB84" t="n">
         <v>13</v>
       </c>
-      <c r="BB84" t="n">
+      <c r="BC84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -15032,9 +15287,12 @@
         <v>0</v>
       </c>
       <c r="BA85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB85" t="n">
         <v>7</v>
       </c>
-      <c r="BB85" t="n">
+      <c r="BC85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15207,6 +15465,9 @@
       <c r="BB86" t="n">
         <v>0</v>
       </c>
+      <c r="BC86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -15372,9 +15633,12 @@
         <v>1</v>
       </c>
       <c r="BA87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB87" t="n">
         <v>18</v>
       </c>
-      <c r="BB87" t="n">
+      <c r="BC87" t="n">
         <v>18</v>
       </c>
     </row>
@@ -15547,6 +15811,9 @@
       <c r="BB88" t="n">
         <v>0</v>
       </c>
+      <c r="BC88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -15712,9 +15979,12 @@
         <v>0</v>
       </c>
       <c r="BA89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB89" t="n">
         <v>17</v>
       </c>
-      <c r="BB89" t="n">
+      <c r="BC89" t="n">
         <v>17</v>
       </c>
     </row>
@@ -15882,10 +16152,13 @@
         <v>0</v>
       </c>
       <c r="BA90" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="BB90" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="BC90" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="91">
@@ -16052,9 +16325,12 @@
         <v>0</v>
       </c>
       <c r="BA91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB91" t="n">
         <v>42</v>
       </c>
-      <c r="BB91" t="n">
+      <c r="BC91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -16222,9 +16498,12 @@
         <v>0</v>
       </c>
       <c r="BA92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB92" t="n">
         <v>7</v>
       </c>
-      <c r="BB92" t="n">
+      <c r="BC92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16397,6 +16676,9 @@
       <c r="BB93" t="n">
         <v>0</v>
       </c>
+      <c r="BC93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -16562,9 +16844,12 @@
         <v>1</v>
       </c>
       <c r="BA94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB94" t="n">
         <v>16</v>
       </c>
-      <c r="BB94" t="n">
+      <c r="BC94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -16732,9 +17017,12 @@
         <v>0</v>
       </c>
       <c r="BA95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB95" t="n">
         <v>7</v>
       </c>
-      <c r="BB95" t="n">
+      <c r="BC95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16902,9 +17190,12 @@
         <v>1</v>
       </c>
       <c r="BA96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB96" t="n">
         <v>23</v>
       </c>
-      <c r="BB96" t="n">
+      <c r="BC96" t="n">
         <v>23</v>
       </c>
     </row>
@@ -17077,6 +17368,9 @@
       <c r="BB97" t="n">
         <v>0</v>
       </c>
+      <c r="BC97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -17242,10 +17536,13 @@
         <v>1</v>
       </c>
       <c r="BA98" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BB98" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BC98" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="99">
@@ -17412,10 +17709,13 @@
         <v>1</v>
       </c>
       <c r="BA99" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="BB99" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="BC99" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="100">
@@ -17587,6 +17887,9 @@
       <c r="BB100" t="n">
         <v>0</v>
       </c>
+      <c r="BC100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -17752,10 +18055,13 @@
         <v>0</v>
       </c>
       <c r="BA101" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BB101" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BC101" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="102">
@@ -17922,9 +18228,12 @@
         <v>1</v>
       </c>
       <c r="BA102" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB102" t="n">
         <v>26</v>
       </c>
-      <c r="BB102" t="n">
+      <c r="BC102" t="n">
         <v>26</v>
       </c>
     </row>
@@ -18092,10 +18401,13 @@
         <v>1</v>
       </c>
       <c r="BA103" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BB103" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BC103" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="104">
@@ -18262,9 +18574,12 @@
         <v>1</v>
       </c>
       <c r="BA104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB104" t="n">
         <v>12</v>
       </c>
-      <c r="BB104" t="n">
+      <c r="BC104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -18432,10 +18747,13 @@
         <v>1</v>
       </c>
       <c r="BA105" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="BB105" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="BC105" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="106">
@@ -18602,9 +18920,12 @@
         <v>0</v>
       </c>
       <c r="BA106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB106" t="n">
         <v>7</v>
       </c>
-      <c r="BB106" t="n">
+      <c r="BC106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18772,10 +19093,13 @@
         <v>0</v>
       </c>
       <c r="BA107" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="BB107" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="BC107" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="108">
@@ -18942,9 +19266,12 @@
         <v>0</v>
       </c>
       <c r="BA108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB108" t="n">
         <v>2</v>
       </c>
-      <c r="BB108" t="n">
+      <c r="BC108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -19112,9 +19439,12 @@
         <v>0</v>
       </c>
       <c r="BA109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB109" t="n">
         <v>4</v>
       </c>
-      <c r="BB109" t="n">
+      <c r="BC109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3785)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC109"/>
+  <dimension ref="A1:BD109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -483,8 +483,9 @@
     <col width="12" customWidth="1" min="51" max="51"/>
     <col width="12" customWidth="1" min="52" max="52"/>
     <col width="12" customWidth="1" min="53" max="53"/>
-    <col width="13" customWidth="1" min="54" max="54"/>
+    <col width="12" customWidth="1" min="54" max="54"/>
     <col width="13" customWidth="1" min="55" max="55"/>
+    <col width="13" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -753,12 +754,17 @@
           <t>2026-04-16</t>
         </is>
       </c>
-      <c r="BB1" s="2" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="BC1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BC1" s="2" t="inlineStr">
+      <c r="BD1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -931,9 +937,12 @@
         <v>0</v>
       </c>
       <c r="BB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC2" t="n">
         <v>12</v>
       </c>
-      <c r="BC2" t="n">
+      <c r="BD2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1104,9 +1113,12 @@
         <v>0</v>
       </c>
       <c r="BB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC3" t="n">
         <v>9</v>
       </c>
-      <c r="BC3" t="n">
+      <c r="BD3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1277,9 +1289,12 @@
         <v>1</v>
       </c>
       <c r="BB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC4" t="n">
         <v>31</v>
       </c>
-      <c r="BC4" t="n">
+      <c r="BD4" t="n">
         <v>31</v>
       </c>
     </row>
@@ -1450,9 +1465,12 @@
         <v>0</v>
       </c>
       <c r="BB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC5" t="n">
         <v>15</v>
       </c>
-      <c r="BC5" t="n">
+      <c r="BD5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1623,9 +1641,12 @@
         <v>1</v>
       </c>
       <c r="BB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC6" t="n">
         <v>19</v>
       </c>
-      <c r="BC6" t="n">
+      <c r="BD6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1796,9 +1817,12 @@
         <v>0</v>
       </c>
       <c r="BB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC7" t="n">
         <v>19</v>
       </c>
-      <c r="BC7" t="n">
+      <c r="BD7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1969,9 +1993,12 @@
         <v>1</v>
       </c>
       <c r="BB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC8" t="n">
         <v>29</v>
       </c>
-      <c r="BC8" t="n">
+      <c r="BD8" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2142,9 +2169,12 @@
         <v>0</v>
       </c>
       <c r="BB9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC9" t="n">
         <v>25</v>
       </c>
-      <c r="BC9" t="n">
+      <c r="BD9" t="n">
         <v>25</v>
       </c>
     </row>
@@ -2315,9 +2345,12 @@
         <v>1</v>
       </c>
       <c r="BB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC10" t="n">
         <v>31</v>
       </c>
-      <c r="BC10" t="n">
+      <c r="BD10" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2488,9 +2521,12 @@
         <v>1</v>
       </c>
       <c r="BB11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC11" t="n">
         <v>26</v>
       </c>
-      <c r="BC11" t="n">
+      <c r="BD11" t="n">
         <v>26</v>
       </c>
     </row>
@@ -2661,9 +2697,12 @@
         <v>0</v>
       </c>
       <c r="BB12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC12" t="n">
         <v>29</v>
       </c>
-      <c r="BC12" t="n">
+      <c r="BD12" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2834,9 +2873,12 @@
         <v>0</v>
       </c>
       <c r="BB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC13" t="n">
         <v>14</v>
       </c>
-      <c r="BC13" t="n">
+      <c r="BD13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3007,9 +3049,12 @@
         <v>1</v>
       </c>
       <c r="BB14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC14" t="n">
         <v>25</v>
       </c>
-      <c r="BC14" t="n">
+      <c r="BD14" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3180,9 +3225,12 @@
         <v>0</v>
       </c>
       <c r="BB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC15" t="n">
         <v>9</v>
       </c>
-      <c r="BC15" t="n">
+      <c r="BD15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3353,9 +3401,12 @@
         <v>0</v>
       </c>
       <c r="BB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC16" t="n">
         <v>20</v>
       </c>
-      <c r="BC16" t="n">
+      <c r="BD16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3526,9 +3577,12 @@
         <v>0</v>
       </c>
       <c r="BB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC17" t="n">
         <v>17</v>
       </c>
-      <c r="BC17" t="n">
+      <c r="BD17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3699,9 +3753,12 @@
         <v>1</v>
       </c>
       <c r="BB18" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC18" t="n">
         <v>27</v>
       </c>
-      <c r="BC18" t="n">
+      <c r="BD18" t="n">
         <v>27</v>
       </c>
     </row>
@@ -3877,6 +3934,9 @@
       <c r="BC19" t="n">
         <v>0</v>
       </c>
+      <c r="BD19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4045,9 +4105,12 @@
         <v>0</v>
       </c>
       <c r="BB20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC20" t="n">
         <v>18</v>
       </c>
-      <c r="BC20" t="n">
+      <c r="BD20" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4218,9 +4281,12 @@
         <v>1</v>
       </c>
       <c r="BB21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC21" t="n">
         <v>25</v>
       </c>
-      <c r="BC21" t="n">
+      <c r="BD21" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4396,6 +4462,9 @@
       <c r="BC22" t="n">
         <v>0</v>
       </c>
+      <c r="BD22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4564,9 +4633,12 @@
         <v>1</v>
       </c>
       <c r="BB23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC23" t="n">
         <v>20</v>
       </c>
-      <c r="BC23" t="n">
+      <c r="BD23" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4737,9 +4809,12 @@
         <v>1</v>
       </c>
       <c r="BB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC24" t="n">
         <v>25</v>
       </c>
-      <c r="BC24" t="n">
+      <c r="BD24" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4910,9 +4985,12 @@
         <v>0</v>
       </c>
       <c r="BB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC25" t="n">
         <v>10</v>
       </c>
-      <c r="BC25" t="n">
+      <c r="BD25" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5083,9 +5161,12 @@
         <v>1</v>
       </c>
       <c r="BB26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC26" t="n">
         <v>27</v>
       </c>
-      <c r="BC26" t="n">
+      <c r="BD26" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5256,9 +5337,12 @@
         <v>0</v>
       </c>
       <c r="BB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC27" t="n">
         <v>24</v>
       </c>
-      <c r="BC27" t="n">
+      <c r="BD27" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5429,9 +5513,12 @@
         <v>1</v>
       </c>
       <c r="BB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC28" t="n">
         <v>18</v>
       </c>
-      <c r="BC28" t="n">
+      <c r="BD28" t="n">
         <v>18</v>
       </c>
     </row>
@@ -5602,9 +5689,12 @@
         <v>0</v>
       </c>
       <c r="BB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC29" t="n">
         <v>11</v>
       </c>
-      <c r="BC29" t="n">
+      <c r="BD29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5775,10 +5865,13 @@
         <v>1</v>
       </c>
       <c r="BB30" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="BC30" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BD30" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="31">
@@ -5948,9 +6041,12 @@
         <v>1</v>
       </c>
       <c r="BB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC31" t="n">
         <v>20</v>
       </c>
-      <c r="BC31" t="n">
+      <c r="BD31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6121,10 +6217,13 @@
         <v>1</v>
       </c>
       <c r="BB32" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="BC32" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="BD32" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="33">
@@ -6294,9 +6393,12 @@
         <v>1</v>
       </c>
       <c r="BB33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC33" t="n">
         <v>16</v>
       </c>
-      <c r="BC33" t="n">
+      <c r="BD33" t="n">
         <v>16</v>
       </c>
     </row>
@@ -6467,9 +6569,12 @@
         <v>0</v>
       </c>
       <c r="BB34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC34" t="n">
         <v>9</v>
       </c>
-      <c r="BC34" t="n">
+      <c r="BD34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6640,9 +6745,12 @@
         <v>1</v>
       </c>
       <c r="BB35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC35" t="n">
         <v>24</v>
       </c>
-      <c r="BC35" t="n">
+      <c r="BD35" t="n">
         <v>24</v>
       </c>
     </row>
@@ -6813,9 +6921,12 @@
         <v>0</v>
       </c>
       <c r="BB36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC36" t="n">
         <v>15</v>
       </c>
-      <c r="BC36" t="n">
+      <c r="BD36" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6991,6 +7102,9 @@
       <c r="BC37" t="n">
         <v>0</v>
       </c>
+      <c r="BD37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7159,9 +7273,12 @@
         <v>0</v>
       </c>
       <c r="BB38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC38" t="n">
         <v>2</v>
       </c>
-      <c r="BC38" t="n">
+      <c r="BD38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7332,9 +7449,12 @@
         <v>1</v>
       </c>
       <c r="BB39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC39" t="n">
         <v>30</v>
       </c>
-      <c r="BC39" t="n">
+      <c r="BD39" t="n">
         <v>30</v>
       </c>
     </row>
@@ -7505,9 +7625,12 @@
         <v>0</v>
       </c>
       <c r="BB40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC40" t="n">
         <v>23</v>
       </c>
-      <c r="BC40" t="n">
+      <c r="BD40" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7678,9 +7801,12 @@
         <v>1</v>
       </c>
       <c r="BB41" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC41" t="n">
         <v>30</v>
       </c>
-      <c r="BC41" t="n">
+      <c r="BD41" t="n">
         <v>30</v>
       </c>
     </row>
@@ -7851,9 +7977,12 @@
         <v>0</v>
       </c>
       <c r="BB42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC42" t="n">
         <v>21</v>
       </c>
-      <c r="BC42" t="n">
+      <c r="BD42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8024,9 +8153,12 @@
         <v>0</v>
       </c>
       <c r="BB43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC43" t="n">
         <v>60</v>
       </c>
-      <c r="BC43" t="n">
+      <c r="BD43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8197,9 +8329,12 @@
         <v>1</v>
       </c>
       <c r="BB44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC44" t="n">
         <v>23</v>
       </c>
-      <c r="BC44" t="n">
+      <c r="BD44" t="n">
         <v>23</v>
       </c>
     </row>
@@ -8370,9 +8505,12 @@
         <v>1</v>
       </c>
       <c r="BB45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC45" t="n">
         <v>24</v>
       </c>
-      <c r="BC45" t="n">
+      <c r="BD45" t="n">
         <v>24</v>
       </c>
     </row>
@@ -8543,9 +8681,12 @@
         <v>1</v>
       </c>
       <c r="BB46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC46" t="n">
         <v>26</v>
       </c>
-      <c r="BC46" t="n">
+      <c r="BD46" t="n">
         <v>26</v>
       </c>
     </row>
@@ -8721,6 +8862,9 @@
       <c r="BC47" t="n">
         <v>0</v>
       </c>
+      <c r="BD47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8889,9 +9033,12 @@
         <v>0</v>
       </c>
       <c r="BB48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC48" t="n">
         <v>25</v>
       </c>
-      <c r="BC48" t="n">
+      <c r="BD48" t="n">
         <v>25</v>
       </c>
     </row>
@@ -9062,9 +9209,12 @@
         <v>0</v>
       </c>
       <c r="BB49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC49" t="n">
         <v>19</v>
       </c>
-      <c r="BC49" t="n">
+      <c r="BD49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9235,9 +9385,12 @@
         <v>0</v>
       </c>
       <c r="BB50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC50" t="n">
         <v>7</v>
       </c>
-      <c r="BC50" t="n">
+      <c r="BD50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9408,9 +9561,12 @@
         <v>1</v>
       </c>
       <c r="BB51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC51" t="n">
         <v>29</v>
       </c>
-      <c r="BC51" t="n">
+      <c r="BD51" t="n">
         <v>29</v>
       </c>
     </row>
@@ -9586,6 +9742,9 @@
       <c r="BC52" t="n">
         <v>0</v>
       </c>
+      <c r="BD52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9754,9 +9913,12 @@
         <v>0</v>
       </c>
       <c r="BB53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC53" t="n">
         <v>13</v>
       </c>
-      <c r="BC53" t="n">
+      <c r="BD53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9932,6 +10094,9 @@
       <c r="BC54" t="n">
         <v>0</v>
       </c>
+      <c r="BD54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10100,9 +10265,12 @@
         <v>1</v>
       </c>
       <c r="BB55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC55" t="n">
         <v>31</v>
       </c>
-      <c r="BC55" t="n">
+      <c r="BD55" t="n">
         <v>31</v>
       </c>
     </row>
@@ -10273,9 +10441,12 @@
         <v>1</v>
       </c>
       <c r="BB56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC56" t="n">
         <v>27</v>
       </c>
-      <c r="BC56" t="n">
+      <c r="BD56" t="n">
         <v>27</v>
       </c>
     </row>
@@ -10446,9 +10617,12 @@
         <v>0</v>
       </c>
       <c r="BB57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC57" t="n">
         <v>9</v>
       </c>
-      <c r="BC57" t="n">
+      <c r="BD57" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10619,9 +10793,12 @@
         <v>0</v>
       </c>
       <c r="BB58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC58" t="n">
         <v>12</v>
       </c>
-      <c r="BC58" t="n">
+      <c r="BD58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -10792,9 +10969,12 @@
         <v>0</v>
       </c>
       <c r="BB59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC59" t="n">
         <v>6</v>
       </c>
-      <c r="BC59" t="n">
+      <c r="BD59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10970,6 +11150,9 @@
       <c r="BC60" t="n">
         <v>0</v>
       </c>
+      <c r="BD60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -11138,9 +11321,12 @@
         <v>1</v>
       </c>
       <c r="BB61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC61" t="n">
         <v>27</v>
       </c>
-      <c r="BC61" t="n">
+      <c r="BD61" t="n">
         <v>27</v>
       </c>
     </row>
@@ -11311,9 +11497,12 @@
         <v>1</v>
       </c>
       <c r="BB62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC62" t="n">
         <v>27</v>
       </c>
-      <c r="BC62" t="n">
+      <c r="BD62" t="n">
         <v>27</v>
       </c>
     </row>
@@ -11484,9 +11673,12 @@
         <v>1</v>
       </c>
       <c r="BB63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC63" t="n">
         <v>11</v>
       </c>
-      <c r="BC63" t="n">
+      <c r="BD63" t="n">
         <v>11</v>
       </c>
     </row>
@@ -11662,6 +11854,9 @@
       <c r="BC64" t="n">
         <v>0</v>
       </c>
+      <c r="BD64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -11830,9 +12025,12 @@
         <v>1</v>
       </c>
       <c r="BB65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC65" t="n">
         <v>16</v>
       </c>
-      <c r="BC65" t="n">
+      <c r="BD65" t="n">
         <v>16</v>
       </c>
     </row>
@@ -12003,9 +12201,12 @@
         <v>1</v>
       </c>
       <c r="BB66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC66" t="n">
         <v>8</v>
       </c>
-      <c r="BC66" t="n">
+      <c r="BD66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -12176,9 +12377,12 @@
         <v>1</v>
       </c>
       <c r="BB67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC67" t="n">
         <v>31</v>
       </c>
-      <c r="BC67" t="n">
+      <c r="BD67" t="n">
         <v>31</v>
       </c>
     </row>
@@ -12349,9 +12553,12 @@
         <v>0</v>
       </c>
       <c r="BB68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC68" t="n">
         <v>19</v>
       </c>
-      <c r="BC68" t="n">
+      <c r="BD68" t="n">
         <v>18</v>
       </c>
     </row>
@@ -12522,9 +12729,12 @@
         <v>0</v>
       </c>
       <c r="BB69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC69" t="n">
         <v>7</v>
       </c>
-      <c r="BC69" t="n">
+      <c r="BD69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12695,9 +12905,12 @@
         <v>0</v>
       </c>
       <c r="BB70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC70" t="n">
         <v>23</v>
       </c>
-      <c r="BC70" t="n">
+      <c r="BD70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -12868,9 +13081,12 @@
         <v>1</v>
       </c>
       <c r="BB71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC71" t="n">
         <v>22</v>
       </c>
-      <c r="BC71" t="n">
+      <c r="BD71" t="n">
         <v>22</v>
       </c>
     </row>
@@ -13041,9 +13257,12 @@
         <v>1</v>
       </c>
       <c r="BB72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC72" t="n">
         <v>22</v>
       </c>
-      <c r="BC72" t="n">
+      <c r="BD72" t="n">
         <v>22</v>
       </c>
     </row>
@@ -13219,6 +13438,9 @@
       <c r="BC73" t="n">
         <v>0</v>
       </c>
+      <c r="BD73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -13392,6 +13614,9 @@
       <c r="BC74" t="n">
         <v>0</v>
       </c>
+      <c r="BD74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -13560,9 +13785,12 @@
         <v>1</v>
       </c>
       <c r="BB75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC75" t="n">
         <v>22</v>
       </c>
-      <c r="BC75" t="n">
+      <c r="BD75" t="n">
         <v>22</v>
       </c>
     </row>
@@ -13733,9 +13961,12 @@
         <v>0</v>
       </c>
       <c r="BB76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC76" t="n">
         <v>20</v>
       </c>
-      <c r="BC76" t="n">
+      <c r="BD76" t="n">
         <v>20</v>
       </c>
     </row>
@@ -13906,9 +14137,12 @@
         <v>0</v>
       </c>
       <c r="BB77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC77" t="n">
         <v>15</v>
       </c>
-      <c r="BC77" t="n">
+      <c r="BD77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -14079,9 +14313,12 @@
         <v>1</v>
       </c>
       <c r="BB78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC78" t="n">
         <v>28</v>
       </c>
-      <c r="BC78" t="n">
+      <c r="BD78" t="n">
         <v>28</v>
       </c>
     </row>
@@ -14252,9 +14489,12 @@
         <v>1</v>
       </c>
       <c r="BB79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC79" t="n">
         <v>22</v>
       </c>
-      <c r="BC79" t="n">
+      <c r="BD79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -14425,9 +14665,12 @@
         <v>0</v>
       </c>
       <c r="BB80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC80" t="n">
         <v>11</v>
       </c>
-      <c r="BC80" t="n">
+      <c r="BD80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -14598,9 +14841,12 @@
         <v>0</v>
       </c>
       <c r="BB81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC81" t="n">
         <v>4</v>
       </c>
-      <c r="BC81" t="n">
+      <c r="BD81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -14771,9 +15017,12 @@
         <v>1</v>
       </c>
       <c r="BB82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC82" t="n">
         <v>14</v>
       </c>
-      <c r="BC82" t="n">
+      <c r="BD82" t="n">
         <v>14</v>
       </c>
     </row>
@@ -14944,9 +15193,12 @@
         <v>0</v>
       </c>
       <c r="BB83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC83" t="n">
         <v>17</v>
       </c>
-      <c r="BC83" t="n">
+      <c r="BD83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -15117,9 +15369,12 @@
         <v>0</v>
       </c>
       <c r="BB84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC84" t="n">
         <v>13</v>
       </c>
-      <c r="BC84" t="n">
+      <c r="BD84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -15290,9 +15545,12 @@
         <v>0</v>
       </c>
       <c r="BB85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC85" t="n">
         <v>7</v>
       </c>
-      <c r="BC85" t="n">
+      <c r="BD85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15468,6 +15726,9 @@
       <c r="BC86" t="n">
         <v>0</v>
       </c>
+      <c r="BD86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -15636,9 +15897,12 @@
         <v>0</v>
       </c>
       <c r="BB87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC87" t="n">
         <v>18</v>
       </c>
-      <c r="BC87" t="n">
+      <c r="BD87" t="n">
         <v>18</v>
       </c>
     </row>
@@ -15814,6 +16078,9 @@
       <c r="BC88" t="n">
         <v>0</v>
       </c>
+      <c r="BD88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -15982,9 +16249,12 @@
         <v>0</v>
       </c>
       <c r="BB89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC89" t="n">
         <v>17</v>
       </c>
-      <c r="BC89" t="n">
+      <c r="BD89" t="n">
         <v>17</v>
       </c>
     </row>
@@ -16155,9 +16425,12 @@
         <v>1</v>
       </c>
       <c r="BB90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC90" t="n">
         <v>16</v>
       </c>
-      <c r="BC90" t="n">
+      <c r="BD90" t="n">
         <v>16</v>
       </c>
     </row>
@@ -16328,9 +16601,12 @@
         <v>0</v>
       </c>
       <c r="BB91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC91" t="n">
         <v>42</v>
       </c>
-      <c r="BC91" t="n">
+      <c r="BD91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -16501,9 +16777,12 @@
         <v>0</v>
       </c>
       <c r="BB92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC92" t="n">
         <v>7</v>
       </c>
-      <c r="BC92" t="n">
+      <c r="BD92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16679,6 +16958,9 @@
       <c r="BC93" t="n">
         <v>0</v>
       </c>
+      <c r="BD93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -16847,9 +17129,12 @@
         <v>0</v>
       </c>
       <c r="BB94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC94" t="n">
         <v>16</v>
       </c>
-      <c r="BC94" t="n">
+      <c r="BD94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -17020,9 +17305,12 @@
         <v>0</v>
       </c>
       <c r="BB95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC95" t="n">
         <v>7</v>
       </c>
-      <c r="BC95" t="n">
+      <c r="BD95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17193,9 +17481,12 @@
         <v>0</v>
       </c>
       <c r="BB96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC96" t="n">
         <v>23</v>
       </c>
-      <c r="BC96" t="n">
+      <c r="BD96" t="n">
         <v>23</v>
       </c>
     </row>
@@ -17371,6 +17662,9 @@
       <c r="BC97" t="n">
         <v>0</v>
       </c>
+      <c r="BD97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -17539,9 +17833,12 @@
         <v>1</v>
       </c>
       <c r="BB98" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC98" t="n">
         <v>29</v>
       </c>
-      <c r="BC98" t="n">
+      <c r="BD98" t="n">
         <v>29</v>
       </c>
     </row>
@@ -17712,9 +18009,12 @@
         <v>1</v>
       </c>
       <c r="BB99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC99" t="n">
         <v>13</v>
       </c>
-      <c r="BC99" t="n">
+      <c r="BD99" t="n">
         <v>13</v>
       </c>
     </row>
@@ -17890,6 +18190,9 @@
       <c r="BC100" t="n">
         <v>0</v>
       </c>
+      <c r="BD100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -18058,9 +18361,12 @@
         <v>1</v>
       </c>
       <c r="BB101" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC101" t="n">
         <v>27</v>
       </c>
-      <c r="BC101" t="n">
+      <c r="BD101" t="n">
         <v>27</v>
       </c>
     </row>
@@ -18231,9 +18537,12 @@
         <v>0</v>
       </c>
       <c r="BB102" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC102" t="n">
         <v>26</v>
       </c>
-      <c r="BC102" t="n">
+      <c r="BD102" t="n">
         <v>26</v>
       </c>
     </row>
@@ -18404,10 +18713,13 @@
         <v>1</v>
       </c>
       <c r="BB103" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BC103" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BD103" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="104">
@@ -18577,9 +18889,12 @@
         <v>0</v>
       </c>
       <c r="BB104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC104" t="n">
         <v>12</v>
       </c>
-      <c r="BC104" t="n">
+      <c r="BD104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -18750,9 +19065,12 @@
         <v>1</v>
       </c>
       <c r="BB105" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC105" t="n">
         <v>21</v>
       </c>
-      <c r="BC105" t="n">
+      <c r="BD105" t="n">
         <v>21</v>
       </c>
     </row>
@@ -18923,9 +19241,12 @@
         <v>0</v>
       </c>
       <c r="BB106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC106" t="n">
         <v>7</v>
       </c>
-      <c r="BC106" t="n">
+      <c r="BD106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -19096,9 +19417,12 @@
         <v>1</v>
       </c>
       <c r="BB107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC107" t="n">
         <v>13</v>
       </c>
-      <c r="BC107" t="n">
+      <c r="BD107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -19269,9 +19593,12 @@
         <v>0</v>
       </c>
       <c r="BB108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC108" t="n">
         <v>2</v>
       </c>
-      <c r="BC108" t="n">
+      <c r="BD108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -19442,9 +19769,12 @@
         <v>0</v>
       </c>
       <c r="BB109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC109" t="n">
         <v>4</v>
       </c>
-      <c r="BC109" t="n">
+      <c r="BD109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3898)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD109"/>
+  <dimension ref="A1:BE109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -484,8 +484,9 @@
     <col width="12" customWidth="1" min="52" max="52"/>
     <col width="12" customWidth="1" min="53" max="53"/>
     <col width="12" customWidth="1" min="54" max="54"/>
-    <col width="13" customWidth="1" min="55" max="55"/>
+    <col width="12" customWidth="1" min="55" max="55"/>
     <col width="13" customWidth="1" min="56" max="56"/>
+    <col width="13" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -759,12 +760,17 @@
           <t>2026-04-19</t>
         </is>
       </c>
-      <c r="BC1" s="2" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="BD1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BD1" s="2" t="inlineStr">
+      <c r="BE1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -940,9 +946,12 @@
         <v>0</v>
       </c>
       <c r="BC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD2" t="n">
         <v>12</v>
       </c>
-      <c r="BD2" t="n">
+      <c r="BE2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1116,10 +1125,13 @@
         <v>0</v>
       </c>
       <c r="BC3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="BD3" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -1292,10 +1304,13 @@
         <v>0</v>
       </c>
       <c r="BC4" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BD4" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="5">
@@ -1468,9 +1483,12 @@
         <v>0</v>
       </c>
       <c r="BC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD5" t="n">
         <v>15</v>
       </c>
-      <c r="BD5" t="n">
+      <c r="BE5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1644,9 +1662,12 @@
         <v>0</v>
       </c>
       <c r="BC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD6" t="n">
         <v>19</v>
       </c>
-      <c r="BD6" t="n">
+      <c r="BE6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1820,9 +1841,12 @@
         <v>0</v>
       </c>
       <c r="BC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD7" t="n">
         <v>19</v>
       </c>
-      <c r="BD7" t="n">
+      <c r="BE7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1996,9 +2020,12 @@
         <v>0</v>
       </c>
       <c r="BC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD8" t="n">
         <v>29</v>
       </c>
-      <c r="BD8" t="n">
+      <c r="BE8" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2172,9 +2199,12 @@
         <v>0</v>
       </c>
       <c r="BC9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD9" t="n">
         <v>25</v>
       </c>
-      <c r="BD9" t="n">
+      <c r="BE9" t="n">
         <v>25</v>
       </c>
     </row>
@@ -2348,10 +2378,13 @@
         <v>0</v>
       </c>
       <c r="BC10" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BD10" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="11">
@@ -2524,9 +2557,12 @@
         <v>0</v>
       </c>
       <c r="BC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD11" t="n">
         <v>26</v>
       </c>
-      <c r="BD11" t="n">
+      <c r="BE11" t="n">
         <v>26</v>
       </c>
     </row>
@@ -2700,10 +2736,13 @@
         <v>0</v>
       </c>
       <c r="BC12" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BD12" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BE12" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="13">
@@ -2876,9 +2915,12 @@
         <v>0</v>
       </c>
       <c r="BC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD13" t="n">
         <v>14</v>
       </c>
-      <c r="BD13" t="n">
+      <c r="BE13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3052,9 +3094,12 @@
         <v>0</v>
       </c>
       <c r="BC14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD14" t="n">
         <v>25</v>
       </c>
-      <c r="BD14" t="n">
+      <c r="BE14" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3228,9 +3273,12 @@
         <v>0</v>
       </c>
       <c r="BC15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD15" t="n">
         <v>9</v>
       </c>
-      <c r="BD15" t="n">
+      <c r="BE15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3404,9 +3452,12 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD16" t="n">
         <v>20</v>
       </c>
-      <c r="BD16" t="n">
+      <c r="BE16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3580,9 +3631,12 @@
         <v>0</v>
       </c>
       <c r="BC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD17" t="n">
         <v>17</v>
       </c>
-      <c r="BD17" t="n">
+      <c r="BE17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3756,10 +3810,13 @@
         <v>0</v>
       </c>
       <c r="BC18" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BD18" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BE18" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="19">
@@ -3937,6 +3994,9 @@
       <c r="BD19" t="n">
         <v>0</v>
       </c>
+      <c r="BE19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4108,9 +4168,12 @@
         <v>0</v>
       </c>
       <c r="BC20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD20" t="n">
         <v>18</v>
       </c>
-      <c r="BD20" t="n">
+      <c r="BE20" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4284,10 +4347,13 @@
         <v>0</v>
       </c>
       <c r="BC21" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BD21" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BE21" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="22">
@@ -4465,6 +4531,9 @@
       <c r="BD22" t="n">
         <v>0</v>
       </c>
+      <c r="BE22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4636,9 +4705,12 @@
         <v>0</v>
       </c>
       <c r="BC23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD23" t="n">
         <v>20</v>
       </c>
-      <c r="BD23" t="n">
+      <c r="BE23" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4812,10 +4884,13 @@
         <v>0</v>
       </c>
       <c r="BC24" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BD24" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BE24" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="25">
@@ -4988,9 +5063,12 @@
         <v>0</v>
       </c>
       <c r="BC25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD25" t="n">
         <v>10</v>
       </c>
-      <c r="BD25" t="n">
+      <c r="BE25" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5164,10 +5242,13 @@
         <v>0</v>
       </c>
       <c r="BC26" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BD26" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BE26" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="27">
@@ -5340,9 +5421,12 @@
         <v>0</v>
       </c>
       <c r="BC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD27" t="n">
         <v>24</v>
       </c>
-      <c r="BD27" t="n">
+      <c r="BE27" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5516,9 +5600,12 @@
         <v>0</v>
       </c>
       <c r="BC28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD28" t="n">
         <v>18</v>
       </c>
-      <c r="BD28" t="n">
+      <c r="BE28" t="n">
         <v>18</v>
       </c>
     </row>
@@ -5692,9 +5779,12 @@
         <v>0</v>
       </c>
       <c r="BC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD29" t="n">
         <v>11</v>
       </c>
-      <c r="BD29" t="n">
+      <c r="BE29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5868,9 +5958,12 @@
         <v>1</v>
       </c>
       <c r="BC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD30" t="n">
         <v>24</v>
       </c>
-      <c r="BD30" t="n">
+      <c r="BE30" t="n">
         <v>24</v>
       </c>
     </row>
@@ -6044,9 +6137,12 @@
         <v>0</v>
       </c>
       <c r="BC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD31" t="n">
         <v>20</v>
       </c>
-      <c r="BD31" t="n">
+      <c r="BE31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6220,9 +6316,12 @@
         <v>1</v>
       </c>
       <c r="BC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD32" t="n">
         <v>21</v>
       </c>
-      <c r="BD32" t="n">
+      <c r="BE32" t="n">
         <v>21</v>
       </c>
     </row>
@@ -6396,9 +6495,12 @@
         <v>0</v>
       </c>
       <c r="BC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD33" t="n">
         <v>16</v>
       </c>
-      <c r="BD33" t="n">
+      <c r="BE33" t="n">
         <v>16</v>
       </c>
     </row>
@@ -6572,9 +6674,12 @@
         <v>0</v>
       </c>
       <c r="BC34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD34" t="n">
         <v>9</v>
       </c>
-      <c r="BD34" t="n">
+      <c r="BE34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6748,9 +6853,12 @@
         <v>0</v>
       </c>
       <c r="BC35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD35" t="n">
         <v>24</v>
       </c>
-      <c r="BD35" t="n">
+      <c r="BE35" t="n">
         <v>24</v>
       </c>
     </row>
@@ -6924,9 +7032,12 @@
         <v>0</v>
       </c>
       <c r="BC36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD36" t="n">
         <v>15</v>
       </c>
-      <c r="BD36" t="n">
+      <c r="BE36" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7105,6 +7216,9 @@
       <c r="BD37" t="n">
         <v>0</v>
       </c>
+      <c r="BE37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7276,9 +7390,12 @@
         <v>0</v>
       </c>
       <c r="BC38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD38" t="n">
         <v>2</v>
       </c>
-      <c r="BD38" t="n">
+      <c r="BE38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7452,10 +7569,13 @@
         <v>0</v>
       </c>
       <c r="BC39" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BD39" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BE39" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="40">
@@ -7628,9 +7748,12 @@
         <v>0</v>
       </c>
       <c r="BC40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD40" t="n">
         <v>23</v>
       </c>
-      <c r="BD40" t="n">
+      <c r="BE40" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7804,10 +7927,13 @@
         <v>0</v>
       </c>
       <c r="BC41" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BD41" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BE41" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="42">
@@ -7980,9 +8106,12 @@
         <v>0</v>
       </c>
       <c r="BC42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD42" t="n">
         <v>21</v>
       </c>
-      <c r="BD42" t="n">
+      <c r="BE42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8156,9 +8285,12 @@
         <v>0</v>
       </c>
       <c r="BC43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD43" t="n">
         <v>60</v>
       </c>
-      <c r="BD43" t="n">
+      <c r="BE43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8332,9 +8464,12 @@
         <v>0</v>
       </c>
       <c r="BC44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD44" t="n">
         <v>23</v>
       </c>
-      <c r="BD44" t="n">
+      <c r="BE44" t="n">
         <v>23</v>
       </c>
     </row>
@@ -8508,9 +8643,12 @@
         <v>0</v>
       </c>
       <c r="BC45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD45" t="n">
         <v>24</v>
       </c>
-      <c r="BD45" t="n">
+      <c r="BE45" t="n">
         <v>24</v>
       </c>
     </row>
@@ -8684,10 +8822,13 @@
         <v>0</v>
       </c>
       <c r="BC46" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BD46" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BE46" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="47">
@@ -8865,6 +9006,9 @@
       <c r="BD47" t="n">
         <v>0</v>
       </c>
+      <c r="BE47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9036,9 +9180,12 @@
         <v>0</v>
       </c>
       <c r="BC48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD48" t="n">
         <v>25</v>
       </c>
-      <c r="BD48" t="n">
+      <c r="BE48" t="n">
         <v>25</v>
       </c>
     </row>
@@ -9212,9 +9359,12 @@
         <v>0</v>
       </c>
       <c r="BC49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD49" t="n">
         <v>19</v>
       </c>
-      <c r="BD49" t="n">
+      <c r="BE49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9388,9 +9538,12 @@
         <v>0</v>
       </c>
       <c r="BC50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD50" t="n">
         <v>7</v>
       </c>
-      <c r="BD50" t="n">
+      <c r="BE50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9564,10 +9717,13 @@
         <v>0</v>
       </c>
       <c r="BC51" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BD51" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BE51" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="52">
@@ -9745,6 +9901,9 @@
       <c r="BD52" t="n">
         <v>0</v>
       </c>
+      <c r="BE52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9916,9 +10075,12 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD53" t="n">
         <v>13</v>
       </c>
-      <c r="BD53" t="n">
+      <c r="BE53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -10097,6 +10259,9 @@
       <c r="BD54" t="n">
         <v>0</v>
       </c>
+      <c r="BE54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10268,10 +10433,13 @@
         <v>0</v>
       </c>
       <c r="BC55" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BD55" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BE55" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="56">
@@ -10444,10 +10612,13 @@
         <v>0</v>
       </c>
       <c r="BC56" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BD56" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BE56" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="57">
@@ -10620,9 +10791,12 @@
         <v>0</v>
       </c>
       <c r="BC57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD57" t="n">
         <v>9</v>
       </c>
-      <c r="BD57" t="n">
+      <c r="BE57" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10796,9 +10970,12 @@
         <v>0</v>
       </c>
       <c r="BC58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD58" t="n">
         <v>12</v>
       </c>
-      <c r="BD58" t="n">
+      <c r="BE58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -10972,9 +11149,12 @@
         <v>0</v>
       </c>
       <c r="BC59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD59" t="n">
         <v>6</v>
       </c>
-      <c r="BD59" t="n">
+      <c r="BE59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -11153,6 +11333,9 @@
       <c r="BD60" t="n">
         <v>0</v>
       </c>
+      <c r="BE60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -11324,10 +11507,13 @@
         <v>0</v>
       </c>
       <c r="BC61" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BD61" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BE61" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="62">
@@ -11500,10 +11686,13 @@
         <v>0</v>
       </c>
       <c r="BC62" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BD62" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BE62" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="63">
@@ -11676,10 +11865,13 @@
         <v>0</v>
       </c>
       <c r="BC63" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="BD63" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="BE63" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="64">
@@ -11857,6 +12049,9 @@
       <c r="BD64" t="n">
         <v>0</v>
       </c>
+      <c r="BE64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -12028,9 +12223,12 @@
         <v>0</v>
       </c>
       <c r="BC65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD65" t="n">
         <v>16</v>
       </c>
-      <c r="BD65" t="n">
+      <c r="BE65" t="n">
         <v>16</v>
       </c>
     </row>
@@ -12204,9 +12402,12 @@
         <v>0</v>
       </c>
       <c r="BC66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD66" t="n">
         <v>8</v>
       </c>
-      <c r="BD66" t="n">
+      <c r="BE66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -12380,10 +12581,13 @@
         <v>0</v>
       </c>
       <c r="BC67" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BD67" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BE67" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="68">
@@ -12556,9 +12760,12 @@
         <v>0</v>
       </c>
       <c r="BC68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD68" t="n">
         <v>19</v>
       </c>
-      <c r="BD68" t="n">
+      <c r="BE68" t="n">
         <v>18</v>
       </c>
     </row>
@@ -12732,9 +12939,12 @@
         <v>0</v>
       </c>
       <c r="BC69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD69" t="n">
         <v>7</v>
       </c>
-      <c r="BD69" t="n">
+      <c r="BE69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -12908,9 +13118,12 @@
         <v>0</v>
       </c>
       <c r="BC70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD70" t="n">
         <v>23</v>
       </c>
-      <c r="BD70" t="n">
+      <c r="BE70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -13084,10 +13297,13 @@
         <v>0</v>
       </c>
       <c r="BC71" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="BD71" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="BE71" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="72">
@@ -13260,9 +13476,12 @@
         <v>0</v>
       </c>
       <c r="BC72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD72" t="n">
         <v>22</v>
       </c>
-      <c r="BD72" t="n">
+      <c r="BE72" t="n">
         <v>22</v>
       </c>
     </row>
@@ -13441,6 +13660,9 @@
       <c r="BD73" t="n">
         <v>0</v>
       </c>
+      <c r="BE73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -13617,6 +13839,9 @@
       <c r="BD74" t="n">
         <v>0</v>
       </c>
+      <c r="BE74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -13788,9 +14013,12 @@
         <v>0</v>
       </c>
       <c r="BC75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD75" t="n">
         <v>22</v>
       </c>
-      <c r="BD75" t="n">
+      <c r="BE75" t="n">
         <v>22</v>
       </c>
     </row>
@@ -13964,9 +14192,12 @@
         <v>0</v>
       </c>
       <c r="BC76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD76" t="n">
         <v>20</v>
       </c>
-      <c r="BD76" t="n">
+      <c r="BE76" t="n">
         <v>20</v>
       </c>
     </row>
@@ -14140,9 +14371,12 @@
         <v>0</v>
       </c>
       <c r="BC77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD77" t="n">
         <v>15</v>
       </c>
-      <c r="BD77" t="n">
+      <c r="BE77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -14316,10 +14550,13 @@
         <v>0</v>
       </c>
       <c r="BC78" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BD78" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BE78" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="79">
@@ -14492,9 +14729,12 @@
         <v>0</v>
       </c>
       <c r="BC79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD79" t="n">
         <v>22</v>
       </c>
-      <c r="BD79" t="n">
+      <c r="BE79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -14668,9 +14908,12 @@
         <v>0</v>
       </c>
       <c r="BC80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD80" t="n">
         <v>11</v>
       </c>
-      <c r="BD80" t="n">
+      <c r="BE80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -14844,9 +15087,12 @@
         <v>0</v>
       </c>
       <c r="BC81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD81" t="n">
         <v>4</v>
       </c>
-      <c r="BD81" t="n">
+      <c r="BE81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -15020,10 +15266,13 @@
         <v>0</v>
       </c>
       <c r="BC82" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="BD82" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="BE82" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="83">
@@ -15196,9 +15445,12 @@
         <v>0</v>
       </c>
       <c r="BC83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD83" t="n">
         <v>17</v>
       </c>
-      <c r="BD83" t="n">
+      <c r="BE83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -15372,9 +15624,12 @@
         <v>0</v>
       </c>
       <c r="BC84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD84" t="n">
         <v>13</v>
       </c>
-      <c r="BD84" t="n">
+      <c r="BE84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -15548,9 +15803,12 @@
         <v>0</v>
       </c>
       <c r="BC85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD85" t="n">
         <v>7</v>
       </c>
-      <c r="BD85" t="n">
+      <c r="BE85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15729,6 +15987,9 @@
       <c r="BD86" t="n">
         <v>0</v>
       </c>
+      <c r="BE86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -15900,9 +16161,12 @@
         <v>0</v>
       </c>
       <c r="BC87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD87" t="n">
         <v>18</v>
       </c>
-      <c r="BD87" t="n">
+      <c r="BE87" t="n">
         <v>18</v>
       </c>
     </row>
@@ -16081,6 +16345,9 @@
       <c r="BD88" t="n">
         <v>0</v>
       </c>
+      <c r="BE88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -16252,9 +16519,12 @@
         <v>0</v>
       </c>
       <c r="BC89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD89" t="n">
         <v>17</v>
       </c>
-      <c r="BD89" t="n">
+      <c r="BE89" t="n">
         <v>17</v>
       </c>
     </row>
@@ -16428,9 +16698,12 @@
         <v>0</v>
       </c>
       <c r="BC90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD90" t="n">
         <v>16</v>
       </c>
-      <c r="BD90" t="n">
+      <c r="BE90" t="n">
         <v>16</v>
       </c>
     </row>
@@ -16604,9 +16877,12 @@
         <v>0</v>
       </c>
       <c r="BC91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD91" t="n">
         <v>42</v>
       </c>
-      <c r="BD91" t="n">
+      <c r="BE91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -16780,9 +17056,12 @@
         <v>0</v>
       </c>
       <c r="BC92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD92" t="n">
         <v>7</v>
       </c>
-      <c r="BD92" t="n">
+      <c r="BE92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16961,6 +17240,9 @@
       <c r="BD93" t="n">
         <v>0</v>
       </c>
+      <c r="BE93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -17132,9 +17414,12 @@
         <v>0</v>
       </c>
       <c r="BC94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD94" t="n">
         <v>16</v>
       </c>
-      <c r="BD94" t="n">
+      <c r="BE94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -17308,9 +17593,12 @@
         <v>0</v>
       </c>
       <c r="BC95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD95" t="n">
         <v>7</v>
       </c>
-      <c r="BD95" t="n">
+      <c r="BE95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17484,10 +17772,13 @@
         <v>0</v>
       </c>
       <c r="BC96" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="BD96" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BE96" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="97">
@@ -17665,6 +17956,9 @@
       <c r="BD97" t="n">
         <v>0</v>
       </c>
+      <c r="BE97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -17836,9 +18130,12 @@
         <v>0</v>
       </c>
       <c r="BC98" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD98" t="n">
         <v>29</v>
       </c>
-      <c r="BD98" t="n">
+      <c r="BE98" t="n">
         <v>29</v>
       </c>
     </row>
@@ -18012,9 +18309,12 @@
         <v>0</v>
       </c>
       <c r="BC99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD99" t="n">
         <v>13</v>
       </c>
-      <c r="BD99" t="n">
+      <c r="BE99" t="n">
         <v>13</v>
       </c>
     </row>
@@ -18193,6 +18493,9 @@
       <c r="BD100" t="n">
         <v>0</v>
       </c>
+      <c r="BE100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -18364,9 +18667,12 @@
         <v>0</v>
       </c>
       <c r="BC101" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD101" t="n">
         <v>27</v>
       </c>
-      <c r="BD101" t="n">
+      <c r="BE101" t="n">
         <v>27</v>
       </c>
     </row>
@@ -18540,9 +18846,12 @@
         <v>0</v>
       </c>
       <c r="BC102" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD102" t="n">
         <v>26</v>
       </c>
-      <c r="BD102" t="n">
+      <c r="BE102" t="n">
         <v>26</v>
       </c>
     </row>
@@ -18716,10 +19025,13 @@
         <v>1</v>
       </c>
       <c r="BC103" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BD103" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BE103" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="104">
@@ -18892,9 +19204,12 @@
         <v>0</v>
       </c>
       <c r="BC104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD104" t="n">
         <v>12</v>
       </c>
-      <c r="BD104" t="n">
+      <c r="BE104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -19068,9 +19383,12 @@
         <v>0</v>
       </c>
       <c r="BC105" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD105" t="n">
         <v>21</v>
       </c>
-      <c r="BD105" t="n">
+      <c r="BE105" t="n">
         <v>21</v>
       </c>
     </row>
@@ -19244,9 +19562,12 @@
         <v>0</v>
       </c>
       <c r="BC106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD106" t="n">
         <v>7</v>
       </c>
-      <c r="BD106" t="n">
+      <c r="BE106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -19420,9 +19741,12 @@
         <v>0</v>
       </c>
       <c r="BC107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD107" t="n">
         <v>13</v>
       </c>
-      <c r="BD107" t="n">
+      <c r="BE107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -19596,9 +19920,12 @@
         <v>0</v>
       </c>
       <c r="BC108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD108" t="n">
         <v>2</v>
       </c>
-      <c r="BD108" t="n">
+      <c r="BE108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -19772,9 +20099,12 @@
         <v>0</v>
       </c>
       <c r="BC109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD109" t="n">
         <v>4</v>
       </c>
-      <c r="BD109" t="n">
+      <c r="BE109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#3966)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE109"/>
+  <dimension ref="A1:BF109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -485,8 +485,9 @@
     <col width="12" customWidth="1" min="53" max="53"/>
     <col width="12" customWidth="1" min="54" max="54"/>
     <col width="12" customWidth="1" min="55" max="55"/>
-    <col width="13" customWidth="1" min="56" max="56"/>
+    <col width="12" customWidth="1" min="56" max="56"/>
     <col width="13" customWidth="1" min="57" max="57"/>
+    <col width="13" customWidth="1" min="58" max="58"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -765,12 +766,17 @@
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="BD1" s="2" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="BE1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BE1" s="2" t="inlineStr">
+      <c r="BF1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -949,9 +955,12 @@
         <v>0</v>
       </c>
       <c r="BD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" t="n">
         <v>12</v>
       </c>
-      <c r="BE2" t="n">
+      <c r="BF2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1128,9 +1137,12 @@
         <v>1</v>
       </c>
       <c r="BD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE3" t="n">
         <v>10</v>
       </c>
-      <c r="BE3" t="n">
+      <c r="BF3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1307,10 +1319,13 @@
         <v>1</v>
       </c>
       <c r="BD4" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="BE4" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="5">
@@ -1486,9 +1501,12 @@
         <v>0</v>
       </c>
       <c r="BD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE5" t="n">
         <v>15</v>
       </c>
-      <c r="BE5" t="n">
+      <c r="BF5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1665,9 +1683,12 @@
         <v>0</v>
       </c>
       <c r="BD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE6" t="n">
         <v>19</v>
       </c>
-      <c r="BE6" t="n">
+      <c r="BF6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1844,9 +1865,12 @@
         <v>0</v>
       </c>
       <c r="BD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE7" t="n">
         <v>19</v>
       </c>
-      <c r="BE7" t="n">
+      <c r="BF7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2023,9 +2047,12 @@
         <v>0</v>
       </c>
       <c r="BD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE8" t="n">
         <v>29</v>
       </c>
-      <c r="BE8" t="n">
+      <c r="BF8" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2202,10 +2229,13 @@
         <v>0</v>
       </c>
       <c r="BD9" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BE9" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="10">
@@ -2381,10 +2411,13 @@
         <v>1</v>
       </c>
       <c r="BD10" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="BE10" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="11">
@@ -2560,10 +2593,13 @@
         <v>0</v>
       </c>
       <c r="BD11" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BE11" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -2739,10 +2775,13 @@
         <v>1</v>
       </c>
       <c r="BD12" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BE12" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="13">
@@ -2918,9 +2957,12 @@
         <v>0</v>
       </c>
       <c r="BD13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE13" t="n">
         <v>14</v>
       </c>
-      <c r="BE13" t="n">
+      <c r="BF13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3097,9 +3139,12 @@
         <v>0</v>
       </c>
       <c r="BD14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE14" t="n">
         <v>25</v>
       </c>
-      <c r="BE14" t="n">
+      <c r="BF14" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3276,9 +3321,12 @@
         <v>0</v>
       </c>
       <c r="BD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE15" t="n">
         <v>9</v>
       </c>
-      <c r="BE15" t="n">
+      <c r="BF15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3455,9 +3503,12 @@
         <v>0</v>
       </c>
       <c r="BD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE16" t="n">
         <v>20</v>
       </c>
-      <c r="BE16" t="n">
+      <c r="BF16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3634,9 +3685,12 @@
         <v>0</v>
       </c>
       <c r="BD17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE17" t="n">
         <v>17</v>
       </c>
-      <c r="BE17" t="n">
+      <c r="BF17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3813,10 +3867,13 @@
         <v>1</v>
       </c>
       <c r="BD18" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BE18" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BF18" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="19">
@@ -3997,6 +4054,9 @@
       <c r="BE19" t="n">
         <v>0</v>
       </c>
+      <c r="BF19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4171,9 +4231,12 @@
         <v>0</v>
       </c>
       <c r="BD20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE20" t="n">
         <v>18</v>
       </c>
-      <c r="BE20" t="n">
+      <c r="BF20" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4350,10 +4413,13 @@
         <v>1</v>
       </c>
       <c r="BD21" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BE21" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BF21" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="22">
@@ -4534,6 +4600,9 @@
       <c r="BE22" t="n">
         <v>0</v>
       </c>
+      <c r="BF22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4708,10 +4777,13 @@
         <v>0</v>
       </c>
       <c r="BD23" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="BE23" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="BF23" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="24">
@@ -4887,10 +4959,13 @@
         <v>1</v>
       </c>
       <c r="BD24" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BE24" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BF24" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="25">
@@ -5066,9 +5141,12 @@
         <v>0</v>
       </c>
       <c r="BD25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE25" t="n">
         <v>10</v>
       </c>
-      <c r="BE25" t="n">
+      <c r="BF25" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5245,10 +5323,13 @@
         <v>1</v>
       </c>
       <c r="BD26" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BE26" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BF26" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="27">
@@ -5424,9 +5505,12 @@
         <v>0</v>
       </c>
       <c r="BD27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE27" t="n">
         <v>24</v>
       </c>
-      <c r="BE27" t="n">
+      <c r="BF27" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5603,9 +5687,12 @@
         <v>0</v>
       </c>
       <c r="BD28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE28" t="n">
         <v>18</v>
       </c>
-      <c r="BE28" t="n">
+      <c r="BF28" t="n">
         <v>18</v>
       </c>
     </row>
@@ -5782,9 +5869,12 @@
         <v>0</v>
       </c>
       <c r="BD29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE29" t="n">
         <v>11</v>
       </c>
-      <c r="BE29" t="n">
+      <c r="BF29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5961,10 +6051,13 @@
         <v>0</v>
       </c>
       <c r="BD30" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BE30" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BF30" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="31">
@@ -6140,9 +6233,12 @@
         <v>0</v>
       </c>
       <c r="BD31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE31" t="n">
         <v>20</v>
       </c>
-      <c r="BE31" t="n">
+      <c r="BF31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6319,10 +6415,13 @@
         <v>0</v>
       </c>
       <c r="BD32" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="BE32" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="BF32" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="33">
@@ -6498,9 +6597,12 @@
         <v>0</v>
       </c>
       <c r="BD33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE33" t="n">
         <v>16</v>
       </c>
-      <c r="BE33" t="n">
+      <c r="BF33" t="n">
         <v>16</v>
       </c>
     </row>
@@ -6677,9 +6779,12 @@
         <v>0</v>
       </c>
       <c r="BD34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE34" t="n">
         <v>9</v>
       </c>
-      <c r="BE34" t="n">
+      <c r="BF34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6856,9 +6961,12 @@
         <v>0</v>
       </c>
       <c r="BD35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE35" t="n">
         <v>24</v>
       </c>
-      <c r="BE35" t="n">
+      <c r="BF35" t="n">
         <v>24</v>
       </c>
     </row>
@@ -7035,9 +7143,12 @@
         <v>0</v>
       </c>
       <c r="BD36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE36" t="n">
         <v>15</v>
       </c>
-      <c r="BE36" t="n">
+      <c r="BF36" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7219,6 +7330,9 @@
       <c r="BE37" t="n">
         <v>0</v>
       </c>
+      <c r="BF37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7393,9 +7507,12 @@
         <v>0</v>
       </c>
       <c r="BD38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE38" t="n">
         <v>2</v>
       </c>
-      <c r="BE38" t="n">
+      <c r="BF38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7572,10 +7689,13 @@
         <v>1</v>
       </c>
       <c r="BD39" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BE39" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BF39" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="40">
@@ -7751,10 +7871,13 @@
         <v>0</v>
       </c>
       <c r="BD40" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="BE40" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BF40" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="41">
@@ -7930,10 +8053,13 @@
         <v>1</v>
       </c>
       <c r="BD41" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BE41" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BF41" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="42">
@@ -8109,9 +8235,12 @@
         <v>0</v>
       </c>
       <c r="BD42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE42" t="n">
         <v>21</v>
       </c>
-      <c r="BE42" t="n">
+      <c r="BF42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8288,9 +8417,12 @@
         <v>0</v>
       </c>
       <c r="BD43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE43" t="n">
         <v>60</v>
       </c>
-      <c r="BE43" t="n">
+      <c r="BF43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8467,9 +8599,12 @@
         <v>0</v>
       </c>
       <c r="BD44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE44" t="n">
         <v>23</v>
       </c>
-      <c r="BE44" t="n">
+      <c r="BF44" t="n">
         <v>23</v>
       </c>
     </row>
@@ -8646,9 +8781,12 @@
         <v>0</v>
       </c>
       <c r="BD45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE45" t="n">
         <v>24</v>
       </c>
-      <c r="BE45" t="n">
+      <c r="BF45" t="n">
         <v>24</v>
       </c>
     </row>
@@ -8825,10 +8963,13 @@
         <v>1</v>
       </c>
       <c r="BD46" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BE46" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BF46" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="47">
@@ -9009,6 +9150,9 @@
       <c r="BE47" t="n">
         <v>0</v>
       </c>
+      <c r="BF47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9183,10 +9327,13 @@
         <v>0</v>
       </c>
       <c r="BD48" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BE48" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BF48" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="49">
@@ -9362,9 +9509,12 @@
         <v>0</v>
       </c>
       <c r="BD49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE49" t="n">
         <v>19</v>
       </c>
-      <c r="BE49" t="n">
+      <c r="BF49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9541,9 +9691,12 @@
         <v>0</v>
       </c>
       <c r="BD50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE50" t="n">
         <v>7</v>
       </c>
-      <c r="BE50" t="n">
+      <c r="BF50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9720,10 +9873,13 @@
         <v>1</v>
       </c>
       <c r="BD51" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BE51" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BF51" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="52">
@@ -9904,6 +10060,9 @@
       <c r="BE52" t="n">
         <v>0</v>
       </c>
+      <c r="BF52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10078,9 +10237,12 @@
         <v>0</v>
       </c>
       <c r="BD53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE53" t="n">
         <v>13</v>
       </c>
-      <c r="BE53" t="n">
+      <c r="BF53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -10262,6 +10424,9 @@
       <c r="BE54" t="n">
         <v>0</v>
       </c>
+      <c r="BF54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10436,10 +10601,13 @@
         <v>1</v>
       </c>
       <c r="BD55" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="BE55" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="BF55" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="56">
@@ -10615,10 +10783,13 @@
         <v>1</v>
       </c>
       <c r="BD56" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BE56" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BF56" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="57">
@@ -10794,10 +10965,13 @@
         <v>0</v>
       </c>
       <c r="BD57" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="BE57" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="BF57" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="58">
@@ -10973,9 +11147,12 @@
         <v>0</v>
       </c>
       <c r="BD58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE58" t="n">
         <v>12</v>
       </c>
-      <c r="BE58" t="n">
+      <c r="BF58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -11152,9 +11329,12 @@
         <v>0</v>
       </c>
       <c r="BD59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE59" t="n">
         <v>6</v>
       </c>
-      <c r="BE59" t="n">
+      <c r="BF59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -11336,6 +11516,9 @@
       <c r="BE60" t="n">
         <v>0</v>
       </c>
+      <c r="BF60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -11510,9 +11693,12 @@
         <v>1</v>
       </c>
       <c r="BD61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE61" t="n">
         <v>28</v>
       </c>
-      <c r="BE61" t="n">
+      <c r="BF61" t="n">
         <v>28</v>
       </c>
     </row>
@@ -11689,9 +11875,12 @@
         <v>1</v>
       </c>
       <c r="BD62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE62" t="n">
         <v>28</v>
       </c>
-      <c r="BE62" t="n">
+      <c r="BF62" t="n">
         <v>28</v>
       </c>
     </row>
@@ -11868,9 +12057,12 @@
         <v>1</v>
       </c>
       <c r="BD63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE63" t="n">
         <v>12</v>
       </c>
-      <c r="BE63" t="n">
+      <c r="BF63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -12052,6 +12244,9 @@
       <c r="BE64" t="n">
         <v>0</v>
       </c>
+      <c r="BF64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -12226,9 +12421,12 @@
         <v>0</v>
       </c>
       <c r="BD65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE65" t="n">
         <v>16</v>
       </c>
-      <c r="BE65" t="n">
+      <c r="BF65" t="n">
         <v>16</v>
       </c>
     </row>
@@ -12405,9 +12603,12 @@
         <v>0</v>
       </c>
       <c r="BD66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE66" t="n">
         <v>8</v>
       </c>
-      <c r="BE66" t="n">
+      <c r="BF66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -12584,10 +12785,13 @@
         <v>1</v>
       </c>
       <c r="BD67" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="BE67" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="BF67" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="68">
@@ -12763,10 +12967,13 @@
         <v>0</v>
       </c>
       <c r="BD68" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE68" t="n">
+        <v>20</v>
+      </c>
+      <c r="BF68" t="n">
         <v>19</v>
-      </c>
-      <c r="BE68" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="69">
@@ -12942,9 +13149,12 @@
         <v>0</v>
       </c>
       <c r="BD69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE69" t="n">
         <v>7</v>
       </c>
-      <c r="BE69" t="n">
+      <c r="BF69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13121,9 +13331,12 @@
         <v>0</v>
       </c>
       <c r="BD70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE70" t="n">
         <v>23</v>
       </c>
-      <c r="BE70" t="n">
+      <c r="BF70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -13300,9 +13513,12 @@
         <v>1</v>
       </c>
       <c r="BD71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE71" t="n">
         <v>23</v>
       </c>
-      <c r="BE71" t="n">
+      <c r="BF71" t="n">
         <v>23</v>
       </c>
     </row>
@@ -13479,9 +13695,12 @@
         <v>0</v>
       </c>
       <c r="BD72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE72" t="n">
         <v>22</v>
       </c>
-      <c r="BE72" t="n">
+      <c r="BF72" t="n">
         <v>22</v>
       </c>
     </row>
@@ -13663,6 +13882,9 @@
       <c r="BE73" t="n">
         <v>0</v>
       </c>
+      <c r="BF73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -13842,6 +14064,9 @@
       <c r="BE74" t="n">
         <v>0</v>
       </c>
+      <c r="BF74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -14016,10 +14241,13 @@
         <v>0</v>
       </c>
       <c r="BD75" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="BE75" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="BF75" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="76">
@@ -14195,9 +14423,12 @@
         <v>0</v>
       </c>
       <c r="BD76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE76" t="n">
         <v>20</v>
       </c>
-      <c r="BE76" t="n">
+      <c r="BF76" t="n">
         <v>20</v>
       </c>
     </row>
@@ -14374,9 +14605,12 @@
         <v>0</v>
       </c>
       <c r="BD77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE77" t="n">
         <v>15</v>
       </c>
-      <c r="BE77" t="n">
+      <c r="BF77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -14553,10 +14787,13 @@
         <v>1</v>
       </c>
       <c r="BD78" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="BE78" t="n">
-        <v>29</v>
+        <v>31</v>
+      </c>
+      <c r="BF78" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="79">
@@ -14732,9 +14969,12 @@
         <v>0</v>
       </c>
       <c r="BD79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE79" t="n">
         <v>22</v>
       </c>
-      <c r="BE79" t="n">
+      <c r="BF79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -14911,9 +15151,12 @@
         <v>0</v>
       </c>
       <c r="BD80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE80" t="n">
         <v>11</v>
       </c>
-      <c r="BE80" t="n">
+      <c r="BF80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -15090,9 +15333,12 @@
         <v>0</v>
       </c>
       <c r="BD81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE81" t="n">
         <v>4</v>
       </c>
-      <c r="BE81" t="n">
+      <c r="BF81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -15269,10 +15515,13 @@
         <v>1</v>
       </c>
       <c r="BD82" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="BE82" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="BF82" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="83">
@@ -15448,9 +15697,12 @@
         <v>0</v>
       </c>
       <c r="BD83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE83" t="n">
         <v>17</v>
       </c>
-      <c r="BE83" t="n">
+      <c r="BF83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -15627,9 +15879,12 @@
         <v>0</v>
       </c>
       <c r="BD84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE84" t="n">
         <v>13</v>
       </c>
-      <c r="BE84" t="n">
+      <c r="BF84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -15806,9 +16061,12 @@
         <v>0</v>
       </c>
       <c r="BD85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE85" t="n">
         <v>7</v>
       </c>
-      <c r="BE85" t="n">
+      <c r="BF85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15990,6 +16248,9 @@
       <c r="BE86" t="n">
         <v>0</v>
       </c>
+      <c r="BF86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -16164,9 +16425,12 @@
         <v>0</v>
       </c>
       <c r="BD87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE87" t="n">
         <v>18</v>
       </c>
-      <c r="BE87" t="n">
+      <c r="BF87" t="n">
         <v>18</v>
       </c>
     </row>
@@ -16348,6 +16612,9 @@
       <c r="BE88" t="n">
         <v>0</v>
       </c>
+      <c r="BF88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -16522,9 +16789,12 @@
         <v>0</v>
       </c>
       <c r="BD89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE89" t="n">
         <v>17</v>
       </c>
-      <c r="BE89" t="n">
+      <c r="BF89" t="n">
         <v>17</v>
       </c>
     </row>
@@ -16701,9 +16971,12 @@
         <v>0</v>
       </c>
       <c r="BD90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE90" t="n">
         <v>16</v>
       </c>
-      <c r="BE90" t="n">
+      <c r="BF90" t="n">
         <v>16</v>
       </c>
     </row>
@@ -16880,9 +17153,12 @@
         <v>0</v>
       </c>
       <c r="BD91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE91" t="n">
         <v>42</v>
       </c>
-      <c r="BE91" t="n">
+      <c r="BF91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -17059,9 +17335,12 @@
         <v>0</v>
       </c>
       <c r="BD92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE92" t="n">
         <v>7</v>
       </c>
-      <c r="BE92" t="n">
+      <c r="BF92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17243,6 +17522,9 @@
       <c r="BE93" t="n">
         <v>0</v>
       </c>
+      <c r="BF93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -17417,9 +17699,12 @@
         <v>0</v>
       </c>
       <c r="BD94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE94" t="n">
         <v>16</v>
       </c>
-      <c r="BE94" t="n">
+      <c r="BF94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -17596,9 +17881,12 @@
         <v>0</v>
       </c>
       <c r="BD95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE95" t="n">
         <v>7</v>
       </c>
-      <c r="BE95" t="n">
+      <c r="BF95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17775,9 +18063,12 @@
         <v>1</v>
       </c>
       <c r="BD96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE96" t="n">
         <v>24</v>
       </c>
-      <c r="BE96" t="n">
+      <c r="BF96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -17959,6 +18250,9 @@
       <c r="BE97" t="n">
         <v>0</v>
       </c>
+      <c r="BF97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -18133,10 +18427,13 @@
         <v>0</v>
       </c>
       <c r="BD98" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BE98" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BF98" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="99">
@@ -18312,9 +18609,12 @@
         <v>0</v>
       </c>
       <c r="BD99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE99" t="n">
         <v>13</v>
       </c>
-      <c r="BE99" t="n">
+      <c r="BF99" t="n">
         <v>13</v>
       </c>
     </row>
@@ -18496,6 +18796,9 @@
       <c r="BE100" t="n">
         <v>0</v>
       </c>
+      <c r="BF100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -18670,10 +18973,13 @@
         <v>0</v>
       </c>
       <c r="BD101" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BE101" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BF101" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="102">
@@ -18849,10 +19155,13 @@
         <v>0</v>
       </c>
       <c r="BD102" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BE102" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BF102" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="103">
@@ -19028,10 +19337,13 @@
         <v>1</v>
       </c>
       <c r="BD103" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BE103" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BF103" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="104">
@@ -19207,9 +19519,12 @@
         <v>0</v>
       </c>
       <c r="BD104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE104" t="n">
         <v>12</v>
       </c>
-      <c r="BE104" t="n">
+      <c r="BF104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -19386,10 +19701,13 @@
         <v>0</v>
       </c>
       <c r="BD105" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="BE105" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="BF105" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="106">
@@ -19565,9 +19883,12 @@
         <v>0</v>
       </c>
       <c r="BD106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE106" t="n">
         <v>7</v>
       </c>
-      <c r="BE106" t="n">
+      <c r="BF106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -19744,9 +20065,12 @@
         <v>0</v>
       </c>
       <c r="BD107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE107" t="n">
         <v>13</v>
       </c>
-      <c r="BE107" t="n">
+      <c r="BF107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -19923,9 +20247,12 @@
         <v>0</v>
       </c>
       <c r="BD108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE108" t="n">
         <v>2</v>
       </c>
-      <c r="BE108" t="n">
+      <c r="BF108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -20102,9 +20429,12 @@
         <v>0</v>
       </c>
       <c r="BD109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE109" t="n">
         <v>4</v>
       </c>
-      <c r="BE109" t="n">
+      <c r="BF109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#4029)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BF109"/>
+  <dimension ref="A1:BG109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -486,8 +486,9 @@
     <col width="12" customWidth="1" min="54" max="54"/>
     <col width="12" customWidth="1" min="55" max="55"/>
     <col width="12" customWidth="1" min="56" max="56"/>
-    <col width="13" customWidth="1" min="57" max="57"/>
+    <col width="12" customWidth="1" min="57" max="57"/>
     <col width="13" customWidth="1" min="58" max="58"/>
+    <col width="13" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -771,12 +772,17 @@
           <t>2026-04-23</t>
         </is>
       </c>
-      <c r="BE1" s="2" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="BF1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BF1" s="2" t="inlineStr">
+      <c r="BG1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -958,9 +964,12 @@
         <v>0</v>
       </c>
       <c r="BE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
         <v>12</v>
       </c>
-      <c r="BF2" t="n">
+      <c r="BG2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1140,9 +1149,12 @@
         <v>0</v>
       </c>
       <c r="BE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF3" t="n">
         <v>10</v>
       </c>
-      <c r="BF3" t="n">
+      <c r="BG3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1322,9 +1334,12 @@
         <v>1</v>
       </c>
       <c r="BE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" t="n">
         <v>33</v>
       </c>
-      <c r="BF4" t="n">
+      <c r="BG4" t="n">
         <v>33</v>
       </c>
     </row>
@@ -1504,9 +1519,12 @@
         <v>0</v>
       </c>
       <c r="BE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF5" t="n">
         <v>15</v>
       </c>
-      <c r="BF5" t="n">
+      <c r="BG5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1686,9 +1704,12 @@
         <v>0</v>
       </c>
       <c r="BE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF6" t="n">
         <v>19</v>
       </c>
-      <c r="BF6" t="n">
+      <c r="BG6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1868,9 +1889,12 @@
         <v>0</v>
       </c>
       <c r="BE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF7" t="n">
         <v>19</v>
       </c>
-      <c r="BF7" t="n">
+      <c r="BG7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2050,9 +2074,12 @@
         <v>0</v>
       </c>
       <c r="BE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF8" t="n">
         <v>29</v>
       </c>
-      <c r="BF8" t="n">
+      <c r="BG8" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2232,9 +2259,12 @@
         <v>1</v>
       </c>
       <c r="BE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF9" t="n">
         <v>26</v>
       </c>
-      <c r="BF9" t="n">
+      <c r="BG9" t="n">
         <v>26</v>
       </c>
     </row>
@@ -2414,9 +2444,12 @@
         <v>1</v>
       </c>
       <c r="BE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF10" t="n">
         <v>33</v>
       </c>
-      <c r="BF10" t="n">
+      <c r="BG10" t="n">
         <v>33</v>
       </c>
     </row>
@@ -2596,9 +2629,12 @@
         <v>1</v>
       </c>
       <c r="BE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF11" t="n">
         <v>27</v>
       </c>
-      <c r="BF11" t="n">
+      <c r="BG11" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2778,9 +2814,12 @@
         <v>1</v>
       </c>
       <c r="BE12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF12" t="n">
         <v>31</v>
       </c>
-      <c r="BF12" t="n">
+      <c r="BG12" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2960,9 +2999,12 @@
         <v>0</v>
       </c>
       <c r="BE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF13" t="n">
         <v>14</v>
       </c>
-      <c r="BF13" t="n">
+      <c r="BG13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3142,9 +3184,12 @@
         <v>0</v>
       </c>
       <c r="BE14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF14" t="n">
         <v>25</v>
       </c>
-      <c r="BF14" t="n">
+      <c r="BG14" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3324,9 +3369,12 @@
         <v>0</v>
       </c>
       <c r="BE15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF15" t="n">
         <v>9</v>
       </c>
-      <c r="BF15" t="n">
+      <c r="BG15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3506,9 +3554,12 @@
         <v>0</v>
       </c>
       <c r="BE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF16" t="n">
         <v>20</v>
       </c>
-      <c r="BF16" t="n">
+      <c r="BG16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3688,9 +3739,12 @@
         <v>0</v>
       </c>
       <c r="BE17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF17" t="n">
         <v>17</v>
       </c>
-      <c r="BF17" t="n">
+      <c r="BG17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3870,9 +3924,12 @@
         <v>1</v>
       </c>
       <c r="BE18" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF18" t="n">
         <v>29</v>
       </c>
-      <c r="BF18" t="n">
+      <c r="BG18" t="n">
         <v>29</v>
       </c>
     </row>
@@ -4057,6 +4114,9 @@
       <c r="BF19" t="n">
         <v>0</v>
       </c>
+      <c r="BG19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4234,9 +4294,12 @@
         <v>0</v>
       </c>
       <c r="BE20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF20" t="n">
         <v>18</v>
       </c>
-      <c r="BF20" t="n">
+      <c r="BG20" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4416,9 +4479,12 @@
         <v>1</v>
       </c>
       <c r="BE21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF21" t="n">
         <v>27</v>
       </c>
-      <c r="BF21" t="n">
+      <c r="BG21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -4603,6 +4669,9 @@
       <c r="BF22" t="n">
         <v>0</v>
       </c>
+      <c r="BG22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4780,9 +4849,12 @@
         <v>1</v>
       </c>
       <c r="BE23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF23" t="n">
         <v>21</v>
       </c>
-      <c r="BF23" t="n">
+      <c r="BG23" t="n">
         <v>21</v>
       </c>
     </row>
@@ -4962,9 +5034,12 @@
         <v>1</v>
       </c>
       <c r="BE24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF24" t="n">
         <v>27</v>
       </c>
-      <c r="BF24" t="n">
+      <c r="BG24" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5144,9 +5219,12 @@
         <v>0</v>
       </c>
       <c r="BE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF25" t="n">
         <v>10</v>
       </c>
-      <c r="BF25" t="n">
+      <c r="BG25" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5326,9 +5404,12 @@
         <v>1</v>
       </c>
       <c r="BE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF26" t="n">
         <v>29</v>
       </c>
-      <c r="BF26" t="n">
+      <c r="BG26" t="n">
         <v>29</v>
       </c>
     </row>
@@ -5508,9 +5589,12 @@
         <v>0</v>
       </c>
       <c r="BE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF27" t="n">
         <v>24</v>
       </c>
-      <c r="BF27" t="n">
+      <c r="BG27" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5690,9 +5774,12 @@
         <v>0</v>
       </c>
       <c r="BE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF28" t="n">
         <v>18</v>
       </c>
-      <c r="BF28" t="n">
+      <c r="BG28" t="n">
         <v>18</v>
       </c>
     </row>
@@ -5872,9 +5959,12 @@
         <v>0</v>
       </c>
       <c r="BE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF29" t="n">
         <v>11</v>
       </c>
-      <c r="BF29" t="n">
+      <c r="BG29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6054,9 +6144,12 @@
         <v>1</v>
       </c>
       <c r="BE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF30" t="n">
         <v>25</v>
       </c>
-      <c r="BF30" t="n">
+      <c r="BG30" t="n">
         <v>25</v>
       </c>
     </row>
@@ -6236,9 +6329,12 @@
         <v>0</v>
       </c>
       <c r="BE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF31" t="n">
         <v>20</v>
       </c>
-      <c r="BF31" t="n">
+      <c r="BG31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6418,9 +6514,12 @@
         <v>1</v>
       </c>
       <c r="BE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF32" t="n">
         <v>22</v>
       </c>
-      <c r="BF32" t="n">
+      <c r="BG32" t="n">
         <v>22</v>
       </c>
     </row>
@@ -6600,9 +6699,12 @@
         <v>0</v>
       </c>
       <c r="BE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF33" t="n">
         <v>16</v>
       </c>
-      <c r="BF33" t="n">
+      <c r="BG33" t="n">
         <v>16</v>
       </c>
     </row>
@@ -6782,9 +6884,12 @@
         <v>0</v>
       </c>
       <c r="BE34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF34" t="n">
         <v>9</v>
       </c>
-      <c r="BF34" t="n">
+      <c r="BG34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6964,9 +7069,12 @@
         <v>0</v>
       </c>
       <c r="BE35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF35" t="n">
         <v>24</v>
       </c>
-      <c r="BF35" t="n">
+      <c r="BG35" t="n">
         <v>24</v>
       </c>
     </row>
@@ -7146,9 +7254,12 @@
         <v>0</v>
       </c>
       <c r="BE36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF36" t="n">
         <v>15</v>
       </c>
-      <c r="BF36" t="n">
+      <c r="BG36" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7333,6 +7444,9 @@
       <c r="BF37" t="n">
         <v>0</v>
       </c>
+      <c r="BG37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7510,9 +7624,12 @@
         <v>0</v>
       </c>
       <c r="BE38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF38" t="n">
         <v>2</v>
       </c>
-      <c r="BF38" t="n">
+      <c r="BG38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7692,9 +7809,12 @@
         <v>1</v>
       </c>
       <c r="BE39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF39" t="n">
         <v>32</v>
       </c>
-      <c r="BF39" t="n">
+      <c r="BG39" t="n">
         <v>32</v>
       </c>
     </row>
@@ -7874,9 +7994,12 @@
         <v>1</v>
       </c>
       <c r="BE40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF40" t="n">
         <v>24</v>
       </c>
-      <c r="BF40" t="n">
+      <c r="BG40" t="n">
         <v>24</v>
       </c>
     </row>
@@ -8056,9 +8179,12 @@
         <v>1</v>
       </c>
       <c r="BE41" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF41" t="n">
         <v>32</v>
       </c>
-      <c r="BF41" t="n">
+      <c r="BG41" t="n">
         <v>32</v>
       </c>
     </row>
@@ -8238,9 +8364,12 @@
         <v>0</v>
       </c>
       <c r="BE42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF42" t="n">
         <v>21</v>
       </c>
-      <c r="BF42" t="n">
+      <c r="BG42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8420,9 +8549,12 @@
         <v>0</v>
       </c>
       <c r="BE43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF43" t="n">
         <v>60</v>
       </c>
-      <c r="BF43" t="n">
+      <c r="BG43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8602,9 +8734,12 @@
         <v>0</v>
       </c>
       <c r="BE44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF44" t="n">
         <v>23</v>
       </c>
-      <c r="BF44" t="n">
+      <c r="BG44" t="n">
         <v>23</v>
       </c>
     </row>
@@ -8784,9 +8919,12 @@
         <v>0</v>
       </c>
       <c r="BE45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF45" t="n">
         <v>24</v>
       </c>
-      <c r="BF45" t="n">
+      <c r="BG45" t="n">
         <v>24</v>
       </c>
     </row>
@@ -8966,9 +9104,12 @@
         <v>1</v>
       </c>
       <c r="BE46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF46" t="n">
         <v>28</v>
       </c>
-      <c r="BF46" t="n">
+      <c r="BG46" t="n">
         <v>28</v>
       </c>
     </row>
@@ -9153,6 +9294,9 @@
       <c r="BF47" t="n">
         <v>0</v>
       </c>
+      <c r="BG47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9330,9 +9474,12 @@
         <v>1</v>
       </c>
       <c r="BE48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF48" t="n">
         <v>26</v>
       </c>
-      <c r="BF48" t="n">
+      <c r="BG48" t="n">
         <v>26</v>
       </c>
     </row>
@@ -9512,9 +9659,12 @@
         <v>0</v>
       </c>
       <c r="BE49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF49" t="n">
         <v>19</v>
       </c>
-      <c r="BF49" t="n">
+      <c r="BG49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9694,9 +9844,12 @@
         <v>0</v>
       </c>
       <c r="BE50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF50" t="n">
         <v>7</v>
       </c>
-      <c r="BF50" t="n">
+      <c r="BG50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9876,9 +10029,12 @@
         <v>1</v>
       </c>
       <c r="BE51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF51" t="n">
         <v>31</v>
       </c>
-      <c r="BF51" t="n">
+      <c r="BG51" t="n">
         <v>31</v>
       </c>
     </row>
@@ -10063,6 +10219,9 @@
       <c r="BF52" t="n">
         <v>0</v>
       </c>
+      <c r="BG52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10240,9 +10399,12 @@
         <v>0</v>
       </c>
       <c r="BE53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF53" t="n">
         <v>13</v>
       </c>
-      <c r="BF53" t="n">
+      <c r="BG53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -10427,6 +10589,9 @@
       <c r="BF54" t="n">
         <v>0</v>
       </c>
+      <c r="BG54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10604,9 +10769,12 @@
         <v>1</v>
       </c>
       <c r="BE55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF55" t="n">
         <v>33</v>
       </c>
-      <c r="BF55" t="n">
+      <c r="BG55" t="n">
         <v>33</v>
       </c>
     </row>
@@ -10786,9 +10954,12 @@
         <v>1</v>
       </c>
       <c r="BE56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF56" t="n">
         <v>29</v>
       </c>
-      <c r="BF56" t="n">
+      <c r="BG56" t="n">
         <v>29</v>
       </c>
     </row>
@@ -10968,9 +11139,12 @@
         <v>1</v>
       </c>
       <c r="BE57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF57" t="n">
         <v>10</v>
       </c>
-      <c r="BF57" t="n">
+      <c r="BG57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -11150,9 +11324,12 @@
         <v>0</v>
       </c>
       <c r="BE58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF58" t="n">
         <v>12</v>
       </c>
-      <c r="BF58" t="n">
+      <c r="BG58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -11332,9 +11509,12 @@
         <v>0</v>
       </c>
       <c r="BE59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF59" t="n">
         <v>6</v>
       </c>
-      <c r="BF59" t="n">
+      <c r="BG59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -11519,6 +11699,9 @@
       <c r="BF60" t="n">
         <v>0</v>
       </c>
+      <c r="BG60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -11696,9 +11879,12 @@
         <v>0</v>
       </c>
       <c r="BE61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF61" t="n">
         <v>28</v>
       </c>
-      <c r="BF61" t="n">
+      <c r="BG61" t="n">
         <v>28</v>
       </c>
     </row>
@@ -11878,9 +12064,12 @@
         <v>0</v>
       </c>
       <c r="BE62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF62" t="n">
         <v>28</v>
       </c>
-      <c r="BF62" t="n">
+      <c r="BG62" t="n">
         <v>28</v>
       </c>
     </row>
@@ -12060,9 +12249,12 @@
         <v>0</v>
       </c>
       <c r="BE63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF63" t="n">
         <v>12</v>
       </c>
-      <c r="BF63" t="n">
+      <c r="BG63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -12247,6 +12439,9 @@
       <c r="BF64" t="n">
         <v>0</v>
       </c>
+      <c r="BG64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -12424,9 +12619,12 @@
         <v>0</v>
       </c>
       <c r="BE65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF65" t="n">
         <v>16</v>
       </c>
-      <c r="BF65" t="n">
+      <c r="BG65" t="n">
         <v>16</v>
       </c>
     </row>
@@ -12606,9 +12804,12 @@
         <v>0</v>
       </c>
       <c r="BE66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF66" t="n">
         <v>8</v>
       </c>
-      <c r="BF66" t="n">
+      <c r="BG66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -12788,9 +12989,12 @@
         <v>1</v>
       </c>
       <c r="BE67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF67" t="n">
         <v>33</v>
       </c>
-      <c r="BF67" t="n">
+      <c r="BG67" t="n">
         <v>33</v>
       </c>
     </row>
@@ -12970,9 +13174,12 @@
         <v>1</v>
       </c>
       <c r="BE68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF68" t="n">
         <v>20</v>
       </c>
-      <c r="BF68" t="n">
+      <c r="BG68" t="n">
         <v>19</v>
       </c>
     </row>
@@ -13152,9 +13359,12 @@
         <v>0</v>
       </c>
       <c r="BE69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF69" t="n">
         <v>7</v>
       </c>
-      <c r="BF69" t="n">
+      <c r="BG69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13334,9 +13544,12 @@
         <v>0</v>
       </c>
       <c r="BE70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF70" t="n">
         <v>23</v>
       </c>
-      <c r="BF70" t="n">
+      <c r="BG70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -13516,9 +13729,12 @@
         <v>0</v>
       </c>
       <c r="BE71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF71" t="n">
         <v>23</v>
       </c>
-      <c r="BF71" t="n">
+      <c r="BG71" t="n">
         <v>23</v>
       </c>
     </row>
@@ -13698,9 +13914,12 @@
         <v>0</v>
       </c>
       <c r="BE72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF72" t="n">
         <v>22</v>
       </c>
-      <c r="BF72" t="n">
+      <c r="BG72" t="n">
         <v>22</v>
       </c>
     </row>
@@ -13885,6 +14104,9 @@
       <c r="BF73" t="n">
         <v>0</v>
       </c>
+      <c r="BG73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -14067,6 +14289,9 @@
       <c r="BF74" t="n">
         <v>0</v>
       </c>
+      <c r="BG74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -14244,9 +14469,12 @@
         <v>1</v>
       </c>
       <c r="BE75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF75" t="n">
         <v>23</v>
       </c>
-      <c r="BF75" t="n">
+      <c r="BG75" t="n">
         <v>23</v>
       </c>
     </row>
@@ -14426,9 +14654,12 @@
         <v>0</v>
       </c>
       <c r="BE76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF76" t="n">
         <v>20</v>
       </c>
-      <c r="BF76" t="n">
+      <c r="BG76" t="n">
         <v>20</v>
       </c>
     </row>
@@ -14608,9 +14839,12 @@
         <v>0</v>
       </c>
       <c r="BE77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF77" t="n">
         <v>15</v>
       </c>
-      <c r="BF77" t="n">
+      <c r="BG77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -14790,9 +15024,12 @@
         <v>2</v>
       </c>
       <c r="BE78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF78" t="n">
         <v>31</v>
       </c>
-      <c r="BF78" t="n">
+      <c r="BG78" t="n">
         <v>30</v>
       </c>
     </row>
@@ -14972,9 +15209,12 @@
         <v>0</v>
       </c>
       <c r="BE79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF79" t="n">
         <v>22</v>
       </c>
-      <c r="BF79" t="n">
+      <c r="BG79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -15154,9 +15394,12 @@
         <v>0</v>
       </c>
       <c r="BE80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF80" t="n">
         <v>11</v>
       </c>
-      <c r="BF80" t="n">
+      <c r="BG80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -15336,9 +15579,12 @@
         <v>0</v>
       </c>
       <c r="BE81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF81" t="n">
         <v>4</v>
       </c>
-      <c r="BF81" t="n">
+      <c r="BG81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -15518,9 +15764,12 @@
         <v>1</v>
       </c>
       <c r="BE82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF82" t="n">
         <v>16</v>
       </c>
-      <c r="BF82" t="n">
+      <c r="BG82" t="n">
         <v>16</v>
       </c>
     </row>
@@ -15700,9 +15949,12 @@
         <v>0</v>
       </c>
       <c r="BE83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF83" t="n">
         <v>17</v>
       </c>
-      <c r="BF83" t="n">
+      <c r="BG83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -15882,9 +16134,12 @@
         <v>0</v>
       </c>
       <c r="BE84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF84" t="n">
         <v>13</v>
       </c>
-      <c r="BF84" t="n">
+      <c r="BG84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -16064,9 +16319,12 @@
         <v>0</v>
       </c>
       <c r="BE85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF85" t="n">
         <v>7</v>
       </c>
-      <c r="BF85" t="n">
+      <c r="BG85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16251,6 +16509,9 @@
       <c r="BF86" t="n">
         <v>0</v>
       </c>
+      <c r="BG86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -16428,9 +16689,12 @@
         <v>0</v>
       </c>
       <c r="BE87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF87" t="n">
         <v>18</v>
       </c>
-      <c r="BF87" t="n">
+      <c r="BG87" t="n">
         <v>18</v>
       </c>
     </row>
@@ -16615,6 +16879,9 @@
       <c r="BF88" t="n">
         <v>0</v>
       </c>
+      <c r="BG88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -16792,9 +17059,12 @@
         <v>0</v>
       </c>
       <c r="BE89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF89" t="n">
         <v>17</v>
       </c>
-      <c r="BF89" t="n">
+      <c r="BG89" t="n">
         <v>17</v>
       </c>
     </row>
@@ -16974,9 +17244,12 @@
         <v>0</v>
       </c>
       <c r="BE90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF90" t="n">
         <v>16</v>
       </c>
-      <c r="BF90" t="n">
+      <c r="BG90" t="n">
         <v>16</v>
       </c>
     </row>
@@ -17156,9 +17429,12 @@
         <v>0</v>
       </c>
       <c r="BE91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF91" t="n">
         <v>42</v>
       </c>
-      <c r="BF91" t="n">
+      <c r="BG91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -17338,9 +17614,12 @@
         <v>0</v>
       </c>
       <c r="BE92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF92" t="n">
         <v>7</v>
       </c>
-      <c r="BF92" t="n">
+      <c r="BG92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17525,6 +17804,9 @@
       <c r="BF93" t="n">
         <v>0</v>
       </c>
+      <c r="BG93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -17702,9 +17984,12 @@
         <v>0</v>
       </c>
       <c r="BE94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF94" t="n">
         <v>16</v>
       </c>
-      <c r="BF94" t="n">
+      <c r="BG94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -17884,9 +18169,12 @@
         <v>0</v>
       </c>
       <c r="BE95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF95" t="n">
         <v>7</v>
       </c>
-      <c r="BF95" t="n">
+      <c r="BG95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18066,9 +18354,12 @@
         <v>0</v>
       </c>
       <c r="BE96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF96" t="n">
         <v>24</v>
       </c>
-      <c r="BF96" t="n">
+      <c r="BG96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -18253,6 +18544,9 @@
       <c r="BF97" t="n">
         <v>0</v>
       </c>
+      <c r="BG97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -18430,9 +18724,12 @@
         <v>1</v>
       </c>
       <c r="BE98" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF98" t="n">
         <v>30</v>
       </c>
-      <c r="BF98" t="n">
+      <c r="BG98" t="n">
         <v>30</v>
       </c>
     </row>
@@ -18612,9 +18909,12 @@
         <v>0</v>
       </c>
       <c r="BE99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF99" t="n">
         <v>13</v>
       </c>
-      <c r="BF99" t="n">
+      <c r="BG99" t="n">
         <v>13</v>
       </c>
     </row>
@@ -18799,6 +19099,9 @@
       <c r="BF100" t="n">
         <v>0</v>
       </c>
+      <c r="BG100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -18976,9 +19279,12 @@
         <v>1</v>
       </c>
       <c r="BE101" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF101" t="n">
         <v>28</v>
       </c>
-      <c r="BF101" t="n">
+      <c r="BG101" t="n">
         <v>28</v>
       </c>
     </row>
@@ -19158,9 +19464,12 @@
         <v>1</v>
       </c>
       <c r="BE102" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF102" t="n">
         <v>27</v>
       </c>
-      <c r="BF102" t="n">
+      <c r="BG102" t="n">
         <v>27</v>
       </c>
     </row>
@@ -19340,9 +19649,12 @@
         <v>1</v>
       </c>
       <c r="BE103" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF103" t="n">
         <v>31</v>
       </c>
-      <c r="BF103" t="n">
+      <c r="BG103" t="n">
         <v>31</v>
       </c>
     </row>
@@ -19522,9 +19834,12 @@
         <v>0</v>
       </c>
       <c r="BE104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF104" t="n">
         <v>12</v>
       </c>
-      <c r="BF104" t="n">
+      <c r="BG104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -19704,9 +20019,12 @@
         <v>1</v>
       </c>
       <c r="BE105" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF105" t="n">
         <v>22</v>
       </c>
-      <c r="BF105" t="n">
+      <c r="BG105" t="n">
         <v>22</v>
       </c>
     </row>
@@ -19886,9 +20204,12 @@
         <v>0</v>
       </c>
       <c r="BE106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF106" t="n">
         <v>7</v>
       </c>
-      <c r="BF106" t="n">
+      <c r="BG106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -20068,9 +20389,12 @@
         <v>0</v>
       </c>
       <c r="BE107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF107" t="n">
         <v>13</v>
       </c>
-      <c r="BF107" t="n">
+      <c r="BG107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -20250,9 +20574,12 @@
         <v>0</v>
       </c>
       <c r="BE108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF108" t="n">
         <v>2</v>
       </c>
-      <c r="BF108" t="n">
+      <c r="BG108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -20432,9 +20759,12 @@
         <v>0</v>
       </c>
       <c r="BE109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF109" t="n">
         <v>4</v>
       </c>
-      <c r="BF109" t="n">
+      <c r="BG109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#4109)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG109"/>
+  <dimension ref="A1:BH109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -487,8 +487,9 @@
     <col width="12" customWidth="1" min="55" max="55"/>
     <col width="12" customWidth="1" min="56" max="56"/>
     <col width="12" customWidth="1" min="57" max="57"/>
-    <col width="13" customWidth="1" min="58" max="58"/>
+    <col width="12" customWidth="1" min="58" max="58"/>
     <col width="13" customWidth="1" min="59" max="59"/>
+    <col width="13" customWidth="1" min="60" max="60"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -777,12 +778,17 @@
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="BF1" s="2" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="BG1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BG1" s="2" t="inlineStr">
+      <c r="BH1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -967,9 +973,12 @@
         <v>0</v>
       </c>
       <c r="BF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="n">
         <v>12</v>
       </c>
-      <c r="BG2" t="n">
+      <c r="BH2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1152,9 +1161,12 @@
         <v>0</v>
       </c>
       <c r="BF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" t="n">
         <v>10</v>
       </c>
-      <c r="BG3" t="n">
+      <c r="BH3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1337,10 +1349,13 @@
         <v>0</v>
       </c>
       <c r="BF4" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="BG4" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="5">
@@ -1522,9 +1537,12 @@
         <v>0</v>
       </c>
       <c r="BF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG5" t="n">
         <v>15</v>
       </c>
-      <c r="BG5" t="n">
+      <c r="BH5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1707,9 +1725,12 @@
         <v>0</v>
       </c>
       <c r="BF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG6" t="n">
         <v>19</v>
       </c>
-      <c r="BG6" t="n">
+      <c r="BH6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1892,9 +1913,12 @@
         <v>0</v>
       </c>
       <c r="BF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG7" t="n">
         <v>19</v>
       </c>
-      <c r="BG7" t="n">
+      <c r="BH7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2077,10 +2101,13 @@
         <v>0</v>
       </c>
       <c r="BF8" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BG8" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="9">
@@ -2262,10 +2289,13 @@
         <v>0</v>
       </c>
       <c r="BF9" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BG9" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="10">
@@ -2447,10 +2477,13 @@
         <v>0</v>
       </c>
       <c r="BF10" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="BG10" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="11">
@@ -2632,9 +2665,12 @@
         <v>0</v>
       </c>
       <c r="BF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG11" t="n">
         <v>27</v>
       </c>
-      <c r="BG11" t="n">
+      <c r="BH11" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2817,10 +2853,13 @@
         <v>0</v>
       </c>
       <c r="BF12" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BG12" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="13">
@@ -3002,9 +3041,12 @@
         <v>0</v>
       </c>
       <c r="BF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG13" t="n">
         <v>14</v>
       </c>
-      <c r="BG13" t="n">
+      <c r="BH13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3187,9 +3229,12 @@
         <v>0</v>
       </c>
       <c r="BF14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG14" t="n">
         <v>25</v>
       </c>
-      <c r="BG14" t="n">
+      <c r="BH14" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3372,9 +3417,12 @@
         <v>0</v>
       </c>
       <c r="BF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG15" t="n">
         <v>9</v>
       </c>
-      <c r="BG15" t="n">
+      <c r="BH15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3557,9 +3605,12 @@
         <v>0</v>
       </c>
       <c r="BF16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG16" t="n">
         <v>20</v>
       </c>
-      <c r="BG16" t="n">
+      <c r="BH16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3742,9 +3793,12 @@
         <v>0</v>
       </c>
       <c r="BF17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG17" t="n">
         <v>17</v>
       </c>
-      <c r="BG17" t="n">
+      <c r="BH17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3927,10 +3981,13 @@
         <v>0</v>
       </c>
       <c r="BF18" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BG18" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BH18" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="19">
@@ -4117,6 +4174,9 @@
       <c r="BG19" t="n">
         <v>0</v>
       </c>
+      <c r="BH19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4297,9 +4357,12 @@
         <v>0</v>
       </c>
       <c r="BF20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG20" t="n">
         <v>18</v>
       </c>
-      <c r="BG20" t="n">
+      <c r="BH20" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4482,9 +4545,12 @@
         <v>0</v>
       </c>
       <c r="BF21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG21" t="n">
         <v>27</v>
       </c>
-      <c r="BG21" t="n">
+      <c r="BH21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -4672,6 +4738,9 @@
       <c r="BG22" t="n">
         <v>0</v>
       </c>
+      <c r="BH22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4852,9 +4921,12 @@
         <v>0</v>
       </c>
       <c r="BF23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG23" t="n">
         <v>21</v>
       </c>
-      <c r="BG23" t="n">
+      <c r="BH23" t="n">
         <v>21</v>
       </c>
     </row>
@@ -5037,9 +5109,12 @@
         <v>0</v>
       </c>
       <c r="BF24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG24" t="n">
         <v>27</v>
       </c>
-      <c r="BG24" t="n">
+      <c r="BH24" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5222,10 +5297,13 @@
         <v>0</v>
       </c>
       <c r="BF25" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="BG25" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="BH25" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="26">
@@ -5407,10 +5485,13 @@
         <v>0</v>
       </c>
       <c r="BF26" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BG26" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BH26" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="27">
@@ -5592,10 +5673,13 @@
         <v>0</v>
       </c>
       <c r="BF27" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BG27" t="n">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="BH27" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="28">
@@ -5777,9 +5861,12 @@
         <v>0</v>
       </c>
       <c r="BF28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG28" t="n">
         <v>18</v>
       </c>
-      <c r="BG28" t="n">
+      <c r="BH28" t="n">
         <v>18</v>
       </c>
     </row>
@@ -5962,9 +6049,12 @@
         <v>0</v>
       </c>
       <c r="BF29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG29" t="n">
         <v>11</v>
       </c>
-      <c r="BG29" t="n">
+      <c r="BH29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6147,9 +6237,12 @@
         <v>0</v>
       </c>
       <c r="BF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG30" t="n">
         <v>25</v>
       </c>
-      <c r="BG30" t="n">
+      <c r="BH30" t="n">
         <v>25</v>
       </c>
     </row>
@@ -6332,9 +6425,12 @@
         <v>0</v>
       </c>
       <c r="BF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG31" t="n">
         <v>20</v>
       </c>
-      <c r="BG31" t="n">
+      <c r="BH31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6517,9 +6613,12 @@
         <v>0</v>
       </c>
       <c r="BF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG32" t="n">
         <v>22</v>
       </c>
-      <c r="BG32" t="n">
+      <c r="BH32" t="n">
         <v>22</v>
       </c>
     </row>
@@ -6702,10 +6801,13 @@
         <v>0</v>
       </c>
       <c r="BF33" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="BG33" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="BH33" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="34">
@@ -6887,9 +6989,12 @@
         <v>0</v>
       </c>
       <c r="BF34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG34" t="n">
         <v>9</v>
       </c>
-      <c r="BG34" t="n">
+      <c r="BH34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7072,9 +7177,12 @@
         <v>0</v>
       </c>
       <c r="BF35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG35" t="n">
         <v>24</v>
       </c>
-      <c r="BG35" t="n">
+      <c r="BH35" t="n">
         <v>24</v>
       </c>
     </row>
@@ -7257,9 +7365,12 @@
         <v>0</v>
       </c>
       <c r="BF36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG36" t="n">
         <v>15</v>
       </c>
-      <c r="BG36" t="n">
+      <c r="BH36" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7447,6 +7558,9 @@
       <c r="BG37" t="n">
         <v>0</v>
       </c>
+      <c r="BH37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7627,9 +7741,12 @@
         <v>0</v>
       </c>
       <c r="BF38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG38" t="n">
         <v>2</v>
       </c>
-      <c r="BG38" t="n">
+      <c r="BH38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7812,10 +7929,13 @@
         <v>0</v>
       </c>
       <c r="BF39" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="BG39" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="BH39" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="40">
@@ -7997,10 +8117,13 @@
         <v>0</v>
       </c>
       <c r="BF40" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BG40" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BH40" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="41">
@@ -8182,10 +8305,13 @@
         <v>0</v>
       </c>
       <c r="BF41" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="BG41" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="BH41" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="42">
@@ -8367,9 +8493,12 @@
         <v>0</v>
       </c>
       <c r="BF42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG42" t="n">
         <v>21</v>
       </c>
-      <c r="BG42" t="n">
+      <c r="BH42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8552,9 +8681,12 @@
         <v>0</v>
       </c>
       <c r="BF43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG43" t="n">
         <v>60</v>
       </c>
-      <c r="BG43" t="n">
+      <c r="BH43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8737,10 +8869,13 @@
         <v>0</v>
       </c>
       <c r="BF44" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="BG44" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BH44" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="45">
@@ -8922,9 +9057,12 @@
         <v>0</v>
       </c>
       <c r="BF45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG45" t="n">
         <v>24</v>
       </c>
-      <c r="BG45" t="n">
+      <c r="BH45" t="n">
         <v>24</v>
       </c>
     </row>
@@ -9107,10 +9245,13 @@
         <v>0</v>
       </c>
       <c r="BF46" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BG46" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BH46" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="47">
@@ -9297,6 +9438,9 @@
       <c r="BG47" t="n">
         <v>0</v>
       </c>
+      <c r="BH47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9477,9 +9621,12 @@
         <v>0</v>
       </c>
       <c r="BF48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG48" t="n">
         <v>26</v>
       </c>
-      <c r="BG48" t="n">
+      <c r="BH48" t="n">
         <v>26</v>
       </c>
     </row>
@@ -9662,9 +9809,12 @@
         <v>0</v>
       </c>
       <c r="BF49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG49" t="n">
         <v>19</v>
       </c>
-      <c r="BG49" t="n">
+      <c r="BH49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9847,9 +9997,12 @@
         <v>0</v>
       </c>
       <c r="BF50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG50" t="n">
         <v>7</v>
       </c>
-      <c r="BG50" t="n">
+      <c r="BH50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10032,10 +10185,13 @@
         <v>0</v>
       </c>
       <c r="BF51" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BG51" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BH51" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="52">
@@ -10222,6 +10378,9 @@
       <c r="BG52" t="n">
         <v>0</v>
       </c>
+      <c r="BH52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10402,9 +10561,12 @@
         <v>0</v>
       </c>
       <c r="BF53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG53" t="n">
         <v>13</v>
       </c>
-      <c r="BG53" t="n">
+      <c r="BH53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -10592,6 +10754,9 @@
       <c r="BG54" t="n">
         <v>0</v>
       </c>
+      <c r="BH54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10772,9 +10937,12 @@
         <v>0</v>
       </c>
       <c r="BF55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG55" t="n">
         <v>33</v>
       </c>
-      <c r="BG55" t="n">
+      <c r="BH55" t="n">
         <v>33</v>
       </c>
     </row>
@@ -10957,10 +11125,13 @@
         <v>0</v>
       </c>
       <c r="BF56" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BG56" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BH56" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="57">
@@ -11142,9 +11313,12 @@
         <v>0</v>
       </c>
       <c r="BF57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG57" t="n">
         <v>10</v>
       </c>
-      <c r="BG57" t="n">
+      <c r="BH57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -11327,9 +11501,12 @@
         <v>0</v>
       </c>
       <c r="BF58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG58" t="n">
         <v>12</v>
       </c>
-      <c r="BG58" t="n">
+      <c r="BH58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -11512,9 +11689,12 @@
         <v>0</v>
       </c>
       <c r="BF59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG59" t="n">
         <v>6</v>
       </c>
-      <c r="BG59" t="n">
+      <c r="BH59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -11702,6 +11882,9 @@
       <c r="BG60" t="n">
         <v>0</v>
       </c>
+      <c r="BH60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -11882,10 +12065,13 @@
         <v>0</v>
       </c>
       <c r="BF61" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BG61" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BH61" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="62">
@@ -12067,9 +12253,12 @@
         <v>0</v>
       </c>
       <c r="BF62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG62" t="n">
         <v>28</v>
       </c>
-      <c r="BG62" t="n">
+      <c r="BH62" t="n">
         <v>28</v>
       </c>
     </row>
@@ -12252,9 +12441,12 @@
         <v>0</v>
       </c>
       <c r="BF63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG63" t="n">
         <v>12</v>
       </c>
-      <c r="BG63" t="n">
+      <c r="BH63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -12442,6 +12634,9 @@
       <c r="BG64" t="n">
         <v>0</v>
       </c>
+      <c r="BH64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -12622,9 +12817,12 @@
         <v>0</v>
       </c>
       <c r="BF65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG65" t="n">
         <v>16</v>
       </c>
-      <c r="BG65" t="n">
+      <c r="BH65" t="n">
         <v>16</v>
       </c>
     </row>
@@ -12807,9 +13005,12 @@
         <v>0</v>
       </c>
       <c r="BF66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG66" t="n">
         <v>8</v>
       </c>
-      <c r="BG66" t="n">
+      <c r="BH66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -12992,10 +13193,13 @@
         <v>0</v>
       </c>
       <c r="BF67" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="BG67" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="BH67" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="68">
@@ -13177,9 +13381,12 @@
         <v>0</v>
       </c>
       <c r="BF68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG68" t="n">
         <v>20</v>
       </c>
-      <c r="BG68" t="n">
+      <c r="BH68" t="n">
         <v>19</v>
       </c>
     </row>
@@ -13362,9 +13569,12 @@
         <v>0</v>
       </c>
       <c r="BF69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG69" t="n">
         <v>7</v>
       </c>
-      <c r="BG69" t="n">
+      <c r="BH69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13547,9 +13757,12 @@
         <v>0</v>
       </c>
       <c r="BF70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG70" t="n">
         <v>23</v>
       </c>
-      <c r="BG70" t="n">
+      <c r="BH70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -13732,10 +13945,13 @@
         <v>0</v>
       </c>
       <c r="BF71" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="BG71" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BH71" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="72">
@@ -13917,10 +14133,13 @@
         <v>0</v>
       </c>
       <c r="BF72" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="BG72" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="BH72" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="73">
@@ -14107,6 +14326,9 @@
       <c r="BG73" t="n">
         <v>0</v>
       </c>
+      <c r="BH73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -14292,6 +14514,9 @@
       <c r="BG74" t="n">
         <v>0</v>
       </c>
+      <c r="BH74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -14472,9 +14697,12 @@
         <v>0</v>
       </c>
       <c r="BF75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG75" t="n">
         <v>23</v>
       </c>
-      <c r="BG75" t="n">
+      <c r="BH75" t="n">
         <v>23</v>
       </c>
     </row>
@@ -14657,10 +14885,13 @@
         <v>0</v>
       </c>
       <c r="BF76" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="BG76" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="BH76" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="77">
@@ -14842,9 +15073,12 @@
         <v>0</v>
       </c>
       <c r="BF77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG77" t="n">
         <v>15</v>
       </c>
-      <c r="BG77" t="n">
+      <c r="BH77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -15027,10 +15261,13 @@
         <v>0</v>
       </c>
       <c r="BF78" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG78" t="n">
+        <v>32</v>
+      </c>
+      <c r="BH78" t="n">
         <v>31</v>
-      </c>
-      <c r="BG78" t="n">
-        <v>30</v>
       </c>
     </row>
     <row r="79">
@@ -15212,9 +15449,12 @@
         <v>0</v>
       </c>
       <c r="BF79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG79" t="n">
         <v>22</v>
       </c>
-      <c r="BG79" t="n">
+      <c r="BH79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -15397,9 +15637,12 @@
         <v>0</v>
       </c>
       <c r="BF80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG80" t="n">
         <v>11</v>
       </c>
-      <c r="BG80" t="n">
+      <c r="BH80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -15582,9 +15825,12 @@
         <v>0</v>
       </c>
       <c r="BF81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG81" t="n">
         <v>4</v>
       </c>
-      <c r="BG81" t="n">
+      <c r="BH81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -15767,10 +16013,13 @@
         <v>0</v>
       </c>
       <c r="BF82" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="BG82" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="BH82" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="83">
@@ -15952,9 +16201,12 @@
         <v>0</v>
       </c>
       <c r="BF83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG83" t="n">
         <v>17</v>
       </c>
-      <c r="BG83" t="n">
+      <c r="BH83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -16137,9 +16389,12 @@
         <v>0</v>
       </c>
       <c r="BF84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG84" t="n">
         <v>13</v>
       </c>
-      <c r="BG84" t="n">
+      <c r="BH84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -16322,9 +16577,12 @@
         <v>0</v>
       </c>
       <c r="BF85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG85" t="n">
         <v>7</v>
       </c>
-      <c r="BG85" t="n">
+      <c r="BH85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16512,6 +16770,9 @@
       <c r="BG86" t="n">
         <v>0</v>
       </c>
+      <c r="BH86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -16692,9 +16953,12 @@
         <v>0</v>
       </c>
       <c r="BF87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG87" t="n">
         <v>18</v>
       </c>
-      <c r="BG87" t="n">
+      <c r="BH87" t="n">
         <v>18</v>
       </c>
     </row>
@@ -16882,6 +17146,9 @@
       <c r="BG88" t="n">
         <v>0</v>
       </c>
+      <c r="BH88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -17062,9 +17329,12 @@
         <v>0</v>
       </c>
       <c r="BF89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG89" t="n">
         <v>17</v>
       </c>
-      <c r="BG89" t="n">
+      <c r="BH89" t="n">
         <v>17</v>
       </c>
     </row>
@@ -17247,9 +17517,12 @@
         <v>0</v>
       </c>
       <c r="BF90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG90" t="n">
         <v>16</v>
       </c>
-      <c r="BG90" t="n">
+      <c r="BH90" t="n">
         <v>16</v>
       </c>
     </row>
@@ -17432,9 +17705,12 @@
         <v>0</v>
       </c>
       <c r="BF91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG91" t="n">
         <v>42</v>
       </c>
-      <c r="BG91" t="n">
+      <c r="BH91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -17617,9 +17893,12 @@
         <v>0</v>
       </c>
       <c r="BF92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG92" t="n">
         <v>7</v>
       </c>
-      <c r="BG92" t="n">
+      <c r="BH92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17807,6 +18086,9 @@
       <c r="BG93" t="n">
         <v>0</v>
       </c>
+      <c r="BH93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -17987,9 +18269,12 @@
         <v>0</v>
       </c>
       <c r="BF94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG94" t="n">
         <v>16</v>
       </c>
-      <c r="BG94" t="n">
+      <c r="BH94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -18172,9 +18457,12 @@
         <v>0</v>
       </c>
       <c r="BF95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG95" t="n">
         <v>7</v>
       </c>
-      <c r="BG95" t="n">
+      <c r="BH95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18357,9 +18645,12 @@
         <v>0</v>
       </c>
       <c r="BF96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG96" t="n">
         <v>24</v>
       </c>
-      <c r="BG96" t="n">
+      <c r="BH96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -18547,6 +18838,9 @@
       <c r="BG97" t="n">
         <v>0</v>
       </c>
+      <c r="BH97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -18727,10 +19021,13 @@
         <v>0</v>
       </c>
       <c r="BF98" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BG98" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BH98" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="99">
@@ -18912,9 +19209,12 @@
         <v>0</v>
       </c>
       <c r="BF99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG99" t="n">
         <v>13</v>
       </c>
-      <c r="BG99" t="n">
+      <c r="BH99" t="n">
         <v>13</v>
       </c>
     </row>
@@ -19102,6 +19402,9 @@
       <c r="BG100" t="n">
         <v>0</v>
       </c>
+      <c r="BH100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -19282,9 +19585,12 @@
         <v>0</v>
       </c>
       <c r="BF101" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG101" t="n">
         <v>28</v>
       </c>
-      <c r="BG101" t="n">
+      <c r="BH101" t="n">
         <v>28</v>
       </c>
     </row>
@@ -19467,10 +19773,13 @@
         <v>0</v>
       </c>
       <c r="BF102" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BG102" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BH102" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="103">
@@ -19652,9 +19961,12 @@
         <v>0</v>
       </c>
       <c r="BF103" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG103" t="n">
         <v>31</v>
       </c>
-      <c r="BG103" t="n">
+      <c r="BH103" t="n">
         <v>31</v>
       </c>
     </row>
@@ -19837,9 +20149,12 @@
         <v>0</v>
       </c>
       <c r="BF104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG104" t="n">
         <v>12</v>
       </c>
-      <c r="BG104" t="n">
+      <c r="BH104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -20022,10 +20337,13 @@
         <v>0</v>
       </c>
       <c r="BF105" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="BG105" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="BH105" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="106">
@@ -20207,9 +20525,12 @@
         <v>0</v>
       </c>
       <c r="BF106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG106" t="n">
         <v>7</v>
       </c>
-      <c r="BG106" t="n">
+      <c r="BH106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -20392,9 +20713,12 @@
         <v>0</v>
       </c>
       <c r="BF107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG107" t="n">
         <v>13</v>
       </c>
-      <c r="BG107" t="n">
+      <c r="BH107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -20577,9 +20901,12 @@
         <v>0</v>
       </c>
       <c r="BF108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG108" t="n">
         <v>2</v>
       </c>
-      <c r="BG108" t="n">
+      <c r="BH108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -20762,9 +21089,12 @@
         <v>0</v>
       </c>
       <c r="BF109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG109" t="n">
         <v>4</v>
       </c>
-      <c r="BG109" t="n">
+      <c r="BH109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#4176)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH109"/>
+  <dimension ref="A1:BI109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -488,8 +488,9 @@
     <col width="12" customWidth="1" min="56" max="56"/>
     <col width="12" customWidth="1" min="57" max="57"/>
     <col width="12" customWidth="1" min="58" max="58"/>
-    <col width="13" customWidth="1" min="59" max="59"/>
+    <col width="12" customWidth="1" min="59" max="59"/>
     <col width="13" customWidth="1" min="60" max="60"/>
+    <col width="13" customWidth="1" min="61" max="61"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -783,12 +784,17 @@
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="BG1" s="2" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="BH1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BH1" s="2" t="inlineStr">
+      <c r="BI1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -976,9 +982,12 @@
         <v>0</v>
       </c>
       <c r="BG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH2" t="n">
         <v>12</v>
       </c>
-      <c r="BH2" t="n">
+      <c r="BI2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1164,9 +1173,12 @@
         <v>0</v>
       </c>
       <c r="BG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH3" t="n">
         <v>10</v>
       </c>
-      <c r="BH3" t="n">
+      <c r="BI3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1352,10 +1364,13 @@
         <v>1</v>
       </c>
       <c r="BG4" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="BH4" t="n">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="5">
@@ -1540,9 +1555,12 @@
         <v>0</v>
       </c>
       <c r="BG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH5" t="n">
         <v>15</v>
       </c>
-      <c r="BH5" t="n">
+      <c r="BI5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1728,9 +1746,12 @@
         <v>0</v>
       </c>
       <c r="BG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH6" t="n">
         <v>19</v>
       </c>
-      <c r="BH6" t="n">
+      <c r="BI6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1916,9 +1937,12 @@
         <v>0</v>
       </c>
       <c r="BG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH7" t="n">
         <v>19</v>
       </c>
-      <c r="BH7" t="n">
+      <c r="BI7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2104,9 +2128,12 @@
         <v>1</v>
       </c>
       <c r="BG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH8" t="n">
         <v>30</v>
       </c>
-      <c r="BH8" t="n">
+      <c r="BI8" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2292,10 +2319,13 @@
         <v>1</v>
       </c>
       <c r="BG9" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BH9" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="10">
@@ -2480,10 +2510,13 @@
         <v>1</v>
       </c>
       <c r="BG10" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="BH10" t="n">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="11">
@@ -2668,9 +2701,12 @@
         <v>0</v>
       </c>
       <c r="BG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH11" t="n">
         <v>27</v>
       </c>
-      <c r="BH11" t="n">
+      <c r="BI11" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2856,10 +2892,13 @@
         <v>1</v>
       </c>
       <c r="BG12" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="BH12" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="13">
@@ -3044,9 +3083,12 @@
         <v>0</v>
       </c>
       <c r="BG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH13" t="n">
         <v>14</v>
       </c>
-      <c r="BH13" t="n">
+      <c r="BI13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3232,9 +3274,12 @@
         <v>0</v>
       </c>
       <c r="BG14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH14" t="n">
         <v>25</v>
       </c>
-      <c r="BH14" t="n">
+      <c r="BI14" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3420,9 +3465,12 @@
         <v>0</v>
       </c>
       <c r="BG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH15" t="n">
         <v>9</v>
       </c>
-      <c r="BH15" t="n">
+      <c r="BI15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3608,9 +3656,12 @@
         <v>0</v>
       </c>
       <c r="BG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH16" t="n">
         <v>20</v>
       </c>
-      <c r="BH16" t="n">
+      <c r="BI16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3796,9 +3847,12 @@
         <v>0</v>
       </c>
       <c r="BG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH17" t="n">
         <v>17</v>
       </c>
-      <c r="BH17" t="n">
+      <c r="BI17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3984,9 +4038,12 @@
         <v>1</v>
       </c>
       <c r="BG18" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH18" t="n">
         <v>30</v>
       </c>
-      <c r="BH18" t="n">
+      <c r="BI18" t="n">
         <v>30</v>
       </c>
     </row>
@@ -4177,6 +4234,9 @@
       <c r="BH19" t="n">
         <v>0</v>
       </c>
+      <c r="BI19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4360,10 +4420,13 @@
         <v>0</v>
       </c>
       <c r="BG20" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="BH20" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="BI20" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="21">
@@ -4548,9 +4611,12 @@
         <v>0</v>
       </c>
       <c r="BG21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH21" t="n">
         <v>27</v>
       </c>
-      <c r="BH21" t="n">
+      <c r="BI21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -4741,6 +4807,9 @@
       <c r="BH22" t="n">
         <v>0</v>
       </c>
+      <c r="BI22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4924,9 +4993,12 @@
         <v>0</v>
       </c>
       <c r="BG23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH23" t="n">
         <v>21</v>
       </c>
-      <c r="BH23" t="n">
+      <c r="BI23" t="n">
         <v>21</v>
       </c>
     </row>
@@ -5112,9 +5184,12 @@
         <v>0</v>
       </c>
       <c r="BG24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH24" t="n">
         <v>27</v>
       </c>
-      <c r="BH24" t="n">
+      <c r="BI24" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5300,9 +5375,12 @@
         <v>1</v>
       </c>
       <c r="BG25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH25" t="n">
         <v>11</v>
       </c>
-      <c r="BH25" t="n">
+      <c r="BI25" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5488,10 +5566,13 @@
         <v>1</v>
       </c>
       <c r="BG26" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BH26" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BI26" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="27">
@@ -5676,9 +5757,12 @@
         <v>1</v>
       </c>
       <c r="BG27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH27" t="n">
         <v>25</v>
       </c>
-      <c r="BH27" t="n">
+      <c r="BI27" t="n">
         <v>23</v>
       </c>
     </row>
@@ -5864,9 +5948,12 @@
         <v>0</v>
       </c>
       <c r="BG28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH28" t="n">
         <v>18</v>
       </c>
-      <c r="BH28" t="n">
+      <c r="BI28" t="n">
         <v>18</v>
       </c>
     </row>
@@ -6052,9 +6139,12 @@
         <v>0</v>
       </c>
       <c r="BG29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH29" t="n">
         <v>11</v>
       </c>
-      <c r="BH29" t="n">
+      <c r="BI29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6240,9 +6330,12 @@
         <v>0</v>
       </c>
       <c r="BG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH30" t="n">
         <v>25</v>
       </c>
-      <c r="BH30" t="n">
+      <c r="BI30" t="n">
         <v>25</v>
       </c>
     </row>
@@ -6428,9 +6521,12 @@
         <v>0</v>
       </c>
       <c r="BG31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH31" t="n">
         <v>20</v>
       </c>
-      <c r="BH31" t="n">
+      <c r="BI31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6616,9 +6712,12 @@
         <v>0</v>
       </c>
       <c r="BG32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH32" t="n">
         <v>22</v>
       </c>
-      <c r="BH32" t="n">
+      <c r="BI32" t="n">
         <v>22</v>
       </c>
     </row>
@@ -6804,10 +6903,13 @@
         <v>1</v>
       </c>
       <c r="BG33" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="BH33" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="BI33" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="34">
@@ -6992,9 +7094,12 @@
         <v>0</v>
       </c>
       <c r="BG34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH34" t="n">
         <v>9</v>
       </c>
-      <c r="BH34" t="n">
+      <c r="BI34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7180,10 +7285,13 @@
         <v>0</v>
       </c>
       <c r="BG35" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BH35" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BI35" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="36">
@@ -7368,9 +7476,12 @@
         <v>0</v>
       </c>
       <c r="BG36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH36" t="n">
         <v>15</v>
       </c>
-      <c r="BH36" t="n">
+      <c r="BI36" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7561,6 +7672,9 @@
       <c r="BH37" t="n">
         <v>0</v>
       </c>
+      <c r="BI37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7744,9 +7858,12 @@
         <v>0</v>
       </c>
       <c r="BG38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH38" t="n">
         <v>2</v>
       </c>
-      <c r="BH38" t="n">
+      <c r="BI38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7932,10 +8049,13 @@
         <v>1</v>
       </c>
       <c r="BG39" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="BH39" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="BI39" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="40">
@@ -8120,9 +8240,12 @@
         <v>1</v>
       </c>
       <c r="BG40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH40" t="n">
         <v>25</v>
       </c>
-      <c r="BH40" t="n">
+      <c r="BI40" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8308,10 +8431,13 @@
         <v>1</v>
       </c>
       <c r="BG41" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="BH41" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="BI41" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="42">
@@ -8496,9 +8622,12 @@
         <v>0</v>
       </c>
       <c r="BG42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH42" t="n">
         <v>21</v>
       </c>
-      <c r="BH42" t="n">
+      <c r="BI42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8684,9 +8813,12 @@
         <v>0</v>
       </c>
       <c r="BG43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH43" t="n">
         <v>60</v>
       </c>
-      <c r="BH43" t="n">
+      <c r="BI43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -8872,10 +9004,13 @@
         <v>1</v>
       </c>
       <c r="BG44" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BH44" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BI44" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="45">
@@ -9060,10 +9195,13 @@
         <v>0</v>
       </c>
       <c r="BG45" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BH45" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BI45" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="46">
@@ -9248,9 +9386,12 @@
         <v>1</v>
       </c>
       <c r="BG46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH46" t="n">
         <v>29</v>
       </c>
-      <c r="BH46" t="n">
+      <c r="BI46" t="n">
         <v>29</v>
       </c>
     </row>
@@ -9441,6 +9582,9 @@
       <c r="BH47" t="n">
         <v>0</v>
       </c>
+      <c r="BI47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9624,9 +9768,12 @@
         <v>0</v>
       </c>
       <c r="BG48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH48" t="n">
         <v>26</v>
       </c>
-      <c r="BH48" t="n">
+      <c r="BI48" t="n">
         <v>26</v>
       </c>
     </row>
@@ -9812,9 +9959,12 @@
         <v>0</v>
       </c>
       <c r="BG49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH49" t="n">
         <v>19</v>
       </c>
-      <c r="BH49" t="n">
+      <c r="BI49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -10000,9 +10150,12 @@
         <v>0</v>
       </c>
       <c r="BG50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH50" t="n">
         <v>7</v>
       </c>
-      <c r="BH50" t="n">
+      <c r="BI50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10188,9 +10341,12 @@
         <v>1</v>
       </c>
       <c r="BG51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH51" t="n">
         <v>32</v>
       </c>
-      <c r="BH51" t="n">
+      <c r="BI51" t="n">
         <v>32</v>
       </c>
     </row>
@@ -10381,6 +10537,9 @@
       <c r="BH52" t="n">
         <v>0</v>
       </c>
+      <c r="BI52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10564,9 +10723,12 @@
         <v>0</v>
       </c>
       <c r="BG53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH53" t="n">
         <v>13</v>
       </c>
-      <c r="BH53" t="n">
+      <c r="BI53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -10757,6 +10919,9 @@
       <c r="BH54" t="n">
         <v>0</v>
       </c>
+      <c r="BI54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10940,9 +11105,12 @@
         <v>0</v>
       </c>
       <c r="BG55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH55" t="n">
         <v>33</v>
       </c>
-      <c r="BH55" t="n">
+      <c r="BI55" t="n">
         <v>33</v>
       </c>
     </row>
@@ -11128,9 +11296,12 @@
         <v>1</v>
       </c>
       <c r="BG56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH56" t="n">
         <v>30</v>
       </c>
-      <c r="BH56" t="n">
+      <c r="BI56" t="n">
         <v>30</v>
       </c>
     </row>
@@ -11316,9 +11487,12 @@
         <v>0</v>
       </c>
       <c r="BG57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH57" t="n">
         <v>10</v>
       </c>
-      <c r="BH57" t="n">
+      <c r="BI57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -11504,9 +11678,12 @@
         <v>0</v>
       </c>
       <c r="BG58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH58" t="n">
         <v>12</v>
       </c>
-      <c r="BH58" t="n">
+      <c r="BI58" t="n">
         <v>12</v>
       </c>
     </row>
@@ -11692,9 +11869,12 @@
         <v>0</v>
       </c>
       <c r="BG59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH59" t="n">
         <v>6</v>
       </c>
-      <c r="BH59" t="n">
+      <c r="BI59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -11885,6 +12065,9 @@
       <c r="BH60" t="n">
         <v>0</v>
       </c>
+      <c r="BI60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12068,9 +12251,12 @@
         <v>1</v>
       </c>
       <c r="BG61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH61" t="n">
         <v>29</v>
       </c>
-      <c r="BH61" t="n">
+      <c r="BI61" t="n">
         <v>29</v>
       </c>
     </row>
@@ -12256,9 +12442,12 @@
         <v>0</v>
       </c>
       <c r="BG62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH62" t="n">
         <v>28</v>
       </c>
-      <c r="BH62" t="n">
+      <c r="BI62" t="n">
         <v>28</v>
       </c>
     </row>
@@ -12444,9 +12633,12 @@
         <v>0</v>
       </c>
       <c r="BG63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH63" t="n">
         <v>12</v>
       </c>
-      <c r="BH63" t="n">
+      <c r="BI63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -12637,6 +12829,9 @@
       <c r="BH64" t="n">
         <v>0</v>
       </c>
+      <c r="BI64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -12820,10 +13015,13 @@
         <v>0</v>
       </c>
       <c r="BG65" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="BH65" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="BI65" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="66">
@@ -13008,9 +13206,12 @@
         <v>0</v>
       </c>
       <c r="BG66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH66" t="n">
         <v>8</v>
       </c>
-      <c r="BH66" t="n">
+      <c r="BI66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -13196,10 +13397,13 @@
         <v>1</v>
       </c>
       <c r="BG67" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="BH67" t="n">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="BI67" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="68">
@@ -13384,10 +13588,13 @@
         <v>0</v>
       </c>
       <c r="BG68" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH68" t="n">
+        <v>21</v>
+      </c>
+      <c r="BI68" t="n">
         <v>20</v>
-      </c>
-      <c r="BH68" t="n">
-        <v>19</v>
       </c>
     </row>
     <row r="69">
@@ -13572,9 +13779,12 @@
         <v>0</v>
       </c>
       <c r="BG69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH69" t="n">
         <v>7</v>
       </c>
-      <c r="BH69" t="n">
+      <c r="BI69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13760,9 +13970,12 @@
         <v>0</v>
       </c>
       <c r="BG70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH70" t="n">
         <v>23</v>
       </c>
-      <c r="BH70" t="n">
+      <c r="BI70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -13948,9 +14161,12 @@
         <v>1</v>
       </c>
       <c r="BG71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH71" t="n">
         <v>24</v>
       </c>
-      <c r="BH71" t="n">
+      <c r="BI71" t="n">
         <v>24</v>
       </c>
     </row>
@@ -14136,10 +14352,13 @@
         <v>1</v>
       </c>
       <c r="BG72" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="BH72" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BI72" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="73">
@@ -14329,6 +14548,9 @@
       <c r="BH73" t="n">
         <v>0</v>
       </c>
+      <c r="BI73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -14517,6 +14739,9 @@
       <c r="BH74" t="n">
         <v>0</v>
       </c>
+      <c r="BI74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -14700,9 +14925,12 @@
         <v>0</v>
       </c>
       <c r="BG75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH75" t="n">
         <v>23</v>
       </c>
-      <c r="BH75" t="n">
+      <c r="BI75" t="n">
         <v>23</v>
       </c>
     </row>
@@ -14888,9 +15116,12 @@
         <v>1</v>
       </c>
       <c r="BG76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH76" t="n">
         <v>21</v>
       </c>
-      <c r="BH76" t="n">
+      <c r="BI76" t="n">
         <v>21</v>
       </c>
     </row>
@@ -15076,9 +15307,12 @@
         <v>0</v>
       </c>
       <c r="BG77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH77" t="n">
         <v>15</v>
       </c>
-      <c r="BH77" t="n">
+      <c r="BI77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -15264,10 +15498,13 @@
         <v>1</v>
       </c>
       <c r="BG78" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH78" t="n">
+        <v>33</v>
+      </c>
+      <c r="BI78" t="n">
         <v>32</v>
-      </c>
-      <c r="BH78" t="n">
-        <v>31</v>
       </c>
     </row>
     <row r="79">
@@ -15452,9 +15689,12 @@
         <v>0</v>
       </c>
       <c r="BG79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH79" t="n">
         <v>22</v>
       </c>
-      <c r="BH79" t="n">
+      <c r="BI79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -15640,9 +15880,12 @@
         <v>0</v>
       </c>
       <c r="BG80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH80" t="n">
         <v>11</v>
       </c>
-      <c r="BH80" t="n">
+      <c r="BI80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -15828,9 +16071,12 @@
         <v>0</v>
       </c>
       <c r="BG81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH81" t="n">
         <v>4</v>
       </c>
-      <c r="BH81" t="n">
+      <c r="BI81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -16016,9 +16262,12 @@
         <v>1</v>
       </c>
       <c r="BG82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH82" t="n">
         <v>17</v>
       </c>
-      <c r="BH82" t="n">
+      <c r="BI82" t="n">
         <v>17</v>
       </c>
     </row>
@@ -16204,9 +16453,12 @@
         <v>0</v>
       </c>
       <c r="BG83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH83" t="n">
         <v>17</v>
       </c>
-      <c r="BH83" t="n">
+      <c r="BI83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -16392,9 +16644,12 @@
         <v>0</v>
       </c>
       <c r="BG84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH84" t="n">
         <v>13</v>
       </c>
-      <c r="BH84" t="n">
+      <c r="BI84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -16580,9 +16835,12 @@
         <v>0</v>
       </c>
       <c r="BG85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH85" t="n">
         <v>7</v>
       </c>
-      <c r="BH85" t="n">
+      <c r="BI85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -16773,6 +17031,9 @@
       <c r="BH86" t="n">
         <v>0</v>
       </c>
+      <c r="BI86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -16956,9 +17217,12 @@
         <v>0</v>
       </c>
       <c r="BG87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH87" t="n">
         <v>18</v>
       </c>
-      <c r="BH87" t="n">
+      <c r="BI87" t="n">
         <v>18</v>
       </c>
     </row>
@@ -17149,6 +17413,9 @@
       <c r="BH88" t="n">
         <v>0</v>
       </c>
+      <c r="BI88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -17332,10 +17599,13 @@
         <v>0</v>
       </c>
       <c r="BG89" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="BH89" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="BI89" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="90">
@@ -17520,10 +17790,13 @@
         <v>0</v>
       </c>
       <c r="BG90" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="BH90" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="BI90" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="91">
@@ -17708,9 +17981,12 @@
         <v>0</v>
       </c>
       <c r="BG91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH91" t="n">
         <v>42</v>
       </c>
-      <c r="BH91" t="n">
+      <c r="BI91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -17896,9 +18172,12 @@
         <v>0</v>
       </c>
       <c r="BG92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH92" t="n">
         <v>7</v>
       </c>
-      <c r="BH92" t="n">
+      <c r="BI92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18089,6 +18368,9 @@
       <c r="BH93" t="n">
         <v>0</v>
       </c>
+      <c r="BI93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -18272,9 +18554,12 @@
         <v>0</v>
       </c>
       <c r="BG94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH94" t="n">
         <v>16</v>
       </c>
-      <c r="BH94" t="n">
+      <c r="BI94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -18460,9 +18745,12 @@
         <v>0</v>
       </c>
       <c r="BG95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH95" t="n">
         <v>7</v>
       </c>
-      <c r="BH95" t="n">
+      <c r="BI95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18648,9 +18936,12 @@
         <v>0</v>
       </c>
       <c r="BG96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH96" t="n">
         <v>24</v>
       </c>
-      <c r="BH96" t="n">
+      <c r="BI96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -18841,6 +19132,9 @@
       <c r="BH97" t="n">
         <v>0</v>
       </c>
+      <c r="BI97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -19024,10 +19318,13 @@
         <v>1</v>
       </c>
       <c r="BG98" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BH98" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BI98" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="99">
@@ -19212,10 +19509,13 @@
         <v>0</v>
       </c>
       <c r="BG99" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="BH99" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="BI99" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="100">
@@ -19405,6 +19705,9 @@
       <c r="BH100" t="n">
         <v>0</v>
       </c>
+      <c r="BI100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -19588,10 +19891,13 @@
         <v>0</v>
       </c>
       <c r="BG101" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BH101" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BI101" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="102">
@@ -19776,9 +20082,12 @@
         <v>1</v>
       </c>
       <c r="BG102" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH102" t="n">
         <v>28</v>
       </c>
-      <c r="BH102" t="n">
+      <c r="BI102" t="n">
         <v>28</v>
       </c>
     </row>
@@ -19964,9 +20273,12 @@
         <v>0</v>
       </c>
       <c r="BG103" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH103" t="n">
         <v>31</v>
       </c>
-      <c r="BH103" t="n">
+      <c r="BI103" t="n">
         <v>31</v>
       </c>
     </row>
@@ -20152,9 +20464,12 @@
         <v>0</v>
       </c>
       <c r="BG104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH104" t="n">
         <v>12</v>
       </c>
-      <c r="BH104" t="n">
+      <c r="BI104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -20340,10 +20655,13 @@
         <v>1</v>
       </c>
       <c r="BG105" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="BH105" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BI105" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="106">
@@ -20528,9 +20846,12 @@
         <v>0</v>
       </c>
       <c r="BG106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH106" t="n">
         <v>7</v>
       </c>
-      <c r="BH106" t="n">
+      <c r="BI106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -20716,9 +21037,12 @@
         <v>0</v>
       </c>
       <c r="BG107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH107" t="n">
         <v>13</v>
       </c>
-      <c r="BH107" t="n">
+      <c r="BI107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -20904,9 +21228,12 @@
         <v>0</v>
       </c>
       <c r="BG108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH108" t="n">
         <v>2</v>
       </c>
-      <c r="BH108" t="n">
+      <c r="BI108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -21092,9 +21419,12 @@
         <v>0</v>
       </c>
       <c r="BG109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH109" t="n">
         <v>4</v>
       </c>
-      <c r="BH109" t="n">
+      <c r="BI109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#4220)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BI109"/>
+  <dimension ref="A1:BJ109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -489,8 +489,9 @@
     <col width="12" customWidth="1" min="57" max="57"/>
     <col width="12" customWidth="1" min="58" max="58"/>
     <col width="12" customWidth="1" min="59" max="59"/>
-    <col width="13" customWidth="1" min="60" max="60"/>
+    <col width="12" customWidth="1" min="60" max="60"/>
     <col width="13" customWidth="1" min="61" max="61"/>
+    <col width="13" customWidth="1" min="62" max="62"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -789,12 +790,17 @@
           <t>2026-04-29</t>
         </is>
       </c>
-      <c r="BH1" s="2" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="BI1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BI1" s="2" t="inlineStr">
+      <c r="BJ1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -985,9 +991,12 @@
         <v>0</v>
       </c>
       <c r="BH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI2" t="n">
         <v>12</v>
       </c>
-      <c r="BI2" t="n">
+      <c r="BJ2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1176,9 +1185,12 @@
         <v>0</v>
       </c>
       <c r="BH3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI3" t="n">
         <v>10</v>
       </c>
-      <c r="BI3" t="n">
+      <c r="BJ3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1367,10 +1379,13 @@
         <v>1</v>
       </c>
       <c r="BH4" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="BI4" t="n">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -1558,9 +1573,12 @@
         <v>0</v>
       </c>
       <c r="BH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI5" t="n">
         <v>15</v>
       </c>
-      <c r="BI5" t="n">
+      <c r="BJ5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1749,9 +1767,12 @@
         <v>0</v>
       </c>
       <c r="BH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI6" t="n">
         <v>19</v>
       </c>
-      <c r="BI6" t="n">
+      <c r="BJ6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1940,9 +1961,12 @@
         <v>0</v>
       </c>
       <c r="BH7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI7" t="n">
         <v>19</v>
       </c>
-      <c r="BI7" t="n">
+      <c r="BJ7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2131,9 +2155,12 @@
         <v>0</v>
       </c>
       <c r="BH8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI8" t="n">
         <v>30</v>
       </c>
-      <c r="BI8" t="n">
+      <c r="BJ8" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2322,10 +2349,13 @@
         <v>1</v>
       </c>
       <c r="BH9" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BI9" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="10">
@@ -2513,9 +2543,12 @@
         <v>1</v>
       </c>
       <c r="BH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI10" t="n">
         <v>35</v>
       </c>
-      <c r="BI10" t="n">
+      <c r="BJ10" t="n">
         <v>35</v>
       </c>
     </row>
@@ -2704,10 +2737,13 @@
         <v>0</v>
       </c>
       <c r="BH11" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BI11" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="12">
@@ -2895,10 +2931,13 @@
         <v>1</v>
       </c>
       <c r="BH12" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="BI12" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="13">
@@ -3086,9 +3125,12 @@
         <v>0</v>
       </c>
       <c r="BH13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI13" t="n">
         <v>14</v>
       </c>
-      <c r="BI13" t="n">
+      <c r="BJ13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3277,9 +3319,12 @@
         <v>0</v>
       </c>
       <c r="BH14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI14" t="n">
         <v>25</v>
       </c>
-      <c r="BI14" t="n">
+      <c r="BJ14" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3468,9 +3513,12 @@
         <v>0</v>
       </c>
       <c r="BH15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI15" t="n">
         <v>9</v>
       </c>
-      <c r="BI15" t="n">
+      <c r="BJ15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3659,9 +3707,12 @@
         <v>0</v>
       </c>
       <c r="BH16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI16" t="n">
         <v>20</v>
       </c>
-      <c r="BI16" t="n">
+      <c r="BJ16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3850,9 +3901,12 @@
         <v>0</v>
       </c>
       <c r="BH17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI17" t="n">
         <v>17</v>
       </c>
-      <c r="BI17" t="n">
+      <c r="BJ17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4041,9 +4095,12 @@
         <v>0</v>
       </c>
       <c r="BH18" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI18" t="n">
         <v>30</v>
       </c>
-      <c r="BI18" t="n">
+      <c r="BJ18" t="n">
         <v>30</v>
       </c>
     </row>
@@ -4237,6 +4294,9 @@
       <c r="BI19" t="n">
         <v>0</v>
       </c>
+      <c r="BJ19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4423,10 +4483,13 @@
         <v>1</v>
       </c>
       <c r="BH20" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="BI20" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="BJ20" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="21">
@@ -4614,9 +4677,12 @@
         <v>0</v>
       </c>
       <c r="BH21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI21" t="n">
         <v>27</v>
       </c>
-      <c r="BI21" t="n">
+      <c r="BJ21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -4810,6 +4876,9 @@
       <c r="BI22" t="n">
         <v>0</v>
       </c>
+      <c r="BJ22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4996,9 +5065,12 @@
         <v>0</v>
       </c>
       <c r="BH23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI23" t="n">
         <v>21</v>
       </c>
-      <c r="BI23" t="n">
+      <c r="BJ23" t="n">
         <v>21</v>
       </c>
     </row>
@@ -5187,9 +5259,12 @@
         <v>0</v>
       </c>
       <c r="BH24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI24" t="n">
         <v>27</v>
       </c>
-      <c r="BI24" t="n">
+      <c r="BJ24" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5378,9 +5453,12 @@
         <v>0</v>
       </c>
       <c r="BH25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI25" t="n">
         <v>11</v>
       </c>
-      <c r="BI25" t="n">
+      <c r="BJ25" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5569,10 +5647,13 @@
         <v>1</v>
       </c>
       <c r="BH26" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BI26" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BJ26" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="27">
@@ -5760,9 +5841,12 @@
         <v>0</v>
       </c>
       <c r="BH27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI27" t="n">
         <v>25</v>
       </c>
-      <c r="BI27" t="n">
+      <c r="BJ27" t="n">
         <v>23</v>
       </c>
     </row>
@@ -5951,10 +6035,13 @@
         <v>0</v>
       </c>
       <c r="BH28" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="BI28" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="BJ28" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="29">
@@ -6142,9 +6229,12 @@
         <v>0</v>
       </c>
       <c r="BH29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI29" t="n">
         <v>11</v>
       </c>
-      <c r="BI29" t="n">
+      <c r="BJ29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6333,9 +6423,12 @@
         <v>0</v>
       </c>
       <c r="BH30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI30" t="n">
         <v>25</v>
       </c>
-      <c r="BI30" t="n">
+      <c r="BJ30" t="n">
         <v>25</v>
       </c>
     </row>
@@ -6524,9 +6617,12 @@
         <v>0</v>
       </c>
       <c r="BH31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI31" t="n">
         <v>20</v>
       </c>
-      <c r="BI31" t="n">
+      <c r="BJ31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6715,9 +6811,12 @@
         <v>0</v>
       </c>
       <c r="BH32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI32" t="n">
         <v>22</v>
       </c>
-      <c r="BI32" t="n">
+      <c r="BJ32" t="n">
         <v>22</v>
       </c>
     </row>
@@ -6906,10 +7005,13 @@
         <v>1</v>
       </c>
       <c r="BH33" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="BI33" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="BJ33" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="34">
@@ -7097,9 +7199,12 @@
         <v>0</v>
       </c>
       <c r="BH34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI34" t="n">
         <v>9</v>
       </c>
-      <c r="BI34" t="n">
+      <c r="BJ34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7288,9 +7393,12 @@
         <v>1</v>
       </c>
       <c r="BH35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI35" t="n">
         <v>25</v>
       </c>
-      <c r="BI35" t="n">
+      <c r="BJ35" t="n">
         <v>25</v>
       </c>
     </row>
@@ -7479,9 +7587,12 @@
         <v>0</v>
       </c>
       <c r="BH36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI36" t="n">
         <v>15</v>
       </c>
-      <c r="BI36" t="n">
+      <c r="BJ36" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7675,6 +7786,9 @@
       <c r="BI37" t="n">
         <v>0</v>
       </c>
+      <c r="BJ37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7861,9 +7975,12 @@
         <v>0</v>
       </c>
       <c r="BH38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI38" t="n">
         <v>2</v>
       </c>
-      <c r="BI38" t="n">
+      <c r="BJ38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8052,10 +8169,13 @@
         <v>1</v>
       </c>
       <c r="BH39" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="BI39" t="n">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="BJ39" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="40">
@@ -8243,10 +8363,13 @@
         <v>0</v>
       </c>
       <c r="BH40" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BI40" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BJ40" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="41">
@@ -8434,10 +8557,13 @@
         <v>1</v>
       </c>
       <c r="BH41" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="BI41" t="n">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="BJ41" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="42">
@@ -8625,9 +8751,12 @@
         <v>0</v>
       </c>
       <c r="BH42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI42" t="n">
         <v>21</v>
       </c>
-      <c r="BI42" t="n">
+      <c r="BJ42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8816,9 +8945,12 @@
         <v>0</v>
       </c>
       <c r="BH43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI43" t="n">
         <v>60</v>
       </c>
-      <c r="BI43" t="n">
+      <c r="BJ43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9007,9 +9139,12 @@
         <v>1</v>
       </c>
       <c r="BH44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI44" t="n">
         <v>25</v>
       </c>
-      <c r="BI44" t="n">
+      <c r="BJ44" t="n">
         <v>25</v>
       </c>
     </row>
@@ -9198,10 +9333,13 @@
         <v>1</v>
       </c>
       <c r="BH45" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BI45" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BJ45" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="46">
@@ -9389,10 +9527,13 @@
         <v>0</v>
       </c>
       <c r="BH46" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BI46" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BJ46" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="47">
@@ -9585,6 +9726,9 @@
       <c r="BI47" t="n">
         <v>0</v>
       </c>
+      <c r="BJ47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9771,9 +9915,12 @@
         <v>0</v>
       </c>
       <c r="BH48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI48" t="n">
         <v>26</v>
       </c>
-      <c r="BI48" t="n">
+      <c r="BJ48" t="n">
         <v>26</v>
       </c>
     </row>
@@ -9962,9 +10109,12 @@
         <v>0</v>
       </c>
       <c r="BH49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI49" t="n">
         <v>19</v>
       </c>
-      <c r="BI49" t="n">
+      <c r="BJ49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -10153,9 +10303,12 @@
         <v>0</v>
       </c>
       <c r="BH50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI50" t="n">
         <v>7</v>
       </c>
-      <c r="BI50" t="n">
+      <c r="BJ50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10344,9 +10497,12 @@
         <v>0</v>
       </c>
       <c r="BH51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI51" t="n">
         <v>32</v>
       </c>
-      <c r="BI51" t="n">
+      <c r="BJ51" t="n">
         <v>32</v>
       </c>
     </row>
@@ -10540,6 +10696,9 @@
       <c r="BI52" t="n">
         <v>0</v>
       </c>
+      <c r="BJ52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10726,9 +10885,12 @@
         <v>0</v>
       </c>
       <c r="BH53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI53" t="n">
         <v>13</v>
       </c>
-      <c r="BI53" t="n">
+      <c r="BJ53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -10922,6 +11084,9 @@
       <c r="BI54" t="n">
         <v>0</v>
       </c>
+      <c r="BJ54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11108,9 +11273,12 @@
         <v>0</v>
       </c>
       <c r="BH55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI55" t="n">
         <v>33</v>
       </c>
-      <c r="BI55" t="n">
+      <c r="BJ55" t="n">
         <v>33</v>
       </c>
     </row>
@@ -11299,9 +11467,12 @@
         <v>0</v>
       </c>
       <c r="BH56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI56" t="n">
         <v>30</v>
       </c>
-      <c r="BI56" t="n">
+      <c r="BJ56" t="n">
         <v>30</v>
       </c>
     </row>
@@ -11490,9 +11661,12 @@
         <v>0</v>
       </c>
       <c r="BH57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI57" t="n">
         <v>10</v>
       </c>
-      <c r="BI57" t="n">
+      <c r="BJ57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -11681,10 +11855,13 @@
         <v>0</v>
       </c>
       <c r="BH58" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="BI58" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="BJ58" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="59">
@@ -11872,9 +12049,12 @@
         <v>0</v>
       </c>
       <c r="BH59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI59" t="n">
         <v>6</v>
       </c>
-      <c r="BI59" t="n">
+      <c r="BJ59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -12068,6 +12248,9 @@
       <c r="BI60" t="n">
         <v>0</v>
       </c>
+      <c r="BJ60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12254,9 +12437,12 @@
         <v>0</v>
       </c>
       <c r="BH61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI61" t="n">
         <v>29</v>
       </c>
-      <c r="BI61" t="n">
+      <c r="BJ61" t="n">
         <v>29</v>
       </c>
     </row>
@@ -12445,9 +12631,12 @@
         <v>0</v>
       </c>
       <c r="BH62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI62" t="n">
         <v>28</v>
       </c>
-      <c r="BI62" t="n">
+      <c r="BJ62" t="n">
         <v>28</v>
       </c>
     </row>
@@ -12636,9 +12825,12 @@
         <v>0</v>
       </c>
       <c r="BH63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI63" t="n">
         <v>12</v>
       </c>
-      <c r="BI63" t="n">
+      <c r="BJ63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -12832,6 +13024,9 @@
       <c r="BI64" t="n">
         <v>0</v>
       </c>
+      <c r="BJ64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -13018,9 +13213,12 @@
         <v>1</v>
       </c>
       <c r="BH65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI65" t="n">
         <v>17</v>
       </c>
-      <c r="BI65" t="n">
+      <c r="BJ65" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13209,9 +13407,12 @@
         <v>0</v>
       </c>
       <c r="BH66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI66" t="n">
         <v>8</v>
       </c>
-      <c r="BI66" t="n">
+      <c r="BJ66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -13400,10 +13601,13 @@
         <v>1</v>
       </c>
       <c r="BH67" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="BI67" t="n">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="BJ67" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="68">
@@ -13591,10 +13795,13 @@
         <v>1</v>
       </c>
       <c r="BH68" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI68" t="n">
+        <v>22</v>
+      </c>
+      <c r="BJ68" t="n">
         <v>21</v>
-      </c>
-      <c r="BI68" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="69">
@@ -13782,9 +13989,12 @@
         <v>0</v>
       </c>
       <c r="BH69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI69" t="n">
         <v>7</v>
       </c>
-      <c r="BI69" t="n">
+      <c r="BJ69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -13973,9 +14183,12 @@
         <v>0</v>
       </c>
       <c r="BH70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI70" t="n">
         <v>23</v>
       </c>
-      <c r="BI70" t="n">
+      <c r="BJ70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -14164,9 +14377,12 @@
         <v>0</v>
       </c>
       <c r="BH71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI71" t="n">
         <v>24</v>
       </c>
-      <c r="BI71" t="n">
+      <c r="BJ71" t="n">
         <v>24</v>
       </c>
     </row>
@@ -14355,9 +14571,12 @@
         <v>1</v>
       </c>
       <c r="BH72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI72" t="n">
         <v>24</v>
       </c>
-      <c r="BI72" t="n">
+      <c r="BJ72" t="n">
         <v>24</v>
       </c>
     </row>
@@ -14551,6 +14770,9 @@
       <c r="BI73" t="n">
         <v>0</v>
       </c>
+      <c r="BJ73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -14742,6 +14964,9 @@
       <c r="BI74" t="n">
         <v>0</v>
       </c>
+      <c r="BJ74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -14928,9 +15153,12 @@
         <v>0</v>
       </c>
       <c r="BH75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI75" t="n">
         <v>23</v>
       </c>
-      <c r="BI75" t="n">
+      <c r="BJ75" t="n">
         <v>23</v>
       </c>
     </row>
@@ -15119,9 +15347,12 @@
         <v>0</v>
       </c>
       <c r="BH76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI76" t="n">
         <v>21</v>
       </c>
-      <c r="BI76" t="n">
+      <c r="BJ76" t="n">
         <v>21</v>
       </c>
     </row>
@@ -15310,9 +15541,12 @@
         <v>0</v>
       </c>
       <c r="BH77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI77" t="n">
         <v>15</v>
       </c>
-      <c r="BI77" t="n">
+      <c r="BJ77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -15501,9 +15735,12 @@
         <v>1</v>
       </c>
       <c r="BH78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI78" t="n">
         <v>33</v>
       </c>
-      <c r="BI78" t="n">
+      <c r="BJ78" t="n">
         <v>32</v>
       </c>
     </row>
@@ -15692,9 +15929,12 @@
         <v>0</v>
       </c>
       <c r="BH79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI79" t="n">
         <v>22</v>
       </c>
-      <c r="BI79" t="n">
+      <c r="BJ79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -15883,9 +16123,12 @@
         <v>0</v>
       </c>
       <c r="BH80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI80" t="n">
         <v>11</v>
       </c>
-      <c r="BI80" t="n">
+      <c r="BJ80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -16074,9 +16317,12 @@
         <v>0</v>
       </c>
       <c r="BH81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI81" t="n">
         <v>4</v>
       </c>
-      <c r="BI81" t="n">
+      <c r="BJ81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -16265,9 +16511,12 @@
         <v>0</v>
       </c>
       <c r="BH82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI82" t="n">
         <v>17</v>
       </c>
-      <c r="BI82" t="n">
+      <c r="BJ82" t="n">
         <v>17</v>
       </c>
     </row>
@@ -16456,9 +16705,12 @@
         <v>0</v>
       </c>
       <c r="BH83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI83" t="n">
         <v>17</v>
       </c>
-      <c r="BI83" t="n">
+      <c r="BJ83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -16647,9 +16899,12 @@
         <v>0</v>
       </c>
       <c r="BH84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI84" t="n">
         <v>13</v>
       </c>
-      <c r="BI84" t="n">
+      <c r="BJ84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -16838,9 +17093,12 @@
         <v>0</v>
       </c>
       <c r="BH85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI85" t="n">
         <v>7</v>
       </c>
-      <c r="BI85" t="n">
+      <c r="BJ85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17034,6 +17292,9 @@
       <c r="BI86" t="n">
         <v>0</v>
       </c>
+      <c r="BJ86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -17220,9 +17481,12 @@
         <v>0</v>
       </c>
       <c r="BH87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI87" t="n">
         <v>18</v>
       </c>
-      <c r="BI87" t="n">
+      <c r="BJ87" t="n">
         <v>18</v>
       </c>
     </row>
@@ -17416,6 +17680,9 @@
       <c r="BI88" t="n">
         <v>0</v>
       </c>
+      <c r="BJ88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -17602,9 +17869,12 @@
         <v>1</v>
       </c>
       <c r="BH89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI89" t="n">
         <v>18</v>
       </c>
-      <c r="BI89" t="n">
+      <c r="BJ89" t="n">
         <v>18</v>
       </c>
     </row>
@@ -17793,9 +18063,12 @@
         <v>1</v>
       </c>
       <c r="BH90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI90" t="n">
         <v>17</v>
       </c>
-      <c r="BI90" t="n">
+      <c r="BJ90" t="n">
         <v>17</v>
       </c>
     </row>
@@ -17984,9 +18257,12 @@
         <v>0</v>
       </c>
       <c r="BH91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI91" t="n">
         <v>42</v>
       </c>
-      <c r="BI91" t="n">
+      <c r="BJ91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -18175,9 +18451,12 @@
         <v>0</v>
       </c>
       <c r="BH92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI92" t="n">
         <v>7</v>
       </c>
-      <c r="BI92" t="n">
+      <c r="BJ92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18371,6 +18650,9 @@
       <c r="BI93" t="n">
         <v>0</v>
       </c>
+      <c r="BJ93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -18557,9 +18839,12 @@
         <v>0</v>
       </c>
       <c r="BH94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI94" t="n">
         <v>16</v>
       </c>
-      <c r="BI94" t="n">
+      <c r="BJ94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -18748,9 +19033,12 @@
         <v>0</v>
       </c>
       <c r="BH95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI95" t="n">
         <v>7</v>
       </c>
-      <c r="BI95" t="n">
+      <c r="BJ95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18939,9 +19227,12 @@
         <v>0</v>
       </c>
       <c r="BH96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI96" t="n">
         <v>24</v>
       </c>
-      <c r="BI96" t="n">
+      <c r="BJ96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -19135,6 +19426,9 @@
       <c r="BI97" t="n">
         <v>0</v>
       </c>
+      <c r="BJ97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -19321,9 +19615,12 @@
         <v>1</v>
       </c>
       <c r="BH98" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI98" t="n">
         <v>32</v>
       </c>
-      <c r="BI98" t="n">
+      <c r="BJ98" t="n">
         <v>32</v>
       </c>
     </row>
@@ -19512,9 +19809,12 @@
         <v>1</v>
       </c>
       <c r="BH99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI99" t="n">
         <v>14</v>
       </c>
-      <c r="BI99" t="n">
+      <c r="BJ99" t="n">
         <v>14</v>
       </c>
     </row>
@@ -19708,6 +20008,9 @@
       <c r="BI100" t="n">
         <v>0</v>
       </c>
+      <c r="BJ100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -19894,10 +20197,13 @@
         <v>1</v>
       </c>
       <c r="BH101" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BI101" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BJ101" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="102">
@@ -20085,9 +20391,12 @@
         <v>0</v>
       </c>
       <c r="BH102" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI102" t="n">
         <v>28</v>
       </c>
-      <c r="BI102" t="n">
+      <c r="BJ102" t="n">
         <v>28</v>
       </c>
     </row>
@@ -20276,9 +20585,12 @@
         <v>0</v>
       </c>
       <c r="BH103" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI103" t="n">
         <v>31</v>
       </c>
-      <c r="BI103" t="n">
+      <c r="BJ103" t="n">
         <v>31</v>
       </c>
     </row>
@@ -20467,9 +20779,12 @@
         <v>0</v>
       </c>
       <c r="BH104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI104" t="n">
         <v>12</v>
       </c>
-      <c r="BI104" t="n">
+      <c r="BJ104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -20658,10 +20973,13 @@
         <v>1</v>
       </c>
       <c r="BH105" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BI105" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BJ105" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="106">
@@ -20849,9 +21167,12 @@
         <v>0</v>
       </c>
       <c r="BH106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI106" t="n">
         <v>7</v>
       </c>
-      <c r="BI106" t="n">
+      <c r="BJ106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -21040,9 +21361,12 @@
         <v>0</v>
       </c>
       <c r="BH107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI107" t="n">
         <v>13</v>
       </c>
-      <c r="BI107" t="n">
+      <c r="BJ107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -21231,9 +21555,12 @@
         <v>0</v>
       </c>
       <c r="BH108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI108" t="n">
         <v>2</v>
       </c>
-      <c r="BI108" t="n">
+      <c r="BJ108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -21422,9 +21749,12 @@
         <v>0</v>
       </c>
       <c r="BH109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI109" t="n">
         <v>4</v>
       </c>
-      <c r="BI109" t="n">
+      <c r="BJ109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#4251)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ109"/>
+  <dimension ref="A1:BK109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -490,8 +490,9 @@
     <col width="12" customWidth="1" min="58" max="58"/>
     <col width="12" customWidth="1" min="59" max="59"/>
     <col width="12" customWidth="1" min="60" max="60"/>
-    <col width="13" customWidth="1" min="61" max="61"/>
+    <col width="12" customWidth="1" min="61" max="61"/>
     <col width="13" customWidth="1" min="62" max="62"/>
+    <col width="13" customWidth="1" min="63" max="63"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -795,12 +796,17 @@
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="BI1" s="2" t="inlineStr">
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="BJ1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BJ1" s="2" t="inlineStr">
+      <c r="BK1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -994,9 +1000,12 @@
         <v>0</v>
       </c>
       <c r="BI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ2" t="n">
         <v>12</v>
       </c>
-      <c r="BJ2" t="n">
+      <c r="BK2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1188,9 +1197,12 @@
         <v>0</v>
       </c>
       <c r="BI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ3" t="n">
         <v>10</v>
       </c>
-      <c r="BJ3" t="n">
+      <c r="BK3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1382,10 +1394,13 @@
         <v>1</v>
       </c>
       <c r="BI4" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="BJ4" t="n">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -1576,9 +1591,12 @@
         <v>0</v>
       </c>
       <c r="BI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ5" t="n">
         <v>15</v>
       </c>
-      <c r="BJ5" t="n">
+      <c r="BK5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1770,9 +1788,12 @@
         <v>0</v>
       </c>
       <c r="BI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ6" t="n">
         <v>19</v>
       </c>
-      <c r="BJ6" t="n">
+      <c r="BK6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1964,9 +1985,12 @@
         <v>0</v>
       </c>
       <c r="BI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ7" t="n">
         <v>19</v>
       </c>
-      <c r="BJ7" t="n">
+      <c r="BK7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2158,10 +2182,13 @@
         <v>0</v>
       </c>
       <c r="BI8" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BJ8" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -2352,9 +2379,12 @@
         <v>1</v>
       </c>
       <c r="BI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ9" t="n">
         <v>29</v>
       </c>
-      <c r="BJ9" t="n">
+      <c r="BK9" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2546,10 +2576,13 @@
         <v>0</v>
       </c>
       <c r="BI10" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="BJ10" t="n">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="11">
@@ -2740,10 +2773,13 @@
         <v>1</v>
       </c>
       <c r="BI11" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BJ11" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="12">
@@ -2934,10 +2970,13 @@
         <v>1</v>
       </c>
       <c r="BI12" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="BJ12" t="n">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="13">
@@ -3128,9 +3167,12 @@
         <v>0</v>
       </c>
       <c r="BI13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ13" t="n">
         <v>14</v>
       </c>
-      <c r="BJ13" t="n">
+      <c r="BK13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3322,9 +3364,12 @@
         <v>0</v>
       </c>
       <c r="BI14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ14" t="n">
         <v>25</v>
       </c>
-      <c r="BJ14" t="n">
+      <c r="BK14" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3516,9 +3561,12 @@
         <v>0</v>
       </c>
       <c r="BI15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ15" t="n">
         <v>9</v>
       </c>
-      <c r="BJ15" t="n">
+      <c r="BK15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3710,9 +3758,12 @@
         <v>0</v>
       </c>
       <c r="BI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ16" t="n">
         <v>20</v>
       </c>
-      <c r="BJ16" t="n">
+      <c r="BK16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3904,9 +3955,12 @@
         <v>0</v>
       </c>
       <c r="BI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ17" t="n">
         <v>17</v>
       </c>
-      <c r="BJ17" t="n">
+      <c r="BK17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4098,10 +4152,13 @@
         <v>0</v>
       </c>
       <c r="BI18" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BJ18" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BK18" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="19">
@@ -4297,6 +4354,9 @@
       <c r="BJ19" t="n">
         <v>0</v>
       </c>
+      <c r="BK19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4486,9 +4546,12 @@
         <v>1</v>
       </c>
       <c r="BI20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ20" t="n">
         <v>20</v>
       </c>
-      <c r="BJ20" t="n">
+      <c r="BK20" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4680,9 +4743,12 @@
         <v>0</v>
       </c>
       <c r="BI21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ21" t="n">
         <v>27</v>
       </c>
-      <c r="BJ21" t="n">
+      <c r="BK21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -4879,6 +4945,9 @@
       <c r="BJ22" t="n">
         <v>0</v>
       </c>
+      <c r="BK22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5068,9 +5137,12 @@
         <v>0</v>
       </c>
       <c r="BI23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ23" t="n">
         <v>21</v>
       </c>
-      <c r="BJ23" t="n">
+      <c r="BK23" t="n">
         <v>21</v>
       </c>
     </row>
@@ -5262,9 +5334,12 @@
         <v>0</v>
       </c>
       <c r="BI24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ24" t="n">
         <v>27</v>
       </c>
-      <c r="BJ24" t="n">
+      <c r="BK24" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5456,9 +5531,12 @@
         <v>0</v>
       </c>
       <c r="BI25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ25" t="n">
         <v>11</v>
       </c>
-      <c r="BJ25" t="n">
+      <c r="BK25" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5650,10 +5728,13 @@
         <v>1</v>
       </c>
       <c r="BI26" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="BJ26" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="BK26" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="27">
@@ -5844,9 +5925,12 @@
         <v>0</v>
       </c>
       <c r="BI27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ27" t="n">
         <v>25</v>
       </c>
-      <c r="BJ27" t="n">
+      <c r="BK27" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6038,9 +6122,12 @@
         <v>1</v>
       </c>
       <c r="BI28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ28" t="n">
         <v>19</v>
       </c>
-      <c r="BJ28" t="n">
+      <c r="BK28" t="n">
         <v>19</v>
       </c>
     </row>
@@ -6232,9 +6319,12 @@
         <v>0</v>
       </c>
       <c r="BI29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ29" t="n">
         <v>11</v>
       </c>
-      <c r="BJ29" t="n">
+      <c r="BK29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6426,9 +6516,12 @@
         <v>0</v>
       </c>
       <c r="BI30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ30" t="n">
         <v>25</v>
       </c>
-      <c r="BJ30" t="n">
+      <c r="BK30" t="n">
         <v>25</v>
       </c>
     </row>
@@ -6620,9 +6713,12 @@
         <v>0</v>
       </c>
       <c r="BI31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ31" t="n">
         <v>20</v>
       </c>
-      <c r="BJ31" t="n">
+      <c r="BK31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6814,9 +6910,12 @@
         <v>0</v>
       </c>
       <c r="BI32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ32" t="n">
         <v>22</v>
       </c>
-      <c r="BJ32" t="n">
+      <c r="BK32" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7008,10 +7107,13 @@
         <v>1</v>
       </c>
       <c r="BI33" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="BJ33" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="BK33" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="34">
@@ -7202,9 +7304,12 @@
         <v>0</v>
       </c>
       <c r="BI34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ34" t="n">
         <v>9</v>
       </c>
-      <c r="BJ34" t="n">
+      <c r="BK34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7396,9 +7501,12 @@
         <v>0</v>
       </c>
       <c r="BI35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ35" t="n">
         <v>25</v>
       </c>
-      <c r="BJ35" t="n">
+      <c r="BK35" t="n">
         <v>25</v>
       </c>
     </row>
@@ -7590,9 +7698,12 @@
         <v>0</v>
       </c>
       <c r="BI36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ36" t="n">
         <v>15</v>
       </c>
-      <c r="BJ36" t="n">
+      <c r="BK36" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7789,6 +7900,9 @@
       <c r="BJ37" t="n">
         <v>0</v>
       </c>
+      <c r="BK37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7978,9 +8092,12 @@
         <v>0</v>
       </c>
       <c r="BI38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ38" t="n">
         <v>2</v>
       </c>
-      <c r="BJ38" t="n">
+      <c r="BK38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8172,10 +8289,13 @@
         <v>1</v>
       </c>
       <c r="BI39" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="BJ39" t="n">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="BK39" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="40">
@@ -8366,10 +8486,13 @@
         <v>1</v>
       </c>
       <c r="BI40" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BJ40" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BK40" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="41">
@@ -8560,10 +8683,13 @@
         <v>1</v>
       </c>
       <c r="BI41" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="BJ41" t="n">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="BK41" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="42">
@@ -8754,9 +8880,12 @@
         <v>0</v>
       </c>
       <c r="BI42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ42" t="n">
         <v>21</v>
       </c>
-      <c r="BJ42" t="n">
+      <c r="BK42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8948,9 +9077,12 @@
         <v>0</v>
       </c>
       <c r="BI43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ43" t="n">
         <v>60</v>
       </c>
-      <c r="BJ43" t="n">
+      <c r="BK43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9142,9 +9274,12 @@
         <v>0</v>
       </c>
       <c r="BI44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ44" t="n">
         <v>25</v>
       </c>
-      <c r="BJ44" t="n">
+      <c r="BK44" t="n">
         <v>25</v>
       </c>
     </row>
@@ -9336,9 +9471,12 @@
         <v>1</v>
       </c>
       <c r="BI45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ45" t="n">
         <v>26</v>
       </c>
-      <c r="BJ45" t="n">
+      <c r="BK45" t="n">
         <v>26</v>
       </c>
     </row>
@@ -9530,9 +9668,12 @@
         <v>1</v>
       </c>
       <c r="BI46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ46" t="n">
         <v>30</v>
       </c>
-      <c r="BJ46" t="n">
+      <c r="BK46" t="n">
         <v>30</v>
       </c>
     </row>
@@ -9729,6 +9870,9 @@
       <c r="BJ47" t="n">
         <v>0</v>
       </c>
+      <c r="BK47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9918,9 +10062,12 @@
         <v>0</v>
       </c>
       <c r="BI48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ48" t="n">
         <v>26</v>
       </c>
-      <c r="BJ48" t="n">
+      <c r="BK48" t="n">
         <v>26</v>
       </c>
     </row>
@@ -10112,9 +10259,12 @@
         <v>0</v>
       </c>
       <c r="BI49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ49" t="n">
         <v>19</v>
       </c>
-      <c r="BJ49" t="n">
+      <c r="BK49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -10306,9 +10456,12 @@
         <v>0</v>
       </c>
       <c r="BI50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ50" t="n">
         <v>7</v>
       </c>
-      <c r="BJ50" t="n">
+      <c r="BK50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10500,9 +10653,12 @@
         <v>0</v>
       </c>
       <c r="BI51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ51" t="n">
         <v>32</v>
       </c>
-      <c r="BJ51" t="n">
+      <c r="BK51" t="n">
         <v>32</v>
       </c>
     </row>
@@ -10699,6 +10855,9 @@
       <c r="BJ52" t="n">
         <v>0</v>
       </c>
+      <c r="BK52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10888,9 +11047,12 @@
         <v>0</v>
       </c>
       <c r="BI53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ53" t="n">
         <v>13</v>
       </c>
-      <c r="BJ53" t="n">
+      <c r="BK53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -11087,6 +11249,9 @@
       <c r="BJ54" t="n">
         <v>0</v>
       </c>
+      <c r="BK54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11276,10 +11441,13 @@
         <v>0</v>
       </c>
       <c r="BI55" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="BJ55" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="BK55" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="56">
@@ -11470,10 +11638,13 @@
         <v>0</v>
       </c>
       <c r="BI56" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BJ56" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BK56" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="57">
@@ -11664,9 +11835,12 @@
         <v>0</v>
       </c>
       <c r="BI57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ57" t="n">
         <v>10</v>
       </c>
-      <c r="BJ57" t="n">
+      <c r="BK57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -11858,9 +12032,12 @@
         <v>1</v>
       </c>
       <c r="BI58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ58" t="n">
         <v>13</v>
       </c>
-      <c r="BJ58" t="n">
+      <c r="BK58" t="n">
         <v>13</v>
       </c>
     </row>
@@ -12052,9 +12229,12 @@
         <v>0</v>
       </c>
       <c r="BI59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ59" t="n">
         <v>6</v>
       </c>
-      <c r="BJ59" t="n">
+      <c r="BK59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -12251,6 +12431,9 @@
       <c r="BJ60" t="n">
         <v>0</v>
       </c>
+      <c r="BK60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12440,9 +12623,12 @@
         <v>0</v>
       </c>
       <c r="BI61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ61" t="n">
         <v>29</v>
       </c>
-      <c r="BJ61" t="n">
+      <c r="BK61" t="n">
         <v>29</v>
       </c>
     </row>
@@ -12634,10 +12820,13 @@
         <v>0</v>
       </c>
       <c r="BI62" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BJ62" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BK62" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="63">
@@ -12828,9 +13017,12 @@
         <v>0</v>
       </c>
       <c r="BI63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ63" t="n">
         <v>12</v>
       </c>
-      <c r="BJ63" t="n">
+      <c r="BK63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -13027,6 +13219,9 @@
       <c r="BJ64" t="n">
         <v>0</v>
       </c>
+      <c r="BK64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -13216,9 +13411,12 @@
         <v>0</v>
       </c>
       <c r="BI65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ65" t="n">
         <v>17</v>
       </c>
-      <c r="BJ65" t="n">
+      <c r="BK65" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13410,9 +13608,12 @@
         <v>0</v>
       </c>
       <c r="BI66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ66" t="n">
         <v>8</v>
       </c>
-      <c r="BJ66" t="n">
+      <c r="BK66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -13604,10 +13805,13 @@
         <v>1</v>
       </c>
       <c r="BI67" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="BJ67" t="n">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="BK67" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="68">
@@ -13798,9 +14002,12 @@
         <v>1</v>
       </c>
       <c r="BI68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ68" t="n">
         <v>22</v>
       </c>
-      <c r="BJ68" t="n">
+      <c r="BK68" t="n">
         <v>21</v>
       </c>
     </row>
@@ -13992,9 +14199,12 @@
         <v>0</v>
       </c>
       <c r="BI69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ69" t="n">
         <v>7</v>
       </c>
-      <c r="BJ69" t="n">
+      <c r="BK69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14186,9 +14396,12 @@
         <v>0</v>
       </c>
       <c r="BI70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ70" t="n">
         <v>23</v>
       </c>
-      <c r="BJ70" t="n">
+      <c r="BK70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -14380,9 +14593,12 @@
         <v>0</v>
       </c>
       <c r="BI71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ71" t="n">
         <v>24</v>
       </c>
-      <c r="BJ71" t="n">
+      <c r="BK71" t="n">
         <v>24</v>
       </c>
     </row>
@@ -14574,9 +14790,12 @@
         <v>0</v>
       </c>
       <c r="BI72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ72" t="n">
         <v>24</v>
       </c>
-      <c r="BJ72" t="n">
+      <c r="BK72" t="n">
         <v>24</v>
       </c>
     </row>
@@ -14773,6 +14992,9 @@
       <c r="BJ73" t="n">
         <v>0</v>
       </c>
+      <c r="BK73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -14967,6 +15189,9 @@
       <c r="BJ74" t="n">
         <v>0</v>
       </c>
+      <c r="BK74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -15156,9 +15381,12 @@
         <v>0</v>
       </c>
       <c r="BI75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ75" t="n">
         <v>23</v>
       </c>
-      <c r="BJ75" t="n">
+      <c r="BK75" t="n">
         <v>23</v>
       </c>
     </row>
@@ -15350,9 +15578,12 @@
         <v>0</v>
       </c>
       <c r="BI76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ76" t="n">
         <v>21</v>
       </c>
-      <c r="BJ76" t="n">
+      <c r="BK76" t="n">
         <v>21</v>
       </c>
     </row>
@@ -15544,9 +15775,12 @@
         <v>0</v>
       </c>
       <c r="BI77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ77" t="n">
         <v>15</v>
       </c>
-      <c r="BJ77" t="n">
+      <c r="BK77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -15738,10 +15972,13 @@
         <v>0</v>
       </c>
       <c r="BI78" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ78" t="n">
+        <v>34</v>
+      </c>
+      <c r="BK78" t="n">
         <v>33</v>
-      </c>
-      <c r="BJ78" t="n">
-        <v>32</v>
       </c>
     </row>
     <row r="79">
@@ -15932,9 +16169,12 @@
         <v>0</v>
       </c>
       <c r="BI79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ79" t="n">
         <v>22</v>
       </c>
-      <c r="BJ79" t="n">
+      <c r="BK79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -16126,9 +16366,12 @@
         <v>0</v>
       </c>
       <c r="BI80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ80" t="n">
         <v>11</v>
       </c>
-      <c r="BJ80" t="n">
+      <c r="BK80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -16320,9 +16563,12 @@
         <v>0</v>
       </c>
       <c r="BI81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ81" t="n">
         <v>4</v>
       </c>
-      <c r="BJ81" t="n">
+      <c r="BK81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -16514,10 +16760,13 @@
         <v>0</v>
       </c>
       <c r="BI82" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="BJ82" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="BK82" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="83">
@@ -16708,9 +16957,12 @@
         <v>0</v>
       </c>
       <c r="BI83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ83" t="n">
         <v>17</v>
       </c>
-      <c r="BJ83" t="n">
+      <c r="BK83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -16902,9 +17154,12 @@
         <v>0</v>
       </c>
       <c r="BI84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ84" t="n">
         <v>13</v>
       </c>
-      <c r="BJ84" t="n">
+      <c r="BK84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -17096,9 +17351,12 @@
         <v>0</v>
       </c>
       <c r="BI85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ85" t="n">
         <v>7</v>
       </c>
-      <c r="BJ85" t="n">
+      <c r="BK85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17295,6 +17553,9 @@
       <c r="BJ86" t="n">
         <v>0</v>
       </c>
+      <c r="BK86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -17484,9 +17745,12 @@
         <v>0</v>
       </c>
       <c r="BI87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ87" t="n">
         <v>18</v>
       </c>
-      <c r="BJ87" t="n">
+      <c r="BK87" t="n">
         <v>18</v>
       </c>
     </row>
@@ -17683,6 +17947,9 @@
       <c r="BJ88" t="n">
         <v>0</v>
       </c>
+      <c r="BK88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -17872,9 +18139,12 @@
         <v>0</v>
       </c>
       <c r="BI89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ89" t="n">
         <v>18</v>
       </c>
-      <c r="BJ89" t="n">
+      <c r="BK89" t="n">
         <v>18</v>
       </c>
     </row>
@@ -18066,9 +18336,12 @@
         <v>0</v>
       </c>
       <c r="BI90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ90" t="n">
         <v>17</v>
       </c>
-      <c r="BJ90" t="n">
+      <c r="BK90" t="n">
         <v>17</v>
       </c>
     </row>
@@ -18260,9 +18533,12 @@
         <v>0</v>
       </c>
       <c r="BI91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ91" t="n">
         <v>42</v>
       </c>
-      <c r="BJ91" t="n">
+      <c r="BK91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -18454,9 +18730,12 @@
         <v>0</v>
       </c>
       <c r="BI92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ92" t="n">
         <v>7</v>
       </c>
-      <c r="BJ92" t="n">
+      <c r="BK92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18653,6 +18932,9 @@
       <c r="BJ93" t="n">
         <v>0</v>
       </c>
+      <c r="BK93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -18842,9 +19124,12 @@
         <v>0</v>
       </c>
       <c r="BI94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ94" t="n">
         <v>16</v>
       </c>
-      <c r="BJ94" t="n">
+      <c r="BK94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -19036,9 +19321,12 @@
         <v>0</v>
       </c>
       <c r="BI95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ95" t="n">
         <v>7</v>
       </c>
-      <c r="BJ95" t="n">
+      <c r="BK95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -19230,9 +19518,12 @@
         <v>0</v>
       </c>
       <c r="BI96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ96" t="n">
         <v>24</v>
       </c>
-      <c r="BJ96" t="n">
+      <c r="BK96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -19429,6 +19720,9 @@
       <c r="BJ97" t="n">
         <v>0</v>
       </c>
+      <c r="BK97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -19618,10 +19912,13 @@
         <v>0</v>
       </c>
       <c r="BI98" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="BJ98" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="BK98" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="99">
@@ -19812,9 +20109,12 @@
         <v>0</v>
       </c>
       <c r="BI99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ99" t="n">
         <v>14</v>
       </c>
-      <c r="BJ99" t="n">
+      <c r="BK99" t="n">
         <v>14</v>
       </c>
     </row>
@@ -20011,6 +20311,9 @@
       <c r="BJ100" t="n">
         <v>0</v>
       </c>
+      <c r="BK100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -20200,9 +20503,12 @@
         <v>1</v>
       </c>
       <c r="BI101" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ101" t="n">
         <v>30</v>
       </c>
-      <c r="BJ101" t="n">
+      <c r="BK101" t="n">
         <v>30</v>
       </c>
     </row>
@@ -20394,10 +20700,13 @@
         <v>0</v>
       </c>
       <c r="BI102" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="BJ102" t="n">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="BK102" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="103">
@@ -20588,10 +20897,13 @@
         <v>0</v>
       </c>
       <c r="BI103" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BJ103" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BK103" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="104">
@@ -20782,9 +21094,12 @@
         <v>0</v>
       </c>
       <c r="BI104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ104" t="n">
         <v>12</v>
       </c>
-      <c r="BJ104" t="n">
+      <c r="BK104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -20976,10 +21291,13 @@
         <v>1</v>
       </c>
       <c r="BI105" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BJ105" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BK105" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="106">
@@ -21170,9 +21488,12 @@
         <v>0</v>
       </c>
       <c r="BI106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ106" t="n">
         <v>7</v>
       </c>
-      <c r="BJ106" t="n">
+      <c r="BK106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -21364,9 +21685,12 @@
         <v>0</v>
       </c>
       <c r="BI107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ107" t="n">
         <v>13</v>
       </c>
-      <c r="BJ107" t="n">
+      <c r="BK107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -21558,9 +21882,12 @@
         <v>0</v>
       </c>
       <c r="BI108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ108" t="n">
         <v>2</v>
       </c>
-      <c r="BJ108" t="n">
+      <c r="BK108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -21752,9 +22079,12 @@
         <v>0</v>
       </c>
       <c r="BI109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ109" t="n">
         <v>4</v>
       </c>
-      <c r="BJ109" t="n">
+      <c r="BK109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#4355)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK109"/>
+  <dimension ref="A1:BL109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -491,8 +491,9 @@
     <col width="12" customWidth="1" min="59" max="59"/>
     <col width="12" customWidth="1" min="60" max="60"/>
     <col width="12" customWidth="1" min="61" max="61"/>
-    <col width="13" customWidth="1" min="62" max="62"/>
+    <col width="12" customWidth="1" min="62" max="62"/>
     <col width="13" customWidth="1" min="63" max="63"/>
+    <col width="13" customWidth="1" min="64" max="64"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -801,12 +802,17 @@
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="BJ1" s="2" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="BK1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BK1" s="2" t="inlineStr">
+      <c r="BL1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -1003,9 +1009,12 @@
         <v>0</v>
       </c>
       <c r="BJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK2" t="n">
         <v>12</v>
       </c>
-      <c r="BK2" t="n">
+      <c r="BL2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1200,9 +1209,12 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK3" t="n">
         <v>10</v>
       </c>
-      <c r="BK3" t="n">
+      <c r="BL3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1397,10 +1409,13 @@
         <v>1</v>
       </c>
       <c r="BJ4" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="BK4" t="n">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -1594,9 +1609,12 @@
         <v>0</v>
       </c>
       <c r="BJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK5" t="n">
         <v>15</v>
       </c>
-      <c r="BK5" t="n">
+      <c r="BL5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1791,9 +1809,12 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK6" t="n">
         <v>19</v>
       </c>
-      <c r="BK6" t="n">
+      <c r="BL6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1988,9 +2009,12 @@
         <v>0</v>
       </c>
       <c r="BJ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK7" t="n">
         <v>19</v>
       </c>
-      <c r="BK7" t="n">
+      <c r="BL7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2185,9 +2209,12 @@
         <v>1</v>
       </c>
       <c r="BJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK8" t="n">
         <v>31</v>
       </c>
-      <c r="BK8" t="n">
+      <c r="BL8" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2382,10 +2409,13 @@
         <v>0</v>
       </c>
       <c r="BJ9" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BK9" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="10">
@@ -2579,10 +2609,13 @@
         <v>1</v>
       </c>
       <c r="BJ10" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="BK10" t="n">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="11">
@@ -2776,9 +2809,12 @@
         <v>1</v>
       </c>
       <c r="BJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK11" t="n">
         <v>29</v>
       </c>
-      <c r="BK11" t="n">
+      <c r="BL11" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2973,10 +3009,13 @@
         <v>1</v>
       </c>
       <c r="BJ12" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="BK12" t="n">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="BL12" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="13">
@@ -3170,9 +3209,12 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK13" t="n">
         <v>14</v>
       </c>
-      <c r="BK13" t="n">
+      <c r="BL13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3367,10 +3409,13 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="BK14" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="BL14" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="15">
@@ -3564,9 +3609,12 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK15" t="n">
         <v>9</v>
       </c>
-      <c r="BK15" t="n">
+      <c r="BL15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3761,9 +3809,12 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK16" t="n">
         <v>20</v>
       </c>
-      <c r="BK16" t="n">
+      <c r="BL16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3958,9 +4009,12 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK17" t="n">
         <v>17</v>
       </c>
-      <c r="BK17" t="n">
+      <c r="BL17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4155,10 +4209,13 @@
         <v>1</v>
       </c>
       <c r="BJ18" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BK18" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BL18" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="19">
@@ -4357,6 +4414,9 @@
       <c r="BK19" t="n">
         <v>0</v>
       </c>
+      <c r="BL19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4549,9 +4609,12 @@
         <v>0</v>
       </c>
       <c r="BJ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK20" t="n">
         <v>20</v>
       </c>
-      <c r="BK20" t="n">
+      <c r="BL20" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4746,9 +4809,12 @@
         <v>0</v>
       </c>
       <c r="BJ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK21" t="n">
         <v>27</v>
       </c>
-      <c r="BK21" t="n">
+      <c r="BL21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -4948,6 +5014,9 @@
       <c r="BK22" t="n">
         <v>0</v>
       </c>
+      <c r="BL22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5140,10 +5209,13 @@
         <v>0</v>
       </c>
       <c r="BJ23" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="BK23" t="n">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="BL23" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="24">
@@ -5337,9 +5409,12 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK24" t="n">
         <v>27</v>
       </c>
-      <c r="BK24" t="n">
+      <c r="BL24" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5534,9 +5609,12 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK25" t="n">
         <v>11</v>
       </c>
-      <c r="BK25" t="n">
+      <c r="BL25" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5731,10 +5809,13 @@
         <v>1</v>
       </c>
       <c r="BJ26" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="BK26" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="BL26" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="27">
@@ -5928,9 +6009,12 @@
         <v>0</v>
       </c>
       <c r="BJ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK27" t="n">
         <v>25</v>
       </c>
-      <c r="BK27" t="n">
+      <c r="BL27" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6125,9 +6209,12 @@
         <v>0</v>
       </c>
       <c r="BJ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK28" t="n">
         <v>19</v>
       </c>
-      <c r="BK28" t="n">
+      <c r="BL28" t="n">
         <v>19</v>
       </c>
     </row>
@@ -6322,9 +6409,12 @@
         <v>0</v>
       </c>
       <c r="BJ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK29" t="n">
         <v>11</v>
       </c>
-      <c r="BK29" t="n">
+      <c r="BL29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6519,9 +6609,12 @@
         <v>0</v>
       </c>
       <c r="BJ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK30" t="n">
         <v>25</v>
       </c>
-      <c r="BK30" t="n">
+      <c r="BL30" t="n">
         <v>25</v>
       </c>
     </row>
@@ -6716,9 +6809,12 @@
         <v>0</v>
       </c>
       <c r="BJ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK31" t="n">
         <v>20</v>
       </c>
-      <c r="BK31" t="n">
+      <c r="BL31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6913,9 +7009,12 @@
         <v>0</v>
       </c>
       <c r="BJ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK32" t="n">
         <v>22</v>
       </c>
-      <c r="BK32" t="n">
+      <c r="BL32" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7110,10 +7209,13 @@
         <v>1</v>
       </c>
       <c r="BJ33" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="BK33" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="BL33" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="34">
@@ -7307,9 +7409,12 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK34" t="n">
         <v>9</v>
       </c>
-      <c r="BK34" t="n">
+      <c r="BL34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7504,9 +7609,12 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK35" t="n">
         <v>25</v>
       </c>
-      <c r="BK35" t="n">
+      <c r="BL35" t="n">
         <v>25</v>
       </c>
     </row>
@@ -7701,10 +7809,13 @@
         <v>0</v>
       </c>
       <c r="BJ36" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="BK36" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="BL36" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="37">
@@ -7903,6 +8014,9 @@
       <c r="BK37" t="n">
         <v>0</v>
       </c>
+      <c r="BL37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8095,9 +8209,12 @@
         <v>0</v>
       </c>
       <c r="BJ38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK38" t="n">
         <v>2</v>
       </c>
-      <c r="BK38" t="n">
+      <c r="BL38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8292,9 +8409,12 @@
         <v>1</v>
       </c>
       <c r="BJ39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK39" t="n">
         <v>36</v>
       </c>
-      <c r="BK39" t="n">
+      <c r="BL39" t="n">
         <v>36</v>
       </c>
     </row>
@@ -8489,10 +8609,13 @@
         <v>1</v>
       </c>
       <c r="BJ40" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BK40" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BL40" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="41">
@@ -8686,10 +8809,13 @@
         <v>1</v>
       </c>
       <c r="BJ41" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="BK41" t="n">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="BL41" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="42">
@@ -8883,9 +9009,12 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK42" t="n">
         <v>21</v>
       </c>
-      <c r="BK42" t="n">
+      <c r="BL42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9080,9 +9209,12 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK43" t="n">
         <v>60</v>
       </c>
-      <c r="BK43" t="n">
+      <c r="BL43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9277,9 +9409,12 @@
         <v>0</v>
       </c>
       <c r="BJ44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK44" t="n">
         <v>25</v>
       </c>
-      <c r="BK44" t="n">
+      <c r="BL44" t="n">
         <v>25</v>
       </c>
     </row>
@@ -9474,9 +9609,12 @@
         <v>0</v>
       </c>
       <c r="BJ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK45" t="n">
         <v>26</v>
       </c>
-      <c r="BK45" t="n">
+      <c r="BL45" t="n">
         <v>26</v>
       </c>
     </row>
@@ -9671,9 +9809,12 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK46" t="n">
         <v>30</v>
       </c>
-      <c r="BK46" t="n">
+      <c r="BL46" t="n">
         <v>30</v>
       </c>
     </row>
@@ -9873,6 +10014,9 @@
       <c r="BK47" t="n">
         <v>0</v>
       </c>
+      <c r="BL47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -10065,9 +10209,12 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK48" t="n">
         <v>26</v>
       </c>
-      <c r="BK48" t="n">
+      <c r="BL48" t="n">
         <v>26</v>
       </c>
     </row>
@@ -10262,9 +10409,12 @@
         <v>0</v>
       </c>
       <c r="BJ49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK49" t="n">
         <v>19</v>
       </c>
-      <c r="BK49" t="n">
+      <c r="BL49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -10459,9 +10609,12 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK50" t="n">
         <v>7</v>
       </c>
-      <c r="BK50" t="n">
+      <c r="BL50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10656,9 +10809,12 @@
         <v>0</v>
       </c>
       <c r="BJ51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK51" t="n">
         <v>32</v>
       </c>
-      <c r="BK51" t="n">
+      <c r="BL51" t="n">
         <v>32</v>
       </c>
     </row>
@@ -10858,6 +11014,9 @@
       <c r="BK52" t="n">
         <v>0</v>
       </c>
+      <c r="BL52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11050,9 +11209,12 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK53" t="n">
         <v>13</v>
       </c>
-      <c r="BK53" t="n">
+      <c r="BL53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -11252,6 +11414,9 @@
       <c r="BK54" t="n">
         <v>0</v>
       </c>
+      <c r="BL54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11444,10 +11609,13 @@
         <v>1</v>
       </c>
       <c r="BJ55" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="BK55" t="n">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="BL55" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="56">
@@ -11641,9 +11809,12 @@
         <v>1</v>
       </c>
       <c r="BJ56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK56" t="n">
         <v>31</v>
       </c>
-      <c r="BK56" t="n">
+      <c r="BL56" t="n">
         <v>31</v>
       </c>
     </row>
@@ -11838,9 +12009,12 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK57" t="n">
         <v>10</v>
       </c>
-      <c r="BK57" t="n">
+      <c r="BL57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -12035,9 +12209,12 @@
         <v>0</v>
       </c>
       <c r="BJ58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK58" t="n">
         <v>13</v>
       </c>
-      <c r="BK58" t="n">
+      <c r="BL58" t="n">
         <v>13</v>
       </c>
     </row>
@@ -12232,9 +12409,12 @@
         <v>0</v>
       </c>
       <c r="BJ59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK59" t="n">
         <v>6</v>
       </c>
-      <c r="BK59" t="n">
+      <c r="BL59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -12434,6 +12614,9 @@
       <c r="BK60" t="n">
         <v>0</v>
       </c>
+      <c r="BL60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12626,9 +12809,12 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK61" t="n">
         <v>29</v>
       </c>
-      <c r="BK61" t="n">
+      <c r="BL61" t="n">
         <v>29</v>
       </c>
     </row>
@@ -12823,9 +13009,12 @@
         <v>1</v>
       </c>
       <c r="BJ62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK62" t="n">
         <v>29</v>
       </c>
-      <c r="BK62" t="n">
+      <c r="BL62" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13020,9 +13209,12 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK63" t="n">
         <v>12</v>
       </c>
-      <c r="BK63" t="n">
+      <c r="BL63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -13222,6 +13414,9 @@
       <c r="BK64" t="n">
         <v>0</v>
       </c>
+      <c r="BL64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -13414,9 +13609,12 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK65" t="n">
         <v>17</v>
       </c>
-      <c r="BK65" t="n">
+      <c r="BL65" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13611,9 +13809,12 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK66" t="n">
         <v>8</v>
       </c>
-      <c r="BK66" t="n">
+      <c r="BL66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -13808,10 +14009,13 @@
         <v>1</v>
       </c>
       <c r="BJ67" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="BK67" t="n">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="BL67" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="68">
@@ -14005,9 +14209,12 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK68" t="n">
         <v>22</v>
       </c>
-      <c r="BK68" t="n">
+      <c r="BL68" t="n">
         <v>21</v>
       </c>
     </row>
@@ -14202,9 +14409,12 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK69" t="n">
         <v>7</v>
       </c>
-      <c r="BK69" t="n">
+      <c r="BL69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14399,9 +14609,12 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK70" t="n">
         <v>23</v>
       </c>
-      <c r="BK70" t="n">
+      <c r="BL70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -14596,9 +14809,12 @@
         <v>0</v>
       </c>
       <c r="BJ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK71" t="n">
         <v>24</v>
       </c>
-      <c r="BK71" t="n">
+      <c r="BL71" t="n">
         <v>24</v>
       </c>
     </row>
@@ -14793,9 +15009,12 @@
         <v>0</v>
       </c>
       <c r="BJ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK72" t="n">
         <v>24</v>
       </c>
-      <c r="BK72" t="n">
+      <c r="BL72" t="n">
         <v>24</v>
       </c>
     </row>
@@ -14995,6 +15214,9 @@
       <c r="BK73" t="n">
         <v>0</v>
       </c>
+      <c r="BL73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -15192,6 +15414,9 @@
       <c r="BK74" t="n">
         <v>0</v>
       </c>
+      <c r="BL74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -15384,10 +15609,13 @@
         <v>0</v>
       </c>
       <c r="BJ75" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="BK75" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="BL75" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="76">
@@ -15581,9 +15809,12 @@
         <v>0</v>
       </c>
       <c r="BJ76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK76" t="n">
         <v>21</v>
       </c>
-      <c r="BK76" t="n">
+      <c r="BL76" t="n">
         <v>21</v>
       </c>
     </row>
@@ -15778,9 +16009,12 @@
         <v>0</v>
       </c>
       <c r="BJ77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK77" t="n">
         <v>15</v>
       </c>
-      <c r="BK77" t="n">
+      <c r="BL77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -15975,10 +16209,13 @@
         <v>1</v>
       </c>
       <c r="BJ78" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK78" t="n">
+        <v>35</v>
+      </c>
+      <c r="BL78" t="n">
         <v>34</v>
-      </c>
-      <c r="BK78" t="n">
-        <v>33</v>
       </c>
     </row>
     <row r="79">
@@ -16172,9 +16409,12 @@
         <v>0</v>
       </c>
       <c r="BJ79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK79" t="n">
         <v>22</v>
       </c>
-      <c r="BK79" t="n">
+      <c r="BL79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -16369,9 +16609,12 @@
         <v>0</v>
       </c>
       <c r="BJ80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK80" t="n">
         <v>11</v>
       </c>
-      <c r="BK80" t="n">
+      <c r="BL80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -16566,9 +16809,12 @@
         <v>0</v>
       </c>
       <c r="BJ81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK81" t="n">
         <v>4</v>
       </c>
-      <c r="BK81" t="n">
+      <c r="BL81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -16763,9 +17009,12 @@
         <v>1</v>
       </c>
       <c r="BJ82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK82" t="n">
         <v>18</v>
       </c>
-      <c r="BK82" t="n">
+      <c r="BL82" t="n">
         <v>18</v>
       </c>
     </row>
@@ -16960,9 +17209,12 @@
         <v>0</v>
       </c>
       <c r="BJ83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK83" t="n">
         <v>17</v>
       </c>
-      <c r="BK83" t="n">
+      <c r="BL83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -17157,9 +17409,12 @@
         <v>0</v>
       </c>
       <c r="BJ84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK84" t="n">
         <v>13</v>
       </c>
-      <c r="BK84" t="n">
+      <c r="BL84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -17354,9 +17609,12 @@
         <v>0</v>
       </c>
       <c r="BJ85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK85" t="n">
         <v>7</v>
       </c>
-      <c r="BK85" t="n">
+      <c r="BL85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17556,6 +17814,9 @@
       <c r="BK86" t="n">
         <v>0</v>
       </c>
+      <c r="BL86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -17748,10 +18009,13 @@
         <v>0</v>
       </c>
       <c r="BJ87" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="BK87" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="BL87" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="88">
@@ -17950,6 +18214,9 @@
       <c r="BK88" t="n">
         <v>0</v>
       </c>
+      <c r="BL88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -18142,9 +18409,12 @@
         <v>0</v>
       </c>
       <c r="BJ89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK89" t="n">
         <v>18</v>
       </c>
-      <c r="BK89" t="n">
+      <c r="BL89" t="n">
         <v>18</v>
       </c>
     </row>
@@ -18339,9 +18609,12 @@
         <v>0</v>
       </c>
       <c r="BJ90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK90" t="n">
         <v>17</v>
       </c>
-      <c r="BK90" t="n">
+      <c r="BL90" t="n">
         <v>17</v>
       </c>
     </row>
@@ -18536,9 +18809,12 @@
         <v>0</v>
       </c>
       <c r="BJ91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK91" t="n">
         <v>42</v>
       </c>
-      <c r="BK91" t="n">
+      <c r="BL91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -18733,9 +19009,12 @@
         <v>0</v>
       </c>
       <c r="BJ92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK92" t="n">
         <v>7</v>
       </c>
-      <c r="BK92" t="n">
+      <c r="BL92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18935,6 +19214,9 @@
       <c r="BK93" t="n">
         <v>0</v>
       </c>
+      <c r="BL93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -19127,9 +19409,12 @@
         <v>0</v>
       </c>
       <c r="BJ94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK94" t="n">
         <v>16</v>
       </c>
-      <c r="BK94" t="n">
+      <c r="BL94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -19324,9 +19609,12 @@
         <v>0</v>
       </c>
       <c r="BJ95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK95" t="n">
         <v>7</v>
       </c>
-      <c r="BK95" t="n">
+      <c r="BL95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -19521,9 +19809,12 @@
         <v>0</v>
       </c>
       <c r="BJ96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK96" t="n">
         <v>24</v>
       </c>
-      <c r="BK96" t="n">
+      <c r="BL96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -19723,6 +20014,9 @@
       <c r="BK97" t="n">
         <v>0</v>
       </c>
+      <c r="BL97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -19915,10 +20209,13 @@
         <v>1</v>
       </c>
       <c r="BJ98" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="BK98" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="BL98" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="99">
@@ -20112,9 +20409,12 @@
         <v>0</v>
       </c>
       <c r="BJ99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK99" t="n">
         <v>14</v>
       </c>
-      <c r="BK99" t="n">
+      <c r="BL99" t="n">
         <v>14</v>
       </c>
     </row>
@@ -20314,6 +20614,9 @@
       <c r="BK100" t="n">
         <v>0</v>
       </c>
+      <c r="BL100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -20506,10 +20809,13 @@
         <v>0</v>
       </c>
       <c r="BJ101" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BK101" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BL101" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="102">
@@ -20703,10 +21009,13 @@
         <v>1</v>
       </c>
       <c r="BJ102" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="BK102" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="BL102" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="103">
@@ -20900,10 +21209,13 @@
         <v>1</v>
       </c>
       <c r="BJ103" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="BK103" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="BL103" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="104">
@@ -21097,9 +21409,12 @@
         <v>0</v>
       </c>
       <c r="BJ104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK104" t="n">
         <v>12</v>
       </c>
-      <c r="BK104" t="n">
+      <c r="BL104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -21294,10 +21609,13 @@
         <v>1</v>
       </c>
       <c r="BJ105" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BK105" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BL105" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="106">
@@ -21491,9 +21809,12 @@
         <v>0</v>
       </c>
       <c r="BJ106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK106" t="n">
         <v>7</v>
       </c>
-      <c r="BK106" t="n">
+      <c r="BL106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -21688,9 +22009,12 @@
         <v>0</v>
       </c>
       <c r="BJ107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK107" t="n">
         <v>13</v>
       </c>
-      <c r="BK107" t="n">
+      <c r="BL107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -21885,9 +22209,12 @@
         <v>0</v>
       </c>
       <c r="BJ108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK108" t="n">
         <v>2</v>
       </c>
-      <c r="BK108" t="n">
+      <c r="BL108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -22082,9 +22409,12 @@
         <v>0</v>
       </c>
       <c r="BJ109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK109" t="n">
         <v>4</v>
       </c>
-      <c r="BK109" t="n">
+      <c r="BL109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#4396)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL109"/>
+  <dimension ref="A1:BM109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -492,8 +492,9 @@
     <col width="12" customWidth="1" min="60" max="60"/>
     <col width="12" customWidth="1" min="61" max="61"/>
     <col width="12" customWidth="1" min="62" max="62"/>
-    <col width="13" customWidth="1" min="63" max="63"/>
+    <col width="12" customWidth="1" min="63" max="63"/>
     <col width="13" customWidth="1" min="64" max="64"/>
+    <col width="13" customWidth="1" min="65" max="65"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -807,12 +808,17 @@
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="BK1" s="2" t="inlineStr">
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="BL1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BL1" s="2" t="inlineStr">
+      <c r="BM1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -1012,9 +1018,12 @@
         <v>0</v>
       </c>
       <c r="BK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL2" t="n">
         <v>12</v>
       </c>
-      <c r="BL2" t="n">
+      <c r="BM2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1212,9 +1221,12 @@
         <v>0</v>
       </c>
       <c r="BK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL3" t="n">
         <v>10</v>
       </c>
-      <c r="BL3" t="n">
+      <c r="BM3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1412,10 +1424,13 @@
         <v>1</v>
       </c>
       <c r="BK4" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="BL4" t="n">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="BM4" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -1612,9 +1627,12 @@
         <v>0</v>
       </c>
       <c r="BK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL5" t="n">
         <v>15</v>
       </c>
-      <c r="BL5" t="n">
+      <c r="BM5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1812,9 +1830,12 @@
         <v>0</v>
       </c>
       <c r="BK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL6" t="n">
         <v>19</v>
       </c>
-      <c r="BL6" t="n">
+      <c r="BM6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2012,9 +2033,12 @@
         <v>0</v>
       </c>
       <c r="BK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL7" t="n">
         <v>19</v>
       </c>
-      <c r="BL7" t="n">
+      <c r="BM7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2212,10 +2236,13 @@
         <v>0</v>
       </c>
       <c r="BK8" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BL8" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="9">
@@ -2412,10 +2439,13 @@
         <v>1</v>
       </c>
       <c r="BK9" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BL9" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="10">
@@ -2612,10 +2642,13 @@
         <v>1</v>
       </c>
       <c r="BK10" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="BL10" t="n">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="11">
@@ -2812,9 +2845,12 @@
         <v>0</v>
       </c>
       <c r="BK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL11" t="n">
         <v>29</v>
       </c>
-      <c r="BL11" t="n">
+      <c r="BM11" t="n">
         <v>29</v>
       </c>
     </row>
@@ -3012,10 +3048,13 @@
         <v>1</v>
       </c>
       <c r="BK12" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="BL12" t="n">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="BM12" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="13">
@@ -3212,9 +3251,12 @@
         <v>0</v>
       </c>
       <c r="BK13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL13" t="n">
         <v>14</v>
       </c>
-      <c r="BL13" t="n">
+      <c r="BM13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3412,9 +3454,12 @@
         <v>1</v>
       </c>
       <c r="BK14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL14" t="n">
         <v>26</v>
       </c>
-      <c r="BL14" t="n">
+      <c r="BM14" t="n">
         <v>26</v>
       </c>
     </row>
@@ -3612,9 +3657,12 @@
         <v>0</v>
       </c>
       <c r="BK15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL15" t="n">
         <v>9</v>
       </c>
-      <c r="BL15" t="n">
+      <c r="BM15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3812,9 +3860,12 @@
         <v>0</v>
       </c>
       <c r="BK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL16" t="n">
         <v>20</v>
       </c>
-      <c r="BL16" t="n">
+      <c r="BM16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4012,9 +4063,12 @@
         <v>0</v>
       </c>
       <c r="BK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL17" t="n">
         <v>17</v>
       </c>
-      <c r="BL17" t="n">
+      <c r="BM17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4212,10 +4266,13 @@
         <v>1</v>
       </c>
       <c r="BK18" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="BL18" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="BM18" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="19">
@@ -4417,6 +4474,9 @@
       <c r="BL19" t="n">
         <v>0</v>
       </c>
+      <c r="BM19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4612,9 +4672,12 @@
         <v>0</v>
       </c>
       <c r="BK20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL20" t="n">
         <v>20</v>
       </c>
-      <c r="BL20" t="n">
+      <c r="BM20" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4812,9 +4875,12 @@
         <v>0</v>
       </c>
       <c r="BK21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL21" t="n">
         <v>27</v>
       </c>
-      <c r="BL21" t="n">
+      <c r="BM21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5017,6 +5083,9 @@
       <c r="BL22" t="n">
         <v>0</v>
       </c>
+      <c r="BM22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5212,9 +5281,12 @@
         <v>1</v>
       </c>
       <c r="BK23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL23" t="n">
         <v>22</v>
       </c>
-      <c r="BL23" t="n">
+      <c r="BM23" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5412,9 +5484,12 @@
         <v>0</v>
       </c>
       <c r="BK24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL24" t="n">
         <v>27</v>
       </c>
-      <c r="BL24" t="n">
+      <c r="BM24" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5612,9 +5687,12 @@
         <v>0</v>
       </c>
       <c r="BK25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL25" t="n">
         <v>11</v>
       </c>
-      <c r="BL25" t="n">
+      <c r="BM25" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5812,10 +5890,13 @@
         <v>1</v>
       </c>
       <c r="BK26" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="BL26" t="n">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="BM26" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="27">
@@ -6012,9 +6093,12 @@
         <v>0</v>
       </c>
       <c r="BK27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL27" t="n">
         <v>25</v>
       </c>
-      <c r="BL27" t="n">
+      <c r="BM27" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6212,9 +6296,12 @@
         <v>0</v>
       </c>
       <c r="BK28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL28" t="n">
         <v>19</v>
       </c>
-      <c r="BL28" t="n">
+      <c r="BM28" t="n">
         <v>19</v>
       </c>
     </row>
@@ -6412,9 +6499,12 @@
         <v>0</v>
       </c>
       <c r="BK29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL29" t="n">
         <v>11</v>
       </c>
-      <c r="BL29" t="n">
+      <c r="BM29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6612,9 +6702,12 @@
         <v>0</v>
       </c>
       <c r="BK30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL30" t="n">
         <v>25</v>
       </c>
-      <c r="BL30" t="n">
+      <c r="BM30" t="n">
         <v>25</v>
       </c>
     </row>
@@ -6812,9 +6905,12 @@
         <v>0</v>
       </c>
       <c r="BK31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL31" t="n">
         <v>20</v>
       </c>
-      <c r="BL31" t="n">
+      <c r="BM31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -7012,10 +7108,13 @@
         <v>0</v>
       </c>
       <c r="BK32" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="BL32" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="BM32" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="33">
@@ -7212,9 +7311,12 @@
         <v>1</v>
       </c>
       <c r="BK33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL33" t="n">
         <v>21</v>
       </c>
-      <c r="BL33" t="n">
+      <c r="BM33" t="n">
         <v>21</v>
       </c>
     </row>
@@ -7412,9 +7514,12 @@
         <v>0</v>
       </c>
       <c r="BK34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL34" t="n">
         <v>9</v>
       </c>
-      <c r="BL34" t="n">
+      <c r="BM34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7612,9 +7717,12 @@
         <v>0</v>
       </c>
       <c r="BK35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL35" t="n">
         <v>25</v>
       </c>
-      <c r="BL35" t="n">
+      <c r="BM35" t="n">
         <v>25</v>
       </c>
     </row>
@@ -7812,9 +7920,12 @@
         <v>1</v>
       </c>
       <c r="BK36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL36" t="n">
         <v>16</v>
       </c>
-      <c r="BL36" t="n">
+      <c r="BM36" t="n">
         <v>16</v>
       </c>
     </row>
@@ -8017,6 +8128,9 @@
       <c r="BL37" t="n">
         <v>0</v>
       </c>
+      <c r="BM37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8212,9 +8326,12 @@
         <v>0</v>
       </c>
       <c r="BK38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL38" t="n">
         <v>2</v>
       </c>
-      <c r="BL38" t="n">
+      <c r="BM38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8412,10 +8529,13 @@
         <v>0</v>
       </c>
       <c r="BK39" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="BL39" t="n">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="BM39" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="40">
@@ -8612,9 +8732,12 @@
         <v>1</v>
       </c>
       <c r="BK40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL40" t="n">
         <v>28</v>
       </c>
-      <c r="BL40" t="n">
+      <c r="BM40" t="n">
         <v>28</v>
       </c>
     </row>
@@ -8812,10 +8935,13 @@
         <v>1</v>
       </c>
       <c r="BK41" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="BL41" t="n">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="BM41" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="42">
@@ -9012,9 +9138,12 @@
         <v>0</v>
       </c>
       <c r="BK42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL42" t="n">
         <v>21</v>
       </c>
-      <c r="BL42" t="n">
+      <c r="BM42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9212,9 +9341,12 @@
         <v>0</v>
       </c>
       <c r="BK43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL43" t="n">
         <v>60</v>
       </c>
-      <c r="BL43" t="n">
+      <c r="BM43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9412,9 +9544,12 @@
         <v>0</v>
       </c>
       <c r="BK44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL44" t="n">
         <v>25</v>
       </c>
-      <c r="BL44" t="n">
+      <c r="BM44" t="n">
         <v>25</v>
       </c>
     </row>
@@ -9612,9 +9747,12 @@
         <v>0</v>
       </c>
       <c r="BK45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL45" t="n">
         <v>26</v>
       </c>
-      <c r="BL45" t="n">
+      <c r="BM45" t="n">
         <v>26</v>
       </c>
     </row>
@@ -9812,9 +9950,12 @@
         <v>0</v>
       </c>
       <c r="BK46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL46" t="n">
         <v>30</v>
       </c>
-      <c r="BL46" t="n">
+      <c r="BM46" t="n">
         <v>30</v>
       </c>
     </row>
@@ -10017,6 +10158,9 @@
       <c r="BL47" t="n">
         <v>0</v>
       </c>
+      <c r="BM47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -10212,9 +10356,12 @@
         <v>0</v>
       </c>
       <c r="BK48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL48" t="n">
         <v>26</v>
       </c>
-      <c r="BL48" t="n">
+      <c r="BM48" t="n">
         <v>26</v>
       </c>
     </row>
@@ -10412,9 +10559,12 @@
         <v>0</v>
       </c>
       <c r="BK49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL49" t="n">
         <v>19</v>
       </c>
-      <c r="BL49" t="n">
+      <c r="BM49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -10612,9 +10762,12 @@
         <v>0</v>
       </c>
       <c r="BK50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL50" t="n">
         <v>7</v>
       </c>
-      <c r="BL50" t="n">
+      <c r="BM50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10812,9 +10965,12 @@
         <v>0</v>
       </c>
       <c r="BK51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL51" t="n">
         <v>32</v>
       </c>
-      <c r="BL51" t="n">
+      <c r="BM51" t="n">
         <v>32</v>
       </c>
     </row>
@@ -11017,6 +11173,9 @@
       <c r="BL52" t="n">
         <v>0</v>
       </c>
+      <c r="BM52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11212,9 +11371,12 @@
         <v>0</v>
       </c>
       <c r="BK53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL53" t="n">
         <v>13</v>
       </c>
-      <c r="BL53" t="n">
+      <c r="BM53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -11417,6 +11579,9 @@
       <c r="BL54" t="n">
         <v>0</v>
       </c>
+      <c r="BM54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11612,10 +11777,13 @@
         <v>1</v>
       </c>
       <c r="BK55" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="BL55" t="n">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="BM55" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="56">
@@ -11812,9 +11980,12 @@
         <v>0</v>
       </c>
       <c r="BK56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL56" t="n">
         <v>31</v>
       </c>
-      <c r="BL56" t="n">
+      <c r="BM56" t="n">
         <v>31</v>
       </c>
     </row>
@@ -12012,9 +12183,12 @@
         <v>0</v>
       </c>
       <c r="BK57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL57" t="n">
         <v>10</v>
       </c>
-      <c r="BL57" t="n">
+      <c r="BM57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -12212,9 +12386,12 @@
         <v>0</v>
       </c>
       <c r="BK58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL58" t="n">
         <v>13</v>
       </c>
-      <c r="BL58" t="n">
+      <c r="BM58" t="n">
         <v>13</v>
       </c>
     </row>
@@ -12412,9 +12589,12 @@
         <v>0</v>
       </c>
       <c r="BK59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL59" t="n">
         <v>6</v>
       </c>
-      <c r="BL59" t="n">
+      <c r="BM59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -12617,6 +12797,9 @@
       <c r="BL60" t="n">
         <v>0</v>
       </c>
+      <c r="BM60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12812,9 +12995,12 @@
         <v>0</v>
       </c>
       <c r="BK61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL61" t="n">
         <v>29</v>
       </c>
-      <c r="BL61" t="n">
+      <c r="BM61" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13012,9 +13198,12 @@
         <v>0</v>
       </c>
       <c r="BK62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL62" t="n">
         <v>29</v>
       </c>
-      <c r="BL62" t="n">
+      <c r="BM62" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13212,9 +13401,12 @@
         <v>0</v>
       </c>
       <c r="BK63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL63" t="n">
         <v>12</v>
       </c>
-      <c r="BL63" t="n">
+      <c r="BM63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -13417,6 +13609,9 @@
       <c r="BL64" t="n">
         <v>0</v>
       </c>
+      <c r="BM64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -13612,9 +13807,12 @@
         <v>0</v>
       </c>
       <c r="BK65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL65" t="n">
         <v>17</v>
       </c>
-      <c r="BL65" t="n">
+      <c r="BM65" t="n">
         <v>17</v>
       </c>
     </row>
@@ -13812,9 +14010,12 @@
         <v>0</v>
       </c>
       <c r="BK66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL66" t="n">
         <v>8</v>
       </c>
-      <c r="BL66" t="n">
+      <c r="BM66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -14012,10 +14213,13 @@
         <v>1</v>
       </c>
       <c r="BK67" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="BL67" t="n">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="BM67" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="68">
@@ -14212,10 +14416,13 @@
         <v>0</v>
       </c>
       <c r="BK68" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL68" t="n">
+        <v>23</v>
+      </c>
+      <c r="BM68" t="n">
         <v>22</v>
-      </c>
-      <c r="BL68" t="n">
-        <v>21</v>
       </c>
     </row>
     <row r="69">
@@ -14412,9 +14619,12 @@
         <v>0</v>
       </c>
       <c r="BK69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL69" t="n">
         <v>7</v>
       </c>
-      <c r="BL69" t="n">
+      <c r="BM69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14612,9 +14822,12 @@
         <v>0</v>
       </c>
       <c r="BK70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL70" t="n">
         <v>23</v>
       </c>
-      <c r="BL70" t="n">
+      <c r="BM70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -14812,9 +15025,12 @@
         <v>0</v>
       </c>
       <c r="BK71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL71" t="n">
         <v>24</v>
       </c>
-      <c r="BL71" t="n">
+      <c r="BM71" t="n">
         <v>24</v>
       </c>
     </row>
@@ -15012,9 +15228,12 @@
         <v>0</v>
       </c>
       <c r="BK72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL72" t="n">
         <v>24</v>
       </c>
-      <c r="BL72" t="n">
+      <c r="BM72" t="n">
         <v>24</v>
       </c>
     </row>
@@ -15217,6 +15436,9 @@
       <c r="BL73" t="n">
         <v>0</v>
       </c>
+      <c r="BM73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -15417,6 +15639,9 @@
       <c r="BL74" t="n">
         <v>0</v>
       </c>
+      <c r="BM74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -15612,10 +15837,13 @@
         <v>1</v>
       </c>
       <c r="BK75" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="BL75" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="BM75" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="76">
@@ -15812,9 +16040,12 @@
         <v>0</v>
       </c>
       <c r="BK76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL76" t="n">
         <v>21</v>
       </c>
-      <c r="BL76" t="n">
+      <c r="BM76" t="n">
         <v>21</v>
       </c>
     </row>
@@ -16012,9 +16243,12 @@
         <v>0</v>
       </c>
       <c r="BK77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL77" t="n">
         <v>15</v>
       </c>
-      <c r="BL77" t="n">
+      <c r="BM77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -16212,10 +16446,13 @@
         <v>1</v>
       </c>
       <c r="BK78" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL78" t="n">
+        <v>36</v>
+      </c>
+      <c r="BM78" t="n">
         <v>35</v>
-      </c>
-      <c r="BL78" t="n">
-        <v>34</v>
       </c>
     </row>
     <row r="79">
@@ -16412,9 +16649,12 @@
         <v>0</v>
       </c>
       <c r="BK79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL79" t="n">
         <v>22</v>
       </c>
-      <c r="BL79" t="n">
+      <c r="BM79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -16612,9 +16852,12 @@
         <v>0</v>
       </c>
       <c r="BK80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL80" t="n">
         <v>11</v>
       </c>
-      <c r="BL80" t="n">
+      <c r="BM80" t="n">
         <v>11</v>
       </c>
     </row>
@@ -16812,9 +17055,12 @@
         <v>0</v>
       </c>
       <c r="BK81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL81" t="n">
         <v>4</v>
       </c>
-      <c r="BL81" t="n">
+      <c r="BM81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -17012,9 +17258,12 @@
         <v>0</v>
       </c>
       <c r="BK82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL82" t="n">
         <v>18</v>
       </c>
-      <c r="BL82" t="n">
+      <c r="BM82" t="n">
         <v>18</v>
       </c>
     </row>
@@ -17212,9 +17461,12 @@
         <v>0</v>
       </c>
       <c r="BK83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL83" t="n">
         <v>17</v>
       </c>
-      <c r="BL83" t="n">
+      <c r="BM83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -17412,9 +17664,12 @@
         <v>0</v>
       </c>
       <c r="BK84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL84" t="n">
         <v>13</v>
       </c>
-      <c r="BL84" t="n">
+      <c r="BM84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -17612,9 +17867,12 @@
         <v>0</v>
       </c>
       <c r="BK85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL85" t="n">
         <v>7</v>
       </c>
-      <c r="BL85" t="n">
+      <c r="BM85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -17817,6 +18075,9 @@
       <c r="BL86" t="n">
         <v>0</v>
       </c>
+      <c r="BM86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -18012,9 +18273,12 @@
         <v>1</v>
       </c>
       <c r="BK87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL87" t="n">
         <v>19</v>
       </c>
-      <c r="BL87" t="n">
+      <c r="BM87" t="n">
         <v>19</v>
       </c>
     </row>
@@ -18217,6 +18481,9 @@
       <c r="BL88" t="n">
         <v>0</v>
       </c>
+      <c r="BM88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -18412,9 +18679,12 @@
         <v>0</v>
       </c>
       <c r="BK89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL89" t="n">
         <v>18</v>
       </c>
-      <c r="BL89" t="n">
+      <c r="BM89" t="n">
         <v>18</v>
       </c>
     </row>
@@ -18612,9 +18882,12 @@
         <v>0</v>
       </c>
       <c r="BK90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL90" t="n">
         <v>17</v>
       </c>
-      <c r="BL90" t="n">
+      <c r="BM90" t="n">
         <v>17</v>
       </c>
     </row>
@@ -18812,9 +19085,12 @@
         <v>0</v>
       </c>
       <c r="BK91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL91" t="n">
         <v>42</v>
       </c>
-      <c r="BL91" t="n">
+      <c r="BM91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -19012,9 +19288,12 @@
         <v>0</v>
       </c>
       <c r="BK92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL92" t="n">
         <v>7</v>
       </c>
-      <c r="BL92" t="n">
+      <c r="BM92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -19217,6 +19496,9 @@
       <c r="BL93" t="n">
         <v>0</v>
       </c>
+      <c r="BM93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -19412,9 +19694,12 @@
         <v>0</v>
       </c>
       <c r="BK94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL94" t="n">
         <v>16</v>
       </c>
-      <c r="BL94" t="n">
+      <c r="BM94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -19612,9 +19897,12 @@
         <v>0</v>
       </c>
       <c r="BK95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL95" t="n">
         <v>7</v>
       </c>
-      <c r="BL95" t="n">
+      <c r="BM95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -19812,9 +20100,12 @@
         <v>0</v>
       </c>
       <c r="BK96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL96" t="n">
         <v>24</v>
       </c>
-      <c r="BL96" t="n">
+      <c r="BM96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -20017,6 +20308,9 @@
       <c r="BL97" t="n">
         <v>0</v>
       </c>
+      <c r="BM97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -20212,10 +20506,13 @@
         <v>1</v>
       </c>
       <c r="BK98" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="BL98" t="n">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="BM98" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="99">
@@ -20412,9 +20709,12 @@
         <v>0</v>
       </c>
       <c r="BK99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL99" t="n">
         <v>14</v>
       </c>
-      <c r="BL99" t="n">
+      <c r="BM99" t="n">
         <v>14</v>
       </c>
     </row>
@@ -20617,6 +20917,9 @@
       <c r="BL100" t="n">
         <v>0</v>
       </c>
+      <c r="BM100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -20812,9 +21115,12 @@
         <v>1</v>
       </c>
       <c r="BK101" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL101" t="n">
         <v>31</v>
       </c>
-      <c r="BL101" t="n">
+      <c r="BM101" t="n">
         <v>31</v>
       </c>
     </row>
@@ -21012,9 +21318,12 @@
         <v>1</v>
       </c>
       <c r="BK102" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL102" t="n">
         <v>30</v>
       </c>
-      <c r="BL102" t="n">
+      <c r="BM102" t="n">
         <v>30</v>
       </c>
     </row>
@@ -21212,10 +21521,13 @@
         <v>1</v>
       </c>
       <c r="BK103" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="BL103" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="BM103" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="104">
@@ -21412,9 +21724,12 @@
         <v>0</v>
       </c>
       <c r="BK104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL104" t="n">
         <v>12</v>
       </c>
-      <c r="BL104" t="n">
+      <c r="BM104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -21612,10 +21927,13 @@
         <v>1</v>
       </c>
       <c r="BK105" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="BL105" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="BM105" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="106">
@@ -21812,9 +22130,12 @@
         <v>0</v>
       </c>
       <c r="BK106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL106" t="n">
         <v>7</v>
       </c>
-      <c r="BL106" t="n">
+      <c r="BM106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -22012,9 +22333,12 @@
         <v>0</v>
       </c>
       <c r="BK107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL107" t="n">
         <v>13</v>
       </c>
-      <c r="BL107" t="n">
+      <c r="BM107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -22212,9 +22536,12 @@
         <v>0</v>
       </c>
       <c r="BK108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL108" t="n">
         <v>2</v>
       </c>
-      <c r="BL108" t="n">
+      <c r="BM108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -22412,9 +22739,12 @@
         <v>0</v>
       </c>
       <c r="BK109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL109" t="n">
         <v>4</v>
       </c>
-      <c r="BL109" t="n">
+      <c r="BM109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#4410)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM109"/>
+  <dimension ref="A1:BN109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -493,8 +493,9 @@
     <col width="12" customWidth="1" min="61" max="61"/>
     <col width="12" customWidth="1" min="62" max="62"/>
     <col width="12" customWidth="1" min="63" max="63"/>
-    <col width="13" customWidth="1" min="64" max="64"/>
+    <col width="12" customWidth="1" min="64" max="64"/>
     <col width="13" customWidth="1" min="65" max="65"/>
+    <col width="13" customWidth="1" min="66" max="66"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -813,12 +814,17 @@
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="BL1" s="2" t="inlineStr">
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="BM1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BM1" s="2" t="inlineStr">
+      <c r="BN1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -1021,9 +1027,12 @@
         <v>0</v>
       </c>
       <c r="BL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="n">
         <v>12</v>
       </c>
-      <c r="BM2" t="n">
+      <c r="BN2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1224,9 +1233,12 @@
         <v>0</v>
       </c>
       <c r="BL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM3" t="n">
         <v>10</v>
       </c>
-      <c r="BM3" t="n">
+      <c r="BN3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1427,10 +1439,13 @@
         <v>1</v>
       </c>
       <c r="BL4" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="BM4" t="n">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="BN4" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -1630,9 +1645,12 @@
         <v>0</v>
       </c>
       <c r="BL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM5" t="n">
         <v>15</v>
       </c>
-      <c r="BM5" t="n">
+      <c r="BN5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1833,9 +1851,12 @@
         <v>0</v>
       </c>
       <c r="BL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM6" t="n">
         <v>19</v>
       </c>
-      <c r="BM6" t="n">
+      <c r="BN6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2036,9 +2057,12 @@
         <v>0</v>
       </c>
       <c r="BL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM7" t="n">
         <v>19</v>
       </c>
-      <c r="BM7" t="n">
+      <c r="BN7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2239,9 +2263,12 @@
         <v>1</v>
       </c>
       <c r="BL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM8" t="n">
         <v>32</v>
       </c>
-      <c r="BM8" t="n">
+      <c r="BN8" t="n">
         <v>32</v>
       </c>
     </row>
@@ -2442,9 +2469,12 @@
         <v>1</v>
       </c>
       <c r="BL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM9" t="n">
         <v>31</v>
       </c>
-      <c r="BM9" t="n">
+      <c r="BN9" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2645,10 +2675,13 @@
         <v>1</v>
       </c>
       <c r="BL10" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="BM10" t="n">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="11">
@@ -2848,9 +2881,12 @@
         <v>0</v>
       </c>
       <c r="BL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM11" t="n">
         <v>29</v>
       </c>
-      <c r="BM11" t="n">
+      <c r="BN11" t="n">
         <v>29</v>
       </c>
     </row>
@@ -3051,9 +3087,12 @@
         <v>1</v>
       </c>
       <c r="BL12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM12" t="n">
         <v>37</v>
       </c>
-      <c r="BM12" t="n">
+      <c r="BN12" t="n">
         <v>37</v>
       </c>
     </row>
@@ -3254,9 +3293,12 @@
         <v>0</v>
       </c>
       <c r="BL13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM13" t="n">
         <v>14</v>
       </c>
-      <c r="BM13" t="n">
+      <c r="BN13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3457,9 +3499,12 @@
         <v>0</v>
       </c>
       <c r="BL14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM14" t="n">
         <v>26</v>
       </c>
-      <c r="BM14" t="n">
+      <c r="BN14" t="n">
         <v>26</v>
       </c>
     </row>
@@ -3660,9 +3705,12 @@
         <v>0</v>
       </c>
       <c r="BL15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM15" t="n">
         <v>9</v>
       </c>
-      <c r="BM15" t="n">
+      <c r="BN15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3863,9 +3911,12 @@
         <v>0</v>
       </c>
       <c r="BL16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM16" t="n">
         <v>20</v>
       </c>
-      <c r="BM16" t="n">
+      <c r="BN16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4066,9 +4117,12 @@
         <v>0</v>
       </c>
       <c r="BL17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM17" t="n">
         <v>17</v>
       </c>
-      <c r="BM17" t="n">
+      <c r="BN17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4269,9 +4323,12 @@
         <v>1</v>
       </c>
       <c r="BL18" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM18" t="n">
         <v>33</v>
       </c>
-      <c r="BM18" t="n">
+      <c r="BN18" t="n">
         <v>33</v>
       </c>
     </row>
@@ -4477,6 +4534,9 @@
       <c r="BM19" t="n">
         <v>0</v>
       </c>
+      <c r="BN19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4675,9 +4735,12 @@
         <v>0</v>
       </c>
       <c r="BL20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM20" t="n">
         <v>20</v>
       </c>
-      <c r="BM20" t="n">
+      <c r="BN20" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4878,9 +4941,12 @@
         <v>0</v>
       </c>
       <c r="BL21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM21" t="n">
         <v>27</v>
       </c>
-      <c r="BM21" t="n">
+      <c r="BN21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5086,6 +5152,9 @@
       <c r="BM22" t="n">
         <v>0</v>
       </c>
+      <c r="BN22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5284,9 +5353,12 @@
         <v>0</v>
       </c>
       <c r="BL23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM23" t="n">
         <v>22</v>
       </c>
-      <c r="BM23" t="n">
+      <c r="BN23" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5487,9 +5559,12 @@
         <v>0</v>
       </c>
       <c r="BL24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM24" t="n">
         <v>27</v>
       </c>
-      <c r="BM24" t="n">
+      <c r="BN24" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5690,9 +5765,12 @@
         <v>0</v>
       </c>
       <c r="BL25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM25" t="n">
         <v>11</v>
       </c>
-      <c r="BM25" t="n">
+      <c r="BN25" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5893,9 +5971,12 @@
         <v>1</v>
       </c>
       <c r="BL26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM26" t="n">
         <v>35</v>
       </c>
-      <c r="BM26" t="n">
+      <c r="BN26" t="n">
         <v>35</v>
       </c>
     </row>
@@ -6096,9 +6177,12 @@
         <v>0</v>
       </c>
       <c r="BL27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM27" t="n">
         <v>25</v>
       </c>
-      <c r="BM27" t="n">
+      <c r="BN27" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6299,9 +6383,12 @@
         <v>0</v>
       </c>
       <c r="BL28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM28" t="n">
         <v>19</v>
       </c>
-      <c r="BM28" t="n">
+      <c r="BN28" t="n">
         <v>19</v>
       </c>
     </row>
@@ -6502,9 +6589,12 @@
         <v>0</v>
       </c>
       <c r="BL29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM29" t="n">
         <v>11</v>
       </c>
-      <c r="BM29" t="n">
+      <c r="BN29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6705,9 +6795,12 @@
         <v>0</v>
       </c>
       <c r="BL30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM30" t="n">
         <v>25</v>
       </c>
-      <c r="BM30" t="n">
+      <c r="BN30" t="n">
         <v>25</v>
       </c>
     </row>
@@ -6908,9 +7001,12 @@
         <v>0</v>
       </c>
       <c r="BL31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM31" t="n">
         <v>20</v>
       </c>
-      <c r="BM31" t="n">
+      <c r="BN31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -7111,9 +7207,12 @@
         <v>1</v>
       </c>
       <c r="BL32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM32" t="n">
         <v>23</v>
       </c>
-      <c r="BM32" t="n">
+      <c r="BN32" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7314,9 +7413,12 @@
         <v>0</v>
       </c>
       <c r="BL33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM33" t="n">
         <v>21</v>
       </c>
-      <c r="BM33" t="n">
+      <c r="BN33" t="n">
         <v>21</v>
       </c>
     </row>
@@ -7517,9 +7619,12 @@
         <v>0</v>
       </c>
       <c r="BL34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM34" t="n">
         <v>9</v>
       </c>
-      <c r="BM34" t="n">
+      <c r="BN34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7720,9 +7825,12 @@
         <v>0</v>
       </c>
       <c r="BL35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM35" t="n">
         <v>25</v>
       </c>
-      <c r="BM35" t="n">
+      <c r="BN35" t="n">
         <v>25</v>
       </c>
     </row>
@@ -7923,9 +8031,12 @@
         <v>0</v>
       </c>
       <c r="BL36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM36" t="n">
         <v>16</v>
       </c>
-      <c r="BM36" t="n">
+      <c r="BN36" t="n">
         <v>16</v>
       </c>
     </row>
@@ -8131,6 +8242,9 @@
       <c r="BM37" t="n">
         <v>0</v>
       </c>
+      <c r="BN37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8329,9 +8443,12 @@
         <v>0</v>
       </c>
       <c r="BL38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM38" t="n">
         <v>2</v>
       </c>
-      <c r="BM38" t="n">
+      <c r="BN38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8532,9 +8649,12 @@
         <v>1</v>
       </c>
       <c r="BL39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM39" t="n">
         <v>37</v>
       </c>
-      <c r="BM39" t="n">
+      <c r="BN39" t="n">
         <v>37</v>
       </c>
     </row>
@@ -8735,9 +8855,12 @@
         <v>0</v>
       </c>
       <c r="BL40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM40" t="n">
         <v>28</v>
       </c>
-      <c r="BM40" t="n">
+      <c r="BN40" t="n">
         <v>28</v>
       </c>
     </row>
@@ -8938,10 +9061,13 @@
         <v>1</v>
       </c>
       <c r="BL41" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="BM41" t="n">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="BN41" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="42">
@@ -9141,9 +9267,12 @@
         <v>0</v>
       </c>
       <c r="BL42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM42" t="n">
         <v>21</v>
       </c>
-      <c r="BM42" t="n">
+      <c r="BN42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9344,9 +9473,12 @@
         <v>0</v>
       </c>
       <c r="BL43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM43" t="n">
         <v>60</v>
       </c>
-      <c r="BM43" t="n">
+      <c r="BN43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9547,9 +9679,12 @@
         <v>0</v>
       </c>
       <c r="BL44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM44" t="n">
         <v>25</v>
       </c>
-      <c r="BM44" t="n">
+      <c r="BN44" t="n">
         <v>25</v>
       </c>
     </row>
@@ -9750,9 +9885,12 @@
         <v>0</v>
       </c>
       <c r="BL45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM45" t="n">
         <v>26</v>
       </c>
-      <c r="BM45" t="n">
+      <c r="BN45" t="n">
         <v>26</v>
       </c>
     </row>
@@ -9953,9 +10091,12 @@
         <v>0</v>
       </c>
       <c r="BL46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM46" t="n">
         <v>30</v>
       </c>
-      <c r="BM46" t="n">
+      <c r="BN46" t="n">
         <v>30</v>
       </c>
     </row>
@@ -10161,6 +10302,9 @@
       <c r="BM47" t="n">
         <v>0</v>
       </c>
+      <c r="BN47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -10359,10 +10503,13 @@
         <v>0</v>
       </c>
       <c r="BL48" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="BM48" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="BN48" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="49">
@@ -10562,9 +10709,12 @@
         <v>0</v>
       </c>
       <c r="BL49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM49" t="n">
         <v>19</v>
       </c>
-      <c r="BM49" t="n">
+      <c r="BN49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -10765,9 +10915,12 @@
         <v>0</v>
       </c>
       <c r="BL50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM50" t="n">
         <v>7</v>
       </c>
-      <c r="BM50" t="n">
+      <c r="BN50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10968,9 +11121,12 @@
         <v>0</v>
       </c>
       <c r="BL51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM51" t="n">
         <v>32</v>
       </c>
-      <c r="BM51" t="n">
+      <c r="BN51" t="n">
         <v>32</v>
       </c>
     </row>
@@ -11176,6 +11332,9 @@
       <c r="BM52" t="n">
         <v>0</v>
       </c>
+      <c r="BN52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11374,9 +11533,12 @@
         <v>0</v>
       </c>
       <c r="BL53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM53" t="n">
         <v>13</v>
       </c>
-      <c r="BM53" t="n">
+      <c r="BN53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -11582,6 +11744,9 @@
       <c r="BM54" t="n">
         <v>0</v>
       </c>
+      <c r="BN54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11780,9 +11945,12 @@
         <v>1</v>
       </c>
       <c r="BL55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM55" t="n">
         <v>36</v>
       </c>
-      <c r="BM55" t="n">
+      <c r="BN55" t="n">
         <v>36</v>
       </c>
     </row>
@@ -11983,9 +12151,12 @@
         <v>0</v>
       </c>
       <c r="BL56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM56" t="n">
         <v>31</v>
       </c>
-      <c r="BM56" t="n">
+      <c r="BN56" t="n">
         <v>31</v>
       </c>
     </row>
@@ -12186,9 +12357,12 @@
         <v>0</v>
       </c>
       <c r="BL57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM57" t="n">
         <v>10</v>
       </c>
-      <c r="BM57" t="n">
+      <c r="BN57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -12389,9 +12563,12 @@
         <v>0</v>
       </c>
       <c r="BL58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM58" t="n">
         <v>13</v>
       </c>
-      <c r="BM58" t="n">
+      <c r="BN58" t="n">
         <v>13</v>
       </c>
     </row>
@@ -12592,9 +12769,12 @@
         <v>0</v>
       </c>
       <c r="BL59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM59" t="n">
         <v>6</v>
       </c>
-      <c r="BM59" t="n">
+      <c r="BN59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -12800,6 +12980,9 @@
       <c r="BM60" t="n">
         <v>0</v>
       </c>
+      <c r="BN60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12998,9 +13181,12 @@
         <v>0</v>
       </c>
       <c r="BL61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM61" t="n">
         <v>29</v>
       </c>
-      <c r="BM61" t="n">
+      <c r="BN61" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13201,9 +13387,12 @@
         <v>0</v>
       </c>
       <c r="BL62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM62" t="n">
         <v>29</v>
       </c>
-      <c r="BM62" t="n">
+      <c r="BN62" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13404,9 +13593,12 @@
         <v>0</v>
       </c>
       <c r="BL63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM63" t="n">
         <v>12</v>
       </c>
-      <c r="BM63" t="n">
+      <c r="BN63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -13612,6 +13804,9 @@
       <c r="BM64" t="n">
         <v>0</v>
       </c>
+      <c r="BN64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -13810,9 +14005,12 @@
         <v>0</v>
       </c>
       <c r="BL65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM65" t="n">
         <v>17</v>
       </c>
-      <c r="BM65" t="n">
+      <c r="BN65" t="n">
         <v>17</v>
       </c>
     </row>
@@ -14013,9 +14211,12 @@
         <v>0</v>
       </c>
       <c r="BL66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM66" t="n">
         <v>8</v>
       </c>
-      <c r="BM66" t="n">
+      <c r="BN66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -14216,10 +14417,13 @@
         <v>1</v>
       </c>
       <c r="BL67" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="BM67" t="n">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="BN67" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="68">
@@ -14419,9 +14623,12 @@
         <v>1</v>
       </c>
       <c r="BL68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM68" t="n">
         <v>23</v>
       </c>
-      <c r="BM68" t="n">
+      <c r="BN68" t="n">
         <v>22</v>
       </c>
     </row>
@@ -14622,9 +14829,12 @@
         <v>0</v>
       </c>
       <c r="BL69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM69" t="n">
         <v>7</v>
       </c>
-      <c r="BM69" t="n">
+      <c r="BN69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -14825,9 +15035,12 @@
         <v>0</v>
       </c>
       <c r="BL70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM70" t="n">
         <v>23</v>
       </c>
-      <c r="BM70" t="n">
+      <c r="BN70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -15028,9 +15241,12 @@
         <v>0</v>
       </c>
       <c r="BL71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM71" t="n">
         <v>24</v>
       </c>
-      <c r="BM71" t="n">
+      <c r="BN71" t="n">
         <v>24</v>
       </c>
     </row>
@@ -15231,9 +15447,12 @@
         <v>0</v>
       </c>
       <c r="BL72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM72" t="n">
         <v>24</v>
       </c>
-      <c r="BM72" t="n">
+      <c r="BN72" t="n">
         <v>24</v>
       </c>
     </row>
@@ -15439,6 +15658,9 @@
       <c r="BM73" t="n">
         <v>0</v>
       </c>
+      <c r="BN73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -15642,6 +15864,9 @@
       <c r="BM74" t="n">
         <v>0</v>
       </c>
+      <c r="BN74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -15840,9 +16065,12 @@
         <v>1</v>
       </c>
       <c r="BL75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM75" t="n">
         <v>25</v>
       </c>
-      <c r="BM75" t="n">
+      <c r="BN75" t="n">
         <v>25</v>
       </c>
     </row>
@@ -16043,9 +16271,12 @@
         <v>0</v>
       </c>
       <c r="BL76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM76" t="n">
         <v>21</v>
       </c>
-      <c r="BM76" t="n">
+      <c r="BN76" t="n">
         <v>21</v>
       </c>
     </row>
@@ -16246,9 +16477,12 @@
         <v>0</v>
       </c>
       <c r="BL77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM77" t="n">
         <v>15</v>
       </c>
-      <c r="BM77" t="n">
+      <c r="BN77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -16449,9 +16683,12 @@
         <v>1</v>
       </c>
       <c r="BL78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM78" t="n">
         <v>36</v>
       </c>
-      <c r="BM78" t="n">
+      <c r="BN78" t="n">
         <v>35</v>
       </c>
     </row>
@@ -16652,9 +16889,12 @@
         <v>0</v>
       </c>
       <c r="BL79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM79" t="n">
         <v>22</v>
       </c>
-      <c r="BM79" t="n">
+      <c r="BN79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -16855,10 +17095,13 @@
         <v>0</v>
       </c>
       <c r="BL80" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="BM80" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="BN80" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="81">
@@ -17058,9 +17301,12 @@
         <v>0</v>
       </c>
       <c r="BL81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM81" t="n">
         <v>4</v>
       </c>
-      <c r="BM81" t="n">
+      <c r="BN81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -17261,9 +17507,12 @@
         <v>0</v>
       </c>
       <c r="BL82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM82" t="n">
         <v>18</v>
       </c>
-      <c r="BM82" t="n">
+      <c r="BN82" t="n">
         <v>18</v>
       </c>
     </row>
@@ -17464,9 +17713,12 @@
         <v>0</v>
       </c>
       <c r="BL83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM83" t="n">
         <v>17</v>
       </c>
-      <c r="BM83" t="n">
+      <c r="BN83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -17667,9 +17919,12 @@
         <v>0</v>
       </c>
       <c r="BL84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM84" t="n">
         <v>13</v>
       </c>
-      <c r="BM84" t="n">
+      <c r="BN84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -17870,9 +18125,12 @@
         <v>0</v>
       </c>
       <c r="BL85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM85" t="n">
         <v>7</v>
       </c>
-      <c r="BM85" t="n">
+      <c r="BN85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18078,6 +18336,9 @@
       <c r="BM86" t="n">
         <v>0</v>
       </c>
+      <c r="BN86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -18276,9 +18537,12 @@
         <v>0</v>
       </c>
       <c r="BL87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM87" t="n">
         <v>19</v>
       </c>
-      <c r="BM87" t="n">
+      <c r="BN87" t="n">
         <v>19</v>
       </c>
     </row>
@@ -18484,6 +18748,9 @@
       <c r="BM88" t="n">
         <v>0</v>
       </c>
+      <c r="BN88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -18682,9 +18949,12 @@
         <v>0</v>
       </c>
       <c r="BL89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM89" t="n">
         <v>18</v>
       </c>
-      <c r="BM89" t="n">
+      <c r="BN89" t="n">
         <v>18</v>
       </c>
     </row>
@@ -18885,9 +19155,12 @@
         <v>0</v>
       </c>
       <c r="BL90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM90" t="n">
         <v>17</v>
       </c>
-      <c r="BM90" t="n">
+      <c r="BN90" t="n">
         <v>17</v>
       </c>
     </row>
@@ -19088,9 +19361,12 @@
         <v>0</v>
       </c>
       <c r="BL91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM91" t="n">
         <v>42</v>
       </c>
-      <c r="BM91" t="n">
+      <c r="BN91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -19291,9 +19567,12 @@
         <v>0</v>
       </c>
       <c r="BL92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM92" t="n">
         <v>7</v>
       </c>
-      <c r="BM92" t="n">
+      <c r="BN92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -19499,6 +19778,9 @@
       <c r="BM93" t="n">
         <v>0</v>
       </c>
+      <c r="BN93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -19697,9 +19979,12 @@
         <v>0</v>
       </c>
       <c r="BL94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM94" t="n">
         <v>16</v>
       </c>
-      <c r="BM94" t="n">
+      <c r="BN94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -19900,9 +20185,12 @@
         <v>0</v>
       </c>
       <c r="BL95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM95" t="n">
         <v>7</v>
       </c>
-      <c r="BM95" t="n">
+      <c r="BN95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -20103,9 +20391,12 @@
         <v>0</v>
       </c>
       <c r="BL96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM96" t="n">
         <v>24</v>
       </c>
-      <c r="BM96" t="n">
+      <c r="BN96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -20311,6 +20602,9 @@
       <c r="BM97" t="n">
         <v>0</v>
       </c>
+      <c r="BN97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -20509,9 +20803,12 @@
         <v>1</v>
       </c>
       <c r="BL98" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM98" t="n">
         <v>35</v>
       </c>
-      <c r="BM98" t="n">
+      <c r="BN98" t="n">
         <v>35</v>
       </c>
     </row>
@@ -20712,9 +21009,12 @@
         <v>0</v>
       </c>
       <c r="BL99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM99" t="n">
         <v>14</v>
       </c>
-      <c r="BM99" t="n">
+      <c r="BN99" t="n">
         <v>14</v>
       </c>
     </row>
@@ -20920,6 +21220,9 @@
       <c r="BM100" t="n">
         <v>0</v>
       </c>
+      <c r="BN100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -21118,9 +21421,12 @@
         <v>0</v>
       </c>
       <c r="BL101" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM101" t="n">
         <v>31</v>
       </c>
-      <c r="BM101" t="n">
+      <c r="BN101" t="n">
         <v>31</v>
       </c>
     </row>
@@ -21321,10 +21627,13 @@
         <v>0</v>
       </c>
       <c r="BL102" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="BM102" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="BN102" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="103">
@@ -21524,9 +21833,12 @@
         <v>1</v>
       </c>
       <c r="BL103" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM103" t="n">
         <v>34</v>
       </c>
-      <c r="BM103" t="n">
+      <c r="BN103" t="n">
         <v>34</v>
       </c>
     </row>
@@ -21727,9 +22039,12 @@
         <v>0</v>
       </c>
       <c r="BL104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM104" t="n">
         <v>12</v>
       </c>
-      <c r="BM104" t="n">
+      <c r="BN104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -21930,9 +22245,12 @@
         <v>1</v>
       </c>
       <c r="BL105" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM105" t="n">
         <v>28</v>
       </c>
-      <c r="BM105" t="n">
+      <c r="BN105" t="n">
         <v>28</v>
       </c>
     </row>
@@ -22133,9 +22451,12 @@
         <v>0</v>
       </c>
       <c r="BL106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM106" t="n">
         <v>7</v>
       </c>
-      <c r="BM106" t="n">
+      <c r="BN106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -22336,9 +22657,12 @@
         <v>0</v>
       </c>
       <c r="BL107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM107" t="n">
         <v>13</v>
       </c>
-      <c r="BM107" t="n">
+      <c r="BN107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -22539,9 +22863,12 @@
         <v>0</v>
       </c>
       <c r="BL108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM108" t="n">
         <v>2</v>
       </c>
-      <c r="BM108" t="n">
+      <c r="BN108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -22742,9 +23069,12 @@
         <v>0</v>
       </c>
       <c r="BL109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM109" t="n">
         <v>4</v>
       </c>
-      <c r="BM109" t="n">
+      <c r="BN109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#4433)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BN109"/>
+  <dimension ref="A1:BO109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -494,8 +494,9 @@
     <col width="12" customWidth="1" min="62" max="62"/>
     <col width="12" customWidth="1" min="63" max="63"/>
     <col width="12" customWidth="1" min="64" max="64"/>
-    <col width="13" customWidth="1" min="65" max="65"/>
+    <col width="12" customWidth="1" min="65" max="65"/>
     <col width="13" customWidth="1" min="66" max="66"/>
+    <col width="13" customWidth="1" min="67" max="67"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -819,12 +820,17 @@
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="BM1" s="2" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="BN1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BN1" s="2" t="inlineStr">
+      <c r="BO1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -1030,9 +1036,12 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN2" t="n">
         <v>12</v>
       </c>
-      <c r="BN2" t="n">
+      <c r="BO2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1236,9 +1245,12 @@
         <v>0</v>
       </c>
       <c r="BM3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN3" t="n">
         <v>10</v>
       </c>
-      <c r="BN3" t="n">
+      <c r="BO3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1442,9 +1454,12 @@
         <v>1</v>
       </c>
       <c r="BM4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN4" t="n">
         <v>40</v>
       </c>
-      <c r="BN4" t="n">
+      <c r="BO4" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1648,9 +1663,12 @@
         <v>0</v>
       </c>
       <c r="BM5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN5" t="n">
         <v>15</v>
       </c>
-      <c r="BN5" t="n">
+      <c r="BO5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1854,9 +1872,12 @@
         <v>0</v>
       </c>
       <c r="BM6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN6" t="n">
         <v>19</v>
       </c>
-      <c r="BN6" t="n">
+      <c r="BO6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2060,9 +2081,12 @@
         <v>0</v>
       </c>
       <c r="BM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN7" t="n">
         <v>19</v>
       </c>
-      <c r="BN7" t="n">
+      <c r="BO7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2266,9 +2290,12 @@
         <v>0</v>
       </c>
       <c r="BM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN8" t="n">
         <v>32</v>
       </c>
-      <c r="BN8" t="n">
+      <c r="BO8" t="n">
         <v>32</v>
       </c>
     </row>
@@ -2472,9 +2499,12 @@
         <v>0</v>
       </c>
       <c r="BM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN9" t="n">
         <v>31</v>
       </c>
-      <c r="BN9" t="n">
+      <c r="BO9" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2678,9 +2708,12 @@
         <v>1</v>
       </c>
       <c r="BM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN10" t="n">
         <v>39</v>
       </c>
-      <c r="BN10" t="n">
+      <c r="BO10" t="n">
         <v>39</v>
       </c>
     </row>
@@ -2884,9 +2917,12 @@
         <v>0</v>
       </c>
       <c r="BM11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN11" t="n">
         <v>29</v>
       </c>
-      <c r="BN11" t="n">
+      <c r="BO11" t="n">
         <v>29</v>
       </c>
     </row>
@@ -3090,9 +3126,12 @@
         <v>0</v>
       </c>
       <c r="BM12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN12" t="n">
         <v>37</v>
       </c>
-      <c r="BN12" t="n">
+      <c r="BO12" t="n">
         <v>37</v>
       </c>
     </row>
@@ -3296,9 +3335,12 @@
         <v>0</v>
       </c>
       <c r="BM13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN13" t="n">
         <v>14</v>
       </c>
-      <c r="BN13" t="n">
+      <c r="BO13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3502,9 +3544,12 @@
         <v>0</v>
       </c>
       <c r="BM14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN14" t="n">
         <v>26</v>
       </c>
-      <c r="BN14" t="n">
+      <c r="BO14" t="n">
         <v>26</v>
       </c>
     </row>
@@ -3708,9 +3753,12 @@
         <v>0</v>
       </c>
       <c r="BM15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN15" t="n">
         <v>9</v>
       </c>
-      <c r="BN15" t="n">
+      <c r="BO15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3914,9 +3962,12 @@
         <v>0</v>
       </c>
       <c r="BM16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN16" t="n">
         <v>20</v>
       </c>
-      <c r="BN16" t="n">
+      <c r="BO16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4120,9 +4171,12 @@
         <v>0</v>
       </c>
       <c r="BM17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN17" t="n">
         <v>17</v>
       </c>
-      <c r="BN17" t="n">
+      <c r="BO17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4326,9 +4380,12 @@
         <v>0</v>
       </c>
       <c r="BM18" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN18" t="n">
         <v>33</v>
       </c>
-      <c r="BN18" t="n">
+      <c r="BO18" t="n">
         <v>33</v>
       </c>
     </row>
@@ -4537,6 +4594,9 @@
       <c r="BN19" t="n">
         <v>0</v>
       </c>
+      <c r="BO19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4738,9 +4798,12 @@
         <v>0</v>
       </c>
       <c r="BM20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN20" t="n">
         <v>20</v>
       </c>
-      <c r="BN20" t="n">
+      <c r="BO20" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4944,9 +5007,12 @@
         <v>0</v>
       </c>
       <c r="BM21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN21" t="n">
         <v>27</v>
       </c>
-      <c r="BN21" t="n">
+      <c r="BO21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5155,6 +5221,9 @@
       <c r="BN22" t="n">
         <v>0</v>
       </c>
+      <c r="BO22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5356,9 +5425,12 @@
         <v>0</v>
       </c>
       <c r="BM23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN23" t="n">
         <v>22</v>
       </c>
-      <c r="BN23" t="n">
+      <c r="BO23" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5562,9 +5634,12 @@
         <v>0</v>
       </c>
       <c r="BM24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN24" t="n">
         <v>27</v>
       </c>
-      <c r="BN24" t="n">
+      <c r="BO24" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5768,9 +5843,12 @@
         <v>0</v>
       </c>
       <c r="BM25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN25" t="n">
         <v>11</v>
       </c>
-      <c r="BN25" t="n">
+      <c r="BO25" t="n">
         <v>11</v>
       </c>
     </row>
@@ -5974,9 +6052,12 @@
         <v>0</v>
       </c>
       <c r="BM26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN26" t="n">
         <v>35</v>
       </c>
-      <c r="BN26" t="n">
+      <c r="BO26" t="n">
         <v>35</v>
       </c>
     </row>
@@ -6180,9 +6261,12 @@
         <v>0</v>
       </c>
       <c r="BM27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN27" t="n">
         <v>25</v>
       </c>
-      <c r="BN27" t="n">
+      <c r="BO27" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6386,9 +6470,12 @@
         <v>0</v>
       </c>
       <c r="BM28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN28" t="n">
         <v>19</v>
       </c>
-      <c r="BN28" t="n">
+      <c r="BO28" t="n">
         <v>19</v>
       </c>
     </row>
@@ -6592,9 +6679,12 @@
         <v>0</v>
       </c>
       <c r="BM29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN29" t="n">
         <v>11</v>
       </c>
-      <c r="BN29" t="n">
+      <c r="BO29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6798,9 +6888,12 @@
         <v>0</v>
       </c>
       <c r="BM30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN30" t="n">
         <v>25</v>
       </c>
-      <c r="BN30" t="n">
+      <c r="BO30" t="n">
         <v>25</v>
       </c>
     </row>
@@ -7004,9 +7097,12 @@
         <v>0</v>
       </c>
       <c r="BM31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN31" t="n">
         <v>20</v>
       </c>
-      <c r="BN31" t="n">
+      <c r="BO31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -7210,9 +7306,12 @@
         <v>0</v>
       </c>
       <c r="BM32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN32" t="n">
         <v>23</v>
       </c>
-      <c r="BN32" t="n">
+      <c r="BO32" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7416,9 +7515,12 @@
         <v>0</v>
       </c>
       <c r="BM33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN33" t="n">
         <v>21</v>
       </c>
-      <c r="BN33" t="n">
+      <c r="BO33" t="n">
         <v>21</v>
       </c>
     </row>
@@ -7622,9 +7724,12 @@
         <v>0</v>
       </c>
       <c r="BM34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN34" t="n">
         <v>9</v>
       </c>
-      <c r="BN34" t="n">
+      <c r="BO34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7828,9 +7933,12 @@
         <v>0</v>
       </c>
       <c r="BM35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN35" t="n">
         <v>25</v>
       </c>
-      <c r="BN35" t="n">
+      <c r="BO35" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8034,9 +8142,12 @@
         <v>0</v>
       </c>
       <c r="BM36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN36" t="n">
         <v>16</v>
       </c>
-      <c r="BN36" t="n">
+      <c r="BO36" t="n">
         <v>16</v>
       </c>
     </row>
@@ -8245,6 +8356,9 @@
       <c r="BN37" t="n">
         <v>0</v>
       </c>
+      <c r="BO37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8446,9 +8560,12 @@
         <v>0</v>
       </c>
       <c r="BM38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN38" t="n">
         <v>2</v>
       </c>
-      <c r="BN38" t="n">
+      <c r="BO38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8652,9 +8769,12 @@
         <v>0</v>
       </c>
       <c r="BM39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN39" t="n">
         <v>37</v>
       </c>
-      <c r="BN39" t="n">
+      <c r="BO39" t="n">
         <v>37</v>
       </c>
     </row>
@@ -8858,9 +8978,12 @@
         <v>0</v>
       </c>
       <c r="BM40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN40" t="n">
         <v>28</v>
       </c>
-      <c r="BN40" t="n">
+      <c r="BO40" t="n">
         <v>28</v>
       </c>
     </row>
@@ -9064,9 +9187,12 @@
         <v>1</v>
       </c>
       <c r="BM41" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN41" t="n">
         <v>39</v>
       </c>
-      <c r="BN41" t="n">
+      <c r="BO41" t="n">
         <v>39</v>
       </c>
     </row>
@@ -9270,9 +9396,12 @@
         <v>0</v>
       </c>
       <c r="BM42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN42" t="n">
         <v>21</v>
       </c>
-      <c r="BN42" t="n">
+      <c r="BO42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9476,9 +9605,12 @@
         <v>0</v>
       </c>
       <c r="BM43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN43" t="n">
         <v>60</v>
       </c>
-      <c r="BN43" t="n">
+      <c r="BO43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9682,9 +9814,12 @@
         <v>0</v>
       </c>
       <c r="BM44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN44" t="n">
         <v>25</v>
       </c>
-      <c r="BN44" t="n">
+      <c r="BO44" t="n">
         <v>25</v>
       </c>
     </row>
@@ -9888,9 +10023,12 @@
         <v>0</v>
       </c>
       <c r="BM45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN45" t="n">
         <v>26</v>
       </c>
-      <c r="BN45" t="n">
+      <c r="BO45" t="n">
         <v>26</v>
       </c>
     </row>
@@ -10094,9 +10232,12 @@
         <v>0</v>
       </c>
       <c r="BM46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN46" t="n">
         <v>30</v>
       </c>
-      <c r="BN46" t="n">
+      <c r="BO46" t="n">
         <v>30</v>
       </c>
     </row>
@@ -10305,6 +10446,9 @@
       <c r="BN47" t="n">
         <v>0</v>
       </c>
+      <c r="BO47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -10506,9 +10650,12 @@
         <v>1</v>
       </c>
       <c r="BM48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN48" t="n">
         <v>27</v>
       </c>
-      <c r="BN48" t="n">
+      <c r="BO48" t="n">
         <v>27</v>
       </c>
     </row>
@@ -10712,9 +10859,12 @@
         <v>0</v>
       </c>
       <c r="BM49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN49" t="n">
         <v>19</v>
       </c>
-      <c r="BN49" t="n">
+      <c r="BO49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -10918,9 +11068,12 @@
         <v>0</v>
       </c>
       <c r="BM50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN50" t="n">
         <v>7</v>
       </c>
-      <c r="BN50" t="n">
+      <c r="BO50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11124,9 +11277,12 @@
         <v>0</v>
       </c>
       <c r="BM51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN51" t="n">
         <v>32</v>
       </c>
-      <c r="BN51" t="n">
+      <c r="BO51" t="n">
         <v>32</v>
       </c>
     </row>
@@ -11335,6 +11491,9 @@
       <c r="BN52" t="n">
         <v>0</v>
       </c>
+      <c r="BO52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11536,9 +11695,12 @@
         <v>0</v>
       </c>
       <c r="BM53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN53" t="n">
         <v>13</v>
       </c>
-      <c r="BN53" t="n">
+      <c r="BO53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -11747,6 +11909,9 @@
       <c r="BN54" t="n">
         <v>0</v>
       </c>
+      <c r="BO54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11948,9 +12113,12 @@
         <v>0</v>
       </c>
       <c r="BM55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN55" t="n">
         <v>36</v>
       </c>
-      <c r="BN55" t="n">
+      <c r="BO55" t="n">
         <v>36</v>
       </c>
     </row>
@@ -12154,9 +12322,12 @@
         <v>0</v>
       </c>
       <c r="BM56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN56" t="n">
         <v>31</v>
       </c>
-      <c r="BN56" t="n">
+      <c r="BO56" t="n">
         <v>31</v>
       </c>
     </row>
@@ -12360,9 +12531,12 @@
         <v>0</v>
       </c>
       <c r="BM57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN57" t="n">
         <v>10</v>
       </c>
-      <c r="BN57" t="n">
+      <c r="BO57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -12566,9 +12740,12 @@
         <v>0</v>
       </c>
       <c r="BM58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN58" t="n">
         <v>13</v>
       </c>
-      <c r="BN58" t="n">
+      <c r="BO58" t="n">
         <v>13</v>
       </c>
     </row>
@@ -12772,9 +12949,12 @@
         <v>0</v>
       </c>
       <c r="BM59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN59" t="n">
         <v>6</v>
       </c>
-      <c r="BN59" t="n">
+      <c r="BO59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -12983,6 +13163,9 @@
       <c r="BN60" t="n">
         <v>0</v>
       </c>
+      <c r="BO60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -13184,9 +13367,12 @@
         <v>0</v>
       </c>
       <c r="BM61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN61" t="n">
         <v>29</v>
       </c>
-      <c r="BN61" t="n">
+      <c r="BO61" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13390,9 +13576,12 @@
         <v>0</v>
       </c>
       <c r="BM62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN62" t="n">
         <v>29</v>
       </c>
-      <c r="BN62" t="n">
+      <c r="BO62" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13596,9 +13785,12 @@
         <v>0</v>
       </c>
       <c r="BM63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN63" t="n">
         <v>12</v>
       </c>
-      <c r="BN63" t="n">
+      <c r="BO63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -13807,6 +13999,9 @@
       <c r="BN64" t="n">
         <v>0</v>
       </c>
+      <c r="BO64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -14008,9 +14203,12 @@
         <v>0</v>
       </c>
       <c r="BM65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN65" t="n">
         <v>17</v>
       </c>
-      <c r="BN65" t="n">
+      <c r="BO65" t="n">
         <v>17</v>
       </c>
     </row>
@@ -14214,9 +14412,12 @@
         <v>0</v>
       </c>
       <c r="BM66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN66" t="n">
         <v>8</v>
       </c>
-      <c r="BN66" t="n">
+      <c r="BO66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -14420,9 +14621,12 @@
         <v>1</v>
       </c>
       <c r="BM67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN67" t="n">
         <v>40</v>
       </c>
-      <c r="BN67" t="n">
+      <c r="BO67" t="n">
         <v>40</v>
       </c>
     </row>
@@ -14626,9 +14830,12 @@
         <v>0</v>
       </c>
       <c r="BM68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN68" t="n">
         <v>23</v>
       </c>
-      <c r="BN68" t="n">
+      <c r="BO68" t="n">
         <v>22</v>
       </c>
     </row>
@@ -14832,9 +15039,12 @@
         <v>0</v>
       </c>
       <c r="BM69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN69" t="n">
         <v>7</v>
       </c>
-      <c r="BN69" t="n">
+      <c r="BO69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15038,9 +15248,12 @@
         <v>0</v>
       </c>
       <c r="BM70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN70" t="n">
         <v>23</v>
       </c>
-      <c r="BN70" t="n">
+      <c r="BO70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -15244,9 +15457,12 @@
         <v>0</v>
       </c>
       <c r="BM71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN71" t="n">
         <v>24</v>
       </c>
-      <c r="BN71" t="n">
+      <c r="BO71" t="n">
         <v>24</v>
       </c>
     </row>
@@ -15450,9 +15666,12 @@
         <v>0</v>
       </c>
       <c r="BM72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN72" t="n">
         <v>24</v>
       </c>
-      <c r="BN72" t="n">
+      <c r="BO72" t="n">
         <v>24</v>
       </c>
     </row>
@@ -15661,6 +15880,9 @@
       <c r="BN73" t="n">
         <v>0</v>
       </c>
+      <c r="BO73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -15867,6 +16089,9 @@
       <c r="BN74" t="n">
         <v>0</v>
       </c>
+      <c r="BO74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -16068,9 +16293,12 @@
         <v>0</v>
       </c>
       <c r="BM75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN75" t="n">
         <v>25</v>
       </c>
-      <c r="BN75" t="n">
+      <c r="BO75" t="n">
         <v>25</v>
       </c>
     </row>
@@ -16274,9 +16502,12 @@
         <v>0</v>
       </c>
       <c r="BM76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN76" t="n">
         <v>21</v>
       </c>
-      <c r="BN76" t="n">
+      <c r="BO76" t="n">
         <v>21</v>
       </c>
     </row>
@@ -16480,9 +16711,12 @@
         <v>0</v>
       </c>
       <c r="BM77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN77" t="n">
         <v>15</v>
       </c>
-      <c r="BN77" t="n">
+      <c r="BO77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -16686,9 +16920,12 @@
         <v>0</v>
       </c>
       <c r="BM78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN78" t="n">
         <v>36</v>
       </c>
-      <c r="BN78" t="n">
+      <c r="BO78" t="n">
         <v>35</v>
       </c>
     </row>
@@ -16892,9 +17129,12 @@
         <v>0</v>
       </c>
       <c r="BM79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN79" t="n">
         <v>22</v>
       </c>
-      <c r="BN79" t="n">
+      <c r="BO79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -17098,9 +17338,12 @@
         <v>1</v>
       </c>
       <c r="BM80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN80" t="n">
         <v>12</v>
       </c>
-      <c r="BN80" t="n">
+      <c r="BO80" t="n">
         <v>12</v>
       </c>
     </row>
@@ -17304,9 +17547,12 @@
         <v>0</v>
       </c>
       <c r="BM81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN81" t="n">
         <v>4</v>
       </c>
-      <c r="BN81" t="n">
+      <c r="BO81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -17510,9 +17756,12 @@
         <v>0</v>
       </c>
       <c r="BM82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN82" t="n">
         <v>18</v>
       </c>
-      <c r="BN82" t="n">
+      <c r="BO82" t="n">
         <v>18</v>
       </c>
     </row>
@@ -17716,9 +17965,12 @@
         <v>0</v>
       </c>
       <c r="BM83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN83" t="n">
         <v>17</v>
       </c>
-      <c r="BN83" t="n">
+      <c r="BO83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -17922,9 +18174,12 @@
         <v>0</v>
       </c>
       <c r="BM84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN84" t="n">
         <v>13</v>
       </c>
-      <c r="BN84" t="n">
+      <c r="BO84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -18128,9 +18383,12 @@
         <v>0</v>
       </c>
       <c r="BM85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN85" t="n">
         <v>7</v>
       </c>
-      <c r="BN85" t="n">
+      <c r="BO85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18339,6 +18597,9 @@
       <c r="BN86" t="n">
         <v>0</v>
       </c>
+      <c r="BO86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -18540,9 +18801,12 @@
         <v>0</v>
       </c>
       <c r="BM87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN87" t="n">
         <v>19</v>
       </c>
-      <c r="BN87" t="n">
+      <c r="BO87" t="n">
         <v>19</v>
       </c>
     </row>
@@ -18751,6 +19015,9 @@
       <c r="BN88" t="n">
         <v>0</v>
       </c>
+      <c r="BO88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -18952,9 +19219,12 @@
         <v>0</v>
       </c>
       <c r="BM89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN89" t="n">
         <v>18</v>
       </c>
-      <c r="BN89" t="n">
+      <c r="BO89" t="n">
         <v>18</v>
       </c>
     </row>
@@ -19158,9 +19428,12 @@
         <v>0</v>
       </c>
       <c r="BM90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN90" t="n">
         <v>17</v>
       </c>
-      <c r="BN90" t="n">
+      <c r="BO90" t="n">
         <v>17</v>
       </c>
     </row>
@@ -19364,9 +19637,12 @@
         <v>0</v>
       </c>
       <c r="BM91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN91" t="n">
         <v>42</v>
       </c>
-      <c r="BN91" t="n">
+      <c r="BO91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -19570,9 +19846,12 @@
         <v>0</v>
       </c>
       <c r="BM92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN92" t="n">
         <v>7</v>
       </c>
-      <c r="BN92" t="n">
+      <c r="BO92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -19781,6 +20060,9 @@
       <c r="BN93" t="n">
         <v>0</v>
       </c>
+      <c r="BO93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -19982,9 +20264,12 @@
         <v>0</v>
       </c>
       <c r="BM94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN94" t="n">
         <v>16</v>
       </c>
-      <c r="BN94" t="n">
+      <c r="BO94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -20188,9 +20473,12 @@
         <v>0</v>
       </c>
       <c r="BM95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN95" t="n">
         <v>7</v>
       </c>
-      <c r="BN95" t="n">
+      <c r="BO95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -20394,9 +20682,12 @@
         <v>0</v>
       </c>
       <c r="BM96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN96" t="n">
         <v>24</v>
       </c>
-      <c r="BN96" t="n">
+      <c r="BO96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -20605,6 +20896,9 @@
       <c r="BN97" t="n">
         <v>0</v>
       </c>
+      <c r="BO97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -20806,9 +21100,12 @@
         <v>0</v>
       </c>
       <c r="BM98" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN98" t="n">
         <v>35</v>
       </c>
-      <c r="BN98" t="n">
+      <c r="BO98" t="n">
         <v>35</v>
       </c>
     </row>
@@ -21012,9 +21309,12 @@
         <v>0</v>
       </c>
       <c r="BM99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN99" t="n">
         <v>14</v>
       </c>
-      <c r="BN99" t="n">
+      <c r="BO99" t="n">
         <v>14</v>
       </c>
     </row>
@@ -21223,6 +21523,9 @@
       <c r="BN100" t="n">
         <v>0</v>
       </c>
+      <c r="BO100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -21424,9 +21727,12 @@
         <v>0</v>
       </c>
       <c r="BM101" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN101" t="n">
         <v>31</v>
       </c>
-      <c r="BN101" t="n">
+      <c r="BO101" t="n">
         <v>31</v>
       </c>
     </row>
@@ -21630,9 +21936,12 @@
         <v>1</v>
       </c>
       <c r="BM102" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN102" t="n">
         <v>31</v>
       </c>
-      <c r="BN102" t="n">
+      <c r="BO102" t="n">
         <v>31</v>
       </c>
     </row>
@@ -21836,9 +22145,12 @@
         <v>0</v>
       </c>
       <c r="BM103" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN103" t="n">
         <v>34</v>
       </c>
-      <c r="BN103" t="n">
+      <c r="BO103" t="n">
         <v>34</v>
       </c>
     </row>
@@ -22042,9 +22354,12 @@
         <v>0</v>
       </c>
       <c r="BM104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN104" t="n">
         <v>12</v>
       </c>
-      <c r="BN104" t="n">
+      <c r="BO104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -22248,9 +22563,12 @@
         <v>0</v>
       </c>
       <c r="BM105" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN105" t="n">
         <v>28</v>
       </c>
-      <c r="BN105" t="n">
+      <c r="BO105" t="n">
         <v>28</v>
       </c>
     </row>
@@ -22454,9 +22772,12 @@
         <v>0</v>
       </c>
       <c r="BM106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN106" t="n">
         <v>7</v>
       </c>
-      <c r="BN106" t="n">
+      <c r="BO106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -22660,9 +22981,12 @@
         <v>0</v>
       </c>
       <c r="BM107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN107" t="n">
         <v>13</v>
       </c>
-      <c r="BN107" t="n">
+      <c r="BO107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -22866,9 +23190,12 @@
         <v>0</v>
       </c>
       <c r="BM108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN108" t="n">
         <v>2</v>
       </c>
-      <c r="BN108" t="n">
+      <c r="BO108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -23072,9 +23399,12 @@
         <v>0</v>
       </c>
       <c r="BM109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN109" t="n">
         <v>4</v>
       </c>
-      <c r="BN109" t="n">
+      <c r="BO109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily IST report: add CSV/MD/XLSX (#4497)
Co-authored-by: codethesept <198977775+codethesept@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO109"/>
+  <dimension ref="A1:BP109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -495,8 +495,9 @@
     <col width="12" customWidth="1" min="63" max="63"/>
     <col width="12" customWidth="1" min="64" max="64"/>
     <col width="12" customWidth="1" min="65" max="65"/>
-    <col width="13" customWidth="1" min="66" max="66"/>
+    <col width="12" customWidth="1" min="66" max="66"/>
     <col width="13" customWidth="1" min="67" max="67"/>
+    <col width="13" customWidth="1" min="68" max="68"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -825,12 +826,17 @@
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="BN1" s="2" t="inlineStr">
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="BO1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BO1" s="2" t="inlineStr">
+      <c r="BP1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -1039,9 +1045,12 @@
         <v>0</v>
       </c>
       <c r="BN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO2" t="n">
         <v>12</v>
       </c>
-      <c r="BO2" t="n">
+      <c r="BP2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1248,9 +1257,12 @@
         <v>0</v>
       </c>
       <c r="BN3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO3" t="n">
         <v>10</v>
       </c>
-      <c r="BO3" t="n">
+      <c r="BP3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1457,9 +1469,12 @@
         <v>0</v>
       </c>
       <c r="BN4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO4" t="n">
         <v>40</v>
       </c>
-      <c r="BO4" t="n">
+      <c r="BP4" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1666,9 +1681,12 @@
         <v>0</v>
       </c>
       <c r="BN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO5" t="n">
         <v>15</v>
       </c>
-      <c r="BO5" t="n">
+      <c r="BP5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1875,9 +1893,12 @@
         <v>0</v>
       </c>
       <c r="BN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO6" t="n">
         <v>19</v>
       </c>
-      <c r="BO6" t="n">
+      <c r="BP6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2084,9 +2105,12 @@
         <v>0</v>
       </c>
       <c r="BN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO7" t="n">
         <v>19</v>
       </c>
-      <c r="BO7" t="n">
+      <c r="BP7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2293,9 +2317,12 @@
         <v>0</v>
       </c>
       <c r="BN8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO8" t="n">
         <v>32</v>
       </c>
-      <c r="BO8" t="n">
+      <c r="BP8" t="n">
         <v>32</v>
       </c>
     </row>
@@ -2502,9 +2529,12 @@
         <v>0</v>
       </c>
       <c r="BN9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO9" t="n">
         <v>31</v>
       </c>
-      <c r="BO9" t="n">
+      <c r="BP9" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2711,9 +2741,12 @@
         <v>0</v>
       </c>
       <c r="BN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO10" t="n">
         <v>39</v>
       </c>
-      <c r="BO10" t="n">
+      <c r="BP10" t="n">
         <v>39</v>
       </c>
     </row>
@@ -2920,9 +2953,12 @@
         <v>0</v>
       </c>
       <c r="BN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO11" t="n">
         <v>29</v>
       </c>
-      <c r="BO11" t="n">
+      <c r="BP11" t="n">
         <v>29</v>
       </c>
     </row>
@@ -3129,9 +3165,12 @@
         <v>0</v>
       </c>
       <c r="BN12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO12" t="n">
         <v>37</v>
       </c>
-      <c r="BO12" t="n">
+      <c r="BP12" t="n">
         <v>37</v>
       </c>
     </row>
@@ -3338,9 +3377,12 @@
         <v>0</v>
       </c>
       <c r="BN13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO13" t="n">
         <v>14</v>
       </c>
-      <c r="BO13" t="n">
+      <c r="BP13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3547,9 +3589,12 @@
         <v>0</v>
       </c>
       <c r="BN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO14" t="n">
         <v>26</v>
       </c>
-      <c r="BO14" t="n">
+      <c r="BP14" t="n">
         <v>26</v>
       </c>
     </row>
@@ -3756,9 +3801,12 @@
         <v>0</v>
       </c>
       <c r="BN15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO15" t="n">
         <v>9</v>
       </c>
-      <c r="BO15" t="n">
+      <c r="BP15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3965,9 +4013,12 @@
         <v>0</v>
       </c>
       <c r="BN16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO16" t="n">
         <v>20</v>
       </c>
-      <c r="BO16" t="n">
+      <c r="BP16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4174,9 +4225,12 @@
         <v>0</v>
       </c>
       <c r="BN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO17" t="n">
         <v>17</v>
       </c>
-      <c r="BO17" t="n">
+      <c r="BP17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4383,9 +4437,12 @@
         <v>0</v>
       </c>
       <c r="BN18" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO18" t="n">
         <v>33</v>
       </c>
-      <c r="BO18" t="n">
+      <c r="BP18" t="n">
         <v>33</v>
       </c>
     </row>
@@ -4597,6 +4654,9 @@
       <c r="BO19" t="n">
         <v>0</v>
       </c>
+      <c r="BP19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4801,9 +4861,12 @@
         <v>0</v>
       </c>
       <c r="BN20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO20" t="n">
         <v>20</v>
       </c>
-      <c r="BO20" t="n">
+      <c r="BP20" t="n">
         <v>20</v>
       </c>
     </row>
@@ -5010,9 +5073,12 @@
         <v>0</v>
       </c>
       <c r="BN21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO21" t="n">
         <v>27</v>
       </c>
-      <c r="BO21" t="n">
+      <c r="BP21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5224,6 +5290,9 @@
       <c r="BO22" t="n">
         <v>0</v>
       </c>
+      <c r="BP22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5428,9 +5497,12 @@
         <v>0</v>
       </c>
       <c r="BN23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO23" t="n">
         <v>22</v>
       </c>
-      <c r="BO23" t="n">
+      <c r="BP23" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5637,9 +5709,12 @@
         <v>0</v>
       </c>
       <c r="BN24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO24" t="n">
         <v>27</v>
       </c>
-      <c r="BO24" t="n">
+      <c r="BP24" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5846,9 +5921,12 @@
         <v>0</v>
       </c>
       <c r="BN25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO25" t="n">
         <v>11</v>
       </c>
-      <c r="BO25" t="n">
+      <c r="BP25" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6055,9 +6133,12 @@
         <v>0</v>
       </c>
       <c r="BN26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO26" t="n">
         <v>35</v>
       </c>
-      <c r="BO26" t="n">
+      <c r="BP26" t="n">
         <v>35</v>
       </c>
     </row>
@@ -6264,9 +6345,12 @@
         <v>0</v>
       </c>
       <c r="BN27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO27" t="n">
         <v>25</v>
       </c>
-      <c r="BO27" t="n">
+      <c r="BP27" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6473,9 +6557,12 @@
         <v>0</v>
       </c>
       <c r="BN28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO28" t="n">
         <v>19</v>
       </c>
-      <c r="BO28" t="n">
+      <c r="BP28" t="n">
         <v>19</v>
       </c>
     </row>
@@ -6682,9 +6769,12 @@
         <v>0</v>
       </c>
       <c r="BN29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO29" t="n">
         <v>11</v>
       </c>
-      <c r="BO29" t="n">
+      <c r="BP29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6891,9 +6981,12 @@
         <v>0</v>
       </c>
       <c r="BN30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO30" t="n">
         <v>25</v>
       </c>
-      <c r="BO30" t="n">
+      <c r="BP30" t="n">
         <v>25</v>
       </c>
     </row>
@@ -7100,9 +7193,12 @@
         <v>0</v>
       </c>
       <c r="BN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO31" t="n">
         <v>20</v>
       </c>
-      <c r="BO31" t="n">
+      <c r="BP31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -7309,9 +7405,12 @@
         <v>0</v>
       </c>
       <c r="BN32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO32" t="n">
         <v>23</v>
       </c>
-      <c r="BO32" t="n">
+      <c r="BP32" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7518,9 +7617,12 @@
         <v>0</v>
       </c>
       <c r="BN33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO33" t="n">
         <v>21</v>
       </c>
-      <c r="BO33" t="n">
+      <c r="BP33" t="n">
         <v>21</v>
       </c>
     </row>
@@ -7727,9 +7829,12 @@
         <v>0</v>
       </c>
       <c r="BN34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO34" t="n">
         <v>9</v>
       </c>
-      <c r="BO34" t="n">
+      <c r="BP34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7936,9 +8041,12 @@
         <v>0</v>
       </c>
       <c r="BN35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO35" t="n">
         <v>25</v>
       </c>
-      <c r="BO35" t="n">
+      <c r="BP35" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8145,9 +8253,12 @@
         <v>0</v>
       </c>
       <c r="BN36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO36" t="n">
         <v>16</v>
       </c>
-      <c r="BO36" t="n">
+      <c r="BP36" t="n">
         <v>16</v>
       </c>
     </row>
@@ -8359,6 +8470,9 @@
       <c r="BO37" t="n">
         <v>0</v>
       </c>
+      <c r="BP37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8563,9 +8677,12 @@
         <v>0</v>
       </c>
       <c r="BN38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO38" t="n">
         <v>2</v>
       </c>
-      <c r="BO38" t="n">
+      <c r="BP38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8772,9 +8889,12 @@
         <v>0</v>
       </c>
       <c r="BN39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO39" t="n">
         <v>37</v>
       </c>
-      <c r="BO39" t="n">
+      <c r="BP39" t="n">
         <v>37</v>
       </c>
     </row>
@@ -8981,9 +9101,12 @@
         <v>0</v>
       </c>
       <c r="BN40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO40" t="n">
         <v>28</v>
       </c>
-      <c r="BO40" t="n">
+      <c r="BP40" t="n">
         <v>28</v>
       </c>
     </row>
@@ -9190,9 +9313,12 @@
         <v>0</v>
       </c>
       <c r="BN41" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO41" t="n">
         <v>39</v>
       </c>
-      <c r="BO41" t="n">
+      <c r="BP41" t="n">
         <v>39</v>
       </c>
     </row>
@@ -9399,9 +9525,12 @@
         <v>0</v>
       </c>
       <c r="BN42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO42" t="n">
         <v>21</v>
       </c>
-      <c r="BO42" t="n">
+      <c r="BP42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9608,9 +9737,12 @@
         <v>0</v>
       </c>
       <c r="BN43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO43" t="n">
         <v>60</v>
       </c>
-      <c r="BO43" t="n">
+      <c r="BP43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9817,9 +9949,12 @@
         <v>0</v>
       </c>
       <c r="BN44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO44" t="n">
         <v>25</v>
       </c>
-      <c r="BO44" t="n">
+      <c r="BP44" t="n">
         <v>25</v>
       </c>
     </row>
@@ -10026,9 +10161,12 @@
         <v>0</v>
       </c>
       <c r="BN45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO45" t="n">
         <v>26</v>
       </c>
-      <c r="BO45" t="n">
+      <c r="BP45" t="n">
         <v>26</v>
       </c>
     </row>
@@ -10235,9 +10373,12 @@
         <v>0</v>
       </c>
       <c r="BN46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO46" t="n">
         <v>30</v>
       </c>
-      <c r="BO46" t="n">
+      <c r="BP46" t="n">
         <v>30</v>
       </c>
     </row>
@@ -10449,6 +10590,9 @@
       <c r="BO47" t="n">
         <v>0</v>
       </c>
+      <c r="BP47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -10653,9 +10797,12 @@
         <v>0</v>
       </c>
       <c r="BN48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO48" t="n">
         <v>27</v>
       </c>
-      <c r="BO48" t="n">
+      <c r="BP48" t="n">
         <v>27</v>
       </c>
     </row>
@@ -10862,9 +11009,12 @@
         <v>0</v>
       </c>
       <c r="BN49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO49" t="n">
         <v>19</v>
       </c>
-      <c r="BO49" t="n">
+      <c r="BP49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -11071,9 +11221,12 @@
         <v>0</v>
       </c>
       <c r="BN50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO50" t="n">
         <v>7</v>
       </c>
-      <c r="BO50" t="n">
+      <c r="BP50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11280,9 +11433,12 @@
         <v>0</v>
       </c>
       <c r="BN51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO51" t="n">
         <v>32</v>
       </c>
-      <c r="BO51" t="n">
+      <c r="BP51" t="n">
         <v>32</v>
       </c>
     </row>
@@ -11494,6 +11650,9 @@
       <c r="BO52" t="n">
         <v>0</v>
       </c>
+      <c r="BP52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11698,9 +11857,12 @@
         <v>0</v>
       </c>
       <c r="BN53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO53" t="n">
         <v>13</v>
       </c>
-      <c r="BO53" t="n">
+      <c r="BP53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -11912,6 +12074,9 @@
       <c r="BO54" t="n">
         <v>0</v>
       </c>
+      <c r="BP54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -12116,9 +12281,12 @@
         <v>0</v>
       </c>
       <c r="BN55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO55" t="n">
         <v>36</v>
       </c>
-      <c r="BO55" t="n">
+      <c r="BP55" t="n">
         <v>36</v>
       </c>
     </row>
@@ -12325,9 +12493,12 @@
         <v>0</v>
       </c>
       <c r="BN56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO56" t="n">
         <v>31</v>
       </c>
-      <c r="BO56" t="n">
+      <c r="BP56" t="n">
         <v>31</v>
       </c>
     </row>
@@ -12534,9 +12705,12 @@
         <v>0</v>
       </c>
       <c r="BN57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO57" t="n">
         <v>10</v>
       </c>
-      <c r="BO57" t="n">
+      <c r="BP57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -12743,9 +12917,12 @@
         <v>0</v>
       </c>
       <c r="BN58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO58" t="n">
         <v>13</v>
       </c>
-      <c r="BO58" t="n">
+      <c r="BP58" t="n">
         <v>13</v>
       </c>
     </row>
@@ -12952,9 +13129,12 @@
         <v>0</v>
       </c>
       <c r="BN59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO59" t="n">
         <v>6</v>
       </c>
-      <c r="BO59" t="n">
+      <c r="BP59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -13166,6 +13346,9 @@
       <c r="BO60" t="n">
         <v>0</v>
       </c>
+      <c r="BP60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -13370,9 +13553,12 @@
         <v>0</v>
       </c>
       <c r="BN61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO61" t="n">
         <v>29</v>
       </c>
-      <c r="BO61" t="n">
+      <c r="BP61" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13579,9 +13765,12 @@
         <v>0</v>
       </c>
       <c r="BN62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO62" t="n">
         <v>29</v>
       </c>
-      <c r="BO62" t="n">
+      <c r="BP62" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13788,9 +13977,12 @@
         <v>0</v>
       </c>
       <c r="BN63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO63" t="n">
         <v>12</v>
       </c>
-      <c r="BO63" t="n">
+      <c r="BP63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -14002,6 +14194,9 @@
       <c r="BO64" t="n">
         <v>0</v>
       </c>
+      <c r="BP64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -14206,9 +14401,12 @@
         <v>0</v>
       </c>
       <c r="BN65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO65" t="n">
         <v>17</v>
       </c>
-      <c r="BO65" t="n">
+      <c r="BP65" t="n">
         <v>17</v>
       </c>
     </row>
@@ -14415,9 +14613,12 @@
         <v>0</v>
       </c>
       <c r="BN66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO66" t="n">
         <v>8</v>
       </c>
-      <c r="BO66" t="n">
+      <c r="BP66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -14624,9 +14825,12 @@
         <v>0</v>
       </c>
       <c r="BN67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO67" t="n">
         <v>40</v>
       </c>
-      <c r="BO67" t="n">
+      <c r="BP67" t="n">
         <v>40</v>
       </c>
     </row>
@@ -14833,9 +15037,12 @@
         <v>0</v>
       </c>
       <c r="BN68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO68" t="n">
         <v>23</v>
       </c>
-      <c r="BO68" t="n">
+      <c r="BP68" t="n">
         <v>22</v>
       </c>
     </row>
@@ -15042,9 +15249,12 @@
         <v>0</v>
       </c>
       <c r="BN69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO69" t="n">
         <v>7</v>
       </c>
-      <c r="BO69" t="n">
+      <c r="BP69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15251,9 +15461,12 @@
         <v>0</v>
       </c>
       <c r="BN70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO70" t="n">
         <v>23</v>
       </c>
-      <c r="BO70" t="n">
+      <c r="BP70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -15460,9 +15673,12 @@
         <v>0</v>
       </c>
       <c r="BN71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO71" t="n">
         <v>24</v>
       </c>
-      <c r="BO71" t="n">
+      <c r="BP71" t="n">
         <v>24</v>
       </c>
     </row>
@@ -15669,9 +15885,12 @@
         <v>0</v>
       </c>
       <c r="BN72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO72" t="n">
         <v>24</v>
       </c>
-      <c r="BO72" t="n">
+      <c r="BP72" t="n">
         <v>24</v>
       </c>
     </row>
@@ -15883,6 +16102,9 @@
       <c r="BO73" t="n">
         <v>0</v>
       </c>
+      <c r="BP73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -16092,6 +16314,9 @@
       <c r="BO74" t="n">
         <v>0</v>
       </c>
+      <c r="BP74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -16296,9 +16521,12 @@
         <v>0</v>
       </c>
       <c r="BN75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO75" t="n">
         <v>25</v>
       </c>
-      <c r="BO75" t="n">
+      <c r="BP75" t="n">
         <v>25</v>
       </c>
     </row>
@@ -16505,9 +16733,12 @@
         <v>0</v>
       </c>
       <c r="BN76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO76" t="n">
         <v>21</v>
       </c>
-      <c r="BO76" t="n">
+      <c r="BP76" t="n">
         <v>21</v>
       </c>
     </row>
@@ -16714,9 +16945,12 @@
         <v>0</v>
       </c>
       <c r="BN77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO77" t="n">
         <v>15</v>
       </c>
-      <c r="BO77" t="n">
+      <c r="BP77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -16923,9 +17157,12 @@
         <v>0</v>
       </c>
       <c r="BN78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO78" t="n">
         <v>36</v>
       </c>
-      <c r="BO78" t="n">
+      <c r="BP78" t="n">
         <v>35</v>
       </c>
     </row>
@@ -17132,9 +17369,12 @@
         <v>0</v>
       </c>
       <c r="BN79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO79" t="n">
         <v>22</v>
       </c>
-      <c r="BO79" t="n">
+      <c r="BP79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -17341,9 +17581,12 @@
         <v>0</v>
       </c>
       <c r="BN80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO80" t="n">
         <v>12</v>
       </c>
-      <c r="BO80" t="n">
+      <c r="BP80" t="n">
         <v>12</v>
       </c>
     </row>
@@ -17550,9 +17793,12 @@
         <v>0</v>
       </c>
       <c r="BN81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO81" t="n">
         <v>4</v>
       </c>
-      <c r="BO81" t="n">
+      <c r="BP81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -17759,9 +18005,12 @@
         <v>0</v>
       </c>
       <c r="BN82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO82" t="n">
         <v>18</v>
       </c>
-      <c r="BO82" t="n">
+      <c r="BP82" t="n">
         <v>18</v>
       </c>
     </row>
@@ -17968,9 +18217,12 @@
         <v>0</v>
       </c>
       <c r="BN83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO83" t="n">
         <v>17</v>
       </c>
-      <c r="BO83" t="n">
+      <c r="BP83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -18177,9 +18429,12 @@
         <v>0</v>
       </c>
       <c r="BN84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO84" t="n">
         <v>13</v>
       </c>
-      <c r="BO84" t="n">
+      <c r="BP84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -18386,9 +18641,12 @@
         <v>0</v>
       </c>
       <c r="BN85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO85" t="n">
         <v>7</v>
       </c>
-      <c r="BO85" t="n">
+      <c r="BP85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18600,6 +18858,9 @@
       <c r="BO86" t="n">
         <v>0</v>
       </c>
+      <c r="BP86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -18804,9 +19065,12 @@
         <v>0</v>
       </c>
       <c r="BN87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO87" t="n">
         <v>19</v>
       </c>
-      <c r="BO87" t="n">
+      <c r="BP87" t="n">
         <v>19</v>
       </c>
     </row>
@@ -19018,6 +19282,9 @@
       <c r="BO88" t="n">
         <v>0</v>
       </c>
+      <c r="BP88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -19222,9 +19489,12 @@
         <v>0</v>
       </c>
       <c r="BN89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO89" t="n">
         <v>18</v>
       </c>
-      <c r="BO89" t="n">
+      <c r="BP89" t="n">
         <v>18</v>
       </c>
     </row>
@@ -19431,9 +19701,12 @@
         <v>0</v>
       </c>
       <c r="BN90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO90" t="n">
         <v>17</v>
       </c>
-      <c r="BO90" t="n">
+      <c r="BP90" t="n">
         <v>17</v>
       </c>
     </row>
@@ -19640,9 +19913,12 @@
         <v>0</v>
       </c>
       <c r="BN91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO91" t="n">
         <v>42</v>
       </c>
-      <c r="BO91" t="n">
+      <c r="BP91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -19849,9 +20125,12 @@
         <v>0</v>
       </c>
       <c r="BN92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO92" t="n">
         <v>7</v>
       </c>
-      <c r="BO92" t="n">
+      <c r="BP92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -20063,6 +20342,9 @@
       <c r="BO93" t="n">
         <v>0</v>
       </c>
+      <c r="BP93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -20267,9 +20549,12 @@
         <v>0</v>
       </c>
       <c r="BN94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO94" t="n">
         <v>16</v>
       </c>
-      <c r="BO94" t="n">
+      <c r="BP94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -20476,9 +20761,12 @@
         <v>0</v>
       </c>
       <c r="BN95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO95" t="n">
         <v>7</v>
       </c>
-      <c r="BO95" t="n">
+      <c r="BP95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -20685,9 +20973,12 @@
         <v>0</v>
       </c>
       <c r="BN96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO96" t="n">
         <v>24</v>
       </c>
-      <c r="BO96" t="n">
+      <c r="BP96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -20899,6 +21190,9 @@
       <c r="BO97" t="n">
         <v>0</v>
       </c>
+      <c r="BP97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -21103,9 +21397,12 @@
         <v>0</v>
       </c>
       <c r="BN98" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO98" t="n">
         <v>35</v>
       </c>
-      <c r="BO98" t="n">
+      <c r="BP98" t="n">
         <v>35</v>
       </c>
     </row>
@@ -21312,9 +21609,12 @@
         <v>0</v>
       </c>
       <c r="BN99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO99" t="n">
         <v>14</v>
       </c>
-      <c r="BO99" t="n">
+      <c r="BP99" t="n">
         <v>14</v>
       </c>
     </row>
@@ -21526,6 +21826,9 @@
       <c r="BO100" t="n">
         <v>0</v>
       </c>
+      <c r="BP100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -21730,10 +22033,13 @@
         <v>0</v>
       </c>
       <c r="BN101" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="BO101" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="BP101" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="102">
@@ -21939,9 +22245,12 @@
         <v>0</v>
       </c>
       <c r="BN102" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO102" t="n">
         <v>31</v>
       </c>
-      <c r="BO102" t="n">
+      <c r="BP102" t="n">
         <v>31</v>
       </c>
     </row>
@@ -22148,9 +22457,12 @@
         <v>0</v>
       </c>
       <c r="BN103" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO103" t="n">
         <v>34</v>
       </c>
-      <c r="BO103" t="n">
+      <c r="BP103" t="n">
         <v>34</v>
       </c>
     </row>
@@ -22357,9 +22669,12 @@
         <v>0</v>
       </c>
       <c r="BN104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO104" t="n">
         <v>12</v>
       </c>
-      <c r="BO104" t="n">
+      <c r="BP104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -22566,9 +22881,12 @@
         <v>0</v>
       </c>
       <c r="BN105" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO105" t="n">
         <v>28</v>
       </c>
-      <c r="BO105" t="n">
+      <c r="BP105" t="n">
         <v>28</v>
       </c>
     </row>
@@ -22775,9 +23093,12 @@
         <v>0</v>
       </c>
       <c r="BN106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO106" t="n">
         <v>7</v>
       </c>
-      <c r="BO106" t="n">
+      <c r="BP106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -22984,9 +23305,12 @@
         <v>0</v>
       </c>
       <c r="BN107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO107" t="n">
         <v>13</v>
       </c>
-      <c r="BO107" t="n">
+      <c r="BP107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -23193,9 +23517,12 @@
         <v>0</v>
       </c>
       <c r="BN108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO108" t="n">
         <v>2</v>
       </c>
-      <c r="BO108" t="n">
+      <c r="BP108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -23402,9 +23729,12 @@
         <v>0</v>
       </c>
       <c r="BN109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO109" t="n">
         <v>4</v>
       </c>
-      <c r="BO109" t="n">
+      <c r="BP109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>